<commit_message>
070 => fase IV => backlog millores pendents, ZUP-023 OK (Chrome/USER) i backup Excel proves
</commit_message>
<xml_diff>
--- a/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
+++ b/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4271" uniqueCount="713">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4272" uniqueCount="714">
   <si>
     <t>Zuppeto — Joc de probes manual (totes les pantalles)</t>
   </si>
@@ -558,6 +558,9 @@
   </si>
   <si>
     <t>Cada pantalla carrega sense error 404 ni pantalla en blanc</t>
+  </si>
+  <si>
+    <t>23-08-2026</t>
   </si>
   <si>
     <t>DEVELOPER</t>
@@ -6736,9 +6739,11 @@
       <c r="H140" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="I140" s="29"/>
+      <c r="I140" s="29" t="s">
+        <v>178</v>
+      </c>
       <c r="J140" s="17" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K140" s="15"/>
       <c r="L140" s="1"/>
@@ -6866,7 +6871,7 @@
         <v>58</v>
       </c>
       <c r="H146" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I146" s="18"/>
       <c r="J146" s="17" t="s">
@@ -6888,7 +6893,7 @@
         <v>61</v>
       </c>
       <c r="H147" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I147" s="18"/>
       <c r="J147" s="17" t="s">
@@ -6910,7 +6915,7 @@
         <v>62</v>
       </c>
       <c r="H148" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I148" s="18"/>
       <c r="J148" s="17" t="s">
@@ -6932,7 +6937,7 @@
         <v>63</v>
       </c>
       <c r="H149" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I149" s="18"/>
       <c r="J149" s="17" t="s">
@@ -6954,7 +6959,7 @@
         <v>64</v>
       </c>
       <c r="H150" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I150" s="18"/>
       <c r="J150" s="17" t="s">
@@ -6976,7 +6981,7 @@
         <v>65</v>
       </c>
       <c r="H151" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I151" s="18"/>
       <c r="J151" s="17" t="s">
@@ -7127,16 +7132,16 @@
         <v>53</v>
       </c>
       <c r="C158" s="27" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D158" s="28" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="E158" s="28" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F158" s="28" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="G158" s="16" t="s">
         <v>58</v>
@@ -7406,7 +7411,7 @@
         <v>58</v>
       </c>
       <c r="H170" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I170" s="18"/>
       <c r="J170" s="17" t="s">
@@ -7428,7 +7433,7 @@
         <v>61</v>
       </c>
       <c r="H171" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I171" s="18"/>
       <c r="J171" s="17" t="s">
@@ -7450,7 +7455,7 @@
         <v>62</v>
       </c>
       <c r="H172" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I172" s="18"/>
       <c r="J172" s="17" t="s">
@@ -7472,7 +7477,7 @@
         <v>63</v>
       </c>
       <c r="H173" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I173" s="18"/>
       <c r="J173" s="17" t="s">
@@ -7494,7 +7499,7 @@
         <v>64</v>
       </c>
       <c r="H174" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I174" s="18"/>
       <c r="J174" s="17" t="s">
@@ -7516,7 +7521,7 @@
         <v>65</v>
       </c>
       <c r="H175" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I175" s="18"/>
       <c r="J175" s="17" t="s">
@@ -7667,16 +7672,16 @@
         <v>90</v>
       </c>
       <c r="C182" s="14" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D182" s="15" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="E182" s="15" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F182" s="15" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="G182" s="16" t="s">
         <v>58</v>
@@ -7811,16 +7816,16 @@
         <v>53</v>
       </c>
       <c r="C188" s="27" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="D188" s="28" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="E188" s="28" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F188" s="28" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="G188" s="16" t="s">
         <v>58</v>
@@ -7949,28 +7954,28 @@
     </row>
     <row r="194" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A194" s="36" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B194" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C194" s="14" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D194" s="15" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E194" s="15" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="F194" s="15" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G194" s="16" t="s">
         <v>58</v>
       </c>
       <c r="H194" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I194" s="18"/>
       <c r="J194" s="17" t="s">
@@ -7992,7 +7997,7 @@
         <v>61</v>
       </c>
       <c r="H195" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I195" s="18"/>
       <c r="J195" s="17" t="s">
@@ -8014,7 +8019,7 @@
         <v>62</v>
       </c>
       <c r="H196" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I196" s="18"/>
       <c r="J196" s="17" t="s">
@@ -8036,7 +8041,7 @@
         <v>63</v>
       </c>
       <c r="H197" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I197" s="18"/>
       <c r="J197" s="17" t="s">
@@ -8058,7 +8063,7 @@
         <v>64</v>
       </c>
       <c r="H198" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I198" s="18"/>
       <c r="J198" s="17" t="s">
@@ -8080,7 +8085,7 @@
         <v>65</v>
       </c>
       <c r="H199" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I199" s="18"/>
       <c r="J199" s="17" t="s">
@@ -8093,22 +8098,22 @@
     </row>
     <row r="200" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A200" s="36" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B200" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C200" s="27" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="D200" s="28" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="E200" s="28" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F200" s="28" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="G200" s="16" t="s">
         <v>58</v>
@@ -8237,22 +8242,22 @@
     </row>
     <row r="206" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A206" s="36" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B206" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C206" s="14" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D206" s="15" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="E206" s="15" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="F206" s="15" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="G206" s="16" t="s">
         <v>58</v>
@@ -8381,22 +8386,22 @@
     </row>
     <row r="212" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A212" s="37" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B212" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C212" s="27" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="D212" s="28" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="E212" s="28" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="F212" s="28" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="G212" s="16" t="s">
         <v>58</v>
@@ -8666,7 +8671,7 @@
         <v>58</v>
       </c>
       <c r="H224" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I224" s="18"/>
       <c r="J224" s="17" t="s">
@@ -8688,7 +8693,7 @@
         <v>61</v>
       </c>
       <c r="H225" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I225" s="18"/>
       <c r="J225" s="17" t="s">
@@ -8710,7 +8715,7 @@
         <v>62</v>
       </c>
       <c r="H226" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I226" s="18"/>
       <c r="J226" s="17" t="s">
@@ -8732,7 +8737,7 @@
         <v>63</v>
       </c>
       <c r="H227" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I227" s="18"/>
       <c r="J227" s="17" t="s">
@@ -8754,7 +8759,7 @@
         <v>64</v>
       </c>
       <c r="H228" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I228" s="18"/>
       <c r="J228" s="17" t="s">
@@ -8776,7 +8781,7 @@
         <v>65</v>
       </c>
       <c r="H229" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I229" s="18"/>
       <c r="J229" s="17" t="s">
@@ -8921,22 +8926,22 @@
     </row>
     <row r="236" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A236" s="37" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B236" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C236" s="14" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D236" s="15" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="E236" s="15" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="F236" s="15" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="G236" s="16" t="s">
         <v>58</v>
@@ -9065,22 +9070,22 @@
     </row>
     <row r="242" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A242" s="37" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B242" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C242" s="27" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="D242" s="28" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="E242" s="28" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="F242" s="28" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="G242" s="16" t="s">
         <v>58</v>
@@ -9209,22 +9214,22 @@
     </row>
     <row r="248" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A248" s="37" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B248" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C248" s="14" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D248" s="15" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="E248" s="15" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="F248" s="15" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="G248" s="16" t="s">
         <v>58</v>
@@ -9353,22 +9358,22 @@
     </row>
     <row r="254" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A254" s="37" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B254" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C254" s="27" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="D254" s="28" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="E254" s="28" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="F254" s="28" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="G254" s="16" t="s">
         <v>58</v>
@@ -9497,22 +9502,22 @@
     </row>
     <row r="260" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A260" s="37" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B260" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C260" s="14" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="D260" s="15" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="E260" s="15" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="F260" s="15" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="G260" s="16" t="s">
         <v>58</v>
@@ -9641,22 +9646,22 @@
     </row>
     <row r="266" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A266" s="37" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B266" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C266" s="27" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="D266" s="28" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E266" s="28" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="F266" s="28" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="G266" s="16" t="s">
         <v>58</v>
@@ -9785,22 +9790,22 @@
     </row>
     <row r="272" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A272" s="37" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B272" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C272" s="14" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D272" s="15" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E272" s="15" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="F272" s="15" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="G272" s="16" t="s">
         <v>58</v>
@@ -9929,22 +9934,22 @@
     </row>
     <row r="278" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A278" s="38" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B278" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C278" s="27" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="D278" s="28" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="E278" s="28" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="F278" s="28" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="G278" s="16" t="s">
         <v>58</v>
@@ -10214,7 +10219,7 @@
         <v>58</v>
       </c>
       <c r="H290" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I290" s="18"/>
       <c r="J290" s="17" t="s">
@@ -10236,7 +10241,7 @@
         <v>61</v>
       </c>
       <c r="H291" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I291" s="18"/>
       <c r="J291" s="17" t="s">
@@ -10258,7 +10263,7 @@
         <v>62</v>
       </c>
       <c r="H292" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I292" s="18"/>
       <c r="J292" s="17" t="s">
@@ -10280,7 +10285,7 @@
         <v>63</v>
       </c>
       <c r="H293" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I293" s="18"/>
       <c r="J293" s="17" t="s">
@@ -10302,7 +10307,7 @@
         <v>64</v>
       </c>
       <c r="H294" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I294" s="18"/>
       <c r="J294" s="17" t="s">
@@ -10324,7 +10329,7 @@
         <v>65</v>
       </c>
       <c r="H295" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I295" s="18"/>
       <c r="J295" s="17" t="s">
@@ -10469,22 +10474,22 @@
     </row>
     <row r="302" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A302" s="38" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B302" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C302" s="14" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="D302" s="15" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="E302" s="15" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="F302" s="15" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="G302" s="16" t="s">
         <v>58</v>
@@ -10613,22 +10618,22 @@
     </row>
     <row r="308" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A308" s="38" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B308" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C308" s="27" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="D308" s="28" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="E308" s="28" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="F308" s="28" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="G308" s="16" t="s">
         <v>58</v>
@@ -10757,22 +10762,22 @@
     </row>
     <row r="314" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A314" s="38" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B314" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C314" s="14" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="D314" s="15" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="E314" s="15" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="F314" s="15" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="G314" s="16" t="s">
         <v>58</v>
@@ -10901,22 +10906,22 @@
     </row>
     <row r="320" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A320" s="38" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B320" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C320" s="27" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D320" s="28" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="E320" s="28" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="F320" s="28" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="G320" s="16" t="s">
         <v>58</v>
@@ -11045,22 +11050,22 @@
     </row>
     <row r="326" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A326" s="38" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B326" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C326" s="14" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D326" s="15" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="E326" s="15" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="F326" s="15" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="G326" s="16" t="s">
         <v>58</v>
@@ -11189,22 +11194,22 @@
     </row>
     <row r="332" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A332" s="38" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B332" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C332" s="27" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D332" s="28" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="E332" s="28" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="F332" s="28" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="G332" s="16" t="s">
         <v>58</v>
@@ -11333,22 +11338,22 @@
     </row>
     <row r="338" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A338" s="38" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B338" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C338" s="14" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D338" s="15" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="E338" s="15" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="F338" s="15" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="G338" s="16" t="s">
         <v>58</v>
@@ -11477,22 +11482,22 @@
     </row>
     <row r="344" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A344" s="38" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B344" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C344" s="27" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D344" s="28" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="E344" s="28" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F344" s="28" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="G344" s="16" t="s">
         <v>58</v>
@@ -11621,22 +11626,22 @@
     </row>
     <row r="350" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A350" s="38" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B350" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C350" s="14" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="D350" s="15" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="E350" s="15" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="F350" s="15" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="G350" s="16" t="s">
         <v>58</v>
@@ -11765,22 +11770,22 @@
     </row>
     <row r="356" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A356" s="38" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B356" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C356" s="27" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="D356" s="28" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="E356" s="28" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="F356" s="28" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="G356" s="16" t="s">
         <v>58</v>
@@ -11909,22 +11914,22 @@
     </row>
     <row r="362" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A362" s="38" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B362" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C362" s="14" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D362" s="15" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="E362" s="15" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="F362" s="15" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="G362" s="16" t="s">
         <v>58</v>
@@ -12053,22 +12058,22 @@
     </row>
     <row r="368" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A368" s="38" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B368" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C368" s="27" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="D368" s="28" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E368" s="28" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="F368" s="28" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="G368" s="16" t="s">
         <v>58</v>
@@ -12197,22 +12202,22 @@
     </row>
     <row r="374" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A374" s="38" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B374" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C374" s="14" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="D374" s="15" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="E374" s="15" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="F374" s="15" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="G374" s="16" t="s">
         <v>58</v>
@@ -12341,22 +12346,22 @@
     </row>
     <row r="380" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A380" s="38" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B380" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C380" s="27" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="D380" s="28" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="E380" s="28" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="F380" s="28" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="G380" s="16" t="s">
         <v>58</v>
@@ -12485,22 +12490,22 @@
     </row>
     <row r="386" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A386" s="38" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B386" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C386" s="14" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="D386" s="15" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E386" s="15" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="F386" s="15" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="G386" s="16" t="s">
         <v>58</v>
@@ -12629,22 +12634,22 @@
     </row>
     <row r="392" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A392" s="38" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B392" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C392" s="27" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D392" s="28" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="E392" s="28" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="F392" s="28" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="G392" s="16" t="s">
         <v>58</v>
@@ -12773,22 +12778,22 @@
     </row>
     <row r="398" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A398" s="39" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B398" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C398" s="14" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="D398" s="15" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="E398" s="15" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="F398" s="15" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="G398" s="16" t="s">
         <v>58</v>
@@ -13058,7 +13063,7 @@
         <v>58</v>
       </c>
       <c r="H410" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I410" s="18"/>
       <c r="J410" s="17" t="s">
@@ -13080,7 +13085,7 @@
         <v>61</v>
       </c>
       <c r="H411" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I411" s="18"/>
       <c r="J411" s="17" t="s">
@@ -13102,7 +13107,7 @@
         <v>62</v>
       </c>
       <c r="H412" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I412" s="18"/>
       <c r="J412" s="17" t="s">
@@ -13124,7 +13129,7 @@
         <v>63</v>
       </c>
       <c r="H413" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I413" s="18"/>
       <c r="J413" s="17" t="s">
@@ -13146,7 +13151,7 @@
         <v>64</v>
       </c>
       <c r="H414" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I414" s="18"/>
       <c r="J414" s="17" t="s">
@@ -13168,7 +13173,7 @@
         <v>65</v>
       </c>
       <c r="H415" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I415" s="18"/>
       <c r="J415" s="17" t="s">
@@ -13313,22 +13318,22 @@
     </row>
     <row r="422" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A422" s="39" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B422" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C422" s="27" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="D422" s="28" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E422" s="28" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="F422" s="28" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="G422" s="16" t="s">
         <v>58</v>
@@ -13457,22 +13462,22 @@
     </row>
     <row r="428" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A428" s="39" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B428" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C428" s="14" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="D428" s="15" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E428" s="15" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="F428" s="15" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="G428" s="16" t="s">
         <v>58</v>
@@ -13601,22 +13606,22 @@
     </row>
     <row r="434" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A434" s="39" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B434" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C434" s="27" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="D434" s="28" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="E434" s="28" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="F434" s="28" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="G434" s="16" t="s">
         <v>58</v>
@@ -13745,22 +13750,22 @@
     </row>
     <row r="440" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A440" s="39" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B440" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C440" s="14" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="D440" s="15" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="E440" s="15" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="F440" s="15" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="G440" s="16" t="s">
         <v>58</v>
@@ -13889,22 +13894,22 @@
     </row>
     <row r="446" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A446" s="39" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B446" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C446" s="27" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="D446" s="28" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="E446" s="28" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="F446" s="28" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="G446" s="16" t="s">
         <v>58</v>
@@ -14033,22 +14038,22 @@
     </row>
     <row r="452" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A452" s="39" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B452" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C452" s="14" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D452" s="15" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="E452" s="15" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="F452" s="15" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G452" s="16" t="s">
         <v>58</v>
@@ -14177,22 +14182,22 @@
     </row>
     <row r="458" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A458" s="39" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B458" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C458" s="27" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="D458" s="28" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="E458" s="28" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="F458" s="28" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="G458" s="16" t="s">
         <v>58</v>
@@ -14321,22 +14326,22 @@
     </row>
     <row r="464" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A464" s="39" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B464" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C464" s="14" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="D464" s="15" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="E464" s="15" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="F464" s="15" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="G464" s="16" t="s">
         <v>58</v>
@@ -14465,22 +14470,22 @@
     </row>
     <row r="470" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A470" s="39" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B470" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C470" s="27" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="D470" s="28" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="E470" s="28" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="F470" s="28" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="G470" s="16" t="s">
         <v>58</v>
@@ -14609,22 +14614,22 @@
     </row>
     <row r="476" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A476" s="40" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B476" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C476" s="14" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="D476" s="15" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="E476" s="15" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="F476" s="15" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="G476" s="16" t="s">
         <v>58</v>
@@ -14753,22 +14758,22 @@
     </row>
     <row r="482" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A482" s="40" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B482" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C482" s="27" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="D482" s="28" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="E482" s="28" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="F482" s="28" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="G482" s="16" t="s">
         <v>58</v>
@@ -14897,22 +14902,22 @@
     </row>
     <row r="488" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A488" s="40" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B488" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C488" s="14" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="D488" s="15" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="E488" s="15" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="F488" s="15" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="G488" s="16" t="s">
         <v>58</v>
@@ -15041,22 +15046,22 @@
     </row>
     <row r="494" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A494" s="40" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B494" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C494" s="27" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="D494" s="28" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="E494" s="28" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="F494" s="28" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="G494" s="16" t="s">
         <v>58</v>
@@ -15185,22 +15190,22 @@
     </row>
     <row r="500" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A500" s="40" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B500" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C500" s="14" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="D500" s="15" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="E500" s="15" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="F500" s="15" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="G500" s="16" t="s">
         <v>58</v>
@@ -15329,22 +15334,22 @@
     </row>
     <row r="506" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A506" s="40" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B506" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C506" s="27" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="D506" s="28" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="E506" s="28" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="F506" s="28" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="G506" s="16" t="s">
         <v>58</v>
@@ -15473,22 +15478,22 @@
     </row>
     <row r="512" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A512" s="40" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B512" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C512" s="14" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="D512" s="15" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E512" s="15" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="F512" s="15" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="G512" s="16" t="s">
         <v>58</v>
@@ -15617,22 +15622,22 @@
     </row>
     <row r="518" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A518" s="40" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B518" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C518" s="27" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="D518" s="28" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="E518" s="28" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="F518" s="28" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="G518" s="16" t="s">
         <v>58</v>
@@ -15761,22 +15766,22 @@
     </row>
     <row r="524" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A524" s="40" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B524" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C524" s="14" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="D524" s="15" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="E524" s="15" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="F524" s="15" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="G524" s="16" t="s">
         <v>58</v>
@@ -15905,22 +15910,22 @@
     </row>
     <row r="530" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A530" s="40" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B530" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C530" s="27" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="D530" s="28" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="E530" s="28" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="F530" s="28" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="G530" s="16" t="s">
         <v>58</v>
@@ -16049,22 +16054,22 @@
     </row>
     <row r="536" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A536" s="40" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B536" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C536" s="14" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="D536" s="15" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="E536" s="15" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="F536" s="15" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="G536" s="16" t="s">
         <v>58</v>
@@ -16193,22 +16198,22 @@
     </row>
     <row r="542" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A542" s="41" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B542" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C542" s="27" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="D542" s="28" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="E542" s="28" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="F542" s="28" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="G542" s="16" t="s">
         <v>58</v>
@@ -16337,22 +16342,22 @@
     </row>
     <row r="548" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A548" s="41" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B548" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C548" s="14" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="D548" s="15" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="E548" s="15" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="F548" s="15" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="G548" s="16" t="s">
         <v>58</v>
@@ -16481,22 +16486,22 @@
     </row>
     <row r="554" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A554" s="41" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B554" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C554" s="27" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="D554" s="28" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="E554" s="28" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="F554" s="28" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="G554" s="16" t="s">
         <v>58</v>
@@ -16625,22 +16630,22 @@
     </row>
     <row r="560" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A560" s="41" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B560" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C560" s="14" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="D560" s="15" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="E560" s="15" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="F560" s="15" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="G560" s="16" t="s">
         <v>58</v>
@@ -16769,22 +16774,22 @@
     </row>
     <row r="566" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A566" s="41" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B566" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C566" s="27" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="D566" s="28" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="E566" s="28" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="F566" s="28" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="G566" s="16" t="s">
         <v>58</v>
@@ -16913,22 +16918,22 @@
     </row>
     <row r="572" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A572" s="41" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B572" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C572" s="14" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="D572" s="15" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="E572" s="15" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="F572" s="15" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="G572" s="16" t="s">
         <v>58</v>
@@ -17057,22 +17062,22 @@
     </row>
     <row r="578" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A578" s="41" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B578" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C578" s="27" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="D578" s="28" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="E578" s="28" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="F578" s="28" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="G578" s="16" t="s">
         <v>58</v>
@@ -17201,22 +17206,22 @@
     </row>
     <row r="584" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A584" s="41" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B584" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C584" s="14" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="D584" s="15" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="E584" s="15" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="F584" s="15" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="G584" s="16" t="s">
         <v>58</v>
@@ -17345,22 +17350,22 @@
     </row>
     <row r="590" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A590" s="41" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B590" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C590" s="27" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="D590" s="28" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="E590" s="28" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="F590" s="28" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="G590" s="16" t="s">
         <v>58</v>
@@ -17489,22 +17494,22 @@
     </row>
     <row r="596" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A596" s="42" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="B596" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C596" s="14" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="D596" s="15" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="E596" s="15" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="F596" s="15" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="G596" s="16" t="s">
         <v>58</v>
@@ -17774,7 +17779,7 @@
         <v>58</v>
       </c>
       <c r="H608" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I608" s="18"/>
       <c r="J608" s="17" t="s">
@@ -17796,7 +17801,7 @@
         <v>61</v>
       </c>
       <c r="H609" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I609" s="18"/>
       <c r="J609" s="17" t="s">
@@ -17818,7 +17823,7 @@
         <v>62</v>
       </c>
       <c r="H610" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I610" s="18"/>
       <c r="J610" s="17" t="s">
@@ -17840,7 +17845,7 @@
         <v>63</v>
       </c>
       <c r="H611" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I611" s="18"/>
       <c r="J611" s="17" t="s">
@@ -17862,7 +17867,7 @@
         <v>64</v>
       </c>
       <c r="H612" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I612" s="18"/>
       <c r="J612" s="17" t="s">
@@ -17884,7 +17889,7 @@
         <v>65</v>
       </c>
       <c r="H613" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I613" s="18"/>
       <c r="J613" s="17" t="s">
@@ -18029,22 +18034,22 @@
     </row>
     <row r="620" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A620" s="42" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="B620" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C620" s="27" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="D620" s="28" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="E620" s="28" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="F620" s="28" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="G620" s="16" t="s">
         <v>58</v>
@@ -18173,22 +18178,22 @@
     </row>
     <row r="626" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A626" s="42" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="B626" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C626" s="14" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="D626" s="15" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="E626" s="15" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="F626" s="15" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="G626" s="16" t="s">
         <v>58</v>
@@ -18317,22 +18322,22 @@
     </row>
     <row r="632" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A632" s="42" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="B632" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C632" s="27" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="D632" s="28" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="E632" s="28" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="F632" s="28" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="G632" s="16" t="s">
         <v>58</v>
@@ -18461,22 +18466,22 @@
     </row>
     <row r="638" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A638" s="42" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="B638" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C638" s="14" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="D638" s="15" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="E638" s="15" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="F638" s="15" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="G638" s="16" t="s">
         <v>58</v>
@@ -18605,22 +18610,22 @@
     </row>
     <row r="644" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A644" s="43" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="B644" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C644" s="27" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="D644" s="28" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="E644" s="28" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="F644" s="28" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="G644" s="16" t="s">
         <v>58</v>
@@ -18890,7 +18895,7 @@
         <v>58</v>
       </c>
       <c r="H656" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I656" s="18"/>
       <c r="J656" s="17" t="s">
@@ -18912,7 +18917,7 @@
         <v>61</v>
       </c>
       <c r="H657" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I657" s="18"/>
       <c r="J657" s="17" t="s">
@@ -18934,7 +18939,7 @@
         <v>62</v>
       </c>
       <c r="H658" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I658" s="18"/>
       <c r="J658" s="17" t="s">
@@ -18956,7 +18961,7 @@
         <v>63</v>
       </c>
       <c r="H659" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I659" s="18"/>
       <c r="J659" s="17" t="s">
@@ -18978,7 +18983,7 @@
         <v>64</v>
       </c>
       <c r="H660" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I660" s="18"/>
       <c r="J660" s="17" t="s">
@@ -19000,7 +19005,7 @@
         <v>65</v>
       </c>
       <c r="H661" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I661" s="18"/>
       <c r="J661" s="17" t="s">
@@ -19145,22 +19150,22 @@
     </row>
     <row r="668" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A668" s="43" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="B668" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C668" s="14" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="D668" s="15" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="E668" s="15" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="F668" s="15" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="G668" s="16" t="s">
         <v>58</v>
@@ -19289,22 +19294,22 @@
     </row>
     <row r="674" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A674" s="43" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="B674" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C674" s="27" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="D674" s="28" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="E674" s="28" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="F674" s="28" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="G674" s="16" t="s">
         <v>58</v>
@@ -19433,22 +19438,22 @@
     </row>
     <row r="680" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A680" s="43" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="B680" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C680" s="14" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="D680" s="15" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="E680" s="15" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="F680" s="15" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="G680" s="16" t="s">
         <v>58</v>
@@ -19577,22 +19582,22 @@
     </row>
     <row r="686" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A686" s="43" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="B686" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C686" s="27" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="D686" s="28" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="E686" s="28" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="F686" s="28" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="G686" s="16" t="s">
         <v>58</v>
@@ -19721,22 +19726,22 @@
     </row>
     <row r="692" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A692" s="44" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="B692" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C692" s="14" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="D692" s="15" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="E692" s="15" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="F692" s="15" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="G692" s="16" t="s">
         <v>58</v>
@@ -20006,7 +20011,7 @@
         <v>58</v>
       </c>
       <c r="H704" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I704" s="18"/>
       <c r="J704" s="17" t="s">
@@ -20028,7 +20033,7 @@
         <v>61</v>
       </c>
       <c r="H705" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I705" s="18"/>
       <c r="J705" s="17" t="s">
@@ -20050,7 +20055,7 @@
         <v>62</v>
       </c>
       <c r="H706" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I706" s="18"/>
       <c r="J706" s="17" t="s">
@@ -20072,7 +20077,7 @@
         <v>63</v>
       </c>
       <c r="H707" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I707" s="18"/>
       <c r="J707" s="17" t="s">
@@ -20094,7 +20099,7 @@
         <v>64</v>
       </c>
       <c r="H708" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I708" s="18"/>
       <c r="J708" s="17" t="s">
@@ -20116,7 +20121,7 @@
         <v>65</v>
       </c>
       <c r="H709" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I709" s="18"/>
       <c r="J709" s="17" t="s">
@@ -20261,22 +20266,22 @@
     </row>
     <row r="716" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A716" s="44" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="B716" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C716" s="27" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="D716" s="28" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="E716" s="28" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="F716" s="28" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="G716" s="16" t="s">
         <v>58</v>
@@ -20405,22 +20410,22 @@
     </row>
     <row r="722" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A722" s="44" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="B722" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C722" s="14" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="D722" s="15" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="E722" s="15" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="F722" s="15" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="G722" s="16" t="s">
         <v>58</v>
@@ -20549,22 +20554,22 @@
     </row>
     <row r="728" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A728" s="44" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="B728" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C728" s="27" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="D728" s="28" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="E728" s="28" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="F728" s="28" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="G728" s="16" t="s">
         <v>58</v>
@@ -20693,22 +20698,22 @@
     </row>
     <row r="734" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A734" s="45" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="B734" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C734" s="14" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="D734" s="15" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="E734" s="15" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="F734" s="15" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="G734" s="16" t="s">
         <v>58</v>
@@ -20837,22 +20842,22 @@
     </row>
     <row r="740" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A740" s="45" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="B740" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C740" s="27" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="D740" s="28" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="E740" s="28" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="F740" s="28" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="G740" s="16" t="s">
         <v>58</v>
@@ -20981,22 +20986,22 @@
     </row>
     <row r="746" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A746" s="45" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="B746" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C746" s="14" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="D746" s="15" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="E746" s="15" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="F746" s="15" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="G746" s="16" t="s">
         <v>58</v>
@@ -21125,22 +21130,22 @@
     </row>
     <row r="752" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A752" s="45" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="B752" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C752" s="27" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="D752" s="28" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="E752" s="28" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="F752" s="28" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="G752" s="16" t="s">
         <v>58</v>
@@ -21269,22 +21274,22 @@
     </row>
     <row r="758" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A758" s="45" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="B758" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C758" s="14" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="D758" s="15" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="E758" s="15" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="F758" s="15" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="G758" s="16" t="s">
         <v>58</v>
@@ -21413,22 +21418,22 @@
     </row>
     <row r="764" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A764" s="46" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B764" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C764" s="27" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="D764" s="28" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="E764" s="28" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="F764" s="28" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="G764" s="16" t="s">
         <v>58</v>
@@ -21557,22 +21562,22 @@
     </row>
     <row r="770" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A770" s="46" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B770" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C770" s="14" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="D770" s="15" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="E770" s="15" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="F770" s="15" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="G770" s="16" t="s">
         <v>58</v>
@@ -21701,22 +21706,22 @@
     </row>
     <row r="776" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A776" s="46" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B776" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C776" s="27" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="D776" s="28" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="E776" s="28" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="F776" s="28" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="G776" s="16" t="s">
         <v>58</v>
@@ -21845,22 +21850,22 @@
     </row>
     <row r="782" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A782" s="46" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B782" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C782" s="14" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="D782" s="15" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="E782" s="15" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="F782" s="15" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="G782" s="16" t="s">
         <v>58</v>
@@ -21989,22 +21994,22 @@
     </row>
     <row r="788" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A788" s="46" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B788" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C788" s="27" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="D788" s="28" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="E788" s="28" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="F788" s="28" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="G788" s="16" t="s">
         <v>58</v>
@@ -22133,28 +22138,28 @@
     </row>
     <row r="794" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A794" s="46" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B794" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C794" s="14" t="s">
+        <v>526</v>
+      </c>
+      <c r="D794" s="15" t="s">
+        <v>527</v>
+      </c>
+      <c r="E794" s="15" t="s">
+        <v>528</v>
+      </c>
+      <c r="F794" s="15" t="s">
         <v>525</v>
-      </c>
-      <c r="D794" s="15" t="s">
-        <v>526</v>
-      </c>
-      <c r="E794" s="15" t="s">
-        <v>527</v>
-      </c>
-      <c r="F794" s="15" t="s">
-        <v>524</v>
       </c>
       <c r="G794" s="16" t="s">
         <v>58</v>
       </c>
       <c r="H794" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I794" s="18"/>
       <c r="J794" s="17" t="s">
@@ -22176,7 +22181,7 @@
         <v>61</v>
       </c>
       <c r="H795" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I795" s="18"/>
       <c r="J795" s="17" t="s">
@@ -22198,7 +22203,7 @@
         <v>62</v>
       </c>
       <c r="H796" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I796" s="18"/>
       <c r="J796" s="17" t="s">
@@ -22220,7 +22225,7 @@
         <v>63</v>
       </c>
       <c r="H797" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I797" s="18"/>
       <c r="J797" s="17" t="s">
@@ -22242,7 +22247,7 @@
         <v>64</v>
       </c>
       <c r="H798" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I798" s="18"/>
       <c r="J798" s="17" t="s">
@@ -22264,7 +22269,7 @@
         <v>65</v>
       </c>
       <c r="H799" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I799" s="18"/>
       <c r="J799" s="17" t="s">
@@ -22277,22 +22282,22 @@
     </row>
     <row r="800" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A800" s="46" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B800" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C800" s="27" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="D800" s="28" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="E800" s="28" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="F800" s="28" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="G800" s="16" t="s">
         <v>58</v>
@@ -22421,22 +22426,22 @@
     </row>
     <row r="806" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A806" s="46" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B806" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C806" s="14" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="D806" s="15" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="E806" s="15" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="F806" s="15" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="G806" s="16" t="s">
         <v>58</v>
@@ -22565,22 +22570,22 @@
     </row>
     <row r="812" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A812" s="46" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B812" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C812" s="27" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="D812" s="28" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="E812" s="28" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="F812" s="28" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="G812" s="16" t="s">
         <v>58</v>
@@ -22709,22 +22714,22 @@
     </row>
     <row r="818" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A818" s="46" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B818" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C818" s="14" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="D818" s="15" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="E818" s="15" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="F818" s="15" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="G818" s="16" t="s">
         <v>58</v>
@@ -22853,22 +22858,22 @@
     </row>
     <row r="824" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A824" s="46" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B824" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C824" s="27" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="D824" s="28" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="E824" s="28" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="F824" s="28" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="G824" s="16" t="s">
         <v>58</v>
@@ -22997,28 +23002,28 @@
     </row>
     <row r="830" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A830" s="46" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B830" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C830" s="14" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="D830" s="15" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="E830" s="15" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="F830" s="15" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="G830" s="16" t="s">
         <v>58</v>
       </c>
       <c r="H830" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I830" s="18"/>
       <c r="J830" s="17" t="s">
@@ -23040,7 +23045,7 @@
         <v>61</v>
       </c>
       <c r="H831" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I831" s="18"/>
       <c r="J831" s="17" t="s">
@@ -23062,7 +23067,7 @@
         <v>62</v>
       </c>
       <c r="H832" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I832" s="18"/>
       <c r="J832" s="17" t="s">
@@ -23084,7 +23089,7 @@
         <v>63</v>
       </c>
       <c r="H833" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I833" s="18"/>
       <c r="J833" s="17" t="s">
@@ -23106,7 +23111,7 @@
         <v>64</v>
       </c>
       <c r="H834" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I834" s="18"/>
       <c r="J834" s="17" t="s">
@@ -23128,7 +23133,7 @@
         <v>65</v>
       </c>
       <c r="H835" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I835" s="18"/>
       <c r="J835" s="17" t="s">
@@ -23141,22 +23146,22 @@
     </row>
     <row r="836" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A836" s="47" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="B836" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C836" s="27" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="D836" s="28" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="E836" s="28" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="F836" s="28" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="G836" s="16" t="s">
         <v>58</v>
@@ -23285,22 +23290,22 @@
     </row>
     <row r="842" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A842" s="47" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="B842" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C842" s="14" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="D842" s="15" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="E842" s="15" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="F842" s="15" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="G842" s="16" t="s">
         <v>58</v>
@@ -23429,28 +23434,28 @@
     </row>
     <row r="848" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A848" s="47" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="B848" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C848" s="27" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="D848" s="28" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="E848" s="28" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="F848" s="28" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="G848" s="16" t="s">
         <v>58</v>
       </c>
       <c r="H848" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I848" s="18"/>
       <c r="J848" s="17" t="s">
@@ -23472,7 +23477,7 @@
         <v>61</v>
       </c>
       <c r="H849" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I849" s="18"/>
       <c r="J849" s="17" t="s">
@@ -23494,7 +23499,7 @@
         <v>62</v>
       </c>
       <c r="H850" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I850" s="18"/>
       <c r="J850" s="17" t="s">
@@ -23516,7 +23521,7 @@
         <v>63</v>
       </c>
       <c r="H851" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I851" s="18"/>
       <c r="J851" s="17" t="s">
@@ -23538,7 +23543,7 @@
         <v>64</v>
       </c>
       <c r="H852" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I852" s="18"/>
       <c r="J852" s="17" t="s">
@@ -23560,7 +23565,7 @@
         <v>65</v>
       </c>
       <c r="H853" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I853" s="18"/>
       <c r="J853" s="17" t="s">
@@ -23573,22 +23578,22 @@
     </row>
     <row r="854" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A854" s="47" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="B854" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C854" s="14" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="D854" s="15" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="E854" s="15" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="F854" s="15" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="G854" s="16" t="s">
         <v>58</v>
@@ -23717,22 +23722,22 @@
     </row>
     <row r="860" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A860" s="48" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="B860" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C860" s="27" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="D860" s="28" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="E860" s="28" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="F860" s="28" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="G860" s="16" t="s">
         <v>58</v>
@@ -23861,22 +23866,22 @@
     </row>
     <row r="866" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A866" s="48" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="B866" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C866" s="14" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="D866" s="15" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="E866" s="15" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="F866" s="15" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="G866" s="16" t="s">
         <v>58</v>
@@ -24005,22 +24010,22 @@
     </row>
     <row r="872" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A872" s="48" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="B872" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C872" s="27" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="D872" s="28" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="E872" s="28" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="F872" s="28" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="G872" s="16" t="s">
         <v>58</v>
@@ -24149,22 +24154,22 @@
     </row>
     <row r="878" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A878" s="48" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="B878" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C878" s="14" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="D878" s="15" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E878" s="15" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="F878" s="15" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="G878" s="16" t="s">
         <v>58</v>
@@ -24293,22 +24298,22 @@
     </row>
     <row r="884" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A884" s="48" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="B884" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C884" s="27" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="D884" s="28" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="E884" s="28" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="F884" s="28" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="G884" s="16" t="s">
         <v>58</v>
@@ -24437,22 +24442,22 @@
     </row>
     <row r="890" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A890" s="48" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="B890" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C890" s="14" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="D890" s="15" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="E890" s="15" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="F890" s="15" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="G890" s="16" t="s">
         <v>58</v>
@@ -24581,22 +24586,22 @@
     </row>
     <row r="896" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A896" s="48" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="B896" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C896" s="27" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="D896" s="28" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="E896" s="28" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="F896" s="28" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="G896" s="16" t="s">
         <v>58</v>
@@ -24725,22 +24730,22 @@
     </row>
     <row r="902" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A902" s="49" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="B902" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C902" s="14" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="D902" s="15" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="E902" s="15" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="F902" s="15" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="G902" s="16" t="s">
         <v>58</v>
@@ -24869,22 +24874,22 @@
     </row>
     <row r="908" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A908" s="49" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="B908" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C908" s="27" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="D908" s="28" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="E908" s="28" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="F908" s="28" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="G908" s="16" t="s">
         <v>58</v>
@@ -25013,22 +25018,22 @@
     </row>
     <row r="914" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A914" s="49" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="B914" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C914" s="14" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="D914" s="15" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="E914" s="15" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="F914" s="15" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="G914" s="16" t="s">
         <v>58</v>
@@ -25157,22 +25162,22 @@
     </row>
     <row r="920" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A920" s="49" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="B920" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C920" s="27" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="D920" s="28" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="E920" s="28" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="F920" s="28" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="G920" s="16" t="s">
         <v>58</v>
@@ -25301,22 +25306,22 @@
     </row>
     <row r="926" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A926" s="49" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="B926" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C926" s="14" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="D926" s="15" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="E926" s="15" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="F926" s="15" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="G926" s="16" t="s">
         <v>58</v>
@@ -25445,22 +25450,22 @@
     </row>
     <row r="932" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A932" s="49" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="B932" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C932" s="27" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="D932" s="28" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="E932" s="28" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="F932" s="28" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="G932" s="16" t="s">
         <v>58</v>
@@ -25589,22 +25594,22 @@
     </row>
     <row r="938" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A938" s="50" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="B938" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C938" s="14" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="D938" s="15" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="E938" s="15" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="F938" s="15" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="G938" s="16" t="s">
         <v>58</v>
@@ -25733,22 +25738,22 @@
     </row>
     <row r="944" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A944" s="50" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="B944" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C944" s="27" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="D944" s="28" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="E944" s="28" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="F944" s="28" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="G944" s="16" t="s">
         <v>58</v>
@@ -25877,22 +25882,22 @@
     </row>
     <row r="950" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A950" s="50" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="B950" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C950" s="14" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="D950" s="15" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="E950" s="15" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="F950" s="15" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="G950" s="16" t="s">
         <v>58</v>
@@ -26021,22 +26026,22 @@
     </row>
     <row r="956" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A956" s="50" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="B956" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C956" s="27" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="D956" s="28" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="E956" s="28" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="F956" s="28" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="G956" s="16" t="s">
         <v>58</v>
@@ -26165,22 +26170,22 @@
     </row>
     <row r="962" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A962" s="50" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="B962" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C962" s="14" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="D962" s="15" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="E962" s="15" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="F962" s="15" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="G962" s="16" t="s">
         <v>58</v>
@@ -26309,22 +26314,22 @@
     </row>
     <row r="968" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A968" s="50" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="B968" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C968" s="27" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="D968" s="28" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="E968" s="28" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="F968" s="28" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="G968" s="16" t="s">
         <v>58</v>
@@ -26453,22 +26458,22 @@
     </row>
     <row r="974" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A974" s="51" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="B974" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C974" s="14" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="D974" s="15" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="E974" s="15" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="F974" s="15" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="G974" s="16" t="s">
         <v>58</v>
@@ -26597,22 +26602,22 @@
     </row>
     <row r="980" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A980" s="51" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="B980" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C980" s="27" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="D980" s="28" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="E980" s="28" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="F980" s="28" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="G980" s="16" t="s">
         <v>58</v>
@@ -26741,22 +26746,22 @@
     </row>
     <row r="986" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A986" s="51" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="B986" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C986" s="14" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="D986" s="15" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="E986" s="15" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="F986" s="15" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="G986" s="16" t="s">
         <v>58</v>
@@ -26885,22 +26890,22 @@
     </row>
     <row r="992" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A992" s="51" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="B992" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C992" s="27" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="D992" s="28" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="E992" s="28" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="F992" s="28" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="G992" s="16" t="s">
         <v>58</v>
@@ -27029,22 +27034,22 @@
     </row>
     <row r="998" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A998" s="51" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="B998" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C998" s="14" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="D998" s="15" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="E998" s="15" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="F998" s="15" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="G998" s="16" t="s">
         <v>58</v>
@@ -27173,22 +27178,22 @@
     </row>
     <row r="1004" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1004" s="52" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="B1004" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1004" s="27" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="D1004" s="28" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="E1004" s="28" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="F1004" s="28" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="G1004" s="16" t="s">
         <v>58</v>
@@ -27317,22 +27322,22 @@
     </row>
     <row r="1010" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1010" s="52" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="B1010" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1010" s="14" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="D1010" s="15" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="E1010" s="15" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="F1010" s="15" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="G1010" s="16" t="s">
         <v>58</v>
@@ -27461,28 +27466,28 @@
     </row>
     <row r="1016" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1016" s="52" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="B1016" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1016" s="27" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="D1016" s="28" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="E1016" s="28" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="F1016" s="28" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="G1016" s="16" t="s">
         <v>58</v>
       </c>
       <c r="H1016" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I1016" s="18"/>
       <c r="J1016" s="17" t="s">
@@ -27504,7 +27509,7 @@
         <v>61</v>
       </c>
       <c r="H1017" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I1017" s="18"/>
       <c r="J1017" s="17" t="s">
@@ -27526,7 +27531,7 @@
         <v>62</v>
       </c>
       <c r="H1018" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I1018" s="18"/>
       <c r="J1018" s="17" t="s">
@@ -27548,7 +27553,7 @@
         <v>63</v>
       </c>
       <c r="H1019" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I1019" s="18"/>
       <c r="J1019" s="17" t="s">
@@ -27570,7 +27575,7 @@
         <v>64</v>
       </c>
       <c r="H1020" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I1020" s="18"/>
       <c r="J1020" s="17" t="s">
@@ -27592,7 +27597,7 @@
         <v>65</v>
       </c>
       <c r="H1021" s="34" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I1021" s="18"/>
       <c r="J1021" s="17" t="s">
@@ -27605,22 +27610,22 @@
     </row>
     <row r="1022" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1022" s="52" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="B1022" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1022" s="14" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="D1022" s="15" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="E1022" s="15" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="F1022" s="15" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="G1022" s="16" t="s">
         <v>58</v>
@@ -27749,22 +27754,22 @@
     </row>
     <row r="1028" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1028" s="52" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="B1028" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C1028" s="27" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="D1028" s="28" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="E1028" s="28" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="F1028" s="28" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="G1028" s="16" t="s">
         <v>58</v>
@@ -27893,22 +27898,22 @@
     </row>
     <row r="1034" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1034" s="52" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="B1034" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C1034" s="14" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="D1034" s="15" t="s">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="E1034" s="15" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="F1034" s="15" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="G1034" s="16" t="s">
         <v>58</v>
@@ -28037,22 +28042,22 @@
     </row>
     <row r="1040" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1040" s="53" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="B1040" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C1040" s="27" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="D1040" s="28" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="E1040" s="28" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="F1040" s="28" t="s">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="G1040" s="16" t="s">
         <v>58</v>
@@ -28181,22 +28186,22 @@
     </row>
     <row r="1046" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1046" s="53" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="B1046" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1046" s="14" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="D1046" s="15" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="E1046" s="15" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="F1046" s="15" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="G1046" s="16" t="s">
         <v>58</v>
@@ -28325,22 +28330,22 @@
     </row>
     <row r="1052" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1052" s="36" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B1052" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1052" s="27" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="D1052" s="28" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="E1052" s="28" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="F1052" s="28" t="s">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="G1052" s="16" t="s">
         <v>58</v>
@@ -28469,22 +28474,22 @@
     </row>
     <row r="1058" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1058" s="36" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B1058" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1058" s="14" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="D1058" s="15" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="E1058" s="15" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="F1058" s="15" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="G1058" s="16" t="s">
         <v>58</v>
@@ -29574,10 +29579,10 @@
         <v>39</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>53</v>
@@ -29595,7 +29600,7 @@
         <v>87</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -29687,7 +29692,7 @@
     </row>
     <row r="5" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="57" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B5" s="1">
         <v>5</v>
@@ -29716,7 +29721,7 @@
     </row>
     <row r="6" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="58" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B6" s="1">
         <v>8</v>
@@ -29745,7 +29750,7 @@
     </row>
     <row r="7" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="59" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B7" s="1">
         <v>17</v>
@@ -29774,7 +29779,7 @@
     </row>
     <row r="8" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="60" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B8" s="1">
         <v>10</v>
@@ -29803,7 +29808,7 @@
     </row>
     <row r="9" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="61" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B9" s="1">
         <v>11</v>
@@ -29832,7 +29837,7 @@
     </row>
     <row r="10" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="62" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B10" s="1">
         <v>9</v>
@@ -29861,7 +29866,7 @@
     </row>
     <row r="11" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="63" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="B11" s="1">
         <v>5</v>
@@ -29890,7 +29895,7 @@
     </row>
     <row r="12" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="64" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="B12" s="1">
         <v>5</v>
@@ -29919,7 +29924,7 @@
     </row>
     <row r="13" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="65" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="B13" s="1">
         <v>4</v>
@@ -29948,7 +29953,7 @@
     </row>
     <row r="14" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="66" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="B14" s="1">
         <v>5</v>
@@ -29977,7 +29982,7 @@
     </row>
     <row r="15" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="67" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B15" s="1">
         <v>12</v>
@@ -30006,7 +30011,7 @@
     </row>
     <row r="16" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="68" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="B16" s="1">
         <v>4</v>
@@ -30035,7 +30040,7 @@
     </row>
     <row r="17" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="69" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="B17" s="1">
         <v>7</v>
@@ -30064,7 +30069,7 @@
     </row>
     <row r="18" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="70" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="B18" s="1">
         <v>6</v>
@@ -30093,7 +30098,7 @@
     </row>
     <row r="19" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="71" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="B19" s="1">
         <v>6</v>
@@ -30122,7 +30127,7 @@
     </row>
     <row r="20" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="72" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="B20" s="1">
         <v>5</v>
@@ -30151,7 +30156,7 @@
     </row>
     <row r="21" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="73" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="B21" s="1">
         <v>6</v>
@@ -30180,7 +30185,7 @@
     </row>
     <row r="22" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="74" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="B22" s="1">
         <v>2</v>
@@ -30209,7 +30214,7 @@
     </row>
     <row r="23" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="75" t="s">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="B23" s="75">
         <v>153</v>
@@ -30260,7 +30265,7 @@
         <v>44</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="C1" s="10" t="s">
         <v>71</v>
@@ -30269,7 +30274,7 @@
         <v>87</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="F1" s="10" t="s">
         <v>95</v>
@@ -30420,10 +30425,10 @@
         <v>45</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>71</v>
@@ -30432,7 +30437,7 @@
         <v>87</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="G1" s="10" t="s">
         <v>95</v>
@@ -30443,7 +30448,7 @@
         <v>59</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="C2" s="1">
         <v>18</v>
@@ -30509,7 +30514,7 @@
     </row>
     <row r="5" ht="15" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="83" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>12</v>

</xml_diff>

<commit_message>
071 => fase IV => ZUP-024 ZUP-028 OK (Chrome/USER), fix doble línia menú Ajuda/Sortir i backups Excel
</commit_message>
<xml_diff>
--- a/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
+++ b/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4272" uniqueCount="714">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4274" uniqueCount="714">
   <si>
     <t>Zuppeto — Joc de probes manual (totes les pantalles)</t>
   </si>
@@ -7281,9 +7281,11 @@
       <c r="H164" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="I164" s="29"/>
+      <c r="I164" s="29" t="s">
+        <v>178</v>
+      </c>
       <c r="J164" s="17" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K164" s="15"/>
       <c r="L164" s="1"/>
@@ -8121,9 +8123,11 @@
       <c r="H200" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="I200" s="29"/>
+      <c r="I200" s="29" t="s">
+        <v>178</v>
+      </c>
       <c r="J200" s="17" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K200" s="15"/>
       <c r="L200" s="1"/>

</xml_diff>

<commit_message>
072 => fase IV => Excel proves sense argot (generador+MAIN), criteri backup només estructura/demanda i nota millores pendents
</commit_message>
<xml_diff>
--- a/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
+++ b/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4274" uniqueCount="714">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4274" uniqueCount="713">
   <si>
     <t>Zuppeto — Joc de probes manual (totes les pantalles)</t>
   </si>
@@ -29,13 +29,13 @@
     <t>Entorn</t>
   </si>
   <si>
-    <t>http://localhost:4200 (web) · http://localhost:5211/swagger (API)</t>
+    <t>http://localhost:4200 (web) · http://localhost:5211/swagger (servidor)</t>
   </si>
   <si>
     <t>Ordre recomanat</t>
   </si>
   <si>
-    <t>Login → Auth → Capçalera → Rols UX → Inici → Llocs → Detall → Favorits → Perfil → Notificacions → Ajuda → Contacte → Admin (Rols→Usuaris→Permisos→Menús→Països→Ciutats→Llocs→Docs) → API</t>
+    <t>Login → Auth → Capçalera → Rols UX → Inici → Llocs → Detall → Favorits → Perfil → Notificacions → Ajuda → Contacte → Admin (Rols→Usuaris→Permisos→Menús→Països→Ciutats→Llocs→Docs) → servidor</t>
   </si>
   <si>
     <t>Codi prova</t>
@@ -101,7 +101,7 @@
     <t>Pantalles cobertes</t>
   </si>
   <si>
-    <t>Capçalera / Navegació · Login (/login) · Auth callback (/auth/callback) · Inici (/) · Llocs (/places) · Detall lloc (/places/:id) · Favorits (/favorites) · Perfil (/perfil) · Notificacions (/notificacions) · Contacte (/contacte) · Ajuda (/ajuda) · Permisos stub (/permissions) · Admin · Documentació (/admin/documentacio) · Admin · Usuaris (/admin/usuaris) · Admin · Permisos (/admin/permisos) · Admin · Menús (/admin/menus) · Admin · Rols (/admin/rols) · Admin · Països (/admin/paisos) · Admin · Ciutats (/admin/ciutats) · Admin · Llocs (/admin/llocs) · Rols i seguretat</t>
+    <t>Capçalera / Navegació · Login (/login) · Retorn del login (/auth/callback) · Inici (/) · Llocs (/places) · Detall lloc (/places/:id) · Favorits (/favorites) · Perfil (/perfil) · Notificacions (/notificacions) · Contacte (/contacte) · Ajuda (/ajuda) · Permisos stub (/permissions) · Admin · Documentació (/admin/documentacio) · Admin · Usuaris (/admin/usuaris) · Admin · Permisos (/admin/permisos) · Admin · Menús (/admin/menus) · Admin · Rols (/admin/rols) · Admin · Països (/admin/paisos) · Admin · Ciutats (/admin/ciutats) · Admin · Llocs (/admin/llocs) · Rols i seguretat</t>
   </si>
   <si>
     <t>Proves lògiques: 153 · Files totals: 1062 · Codis: ZUP-001–ZUP-153</t>
@@ -323,7 +323,7 @@
     <t>Clic LinkedIn si disponible</t>
   </si>
   <si>
-    <t>Redirecció OAuth o botó desactivat si pendent</t>
+    <t>Redirecció al proveïdor de login o botó desactivat si pendent</t>
   </si>
   <si>
     <t>Baixa</t>
@@ -356,7 +356,7 @@
     <t>05-08-2026</t>
   </si>
   <si>
-    <t>Prova conjunta amb ZUP-010 i ZUP-011. Explorador: filtres/cerca sense feedback útil (mosaic/API).</t>
+    <t>Prova conjunta amb ZUP-010 i ZUP-011. Explorador: filtres/cerca sense feedback útil (mosaic/servidor).</t>
   </si>
   <si>
     <t xml:space="preserve">Catàleg real + cerca ≥2.
@@ -372,7 +372,7 @@
     <t>Revisar bloc «Mapa inicial»</t>
   </si>
   <si>
-    <t>Mapa Leaflet centrat a Espanya sense dades carregades</t>
+    <t>Mapa centrat a Espanya sense dades carregades</t>
   </si>
   <si>
     <t>Prova conjunta amb ZUP-009 i ZUP-011. Mapa sense zoom/pan ni marcadors.</t>
@@ -391,7 +391,7 @@
     <t>Clic «Obrir cerca» amb filtres aplicats</t>
   </si>
   <si>
-    <t>Navega cap al flux de places (guest/login segons estat)</t>
+    <t>Navega cap al cerca de llocs (amb o sense sessió, segons l'estat)</t>
   </si>
   <si>
     <t>Prova conjunta amb ZUP-009 i ZUP-010. «Obrir cerca» lligat al mateix explorador.</t>
@@ -409,7 +409,7 @@
     <t>Clic «Generar rutes»</t>
   </si>
   <si>
-    <t>Acció de preview sense trencar la UI</t>
+    <t>Acció de preview sense trencar la pantalla</t>
   </si>
   <si>
     <t>ZUP-013</t>
@@ -427,7 +427,7 @@
     <t>ZUP-014</t>
   </si>
   <si>
-    <t>Guest guard: usuari logat no veu login</t>
+    <t>Control d'accés: usuari logat no veu login</t>
   </si>
   <si>
     <t>Amb sessió activa anar a /login</t>
@@ -436,13 +436,13 @@
     <t>Redirecció fora del login (p.ex. home)</t>
   </si>
   <si>
-    <t>Auth callback (/auth/callback)</t>
+    <t>Retorn del login (/auth/callback)</t>
   </si>
   <si>
     <t>ZUP-015</t>
   </si>
   <si>
-    <t>Callback OAuth sense paràmetres</t>
+    <t>Retorn del login sense dades del proveïdor</t>
   </si>
   <si>
     <t>Anar a /auth/callback directament</t>
@@ -454,10 +454,10 @@
     <t>ZUP-016</t>
   </si>
   <si>
-    <t>Callback OAuth Google/LinkedIn (flux complet)</t>
-  </si>
-  <si>
-    <t>Completar login federat des del proveïdor</t>
+    <t>Retorn del login amb Google o LinkedIn (flux complet)</t>
+  </si>
+  <si>
+    <t>Completar el login amb Google o LinkedIn</t>
   </si>
   <si>
     <t>Sessió creada i redirecció al producte</t>
@@ -496,7 +496,7 @@
     <t>ZUP-019</t>
   </si>
   <si>
-    <t>Dropdown de compte (rodona)</t>
+    <t>Menú del compte (rodona)</t>
   </si>
   <si>
     <t>Clic a la rodona del compte</t>
@@ -535,13 +535,13 @@
     <t>Campana de notificacions</t>
   </si>
   <si>
-    <t>Revisar icona campana al header amb notificacions pendents</t>
+    <t>Revisar icona campana a la capçalera amb notificacions pendents</t>
   </si>
   <si>
     <t>Indicador de no llegides i enllaç a /notificacions</t>
   </si>
   <si>
-    <t>Al generar notificació desant el perfil: camps obligatoris sense marquejar; toast d’èxit sortia en vermell (to error per defecte).</t>
+    <t>Al generar notificació desant el perfil: camps obligatoris sense marquejar; missatge emergent d’èxit sortia en vermell (to error per defecte).</t>
   </si>
   <si>
     <t xml:space="preserve">Asterisc (*) en camps obligatoris.
@@ -569,13 +569,13 @@
     <t>ZUP-024</t>
   </si>
   <si>
-    <t>Peu de pàgina (footer)</t>
+    <t>Peu de pàgina</t>
   </si>
   <si>
     <t>Desplaçar-se al final de Home, Llocs i Ajuda</t>
   </si>
   <si>
-    <t>Footer visible amb enllaços/coherència visual</t>
+    <t>Peu de pàgina visible amb enllaços/coherència visual</t>
   </si>
   <si>
     <t>ZUP-025</t>
@@ -584,7 +584,7 @@
     <t>Refresc després de canvis de permisos</t>
   </si>
   <si>
-    <t>Canviar permisos/menús com ADMIN → Ctrl+Shift+R</t>
+    <t>Canviar permisos/menús com ADMIN → recarregar la pàgina amb força (recarregar la pàgina amb força (recarregar la pàgina amb força (recarregar la pàgina amb força (recarregar la pàgina amb força (recarregar la pàgina amb força (Ctrl+Shift+R))))))</t>
   </si>
   <si>
     <t>Capçalera es reconstrueix correctament</t>
@@ -611,7 +611,7 @@
     <t>Login DEVELOPER — menú</t>
   </si>
   <si>
-    <t>Login DEVELOPER → revisar header</t>
+    <t>Login DEVELOPER → revisar la capçalera</t>
   </si>
   <si>
     <t>Del desenvolupador (documentació); no Del administrador complet</t>
@@ -623,7 +623,7 @@
     <t>Login USER — sense admin</t>
   </si>
   <si>
-    <t>Login USER → revisar header</t>
+    <t>Login USER → revisar la capçalera</t>
   </si>
   <si>
     <t>Cap opció admin ni documentació interna</t>
@@ -647,31 +647,31 @@
     <t>ZUP-030</t>
   </si>
   <si>
-    <t>Hero principal</t>
+    <t>Franja principal de la portada</t>
   </si>
   <si>
     <t>Anar a / autenticat</t>
   </si>
   <si>
-    <t>Títol hero, chips pet-friendly i CTAs «Explora llocs» / «Entén el flux»</t>
+    <t>Títol de la portada, etiquetes pet-friendly i botons «Explora llocs» / «Entén el flux»</t>
   </si>
   <si>
     <t>ZUP-031</t>
   </si>
   <si>
-    <t>Chips del hero cap a places filtrats</t>
-  </si>
-  <si>
-    <t>Clic a un chip del hero</t>
-  </si>
-  <si>
-    <t>Obre /places amb query params de filtre</t>
+    <t>Etiquetes de la franja principal cap a places filtrats</t>
+  </si>
+  <si>
+    <t>Clic a una etiqueta de la franja principal</t>
+  </si>
+  <si>
+    <t>Obre /places amb filtres aplicats a l'adreça de la pàgina</t>
   </si>
   <si>
     <t>ZUP-032</t>
   </si>
   <si>
-    <t>CTA «Anar a llocs»</t>
+    <t>Botó «Anar a llocs»</t>
   </si>
   <si>
     <t>Clic al botó primari del tancament</t>
@@ -683,7 +683,7 @@
     <t>ZUP-033</t>
   </si>
   <si>
-    <t>CTA «Revisar favorits»</t>
+    <t>Botó «Revisar favorits»</t>
   </si>
   <si>
     <t>Clic al botó secundari del tancament</t>
@@ -695,13 +695,13 @@
     <t>ZUP-034</t>
   </si>
   <si>
-    <t>Top favorits al hero</t>
-  </si>
-  <si>
-    <t>Amb favorits existents revisar hero</t>
-  </si>
-  <si>
-    <t>Fins a 10 llocs favorits destacats al hero</t>
+    <t>Favorits destacats a la franja principal</t>
+  </si>
+  <si>
+    <t>Amb favorits existents revisar la franja principal</t>
+  </si>
+  <si>
+    <t>Fins a 10 llocs favorits destacats a la franja principal</t>
   </si>
   <si>
     <t>ZUP-035</t>
@@ -722,7 +722,7 @@
     <t>Secció «Com es fa servir» (3 passos)</t>
   </si>
   <si>
-    <t>Revisar journey cards 01-03</t>
+    <t>Revisar targetes del recorregut 01-03</t>
   </si>
   <si>
     <t>Textos Filtra / Valida al mapa / Guarda i reprèn visibles</t>
@@ -764,16 +764,16 @@
     <t>Escriure terme al camp cerca</t>
   </si>
   <si>
-    <t>Filtre aplicat; chips de filtres actius actualitzats</t>
+    <t>Filtre aplicat; etiquetes de filtres actius actualitzats</t>
   </si>
   <si>
     <t>ZUP-040</t>
   </si>
   <si>
-    <t>Filtres: ciutat (combobox)</t>
-  </si>
-  <si>
-    <t>Seleccionar ciutat al combobox</t>
+    <t>Filtres: ciutat (llista desplegable)</t>
+  </si>
+  <si>
+    <t>Seleccionar ciutat a la llista desplegable</t>
   </si>
   <si>
     <t>Llista i mapa es filtren per ciutat</t>
@@ -806,13 +806,13 @@
     <t>ZUP-043</t>
   </si>
   <si>
-    <t>Obrir cerca (lazy load)</t>
+    <t>Obrir cerca (càrrega sota demanda)</t>
   </si>
   <si>
     <t>Configurar filtres → «Obrir cerca»</t>
   </si>
   <si>
-    <t>Es carreguen resultats des de l'API amb caché</t>
+    <t>Es carreguen resultats des del servidor (amb memòria de cerca)</t>
   </si>
   <si>
     <t>ZUP-044</t>
@@ -848,7 +848,7 @@
     <t>Revisar llistat sota el mapa</t>
   </si>
   <si>
-    <t>Place cards amb imatge, tipus, favorit</t>
+    <t>Targetes de lloc amb imatge, tipus, favorit</t>
   </si>
   <si>
     <t>ZUP-047</t>
@@ -893,7 +893,7 @@
     <t>Després d'una cerca amb resultats</t>
   </si>
   <si>
-    <t>Marcadors al mapa Leaflet</t>
+    <t>Marcadors al Mapa</t>
   </si>
   <si>
     <t>ZUP-051</t>
@@ -1004,7 +1004,7 @@
     <t>Revisar mapa centrat al lloc</t>
   </si>
   <si>
-    <t>Marcador únic amb coordenades del backend</t>
+    <t>Marcador únic amb coordenades del lloc</t>
   </si>
   <si>
     <t>ZUP-060</t>
@@ -1040,7 +1040,7 @@
     <t>Entrar al detall des del mapa de places</t>
   </si>
   <si>
-    <t>Badge/indicador visible si escau</t>
+    <t>Indicador visible si escau</t>
   </si>
   <si>
     <t>ZUP-063</t>
@@ -1079,7 +1079,7 @@
     <t>USER sense favorits → /favorites</t>
   </si>
   <si>
-    <t>Empty state «Encara no tens favorits» + enllaç Explorar</t>
+    <t>Pantalla buida «Encara no tens favorits» + enllaç Explorar</t>
   </si>
   <si>
     <t>ZUP-066</t>
@@ -1109,7 +1109,7 @@
     <t>ZUP-068</t>
   </si>
   <si>
-    <t>Spotlight últim guardat</t>
+    <t>Destacat de l'últim guardat</t>
   </si>
   <si>
     <t>Amb diversos favorits</t>
@@ -1235,7 +1235,7 @@
     <t>Canviar nom → Guardar canvis</t>
   </si>
   <si>
-    <t>Canvi persistit; visible al header/compte</t>
+    <t>Canvi persistit; visible a la capçalera i al menú del compte</t>
   </si>
   <si>
     <t>ZUP-079</t>
@@ -1256,7 +1256,7 @@
     <t>Avatar drag &amp; drop</t>
   </si>
   <si>
-    <t>Arrossegar imatge a la dropzone</t>
+    <t>Arrossegar imatge a la zona per deixar el fitxer</t>
   </si>
   <si>
     <t>Avatar actualitzat</t>
@@ -1322,7 +1322,7 @@
     <t>Usuari sense notificacions</t>
   </si>
   <si>
-    <t>Empty state «No hi ha notificacions»</t>
+    <t>Pantalla buida «No hi ha notificacions»</t>
   </si>
   <si>
     <t>ZUP-086</t>
@@ -1397,7 +1397,7 @@
     <t>Revisar secció Flux</t>
   </si>
   <si>
-    <t>Tres info cards explicatives</t>
+    <t>Tres Targetes informatives explicatives</t>
   </si>
   <si>
     <t>ZUP-092</t>
@@ -1415,10 +1415,10 @@
     <t>ZUP-093</t>
   </si>
   <si>
-    <t>CTAs cap a places i favorits</t>
-  </si>
-  <si>
-    <t>Provar enllaços del hero</t>
+    <t>Botons cap a llocs i favorits</t>
+  </si>
+  <si>
+    <t>Provar enllaços de la franja principal</t>
   </si>
   <si>
     <t>ZUP-094</t>
@@ -1445,7 +1445,7 @@
     <t>Anar a /contacte</t>
   </si>
   <si>
-    <t>Heading contacte, chips i canal suport@zuppeto.fake</t>
+    <t>Heading contacte, etiquetes i canal suport@zuppeto.fake</t>
   </si>
   <si>
     <t>ZUP-096</t>
@@ -1457,13 +1457,13 @@
     <t>Revisar graella Partnerships / Feedback / Ciutats</t>
   </si>
   <si>
-    <t>Info cards amb text coherent</t>
+    <t>Targetes informatives amb text coherent</t>
   </si>
   <si>
     <t>ZUP-097</t>
   </si>
   <si>
-    <t>CTA Veure com funciona</t>
+    <t>Botó «Veure com funciona»</t>
   </si>
   <si>
     <t>Clic enllaç</t>
@@ -1475,9 +1475,6 @@
     <t>ZUP-098</t>
   </si>
   <si>
-    <t>CTA Anar a llocs</t>
-  </si>
-  <si>
     <t>Admin · Rols (/admin/rols)</t>
   </si>
   <si>
@@ -1571,7 +1568,7 @@
     <t>ZUP-106</t>
   </si>
   <si>
-    <t>Modal crear usuari — validació</t>
+    <t>finestra crear usuari — validació</t>
   </si>
   <si>
     <t>Obrir Crear usuari amb camps buits</t>
@@ -1634,7 +1631,7 @@
     <t>Clic fila o icona ull</t>
   </si>
   <si>
-    <t>Panell/modal detall amb dades editables</t>
+    <t>Panell o finestra de detall amb dades editables</t>
   </si>
   <si>
     <t>ZUP-112</t>
@@ -1715,7 +1712,7 @@
     <t>Editar permisos DEVELOPER</t>
   </si>
   <si>
-    <t>Donar/treure page.admin.documentation</t>
+    <t>Donar/treure accés a documentació interna</t>
   </si>
   <si>
     <t>Canvi reflectit en accés real</t>
@@ -1730,7 +1727,7 @@
     <t>Desar canvis que afecten menú</t>
   </si>
   <si>
-    <t>Header es refresca sense relogin</t>
+    <t>La capçalera es refresca sense tornar a iniciar sessió</t>
   </si>
   <si>
     <t>Admin · Menús (/admin/menus)</t>
@@ -1754,7 +1751,7 @@
     <t>Crear menú sota Ajuda</t>
   </si>
   <si>
-    <t>Nou menú parentKey help</t>
+    <t>Nou menú dins d'Ajuda</t>
   </si>
   <si>
     <t>Apareix dins submenú Ajuda</t>
@@ -1766,7 +1763,7 @@
     <t>Crear menú sota admin</t>
   </si>
   <si>
-    <t>Nou menú parentKey admin</t>
+    <t>Nou menú dins d'administració</t>
   </si>
   <si>
     <t>Apareix a Del administrador</t>
@@ -1781,7 +1778,7 @@
     <t>Editar label i desar</t>
   </si>
   <si>
-    <t>Text actualitzat al header</t>
+    <t>Text actualitzat a la capçalera</t>
   </si>
   <si>
     <t>ZUP-124</t>
@@ -1790,10 +1787,10 @@
     <t>Desactivar menú</t>
   </si>
   <si>
-    <t>isActive false → desar</t>
-  </si>
-  <si>
-    <t>Opció desapareix del header</t>
+    <t>marcar com a inactiu → desar</t>
+  </si>
+  <si>
+    <t>Opció desapareix de la capçalera</t>
   </si>
   <si>
     <t>ZUP-125</t>
@@ -1811,7 +1808,7 @@
     <t>ZUP-126</t>
   </si>
   <si>
-    <t>Refresc automàtic header</t>
+    <t>Refresc automàtic capçalera</t>
   </si>
   <si>
     <t>Desar canvis a Menús</t>
@@ -1868,7 +1865,7 @@
     <t>Marcar inactiu</t>
   </si>
   <si>
-    <t>Estat actualitzat; coherent amb comboboxs</t>
+    <t>Estat actualitzat; coherent amb les llistes desplegables</t>
   </si>
   <si>
     <t>ZUP-131</t>
@@ -1958,10 +1955,10 @@
     <t>ZUP-138</t>
   </si>
   <si>
-    <t>Ciutat al combobox de places</t>
-  </si>
-  <si>
-    <t>Ciutat creada → provar combobox a /places</t>
+    <t>Ciutat a la llista desplegable de llocs</t>
+  </si>
+  <si>
+    <t>Ciutat creada → provar la llista de ciutats a /places</t>
   </si>
   <si>
     <t>Ciutat disponible a la cerca</t>
@@ -2129,10 +2126,10 @@
     <t>ZUP-152</t>
   </si>
   <si>
-    <t>API admin com USER → 403</t>
-  </si>
-  <si>
-    <t>Cridar /api/admin/* amb token USER</t>
+    <t>servidor admin com USER → 403</t>
+  </si>
+  <si>
+    <t>Cridar /servidor/admin/* amb token USER</t>
   </si>
   <si>
     <t>403 Forbidden</t>
@@ -2141,10 +2138,10 @@
     <t>ZUP-153</t>
   </si>
   <si>
-    <t>API navigation menu ADMIN</t>
-  </si>
-  <si>
-    <t>GET /api/navigation/menu com ADMIN</t>
+    <t>servidor navigation menu ADMIN</t>
+  </si>
+  <si>
+    <t>GET /servidor/navigation/menu com ADMIN</t>
   </si>
   <si>
     <t>200 amb home, places, favorites, help, admin</t>
@@ -20567,7 +20564,7 @@
         <v>482</v>
       </c>
       <c r="D728" s="28" t="s">
-        <v>483</v>
+        <v>215</v>
       </c>
       <c r="E728" s="28" t="s">
         <v>480</v>
@@ -20702,22 +20699,22 @@
     </row>
     <row r="734" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A734" s="45" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="B734" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C734" s="14" t="s">
+        <v>484</v>
+      </c>
+      <c r="D734" s="15" t="s">
         <v>485</v>
       </c>
-      <c r="D734" s="15" t="s">
+      <c r="E734" s="15" t="s">
         <v>486</v>
       </c>
-      <c r="E734" s="15" t="s">
+      <c r="F734" s="15" t="s">
         <v>487</v>
-      </c>
-      <c r="F734" s="15" t="s">
-        <v>488</v>
       </c>
       <c r="G734" s="16" t="s">
         <v>58</v>
@@ -20846,22 +20843,22 @@
     </row>
     <row r="740" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A740" s="45" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="B740" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C740" s="27" t="s">
+        <v>488</v>
+      </c>
+      <c r="D740" s="28" t="s">
         <v>489</v>
       </c>
-      <c r="D740" s="28" t="s">
+      <c r="E740" s="28" t="s">
         <v>490</v>
       </c>
-      <c r="E740" s="28" t="s">
+      <c r="F740" s="28" t="s">
         <v>491</v>
-      </c>
-      <c r="F740" s="28" t="s">
-        <v>492</v>
       </c>
       <c r="G740" s="16" t="s">
         <v>58</v>
@@ -20990,22 +20987,22 @@
     </row>
     <row r="746" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A746" s="45" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="B746" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C746" s="14" t="s">
+        <v>492</v>
+      </c>
+      <c r="D746" s="15" t="s">
         <v>493</v>
       </c>
-      <c r="D746" s="15" t="s">
+      <c r="E746" s="15" t="s">
         <v>494</v>
       </c>
-      <c r="E746" s="15" t="s">
+      <c r="F746" s="15" t="s">
         <v>495</v>
-      </c>
-      <c r="F746" s="15" t="s">
-        <v>496</v>
       </c>
       <c r="G746" s="16" t="s">
         <v>58</v>
@@ -21134,22 +21131,22 @@
     </row>
     <row r="752" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A752" s="45" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="B752" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C752" s="27" t="s">
+        <v>496</v>
+      </c>
+      <c r="D752" s="28" t="s">
         <v>497</v>
       </c>
-      <c r="D752" s="28" t="s">
+      <c r="E752" s="28" t="s">
         <v>498</v>
       </c>
-      <c r="E752" s="28" t="s">
+      <c r="F752" s="28" t="s">
         <v>499</v>
-      </c>
-      <c r="F752" s="28" t="s">
-        <v>500</v>
       </c>
       <c r="G752" s="16" t="s">
         <v>58</v>
@@ -21278,22 +21275,22 @@
     </row>
     <row r="758" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A758" s="45" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="B758" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C758" s="14" t="s">
+        <v>500</v>
+      </c>
+      <c r="D758" s="15" t="s">
         <v>501</v>
       </c>
-      <c r="D758" s="15" t="s">
+      <c r="E758" s="15" t="s">
         <v>502</v>
       </c>
-      <c r="E758" s="15" t="s">
+      <c r="F758" s="15" t="s">
         <v>503</v>
-      </c>
-      <c r="F758" s="15" t="s">
-        <v>504</v>
       </c>
       <c r="G758" s="16" t="s">
         <v>58</v>
@@ -21422,22 +21419,22 @@
     </row>
     <row r="764" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A764" s="46" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="B764" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C764" s="27" t="s">
+        <v>505</v>
+      </c>
+      <c r="D764" s="28" t="s">
         <v>506</v>
       </c>
-      <c r="D764" s="28" t="s">
+      <c r="E764" s="28" t="s">
         <v>507</v>
       </c>
-      <c r="E764" s="28" t="s">
+      <c r="F764" s="28" t="s">
         <v>508</v>
-      </c>
-      <c r="F764" s="28" t="s">
-        <v>509</v>
       </c>
       <c r="G764" s="16" t="s">
         <v>58</v>
@@ -21566,22 +21563,22 @@
     </row>
     <row r="770" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A770" s="46" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="B770" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C770" s="14" t="s">
+        <v>509</v>
+      </c>
+      <c r="D770" s="15" t="s">
         <v>510</v>
       </c>
-      <c r="D770" s="15" t="s">
+      <c r="E770" s="15" t="s">
         <v>511</v>
       </c>
-      <c r="E770" s="15" t="s">
+      <c r="F770" s="15" t="s">
         <v>512</v>
-      </c>
-      <c r="F770" s="15" t="s">
-        <v>513</v>
       </c>
       <c r="G770" s="16" t="s">
         <v>58</v>
@@ -21710,22 +21707,22 @@
     </row>
     <row r="776" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A776" s="46" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="B776" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C776" s="27" t="s">
+        <v>513</v>
+      </c>
+      <c r="D776" s="28" t="s">
         <v>514</v>
       </c>
-      <c r="D776" s="28" t="s">
+      <c r="E776" s="28" t="s">
         <v>515</v>
       </c>
-      <c r="E776" s="28" t="s">
+      <c r="F776" s="28" t="s">
         <v>516</v>
-      </c>
-      <c r="F776" s="28" t="s">
-        <v>517</v>
       </c>
       <c r="G776" s="16" t="s">
         <v>58</v>
@@ -21854,22 +21851,22 @@
     </row>
     <row r="782" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A782" s="46" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="B782" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C782" s="14" t="s">
+        <v>517</v>
+      </c>
+      <c r="D782" s="15" t="s">
         <v>518</v>
       </c>
-      <c r="D782" s="15" t="s">
+      <c r="E782" s="15" t="s">
         <v>519</v>
       </c>
-      <c r="E782" s="15" t="s">
+      <c r="F782" s="15" t="s">
         <v>520</v>
-      </c>
-      <c r="F782" s="15" t="s">
-        <v>521</v>
       </c>
       <c r="G782" s="16" t="s">
         <v>58</v>
@@ -21998,22 +21995,22 @@
     </row>
     <row r="788" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A788" s="46" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="B788" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C788" s="27" t="s">
+        <v>521</v>
+      </c>
+      <c r="D788" s="28" t="s">
         <v>522</v>
       </c>
-      <c r="D788" s="28" t="s">
+      <c r="E788" s="28" t="s">
         <v>523</v>
       </c>
-      <c r="E788" s="28" t="s">
+      <c r="F788" s="28" t="s">
         <v>524</v>
-      </c>
-      <c r="F788" s="28" t="s">
-        <v>525</v>
       </c>
       <c r="G788" s="16" t="s">
         <v>58</v>
@@ -22142,22 +22139,22 @@
     </row>
     <row r="794" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A794" s="46" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="B794" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C794" s="14" t="s">
+        <v>525</v>
+      </c>
+      <c r="D794" s="15" t="s">
         <v>526</v>
       </c>
-      <c r="D794" s="15" t="s">
+      <c r="E794" s="15" t="s">
         <v>527</v>
       </c>
-      <c r="E794" s="15" t="s">
-        <v>528</v>
-      </c>
       <c r="F794" s="15" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="G794" s="16" t="s">
         <v>58</v>
@@ -22286,22 +22283,22 @@
     </row>
     <row r="800" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A800" s="46" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="B800" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C800" s="27" t="s">
+        <v>528</v>
+      </c>
+      <c r="D800" s="28" t="s">
         <v>529</v>
       </c>
-      <c r="D800" s="28" t="s">
+      <c r="E800" s="28" t="s">
         <v>530</v>
       </c>
-      <c r="E800" s="28" t="s">
+      <c r="F800" s="28" t="s">
         <v>531</v>
-      </c>
-      <c r="F800" s="28" t="s">
-        <v>532</v>
       </c>
       <c r="G800" s="16" t="s">
         <v>58</v>
@@ -22430,22 +22427,22 @@
     </row>
     <row r="806" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A806" s="46" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="B806" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C806" s="14" t="s">
+        <v>532</v>
+      </c>
+      <c r="D806" s="15" t="s">
         <v>533</v>
       </c>
-      <c r="D806" s="15" t="s">
+      <c r="E806" s="15" t="s">
         <v>534</v>
       </c>
-      <c r="E806" s="15" t="s">
+      <c r="F806" s="15" t="s">
         <v>535</v>
-      </c>
-      <c r="F806" s="15" t="s">
-        <v>536</v>
       </c>
       <c r="G806" s="16" t="s">
         <v>58</v>
@@ -22574,22 +22571,22 @@
     </row>
     <row r="812" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A812" s="46" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="B812" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C812" s="27" t="s">
+        <v>536</v>
+      </c>
+      <c r="D812" s="28" t="s">
         <v>537</v>
       </c>
-      <c r="D812" s="28" t="s">
+      <c r="E812" s="28" t="s">
         <v>538</v>
       </c>
-      <c r="E812" s="28" t="s">
+      <c r="F812" s="28" t="s">
         <v>539</v>
-      </c>
-      <c r="F812" s="28" t="s">
-        <v>540</v>
       </c>
       <c r="G812" s="16" t="s">
         <v>58</v>
@@ -22718,22 +22715,22 @@
     </row>
     <row r="818" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A818" s="46" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="B818" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C818" s="14" t="s">
+        <v>540</v>
+      </c>
+      <c r="D818" s="15" t="s">
         <v>541</v>
       </c>
-      <c r="D818" s="15" t="s">
+      <c r="E818" s="15" t="s">
         <v>542</v>
       </c>
-      <c r="E818" s="15" t="s">
+      <c r="F818" s="15" t="s">
         <v>543</v>
-      </c>
-      <c r="F818" s="15" t="s">
-        <v>544</v>
       </c>
       <c r="G818" s="16" t="s">
         <v>58</v>
@@ -22862,22 +22859,22 @@
     </row>
     <row r="824" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A824" s="46" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="B824" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C824" s="27" t="s">
+        <v>544</v>
+      </c>
+      <c r="D824" s="28" t="s">
         <v>545</v>
       </c>
-      <c r="D824" s="28" t="s">
+      <c r="E824" s="28" t="s">
         <v>546</v>
       </c>
-      <c r="E824" s="28" t="s">
+      <c r="F824" s="28" t="s">
         <v>547</v>
-      </c>
-      <c r="F824" s="28" t="s">
-        <v>548</v>
       </c>
       <c r="G824" s="16" t="s">
         <v>58</v>
@@ -23006,22 +23003,22 @@
     </row>
     <row r="830" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A830" s="46" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="B830" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C830" s="14" t="s">
+        <v>548</v>
+      </c>
+      <c r="D830" s="15" t="s">
         <v>549</v>
       </c>
-      <c r="D830" s="15" t="s">
+      <c r="E830" s="15" t="s">
         <v>550</v>
       </c>
-      <c r="E830" s="15" t="s">
+      <c r="F830" s="15" t="s">
         <v>551</v>
-      </c>
-      <c r="F830" s="15" t="s">
-        <v>552</v>
       </c>
       <c r="G830" s="16" t="s">
         <v>58</v>
@@ -23150,22 +23147,22 @@
     </row>
     <row r="836" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A836" s="47" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="B836" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C836" s="27" t="s">
+        <v>553</v>
+      </c>
+      <c r="D836" s="28" t="s">
         <v>554</v>
       </c>
-      <c r="D836" s="28" t="s">
+      <c r="E836" s="28" t="s">
         <v>555</v>
       </c>
-      <c r="E836" s="28" t="s">
+      <c r="F836" s="28" t="s">
         <v>556</v>
-      </c>
-      <c r="F836" s="28" t="s">
-        <v>557</v>
       </c>
       <c r="G836" s="16" t="s">
         <v>58</v>
@@ -23294,22 +23291,22 @@
     </row>
     <row r="842" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A842" s="47" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="B842" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C842" s="14" t="s">
+        <v>557</v>
+      </c>
+      <c r="D842" s="15" t="s">
         <v>558</v>
       </c>
-      <c r="D842" s="15" t="s">
+      <c r="E842" s="15" t="s">
         <v>559</v>
       </c>
-      <c r="E842" s="15" t="s">
-        <v>560</v>
-      </c>
       <c r="F842" s="15" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="G842" s="16" t="s">
         <v>58</v>
@@ -23438,22 +23435,22 @@
     </row>
     <row r="848" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A848" s="47" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="B848" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C848" s="27" t="s">
+        <v>560</v>
+      </c>
+      <c r="D848" s="28" t="s">
         <v>561</v>
       </c>
-      <c r="D848" s="28" t="s">
+      <c r="E848" s="28" t="s">
         <v>562</v>
       </c>
-      <c r="E848" s="28" t="s">
+      <c r="F848" s="28" t="s">
         <v>563</v>
-      </c>
-      <c r="F848" s="28" t="s">
-        <v>564</v>
       </c>
       <c r="G848" s="16" t="s">
         <v>58</v>
@@ -23582,22 +23579,22 @@
     </row>
     <row r="854" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A854" s="47" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="B854" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C854" s="14" t="s">
+        <v>564</v>
+      </c>
+      <c r="D854" s="15" t="s">
         <v>565</v>
       </c>
-      <c r="D854" s="15" t="s">
+      <c r="E854" s="15" t="s">
         <v>566</v>
       </c>
-      <c r="E854" s="15" t="s">
+      <c r="F854" s="15" t="s">
         <v>567</v>
-      </c>
-      <c r="F854" s="15" t="s">
-        <v>568</v>
       </c>
       <c r="G854" s="16" t="s">
         <v>58</v>
@@ -23726,22 +23723,22 @@
     </row>
     <row r="860" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A860" s="48" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="B860" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C860" s="27" t="s">
+        <v>569</v>
+      </c>
+      <c r="D860" s="28" t="s">
         <v>570</v>
       </c>
-      <c r="D860" s="28" t="s">
+      <c r="E860" s="28" t="s">
         <v>571</v>
       </c>
-      <c r="E860" s="28" t="s">
+      <c r="F860" s="28" t="s">
         <v>572</v>
-      </c>
-      <c r="F860" s="28" t="s">
-        <v>573</v>
       </c>
       <c r="G860" s="16" t="s">
         <v>58</v>
@@ -23870,22 +23867,22 @@
     </row>
     <row r="866" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A866" s="48" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="B866" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C866" s="14" t="s">
+        <v>573</v>
+      </c>
+      <c r="D866" s="15" t="s">
         <v>574</v>
       </c>
-      <c r="D866" s="15" t="s">
+      <c r="E866" s="15" t="s">
         <v>575</v>
       </c>
-      <c r="E866" s="15" t="s">
+      <c r="F866" s="15" t="s">
         <v>576</v>
-      </c>
-      <c r="F866" s="15" t="s">
-        <v>577</v>
       </c>
       <c r="G866" s="16" t="s">
         <v>58</v>
@@ -24014,22 +24011,22 @@
     </row>
     <row r="872" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A872" s="48" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="B872" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C872" s="27" t="s">
+        <v>577</v>
+      </c>
+      <c r="D872" s="28" t="s">
         <v>578</v>
       </c>
-      <c r="D872" s="28" t="s">
+      <c r="E872" s="28" t="s">
         <v>579</v>
       </c>
-      <c r="E872" s="28" t="s">
+      <c r="F872" s="28" t="s">
         <v>580</v>
-      </c>
-      <c r="F872" s="28" t="s">
-        <v>581</v>
       </c>
       <c r="G872" s="16" t="s">
         <v>58</v>
@@ -24158,22 +24155,22 @@
     </row>
     <row r="878" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A878" s="48" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="B878" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C878" s="14" t="s">
+        <v>581</v>
+      </c>
+      <c r="D878" s="15" t="s">
         <v>582</v>
       </c>
-      <c r="D878" s="15" t="s">
+      <c r="E878" s="15" t="s">
         <v>583</v>
       </c>
-      <c r="E878" s="15" t="s">
+      <c r="F878" s="15" t="s">
         <v>584</v>
-      </c>
-      <c r="F878" s="15" t="s">
-        <v>585</v>
       </c>
       <c r="G878" s="16" t="s">
         <v>58</v>
@@ -24302,22 +24299,22 @@
     </row>
     <row r="884" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A884" s="48" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="B884" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C884" s="27" t="s">
+        <v>585</v>
+      </c>
+      <c r="D884" s="28" t="s">
         <v>586</v>
       </c>
-      <c r="D884" s="28" t="s">
+      <c r="E884" s="28" t="s">
         <v>587</v>
       </c>
-      <c r="E884" s="28" t="s">
+      <c r="F884" s="28" t="s">
         <v>588</v>
-      </c>
-      <c r="F884" s="28" t="s">
-        <v>589</v>
       </c>
       <c r="G884" s="16" t="s">
         <v>58</v>
@@ -24446,22 +24443,22 @@
     </row>
     <row r="890" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A890" s="48" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="B890" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C890" s="14" t="s">
+        <v>589</v>
+      </c>
+      <c r="D890" s="15" t="s">
         <v>590</v>
       </c>
-      <c r="D890" s="15" t="s">
+      <c r="E890" s="15" t="s">
         <v>591</v>
       </c>
-      <c r="E890" s="15" t="s">
+      <c r="F890" s="15" t="s">
         <v>592</v>
-      </c>
-      <c r="F890" s="15" t="s">
-        <v>593</v>
       </c>
       <c r="G890" s="16" t="s">
         <v>58</v>
@@ -24590,22 +24587,22 @@
     </row>
     <row r="896" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A896" s="48" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="B896" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C896" s="27" t="s">
+        <v>593</v>
+      </c>
+      <c r="D896" s="28" t="s">
         <v>594</v>
       </c>
-      <c r="D896" s="28" t="s">
+      <c r="E896" s="28" t="s">
         <v>595</v>
       </c>
-      <c r="E896" s="28" t="s">
+      <c r="F896" s="28" t="s">
         <v>596</v>
-      </c>
-      <c r="F896" s="28" t="s">
-        <v>597</v>
       </c>
       <c r="G896" s="16" t="s">
         <v>58</v>
@@ -24734,22 +24731,22 @@
     </row>
     <row r="902" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A902" s="49" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="B902" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C902" s="14" t="s">
+        <v>598</v>
+      </c>
+      <c r="D902" s="15" t="s">
         <v>599</v>
       </c>
-      <c r="D902" s="15" t="s">
+      <c r="E902" s="15" t="s">
         <v>600</v>
       </c>
-      <c r="E902" s="15" t="s">
+      <c r="F902" s="15" t="s">
         <v>601</v>
-      </c>
-      <c r="F902" s="15" t="s">
-        <v>602</v>
       </c>
       <c r="G902" s="16" t="s">
         <v>58</v>
@@ -24878,22 +24875,22 @@
     </row>
     <row r="908" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A908" s="49" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="B908" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C908" s="27" t="s">
+        <v>602</v>
+      </c>
+      <c r="D908" s="28" t="s">
         <v>603</v>
       </c>
-      <c r="D908" s="28" t="s">
+      <c r="E908" s="28" t="s">
         <v>604</v>
       </c>
-      <c r="E908" s="28" t="s">
+      <c r="F908" s="28" t="s">
         <v>605</v>
-      </c>
-      <c r="F908" s="28" t="s">
-        <v>606</v>
       </c>
       <c r="G908" s="16" t="s">
         <v>58</v>
@@ -25022,22 +25019,22 @@
     </row>
     <row r="914" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A914" s="49" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="B914" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C914" s="14" t="s">
+        <v>606</v>
+      </c>
+      <c r="D914" s="15" t="s">
         <v>607</v>
       </c>
-      <c r="D914" s="15" t="s">
+      <c r="E914" s="15" t="s">
         <v>608</v>
       </c>
-      <c r="E914" s="15" t="s">
+      <c r="F914" s="15" t="s">
         <v>609</v>
-      </c>
-      <c r="F914" s="15" t="s">
-        <v>610</v>
       </c>
       <c r="G914" s="16" t="s">
         <v>58</v>
@@ -25166,22 +25163,22 @@
     </row>
     <row r="920" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A920" s="49" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="B920" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C920" s="27" t="s">
+        <v>610</v>
+      </c>
+      <c r="D920" s="28" t="s">
         <v>611</v>
       </c>
-      <c r="D920" s="28" t="s">
+      <c r="E920" s="28" t="s">
         <v>612</v>
       </c>
-      <c r="E920" s="28" t="s">
+      <c r="F920" s="28" t="s">
         <v>613</v>
-      </c>
-      <c r="F920" s="28" t="s">
-        <v>614</v>
       </c>
       <c r="G920" s="16" t="s">
         <v>58</v>
@@ -25310,22 +25307,22 @@
     </row>
     <row r="926" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A926" s="49" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="B926" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C926" s="14" t="s">
+        <v>614</v>
+      </c>
+      <c r="D926" s="15" t="s">
         <v>615</v>
       </c>
-      <c r="D926" s="15" t="s">
+      <c r="E926" s="15" t="s">
         <v>616</v>
       </c>
-      <c r="E926" s="15" t="s">
+      <c r="F926" s="15" t="s">
         <v>617</v>
-      </c>
-      <c r="F926" s="15" t="s">
-        <v>618</v>
       </c>
       <c r="G926" s="16" t="s">
         <v>58</v>
@@ -25454,22 +25451,22 @@
     </row>
     <row r="932" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A932" s="49" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="B932" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C932" s="27" t="s">
+        <v>618</v>
+      </c>
+      <c r="D932" s="28" t="s">
         <v>619</v>
       </c>
-      <c r="D932" s="28" t="s">
+      <c r="E932" s="28" t="s">
         <v>620</v>
       </c>
-      <c r="E932" s="28" t="s">
+      <c r="F932" s="28" t="s">
         <v>621</v>
-      </c>
-      <c r="F932" s="28" t="s">
-        <v>622</v>
       </c>
       <c r="G932" s="16" t="s">
         <v>58</v>
@@ -25598,22 +25595,22 @@
     </row>
     <row r="938" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A938" s="50" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="B938" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C938" s="14" t="s">
+        <v>623</v>
+      </c>
+      <c r="D938" s="15" t="s">
         <v>624</v>
       </c>
-      <c r="D938" s="15" t="s">
+      <c r="E938" s="15" t="s">
         <v>625</v>
       </c>
-      <c r="E938" s="15" t="s">
+      <c r="F938" s="15" t="s">
         <v>626</v>
-      </c>
-      <c r="F938" s="15" t="s">
-        <v>627</v>
       </c>
       <c r="G938" s="16" t="s">
         <v>58</v>
@@ -25742,22 +25739,22 @@
     </row>
     <row r="944" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A944" s="50" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="B944" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C944" s="27" t="s">
+        <v>627</v>
+      </c>
+      <c r="D944" s="28" t="s">
         <v>628</v>
       </c>
-      <c r="D944" s="28" t="s">
+      <c r="E944" s="28" t="s">
         <v>629</v>
       </c>
-      <c r="E944" s="28" t="s">
+      <c r="F944" s="28" t="s">
         <v>630</v>
-      </c>
-      <c r="F944" s="28" t="s">
-        <v>631</v>
       </c>
       <c r="G944" s="16" t="s">
         <v>58</v>
@@ -25886,22 +25883,22 @@
     </row>
     <row r="950" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A950" s="50" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="B950" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C950" s="14" t="s">
+        <v>631</v>
+      </c>
+      <c r="D950" s="15" t="s">
         <v>632</v>
       </c>
-      <c r="D950" s="15" t="s">
+      <c r="E950" s="15" t="s">
         <v>633</v>
       </c>
-      <c r="E950" s="15" t="s">
+      <c r="F950" s="15" t="s">
         <v>634</v>
-      </c>
-      <c r="F950" s="15" t="s">
-        <v>635</v>
       </c>
       <c r="G950" s="16" t="s">
         <v>58</v>
@@ -26030,22 +26027,22 @@
     </row>
     <row r="956" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A956" s="50" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="B956" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C956" s="27" t="s">
+        <v>635</v>
+      </c>
+      <c r="D956" s="28" t="s">
         <v>636</v>
       </c>
-      <c r="D956" s="28" t="s">
+      <c r="E956" s="28" t="s">
         <v>637</v>
       </c>
-      <c r="E956" s="28" t="s">
-        <v>638</v>
-      </c>
       <c r="F956" s="28" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="G956" s="16" t="s">
         <v>58</v>
@@ -26174,22 +26171,22 @@
     </row>
     <row r="962" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A962" s="50" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="B962" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C962" s="14" t="s">
+        <v>638</v>
+      </c>
+      <c r="D962" s="15" t="s">
         <v>639</v>
       </c>
-      <c r="D962" s="15" t="s">
+      <c r="E962" s="15" t="s">
         <v>640</v>
       </c>
-      <c r="E962" s="15" t="s">
+      <c r="F962" s="15" t="s">
         <v>641</v>
-      </c>
-      <c r="F962" s="15" t="s">
-        <v>642</v>
       </c>
       <c r="G962" s="16" t="s">
         <v>58</v>
@@ -26318,22 +26315,22 @@
     </row>
     <row r="968" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A968" s="50" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="B968" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C968" s="27" t="s">
+        <v>642</v>
+      </c>
+      <c r="D968" s="28" t="s">
         <v>643</v>
       </c>
-      <c r="D968" s="28" t="s">
+      <c r="E968" s="28" t="s">
         <v>644</v>
       </c>
-      <c r="E968" s="28" t="s">
+      <c r="F968" s="28" t="s">
         <v>645</v>
-      </c>
-      <c r="F968" s="28" t="s">
-        <v>646</v>
       </c>
       <c r="G968" s="16" t="s">
         <v>58</v>
@@ -26462,22 +26459,22 @@
     </row>
     <row r="974" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A974" s="51" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="B974" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C974" s="14" t="s">
+        <v>647</v>
+      </c>
+      <c r="D974" s="15" t="s">
         <v>648</v>
       </c>
-      <c r="D974" s="15" t="s">
+      <c r="E974" s="15" t="s">
         <v>649</v>
       </c>
-      <c r="E974" s="15" t="s">
+      <c r="F974" s="15" t="s">
         <v>650</v>
-      </c>
-      <c r="F974" s="15" t="s">
-        <v>651</v>
       </c>
       <c r="G974" s="16" t="s">
         <v>58</v>
@@ -26606,22 +26603,22 @@
     </row>
     <row r="980" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A980" s="51" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="B980" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C980" s="27" t="s">
+        <v>651</v>
+      </c>
+      <c r="D980" s="28" t="s">
         <v>652</v>
       </c>
-      <c r="D980" s="28" t="s">
+      <c r="E980" s="28" t="s">
         <v>653</v>
       </c>
-      <c r="E980" s="28" t="s">
+      <c r="F980" s="28" t="s">
         <v>654</v>
-      </c>
-      <c r="F980" s="28" t="s">
-        <v>655</v>
       </c>
       <c r="G980" s="16" t="s">
         <v>58</v>
@@ -26750,22 +26747,22 @@
     </row>
     <row r="986" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A986" s="51" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="B986" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C986" s="14" t="s">
+        <v>655</v>
+      </c>
+      <c r="D986" s="15" t="s">
         <v>656</v>
       </c>
-      <c r="D986" s="15" t="s">
+      <c r="E986" s="15" t="s">
         <v>657</v>
       </c>
-      <c r="E986" s="15" t="s">
+      <c r="F986" s="15" t="s">
         <v>658</v>
-      </c>
-      <c r="F986" s="15" t="s">
-        <v>659</v>
       </c>
       <c r="G986" s="16" t="s">
         <v>58</v>
@@ -26894,22 +26891,22 @@
     </row>
     <row r="992" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A992" s="51" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="B992" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C992" s="27" t="s">
+        <v>659</v>
+      </c>
+      <c r="D992" s="28" t="s">
         <v>660</v>
       </c>
-      <c r="D992" s="28" t="s">
+      <c r="E992" s="28" t="s">
         <v>661</v>
       </c>
-      <c r="E992" s="28" t="s">
+      <c r="F992" s="28" t="s">
         <v>662</v>
-      </c>
-      <c r="F992" s="28" t="s">
-        <v>663</v>
       </c>
       <c r="G992" s="16" t="s">
         <v>58</v>
@@ -27038,22 +27035,22 @@
     </row>
     <row r="998" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A998" s="51" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="B998" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C998" s="14" t="s">
+        <v>663</v>
+      </c>
+      <c r="D998" s="15" t="s">
         <v>664</v>
       </c>
-      <c r="D998" s="15" t="s">
+      <c r="E998" s="15" t="s">
         <v>665</v>
       </c>
-      <c r="E998" s="15" t="s">
+      <c r="F998" s="15" t="s">
         <v>666</v>
-      </c>
-      <c r="F998" s="15" t="s">
-        <v>667</v>
       </c>
       <c r="G998" s="16" t="s">
         <v>58</v>
@@ -27182,22 +27179,22 @@
     </row>
     <row r="1004" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1004" s="52" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="B1004" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1004" s="27" t="s">
+        <v>668</v>
+      </c>
+      <c r="D1004" s="28" t="s">
         <v>669</v>
       </c>
-      <c r="D1004" s="28" t="s">
+      <c r="E1004" s="28" t="s">
         <v>670</v>
       </c>
-      <c r="E1004" s="28" t="s">
+      <c r="F1004" s="28" t="s">
         <v>671</v>
-      </c>
-      <c r="F1004" s="28" t="s">
-        <v>672</v>
       </c>
       <c r="G1004" s="16" t="s">
         <v>58</v>
@@ -27326,22 +27323,22 @@
     </row>
     <row r="1010" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1010" s="52" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="B1010" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1010" s="14" t="s">
+        <v>672</v>
+      </c>
+      <c r="D1010" s="15" t="s">
         <v>673</v>
       </c>
-      <c r="D1010" s="15" t="s">
+      <c r="E1010" s="15" t="s">
         <v>674</v>
       </c>
-      <c r="E1010" s="15" t="s">
+      <c r="F1010" s="15" t="s">
         <v>675</v>
-      </c>
-      <c r="F1010" s="15" t="s">
-        <v>676</v>
       </c>
       <c r="G1010" s="16" t="s">
         <v>58</v>
@@ -27470,22 +27467,22 @@
     </row>
     <row r="1016" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1016" s="52" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="B1016" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1016" s="27" t="s">
+        <v>676</v>
+      </c>
+      <c r="D1016" s="28" t="s">
         <v>677</v>
       </c>
-      <c r="D1016" s="28" t="s">
+      <c r="E1016" s="28" t="s">
         <v>678</v>
       </c>
-      <c r="E1016" s="28" t="s">
+      <c r="F1016" s="28" t="s">
         <v>679</v>
-      </c>
-      <c r="F1016" s="28" t="s">
-        <v>680</v>
       </c>
       <c r="G1016" s="16" t="s">
         <v>58</v>
@@ -27614,22 +27611,22 @@
     </row>
     <row r="1022" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1022" s="52" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="B1022" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1022" s="14" t="s">
+        <v>680</v>
+      </c>
+      <c r="D1022" s="15" t="s">
         <v>681</v>
       </c>
-      <c r="D1022" s="15" t="s">
+      <c r="E1022" s="15" t="s">
         <v>682</v>
       </c>
-      <c r="E1022" s="15" t="s">
+      <c r="F1022" s="15" t="s">
         <v>683</v>
-      </c>
-      <c r="F1022" s="15" t="s">
-        <v>684</v>
       </c>
       <c r="G1022" s="16" t="s">
         <v>58</v>
@@ -27758,22 +27755,22 @@
     </row>
     <row r="1028" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1028" s="52" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="B1028" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C1028" s="27" t="s">
+        <v>684</v>
+      </c>
+      <c r="D1028" s="28" t="s">
         <v>685</v>
       </c>
-      <c r="D1028" s="28" t="s">
+      <c r="E1028" s="28" t="s">
         <v>686</v>
       </c>
-      <c r="E1028" s="28" t="s">
+      <c r="F1028" s="28" t="s">
         <v>687</v>
-      </c>
-      <c r="F1028" s="28" t="s">
-        <v>688</v>
       </c>
       <c r="G1028" s="16" t="s">
         <v>58</v>
@@ -27902,22 +27899,22 @@
     </row>
     <row r="1034" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1034" s="52" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="B1034" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C1034" s="14" t="s">
+        <v>688</v>
+      </c>
+      <c r="D1034" s="15" t="s">
         <v>689</v>
       </c>
-      <c r="D1034" s="15" t="s">
+      <c r="E1034" s="15" t="s">
         <v>690</v>
       </c>
-      <c r="E1034" s="15" t="s">
+      <c r="F1034" s="15" t="s">
         <v>691</v>
-      </c>
-      <c r="F1034" s="15" t="s">
-        <v>692</v>
       </c>
       <c r="G1034" s="16" t="s">
         <v>58</v>
@@ -28046,22 +28043,22 @@
     </row>
     <row r="1040" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1040" s="53" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="B1040" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C1040" s="27" t="s">
+        <v>693</v>
+      </c>
+      <c r="D1040" s="28" t="s">
+        <v>681</v>
+      </c>
+      <c r="E1040" s="28" t="s">
         <v>694</v>
       </c>
-      <c r="D1040" s="28" t="s">
-        <v>682</v>
-      </c>
-      <c r="E1040" s="28" t="s">
+      <c r="F1040" s="28" t="s">
         <v>695</v>
-      </c>
-      <c r="F1040" s="28" t="s">
-        <v>696</v>
       </c>
       <c r="G1040" s="16" t="s">
         <v>58</v>
@@ -28190,22 +28187,22 @@
     </row>
     <row r="1046" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1046" s="53" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="B1046" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1046" s="14" t="s">
+        <v>696</v>
+      </c>
+      <c r="D1046" s="15" t="s">
+        <v>673</v>
+      </c>
+      <c r="E1046" s="15" t="s">
         <v>697</v>
       </c>
-      <c r="D1046" s="15" t="s">
-        <v>674</v>
-      </c>
-      <c r="E1046" s="15" t="s">
+      <c r="F1046" s="15" t="s">
         <v>698</v>
-      </c>
-      <c r="F1046" s="15" t="s">
-        <v>699</v>
       </c>
       <c r="G1046" s="16" t="s">
         <v>58</v>
@@ -28340,16 +28337,16 @@
         <v>53</v>
       </c>
       <c r="C1052" s="27" t="s">
+        <v>699</v>
+      </c>
+      <c r="D1052" s="28" t="s">
         <v>700</v>
       </c>
-      <c r="D1052" s="28" t="s">
+      <c r="E1052" s="28" t="s">
         <v>701</v>
       </c>
-      <c r="E1052" s="28" t="s">
+      <c r="F1052" s="28" t="s">
         <v>702</v>
-      </c>
-      <c r="F1052" s="28" t="s">
-        <v>703</v>
       </c>
       <c r="G1052" s="16" t="s">
         <v>58</v>
@@ -28484,16 +28481,16 @@
         <v>53</v>
       </c>
       <c r="C1058" s="14" t="s">
+        <v>703</v>
+      </c>
+      <c r="D1058" s="15" t="s">
         <v>704</v>
       </c>
-      <c r="D1058" s="15" t="s">
+      <c r="E1058" s="15" t="s">
         <v>705</v>
       </c>
-      <c r="E1058" s="15" t="s">
+      <c r="F1058" s="15" t="s">
         <v>706</v>
-      </c>
-      <c r="F1058" s="15" t="s">
-        <v>707</v>
       </c>
       <c r="G1058" s="16" t="s">
         <v>58</v>
@@ -29583,10 +29580,10 @@
         <v>39</v>
       </c>
       <c r="B1" s="10" t="s">
+        <v>707</v>
+      </c>
+      <c r="C1" s="10" t="s">
         <v>708</v>
-      </c>
-      <c r="C1" s="10" t="s">
-        <v>709</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>53</v>
@@ -29604,7 +29601,7 @@
         <v>87</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -29957,7 +29954,7 @@
     </row>
     <row r="14" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="66" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="B14" s="1">
         <v>5</v>
@@ -29986,7 +29983,7 @@
     </row>
     <row r="15" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="67" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="B15" s="1">
         <v>12</v>
@@ -30015,7 +30012,7 @@
     </row>
     <row r="16" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="68" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="B16" s="1">
         <v>4</v>
@@ -30044,7 +30041,7 @@
     </row>
     <row r="17" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="69" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="B17" s="1">
         <v>7</v>
@@ -30073,7 +30070,7 @@
     </row>
     <row r="18" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="70" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="B18" s="1">
         <v>6</v>
@@ -30102,7 +30099,7 @@
     </row>
     <row r="19" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="71" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="B19" s="1">
         <v>6</v>
@@ -30131,7 +30128,7 @@
     </row>
     <row r="20" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="72" t="s">
-        <v>647</v>
+        <v>646</v>
       </c>
       <c r="B20" s="1">
         <v>5</v>
@@ -30160,7 +30157,7 @@
     </row>
     <row r="21" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="73" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="B21" s="1">
         <v>6</v>
@@ -30189,7 +30186,7 @@
     </row>
     <row r="22" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="74" t="s">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="B22" s="1">
         <v>2</v>
@@ -30218,7 +30215,7 @@
     </row>
     <row r="23" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="75" t="s">
-        <v>711</v>
+        <v>710</v>
       </c>
       <c r="B23" s="75">
         <v>153</v>
@@ -30269,7 +30266,7 @@
         <v>44</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="C1" s="10" t="s">
         <v>71</v>
@@ -30278,7 +30275,7 @@
         <v>87</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="F1" s="10" t="s">
         <v>95</v>
@@ -30429,10 +30426,10 @@
         <v>45</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>709</v>
+        <v>708</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>71</v>
@@ -30441,7 +30438,7 @@
         <v>87</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="G1" s="10" t="s">
         <v>95</v>
@@ -30452,7 +30449,7 @@
         <v>59</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>713</v>
+        <v>712</v>
       </c>
       <c r="C2" s="1">
         <v>18</v>

</xml_diff>

<commit_message>
073 => fase IV => ZUP-030 OK (Chrome/USER) i codi peu actualitzat a Fase IV / Angular 22
</commit_message>
<xml_diff>
--- a/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
+++ b/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4274" uniqueCount="713">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4275" uniqueCount="714">
   <si>
     <t>Zuppeto — Joc de probes manual (totes les pantalles)</t>
   </si>
@@ -654,6 +654,9 @@
   </si>
   <si>
     <t>Títol de la portada, etiquetes pet-friendly i botons «Explora llocs» / «Entén el flux»</t>
+  </si>
+  <si>
+    <t>2026-08-24</t>
   </si>
   <si>
     <t>ZUP-031</t>
@@ -8542,9 +8545,11 @@
       <c r="H218" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="I218" s="29"/>
+      <c r="I218" s="29" t="s">
+        <v>210</v>
+      </c>
       <c r="J218" s="17" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K218" s="15"/>
       <c r="L218" s="1"/>
@@ -8933,16 +8938,16 @@
         <v>90</v>
       </c>
       <c r="C236" s="14" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D236" s="15" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="E236" s="15" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F236" s="15" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="G236" s="16" t="s">
         <v>58</v>
@@ -9077,16 +9082,16 @@
         <v>53</v>
       </c>
       <c r="C242" s="27" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D242" s="28" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E242" s="28" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="F242" s="28" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="G242" s="16" t="s">
         <v>58</v>
@@ -9221,16 +9226,16 @@
         <v>53</v>
       </c>
       <c r="C248" s="14" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="D248" s="15" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="E248" s="15" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="F248" s="15" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="G248" s="16" t="s">
         <v>58</v>
@@ -9365,16 +9370,16 @@
         <v>53</v>
       </c>
       <c r="C254" s="27" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="D254" s="28" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="E254" s="28" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="F254" s="28" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="G254" s="16" t="s">
         <v>58</v>
@@ -9509,16 +9514,16 @@
         <v>90</v>
       </c>
       <c r="C260" s="14" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="D260" s="15" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="E260" s="15" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="F260" s="15" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="G260" s="16" t="s">
         <v>58</v>
@@ -9653,16 +9658,16 @@
         <v>90</v>
       </c>
       <c r="C266" s="27" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D266" s="28" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="E266" s="28" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="F266" s="28" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="G266" s="16" t="s">
         <v>58</v>
@@ -9797,16 +9802,16 @@
         <v>90</v>
       </c>
       <c r="C272" s="14" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D272" s="15" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E272" s="15" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="F272" s="15" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="G272" s="16" t="s">
         <v>58</v>
@@ -9935,22 +9940,22 @@
     </row>
     <row r="278" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A278" s="38" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B278" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C278" s="27" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="D278" s="28" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E278" s="28" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="F278" s="28" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="G278" s="16" t="s">
         <v>58</v>
@@ -10475,22 +10480,22 @@
     </row>
     <row r="302" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A302" s="38" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B302" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C302" s="14" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D302" s="15" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="E302" s="15" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="F302" s="15" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="G302" s="16" t="s">
         <v>58</v>
@@ -10619,22 +10624,22 @@
     </row>
     <row r="308" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A308" s="38" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B308" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C308" s="27" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D308" s="28" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="E308" s="28" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="F308" s="28" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="G308" s="16" t="s">
         <v>58</v>
@@ -10763,22 +10768,22 @@
     </row>
     <row r="314" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A314" s="38" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B314" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C314" s="14" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="D314" s="15" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="E314" s="15" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="F314" s="15" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="G314" s="16" t="s">
         <v>58</v>
@@ -10907,22 +10912,22 @@
     </row>
     <row r="320" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A320" s="38" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B320" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C320" s="27" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D320" s="28" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="E320" s="28" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="F320" s="28" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="G320" s="16" t="s">
         <v>58</v>
@@ -11051,22 +11056,22 @@
     </row>
     <row r="326" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A326" s="38" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B326" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C326" s="14" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D326" s="15" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="E326" s="15" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="F326" s="15" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="G326" s="16" t="s">
         <v>58</v>
@@ -11195,22 +11200,22 @@
     </row>
     <row r="332" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A332" s="38" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B332" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C332" s="27" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="D332" s="28" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="E332" s="28" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="F332" s="28" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="G332" s="16" t="s">
         <v>58</v>
@@ -11339,22 +11344,22 @@
     </row>
     <row r="338" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A338" s="38" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B338" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C338" s="14" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D338" s="15" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="E338" s="15" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="F338" s="15" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="G338" s="16" t="s">
         <v>58</v>
@@ -11483,22 +11488,22 @@
     </row>
     <row r="344" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A344" s="38" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B344" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C344" s="27" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D344" s="28" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="E344" s="28" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F344" s="28" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="G344" s="16" t="s">
         <v>58</v>
@@ -11627,22 +11632,22 @@
     </row>
     <row r="350" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A350" s="38" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B350" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C350" s="14" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="D350" s="15" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="E350" s="15" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="F350" s="15" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="G350" s="16" t="s">
         <v>58</v>
@@ -11771,22 +11776,22 @@
     </row>
     <row r="356" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A356" s="38" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B356" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C356" s="27" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D356" s="28" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="E356" s="28" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="F356" s="28" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="G356" s="16" t="s">
         <v>58</v>
@@ -11915,22 +11920,22 @@
     </row>
     <row r="362" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A362" s="38" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B362" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C362" s="14" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="D362" s="15" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="E362" s="15" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="F362" s="15" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="G362" s="16" t="s">
         <v>58</v>
@@ -12059,22 +12064,22 @@
     </row>
     <row r="368" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A368" s="38" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B368" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C368" s="27" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="D368" s="28" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="E368" s="28" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="F368" s="28" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="G368" s="16" t="s">
         <v>58</v>
@@ -12203,22 +12208,22 @@
     </row>
     <row r="374" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A374" s="38" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B374" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C374" s="14" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D374" s="15" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E374" s="15" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F374" s="15" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="G374" s="16" t="s">
         <v>58</v>
@@ -12347,22 +12352,22 @@
     </row>
     <row r="380" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A380" s="38" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B380" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C380" s="27" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D380" s="28" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="E380" s="28" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="F380" s="28" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="G380" s="16" t="s">
         <v>58</v>
@@ -12491,22 +12496,22 @@
     </row>
     <row r="386" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A386" s="38" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B386" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C386" s="14" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D386" s="15" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="E386" s="15" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="F386" s="15" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="G386" s="16" t="s">
         <v>58</v>
@@ -12635,22 +12640,22 @@
     </row>
     <row r="392" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A392" s="38" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B392" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C392" s="27" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="D392" s="28" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="E392" s="28" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="F392" s="28" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="G392" s="16" t="s">
         <v>58</v>
@@ -12779,22 +12784,22 @@
     </row>
     <row r="398" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A398" s="39" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B398" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C398" s="14" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="D398" s="15" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E398" s="15" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="F398" s="15" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="G398" s="16" t="s">
         <v>58</v>
@@ -13319,22 +13324,22 @@
     </row>
     <row r="422" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A422" s="39" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B422" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C422" s="27" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="D422" s="28" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E422" s="28" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="F422" s="28" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="G422" s="16" t="s">
         <v>58</v>
@@ -13463,22 +13468,22 @@
     </row>
     <row r="428" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A428" s="39" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B428" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C428" s="14" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="D428" s="15" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="E428" s="15" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="F428" s="15" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="G428" s="16" t="s">
         <v>58</v>
@@ -13607,22 +13612,22 @@
     </row>
     <row r="434" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A434" s="39" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B434" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C434" s="27" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="D434" s="28" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="E434" s="28" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="F434" s="28" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="G434" s="16" t="s">
         <v>58</v>
@@ -13751,22 +13756,22 @@
     </row>
     <row r="440" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A440" s="39" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B440" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C440" s="14" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="D440" s="15" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="E440" s="15" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="F440" s="15" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="G440" s="16" t="s">
         <v>58</v>
@@ -13895,22 +13900,22 @@
     </row>
     <row r="446" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A446" s="39" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B446" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C446" s="27" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="D446" s="28" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="E446" s="28" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="F446" s="28" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="G446" s="16" t="s">
         <v>58</v>
@@ -14039,22 +14044,22 @@
     </row>
     <row r="452" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A452" s="39" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B452" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C452" s="14" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="D452" s="15" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="E452" s="15" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="F452" s="15" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="G452" s="16" t="s">
         <v>58</v>
@@ -14183,22 +14188,22 @@
     </row>
     <row r="458" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A458" s="39" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B458" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C458" s="27" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="D458" s="28" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="E458" s="28" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="F458" s="28" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="G458" s="16" t="s">
         <v>58</v>
@@ -14327,22 +14332,22 @@
     </row>
     <row r="464" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A464" s="39" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B464" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C464" s="14" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="D464" s="15" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="E464" s="15" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="F464" s="15" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="G464" s="16" t="s">
         <v>58</v>
@@ -14471,22 +14476,22 @@
     </row>
     <row r="470" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A470" s="39" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B470" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C470" s="27" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="D470" s="28" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E470" s="28" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="F470" s="28" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="G470" s="16" t="s">
         <v>58</v>
@@ -14615,22 +14620,22 @@
     </row>
     <row r="476" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A476" s="40" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B476" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C476" s="14" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="D476" s="15" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="E476" s="15" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="F476" s="15" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="G476" s="16" t="s">
         <v>58</v>
@@ -14759,22 +14764,22 @@
     </row>
     <row r="482" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A482" s="40" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B482" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C482" s="27" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="D482" s="28" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="E482" s="28" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="F482" s="28" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="G482" s="16" t="s">
         <v>58</v>
@@ -14903,22 +14908,22 @@
     </row>
     <row r="488" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A488" s="40" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B488" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C488" s="14" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="D488" s="15" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="E488" s="15" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="F488" s="15" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="G488" s="16" t="s">
         <v>58</v>
@@ -15047,22 +15052,22 @@
     </row>
     <row r="494" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A494" s="40" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B494" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C494" s="27" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="D494" s="28" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="E494" s="28" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="F494" s="28" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="G494" s="16" t="s">
         <v>58</v>
@@ -15191,22 +15196,22 @@
     </row>
     <row r="500" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A500" s="40" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B500" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C500" s="14" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="D500" s="15" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="E500" s="15" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="F500" s="15" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="G500" s="16" t="s">
         <v>58</v>
@@ -15335,22 +15340,22 @@
     </row>
     <row r="506" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A506" s="40" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B506" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C506" s="27" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="D506" s="28" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="E506" s="28" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="F506" s="28" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="G506" s="16" t="s">
         <v>58</v>
@@ -15479,22 +15484,22 @@
     </row>
     <row r="512" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A512" s="40" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B512" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C512" s="14" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="D512" s="15" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="E512" s="15" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="F512" s="15" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="G512" s="16" t="s">
         <v>58</v>
@@ -15623,22 +15628,22 @@
     </row>
     <row r="518" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A518" s="40" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B518" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C518" s="27" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="D518" s="28" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="E518" s="28" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="F518" s="28" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="G518" s="16" t="s">
         <v>58</v>
@@ -15767,22 +15772,22 @@
     </row>
     <row r="524" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A524" s="40" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B524" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C524" s="14" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="D524" s="15" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="E524" s="15" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="F524" s="15" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="G524" s="16" t="s">
         <v>58</v>
@@ -15911,22 +15916,22 @@
     </row>
     <row r="530" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A530" s="40" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B530" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C530" s="27" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="D530" s="28" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="E530" s="28" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="F530" s="28" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="G530" s="16" t="s">
         <v>58</v>
@@ -16055,22 +16060,22 @@
     </row>
     <row r="536" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A536" s="40" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B536" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C536" s="14" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="D536" s="15" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="E536" s="15" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="F536" s="15" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="G536" s="16" t="s">
         <v>58</v>
@@ -16199,22 +16204,22 @@
     </row>
     <row r="542" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A542" s="41" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B542" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C542" s="27" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="D542" s="28" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="E542" s="28" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="F542" s="28" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="G542" s="16" t="s">
         <v>58</v>
@@ -16343,22 +16348,22 @@
     </row>
     <row r="548" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A548" s="41" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B548" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C548" s="14" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="D548" s="15" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="E548" s="15" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="F548" s="15" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="G548" s="16" t="s">
         <v>58</v>
@@ -16487,22 +16492,22 @@
     </row>
     <row r="554" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A554" s="41" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B554" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C554" s="27" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="D554" s="28" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="E554" s="28" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="F554" s="28" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="G554" s="16" t="s">
         <v>58</v>
@@ -16631,22 +16636,22 @@
     </row>
     <row r="560" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A560" s="41" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B560" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C560" s="14" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D560" s="15" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="E560" s="15" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="F560" s="15" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="G560" s="16" t="s">
         <v>58</v>
@@ -16775,22 +16780,22 @@
     </row>
     <row r="566" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A566" s="41" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B566" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C566" s="27" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="D566" s="28" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="E566" s="28" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="F566" s="28" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="G566" s="16" t="s">
         <v>58</v>
@@ -16919,22 +16924,22 @@
     </row>
     <row r="572" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A572" s="41" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B572" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C572" s="14" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="D572" s="15" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="E572" s="15" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="F572" s="15" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="G572" s="16" t="s">
         <v>58</v>
@@ -17063,22 +17068,22 @@
     </row>
     <row r="578" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A578" s="41" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B578" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C578" s="27" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="D578" s="28" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="E578" s="28" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="F578" s="28" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="G578" s="16" t="s">
         <v>58</v>
@@ -17207,22 +17212,22 @@
     </row>
     <row r="584" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A584" s="41" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B584" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C584" s="14" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="D584" s="15" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="E584" s="15" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="F584" s="15" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="G584" s="16" t="s">
         <v>58</v>
@@ -17351,22 +17356,22 @@
     </row>
     <row r="590" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A590" s="41" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B590" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C590" s="27" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="D590" s="28" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="E590" s="28" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="F590" s="28" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="G590" s="16" t="s">
         <v>58</v>
@@ -17495,22 +17500,22 @@
     </row>
     <row r="596" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A596" s="42" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="B596" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C596" s="14" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="D596" s="15" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="E596" s="15" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="F596" s="15" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="G596" s="16" t="s">
         <v>58</v>
@@ -18035,22 +18040,22 @@
     </row>
     <row r="620" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A620" s="42" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="B620" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C620" s="27" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="D620" s="28" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="E620" s="28" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="F620" s="28" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="G620" s="16" t="s">
         <v>58</v>
@@ -18179,22 +18184,22 @@
     </row>
     <row r="626" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A626" s="42" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="B626" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C626" s="14" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="D626" s="15" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="E626" s="15" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="F626" s="15" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="G626" s="16" t="s">
         <v>58</v>
@@ -18323,22 +18328,22 @@
     </row>
     <row r="632" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A632" s="42" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="B632" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C632" s="27" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="D632" s="28" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="E632" s="28" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="F632" s="28" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="G632" s="16" t="s">
         <v>58</v>
@@ -18467,22 +18472,22 @@
     </row>
     <row r="638" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A638" s="42" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="B638" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C638" s="14" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="D638" s="15" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E638" s="15" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="F638" s="15" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="G638" s="16" t="s">
         <v>58</v>
@@ -18611,22 +18616,22 @@
     </row>
     <row r="644" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A644" s="43" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="B644" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C644" s="27" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="D644" s="28" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="E644" s="28" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="F644" s="28" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="G644" s="16" t="s">
         <v>58</v>
@@ -19151,22 +19156,22 @@
     </row>
     <row r="668" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A668" s="43" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="B668" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C668" s="14" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="D668" s="15" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="E668" s="15" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="F668" s="15" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="G668" s="16" t="s">
         <v>58</v>
@@ -19295,22 +19300,22 @@
     </row>
     <row r="674" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A674" s="43" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="B674" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C674" s="27" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="D674" s="28" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="E674" s="28" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="F674" s="28" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="G674" s="16" t="s">
         <v>58</v>
@@ -19439,22 +19444,22 @@
     </row>
     <row r="680" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A680" s="43" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="B680" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C680" s="14" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="D680" s="15" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="E680" s="15" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="F680" s="15" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="G680" s="16" t="s">
         <v>58</v>
@@ -19583,22 +19588,22 @@
     </row>
     <row r="686" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A686" s="43" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="B686" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C686" s="27" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="D686" s="28" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="E686" s="28" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="F686" s="28" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="G686" s="16" t="s">
         <v>58</v>
@@ -19727,22 +19732,22 @@
     </row>
     <row r="692" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A692" s="44" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="B692" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C692" s="14" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="D692" s="15" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="E692" s="15" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="F692" s="15" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="G692" s="16" t="s">
         <v>58</v>
@@ -20267,22 +20272,22 @@
     </row>
     <row r="716" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A716" s="44" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="B716" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C716" s="27" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="D716" s="28" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="E716" s="28" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="F716" s="28" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="G716" s="16" t="s">
         <v>58</v>
@@ -20411,22 +20416,22 @@
     </row>
     <row r="722" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A722" s="44" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="B722" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C722" s="14" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="D722" s="15" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="E722" s="15" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="F722" s="15" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="G722" s="16" t="s">
         <v>58</v>
@@ -20555,22 +20560,22 @@
     </row>
     <row r="728" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A728" s="44" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="B728" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C728" s="27" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="D728" s="28" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E728" s="28" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="F728" s="28" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="G728" s="16" t="s">
         <v>58</v>
@@ -20699,22 +20704,22 @@
     </row>
     <row r="734" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A734" s="45" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="B734" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C734" s="14" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="D734" s="15" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="E734" s="15" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="F734" s="15" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="G734" s="16" t="s">
         <v>58</v>
@@ -20843,22 +20848,22 @@
     </row>
     <row r="740" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A740" s="45" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="B740" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C740" s="27" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="D740" s="28" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="E740" s="28" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="F740" s="28" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="G740" s="16" t="s">
         <v>58</v>
@@ -20987,22 +20992,22 @@
     </row>
     <row r="746" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A746" s="45" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="B746" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C746" s="14" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="D746" s="15" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="E746" s="15" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="F746" s="15" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="G746" s="16" t="s">
         <v>58</v>
@@ -21131,22 +21136,22 @@
     </row>
     <row r="752" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A752" s="45" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="B752" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C752" s="27" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="D752" s="28" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="E752" s="28" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="F752" s="28" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="G752" s="16" t="s">
         <v>58</v>
@@ -21275,22 +21280,22 @@
     </row>
     <row r="758" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A758" s="45" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="B758" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C758" s="14" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="D758" s="15" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="E758" s="15" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="F758" s="15" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="G758" s="16" t="s">
         <v>58</v>
@@ -21419,22 +21424,22 @@
     </row>
     <row r="764" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A764" s="46" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B764" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C764" s="27" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="D764" s="28" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="E764" s="28" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="F764" s="28" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="G764" s="16" t="s">
         <v>58</v>
@@ -21563,22 +21568,22 @@
     </row>
     <row r="770" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A770" s="46" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B770" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C770" s="14" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="D770" s="15" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="E770" s="15" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="F770" s="15" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="G770" s="16" t="s">
         <v>58</v>
@@ -21707,22 +21712,22 @@
     </row>
     <row r="776" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A776" s="46" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B776" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C776" s="27" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="D776" s="28" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="E776" s="28" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="F776" s="28" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="G776" s="16" t="s">
         <v>58</v>
@@ -21851,22 +21856,22 @@
     </row>
     <row r="782" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A782" s="46" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B782" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C782" s="14" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="D782" s="15" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="E782" s="15" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="F782" s="15" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="G782" s="16" t="s">
         <v>58</v>
@@ -21995,22 +22000,22 @@
     </row>
     <row r="788" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A788" s="46" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B788" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C788" s="27" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="D788" s="28" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="E788" s="28" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="F788" s="28" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="G788" s="16" t="s">
         <v>58</v>
@@ -22139,22 +22144,22 @@
     </row>
     <row r="794" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A794" s="46" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B794" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C794" s="14" t="s">
+        <v>526</v>
+      </c>
+      <c r="D794" s="15" t="s">
+        <v>527</v>
+      </c>
+      <c r="E794" s="15" t="s">
+        <v>528</v>
+      </c>
+      <c r="F794" s="15" t="s">
         <v>525</v>
-      </c>
-      <c r="D794" s="15" t="s">
-        <v>526</v>
-      </c>
-      <c r="E794" s="15" t="s">
-        <v>527</v>
-      </c>
-      <c r="F794" s="15" t="s">
-        <v>524</v>
       </c>
       <c r="G794" s="16" t="s">
         <v>58</v>
@@ -22283,22 +22288,22 @@
     </row>
     <row r="800" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A800" s="46" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B800" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C800" s="27" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="D800" s="28" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="E800" s="28" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="F800" s="28" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="G800" s="16" t="s">
         <v>58</v>
@@ -22427,22 +22432,22 @@
     </row>
     <row r="806" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A806" s="46" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B806" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C806" s="14" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="D806" s="15" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="E806" s="15" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="F806" s="15" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="G806" s="16" t="s">
         <v>58</v>
@@ -22571,22 +22576,22 @@
     </row>
     <row r="812" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A812" s="46" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B812" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C812" s="27" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="D812" s="28" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="E812" s="28" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="F812" s="28" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="G812" s="16" t="s">
         <v>58</v>
@@ -22715,22 +22720,22 @@
     </row>
     <row r="818" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A818" s="46" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B818" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C818" s="14" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="D818" s="15" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="E818" s="15" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="F818" s="15" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="G818" s="16" t="s">
         <v>58</v>
@@ -22859,22 +22864,22 @@
     </row>
     <row r="824" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A824" s="46" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B824" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C824" s="27" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="D824" s="28" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="E824" s="28" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="F824" s="28" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="G824" s="16" t="s">
         <v>58</v>
@@ -23003,22 +23008,22 @@
     </row>
     <row r="830" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A830" s="46" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B830" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C830" s="14" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="D830" s="15" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="E830" s="15" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="F830" s="15" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="G830" s="16" t="s">
         <v>58</v>
@@ -23147,22 +23152,22 @@
     </row>
     <row r="836" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A836" s="47" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="B836" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C836" s="27" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="D836" s="28" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="E836" s="28" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="F836" s="28" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="G836" s="16" t="s">
         <v>58</v>
@@ -23291,22 +23296,22 @@
     </row>
     <row r="842" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A842" s="47" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="B842" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C842" s="14" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="D842" s="15" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="E842" s="15" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="F842" s="15" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="G842" s="16" t="s">
         <v>58</v>
@@ -23435,22 +23440,22 @@
     </row>
     <row r="848" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A848" s="47" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="B848" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C848" s="27" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="D848" s="28" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="E848" s="28" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="F848" s="28" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="G848" s="16" t="s">
         <v>58</v>
@@ -23579,22 +23584,22 @@
     </row>
     <row r="854" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A854" s="47" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="B854" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C854" s="14" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="D854" s="15" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="E854" s="15" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="F854" s="15" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="G854" s="16" t="s">
         <v>58</v>
@@ -23723,22 +23728,22 @@
     </row>
     <row r="860" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A860" s="48" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="B860" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C860" s="27" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="D860" s="28" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="E860" s="28" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="F860" s="28" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="G860" s="16" t="s">
         <v>58</v>
@@ -23867,22 +23872,22 @@
     </row>
     <row r="866" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A866" s="48" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="B866" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C866" s="14" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="D866" s="15" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="E866" s="15" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="F866" s="15" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="G866" s="16" t="s">
         <v>58</v>
@@ -24011,22 +24016,22 @@
     </row>
     <row r="872" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A872" s="48" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="B872" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C872" s="27" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="D872" s="28" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="E872" s="28" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="F872" s="28" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="G872" s="16" t="s">
         <v>58</v>
@@ -24155,22 +24160,22 @@
     </row>
     <row r="878" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A878" s="48" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="B878" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C878" s="14" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="D878" s="15" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="E878" s="15" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="F878" s="15" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="G878" s="16" t="s">
         <v>58</v>
@@ -24299,22 +24304,22 @@
     </row>
     <row r="884" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A884" s="48" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="B884" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C884" s="27" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="D884" s="28" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="E884" s="28" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="F884" s="28" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="G884" s="16" t="s">
         <v>58</v>
@@ -24443,22 +24448,22 @@
     </row>
     <row r="890" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A890" s="48" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="B890" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C890" s="14" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="D890" s="15" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="E890" s="15" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="F890" s="15" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="G890" s="16" t="s">
         <v>58</v>
@@ -24587,22 +24592,22 @@
     </row>
     <row r="896" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A896" s="48" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="B896" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C896" s="27" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="D896" s="28" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="E896" s="28" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="F896" s="28" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="G896" s="16" t="s">
         <v>58</v>
@@ -24731,22 +24736,22 @@
     </row>
     <row r="902" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A902" s="49" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="B902" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C902" s="14" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="D902" s="15" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="E902" s="15" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="F902" s="15" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="G902" s="16" t="s">
         <v>58</v>
@@ -24875,22 +24880,22 @@
     </row>
     <row r="908" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A908" s="49" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="B908" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C908" s="27" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="D908" s="28" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="E908" s="28" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="F908" s="28" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="G908" s="16" t="s">
         <v>58</v>
@@ -25019,22 +25024,22 @@
     </row>
     <row r="914" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A914" s="49" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="B914" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C914" s="14" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="D914" s="15" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="E914" s="15" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="F914" s="15" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="G914" s="16" t="s">
         <v>58</v>
@@ -25163,22 +25168,22 @@
     </row>
     <row r="920" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A920" s="49" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="B920" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C920" s="27" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="D920" s="28" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="E920" s="28" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="F920" s="28" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="G920" s="16" t="s">
         <v>58</v>
@@ -25307,22 +25312,22 @@
     </row>
     <row r="926" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A926" s="49" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="B926" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C926" s="14" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="D926" s="15" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="E926" s="15" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="F926" s="15" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="G926" s="16" t="s">
         <v>58</v>
@@ -25451,22 +25456,22 @@
     </row>
     <row r="932" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A932" s="49" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="B932" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C932" s="27" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="D932" s="28" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="E932" s="28" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="F932" s="28" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="G932" s="16" t="s">
         <v>58</v>
@@ -25595,22 +25600,22 @@
     </row>
     <row r="938" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A938" s="50" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="B938" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C938" s="14" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="D938" s="15" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="E938" s="15" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="F938" s="15" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="G938" s="16" t="s">
         <v>58</v>
@@ -25739,22 +25744,22 @@
     </row>
     <row r="944" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A944" s="50" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="B944" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C944" s="27" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="D944" s="28" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="E944" s="28" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="F944" s="28" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="G944" s="16" t="s">
         <v>58</v>
@@ -25883,22 +25888,22 @@
     </row>
     <row r="950" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A950" s="50" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="B950" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C950" s="14" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="D950" s="15" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="E950" s="15" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="F950" s="15" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="G950" s="16" t="s">
         <v>58</v>
@@ -26027,22 +26032,22 @@
     </row>
     <row r="956" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A956" s="50" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="B956" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C956" s="27" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="D956" s="28" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="E956" s="28" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="F956" s="28" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="G956" s="16" t="s">
         <v>58</v>
@@ -26171,22 +26176,22 @@
     </row>
     <row r="962" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A962" s="50" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="B962" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C962" s="14" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="D962" s="15" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="E962" s="15" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="F962" s="15" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="G962" s="16" t="s">
         <v>58</v>
@@ -26315,22 +26320,22 @@
     </row>
     <row r="968" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A968" s="50" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="B968" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C968" s="27" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="D968" s="28" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="E968" s="28" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="F968" s="28" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="G968" s="16" t="s">
         <v>58</v>
@@ -26459,22 +26464,22 @@
     </row>
     <row r="974" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A974" s="51" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="B974" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C974" s="14" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="D974" s="15" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="E974" s="15" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="F974" s="15" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="G974" s="16" t="s">
         <v>58</v>
@@ -26603,22 +26608,22 @@
     </row>
     <row r="980" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A980" s="51" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="B980" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C980" s="27" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="D980" s="28" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="E980" s="28" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="F980" s="28" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="G980" s="16" t="s">
         <v>58</v>
@@ -26747,22 +26752,22 @@
     </row>
     <row r="986" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A986" s="51" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="B986" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C986" s="14" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="D986" s="15" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="E986" s="15" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="F986" s="15" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="G986" s="16" t="s">
         <v>58</v>
@@ -26891,22 +26896,22 @@
     </row>
     <row r="992" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A992" s="51" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="B992" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C992" s="27" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="D992" s="28" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="E992" s="28" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="F992" s="28" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="G992" s="16" t="s">
         <v>58</v>
@@ -27035,22 +27040,22 @@
     </row>
     <row r="998" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A998" s="51" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="B998" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C998" s="14" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="D998" s="15" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="E998" s="15" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="F998" s="15" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="G998" s="16" t="s">
         <v>58</v>
@@ -27179,22 +27184,22 @@
     </row>
     <row r="1004" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1004" s="52" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="B1004" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1004" s="27" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="D1004" s="28" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="E1004" s="28" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="F1004" s="28" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="G1004" s="16" t="s">
         <v>58</v>
@@ -27323,22 +27328,22 @@
     </row>
     <row r="1010" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1010" s="52" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="B1010" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1010" s="14" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="D1010" s="15" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="E1010" s="15" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="F1010" s="15" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="G1010" s="16" t="s">
         <v>58</v>
@@ -27467,22 +27472,22 @@
     </row>
     <row r="1016" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1016" s="52" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="B1016" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1016" s="27" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="D1016" s="28" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="E1016" s="28" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="F1016" s="28" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="G1016" s="16" t="s">
         <v>58</v>
@@ -27611,22 +27616,22 @@
     </row>
     <row r="1022" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1022" s="52" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="B1022" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1022" s="14" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="D1022" s="15" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="E1022" s="15" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="F1022" s="15" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="G1022" s="16" t="s">
         <v>58</v>
@@ -27755,22 +27760,22 @@
     </row>
     <row r="1028" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1028" s="52" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="B1028" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C1028" s="27" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="D1028" s="28" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="E1028" s="28" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="F1028" s="28" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="G1028" s="16" t="s">
         <v>58</v>
@@ -27899,22 +27904,22 @@
     </row>
     <row r="1034" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1034" s="52" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="B1034" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C1034" s="14" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="D1034" s="15" t="s">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="E1034" s="15" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="F1034" s="15" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="G1034" s="16" t="s">
         <v>58</v>
@@ -28043,22 +28048,22 @@
     </row>
     <row r="1040" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1040" s="53" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="B1040" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C1040" s="27" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="D1040" s="28" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="E1040" s="28" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="F1040" s="28" t="s">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="G1040" s="16" t="s">
         <v>58</v>
@@ -28187,22 +28192,22 @@
     </row>
     <row r="1046" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1046" s="53" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="B1046" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1046" s="14" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="D1046" s="15" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="E1046" s="15" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="F1046" s="15" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="G1046" s="16" t="s">
         <v>58</v>
@@ -28337,16 +28342,16 @@
         <v>53</v>
       </c>
       <c r="C1052" s="27" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="D1052" s="28" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="E1052" s="28" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="F1052" s="28" t="s">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="G1052" s="16" t="s">
         <v>58</v>
@@ -28481,16 +28486,16 @@
         <v>53</v>
       </c>
       <c r="C1058" s="14" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="D1058" s="15" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="E1058" s="15" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="F1058" s="15" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="G1058" s="16" t="s">
         <v>58</v>
@@ -29580,10 +29585,10 @@
         <v>39</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>53</v>
@@ -29601,7 +29606,7 @@
         <v>87</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -29751,7 +29756,7 @@
     </row>
     <row r="7" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="59" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B7" s="1">
         <v>17</v>
@@ -29780,7 +29785,7 @@
     </row>
     <row r="8" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="60" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B8" s="1">
         <v>10</v>
@@ -29809,7 +29814,7 @@
     </row>
     <row r="9" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="61" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="B9" s="1">
         <v>11</v>
@@ -29838,7 +29843,7 @@
     </row>
     <row r="10" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="62" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B10" s="1">
         <v>9</v>
@@ -29867,7 +29872,7 @@
     </row>
     <row r="11" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="63" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="B11" s="1">
         <v>5</v>
@@ -29896,7 +29901,7 @@
     </row>
     <row r="12" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="64" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="B12" s="1">
         <v>5</v>
@@ -29925,7 +29930,7 @@
     </row>
     <row r="13" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="65" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="B13" s="1">
         <v>4</v>
@@ -29954,7 +29959,7 @@
     </row>
     <row r="14" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="66" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="B14" s="1">
         <v>5</v>
@@ -29983,7 +29988,7 @@
     </row>
     <row r="15" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="67" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="B15" s="1">
         <v>12</v>
@@ -30012,7 +30017,7 @@
     </row>
     <row r="16" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="68" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="B16" s="1">
         <v>4</v>
@@ -30041,7 +30046,7 @@
     </row>
     <row r="17" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="69" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="B17" s="1">
         <v>7</v>
@@ -30070,7 +30075,7 @@
     </row>
     <row r="18" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="70" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="B18" s="1">
         <v>6</v>
@@ -30099,7 +30104,7 @@
     </row>
     <row r="19" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="71" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="B19" s="1">
         <v>6</v>
@@ -30128,7 +30133,7 @@
     </row>
     <row r="20" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="72" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="B20" s="1">
         <v>5</v>
@@ -30157,7 +30162,7 @@
     </row>
     <row r="21" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="73" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="B21" s="1">
         <v>6</v>
@@ -30186,7 +30191,7 @@
     </row>
     <row r="22" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="74" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="B22" s="1">
         <v>2</v>
@@ -30215,7 +30220,7 @@
     </row>
     <row r="23" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="75" t="s">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="B23" s="75">
         <v>153</v>
@@ -30266,7 +30271,7 @@
         <v>44</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="C1" s="10" t="s">
         <v>71</v>
@@ -30275,7 +30280,7 @@
         <v>87</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="F1" s="10" t="s">
         <v>95</v>
@@ -30426,10 +30431,10 @@
         <v>45</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>71</v>
@@ -30438,7 +30443,7 @@
         <v>87</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="G1" s="10" t="s">
         <v>95</v>
@@ -30449,7 +30454,7 @@
         <v>59</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="C2" s="1">
         <v>18</v>

</xml_diff>

<commit_message>
074 => fase IV => ZUP-032 ZUP-033 ZUP-034 OK (Chrome/USER), fix 500 afegir favorits (ZUP-060) i traça KO a Excel/regla
</commit_message>
<xml_diff>
--- a/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
+++ b/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4275" uniqueCount="714">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4284" uniqueCount="717">
   <si>
     <t>Zuppeto — Joc de probes manual (totes les pantalles)</t>
   </si>
@@ -707,6 +707,9 @@
     <t>Fins a 10 llocs favorits destacats a la franja principal</t>
   </si>
   <si>
+    <t>Favorits destacats amb Brisa, Frida i Coco (reals). Correcció ZUP-060 prèvia OK.</t>
+  </si>
+  <si>
     <t>ZUP-035</t>
   </si>
   <si>
@@ -1020,6 +1023,12 @@
   </si>
   <si>
     <t>Estat favorit canvia i persisteix</t>
+  </si>
+  <si>
+    <t>Al clicar «Favorit» al detall d'un segon lloc (ex. Frida) surt error de servidor 500. El primer favorit (ex. Brisa Bistro) sí es guardava.</t>
+  </si>
+  <si>
+    <t>Què s'ha fet: (1) RestorePersistedEntry al carregar. (2) UpdateAsync amb Add/Remove explícits i Id no temporal (IsTemporary=false) perquè EF faci INSERT i no UPDATE. Sense canvi de migració. Fitxers: FavoriteList.cs, FavoriteListPersistenceMapper.cs, FavoriteListRepository.cs. Cal reiniciar API i retest.</t>
   </si>
   <si>
     <t>ZUP-061</t>
@@ -9099,9 +9108,11 @@
       <c r="H242" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="I242" s="29"/>
+      <c r="I242" s="29" t="s">
+        <v>210</v>
+      </c>
       <c r="J242" s="17" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K242" s="15"/>
       <c r="L242" s="1"/>
@@ -9243,9 +9254,11 @@
       <c r="H248" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="I248" s="29"/>
+      <c r="I248" s="29" t="s">
+        <v>210</v>
+      </c>
       <c r="J248" s="17" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K248" s="15"/>
       <c r="L248" s="1"/>
@@ -9387,11 +9400,15 @@
       <c r="H254" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="I254" s="29"/>
+      <c r="I254" s="29" t="s">
+        <v>210</v>
+      </c>
       <c r="J254" s="17" t="s">
-        <v>60</v>
-      </c>
-      <c r="K254" s="15"/>
+        <v>71</v>
+      </c>
+      <c r="K254" s="15" t="s">
+        <v>227</v>
+      </c>
       <c r="L254" s="1"/>
       <c r="M254" s="1"/>
       <c r="N254" s="1"/>
@@ -9514,16 +9531,16 @@
         <v>90</v>
       </c>
       <c r="C260" s="14" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="D260" s="15" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="E260" s="15" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="F260" s="15" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="G260" s="16" t="s">
         <v>58</v>
@@ -9658,16 +9675,16 @@
         <v>90</v>
       </c>
       <c r="C266" s="27" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D266" s="28" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="E266" s="28" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="F266" s="28" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="G266" s="16" t="s">
         <v>58</v>
@@ -9802,16 +9819,16 @@
         <v>90</v>
       </c>
       <c r="C272" s="14" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D272" s="15" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E272" s="15" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="F272" s="15" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="G272" s="16" t="s">
         <v>58</v>
@@ -9940,22 +9957,22 @@
     </row>
     <row r="278" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A278" s="38" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B278" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C278" s="27" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="D278" s="28" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="E278" s="28" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="F278" s="28" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="G278" s="16" t="s">
         <v>58</v>
@@ -10480,22 +10497,22 @@
     </row>
     <row r="302" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A302" s="38" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B302" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C302" s="14" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="D302" s="15" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="E302" s="15" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="F302" s="15" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="G302" s="16" t="s">
         <v>58</v>
@@ -10624,22 +10641,22 @@
     </row>
     <row r="308" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A308" s="38" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B308" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C308" s="27" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="D308" s="28" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="E308" s="28" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="F308" s="28" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="G308" s="16" t="s">
         <v>58</v>
@@ -10768,22 +10785,22 @@
     </row>
     <row r="314" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A314" s="38" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B314" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C314" s="14" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="D314" s="15" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="E314" s="15" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="F314" s="15" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="G314" s="16" t="s">
         <v>58</v>
@@ -10912,22 +10929,22 @@
     </row>
     <row r="320" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A320" s="38" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B320" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C320" s="27" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D320" s="28" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="E320" s="28" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="F320" s="28" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="G320" s="16" t="s">
         <v>58</v>
@@ -11056,22 +11073,22 @@
     </row>
     <row r="326" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A326" s="38" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B326" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C326" s="14" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D326" s="15" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E326" s="15" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="F326" s="15" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="G326" s="16" t="s">
         <v>58</v>
@@ -11200,22 +11217,22 @@
     </row>
     <row r="332" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A332" s="38" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B332" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C332" s="27" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="D332" s="28" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="E332" s="28" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="F332" s="28" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="G332" s="16" t="s">
         <v>58</v>
@@ -11344,22 +11361,22 @@
     </row>
     <row r="338" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A338" s="38" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B338" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C338" s="14" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D338" s="15" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="E338" s="15" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="F338" s="15" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="G338" s="16" t="s">
         <v>58</v>
@@ -11488,22 +11505,22 @@
     </row>
     <row r="344" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A344" s="38" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B344" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C344" s="27" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D344" s="28" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="E344" s="28" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F344" s="28" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="G344" s="16" t="s">
         <v>58</v>
@@ -11632,22 +11649,22 @@
     </row>
     <row r="350" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A350" s="38" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B350" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C350" s="14" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D350" s="15" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="E350" s="15" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="F350" s="15" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="G350" s="16" t="s">
         <v>58</v>
@@ -11776,22 +11793,22 @@
     </row>
     <row r="356" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A356" s="38" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B356" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C356" s="27" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="D356" s="28" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="E356" s="28" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="F356" s="28" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="G356" s="16" t="s">
         <v>58</v>
@@ -11920,19 +11937,19 @@
     </row>
     <row r="362" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A362" s="38" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B362" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C362" s="14" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D362" s="15" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="E362" s="15" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="F362" s="15" t="s">
         <v>222</v>
@@ -12064,22 +12081,22 @@
     </row>
     <row r="368" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A368" s="38" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B368" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C368" s="27" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D368" s="28" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="E368" s="28" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="F368" s="28" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="G368" s="16" t="s">
         <v>58</v>
@@ -12208,22 +12225,22 @@
     </row>
     <row r="374" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A374" s="38" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B374" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C374" s="14" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="D374" s="15" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="E374" s="15" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="F374" s="15" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="G374" s="16" t="s">
         <v>58</v>
@@ -12352,22 +12369,22 @@
     </row>
     <row r="380" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A380" s="38" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B380" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C380" s="27" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D380" s="28" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="E380" s="28" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="F380" s="28" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="G380" s="16" t="s">
         <v>58</v>
@@ -12496,22 +12513,22 @@
     </row>
     <row r="386" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A386" s="38" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B386" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C386" s="14" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D386" s="15" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="E386" s="15" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="F386" s="15" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="G386" s="16" t="s">
         <v>58</v>
@@ -12640,22 +12657,22 @@
     </row>
     <row r="392" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A392" s="38" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B392" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C392" s="27" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="D392" s="28" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="E392" s="28" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="F392" s="28" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="G392" s="16" t="s">
         <v>58</v>
@@ -12784,22 +12801,22 @@
     </row>
     <row r="398" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A398" s="39" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B398" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C398" s="14" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="D398" s="15" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E398" s="15" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="F398" s="15" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="G398" s="16" t="s">
         <v>58</v>
@@ -13324,22 +13341,22 @@
     </row>
     <row r="422" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A422" s="39" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B422" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C422" s="27" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="D422" s="28" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E422" s="28" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="F422" s="28" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="G422" s="16" t="s">
         <v>58</v>
@@ -13468,22 +13485,22 @@
     </row>
     <row r="428" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A428" s="39" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B428" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C428" s="14" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="D428" s="15" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="E428" s="15" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="F428" s="15" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="G428" s="16" t="s">
         <v>58</v>
@@ -13612,22 +13629,22 @@
     </row>
     <row r="434" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A434" s="39" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B434" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C434" s="27" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="D434" s="28" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="E434" s="28" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="F434" s="28" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="G434" s="16" t="s">
         <v>58</v>
@@ -13756,22 +13773,22 @@
     </row>
     <row r="440" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A440" s="39" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B440" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C440" s="14" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="D440" s="15" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="E440" s="15" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="F440" s="15" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="G440" s="16" t="s">
         <v>58</v>
@@ -13900,22 +13917,22 @@
     </row>
     <row r="446" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A446" s="39" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B446" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C446" s="27" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="D446" s="28" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="E446" s="28" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="F446" s="28" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="G446" s="16" t="s">
         <v>58</v>
@@ -13923,14 +13940,24 @@
       <c r="H446" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="I446" s="29"/>
+      <c r="I446" s="29" t="s">
+        <v>210</v>
+      </c>
       <c r="J446" s="17" t="s">
-        <v>60</v>
-      </c>
-      <c r="K446" s="15"/>
-      <c r="L446" s="1"/>
-      <c r="M446" s="1"/>
-      <c r="N446" s="1"/>
+        <v>87</v>
+      </c>
+      <c r="K446" s="15" t="s">
+        <v>333</v>
+      </c>
+      <c r="L446" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="M446" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="N446" s="1" t="s">
+        <v>334</v>
+      </c>
     </row>
     <row r="447" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A447" s="39"/>
@@ -14044,22 +14071,22 @@
     </row>
     <row r="452" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A452" s="39" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B452" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C452" s="14" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="D452" s="15" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="E452" s="15" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="F452" s="15" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="G452" s="16" t="s">
         <v>58</v>
@@ -14188,22 +14215,22 @@
     </row>
     <row r="458" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A458" s="39" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B458" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C458" s="27" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="D458" s="28" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="E458" s="28" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="F458" s="28" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="G458" s="16" t="s">
         <v>58</v>
@@ -14332,22 +14359,22 @@
     </row>
     <row r="464" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A464" s="39" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B464" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C464" s="14" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="D464" s="15" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="E464" s="15" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="F464" s="15" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="G464" s="16" t="s">
         <v>58</v>
@@ -14476,22 +14503,22 @@
     </row>
     <row r="470" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A470" s="39" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B470" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C470" s="27" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="D470" s="28" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="E470" s="28" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="F470" s="28" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="G470" s="16" t="s">
         <v>58</v>
@@ -14620,22 +14647,22 @@
     </row>
     <row r="476" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A476" s="40" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="B476" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C476" s="14" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="D476" s="15" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="E476" s="15" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="F476" s="15" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="G476" s="16" t="s">
         <v>58</v>
@@ -14764,22 +14791,22 @@
     </row>
     <row r="482" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A482" s="40" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="B482" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C482" s="27" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="D482" s="28" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="E482" s="28" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="F482" s="28" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="G482" s="16" t="s">
         <v>58</v>
@@ -14908,22 +14935,22 @@
     </row>
     <row r="488" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A488" s="40" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="B488" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C488" s="14" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="D488" s="15" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="E488" s="15" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="F488" s="15" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="G488" s="16" t="s">
         <v>58</v>
@@ -15052,22 +15079,22 @@
     </row>
     <row r="494" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A494" s="40" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="B494" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C494" s="27" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="D494" s="28" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="E494" s="28" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="F494" s="28" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="G494" s="16" t="s">
         <v>58</v>
@@ -15196,22 +15223,22 @@
     </row>
     <row r="500" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A500" s="40" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="B500" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C500" s="14" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="D500" s="15" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="E500" s="15" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="F500" s="15" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="G500" s="16" t="s">
         <v>58</v>
@@ -15340,22 +15367,22 @@
     </row>
     <row r="506" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A506" s="40" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="B506" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C506" s="27" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="D506" s="28" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="E506" s="28" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="F506" s="28" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="G506" s="16" t="s">
         <v>58</v>
@@ -15484,22 +15511,22 @@
     </row>
     <row r="512" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A512" s="40" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="B512" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C512" s="14" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="D512" s="15" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="E512" s="15" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="F512" s="15" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="G512" s="16" t="s">
         <v>58</v>
@@ -15628,22 +15655,22 @@
     </row>
     <row r="518" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A518" s="40" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="B518" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C518" s="27" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="D518" s="28" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E518" s="28" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
       <c r="F518" s="28" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="G518" s="16" t="s">
         <v>58</v>
@@ -15772,22 +15799,22 @@
     </row>
     <row r="524" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A524" s="40" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="B524" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C524" s="14" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="D524" s="15" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="E524" s="15" t="s">
-        <v>382</v>
+        <v>385</v>
       </c>
       <c r="F524" s="15" t="s">
-        <v>383</v>
+        <v>386</v>
       </c>
       <c r="G524" s="16" t="s">
         <v>58</v>
@@ -15916,22 +15943,22 @@
     </row>
     <row r="530" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A530" s="40" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="B530" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C530" s="27" t="s">
-        <v>384</v>
+        <v>387</v>
       </c>
       <c r="D530" s="28" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="E530" s="28" t="s">
-        <v>386</v>
+        <v>389</v>
       </c>
       <c r="F530" s="28" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="G530" s="16" t="s">
         <v>58</v>
@@ -16060,22 +16087,22 @@
     </row>
     <row r="536" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A536" s="40" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="B536" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C536" s="14" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="D536" s="15" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="E536" s="15" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
       <c r="F536" s="15" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="G536" s="16" t="s">
         <v>58</v>
@@ -16204,22 +16231,22 @@
     </row>
     <row r="542" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A542" s="41" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="B542" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C542" s="27" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
       <c r="D542" s="28" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="E542" s="28" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="F542" s="28" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
       <c r="G542" s="16" t="s">
         <v>58</v>
@@ -16348,22 +16375,22 @@
     </row>
     <row r="548" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A548" s="41" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="B548" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C548" s="14" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="D548" s="15" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="E548" s="15" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
       <c r="F548" s="15" t="s">
-        <v>400</v>
+        <v>403</v>
       </c>
       <c r="G548" s="16" t="s">
         <v>58</v>
@@ -16492,22 +16519,22 @@
     </row>
     <row r="554" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A554" s="41" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="B554" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C554" s="27" t="s">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="D554" s="28" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
       <c r="E554" s="28" t="s">
-        <v>403</v>
+        <v>406</v>
       </c>
       <c r="F554" s="28" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="G554" s="16" t="s">
         <v>58</v>
@@ -16636,22 +16663,22 @@
     </row>
     <row r="560" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A560" s="41" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="B560" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C560" s="14" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
       <c r="D560" s="15" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="E560" s="15" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="F560" s="15" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
       <c r="G560" s="16" t="s">
         <v>58</v>
@@ -16780,22 +16807,22 @@
     </row>
     <row r="566" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A566" s="41" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="B566" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C566" s="27" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
       <c r="D566" s="28" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="E566" s="28" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
       <c r="F566" s="28" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
       <c r="G566" s="16" t="s">
         <v>58</v>
@@ -16924,22 +16951,22 @@
     </row>
     <row r="572" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A572" s="41" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="B572" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C572" s="14" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="D572" s="15" t="s">
-        <v>414</v>
+        <v>417</v>
       </c>
       <c r="E572" s="15" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
       <c r="F572" s="15" t="s">
-        <v>416</v>
+        <v>419</v>
       </c>
       <c r="G572" s="16" t="s">
         <v>58</v>
@@ -17068,22 +17095,22 @@
     </row>
     <row r="578" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A578" s="41" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="B578" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C578" s="27" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="D578" s="28" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
       <c r="E578" s="28" t="s">
-        <v>419</v>
+        <v>422</v>
       </c>
       <c r="F578" s="28" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
       <c r="G578" s="16" t="s">
         <v>58</v>
@@ -17212,22 +17239,22 @@
     </row>
     <row r="584" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A584" s="41" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="B584" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C584" s="14" t="s">
-        <v>421</v>
+        <v>424</v>
       </c>
       <c r="D584" s="15" t="s">
-        <v>422</v>
+        <v>425</v>
       </c>
       <c r="E584" s="15" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="F584" s="15" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="G584" s="16" t="s">
         <v>58</v>
@@ -17356,22 +17383,22 @@
     </row>
     <row r="590" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A590" s="41" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="B590" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C590" s="27" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
       <c r="D590" s="28" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="E590" s="28" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="F590" s="28" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="G590" s="16" t="s">
         <v>58</v>
@@ -17500,22 +17527,22 @@
     </row>
     <row r="596" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A596" s="42" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="B596" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C596" s="14" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="D596" s="15" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="E596" s="15" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="F596" s="15" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
       <c r="G596" s="16" t="s">
         <v>58</v>
@@ -18040,22 +18067,22 @@
     </row>
     <row r="620" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A620" s="42" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="B620" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C620" s="27" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="D620" s="28" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="E620" s="28" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
       <c r="F620" s="28" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="G620" s="16" t="s">
         <v>58</v>
@@ -18184,22 +18211,22 @@
     </row>
     <row r="626" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A626" s="42" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="B626" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C626" s="14" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="D626" s="15" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
       <c r="E626" s="15" t="s">
-        <v>440</v>
+        <v>443</v>
       </c>
       <c r="F626" s="15" t="s">
-        <v>441</v>
+        <v>444</v>
       </c>
       <c r="G626" s="16" t="s">
         <v>58</v>
@@ -18328,22 +18355,22 @@
     </row>
     <row r="632" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A632" s="42" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="B632" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C632" s="27" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="D632" s="28" t="s">
-        <v>443</v>
+        <v>446</v>
       </c>
       <c r="E632" s="28" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
       <c r="F632" s="28" t="s">
-        <v>445</v>
+        <v>448</v>
       </c>
       <c r="G632" s="16" t="s">
         <v>58</v>
@@ -18472,22 +18499,22 @@
     </row>
     <row r="638" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A638" s="42" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="B638" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C638" s="14" t="s">
-        <v>446</v>
+        <v>449</v>
       </c>
       <c r="D638" s="15" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="E638" s="15" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="F638" s="15" t="s">
-        <v>449</v>
+        <v>452</v>
       </c>
       <c r="G638" s="16" t="s">
         <v>58</v>
@@ -18616,22 +18643,22 @@
     </row>
     <row r="644" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A644" s="43" t="s">
-        <v>450</v>
+        <v>453</v>
       </c>
       <c r="B644" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C644" s="27" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="D644" s="28" t="s">
-        <v>452</v>
+        <v>455</v>
       </c>
       <c r="E644" s="28" t="s">
-        <v>453</v>
+        <v>456</v>
       </c>
       <c r="F644" s="28" t="s">
-        <v>454</v>
+        <v>457</v>
       </c>
       <c r="G644" s="16" t="s">
         <v>58</v>
@@ -19156,22 +19183,22 @@
     </row>
     <row r="668" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A668" s="43" t="s">
-        <v>450</v>
+        <v>453</v>
       </c>
       <c r="B668" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C668" s="14" t="s">
-        <v>455</v>
+        <v>458</v>
       </c>
       <c r="D668" s="15" t="s">
-        <v>456</v>
+        <v>459</v>
       </c>
       <c r="E668" s="15" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="F668" s="15" t="s">
-        <v>458</v>
+        <v>461</v>
       </c>
       <c r="G668" s="16" t="s">
         <v>58</v>
@@ -19300,22 +19327,22 @@
     </row>
     <row r="674" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A674" s="43" t="s">
-        <v>450</v>
+        <v>453</v>
       </c>
       <c r="B674" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C674" s="27" t="s">
-        <v>459</v>
+        <v>462</v>
       </c>
       <c r="D674" s="28" t="s">
-        <v>460</v>
+        <v>463</v>
       </c>
       <c r="E674" s="28" t="s">
-        <v>461</v>
+        <v>464</v>
       </c>
       <c r="F674" s="28" t="s">
-        <v>462</v>
+        <v>465</v>
       </c>
       <c r="G674" s="16" t="s">
         <v>58</v>
@@ -19444,22 +19471,22 @@
     </row>
     <row r="680" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A680" s="43" t="s">
-        <v>450</v>
+        <v>453</v>
       </c>
       <c r="B680" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C680" s="14" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="D680" s="15" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="E680" s="15" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
       <c r="F680" s="15" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="G680" s="16" t="s">
         <v>58</v>
@@ -19588,22 +19615,22 @@
     </row>
     <row r="686" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A686" s="43" t="s">
-        <v>450</v>
+        <v>453</v>
       </c>
       <c r="B686" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C686" s="27" t="s">
-        <v>466</v>
+        <v>469</v>
       </c>
       <c r="D686" s="28" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="E686" s="28" t="s">
-        <v>468</v>
+        <v>471</v>
       </c>
       <c r="F686" s="28" t="s">
-        <v>469</v>
+        <v>472</v>
       </c>
       <c r="G686" s="16" t="s">
         <v>58</v>
@@ -19732,22 +19759,22 @@
     </row>
     <row r="692" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A692" s="44" t="s">
-        <v>470</v>
+        <v>473</v>
       </c>
       <c r="B692" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C692" s="14" t="s">
-        <v>471</v>
+        <v>474</v>
       </c>
       <c r="D692" s="15" t="s">
-        <v>472</v>
+        <v>475</v>
       </c>
       <c r="E692" s="15" t="s">
-        <v>473</v>
+        <v>476</v>
       </c>
       <c r="F692" s="15" t="s">
-        <v>474</v>
+        <v>477</v>
       </c>
       <c r="G692" s="16" t="s">
         <v>58</v>
@@ -20272,22 +20299,22 @@
     </row>
     <row r="716" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A716" s="44" t="s">
-        <v>470</v>
+        <v>473</v>
       </c>
       <c r="B716" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C716" s="27" t="s">
-        <v>475</v>
+        <v>478</v>
       </c>
       <c r="D716" s="28" t="s">
-        <v>476</v>
+        <v>479</v>
       </c>
       <c r="E716" s="28" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="F716" s="28" t="s">
-        <v>478</v>
+        <v>481</v>
       </c>
       <c r="G716" s="16" t="s">
         <v>58</v>
@@ -20416,22 +20443,22 @@
     </row>
     <row r="722" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A722" s="44" t="s">
-        <v>470</v>
+        <v>473</v>
       </c>
       <c r="B722" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C722" s="14" t="s">
-        <v>479</v>
+        <v>482</v>
       </c>
       <c r="D722" s="15" t="s">
-        <v>480</v>
+        <v>483</v>
       </c>
       <c r="E722" s="15" t="s">
-        <v>481</v>
+        <v>484</v>
       </c>
       <c r="F722" s="15" t="s">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="G722" s="16" t="s">
         <v>58</v>
@@ -20560,19 +20587,19 @@
     </row>
     <row r="728" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A728" s="44" t="s">
-        <v>470</v>
+        <v>473</v>
       </c>
       <c r="B728" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C728" s="27" t="s">
-        <v>483</v>
+        <v>486</v>
       </c>
       <c r="D728" s="28" t="s">
         <v>216</v>
       </c>
       <c r="E728" s="28" t="s">
-        <v>481</v>
+        <v>484</v>
       </c>
       <c r="F728" s="28" t="s">
         <v>218</v>
@@ -20704,22 +20731,22 @@
     </row>
     <row r="734" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A734" s="45" t="s">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="B734" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C734" s="14" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="D734" s="15" t="s">
-        <v>486</v>
+        <v>489</v>
       </c>
       <c r="E734" s="15" t="s">
-        <v>487</v>
+        <v>490</v>
       </c>
       <c r="F734" s="15" t="s">
-        <v>488</v>
+        <v>491</v>
       </c>
       <c r="G734" s="16" t="s">
         <v>58</v>
@@ -20848,22 +20875,22 @@
     </row>
     <row r="740" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A740" s="45" t="s">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="B740" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C740" s="27" t="s">
-        <v>489</v>
+        <v>492</v>
       </c>
       <c r="D740" s="28" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="E740" s="28" t="s">
-        <v>491</v>
+        <v>494</v>
       </c>
       <c r="F740" s="28" t="s">
-        <v>492</v>
+        <v>495</v>
       </c>
       <c r="G740" s="16" t="s">
         <v>58</v>
@@ -20992,22 +21019,22 @@
     </row>
     <row r="746" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A746" s="45" t="s">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="B746" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C746" s="14" t="s">
-        <v>493</v>
+        <v>496</v>
       </c>
       <c r="D746" s="15" t="s">
-        <v>494</v>
+        <v>497</v>
       </c>
       <c r="E746" s="15" t="s">
-        <v>495</v>
+        <v>498</v>
       </c>
       <c r="F746" s="15" t="s">
-        <v>496</v>
+        <v>499</v>
       </c>
       <c r="G746" s="16" t="s">
         <v>58</v>
@@ -21136,22 +21163,22 @@
     </row>
     <row r="752" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A752" s="45" t="s">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="B752" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C752" s="27" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="D752" s="28" t="s">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="E752" s="28" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
       <c r="F752" s="28" t="s">
-        <v>500</v>
+        <v>503</v>
       </c>
       <c r="G752" s="16" t="s">
         <v>58</v>
@@ -21280,22 +21307,22 @@
     </row>
     <row r="758" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A758" s="45" t="s">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="B758" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C758" s="14" t="s">
-        <v>501</v>
+        <v>504</v>
       </c>
       <c r="D758" s="15" t="s">
-        <v>502</v>
+        <v>505</v>
       </c>
       <c r="E758" s="15" t="s">
-        <v>503</v>
+        <v>506</v>
       </c>
       <c r="F758" s="15" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
       <c r="G758" s="16" t="s">
         <v>58</v>
@@ -21424,22 +21451,22 @@
     </row>
     <row r="764" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A764" s="46" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="B764" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C764" s="27" t="s">
-        <v>506</v>
+        <v>509</v>
       </c>
       <c r="D764" s="28" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="E764" s="28" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="F764" s="28" t="s">
-        <v>509</v>
+        <v>512</v>
       </c>
       <c r="G764" s="16" t="s">
         <v>58</v>
@@ -21568,22 +21595,22 @@
     </row>
     <row r="770" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A770" s="46" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="B770" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C770" s="14" t="s">
-        <v>510</v>
+        <v>513</v>
       </c>
       <c r="D770" s="15" t="s">
-        <v>511</v>
+        <v>514</v>
       </c>
       <c r="E770" s="15" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
       <c r="F770" s="15" t="s">
-        <v>513</v>
+        <v>516</v>
       </c>
       <c r="G770" s="16" t="s">
         <v>58</v>
@@ -21712,22 +21739,22 @@
     </row>
     <row r="776" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A776" s="46" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="B776" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C776" s="27" t="s">
-        <v>514</v>
+        <v>517</v>
       </c>
       <c r="D776" s="28" t="s">
-        <v>515</v>
+        <v>518</v>
       </c>
       <c r="E776" s="28" t="s">
-        <v>516</v>
+        <v>519</v>
       </c>
       <c r="F776" s="28" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
       <c r="G776" s="16" t="s">
         <v>58</v>
@@ -21856,22 +21883,22 @@
     </row>
     <row r="782" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A782" s="46" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="B782" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C782" s="14" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="D782" s="15" t="s">
-        <v>519</v>
+        <v>522</v>
       </c>
       <c r="E782" s="15" t="s">
-        <v>520</v>
+        <v>523</v>
       </c>
       <c r="F782" s="15" t="s">
-        <v>521</v>
+        <v>524</v>
       </c>
       <c r="G782" s="16" t="s">
         <v>58</v>
@@ -22000,22 +22027,22 @@
     </row>
     <row r="788" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A788" s="46" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="B788" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C788" s="27" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="D788" s="28" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="E788" s="28" t="s">
-        <v>524</v>
+        <v>527</v>
       </c>
       <c r="F788" s="28" t="s">
-        <v>525</v>
+        <v>528</v>
       </c>
       <c r="G788" s="16" t="s">
         <v>58</v>
@@ -22144,22 +22171,22 @@
     </row>
     <row r="794" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A794" s="46" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="B794" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C794" s="14" t="s">
-        <v>526</v>
+        <v>529</v>
       </c>
       <c r="D794" s="15" t="s">
-        <v>527</v>
+        <v>530</v>
       </c>
       <c r="E794" s="15" t="s">
+        <v>531</v>
+      </c>
+      <c r="F794" s="15" t="s">
         <v>528</v>
-      </c>
-      <c r="F794" s="15" t="s">
-        <v>525</v>
       </c>
       <c r="G794" s="16" t="s">
         <v>58</v>
@@ -22288,22 +22315,22 @@
     </row>
     <row r="800" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A800" s="46" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="B800" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C800" s="27" t="s">
-        <v>529</v>
+        <v>532</v>
       </c>
       <c r="D800" s="28" t="s">
-        <v>530</v>
+        <v>533</v>
       </c>
       <c r="E800" s="28" t="s">
-        <v>531</v>
+        <v>534</v>
       </c>
       <c r="F800" s="28" t="s">
-        <v>532</v>
+        <v>535</v>
       </c>
       <c r="G800" s="16" t="s">
         <v>58</v>
@@ -22432,22 +22459,22 @@
     </row>
     <row r="806" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A806" s="46" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="B806" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C806" s="14" t="s">
-        <v>533</v>
+        <v>536</v>
       </c>
       <c r="D806" s="15" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="E806" s="15" t="s">
-        <v>535</v>
+        <v>538</v>
       </c>
       <c r="F806" s="15" t="s">
-        <v>536</v>
+        <v>539</v>
       </c>
       <c r="G806" s="16" t="s">
         <v>58</v>
@@ -22576,22 +22603,22 @@
     </row>
     <row r="812" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A812" s="46" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="B812" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C812" s="27" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
       <c r="D812" s="28" t="s">
-        <v>538</v>
+        <v>541</v>
       </c>
       <c r="E812" s="28" t="s">
-        <v>539</v>
+        <v>542</v>
       </c>
       <c r="F812" s="28" t="s">
-        <v>540</v>
+        <v>543</v>
       </c>
       <c r="G812" s="16" t="s">
         <v>58</v>
@@ -22720,22 +22747,22 @@
     </row>
     <row r="818" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A818" s="46" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="B818" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C818" s="14" t="s">
-        <v>541</v>
+        <v>544</v>
       </c>
       <c r="D818" s="15" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
       <c r="E818" s="15" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="F818" s="15" t="s">
-        <v>544</v>
+        <v>547</v>
       </c>
       <c r="G818" s="16" t="s">
         <v>58</v>
@@ -22864,22 +22891,22 @@
     </row>
     <row r="824" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A824" s="46" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="B824" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C824" s="27" t="s">
-        <v>545</v>
+        <v>548</v>
       </c>
       <c r="D824" s="28" t="s">
-        <v>546</v>
+        <v>549</v>
       </c>
       <c r="E824" s="28" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
       <c r="F824" s="28" t="s">
-        <v>548</v>
+        <v>551</v>
       </c>
       <c r="G824" s="16" t="s">
         <v>58</v>
@@ -23008,22 +23035,22 @@
     </row>
     <row r="830" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A830" s="46" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="B830" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C830" s="14" t="s">
-        <v>549</v>
+        <v>552</v>
       </c>
       <c r="D830" s="15" t="s">
-        <v>550</v>
+        <v>553</v>
       </c>
       <c r="E830" s="15" t="s">
-        <v>551</v>
+        <v>554</v>
       </c>
       <c r="F830" s="15" t="s">
-        <v>552</v>
+        <v>555</v>
       </c>
       <c r="G830" s="16" t="s">
         <v>58</v>
@@ -23152,22 +23179,22 @@
     </row>
     <row r="836" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A836" s="47" t="s">
-        <v>553</v>
+        <v>556</v>
       </c>
       <c r="B836" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C836" s="27" t="s">
-        <v>554</v>
+        <v>557</v>
       </c>
       <c r="D836" s="28" t="s">
-        <v>555</v>
+        <v>558</v>
       </c>
       <c r="E836" s="28" t="s">
-        <v>556</v>
+        <v>559</v>
       </c>
       <c r="F836" s="28" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="G836" s="16" t="s">
         <v>58</v>
@@ -23296,22 +23323,22 @@
     </row>
     <row r="842" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A842" s="47" t="s">
-        <v>553</v>
+        <v>556</v>
       </c>
       <c r="B842" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C842" s="14" t="s">
-        <v>558</v>
+        <v>561</v>
       </c>
       <c r="D842" s="15" t="s">
-        <v>559</v>
+        <v>562</v>
       </c>
       <c r="E842" s="15" t="s">
-        <v>560</v>
+        <v>563</v>
       </c>
       <c r="F842" s="15" t="s">
-        <v>496</v>
+        <v>499</v>
       </c>
       <c r="G842" s="16" t="s">
         <v>58</v>
@@ -23440,22 +23467,22 @@
     </row>
     <row r="848" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A848" s="47" t="s">
-        <v>553</v>
+        <v>556</v>
       </c>
       <c r="B848" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C848" s="27" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
       <c r="D848" s="28" t="s">
-        <v>562</v>
+        <v>565</v>
       </c>
       <c r="E848" s="28" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="F848" s="28" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="G848" s="16" t="s">
         <v>58</v>
@@ -23584,22 +23611,22 @@
     </row>
     <row r="854" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A854" s="47" t="s">
-        <v>553</v>
+        <v>556</v>
       </c>
       <c r="B854" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C854" s="14" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="D854" s="15" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="E854" s="15" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="F854" s="15" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="G854" s="16" t="s">
         <v>58</v>
@@ -23728,22 +23755,22 @@
     </row>
     <row r="860" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A860" s="48" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="B860" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C860" s="27" t="s">
-        <v>570</v>
+        <v>573</v>
       </c>
       <c r="D860" s="28" t="s">
-        <v>571</v>
+        <v>574</v>
       </c>
       <c r="E860" s="28" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="F860" s="28" t="s">
-        <v>573</v>
+        <v>576</v>
       </c>
       <c r="G860" s="16" t="s">
         <v>58</v>
@@ -23872,22 +23899,22 @@
     </row>
     <row r="866" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A866" s="48" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="B866" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C866" s="14" t="s">
-        <v>574</v>
+        <v>577</v>
       </c>
       <c r="D866" s="15" t="s">
-        <v>575</v>
+        <v>578</v>
       </c>
       <c r="E866" s="15" t="s">
-        <v>576</v>
+        <v>579</v>
       </c>
       <c r="F866" s="15" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="G866" s="16" t="s">
         <v>58</v>
@@ -24016,22 +24043,22 @@
     </row>
     <row r="872" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A872" s="48" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="B872" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C872" s="27" t="s">
-        <v>578</v>
+        <v>581</v>
       </c>
       <c r="D872" s="28" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="E872" s="28" t="s">
-        <v>580</v>
+        <v>583</v>
       </c>
       <c r="F872" s="28" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="G872" s="16" t="s">
         <v>58</v>
@@ -24160,22 +24187,22 @@
     </row>
     <row r="878" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A878" s="48" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="B878" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C878" s="14" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="D878" s="15" t="s">
-        <v>583</v>
+        <v>586</v>
       </c>
       <c r="E878" s="15" t="s">
-        <v>584</v>
+        <v>587</v>
       </c>
       <c r="F878" s="15" t="s">
-        <v>585</v>
+        <v>588</v>
       </c>
       <c r="G878" s="16" t="s">
         <v>58</v>
@@ -24304,22 +24331,22 @@
     </row>
     <row r="884" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A884" s="48" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="B884" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C884" s="27" t="s">
-        <v>586</v>
+        <v>589</v>
       </c>
       <c r="D884" s="28" t="s">
-        <v>587</v>
+        <v>590</v>
       </c>
       <c r="E884" s="28" t="s">
-        <v>588</v>
+        <v>591</v>
       </c>
       <c r="F884" s="28" t="s">
-        <v>589</v>
+        <v>592</v>
       </c>
       <c r="G884" s="16" t="s">
         <v>58</v>
@@ -24448,22 +24475,22 @@
     </row>
     <row r="890" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A890" s="48" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="B890" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C890" s="14" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="D890" s="15" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
       <c r="E890" s="15" t="s">
-        <v>592</v>
+        <v>595</v>
       </c>
       <c r="F890" s="15" t="s">
-        <v>593</v>
+        <v>596</v>
       </c>
       <c r="G890" s="16" t="s">
         <v>58</v>
@@ -24592,22 +24619,22 @@
     </row>
     <row r="896" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A896" s="48" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="B896" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C896" s="27" t="s">
-        <v>594</v>
+        <v>597</v>
       </c>
       <c r="D896" s="28" t="s">
-        <v>595</v>
+        <v>598</v>
       </c>
       <c r="E896" s="28" t="s">
-        <v>596</v>
+        <v>599</v>
       </c>
       <c r="F896" s="28" t="s">
-        <v>597</v>
+        <v>600</v>
       </c>
       <c r="G896" s="16" t="s">
         <v>58</v>
@@ -24736,22 +24763,22 @@
     </row>
     <row r="902" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A902" s="49" t="s">
-        <v>598</v>
+        <v>601</v>
       </c>
       <c r="B902" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C902" s="14" t="s">
-        <v>599</v>
+        <v>602</v>
       </c>
       <c r="D902" s="15" t="s">
-        <v>600</v>
+        <v>603</v>
       </c>
       <c r="E902" s="15" t="s">
-        <v>601</v>
+        <v>604</v>
       </c>
       <c r="F902" s="15" t="s">
-        <v>602</v>
+        <v>605</v>
       </c>
       <c r="G902" s="16" t="s">
         <v>58</v>
@@ -24880,22 +24907,22 @@
     </row>
     <row r="908" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A908" s="49" t="s">
-        <v>598</v>
+        <v>601</v>
       </c>
       <c r="B908" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C908" s="27" t="s">
-        <v>603</v>
+        <v>606</v>
       </c>
       <c r="D908" s="28" t="s">
-        <v>604</v>
+        <v>607</v>
       </c>
       <c r="E908" s="28" t="s">
-        <v>605</v>
+        <v>608</v>
       </c>
       <c r="F908" s="28" t="s">
-        <v>606</v>
+        <v>609</v>
       </c>
       <c r="G908" s="16" t="s">
         <v>58</v>
@@ -25024,22 +25051,22 @@
     </row>
     <row r="914" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A914" s="49" t="s">
-        <v>598</v>
+        <v>601</v>
       </c>
       <c r="B914" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C914" s="14" t="s">
-        <v>607</v>
+        <v>610</v>
       </c>
       <c r="D914" s="15" t="s">
-        <v>608</v>
+        <v>611</v>
       </c>
       <c r="E914" s="15" t="s">
-        <v>609</v>
+        <v>612</v>
       </c>
       <c r="F914" s="15" t="s">
-        <v>610</v>
+        <v>613</v>
       </c>
       <c r="G914" s="16" t="s">
         <v>58</v>
@@ -25168,22 +25195,22 @@
     </row>
     <row r="920" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A920" s="49" t="s">
-        <v>598</v>
+        <v>601</v>
       </c>
       <c r="B920" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C920" s="27" t="s">
-        <v>611</v>
+        <v>614</v>
       </c>
       <c r="D920" s="28" t="s">
-        <v>612</v>
+        <v>615</v>
       </c>
       <c r="E920" s="28" t="s">
-        <v>613</v>
+        <v>616</v>
       </c>
       <c r="F920" s="28" t="s">
-        <v>614</v>
+        <v>617</v>
       </c>
       <c r="G920" s="16" t="s">
         <v>58</v>
@@ -25312,22 +25339,22 @@
     </row>
     <row r="926" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A926" s="49" t="s">
-        <v>598</v>
+        <v>601</v>
       </c>
       <c r="B926" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C926" s="14" t="s">
-        <v>615</v>
+        <v>618</v>
       </c>
       <c r="D926" s="15" t="s">
-        <v>616</v>
+        <v>619</v>
       </c>
       <c r="E926" s="15" t="s">
-        <v>617</v>
+        <v>620</v>
       </c>
       <c r="F926" s="15" t="s">
-        <v>618</v>
+        <v>621</v>
       </c>
       <c r="G926" s="16" t="s">
         <v>58</v>
@@ -25456,22 +25483,22 @@
     </row>
     <row r="932" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A932" s="49" t="s">
-        <v>598</v>
+        <v>601</v>
       </c>
       <c r="B932" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C932" s="27" t="s">
-        <v>619</v>
+        <v>622</v>
       </c>
       <c r="D932" s="28" t="s">
-        <v>620</v>
+        <v>623</v>
       </c>
       <c r="E932" s="28" t="s">
-        <v>621</v>
+        <v>624</v>
       </c>
       <c r="F932" s="28" t="s">
-        <v>622</v>
+        <v>625</v>
       </c>
       <c r="G932" s="16" t="s">
         <v>58</v>
@@ -25600,22 +25627,22 @@
     </row>
     <row r="938" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A938" s="50" t="s">
-        <v>623</v>
+        <v>626</v>
       </c>
       <c r="B938" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C938" s="14" t="s">
-        <v>624</v>
+        <v>627</v>
       </c>
       <c r="D938" s="15" t="s">
-        <v>625</v>
+        <v>628</v>
       </c>
       <c r="E938" s="15" t="s">
-        <v>626</v>
+        <v>629</v>
       </c>
       <c r="F938" s="15" t="s">
-        <v>627</v>
+        <v>630</v>
       </c>
       <c r="G938" s="16" t="s">
         <v>58</v>
@@ -25744,22 +25771,22 @@
     </row>
     <row r="944" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A944" s="50" t="s">
-        <v>623</v>
+        <v>626</v>
       </c>
       <c r="B944" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C944" s="27" t="s">
-        <v>628</v>
+        <v>631</v>
       </c>
       <c r="D944" s="28" t="s">
-        <v>629</v>
+        <v>632</v>
       </c>
       <c r="E944" s="28" t="s">
-        <v>630</v>
+        <v>633</v>
       </c>
       <c r="F944" s="28" t="s">
-        <v>631</v>
+        <v>634</v>
       </c>
       <c r="G944" s="16" t="s">
         <v>58</v>
@@ -25888,22 +25915,22 @@
     </row>
     <row r="950" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A950" s="50" t="s">
-        <v>623</v>
+        <v>626</v>
       </c>
       <c r="B950" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C950" s="14" t="s">
-        <v>632</v>
+        <v>635</v>
       </c>
       <c r="D950" s="15" t="s">
-        <v>633</v>
+        <v>636</v>
       </c>
       <c r="E950" s="15" t="s">
-        <v>634</v>
+        <v>637</v>
       </c>
       <c r="F950" s="15" t="s">
-        <v>635</v>
+        <v>638</v>
       </c>
       <c r="G950" s="16" t="s">
         <v>58</v>
@@ -26032,22 +26059,22 @@
     </row>
     <row r="956" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A956" s="50" t="s">
-        <v>623</v>
+        <v>626</v>
       </c>
       <c r="B956" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C956" s="27" t="s">
-        <v>636</v>
+        <v>639</v>
       </c>
       <c r="D956" s="28" t="s">
-        <v>637</v>
+        <v>640</v>
       </c>
       <c r="E956" s="28" t="s">
-        <v>638</v>
+        <v>641</v>
       </c>
       <c r="F956" s="28" t="s">
-        <v>610</v>
+        <v>613</v>
       </c>
       <c r="G956" s="16" t="s">
         <v>58</v>
@@ -26176,22 +26203,22 @@
     </row>
     <row r="962" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A962" s="50" t="s">
-        <v>623</v>
+        <v>626</v>
       </c>
       <c r="B962" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C962" s="14" t="s">
-        <v>639</v>
+        <v>642</v>
       </c>
       <c r="D962" s="15" t="s">
-        <v>640</v>
+        <v>643</v>
       </c>
       <c r="E962" s="15" t="s">
-        <v>641</v>
+        <v>644</v>
       </c>
       <c r="F962" s="15" t="s">
-        <v>642</v>
+        <v>645</v>
       </c>
       <c r="G962" s="16" t="s">
         <v>58</v>
@@ -26320,22 +26347,22 @@
     </row>
     <row r="968" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A968" s="50" t="s">
-        <v>623</v>
+        <v>626</v>
       </c>
       <c r="B968" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C968" s="27" t="s">
-        <v>643</v>
+        <v>646</v>
       </c>
       <c r="D968" s="28" t="s">
-        <v>644</v>
+        <v>647</v>
       </c>
       <c r="E968" s="28" t="s">
-        <v>645</v>
+        <v>648</v>
       </c>
       <c r="F968" s="28" t="s">
-        <v>646</v>
+        <v>649</v>
       </c>
       <c r="G968" s="16" t="s">
         <v>58</v>
@@ -26464,22 +26491,22 @@
     </row>
     <row r="974" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A974" s="51" t="s">
-        <v>647</v>
+        <v>650</v>
       </c>
       <c r="B974" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C974" s="14" t="s">
-        <v>648</v>
+        <v>651</v>
       </c>
       <c r="D974" s="15" t="s">
-        <v>649</v>
+        <v>652</v>
       </c>
       <c r="E974" s="15" t="s">
-        <v>650</v>
+        <v>653</v>
       </c>
       <c r="F974" s="15" t="s">
-        <v>651</v>
+        <v>654</v>
       </c>
       <c r="G974" s="16" t="s">
         <v>58</v>
@@ -26608,22 +26635,22 @@
     </row>
     <row r="980" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A980" s="51" t="s">
-        <v>647</v>
+        <v>650</v>
       </c>
       <c r="B980" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C980" s="27" t="s">
-        <v>652</v>
+        <v>655</v>
       </c>
       <c r="D980" s="28" t="s">
-        <v>653</v>
+        <v>656</v>
       </c>
       <c r="E980" s="28" t="s">
-        <v>654</v>
+        <v>657</v>
       </c>
       <c r="F980" s="28" t="s">
-        <v>655</v>
+        <v>658</v>
       </c>
       <c r="G980" s="16" t="s">
         <v>58</v>
@@ -26752,22 +26779,22 @@
     </row>
     <row r="986" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A986" s="51" t="s">
-        <v>647</v>
+        <v>650</v>
       </c>
       <c r="B986" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C986" s="14" t="s">
-        <v>656</v>
+        <v>659</v>
       </c>
       <c r="D986" s="15" t="s">
-        <v>657</v>
+        <v>660</v>
       </c>
       <c r="E986" s="15" t="s">
-        <v>658</v>
+        <v>661</v>
       </c>
       <c r="F986" s="15" t="s">
-        <v>659</v>
+        <v>662</v>
       </c>
       <c r="G986" s="16" t="s">
         <v>58</v>
@@ -26896,22 +26923,22 @@
     </row>
     <row r="992" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A992" s="51" t="s">
-        <v>647</v>
+        <v>650</v>
       </c>
       <c r="B992" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C992" s="27" t="s">
-        <v>660</v>
+        <v>663</v>
       </c>
       <c r="D992" s="28" t="s">
-        <v>661</v>
+        <v>664</v>
       </c>
       <c r="E992" s="28" t="s">
-        <v>662</v>
+        <v>665</v>
       </c>
       <c r="F992" s="28" t="s">
-        <v>663</v>
+        <v>666</v>
       </c>
       <c r="G992" s="16" t="s">
         <v>58</v>
@@ -27040,22 +27067,22 @@
     </row>
     <row r="998" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A998" s="51" t="s">
-        <v>647</v>
+        <v>650</v>
       </c>
       <c r="B998" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C998" s="14" t="s">
-        <v>664</v>
+        <v>667</v>
       </c>
       <c r="D998" s="15" t="s">
-        <v>665</v>
+        <v>668</v>
       </c>
       <c r="E998" s="15" t="s">
-        <v>666</v>
+        <v>669</v>
       </c>
       <c r="F998" s="15" t="s">
-        <v>667</v>
+        <v>670</v>
       </c>
       <c r="G998" s="16" t="s">
         <v>58</v>
@@ -27184,22 +27211,22 @@
     </row>
     <row r="1004" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1004" s="52" t="s">
-        <v>668</v>
+        <v>671</v>
       </c>
       <c r="B1004" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1004" s="27" t="s">
-        <v>669</v>
+        <v>672</v>
       </c>
       <c r="D1004" s="28" t="s">
-        <v>670</v>
+        <v>673</v>
       </c>
       <c r="E1004" s="28" t="s">
-        <v>671</v>
+        <v>674</v>
       </c>
       <c r="F1004" s="28" t="s">
-        <v>672</v>
+        <v>675</v>
       </c>
       <c r="G1004" s="16" t="s">
         <v>58</v>
@@ -27328,22 +27355,22 @@
     </row>
     <row r="1010" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1010" s="52" t="s">
-        <v>668</v>
+        <v>671</v>
       </c>
       <c r="B1010" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1010" s="14" t="s">
-        <v>673</v>
+        <v>676</v>
       </c>
       <c r="D1010" s="15" t="s">
-        <v>674</v>
+        <v>677</v>
       </c>
       <c r="E1010" s="15" t="s">
-        <v>675</v>
+        <v>678</v>
       </c>
       <c r="F1010" s="15" t="s">
-        <v>676</v>
+        <v>679</v>
       </c>
       <c r="G1010" s="16" t="s">
         <v>58</v>
@@ -27472,22 +27499,22 @@
     </row>
     <row r="1016" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1016" s="52" t="s">
-        <v>668</v>
+        <v>671</v>
       </c>
       <c r="B1016" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1016" s="27" t="s">
-        <v>677</v>
+        <v>680</v>
       </c>
       <c r="D1016" s="28" t="s">
-        <v>678</v>
+        <v>681</v>
       </c>
       <c r="E1016" s="28" t="s">
-        <v>679</v>
+        <v>682</v>
       </c>
       <c r="F1016" s="28" t="s">
-        <v>680</v>
+        <v>683</v>
       </c>
       <c r="G1016" s="16" t="s">
         <v>58</v>
@@ -27616,22 +27643,22 @@
     </row>
     <row r="1022" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1022" s="52" t="s">
-        <v>668</v>
+        <v>671</v>
       </c>
       <c r="B1022" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1022" s="14" t="s">
-        <v>681</v>
+        <v>684</v>
       </c>
       <c r="D1022" s="15" t="s">
-        <v>682</v>
+        <v>685</v>
       </c>
       <c r="E1022" s="15" t="s">
-        <v>683</v>
+        <v>686</v>
       </c>
       <c r="F1022" s="15" t="s">
-        <v>684</v>
+        <v>687</v>
       </c>
       <c r="G1022" s="16" t="s">
         <v>58</v>
@@ -27760,22 +27787,22 @@
     </row>
     <row r="1028" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1028" s="52" t="s">
-        <v>668</v>
+        <v>671</v>
       </c>
       <c r="B1028" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C1028" s="27" t="s">
-        <v>685</v>
+        <v>688</v>
       </c>
       <c r="D1028" s="28" t="s">
-        <v>686</v>
+        <v>689</v>
       </c>
       <c r="E1028" s="28" t="s">
-        <v>687</v>
+        <v>690</v>
       </c>
       <c r="F1028" s="28" t="s">
-        <v>688</v>
+        <v>691</v>
       </c>
       <c r="G1028" s="16" t="s">
         <v>58</v>
@@ -27904,22 +27931,22 @@
     </row>
     <row r="1034" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1034" s="52" t="s">
-        <v>668</v>
+        <v>671</v>
       </c>
       <c r="B1034" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C1034" s="14" t="s">
-        <v>689</v>
+        <v>692</v>
       </c>
       <c r="D1034" s="15" t="s">
-        <v>690</v>
+        <v>693</v>
       </c>
       <c r="E1034" s="15" t="s">
-        <v>691</v>
+        <v>694</v>
       </c>
       <c r="F1034" s="15" t="s">
-        <v>692</v>
+        <v>695</v>
       </c>
       <c r="G1034" s="16" t="s">
         <v>58</v>
@@ -28048,22 +28075,22 @@
     </row>
     <row r="1040" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1040" s="53" t="s">
-        <v>693</v>
+        <v>696</v>
       </c>
       <c r="B1040" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C1040" s="27" t="s">
-        <v>694</v>
+        <v>697</v>
       </c>
       <c r="D1040" s="28" t="s">
-        <v>682</v>
+        <v>685</v>
       </c>
       <c r="E1040" s="28" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="F1040" s="28" t="s">
-        <v>696</v>
+        <v>699</v>
       </c>
       <c r="G1040" s="16" t="s">
         <v>58</v>
@@ -28192,22 +28219,22 @@
     </row>
     <row r="1046" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1046" s="53" t="s">
-        <v>693</v>
+        <v>696</v>
       </c>
       <c r="B1046" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1046" s="14" t="s">
-        <v>697</v>
+        <v>700</v>
       </c>
       <c r="D1046" s="15" t="s">
-        <v>674</v>
+        <v>677</v>
       </c>
       <c r="E1046" s="15" t="s">
-        <v>698</v>
+        <v>701</v>
       </c>
       <c r="F1046" s="15" t="s">
-        <v>699</v>
+        <v>702</v>
       </c>
       <c r="G1046" s="16" t="s">
         <v>58</v>
@@ -28342,16 +28369,16 @@
         <v>53</v>
       </c>
       <c r="C1052" s="27" t="s">
-        <v>700</v>
+        <v>703</v>
       </c>
       <c r="D1052" s="28" t="s">
-        <v>701</v>
+        <v>704</v>
       </c>
       <c r="E1052" s="28" t="s">
-        <v>702</v>
+        <v>705</v>
       </c>
       <c r="F1052" s="28" t="s">
-        <v>703</v>
+        <v>706</v>
       </c>
       <c r="G1052" s="16" t="s">
         <v>58</v>
@@ -28486,16 +28513,16 @@
         <v>53</v>
       </c>
       <c r="C1058" s="14" t="s">
-        <v>704</v>
+        <v>707</v>
       </c>
       <c r="D1058" s="15" t="s">
-        <v>705</v>
+        <v>708</v>
       </c>
       <c r="E1058" s="15" t="s">
-        <v>706</v>
+        <v>709</v>
       </c>
       <c r="F1058" s="15" t="s">
-        <v>707</v>
+        <v>710</v>
       </c>
       <c r="G1058" s="16" t="s">
         <v>58</v>
@@ -29585,10 +29612,10 @@
         <v>39</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>708</v>
+        <v>711</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>709</v>
+        <v>712</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>53</v>
@@ -29606,7 +29633,7 @@
         <v>87</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>710</v>
+        <v>713</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -29756,7 +29783,7 @@
     </row>
     <row r="7" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="59" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B7" s="1">
         <v>17</v>
@@ -29785,7 +29812,7 @@
     </row>
     <row r="8" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="60" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B8" s="1">
         <v>10</v>
@@ -29814,7 +29841,7 @@
     </row>
     <row r="9" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="61" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="B9" s="1">
         <v>11</v>
@@ -29843,7 +29870,7 @@
     </row>
     <row r="10" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="62" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="B10" s="1">
         <v>9</v>
@@ -29872,7 +29899,7 @@
     </row>
     <row r="11" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="63" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="B11" s="1">
         <v>5</v>
@@ -29901,7 +29928,7 @@
     </row>
     <row r="12" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="64" t="s">
-        <v>450</v>
+        <v>453</v>
       </c>
       <c r="B12" s="1">
         <v>5</v>
@@ -29930,7 +29957,7 @@
     </row>
     <row r="13" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="65" t="s">
-        <v>470</v>
+        <v>473</v>
       </c>
       <c r="B13" s="1">
         <v>4</v>
@@ -29959,7 +29986,7 @@
     </row>
     <row r="14" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="66" t="s">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="B14" s="1">
         <v>5</v>
@@ -29988,7 +30015,7 @@
     </row>
     <row r="15" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="67" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="B15" s="1">
         <v>12</v>
@@ -30017,7 +30044,7 @@
     </row>
     <row r="16" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="68" t="s">
-        <v>553</v>
+        <v>556</v>
       </c>
       <c r="B16" s="1">
         <v>4</v>
@@ -30046,7 +30073,7 @@
     </row>
     <row r="17" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="69" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="B17" s="1">
         <v>7</v>
@@ -30075,7 +30102,7 @@
     </row>
     <row r="18" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="70" t="s">
-        <v>598</v>
+        <v>601</v>
       </c>
       <c r="B18" s="1">
         <v>6</v>
@@ -30104,7 +30131,7 @@
     </row>
     <row r="19" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="71" t="s">
-        <v>623</v>
+        <v>626</v>
       </c>
       <c r="B19" s="1">
         <v>6</v>
@@ -30133,7 +30160,7 @@
     </row>
     <row r="20" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="72" t="s">
-        <v>647</v>
+        <v>650</v>
       </c>
       <c r="B20" s="1">
         <v>5</v>
@@ -30162,7 +30189,7 @@
     </row>
     <row r="21" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="73" t="s">
-        <v>668</v>
+        <v>671</v>
       </c>
       <c r="B21" s="1">
         <v>6</v>
@@ -30191,7 +30218,7 @@
     </row>
     <row r="22" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="74" t="s">
-        <v>693</v>
+        <v>696</v>
       </c>
       <c r="B22" s="1">
         <v>2</v>
@@ -30220,7 +30247,7 @@
     </row>
     <row r="23" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="75" t="s">
-        <v>711</v>
+        <v>714</v>
       </c>
       <c r="B23" s="75">
         <v>153</v>
@@ -30271,7 +30298,7 @@
         <v>44</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>709</v>
+        <v>712</v>
       </c>
       <c r="C1" s="10" t="s">
         <v>71</v>
@@ -30280,7 +30307,7 @@
         <v>87</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>710</v>
+        <v>713</v>
       </c>
       <c r="F1" s="10" t="s">
         <v>95</v>
@@ -30431,10 +30458,10 @@
         <v>45</v>
       </c>
       <c r="B1" s="10" t="s">
+        <v>715</v>
+      </c>
+      <c r="C1" s="10" t="s">
         <v>712</v>
-      </c>
-      <c r="C1" s="10" t="s">
-        <v>709</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>71</v>
@@ -30443,7 +30470,7 @@
         <v>87</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>710</v>
+        <v>713</v>
       </c>
       <c r="G1" s="10" t="s">
         <v>95</v>
@@ -30454,7 +30481,7 @@
         <v>59</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>713</v>
+        <v>716</v>
       </c>
       <c r="C2" s="1">
         <v>18</v>

</xml_diff>

<commit_message>
075 => fase IV => ZUP-038 OK (Chrome/USER) i fix combo Ciutat que no tancava (ZUP-040)
</commit_message>
<xml_diff>
--- a/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
+++ b/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4284" uniqueCount="717">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4291" uniqueCount="720">
   <si>
     <t>Zuppeto — Joc de probes manual (totes les pantalles)</t>
   </si>
@@ -761,6 +761,9 @@
     <t>Heading «Descobreix… llocs pet-friendly», filtres i mapa visibles</t>
   </si>
   <si>
+    <t>Càrrega OK. Incidència combo Ciutat (no tancava) → veure ZUP-040.</t>
+  </si>
+  <si>
     <t>ZUP-039</t>
   </si>
   <si>
@@ -783,6 +786,12 @@
   </si>
   <si>
     <t>Llista i mapa es filtren per ciutat</t>
+  </si>
+  <si>
+    <t>El combo de Ciutat (app-city-combobox) no es tancava en clicar fora de la pantalla; Tipus/Mascota (select natiu) sí. Detectat durant ZUP-038.</t>
+  </si>
+  <si>
+    <t>Què s'ha fet: Tancar el panell amb document:click (fora del host) i Escape, com el menú de capçalera. El blur sol no basta perquè un clic en elements no focusables (mapa, etc.) no treu el focus de l'input. Fitxer: city-combobox.component.ts. Pendent retest.</t>
   </si>
   <si>
     <t>ZUP-041</t>
@@ -10112,11 +10121,15 @@
       <c r="H284" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="I284" s="29"/>
+      <c r="I284" s="29" t="s">
+        <v>210</v>
+      </c>
       <c r="J284" s="17" t="s">
-        <v>60</v>
-      </c>
-      <c r="K284" s="15"/>
+        <v>71</v>
+      </c>
+      <c r="K284" s="15" t="s">
+        <v>245</v>
+      </c>
       <c r="L284" s="1"/>
       <c r="M284" s="1"/>
       <c r="N284" s="1"/>
@@ -10503,16 +10516,16 @@
         <v>53</v>
       </c>
       <c r="C302" s="14" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="D302" s="15" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="E302" s="15" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="F302" s="15" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="G302" s="16" t="s">
         <v>58</v>
@@ -10647,16 +10660,16 @@
         <v>53</v>
       </c>
       <c r="C308" s="27" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D308" s="28" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="E308" s="28" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="F308" s="28" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="G308" s="16" t="s">
         <v>58</v>
@@ -10664,14 +10677,24 @@
       <c r="H308" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="I308" s="29"/>
+      <c r="I308" s="29" t="s">
+        <v>210</v>
+      </c>
       <c r="J308" s="17" t="s">
-        <v>60</v>
-      </c>
-      <c r="K308" s="15"/>
-      <c r="L308" s="1"/>
-      <c r="M308" s="1"/>
-      <c r="N308" s="1"/>
+        <v>87</v>
+      </c>
+      <c r="K308" s="15" t="s">
+        <v>254</v>
+      </c>
+      <c r="L308" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="M308" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="N308" s="1" t="s">
+        <v>255</v>
+      </c>
     </row>
     <row r="309" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A309" s="38"/>
@@ -10791,16 +10814,16 @@
         <v>53</v>
       </c>
       <c r="C314" s="14" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="D314" s="15" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="E314" s="15" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="F314" s="15" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="G314" s="16" t="s">
         <v>58</v>
@@ -10935,16 +10958,16 @@
         <v>53</v>
       </c>
       <c r="C320" s="27" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="D320" s="28" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="E320" s="28" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="F320" s="28" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="G320" s="16" t="s">
         <v>58</v>
@@ -11079,16 +11102,16 @@
         <v>53</v>
       </c>
       <c r="C326" s="14" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="D326" s="15" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="E326" s="15" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="F326" s="15" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="G326" s="16" t="s">
         <v>58</v>
@@ -11223,16 +11246,16 @@
         <v>53</v>
       </c>
       <c r="C332" s="27" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="D332" s="28" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="E332" s="28" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="F332" s="28" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="G332" s="16" t="s">
         <v>58</v>
@@ -11367,16 +11390,16 @@
         <v>53</v>
       </c>
       <c r="C338" s="14" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="D338" s="15" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="E338" s="15" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="F338" s="15" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="G338" s="16" t="s">
         <v>58</v>
@@ -11511,16 +11534,16 @@
         <v>53</v>
       </c>
       <c r="C344" s="27" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="D344" s="28" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="E344" s="28" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="F344" s="28" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="G344" s="16" t="s">
         <v>58</v>
@@ -11655,16 +11678,16 @@
         <v>53</v>
       </c>
       <c r="C350" s="14" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="D350" s="15" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="E350" s="15" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="F350" s="15" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="G350" s="16" t="s">
         <v>58</v>
@@ -11799,16 +11822,16 @@
         <v>53</v>
       </c>
       <c r="C356" s="27" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="D356" s="28" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="E356" s="28" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="F356" s="28" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="G356" s="16" t="s">
         <v>58</v>
@@ -11943,13 +11966,13 @@
         <v>90</v>
       </c>
       <c r="C362" s="14" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="D362" s="15" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="E362" s="15" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="F362" s="15" t="s">
         <v>222</v>
@@ -12087,16 +12110,16 @@
         <v>53</v>
       </c>
       <c r="C368" s="27" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="D368" s="28" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="E368" s="28" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="F368" s="28" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="G368" s="16" t="s">
         <v>58</v>
@@ -12231,16 +12254,16 @@
         <v>90</v>
       </c>
       <c r="C374" s="14" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="D374" s="15" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="E374" s="15" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="F374" s="15" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="G374" s="16" t="s">
         <v>58</v>
@@ -12375,16 +12398,16 @@
         <v>53</v>
       </c>
       <c r="C380" s="27" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="D380" s="28" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="E380" s="28" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="F380" s="28" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="G380" s="16" t="s">
         <v>58</v>
@@ -12519,16 +12542,16 @@
         <v>53</v>
       </c>
       <c r="C386" s="14" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="D386" s="15" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="E386" s="15" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="F386" s="15" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="G386" s="16" t="s">
         <v>58</v>
@@ -12663,16 +12686,16 @@
         <v>90</v>
       </c>
       <c r="C392" s="27" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="D392" s="28" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="E392" s="28" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="F392" s="28" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="G392" s="16" t="s">
         <v>58</v>
@@ -12801,22 +12824,22 @@
     </row>
     <row r="398" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A398" s="39" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="B398" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C398" s="14" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="D398" s="15" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="E398" s="15" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="F398" s="15" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="G398" s="16" t="s">
         <v>58</v>
@@ -13341,22 +13364,22 @@
     </row>
     <row r="422" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A422" s="39" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="B422" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C422" s="27" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="D422" s="28" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="E422" s="28" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="F422" s="28" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="G422" s="16" t="s">
         <v>58</v>
@@ -13485,22 +13508,22 @@
     </row>
     <row r="428" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A428" s="39" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="B428" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C428" s="14" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="D428" s="15" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="E428" s="15" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="F428" s="15" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="G428" s="16" t="s">
         <v>58</v>
@@ -13629,22 +13652,22 @@
     </row>
     <row r="434" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A434" s="39" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="B434" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C434" s="27" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="D434" s="28" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="E434" s="28" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="F434" s="28" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="G434" s="16" t="s">
         <v>58</v>
@@ -13773,22 +13796,22 @@
     </row>
     <row r="440" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A440" s="39" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="B440" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C440" s="14" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="D440" s="15" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="E440" s="15" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="F440" s="15" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="G440" s="16" t="s">
         <v>58</v>
@@ -13917,22 +13940,22 @@
     </row>
     <row r="446" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A446" s="39" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="B446" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C446" s="27" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="D446" s="28" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="E446" s="28" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="F446" s="28" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="G446" s="16" t="s">
         <v>58</v>
@@ -13947,7 +13970,7 @@
         <v>87</v>
       </c>
       <c r="K446" s="15" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="L446" s="1" t="s">
         <v>210</v>
@@ -13956,7 +13979,7 @@
         <v>71</v>
       </c>
       <c r="N446" s="1" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
     </row>
     <row r="447" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -14071,22 +14094,22 @@
     </row>
     <row r="452" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A452" s="39" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="B452" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C452" s="14" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="D452" s="15" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="E452" s="15" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="F452" s="15" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="G452" s="16" t="s">
         <v>58</v>
@@ -14215,22 +14238,22 @@
     </row>
     <row r="458" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A458" s="39" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="B458" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C458" s="27" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="D458" s="28" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="E458" s="28" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="F458" s="28" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="G458" s="16" t="s">
         <v>58</v>
@@ -14359,22 +14382,22 @@
     </row>
     <row r="464" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A464" s="39" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="B464" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C464" s="14" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="D464" s="15" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="E464" s="15" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="F464" s="15" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="G464" s="16" t="s">
         <v>58</v>
@@ -14503,22 +14526,22 @@
     </row>
     <row r="470" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A470" s="39" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="B470" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C470" s="27" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="D470" s="28" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="E470" s="28" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="F470" s="28" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="G470" s="16" t="s">
         <v>58</v>
@@ -14647,22 +14670,22 @@
     </row>
     <row r="476" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A476" s="40" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="B476" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C476" s="14" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="D476" s="15" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="E476" s="15" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="F476" s="15" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="G476" s="16" t="s">
         <v>58</v>
@@ -14791,22 +14814,22 @@
     </row>
     <row r="482" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A482" s="40" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="B482" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C482" s="27" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="D482" s="28" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="E482" s="28" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="F482" s="28" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="G482" s="16" t="s">
         <v>58</v>
@@ -14935,22 +14958,22 @@
     </row>
     <row r="488" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A488" s="40" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="B488" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C488" s="14" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="D488" s="15" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="E488" s="15" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="F488" s="15" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="G488" s="16" t="s">
         <v>58</v>
@@ -15079,22 +15102,22 @@
     </row>
     <row r="494" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A494" s="40" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="B494" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C494" s="27" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="D494" s="28" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="E494" s="28" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="F494" s="28" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="G494" s="16" t="s">
         <v>58</v>
@@ -15223,22 +15246,22 @@
     </row>
     <row r="500" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A500" s="40" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="B500" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C500" s="14" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="D500" s="15" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="E500" s="15" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="F500" s="15" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="G500" s="16" t="s">
         <v>58</v>
@@ -15367,22 +15390,22 @@
     </row>
     <row r="506" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A506" s="40" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="B506" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C506" s="27" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="D506" s="28" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="E506" s="28" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="F506" s="28" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="G506" s="16" t="s">
         <v>58</v>
@@ -15511,22 +15534,22 @@
     </row>
     <row r="512" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A512" s="40" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="B512" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C512" s="14" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="D512" s="15" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="E512" s="15" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="F512" s="15" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
       <c r="G512" s="16" t="s">
         <v>58</v>
@@ -15655,22 +15678,22 @@
     </row>
     <row r="518" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A518" s="40" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="B518" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C518" s="27" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="D518" s="28" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E518" s="28" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="F518" s="28" t="s">
-        <v>382</v>
+        <v>385</v>
       </c>
       <c r="G518" s="16" t="s">
         <v>58</v>
@@ -15799,22 +15822,22 @@
     </row>
     <row r="524" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A524" s="40" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="B524" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C524" s="14" t="s">
-        <v>383</v>
+        <v>386</v>
       </c>
       <c r="D524" s="15" t="s">
-        <v>384</v>
+        <v>387</v>
       </c>
       <c r="E524" s="15" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="F524" s="15" t="s">
-        <v>386</v>
+        <v>389</v>
       </c>
       <c r="G524" s="16" t="s">
         <v>58</v>
@@ -15943,22 +15966,22 @@
     </row>
     <row r="530" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A530" s="40" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="B530" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C530" s="27" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="D530" s="28" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="E530" s="28" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="F530" s="28" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
       <c r="G530" s="16" t="s">
         <v>58</v>
@@ -16087,22 +16110,22 @@
     </row>
     <row r="536" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A536" s="40" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="B536" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C536" s="14" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="D536" s="15" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="E536" s="15" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
       <c r="F536" s="15" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="G536" s="16" t="s">
         <v>58</v>
@@ -16231,22 +16254,22 @@
     </row>
     <row r="542" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A542" s="41" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="B542" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C542" s="27" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
       <c r="D542" s="28" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="E542" s="28" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="F542" s="28" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
       <c r="G542" s="16" t="s">
         <v>58</v>
@@ -16375,22 +16398,22 @@
     </row>
     <row r="548" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A548" s="41" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="B548" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C548" s="14" t="s">
-        <v>400</v>
+        <v>403</v>
       </c>
       <c r="D548" s="15" t="s">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="E548" s="15" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
       <c r="F548" s="15" t="s">
-        <v>403</v>
+        <v>406</v>
       </c>
       <c r="G548" s="16" t="s">
         <v>58</v>
@@ -16519,22 +16542,22 @@
     </row>
     <row r="554" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A554" s="41" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="B554" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C554" s="27" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="D554" s="28" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
       <c r="E554" s="28" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="F554" s="28" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="G554" s="16" t="s">
         <v>58</v>
@@ -16663,22 +16686,22 @@
     </row>
     <row r="560" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A560" s="41" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="B560" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C560" s="14" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
       <c r="D560" s="15" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
       <c r="E560" s="15" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="F560" s="15" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
       <c r="G560" s="16" t="s">
         <v>58</v>
@@ -16807,22 +16830,22 @@
     </row>
     <row r="566" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A566" s="41" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="B566" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C566" s="27" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
       <c r="D566" s="28" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="E566" s="28" t="s">
-        <v>414</v>
+        <v>417</v>
       </c>
       <c r="F566" s="28" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
       <c r="G566" s="16" t="s">
         <v>58</v>
@@ -16951,22 +16974,22 @@
     </row>
     <row r="572" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A572" s="41" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="B572" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C572" s="14" t="s">
-        <v>416</v>
+        <v>419</v>
       </c>
       <c r="D572" s="15" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="E572" s="15" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
       <c r="F572" s="15" t="s">
-        <v>419</v>
+        <v>422</v>
       </c>
       <c r="G572" s="16" t="s">
         <v>58</v>
@@ -17095,22 +17118,22 @@
     </row>
     <row r="578" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A578" s="41" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="B578" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C578" s="27" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
       <c r="D578" s="28" t="s">
-        <v>421</v>
+        <v>424</v>
       </c>
       <c r="E578" s="28" t="s">
-        <v>422</v>
+        <v>425</v>
       </c>
       <c r="F578" s="28" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="G578" s="16" t="s">
         <v>58</v>
@@ -17239,22 +17262,22 @@
     </row>
     <row r="584" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A584" s="41" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="B584" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C584" s="14" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="D584" s="15" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
       <c r="E584" s="15" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="F584" s="15" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="G584" s="16" t="s">
         <v>58</v>
@@ -17383,22 +17406,22 @@
     </row>
     <row r="590" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A590" s="41" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="B590" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C590" s="27" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="D590" s="28" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="E590" s="28" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="F590" s="28" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="G590" s="16" t="s">
         <v>58</v>
@@ -17527,22 +17550,22 @@
     </row>
     <row r="596" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A596" s="42" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="B596" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C596" s="14" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
       <c r="D596" s="15" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="E596" s="15" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="F596" s="15" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
       <c r="G596" s="16" t="s">
         <v>58</v>
@@ -18067,22 +18090,22 @@
     </row>
     <row r="620" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A620" s="42" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="B620" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C620" s="27" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="D620" s="28" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E620" s="28" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
       <c r="F620" s="28" t="s">
-        <v>440</v>
+        <v>443</v>
       </c>
       <c r="G620" s="16" t="s">
         <v>58</v>
@@ -18211,22 +18234,22 @@
     </row>
     <row r="626" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A626" s="42" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="B626" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C626" s="14" t="s">
-        <v>441</v>
+        <v>444</v>
       </c>
       <c r="D626" s="15" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="E626" s="15" t="s">
-        <v>443</v>
+        <v>446</v>
       </c>
       <c r="F626" s="15" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
       <c r="G626" s="16" t="s">
         <v>58</v>
@@ -18355,22 +18378,22 @@
     </row>
     <row r="632" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A632" s="42" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="B632" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C632" s="27" t="s">
-        <v>445</v>
+        <v>448</v>
       </c>
       <c r="D632" s="28" t="s">
-        <v>446</v>
+        <v>449</v>
       </c>
       <c r="E632" s="28" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="F632" s="28" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="G632" s="16" t="s">
         <v>58</v>
@@ -18499,22 +18522,22 @@
     </row>
     <row r="638" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A638" s="42" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="B638" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C638" s="14" t="s">
-        <v>449</v>
+        <v>452</v>
       </c>
       <c r="D638" s="15" t="s">
-        <v>450</v>
+        <v>453</v>
       </c>
       <c r="E638" s="15" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="F638" s="15" t="s">
-        <v>452</v>
+        <v>455</v>
       </c>
       <c r="G638" s="16" t="s">
         <v>58</v>
@@ -18643,22 +18666,22 @@
     </row>
     <row r="644" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A644" s="43" t="s">
-        <v>453</v>
+        <v>456</v>
       </c>
       <c r="B644" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C644" s="27" t="s">
-        <v>454</v>
+        <v>457</v>
       </c>
       <c r="D644" s="28" t="s">
-        <v>455</v>
+        <v>458</v>
       </c>
       <c r="E644" s="28" t="s">
-        <v>456</v>
+        <v>459</v>
       </c>
       <c r="F644" s="28" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="G644" s="16" t="s">
         <v>58</v>
@@ -19183,22 +19206,22 @@
     </row>
     <row r="668" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A668" s="43" t="s">
-        <v>453</v>
+        <v>456</v>
       </c>
       <c r="B668" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C668" s="14" t="s">
-        <v>458</v>
+        <v>461</v>
       </c>
       <c r="D668" s="15" t="s">
-        <v>459</v>
+        <v>462</v>
       </c>
       <c r="E668" s="15" t="s">
-        <v>460</v>
+        <v>463</v>
       </c>
       <c r="F668" s="15" t="s">
-        <v>461</v>
+        <v>464</v>
       </c>
       <c r="G668" s="16" t="s">
         <v>58</v>
@@ -19327,22 +19350,22 @@
     </row>
     <row r="674" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A674" s="43" t="s">
-        <v>453</v>
+        <v>456</v>
       </c>
       <c r="B674" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C674" s="27" t="s">
-        <v>462</v>
+        <v>465</v>
       </c>
       <c r="D674" s="28" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="E674" s="28" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="F674" s="28" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
       <c r="G674" s="16" t="s">
         <v>58</v>
@@ -19471,22 +19494,22 @@
     </row>
     <row r="680" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A680" s="43" t="s">
-        <v>453</v>
+        <v>456</v>
       </c>
       <c r="B680" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C680" s="14" t="s">
-        <v>466</v>
+        <v>469</v>
       </c>
       <c r="D680" s="15" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="E680" s="15" t="s">
-        <v>468</v>
+        <v>471</v>
       </c>
       <c r="F680" s="15" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="G680" s="16" t="s">
         <v>58</v>
@@ -19615,22 +19638,22 @@
     </row>
     <row r="686" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A686" s="43" t="s">
-        <v>453</v>
+        <v>456</v>
       </c>
       <c r="B686" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C686" s="27" t="s">
-        <v>469</v>
+        <v>472</v>
       </c>
       <c r="D686" s="28" t="s">
-        <v>470</v>
+        <v>473</v>
       </c>
       <c r="E686" s="28" t="s">
-        <v>471</v>
+        <v>474</v>
       </c>
       <c r="F686" s="28" t="s">
-        <v>472</v>
+        <v>475</v>
       </c>
       <c r="G686" s="16" t="s">
         <v>58</v>
@@ -19759,22 +19782,22 @@
     </row>
     <row r="692" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A692" s="44" t="s">
-        <v>473</v>
+        <v>476</v>
       </c>
       <c r="B692" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C692" s="14" t="s">
-        <v>474</v>
+        <v>477</v>
       </c>
       <c r="D692" s="15" t="s">
-        <v>475</v>
+        <v>478</v>
       </c>
       <c r="E692" s="15" t="s">
-        <v>476</v>
+        <v>479</v>
       </c>
       <c r="F692" s="15" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="G692" s="16" t="s">
         <v>58</v>
@@ -20299,22 +20322,22 @@
     </row>
     <row r="716" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A716" s="44" t="s">
-        <v>473</v>
+        <v>476</v>
       </c>
       <c r="B716" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C716" s="27" t="s">
-        <v>478</v>
+        <v>481</v>
       </c>
       <c r="D716" s="28" t="s">
-        <v>479</v>
+        <v>482</v>
       </c>
       <c r="E716" s="28" t="s">
-        <v>480</v>
+        <v>483</v>
       </c>
       <c r="F716" s="28" t="s">
-        <v>481</v>
+        <v>484</v>
       </c>
       <c r="G716" s="16" t="s">
         <v>58</v>
@@ -20443,22 +20466,22 @@
     </row>
     <row r="722" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A722" s="44" t="s">
-        <v>473</v>
+        <v>476</v>
       </c>
       <c r="B722" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C722" s="14" t="s">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="D722" s="15" t="s">
-        <v>483</v>
+        <v>486</v>
       </c>
       <c r="E722" s="15" t="s">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="F722" s="15" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="G722" s="16" t="s">
         <v>58</v>
@@ -20587,19 +20610,19 @@
     </row>
     <row r="728" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A728" s="44" t="s">
-        <v>473</v>
+        <v>476</v>
       </c>
       <c r="B728" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C728" s="27" t="s">
-        <v>486</v>
+        <v>489</v>
       </c>
       <c r="D728" s="28" t="s">
         <v>216</v>
       </c>
       <c r="E728" s="28" t="s">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="F728" s="28" t="s">
         <v>218</v>
@@ -20731,22 +20754,22 @@
     </row>
     <row r="734" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A734" s="45" t="s">
-        <v>487</v>
+        <v>490</v>
       </c>
       <c r="B734" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C734" s="14" t="s">
-        <v>488</v>
+        <v>491</v>
       </c>
       <c r="D734" s="15" t="s">
-        <v>489</v>
+        <v>492</v>
       </c>
       <c r="E734" s="15" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="F734" s="15" t="s">
-        <v>491</v>
+        <v>494</v>
       </c>
       <c r="G734" s="16" t="s">
         <v>58</v>
@@ -20875,22 +20898,22 @@
     </row>
     <row r="740" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A740" s="45" t="s">
-        <v>487</v>
+        <v>490</v>
       </c>
       <c r="B740" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C740" s="27" t="s">
-        <v>492</v>
+        <v>495</v>
       </c>
       <c r="D740" s="28" t="s">
-        <v>493</v>
+        <v>496</v>
       </c>
       <c r="E740" s="28" t="s">
-        <v>494</v>
+        <v>497</v>
       </c>
       <c r="F740" s="28" t="s">
-        <v>495</v>
+        <v>498</v>
       </c>
       <c r="G740" s="16" t="s">
         <v>58</v>
@@ -21019,22 +21042,22 @@
     </row>
     <row r="746" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A746" s="45" t="s">
-        <v>487</v>
+        <v>490</v>
       </c>
       <c r="B746" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C746" s="14" t="s">
-        <v>496</v>
+        <v>499</v>
       </c>
       <c r="D746" s="15" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="E746" s="15" t="s">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="F746" s="15" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
       <c r="G746" s="16" t="s">
         <v>58</v>
@@ -21163,22 +21186,22 @@
     </row>
     <row r="752" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A752" s="45" t="s">
-        <v>487</v>
+        <v>490</v>
       </c>
       <c r="B752" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C752" s="27" t="s">
-        <v>500</v>
+        <v>503</v>
       </c>
       <c r="D752" s="28" t="s">
-        <v>501</v>
+        <v>504</v>
       </c>
       <c r="E752" s="28" t="s">
-        <v>502</v>
+        <v>505</v>
       </c>
       <c r="F752" s="28" t="s">
-        <v>503</v>
+        <v>506</v>
       </c>
       <c r="G752" s="16" t="s">
         <v>58</v>
@@ -21307,22 +21330,22 @@
     </row>
     <row r="758" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A758" s="45" t="s">
-        <v>487</v>
+        <v>490</v>
       </c>
       <c r="B758" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C758" s="14" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
       <c r="D758" s="15" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="E758" s="15" t="s">
-        <v>506</v>
+        <v>509</v>
       </c>
       <c r="F758" s="15" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="G758" s="16" t="s">
         <v>58</v>
@@ -21451,22 +21474,22 @@
     </row>
     <row r="764" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A764" s="46" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="B764" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C764" s="27" t="s">
-        <v>509</v>
+        <v>512</v>
       </c>
       <c r="D764" s="28" t="s">
-        <v>510</v>
+        <v>513</v>
       </c>
       <c r="E764" s="28" t="s">
-        <v>511</v>
+        <v>514</v>
       </c>
       <c r="F764" s="28" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
       <c r="G764" s="16" t="s">
         <v>58</v>
@@ -21595,22 +21618,22 @@
     </row>
     <row r="770" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A770" s="46" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="B770" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C770" s="14" t="s">
-        <v>513</v>
+        <v>516</v>
       </c>
       <c r="D770" s="15" t="s">
-        <v>514</v>
+        <v>517</v>
       </c>
       <c r="E770" s="15" t="s">
-        <v>515</v>
+        <v>518</v>
       </c>
       <c r="F770" s="15" t="s">
-        <v>516</v>
+        <v>519</v>
       </c>
       <c r="G770" s="16" t="s">
         <v>58</v>
@@ -21739,22 +21762,22 @@
     </row>
     <row r="776" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A776" s="46" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="B776" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C776" s="27" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
       <c r="D776" s="28" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="E776" s="28" t="s">
-        <v>519</v>
+        <v>522</v>
       </c>
       <c r="F776" s="28" t="s">
-        <v>520</v>
+        <v>523</v>
       </c>
       <c r="G776" s="16" t="s">
         <v>58</v>
@@ -21883,22 +21906,22 @@
     </row>
     <row r="782" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A782" s="46" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="B782" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C782" s="14" t="s">
-        <v>521</v>
+        <v>524</v>
       </c>
       <c r="D782" s="15" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="E782" s="15" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="F782" s="15" t="s">
-        <v>524</v>
+        <v>527</v>
       </c>
       <c r="G782" s="16" t="s">
         <v>58</v>
@@ -22027,22 +22050,22 @@
     </row>
     <row r="788" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A788" s="46" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="B788" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C788" s="27" t="s">
-        <v>525</v>
+        <v>528</v>
       </c>
       <c r="D788" s="28" t="s">
-        <v>526</v>
+        <v>529</v>
       </c>
       <c r="E788" s="28" t="s">
-        <v>527</v>
+        <v>530</v>
       </c>
       <c r="F788" s="28" t="s">
-        <v>528</v>
+        <v>531</v>
       </c>
       <c r="G788" s="16" t="s">
         <v>58</v>
@@ -22171,22 +22194,22 @@
     </row>
     <row r="794" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A794" s="46" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="B794" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C794" s="14" t="s">
-        <v>529</v>
+        <v>532</v>
       </c>
       <c r="D794" s="15" t="s">
-        <v>530</v>
+        <v>533</v>
       </c>
       <c r="E794" s="15" t="s">
+        <v>534</v>
+      </c>
+      <c r="F794" s="15" t="s">
         <v>531</v>
-      </c>
-      <c r="F794" s="15" t="s">
-        <v>528</v>
       </c>
       <c r="G794" s="16" t="s">
         <v>58</v>
@@ -22315,22 +22338,22 @@
     </row>
     <row r="800" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A800" s="46" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="B800" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C800" s="27" t="s">
-        <v>532</v>
+        <v>535</v>
       </c>
       <c r="D800" s="28" t="s">
-        <v>533</v>
+        <v>536</v>
       </c>
       <c r="E800" s="28" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="F800" s="28" t="s">
-        <v>535</v>
+        <v>538</v>
       </c>
       <c r="G800" s="16" t="s">
         <v>58</v>
@@ -22459,22 +22482,22 @@
     </row>
     <row r="806" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A806" s="46" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="B806" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C806" s="14" t="s">
-        <v>536</v>
+        <v>539</v>
       </c>
       <c r="D806" s="15" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
       <c r="E806" s="15" t="s">
-        <v>538</v>
+        <v>541</v>
       </c>
       <c r="F806" s="15" t="s">
-        <v>539</v>
+        <v>542</v>
       </c>
       <c r="G806" s="16" t="s">
         <v>58</v>
@@ -22603,22 +22626,22 @@
     </row>
     <row r="812" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A812" s="46" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="B812" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C812" s="27" t="s">
-        <v>540</v>
+        <v>543</v>
       </c>
       <c r="D812" s="28" t="s">
-        <v>541</v>
+        <v>544</v>
       </c>
       <c r="E812" s="28" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
       <c r="F812" s="28" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="G812" s="16" t="s">
         <v>58</v>
@@ -22747,22 +22770,22 @@
     </row>
     <row r="818" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A818" s="46" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="B818" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C818" s="14" t="s">
-        <v>544</v>
+        <v>547</v>
       </c>
       <c r="D818" s="15" t="s">
-        <v>545</v>
+        <v>548</v>
       </c>
       <c r="E818" s="15" t="s">
-        <v>546</v>
+        <v>549</v>
       </c>
       <c r="F818" s="15" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
       <c r="G818" s="16" t="s">
         <v>58</v>
@@ -22891,22 +22914,22 @@
     </row>
     <row r="824" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A824" s="46" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="B824" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C824" s="27" t="s">
-        <v>548</v>
+        <v>551</v>
       </c>
       <c r="D824" s="28" t="s">
-        <v>549</v>
+        <v>552</v>
       </c>
       <c r="E824" s="28" t="s">
-        <v>550</v>
+        <v>553</v>
       </c>
       <c r="F824" s="28" t="s">
-        <v>551</v>
+        <v>554</v>
       </c>
       <c r="G824" s="16" t="s">
         <v>58</v>
@@ -23035,22 +23058,22 @@
     </row>
     <row r="830" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A830" s="46" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="B830" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C830" s="14" t="s">
-        <v>552</v>
+        <v>555</v>
       </c>
       <c r="D830" s="15" t="s">
-        <v>553</v>
+        <v>556</v>
       </c>
       <c r="E830" s="15" t="s">
-        <v>554</v>
+        <v>557</v>
       </c>
       <c r="F830" s="15" t="s">
-        <v>555</v>
+        <v>558</v>
       </c>
       <c r="G830" s="16" t="s">
         <v>58</v>
@@ -23179,22 +23202,22 @@
     </row>
     <row r="836" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A836" s="47" t="s">
-        <v>556</v>
+        <v>559</v>
       </c>
       <c r="B836" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C836" s="27" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="D836" s="28" t="s">
-        <v>558</v>
+        <v>561</v>
       </c>
       <c r="E836" s="28" t="s">
-        <v>559</v>
+        <v>562</v>
       </c>
       <c r="F836" s="28" t="s">
-        <v>560</v>
+        <v>563</v>
       </c>
       <c r="G836" s="16" t="s">
         <v>58</v>
@@ -23323,22 +23346,22 @@
     </row>
     <row r="842" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A842" s="47" t="s">
-        <v>556</v>
+        <v>559</v>
       </c>
       <c r="B842" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C842" s="14" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
       <c r="D842" s="15" t="s">
-        <v>562</v>
+        <v>565</v>
       </c>
       <c r="E842" s="15" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="F842" s="15" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
       <c r="G842" s="16" t="s">
         <v>58</v>
@@ -23467,22 +23490,22 @@
     </row>
     <row r="848" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A848" s="47" t="s">
-        <v>556</v>
+        <v>559</v>
       </c>
       <c r="B848" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C848" s="27" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="D848" s="28" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="E848" s="28" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="F848" s="28" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="G848" s="16" t="s">
         <v>58</v>
@@ -23611,22 +23634,22 @@
     </row>
     <row r="854" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A854" s="47" t="s">
-        <v>556</v>
+        <v>559</v>
       </c>
       <c r="B854" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C854" s="14" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="D854" s="15" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="E854" s="15" t="s">
-        <v>570</v>
+        <v>573</v>
       </c>
       <c r="F854" s="15" t="s">
-        <v>571</v>
+        <v>574</v>
       </c>
       <c r="G854" s="16" t="s">
         <v>58</v>
@@ -23755,22 +23778,22 @@
     </row>
     <row r="860" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A860" s="48" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="B860" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C860" s="27" t="s">
-        <v>573</v>
+        <v>576</v>
       </c>
       <c r="D860" s="28" t="s">
-        <v>574</v>
+        <v>577</v>
       </c>
       <c r="E860" s="28" t="s">
-        <v>575</v>
+        <v>578</v>
       </c>
       <c r="F860" s="28" t="s">
-        <v>576</v>
+        <v>579</v>
       </c>
       <c r="G860" s="16" t="s">
         <v>58</v>
@@ -23899,22 +23922,22 @@
     </row>
     <row r="866" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A866" s="48" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="B866" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C866" s="14" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="D866" s="15" t="s">
-        <v>578</v>
+        <v>581</v>
       </c>
       <c r="E866" s="15" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="F866" s="15" t="s">
-        <v>580</v>
+        <v>583</v>
       </c>
       <c r="G866" s="16" t="s">
         <v>58</v>
@@ -24043,22 +24066,22 @@
     </row>
     <row r="872" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A872" s="48" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="B872" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C872" s="27" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="D872" s="28" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="E872" s="28" t="s">
-        <v>583</v>
+        <v>586</v>
       </c>
       <c r="F872" s="28" t="s">
-        <v>584</v>
+        <v>587</v>
       </c>
       <c r="G872" s="16" t="s">
         <v>58</v>
@@ -24187,22 +24210,22 @@
     </row>
     <row r="878" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A878" s="48" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="B878" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C878" s="14" t="s">
-        <v>585</v>
+        <v>588</v>
       </c>
       <c r="D878" s="15" t="s">
-        <v>586</v>
+        <v>589</v>
       </c>
       <c r="E878" s="15" t="s">
-        <v>587</v>
+        <v>590</v>
       </c>
       <c r="F878" s="15" t="s">
-        <v>588</v>
+        <v>591</v>
       </c>
       <c r="G878" s="16" t="s">
         <v>58</v>
@@ -24331,22 +24354,22 @@
     </row>
     <row r="884" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A884" s="48" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="B884" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C884" s="27" t="s">
-        <v>589</v>
+        <v>592</v>
       </c>
       <c r="D884" s="28" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="E884" s="28" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
       <c r="F884" s="28" t="s">
-        <v>592</v>
+        <v>595</v>
       </c>
       <c r="G884" s="16" t="s">
         <v>58</v>
@@ -24475,22 +24498,22 @@
     </row>
     <row r="890" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A890" s="48" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="B890" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C890" s="14" t="s">
-        <v>593</v>
+        <v>596</v>
       </c>
       <c r="D890" s="15" t="s">
-        <v>594</v>
+        <v>597</v>
       </c>
       <c r="E890" s="15" t="s">
-        <v>595</v>
+        <v>598</v>
       </c>
       <c r="F890" s="15" t="s">
-        <v>596</v>
+        <v>599</v>
       </c>
       <c r="G890" s="16" t="s">
         <v>58</v>
@@ -24619,22 +24642,22 @@
     </row>
     <row r="896" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A896" s="48" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="B896" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C896" s="27" t="s">
-        <v>597</v>
+        <v>600</v>
       </c>
       <c r="D896" s="28" t="s">
-        <v>598</v>
+        <v>601</v>
       </c>
       <c r="E896" s="28" t="s">
-        <v>599</v>
+        <v>602</v>
       </c>
       <c r="F896" s="28" t="s">
-        <v>600</v>
+        <v>603</v>
       </c>
       <c r="G896" s="16" t="s">
         <v>58</v>
@@ -24763,22 +24786,22 @@
     </row>
     <row r="902" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A902" s="49" t="s">
-        <v>601</v>
+        <v>604</v>
       </c>
       <c r="B902" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C902" s="14" t="s">
-        <v>602</v>
+        <v>605</v>
       </c>
       <c r="D902" s="15" t="s">
-        <v>603</v>
+        <v>606</v>
       </c>
       <c r="E902" s="15" t="s">
-        <v>604</v>
+        <v>607</v>
       </c>
       <c r="F902" s="15" t="s">
-        <v>605</v>
+        <v>608</v>
       </c>
       <c r="G902" s="16" t="s">
         <v>58</v>
@@ -24907,22 +24930,22 @@
     </row>
     <row r="908" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A908" s="49" t="s">
-        <v>601</v>
+        <v>604</v>
       </c>
       <c r="B908" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C908" s="27" t="s">
-        <v>606</v>
+        <v>609</v>
       </c>
       <c r="D908" s="28" t="s">
-        <v>607</v>
+        <v>610</v>
       </c>
       <c r="E908" s="28" t="s">
-        <v>608</v>
+        <v>611</v>
       </c>
       <c r="F908" s="28" t="s">
-        <v>609</v>
+        <v>612</v>
       </c>
       <c r="G908" s="16" t="s">
         <v>58</v>
@@ -25051,22 +25074,22 @@
     </row>
     <row r="914" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A914" s="49" t="s">
-        <v>601</v>
+        <v>604</v>
       </c>
       <c r="B914" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C914" s="14" t="s">
-        <v>610</v>
+        <v>613</v>
       </c>
       <c r="D914" s="15" t="s">
-        <v>611</v>
+        <v>614</v>
       </c>
       <c r="E914" s="15" t="s">
-        <v>612</v>
+        <v>615</v>
       </c>
       <c r="F914" s="15" t="s">
-        <v>613</v>
+        <v>616</v>
       </c>
       <c r="G914" s="16" t="s">
         <v>58</v>
@@ -25195,22 +25218,22 @@
     </row>
     <row r="920" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A920" s="49" t="s">
-        <v>601</v>
+        <v>604</v>
       </c>
       <c r="B920" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C920" s="27" t="s">
-        <v>614</v>
+        <v>617</v>
       </c>
       <c r="D920" s="28" t="s">
-        <v>615</v>
+        <v>618</v>
       </c>
       <c r="E920" s="28" t="s">
-        <v>616</v>
+        <v>619</v>
       </c>
       <c r="F920" s="28" t="s">
-        <v>617</v>
+        <v>620</v>
       </c>
       <c r="G920" s="16" t="s">
         <v>58</v>
@@ -25339,22 +25362,22 @@
     </row>
     <row r="926" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A926" s="49" t="s">
-        <v>601</v>
+        <v>604</v>
       </c>
       <c r="B926" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C926" s="14" t="s">
-        <v>618</v>
+        <v>621</v>
       </c>
       <c r="D926" s="15" t="s">
-        <v>619</v>
+        <v>622</v>
       </c>
       <c r="E926" s="15" t="s">
-        <v>620</v>
+        <v>623</v>
       </c>
       <c r="F926" s="15" t="s">
-        <v>621</v>
+        <v>624</v>
       </c>
       <c r="G926" s="16" t="s">
         <v>58</v>
@@ -25483,22 +25506,22 @@
     </row>
     <row r="932" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A932" s="49" t="s">
-        <v>601</v>
+        <v>604</v>
       </c>
       <c r="B932" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C932" s="27" t="s">
-        <v>622</v>
+        <v>625</v>
       </c>
       <c r="D932" s="28" t="s">
-        <v>623</v>
+        <v>626</v>
       </c>
       <c r="E932" s="28" t="s">
-        <v>624</v>
+        <v>627</v>
       </c>
       <c r="F932" s="28" t="s">
-        <v>625</v>
+        <v>628</v>
       </c>
       <c r="G932" s="16" t="s">
         <v>58</v>
@@ -25627,22 +25650,22 @@
     </row>
     <row r="938" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A938" s="50" t="s">
-        <v>626</v>
+        <v>629</v>
       </c>
       <c r="B938" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C938" s="14" t="s">
-        <v>627</v>
+        <v>630</v>
       </c>
       <c r="D938" s="15" t="s">
-        <v>628</v>
+        <v>631</v>
       </c>
       <c r="E938" s="15" t="s">
-        <v>629</v>
+        <v>632</v>
       </c>
       <c r="F938" s="15" t="s">
-        <v>630</v>
+        <v>633</v>
       </c>
       <c r="G938" s="16" t="s">
         <v>58</v>
@@ -25771,22 +25794,22 @@
     </row>
     <row r="944" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A944" s="50" t="s">
-        <v>626</v>
+        <v>629</v>
       </c>
       <c r="B944" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C944" s="27" t="s">
-        <v>631</v>
+        <v>634</v>
       </c>
       <c r="D944" s="28" t="s">
-        <v>632</v>
+        <v>635</v>
       </c>
       <c r="E944" s="28" t="s">
-        <v>633</v>
+        <v>636</v>
       </c>
       <c r="F944" s="28" t="s">
-        <v>634</v>
+        <v>637</v>
       </c>
       <c r="G944" s="16" t="s">
         <v>58</v>
@@ -25915,22 +25938,22 @@
     </row>
     <row r="950" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A950" s="50" t="s">
-        <v>626</v>
+        <v>629</v>
       </c>
       <c r="B950" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C950" s="14" t="s">
-        <v>635</v>
+        <v>638</v>
       </c>
       <c r="D950" s="15" t="s">
-        <v>636</v>
+        <v>639</v>
       </c>
       <c r="E950" s="15" t="s">
-        <v>637</v>
+        <v>640</v>
       </c>
       <c r="F950" s="15" t="s">
-        <v>638</v>
+        <v>641</v>
       </c>
       <c r="G950" s="16" t="s">
         <v>58</v>
@@ -26059,22 +26082,22 @@
     </row>
     <row r="956" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A956" s="50" t="s">
-        <v>626</v>
+        <v>629</v>
       </c>
       <c r="B956" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C956" s="27" t="s">
-        <v>639</v>
+        <v>642</v>
       </c>
       <c r="D956" s="28" t="s">
-        <v>640</v>
+        <v>643</v>
       </c>
       <c r="E956" s="28" t="s">
-        <v>641</v>
+        <v>644</v>
       </c>
       <c r="F956" s="28" t="s">
-        <v>613</v>
+        <v>616</v>
       </c>
       <c r="G956" s="16" t="s">
         <v>58</v>
@@ -26203,22 +26226,22 @@
     </row>
     <row r="962" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A962" s="50" t="s">
-        <v>626</v>
+        <v>629</v>
       </c>
       <c r="B962" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C962" s="14" t="s">
-        <v>642</v>
+        <v>645</v>
       </c>
       <c r="D962" s="15" t="s">
-        <v>643</v>
+        <v>646</v>
       </c>
       <c r="E962" s="15" t="s">
-        <v>644</v>
+        <v>647</v>
       </c>
       <c r="F962" s="15" t="s">
-        <v>645</v>
+        <v>648</v>
       </c>
       <c r="G962" s="16" t="s">
         <v>58</v>
@@ -26347,22 +26370,22 @@
     </row>
     <row r="968" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A968" s="50" t="s">
-        <v>626</v>
+        <v>629</v>
       </c>
       <c r="B968" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C968" s="27" t="s">
-        <v>646</v>
+        <v>649</v>
       </c>
       <c r="D968" s="28" t="s">
-        <v>647</v>
+        <v>650</v>
       </c>
       <c r="E968" s="28" t="s">
-        <v>648</v>
+        <v>651</v>
       </c>
       <c r="F968" s="28" t="s">
-        <v>649</v>
+        <v>652</v>
       </c>
       <c r="G968" s="16" t="s">
         <v>58</v>
@@ -26491,22 +26514,22 @@
     </row>
     <row r="974" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A974" s="51" t="s">
-        <v>650</v>
+        <v>653</v>
       </c>
       <c r="B974" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C974" s="14" t="s">
-        <v>651</v>
+        <v>654</v>
       </c>
       <c r="D974" s="15" t="s">
-        <v>652</v>
+        <v>655</v>
       </c>
       <c r="E974" s="15" t="s">
-        <v>653</v>
+        <v>656</v>
       </c>
       <c r="F974" s="15" t="s">
-        <v>654</v>
+        <v>657</v>
       </c>
       <c r="G974" s="16" t="s">
         <v>58</v>
@@ -26635,22 +26658,22 @@
     </row>
     <row r="980" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A980" s="51" t="s">
-        <v>650</v>
+        <v>653</v>
       </c>
       <c r="B980" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C980" s="27" t="s">
-        <v>655</v>
+        <v>658</v>
       </c>
       <c r="D980" s="28" t="s">
-        <v>656</v>
+        <v>659</v>
       </c>
       <c r="E980" s="28" t="s">
-        <v>657</v>
+        <v>660</v>
       </c>
       <c r="F980" s="28" t="s">
-        <v>658</v>
+        <v>661</v>
       </c>
       <c r="G980" s="16" t="s">
         <v>58</v>
@@ -26779,22 +26802,22 @@
     </row>
     <row r="986" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A986" s="51" t="s">
-        <v>650</v>
+        <v>653</v>
       </c>
       <c r="B986" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C986" s="14" t="s">
-        <v>659</v>
+        <v>662</v>
       </c>
       <c r="D986" s="15" t="s">
-        <v>660</v>
+        <v>663</v>
       </c>
       <c r="E986" s="15" t="s">
-        <v>661</v>
+        <v>664</v>
       </c>
       <c r="F986" s="15" t="s">
-        <v>662</v>
+        <v>665</v>
       </c>
       <c r="G986" s="16" t="s">
         <v>58</v>
@@ -26923,22 +26946,22 @@
     </row>
     <row r="992" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A992" s="51" t="s">
-        <v>650</v>
+        <v>653</v>
       </c>
       <c r="B992" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C992" s="27" t="s">
-        <v>663</v>
+        <v>666</v>
       </c>
       <c r="D992" s="28" t="s">
-        <v>664</v>
+        <v>667</v>
       </c>
       <c r="E992" s="28" t="s">
-        <v>665</v>
+        <v>668</v>
       </c>
       <c r="F992" s="28" t="s">
-        <v>666</v>
+        <v>669</v>
       </c>
       <c r="G992" s="16" t="s">
         <v>58</v>
@@ -27067,22 +27090,22 @@
     </row>
     <row r="998" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A998" s="51" t="s">
-        <v>650</v>
+        <v>653</v>
       </c>
       <c r="B998" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C998" s="14" t="s">
-        <v>667</v>
+        <v>670</v>
       </c>
       <c r="D998" s="15" t="s">
-        <v>668</v>
+        <v>671</v>
       </c>
       <c r="E998" s="15" t="s">
-        <v>669</v>
+        <v>672</v>
       </c>
       <c r="F998" s="15" t="s">
-        <v>670</v>
+        <v>673</v>
       </c>
       <c r="G998" s="16" t="s">
         <v>58</v>
@@ -27211,22 +27234,22 @@
     </row>
     <row r="1004" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1004" s="52" t="s">
-        <v>671</v>
+        <v>674</v>
       </c>
       <c r="B1004" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1004" s="27" t="s">
-        <v>672</v>
+        <v>675</v>
       </c>
       <c r="D1004" s="28" t="s">
-        <v>673</v>
+        <v>676</v>
       </c>
       <c r="E1004" s="28" t="s">
-        <v>674</v>
+        <v>677</v>
       </c>
       <c r="F1004" s="28" t="s">
-        <v>675</v>
+        <v>678</v>
       </c>
       <c r="G1004" s="16" t="s">
         <v>58</v>
@@ -27355,22 +27378,22 @@
     </row>
     <row r="1010" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1010" s="52" t="s">
-        <v>671</v>
+        <v>674</v>
       </c>
       <c r="B1010" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1010" s="14" t="s">
-        <v>676</v>
+        <v>679</v>
       </c>
       <c r="D1010" s="15" t="s">
-        <v>677</v>
+        <v>680</v>
       </c>
       <c r="E1010" s="15" t="s">
-        <v>678</v>
+        <v>681</v>
       </c>
       <c r="F1010" s="15" t="s">
-        <v>679</v>
+        <v>682</v>
       </c>
       <c r="G1010" s="16" t="s">
         <v>58</v>
@@ -27499,22 +27522,22 @@
     </row>
     <row r="1016" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1016" s="52" t="s">
-        <v>671</v>
+        <v>674</v>
       </c>
       <c r="B1016" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1016" s="27" t="s">
-        <v>680</v>
+        <v>683</v>
       </c>
       <c r="D1016" s="28" t="s">
-        <v>681</v>
+        <v>684</v>
       </c>
       <c r="E1016" s="28" t="s">
-        <v>682</v>
+        <v>685</v>
       </c>
       <c r="F1016" s="28" t="s">
-        <v>683</v>
+        <v>686</v>
       </c>
       <c r="G1016" s="16" t="s">
         <v>58</v>
@@ -27643,22 +27666,22 @@
     </row>
     <row r="1022" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1022" s="52" t="s">
-        <v>671</v>
+        <v>674</v>
       </c>
       <c r="B1022" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1022" s="14" t="s">
-        <v>684</v>
+        <v>687</v>
       </c>
       <c r="D1022" s="15" t="s">
-        <v>685</v>
+        <v>688</v>
       </c>
       <c r="E1022" s="15" t="s">
-        <v>686</v>
+        <v>689</v>
       </c>
       <c r="F1022" s="15" t="s">
-        <v>687</v>
+        <v>690</v>
       </c>
       <c r="G1022" s="16" t="s">
         <v>58</v>
@@ -27787,22 +27810,22 @@
     </row>
     <row r="1028" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1028" s="52" t="s">
-        <v>671</v>
+        <v>674</v>
       </c>
       <c r="B1028" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C1028" s="27" t="s">
-        <v>688</v>
+        <v>691</v>
       </c>
       <c r="D1028" s="28" t="s">
-        <v>689</v>
+        <v>692</v>
       </c>
       <c r="E1028" s="28" t="s">
-        <v>690</v>
+        <v>693</v>
       </c>
       <c r="F1028" s="28" t="s">
-        <v>691</v>
+        <v>694</v>
       </c>
       <c r="G1028" s="16" t="s">
         <v>58</v>
@@ -27931,22 +27954,22 @@
     </row>
     <row r="1034" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1034" s="52" t="s">
-        <v>671</v>
+        <v>674</v>
       </c>
       <c r="B1034" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C1034" s="14" t="s">
-        <v>692</v>
+        <v>695</v>
       </c>
       <c r="D1034" s="15" t="s">
-        <v>693</v>
+        <v>696</v>
       </c>
       <c r="E1034" s="15" t="s">
-        <v>694</v>
+        <v>697</v>
       </c>
       <c r="F1034" s="15" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="G1034" s="16" t="s">
         <v>58</v>
@@ -28075,22 +28098,22 @@
     </row>
     <row r="1040" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1040" s="53" t="s">
-        <v>696</v>
+        <v>699</v>
       </c>
       <c r="B1040" s="30" t="s">
         <v>90</v>
       </c>
       <c r="C1040" s="27" t="s">
-        <v>697</v>
+        <v>700</v>
       </c>
       <c r="D1040" s="28" t="s">
-        <v>685</v>
+        <v>688</v>
       </c>
       <c r="E1040" s="28" t="s">
-        <v>698</v>
+        <v>701</v>
       </c>
       <c r="F1040" s="28" t="s">
-        <v>699</v>
+        <v>702</v>
       </c>
       <c r="G1040" s="16" t="s">
         <v>58</v>
@@ -28219,22 +28242,22 @@
     </row>
     <row r="1046" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1046" s="53" t="s">
-        <v>696</v>
+        <v>699</v>
       </c>
       <c r="B1046" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1046" s="14" t="s">
-        <v>700</v>
+        <v>703</v>
       </c>
       <c r="D1046" s="15" t="s">
-        <v>677</v>
+        <v>680</v>
       </c>
       <c r="E1046" s="15" t="s">
-        <v>701</v>
+        <v>704</v>
       </c>
       <c r="F1046" s="15" t="s">
-        <v>702</v>
+        <v>705</v>
       </c>
       <c r="G1046" s="16" t="s">
         <v>58</v>
@@ -28369,16 +28392,16 @@
         <v>53</v>
       </c>
       <c r="C1052" s="27" t="s">
-        <v>703</v>
+        <v>706</v>
       </c>
       <c r="D1052" s="28" t="s">
-        <v>704</v>
+        <v>707</v>
       </c>
       <c r="E1052" s="28" t="s">
-        <v>705</v>
+        <v>708</v>
       </c>
       <c r="F1052" s="28" t="s">
-        <v>706</v>
+        <v>709</v>
       </c>
       <c r="G1052" s="16" t="s">
         <v>58</v>
@@ -28513,16 +28536,16 @@
         <v>53</v>
       </c>
       <c r="C1058" s="14" t="s">
-        <v>707</v>
+        <v>710</v>
       </c>
       <c r="D1058" s="15" t="s">
-        <v>708</v>
+        <v>711</v>
       </c>
       <c r="E1058" s="15" t="s">
-        <v>709</v>
+        <v>712</v>
       </c>
       <c r="F1058" s="15" t="s">
-        <v>710</v>
+        <v>713</v>
       </c>
       <c r="G1058" s="16" t="s">
         <v>58</v>
@@ -29612,10 +29635,10 @@
         <v>39</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>711</v>
+        <v>714</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>712</v>
+        <v>715</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>53</v>
@@ -29633,7 +29656,7 @@
         <v>87</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>713</v>
+        <v>716</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -29812,7 +29835,7 @@
     </row>
     <row r="8" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="60" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="B8" s="1">
         <v>10</v>
@@ -29841,7 +29864,7 @@
     </row>
     <row r="9" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="61" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="B9" s="1">
         <v>11</v>
@@ -29870,7 +29893,7 @@
     </row>
     <row r="10" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="62" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="B10" s="1">
         <v>9</v>
@@ -29899,7 +29922,7 @@
     </row>
     <row r="11" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="63" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="B11" s="1">
         <v>5</v>
@@ -29928,7 +29951,7 @@
     </row>
     <row r="12" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="64" t="s">
-        <v>453</v>
+        <v>456</v>
       </c>
       <c r="B12" s="1">
         <v>5</v>
@@ -29957,7 +29980,7 @@
     </row>
     <row r="13" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="65" t="s">
-        <v>473</v>
+        <v>476</v>
       </c>
       <c r="B13" s="1">
         <v>4</v>
@@ -29986,7 +30009,7 @@
     </row>
     <row r="14" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="66" t="s">
-        <v>487</v>
+        <v>490</v>
       </c>
       <c r="B14" s="1">
         <v>5</v>
@@ -30015,7 +30038,7 @@
     </row>
     <row r="15" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="67" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="B15" s="1">
         <v>12</v>
@@ -30044,7 +30067,7 @@
     </row>
     <row r="16" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="68" t="s">
-        <v>556</v>
+        <v>559</v>
       </c>
       <c r="B16" s="1">
         <v>4</v>
@@ -30073,7 +30096,7 @@
     </row>
     <row r="17" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="69" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="B17" s="1">
         <v>7</v>
@@ -30102,7 +30125,7 @@
     </row>
     <row r="18" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="70" t="s">
-        <v>601</v>
+        <v>604</v>
       </c>
       <c r="B18" s="1">
         <v>6</v>
@@ -30131,7 +30154,7 @@
     </row>
     <row r="19" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="71" t="s">
-        <v>626</v>
+        <v>629</v>
       </c>
       <c r="B19" s="1">
         <v>6</v>
@@ -30160,7 +30183,7 @@
     </row>
     <row r="20" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="72" t="s">
-        <v>650</v>
+        <v>653</v>
       </c>
       <c r="B20" s="1">
         <v>5</v>
@@ -30189,7 +30212,7 @@
     </row>
     <row r="21" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="73" t="s">
-        <v>671</v>
+        <v>674</v>
       </c>
       <c r="B21" s="1">
         <v>6</v>
@@ -30218,7 +30241,7 @@
     </row>
     <row r="22" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="74" t="s">
-        <v>696</v>
+        <v>699</v>
       </c>
       <c r="B22" s="1">
         <v>2</v>
@@ -30247,7 +30270,7 @@
     </row>
     <row r="23" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="75" t="s">
-        <v>714</v>
+        <v>717</v>
       </c>
       <c r="B23" s="75">
         <v>153</v>
@@ -30298,7 +30321,7 @@
         <v>44</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>712</v>
+        <v>715</v>
       </c>
       <c r="C1" s="10" t="s">
         <v>71</v>
@@ -30307,7 +30330,7 @@
         <v>87</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>713</v>
+        <v>716</v>
       </c>
       <c r="F1" s="10" t="s">
         <v>95</v>
@@ -30458,10 +30481,10 @@
         <v>45</v>
       </c>
       <c r="B1" s="10" t="s">
+        <v>718</v>
+      </c>
+      <c r="C1" s="10" t="s">
         <v>715</v>
-      </c>
-      <c r="C1" s="10" t="s">
-        <v>712</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>71</v>
@@ -30470,7 +30493,7 @@
         <v>87</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>713</v>
+        <v>716</v>
       </c>
       <c r="G1" s="10" t="s">
         <v>95</v>
@@ -30481,7 +30504,7 @@
         <v>59</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>716</v>
+        <v>719</v>
       </c>
       <c r="C2" s="1">
         <v>18</v>

</xml_diff>

<commit_message>
078 => fase IV => ZUP-045 OK, ZUP-046 KO mapa≠llistat (fix pins Google amb caché) i traça Excel
</commit_message>
<xml_diff>
--- a/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
+++ b/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4297" uniqueCount="721">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4303" uniqueCount="724">
   <si>
     <t>Zuppeto — Joc de probes manual (totes les pantalles)</t>
   </si>
@@ -864,6 +864,9 @@
     <t>Missatge «No hi ha resultats amb aquest filtre»</t>
   </si>
   <si>
+    <t>26-08-2026</t>
+  </si>
+  <si>
     <t>ZUP-046</t>
   </si>
   <si>
@@ -874,6 +877,12 @@
   </si>
   <si>
     <t>Targetes de lloc amb imatge, tipus, favorit</t>
+  </si>
+  <si>
+    <t>KO: cerca «Arenys de Mar» + Hotel → 4 llocs al llistat (La Premsa, Vila Arenys Hotel, L'Hostalet, Sa Voga) però el mapa diu «Cap resultat al mapa» sense pins. Diferència llista/mapa.</t>
+  </si>
+  <si>
+    <t>Què s'ha fet: els locals Google tenien coordenades però excludeFromOsmMap=true (API viva i BD). Frontend places/detail: pintar també si requiresGoogleMapForGoogleCoordinates. Application ToSummary/ToDetail: no excloure pin mentre la caché Google de coordenades sigui vàlida. UPDATE BD exclude_from_osm_map=false on hi ha lat/lng. Fitxers: places-page.component.ts, place-detail-page.component.ts, PlaceApplicationService.cs.</t>
   </si>
   <si>
     <t>ZUP-047</t>
@@ -2221,7 +2230,7 @@
     <numFmt numFmtId="164" formatCode="dd/mm/yy"/>
     <numFmt numFmtId="165" formatCode="dd-mm-yyyy"/>
   </numFmts>
-  <fonts count="27" x14ac:knownFonts="1">
+  <fonts count="28" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -2230,9 +2239,8 @@
       <name val="Calibri"/>
     </font>
     <font>
-      <color rgb="FF94A3B8"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
+      <b/>
+      <color rgb="FF595959"/>
     </font>
     <font>
       <b/>
@@ -2311,6 +2319,10 @@
       <color rgb="FF334155"/>
       <sz val="10"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF9C0006"/>
     </font>
     <font>
       <b/>
@@ -2399,7 +2411,7 @@
       <name val="Cambria"/>
     </font>
   </fonts>
-  <fills count="42">
+  <fills count="43">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2408,7 +2420,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF8FAFC"/>
+        <fgColor rgb="FFD9D9D9"/>
       </patternFill>
     </fill>
     <fill>
@@ -2450,6 +2462,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF1F5F9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
       </patternFill>
     </fill>
     <fill>
@@ -2740,16 +2757,13 @@
     <xf numFmtId="165" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2761,41 +2775,41 @@
     <xf numFmtId="0" fontId="18" fillId="13" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="17" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="11" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="19" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="20" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="21" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="7" fillId="21" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="22" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="23" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="25" fillId="23" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="24" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -2848,79 +2862,79 @@
     <xf numFmtId="0" fontId="7" fillId="40" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="41" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="23" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="24" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="24" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="25" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="25" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="26" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="26" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="27" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="27" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="28" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="28" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="29" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="29" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="30" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="30" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="31" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="31" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="32" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="32" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="35" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="35" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="36" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="36" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="37" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="37" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="38" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="38" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="39" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="39" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="40" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="40" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="41" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -2932,13 +2946,16 @@
     <xf numFmtId="0" fontId="18" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="41" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="42" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="22" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="23" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="bottom"/>
     </xf>
   </cellXfs>
@@ -11495,9 +11512,11 @@
       <c r="H338" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="I338" s="18"/>
+      <c r="I338" s="18" t="s">
+        <v>277</v>
+      </c>
       <c r="J338" s="19" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K338" s="20"/>
       <c r="L338" s="18"/>
@@ -11622,16 +11641,16 @@
         <v>53</v>
       </c>
       <c r="C344" s="26" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D344" s="27" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="E344" s="27" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="F344" s="27" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="G344" s="16" t="s">
         <v>58</v>
@@ -11639,14 +11658,24 @@
       <c r="H344" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="I344" s="18"/>
+      <c r="I344" s="18" t="s">
+        <v>277</v>
+      </c>
       <c r="J344" s="19" t="s">
-        <v>60</v>
-      </c>
-      <c r="K344" s="20"/>
-      <c r="L344" s="18"/>
-      <c r="M344" s="1"/>
-      <c r="N344" s="20"/>
+        <v>86</v>
+      </c>
+      <c r="K344" s="20" t="s">
+        <v>282</v>
+      </c>
+      <c r="L344" s="18" t="s">
+        <v>277</v>
+      </c>
+      <c r="M344" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="N344" s="20" t="s">
+        <v>283</v>
+      </c>
     </row>
     <row r="345" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A345" s="39"/>
@@ -11766,16 +11795,16 @@
         <v>53</v>
       </c>
       <c r="C350" s="14" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="D350" s="15" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="E350" s="15" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="F350" s="15" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="G350" s="16" t="s">
         <v>58</v>
@@ -11910,16 +11939,16 @@
         <v>53</v>
       </c>
       <c r="C356" s="26" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="D356" s="27" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="E356" s="27" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="F356" s="27" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="G356" s="16" t="s">
         <v>58</v>
@@ -12054,13 +12083,13 @@
         <v>89</v>
       </c>
       <c r="C362" s="14" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="D362" s="15" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="E362" s="15" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="F362" s="15" t="s">
         <v>221</v>
@@ -12198,16 +12227,16 @@
         <v>53</v>
       </c>
       <c r="C368" s="26" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="D368" s="27" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="E368" s="27" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="F368" s="27" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="G368" s="16" t="s">
         <v>58</v>
@@ -12342,16 +12371,16 @@
         <v>89</v>
       </c>
       <c r="C374" s="14" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="D374" s="15" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="E374" s="15" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="F374" s="15" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="G374" s="16" t="s">
         <v>58</v>
@@ -12486,16 +12515,16 @@
         <v>53</v>
       </c>
       <c r="C380" s="26" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="D380" s="27" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="E380" s="27" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="F380" s="27" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="G380" s="16" t="s">
         <v>58</v>
@@ -12630,16 +12659,16 @@
         <v>53</v>
       </c>
       <c r="C386" s="14" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="D386" s="15" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="E386" s="15" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="F386" s="15" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="G386" s="16" t="s">
         <v>58</v>
@@ -12774,16 +12803,16 @@
         <v>89</v>
       </c>
       <c r="C392" s="26" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="D392" s="27" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="E392" s="27" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="F392" s="27" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="G392" s="16" t="s">
         <v>58</v>
@@ -12912,22 +12941,22 @@
     </row>
     <row r="398" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A398" s="40" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="B398" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C398" s="14" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="D398" s="15" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="E398" s="15" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="F398" s="15" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="G398" s="16" t="s">
         <v>58</v>
@@ -13452,22 +13481,22 @@
     </row>
     <row r="422" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A422" s="40" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="B422" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C422" s="26" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="D422" s="27" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="E422" s="27" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="F422" s="27" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="G422" s="16" t="s">
         <v>58</v>
@@ -13596,22 +13625,22 @@
     </row>
     <row r="428" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A428" s="40" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="B428" s="30" t="s">
         <v>89</v>
       </c>
       <c r="C428" s="14" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="D428" s="15" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="E428" s="15" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="F428" s="15" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="G428" s="16" t="s">
         <v>58</v>
@@ -13740,22 +13769,22 @@
     </row>
     <row r="434" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A434" s="40" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="B434" s="30" t="s">
         <v>89</v>
       </c>
       <c r="C434" s="26" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="D434" s="27" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="E434" s="27" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="F434" s="27" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="G434" s="16" t="s">
         <v>58</v>
@@ -13884,22 +13913,22 @@
     </row>
     <row r="440" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A440" s="40" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="B440" s="30" t="s">
         <v>89</v>
       </c>
       <c r="C440" s="14" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="D440" s="15" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="E440" s="15" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="F440" s="15" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="G440" s="16" t="s">
         <v>58</v>
@@ -14028,22 +14057,22 @@
     </row>
     <row r="446" ht="77" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A446" s="40" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="B446" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C446" s="26" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="D446" s="27" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="E446" s="27" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="F446" s="27" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="G446" s="16" t="s">
         <v>58</v>
@@ -14058,7 +14087,7 @@
         <v>86</v>
       </c>
       <c r="K446" s="20" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="L446" s="18" t="s">
         <v>209</v>
@@ -14067,7 +14096,7 @@
         <v>71</v>
       </c>
       <c r="N446" s="20" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
     </row>
     <row r="447" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -14182,22 +14211,22 @@
     </row>
     <row r="452" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A452" s="40" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="B452" s="30" t="s">
         <v>89</v>
       </c>
       <c r="C452" s="14" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="D452" s="15" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="E452" s="15" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="F452" s="15" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="G452" s="16" t="s">
         <v>58</v>
@@ -14326,22 +14355,22 @@
     </row>
     <row r="458" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A458" s="40" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="B458" s="30" t="s">
         <v>89</v>
       </c>
       <c r="C458" s="26" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="D458" s="27" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="E458" s="27" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="F458" s="27" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="G458" s="16" t="s">
         <v>58</v>
@@ -14470,22 +14499,22 @@
     </row>
     <row r="464" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A464" s="40" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="B464" s="30" t="s">
         <v>89</v>
       </c>
       <c r="C464" s="14" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="D464" s="15" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="E464" s="15" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="F464" s="15" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="G464" s="16" t="s">
         <v>58</v>
@@ -14614,22 +14643,22 @@
     </row>
     <row r="470" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A470" s="40" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="B470" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C470" s="26" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="D470" s="27" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="E470" s="27" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="F470" s="27" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="G470" s="16" t="s">
         <v>58</v>
@@ -14758,22 +14787,22 @@
     </row>
     <row r="476" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A476" s="41" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="B476" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C476" s="14" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="D476" s="15" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="E476" s="15" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="F476" s="15" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="G476" s="16" t="s">
         <v>58</v>
@@ -14902,22 +14931,22 @@
     </row>
     <row r="482" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A482" s="41" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="B482" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C482" s="26" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="D482" s="27" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="E482" s="27" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="F482" s="27" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="G482" s="16" t="s">
         <v>58</v>
@@ -15046,22 +15075,22 @@
     </row>
     <row r="488" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A488" s="41" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="B488" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C488" s="14" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="D488" s="15" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="E488" s="15" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="F488" s="15" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="G488" s="16" t="s">
         <v>58</v>
@@ -15190,22 +15219,22 @@
     </row>
     <row r="494" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A494" s="41" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="B494" s="30" t="s">
         <v>89</v>
       </c>
       <c r="C494" s="26" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="D494" s="27" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="E494" s="27" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="F494" s="27" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="G494" s="16" t="s">
         <v>58</v>
@@ -15334,22 +15363,22 @@
     </row>
     <row r="500" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A500" s="41" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="B500" s="30" t="s">
         <v>89</v>
       </c>
       <c r="C500" s="14" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="D500" s="15" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="E500" s="15" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="F500" s="15" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="G500" s="16" t="s">
         <v>58</v>
@@ -15478,22 +15507,22 @@
     </row>
     <row r="506" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A506" s="41" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="B506" s="30" t="s">
         <v>89</v>
       </c>
       <c r="C506" s="26" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="D506" s="27" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="E506" s="27" t="s">
         <v>251</v>
       </c>
       <c r="F506" s="27" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
       <c r="G506" s="16" t="s">
         <v>58</v>
@@ -15622,22 +15651,22 @@
     </row>
     <row r="512" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A512" s="41" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="B512" s="30" t="s">
         <v>89</v>
       </c>
       <c r="C512" s="14" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="D512" s="15" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="E512" s="15" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="F512" s="15" t="s">
-        <v>382</v>
+        <v>385</v>
       </c>
       <c r="G512" s="16" t="s">
         <v>58</v>
@@ -15766,22 +15795,22 @@
     </row>
     <row r="518" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A518" s="41" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="B518" s="30" t="s">
         <v>89</v>
       </c>
       <c r="C518" s="26" t="s">
-        <v>383</v>
+        <v>386</v>
       </c>
       <c r="D518" s="27" t="s">
-        <v>384</v>
+        <v>387</v>
       </c>
       <c r="E518" s="27" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="F518" s="27" t="s">
-        <v>386</v>
+        <v>389</v>
       </c>
       <c r="G518" s="16" t="s">
         <v>58</v>
@@ -15910,22 +15939,22 @@
     </row>
     <row r="524" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A524" s="41" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="B524" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C524" s="14" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="D524" s="15" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="E524" s="15" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="F524" s="15" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
       <c r="G524" s="16" t="s">
         <v>58</v>
@@ -16054,22 +16083,22 @@
     </row>
     <row r="530" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A530" s="41" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="B530" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C530" s="26" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="D530" s="27" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="E530" s="27" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
       <c r="F530" s="27" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="G530" s="16" t="s">
         <v>58</v>
@@ -16198,22 +16227,22 @@
     </row>
     <row r="536" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A536" s="41" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="B536" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C536" s="14" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="D536" s="15" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
       <c r="E536" s="15" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="F536" s="15" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="G536" s="16" t="s">
         <v>58</v>
@@ -16342,22 +16371,22 @@
     </row>
     <row r="542" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A542" s="42" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
       <c r="B542" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C542" s="26" t="s">
-        <v>400</v>
+        <v>403</v>
       </c>
       <c r="D542" s="27" t="s">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="E542" s="27" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
       <c r="F542" s="27" t="s">
-        <v>403</v>
+        <v>406</v>
       </c>
       <c r="G542" s="16" t="s">
         <v>58</v>
@@ -16486,22 +16515,22 @@
     </row>
     <row r="548" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A548" s="42" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
       <c r="B548" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C548" s="14" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="D548" s="15" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
       <c r="E548" s="15" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="F548" s="15" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="G548" s="16" t="s">
         <v>58</v>
@@ -16630,22 +16659,22 @@
     </row>
     <row r="554" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A554" s="42" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
       <c r="B554" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C554" s="26" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
       <c r="D554" s="27" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
       <c r="E554" s="27" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="F554" s="27" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
       <c r="G554" s="16" t="s">
         <v>58</v>
@@ -16774,22 +16803,22 @@
     </row>
     <row r="560" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A560" s="42" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
       <c r="B560" s="30" t="s">
         <v>89</v>
       </c>
       <c r="C560" s="14" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
       <c r="D560" s="15" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="E560" s="15" t="s">
-        <v>414</v>
+        <v>417</v>
       </c>
       <c r="F560" s="15" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
       <c r="G560" s="16" t="s">
         <v>58</v>
@@ -16918,22 +16947,22 @@
     </row>
     <row r="566" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A566" s="42" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
       <c r="B566" s="30" t="s">
         <v>89</v>
       </c>
       <c r="C566" s="26" t="s">
-        <v>416</v>
+        <v>419</v>
       </c>
       <c r="D566" s="27" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="E566" s="27" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
       <c r="F566" s="27" t="s">
-        <v>419</v>
+        <v>422</v>
       </c>
       <c r="G566" s="16" t="s">
         <v>58</v>
@@ -17062,22 +17091,22 @@
     </row>
     <row r="572" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A572" s="42" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
       <c r="B572" s="30" t="s">
         <v>89</v>
       </c>
       <c r="C572" s="14" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
       <c r="D572" s="15" t="s">
-        <v>421</v>
+        <v>424</v>
       </c>
       <c r="E572" s="15" t="s">
-        <v>422</v>
+        <v>425</v>
       </c>
       <c r="F572" s="15" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="G572" s="16" t="s">
         <v>58</v>
@@ -17206,22 +17235,22 @@
     </row>
     <row r="578" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A578" s="42" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
       <c r="B578" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C578" s="26" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="D578" s="27" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
       <c r="E578" s="27" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="F578" s="27" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="G578" s="16" t="s">
         <v>58</v>
@@ -17350,22 +17379,22 @@
     </row>
     <row r="584" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A584" s="42" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
       <c r="B584" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C584" s="14" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="D584" s="15" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="E584" s="15" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="F584" s="15" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="G584" s="16" t="s">
         <v>58</v>
@@ -17494,22 +17523,22 @@
     </row>
     <row r="590" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A590" s="42" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
       <c r="B590" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C590" s="26" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="D590" s="27" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
       <c r="E590" s="27" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="F590" s="27" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="G590" s="16" t="s">
         <v>58</v>
@@ -17638,22 +17667,22 @@
     </row>
     <row r="596" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A596" s="43" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
       <c r="B596" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C596" s="14" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="D596" s="15" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="E596" s="15" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
       <c r="F596" s="15" t="s">
-        <v>440</v>
+        <v>443</v>
       </c>
       <c r="G596" s="16" t="s">
         <v>58</v>
@@ -18178,22 +18207,22 @@
     </row>
     <row r="620" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A620" s="43" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
       <c r="B620" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C620" s="26" t="s">
-        <v>441</v>
+        <v>444</v>
       </c>
       <c r="D620" s="27" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="E620" s="27" t="s">
-        <v>443</v>
+        <v>446</v>
       </c>
       <c r="F620" s="27" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
       <c r="G620" s="16" t="s">
         <v>58</v>
@@ -18322,22 +18351,22 @@
     </row>
     <row r="626" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A626" s="43" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
       <c r="B626" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C626" s="14" t="s">
-        <v>445</v>
+        <v>448</v>
       </c>
       <c r="D626" s="15" t="s">
-        <v>446</v>
+        <v>449</v>
       </c>
       <c r="E626" s="15" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="F626" s="15" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="G626" s="16" t="s">
         <v>58</v>
@@ -18466,22 +18495,22 @@
     </row>
     <row r="632" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A632" s="43" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
       <c r="B632" s="30" t="s">
         <v>89</v>
       </c>
       <c r="C632" s="26" t="s">
-        <v>449</v>
+        <v>452</v>
       </c>
       <c r="D632" s="27" t="s">
-        <v>450</v>
+        <v>453</v>
       </c>
       <c r="E632" s="27" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="F632" s="27" t="s">
-        <v>452</v>
+        <v>455</v>
       </c>
       <c r="G632" s="16" t="s">
         <v>58</v>
@@ -18610,22 +18639,22 @@
     </row>
     <row r="638" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A638" s="43" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
       <c r="B638" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C638" s="14" t="s">
-        <v>453</v>
+        <v>456</v>
       </c>
       <c r="D638" s="15" t="s">
-        <v>454</v>
+        <v>457</v>
       </c>
       <c r="E638" s="15" t="s">
-        <v>455</v>
+        <v>458</v>
       </c>
       <c r="F638" s="15" t="s">
-        <v>456</v>
+        <v>459</v>
       </c>
       <c r="G638" s="16" t="s">
         <v>58</v>
@@ -18754,22 +18783,22 @@
     </row>
     <row r="644" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A644" s="44" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="B644" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C644" s="26" t="s">
-        <v>458</v>
+        <v>461</v>
       </c>
       <c r="D644" s="27" t="s">
-        <v>459</v>
+        <v>462</v>
       </c>
       <c r="E644" s="27" t="s">
-        <v>460</v>
+        <v>463</v>
       </c>
       <c r="F644" s="27" t="s">
-        <v>461</v>
+        <v>464</v>
       </c>
       <c r="G644" s="16" t="s">
         <v>58</v>
@@ -19294,22 +19323,22 @@
     </row>
     <row r="668" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A668" s="44" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="B668" s="30" t="s">
         <v>89</v>
       </c>
       <c r="C668" s="14" t="s">
-        <v>462</v>
+        <v>465</v>
       </c>
       <c r="D668" s="15" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="E668" s="15" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="F668" s="15" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
       <c r="G668" s="16" t="s">
         <v>58</v>
@@ -19438,22 +19467,22 @@
     </row>
     <row r="674" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A674" s="44" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="B674" s="30" t="s">
         <v>89</v>
       </c>
       <c r="C674" s="26" t="s">
-        <v>466</v>
+        <v>469</v>
       </c>
       <c r="D674" s="27" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="E674" s="27" t="s">
-        <v>468</v>
+        <v>471</v>
       </c>
       <c r="F674" s="27" t="s">
-        <v>469</v>
+        <v>472</v>
       </c>
       <c r="G674" s="16" t="s">
         <v>58</v>
@@ -19582,22 +19611,22 @@
     </row>
     <row r="680" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A680" s="44" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="B680" s="30" t="s">
         <v>89</v>
       </c>
       <c r="C680" s="14" t="s">
-        <v>470</v>
+        <v>473</v>
       </c>
       <c r="D680" s="15" t="s">
-        <v>471</v>
+        <v>474</v>
       </c>
       <c r="E680" s="15" t="s">
-        <v>472</v>
+        <v>475</v>
       </c>
       <c r="F680" s="15" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="G680" s="16" t="s">
         <v>58</v>
@@ -19726,22 +19755,22 @@
     </row>
     <row r="686" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A686" s="44" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="B686" s="30" t="s">
         <v>89</v>
       </c>
       <c r="C686" s="26" t="s">
-        <v>473</v>
+        <v>476</v>
       </c>
       <c r="D686" s="27" t="s">
-        <v>474</v>
+        <v>477</v>
       </c>
       <c r="E686" s="27" t="s">
-        <v>475</v>
+        <v>478</v>
       </c>
       <c r="F686" s="27" t="s">
-        <v>476</v>
+        <v>479</v>
       </c>
       <c r="G686" s="16" t="s">
         <v>58</v>
@@ -19870,22 +19899,22 @@
     </row>
     <row r="692" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A692" s="45" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="B692" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C692" s="14" t="s">
-        <v>478</v>
+        <v>481</v>
       </c>
       <c r="D692" s="15" t="s">
-        <v>479</v>
+        <v>482</v>
       </c>
       <c r="E692" s="15" t="s">
-        <v>480</v>
+        <v>483</v>
       </c>
       <c r="F692" s="15" t="s">
-        <v>481</v>
+        <v>484</v>
       </c>
       <c r="G692" s="16" t="s">
         <v>58</v>
@@ -20410,22 +20439,22 @@
     </row>
     <row r="716" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A716" s="45" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="B716" s="30" t="s">
         <v>89</v>
       </c>
       <c r="C716" s="26" t="s">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="D716" s="27" t="s">
-        <v>483</v>
+        <v>486</v>
       </c>
       <c r="E716" s="27" t="s">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="F716" s="27" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="G716" s="16" t="s">
         <v>58</v>
@@ -20554,22 +20583,22 @@
     </row>
     <row r="722" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A722" s="45" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="B722" s="30" t="s">
         <v>89</v>
       </c>
       <c r="C722" s="14" t="s">
-        <v>486</v>
+        <v>489</v>
       </c>
       <c r="D722" s="15" t="s">
-        <v>487</v>
+        <v>490</v>
       </c>
       <c r="E722" s="15" t="s">
-        <v>488</v>
+        <v>491</v>
       </c>
       <c r="F722" s="15" t="s">
-        <v>489</v>
+        <v>492</v>
       </c>
       <c r="G722" s="16" t="s">
         <v>58</v>
@@ -20698,19 +20727,19 @@
     </row>
     <row r="728" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A728" s="45" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="B728" s="30" t="s">
         <v>89</v>
       </c>
       <c r="C728" s="26" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="D728" s="27" t="s">
         <v>215</v>
       </c>
       <c r="E728" s="27" t="s">
-        <v>488</v>
+        <v>491</v>
       </c>
       <c r="F728" s="27" t="s">
         <v>217</v>
@@ -20842,22 +20871,22 @@
     </row>
     <row r="734" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A734" s="46" t="s">
-        <v>491</v>
+        <v>494</v>
       </c>
       <c r="B734" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C734" s="14" t="s">
-        <v>492</v>
+        <v>495</v>
       </c>
       <c r="D734" s="15" t="s">
-        <v>493</v>
+        <v>496</v>
       </c>
       <c r="E734" s="15" t="s">
-        <v>494</v>
+        <v>497</v>
       </c>
       <c r="F734" s="15" t="s">
-        <v>495</v>
+        <v>498</v>
       </c>
       <c r="G734" s="16" t="s">
         <v>58</v>
@@ -20986,22 +21015,22 @@
     </row>
     <row r="740" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A740" s="46" t="s">
-        <v>491</v>
+        <v>494</v>
       </c>
       <c r="B740" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C740" s="26" t="s">
-        <v>496</v>
+        <v>499</v>
       </c>
       <c r="D740" s="27" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="E740" s="27" t="s">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="F740" s="27" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
       <c r="G740" s="16" t="s">
         <v>58</v>
@@ -21130,22 +21159,22 @@
     </row>
     <row r="746" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A746" s="46" t="s">
-        <v>491</v>
+        <v>494</v>
       </c>
       <c r="B746" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C746" s="14" t="s">
-        <v>500</v>
+        <v>503</v>
       </c>
       <c r="D746" s="15" t="s">
-        <v>501</v>
+        <v>504</v>
       </c>
       <c r="E746" s="15" t="s">
-        <v>502</v>
+        <v>505</v>
       </c>
       <c r="F746" s="15" t="s">
-        <v>503</v>
+        <v>506</v>
       </c>
       <c r="G746" s="16" t="s">
         <v>58</v>
@@ -21274,22 +21303,22 @@
     </row>
     <row r="752" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A752" s="46" t="s">
-        <v>491</v>
+        <v>494</v>
       </c>
       <c r="B752" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C752" s="26" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
       <c r="D752" s="27" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="E752" s="27" t="s">
-        <v>506</v>
+        <v>509</v>
       </c>
       <c r="F752" s="27" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="G752" s="16" t="s">
         <v>58</v>
@@ -21418,22 +21447,22 @@
     </row>
     <row r="758" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A758" s="46" t="s">
-        <v>491</v>
+        <v>494</v>
       </c>
       <c r="B758" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C758" s="14" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="D758" s="15" t="s">
-        <v>509</v>
+        <v>512</v>
       </c>
       <c r="E758" s="15" t="s">
-        <v>510</v>
+        <v>513</v>
       </c>
       <c r="F758" s="15" t="s">
-        <v>511</v>
+        <v>514</v>
       </c>
       <c r="G758" s="16" t="s">
         <v>58</v>
@@ -21562,22 +21591,22 @@
     </row>
     <row r="764" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A764" s="47" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
       <c r="B764" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C764" s="26" t="s">
-        <v>513</v>
+        <v>516</v>
       </c>
       <c r="D764" s="27" t="s">
-        <v>514</v>
+        <v>517</v>
       </c>
       <c r="E764" s="27" t="s">
-        <v>515</v>
+        <v>518</v>
       </c>
       <c r="F764" s="27" t="s">
-        <v>516</v>
+        <v>519</v>
       </c>
       <c r="G764" s="16" t="s">
         <v>58</v>
@@ -21706,22 +21735,22 @@
     </row>
     <row r="770" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A770" s="47" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
       <c r="B770" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C770" s="14" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
       <c r="D770" s="15" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="E770" s="15" t="s">
-        <v>519</v>
+        <v>522</v>
       </c>
       <c r="F770" s="15" t="s">
-        <v>520</v>
+        <v>523</v>
       </c>
       <c r="G770" s="16" t="s">
         <v>58</v>
@@ -21850,22 +21879,22 @@
     </row>
     <row r="776" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A776" s="47" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
       <c r="B776" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C776" s="26" t="s">
-        <v>521</v>
+        <v>524</v>
       </c>
       <c r="D776" s="27" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="E776" s="27" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="F776" s="27" t="s">
-        <v>524</v>
+        <v>527</v>
       </c>
       <c r="G776" s="16" t="s">
         <v>58</v>
@@ -21994,22 +22023,22 @@
     </row>
     <row r="782" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A782" s="47" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
       <c r="B782" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C782" s="14" t="s">
-        <v>525</v>
+        <v>528</v>
       </c>
       <c r="D782" s="15" t="s">
-        <v>526</v>
+        <v>529</v>
       </c>
       <c r="E782" s="15" t="s">
-        <v>527</v>
+        <v>530</v>
       </c>
       <c r="F782" s="15" t="s">
-        <v>528</v>
+        <v>531</v>
       </c>
       <c r="G782" s="16" t="s">
         <v>58</v>
@@ -22138,22 +22167,22 @@
     </row>
     <row r="788" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A788" s="47" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
       <c r="B788" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C788" s="26" t="s">
-        <v>529</v>
+        <v>532</v>
       </c>
       <c r="D788" s="27" t="s">
-        <v>530</v>
+        <v>533</v>
       </c>
       <c r="E788" s="27" t="s">
-        <v>531</v>
+        <v>534</v>
       </c>
       <c r="F788" s="27" t="s">
-        <v>532</v>
+        <v>535</v>
       </c>
       <c r="G788" s="16" t="s">
         <v>58</v>
@@ -22282,22 +22311,22 @@
     </row>
     <row r="794" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A794" s="47" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
       <c r="B794" s="30" t="s">
         <v>89</v>
       </c>
       <c r="C794" s="14" t="s">
-        <v>533</v>
+        <v>536</v>
       </c>
       <c r="D794" s="15" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="E794" s="15" t="s">
+        <v>538</v>
+      </c>
+      <c r="F794" s="15" t="s">
         <v>535</v>
-      </c>
-      <c r="F794" s="15" t="s">
-        <v>532</v>
       </c>
       <c r="G794" s="16" t="s">
         <v>58</v>
@@ -22426,22 +22455,22 @@
     </row>
     <row r="800" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A800" s="47" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
       <c r="B800" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C800" s="26" t="s">
-        <v>536</v>
+        <v>539</v>
       </c>
       <c r="D800" s="27" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
       <c r="E800" s="27" t="s">
-        <v>538</v>
+        <v>541</v>
       </c>
       <c r="F800" s="27" t="s">
-        <v>539</v>
+        <v>542</v>
       </c>
       <c r="G800" s="16" t="s">
         <v>58</v>
@@ -22570,22 +22599,22 @@
     </row>
     <row r="806" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A806" s="47" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
       <c r="B806" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C806" s="14" t="s">
-        <v>540</v>
+        <v>543</v>
       </c>
       <c r="D806" s="15" t="s">
-        <v>541</v>
+        <v>544</v>
       </c>
       <c r="E806" s="15" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
       <c r="F806" s="15" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="G806" s="16" t="s">
         <v>58</v>
@@ -22714,22 +22743,22 @@
     </row>
     <row r="812" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A812" s="47" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
       <c r="B812" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C812" s="26" t="s">
-        <v>544</v>
+        <v>547</v>
       </c>
       <c r="D812" s="27" t="s">
-        <v>545</v>
+        <v>548</v>
       </c>
       <c r="E812" s="27" t="s">
-        <v>546</v>
+        <v>549</v>
       </c>
       <c r="F812" s="27" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
       <c r="G812" s="16" t="s">
         <v>58</v>
@@ -22858,22 +22887,22 @@
     </row>
     <row r="818" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A818" s="47" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
       <c r="B818" s="30" t="s">
         <v>89</v>
       </c>
       <c r="C818" s="14" t="s">
-        <v>548</v>
+        <v>551</v>
       </c>
       <c r="D818" s="15" t="s">
-        <v>549</v>
+        <v>552</v>
       </c>
       <c r="E818" s="15" t="s">
-        <v>550</v>
+        <v>553</v>
       </c>
       <c r="F818" s="15" t="s">
-        <v>551</v>
+        <v>554</v>
       </c>
       <c r="G818" s="16" t="s">
         <v>58</v>
@@ -23002,22 +23031,22 @@
     </row>
     <row r="824" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A824" s="47" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
       <c r="B824" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C824" s="26" t="s">
-        <v>552</v>
+        <v>555</v>
       </c>
       <c r="D824" s="27" t="s">
-        <v>553</v>
+        <v>556</v>
       </c>
       <c r="E824" s="27" t="s">
-        <v>554</v>
+        <v>557</v>
       </c>
       <c r="F824" s="27" t="s">
-        <v>555</v>
+        <v>558</v>
       </c>
       <c r="G824" s="16" t="s">
         <v>58</v>
@@ -23146,22 +23175,22 @@
     </row>
     <row r="830" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A830" s="47" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
       <c r="B830" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C830" s="14" t="s">
-        <v>556</v>
+        <v>559</v>
       </c>
       <c r="D830" s="15" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="E830" s="15" t="s">
-        <v>558</v>
+        <v>561</v>
       </c>
       <c r="F830" s="15" t="s">
-        <v>559</v>
+        <v>562</v>
       </c>
       <c r="G830" s="16" t="s">
         <v>58</v>
@@ -23290,22 +23319,22 @@
     </row>
     <row r="836" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A836" s="48" t="s">
-        <v>560</v>
+        <v>563</v>
       </c>
       <c r="B836" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C836" s="26" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
       <c r="D836" s="27" t="s">
-        <v>562</v>
+        <v>565</v>
       </c>
       <c r="E836" s="27" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="F836" s="27" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="G836" s="16" t="s">
         <v>58</v>
@@ -23434,22 +23463,22 @@
     </row>
     <row r="842" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A842" s="48" t="s">
-        <v>560</v>
+        <v>563</v>
       </c>
       <c r="B842" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C842" s="14" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="D842" s="15" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="E842" s="15" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="F842" s="15" t="s">
-        <v>503</v>
+        <v>506</v>
       </c>
       <c r="G842" s="16" t="s">
         <v>58</v>
@@ -23578,22 +23607,22 @@
     </row>
     <row r="848" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A848" s="48" t="s">
-        <v>560</v>
+        <v>563</v>
       </c>
       <c r="B848" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C848" s="26" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="D848" s="27" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="E848" s="27" t="s">
-        <v>570</v>
+        <v>573</v>
       </c>
       <c r="F848" s="27" t="s">
-        <v>571</v>
+        <v>574</v>
       </c>
       <c r="G848" s="16" t="s">
         <v>58</v>
@@ -23722,22 +23751,22 @@
     </row>
     <row r="854" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A854" s="48" t="s">
-        <v>560</v>
+        <v>563</v>
       </c>
       <c r="B854" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C854" s="14" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="D854" s="15" t="s">
-        <v>573</v>
+        <v>576</v>
       </c>
       <c r="E854" s="15" t="s">
-        <v>574</v>
+        <v>577</v>
       </c>
       <c r="F854" s="15" t="s">
-        <v>575</v>
+        <v>578</v>
       </c>
       <c r="G854" s="16" t="s">
         <v>58</v>
@@ -23866,22 +23895,22 @@
     </row>
     <row r="860" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A860" s="49" t="s">
-        <v>576</v>
+        <v>579</v>
       </c>
       <c r="B860" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C860" s="26" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="D860" s="27" t="s">
-        <v>578</v>
+        <v>581</v>
       </c>
       <c r="E860" s="27" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="F860" s="27" t="s">
-        <v>580</v>
+        <v>583</v>
       </c>
       <c r="G860" s="16" t="s">
         <v>58</v>
@@ -24010,22 +24039,22 @@
     </row>
     <row r="866" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A866" s="49" t="s">
-        <v>576</v>
+        <v>579</v>
       </c>
       <c r="B866" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C866" s="14" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="D866" s="15" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="E866" s="15" t="s">
-        <v>583</v>
+        <v>586</v>
       </c>
       <c r="F866" s="15" t="s">
-        <v>584</v>
+        <v>587</v>
       </c>
       <c r="G866" s="16" t="s">
         <v>58</v>
@@ -24154,22 +24183,22 @@
     </row>
     <row r="872" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A872" s="49" t="s">
-        <v>576</v>
+        <v>579</v>
       </c>
       <c r="B872" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C872" s="26" t="s">
-        <v>585</v>
+        <v>588</v>
       </c>
       <c r="D872" s="27" t="s">
-        <v>586</v>
+        <v>589</v>
       </c>
       <c r="E872" s="27" t="s">
-        <v>587</v>
+        <v>590</v>
       </c>
       <c r="F872" s="27" t="s">
-        <v>588</v>
+        <v>591</v>
       </c>
       <c r="G872" s="16" t="s">
         <v>58</v>
@@ -24298,22 +24327,22 @@
     </row>
     <row r="878" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A878" s="49" t="s">
-        <v>576</v>
+        <v>579</v>
       </c>
       <c r="B878" s="30" t="s">
         <v>89</v>
       </c>
       <c r="C878" s="14" t="s">
-        <v>589</v>
+        <v>592</v>
       </c>
       <c r="D878" s="15" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="E878" s="15" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
       <c r="F878" s="15" t="s">
-        <v>592</v>
+        <v>595</v>
       </c>
       <c r="G878" s="16" t="s">
         <v>58</v>
@@ -24442,22 +24471,22 @@
     </row>
     <row r="884" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A884" s="49" t="s">
-        <v>576</v>
+        <v>579</v>
       </c>
       <c r="B884" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C884" s="26" t="s">
-        <v>593</v>
+        <v>596</v>
       </c>
       <c r="D884" s="27" t="s">
-        <v>594</v>
+        <v>597</v>
       </c>
       <c r="E884" s="27" t="s">
-        <v>595</v>
+        <v>598</v>
       </c>
       <c r="F884" s="27" t="s">
-        <v>596</v>
+        <v>599</v>
       </c>
       <c r="G884" s="16" t="s">
         <v>58</v>
@@ -24586,22 +24615,22 @@
     </row>
     <row r="890" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A890" s="49" t="s">
-        <v>576</v>
+        <v>579</v>
       </c>
       <c r="B890" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C890" s="14" t="s">
-        <v>597</v>
+        <v>600</v>
       </c>
       <c r="D890" s="15" t="s">
-        <v>598</v>
+        <v>601</v>
       </c>
       <c r="E890" s="15" t="s">
-        <v>599</v>
+        <v>602</v>
       </c>
       <c r="F890" s="15" t="s">
-        <v>600</v>
+        <v>603</v>
       </c>
       <c r="G890" s="16" t="s">
         <v>58</v>
@@ -24730,22 +24759,22 @@
     </row>
     <row r="896" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A896" s="49" t="s">
-        <v>576</v>
+        <v>579</v>
       </c>
       <c r="B896" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C896" s="26" t="s">
-        <v>601</v>
+        <v>604</v>
       </c>
       <c r="D896" s="27" t="s">
-        <v>602</v>
+        <v>605</v>
       </c>
       <c r="E896" s="27" t="s">
-        <v>603</v>
+        <v>606</v>
       </c>
       <c r="F896" s="27" t="s">
-        <v>604</v>
+        <v>607</v>
       </c>
       <c r="G896" s="16" t="s">
         <v>58</v>
@@ -24874,22 +24903,22 @@
     </row>
     <row r="902" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A902" s="50" t="s">
-        <v>605</v>
+        <v>608</v>
       </c>
       <c r="B902" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C902" s="14" t="s">
-        <v>606</v>
+        <v>609</v>
       </c>
       <c r="D902" s="15" t="s">
-        <v>607</v>
+        <v>610</v>
       </c>
       <c r="E902" s="15" t="s">
-        <v>608</v>
+        <v>611</v>
       </c>
       <c r="F902" s="15" t="s">
-        <v>609</v>
+        <v>612</v>
       </c>
       <c r="G902" s="16" t="s">
         <v>58</v>
@@ -25018,22 +25047,22 @@
     </row>
     <row r="908" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A908" s="50" t="s">
-        <v>605</v>
+        <v>608</v>
       </c>
       <c r="B908" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C908" s="26" t="s">
-        <v>610</v>
+        <v>613</v>
       </c>
       <c r="D908" s="27" t="s">
-        <v>611</v>
+        <v>614</v>
       </c>
       <c r="E908" s="27" t="s">
-        <v>612</v>
+        <v>615</v>
       </c>
       <c r="F908" s="27" t="s">
-        <v>613</v>
+        <v>616</v>
       </c>
       <c r="G908" s="16" t="s">
         <v>58</v>
@@ -25162,22 +25191,22 @@
     </row>
     <row r="914" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A914" s="50" t="s">
-        <v>605</v>
+        <v>608</v>
       </c>
       <c r="B914" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C914" s="14" t="s">
-        <v>614</v>
+        <v>617</v>
       </c>
       <c r="D914" s="15" t="s">
-        <v>615</v>
+        <v>618</v>
       </c>
       <c r="E914" s="15" t="s">
-        <v>616</v>
+        <v>619</v>
       </c>
       <c r="F914" s="15" t="s">
-        <v>617</v>
+        <v>620</v>
       </c>
       <c r="G914" s="16" t="s">
         <v>58</v>
@@ -25306,22 +25335,22 @@
     </row>
     <row r="920" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A920" s="50" t="s">
-        <v>605</v>
+        <v>608</v>
       </c>
       <c r="B920" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C920" s="26" t="s">
-        <v>618</v>
+        <v>621</v>
       </c>
       <c r="D920" s="27" t="s">
-        <v>619</v>
+        <v>622</v>
       </c>
       <c r="E920" s="27" t="s">
-        <v>620</v>
+        <v>623</v>
       </c>
       <c r="F920" s="27" t="s">
-        <v>621</v>
+        <v>624</v>
       </c>
       <c r="G920" s="16" t="s">
         <v>58</v>
@@ -25450,22 +25479,22 @@
     </row>
     <row r="926" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A926" s="50" t="s">
-        <v>605</v>
+        <v>608</v>
       </c>
       <c r="B926" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C926" s="14" t="s">
-        <v>622</v>
+        <v>625</v>
       </c>
       <c r="D926" s="15" t="s">
-        <v>623</v>
+        <v>626</v>
       </c>
       <c r="E926" s="15" t="s">
-        <v>624</v>
+        <v>627</v>
       </c>
       <c r="F926" s="15" t="s">
-        <v>625</v>
+        <v>628</v>
       </c>
       <c r="G926" s="16" t="s">
         <v>58</v>
@@ -25594,22 +25623,22 @@
     </row>
     <row r="932" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A932" s="50" t="s">
-        <v>605</v>
+        <v>608</v>
       </c>
       <c r="B932" s="30" t="s">
         <v>89</v>
       </c>
       <c r="C932" s="26" t="s">
-        <v>626</v>
+        <v>629</v>
       </c>
       <c r="D932" s="27" t="s">
-        <v>627</v>
+        <v>630</v>
       </c>
       <c r="E932" s="27" t="s">
-        <v>628</v>
+        <v>631</v>
       </c>
       <c r="F932" s="27" t="s">
-        <v>629</v>
+        <v>632</v>
       </c>
       <c r="G932" s="16" t="s">
         <v>58</v>
@@ -25738,22 +25767,22 @@
     </row>
     <row r="938" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A938" s="51" t="s">
-        <v>630</v>
+        <v>633</v>
       </c>
       <c r="B938" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C938" s="14" t="s">
-        <v>631</v>
+        <v>634</v>
       </c>
       <c r="D938" s="15" t="s">
-        <v>632</v>
+        <v>635</v>
       </c>
       <c r="E938" s="15" t="s">
-        <v>633</v>
+        <v>636</v>
       </c>
       <c r="F938" s="15" t="s">
-        <v>634</v>
+        <v>637</v>
       </c>
       <c r="G938" s="16" t="s">
         <v>58</v>
@@ -25882,22 +25911,22 @@
     </row>
     <row r="944" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A944" s="51" t="s">
-        <v>630</v>
+        <v>633</v>
       </c>
       <c r="B944" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C944" s="26" t="s">
-        <v>635</v>
+        <v>638</v>
       </c>
       <c r="D944" s="27" t="s">
-        <v>636</v>
+        <v>639</v>
       </c>
       <c r="E944" s="27" t="s">
-        <v>637</v>
+        <v>640</v>
       </c>
       <c r="F944" s="27" t="s">
-        <v>638</v>
+        <v>641</v>
       </c>
       <c r="G944" s="16" t="s">
         <v>58</v>
@@ -26026,22 +26055,22 @@
     </row>
     <row r="950" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A950" s="51" t="s">
-        <v>630</v>
+        <v>633</v>
       </c>
       <c r="B950" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C950" s="14" t="s">
-        <v>639</v>
+        <v>642</v>
       </c>
       <c r="D950" s="15" t="s">
-        <v>640</v>
+        <v>643</v>
       </c>
       <c r="E950" s="15" t="s">
-        <v>641</v>
+        <v>644</v>
       </c>
       <c r="F950" s="15" t="s">
-        <v>642</v>
+        <v>645</v>
       </c>
       <c r="G950" s="16" t="s">
         <v>58</v>
@@ -26170,22 +26199,22 @@
     </row>
     <row r="956" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A956" s="51" t="s">
-        <v>630</v>
+        <v>633</v>
       </c>
       <c r="B956" s="30" t="s">
         <v>89</v>
       </c>
       <c r="C956" s="26" t="s">
-        <v>643</v>
+        <v>646</v>
       </c>
       <c r="D956" s="27" t="s">
-        <v>644</v>
+        <v>647</v>
       </c>
       <c r="E956" s="27" t="s">
-        <v>645</v>
+        <v>648</v>
       </c>
       <c r="F956" s="27" t="s">
-        <v>617</v>
+        <v>620</v>
       </c>
       <c r="G956" s="16" t="s">
         <v>58</v>
@@ -26314,22 +26343,22 @@
     </row>
     <row r="962" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A962" s="51" t="s">
-        <v>630</v>
+        <v>633</v>
       </c>
       <c r="B962" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C962" s="14" t="s">
-        <v>646</v>
+        <v>649</v>
       </c>
       <c r="D962" s="15" t="s">
-        <v>647</v>
+        <v>650</v>
       </c>
       <c r="E962" s="15" t="s">
-        <v>648</v>
+        <v>651</v>
       </c>
       <c r="F962" s="15" t="s">
-        <v>649</v>
+        <v>652</v>
       </c>
       <c r="G962" s="16" t="s">
         <v>58</v>
@@ -26458,22 +26487,22 @@
     </row>
     <row r="968" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A968" s="51" t="s">
-        <v>630</v>
+        <v>633</v>
       </c>
       <c r="B968" s="30" t="s">
         <v>89</v>
       </c>
       <c r="C968" s="26" t="s">
-        <v>650</v>
+        <v>653</v>
       </c>
       <c r="D968" s="27" t="s">
-        <v>651</v>
+        <v>654</v>
       </c>
       <c r="E968" s="27" t="s">
-        <v>652</v>
+        <v>655</v>
       </c>
       <c r="F968" s="27" t="s">
-        <v>653</v>
+        <v>656</v>
       </c>
       <c r="G968" s="16" t="s">
         <v>58</v>
@@ -26602,22 +26631,22 @@
     </row>
     <row r="974" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A974" s="52" t="s">
-        <v>654</v>
+        <v>657</v>
       </c>
       <c r="B974" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C974" s="14" t="s">
-        <v>655</v>
+        <v>658</v>
       </c>
       <c r="D974" s="15" t="s">
-        <v>656</v>
+        <v>659</v>
       </c>
       <c r="E974" s="15" t="s">
-        <v>657</v>
+        <v>660</v>
       </c>
       <c r="F974" s="15" t="s">
-        <v>658</v>
+        <v>661</v>
       </c>
       <c r="G974" s="16" t="s">
         <v>58</v>
@@ -26746,22 +26775,22 @@
     </row>
     <row r="980" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A980" s="52" t="s">
-        <v>654</v>
+        <v>657</v>
       </c>
       <c r="B980" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C980" s="26" t="s">
-        <v>659</v>
+        <v>662</v>
       </c>
       <c r="D980" s="27" t="s">
-        <v>660</v>
+        <v>663</v>
       </c>
       <c r="E980" s="27" t="s">
-        <v>661</v>
+        <v>664</v>
       </c>
       <c r="F980" s="27" t="s">
-        <v>662</v>
+        <v>665</v>
       </c>
       <c r="G980" s="16" t="s">
         <v>58</v>
@@ -26890,22 +26919,22 @@
     </row>
     <row r="986" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A986" s="52" t="s">
-        <v>654</v>
+        <v>657</v>
       </c>
       <c r="B986" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C986" s="14" t="s">
-        <v>663</v>
+        <v>666</v>
       </c>
       <c r="D986" s="15" t="s">
-        <v>664</v>
+        <v>667</v>
       </c>
       <c r="E986" s="15" t="s">
-        <v>665</v>
+        <v>668</v>
       </c>
       <c r="F986" s="15" t="s">
-        <v>666</v>
+        <v>669</v>
       </c>
       <c r="G986" s="16" t="s">
         <v>58</v>
@@ -27034,22 +27063,22 @@
     </row>
     <row r="992" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A992" s="52" t="s">
-        <v>654</v>
+        <v>657</v>
       </c>
       <c r="B992" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C992" s="26" t="s">
-        <v>667</v>
+        <v>670</v>
       </c>
       <c r="D992" s="27" t="s">
-        <v>668</v>
+        <v>671</v>
       </c>
       <c r="E992" s="27" t="s">
-        <v>669</v>
+        <v>672</v>
       </c>
       <c r="F992" s="27" t="s">
-        <v>670</v>
+        <v>673</v>
       </c>
       <c r="G992" s="16" t="s">
         <v>58</v>
@@ -27178,22 +27207,22 @@
     </row>
     <row r="998" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A998" s="52" t="s">
-        <v>654</v>
+        <v>657</v>
       </c>
       <c r="B998" s="30" t="s">
         <v>89</v>
       </c>
       <c r="C998" s="14" t="s">
-        <v>671</v>
+        <v>674</v>
       </c>
       <c r="D998" s="15" t="s">
-        <v>672</v>
+        <v>675</v>
       </c>
       <c r="E998" s="15" t="s">
-        <v>673</v>
+        <v>676</v>
       </c>
       <c r="F998" s="15" t="s">
-        <v>674</v>
+        <v>677</v>
       </c>
       <c r="G998" s="16" t="s">
         <v>58</v>
@@ -27322,22 +27351,22 @@
     </row>
     <row r="1004" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1004" s="53" t="s">
-        <v>675</v>
+        <v>678</v>
       </c>
       <c r="B1004" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1004" s="26" t="s">
-        <v>676</v>
+        <v>679</v>
       </c>
       <c r="D1004" s="27" t="s">
-        <v>677</v>
+        <v>680</v>
       </c>
       <c r="E1004" s="27" t="s">
-        <v>678</v>
+        <v>681</v>
       </c>
       <c r="F1004" s="27" t="s">
-        <v>679</v>
+        <v>682</v>
       </c>
       <c r="G1004" s="16" t="s">
         <v>58</v>
@@ -27466,22 +27495,22 @@
     </row>
     <row r="1010" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1010" s="53" t="s">
-        <v>675</v>
+        <v>678</v>
       </c>
       <c r="B1010" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1010" s="14" t="s">
-        <v>680</v>
+        <v>683</v>
       </c>
       <c r="D1010" s="15" t="s">
-        <v>681</v>
+        <v>684</v>
       </c>
       <c r="E1010" s="15" t="s">
-        <v>682</v>
+        <v>685</v>
       </c>
       <c r="F1010" s="15" t="s">
-        <v>683</v>
+        <v>686</v>
       </c>
       <c r="G1010" s="16" t="s">
         <v>58</v>
@@ -27610,22 +27639,22 @@
     </row>
     <row r="1016" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1016" s="53" t="s">
-        <v>675</v>
+        <v>678</v>
       </c>
       <c r="B1016" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1016" s="26" t="s">
-        <v>684</v>
+        <v>687</v>
       </c>
       <c r="D1016" s="27" t="s">
-        <v>685</v>
+        <v>688</v>
       </c>
       <c r="E1016" s="27" t="s">
-        <v>686</v>
+        <v>689</v>
       </c>
       <c r="F1016" s="27" t="s">
-        <v>687</v>
+        <v>690</v>
       </c>
       <c r="G1016" s="16" t="s">
         <v>58</v>
@@ -27754,22 +27783,22 @@
     </row>
     <row r="1022" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1022" s="53" t="s">
-        <v>675</v>
+        <v>678</v>
       </c>
       <c r="B1022" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1022" s="14" t="s">
-        <v>688</v>
+        <v>691</v>
       </c>
       <c r="D1022" s="15" t="s">
-        <v>689</v>
+        <v>692</v>
       </c>
       <c r="E1022" s="15" t="s">
-        <v>690</v>
+        <v>693</v>
       </c>
       <c r="F1022" s="15" t="s">
-        <v>691</v>
+        <v>694</v>
       </c>
       <c r="G1022" s="16" t="s">
         <v>58</v>
@@ -27898,22 +27927,22 @@
     </row>
     <row r="1028" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1028" s="53" t="s">
-        <v>675</v>
+        <v>678</v>
       </c>
       <c r="B1028" s="30" t="s">
         <v>89</v>
       </c>
       <c r="C1028" s="26" t="s">
-        <v>692</v>
+        <v>695</v>
       </c>
       <c r="D1028" s="27" t="s">
-        <v>693</v>
+        <v>696</v>
       </c>
       <c r="E1028" s="27" t="s">
-        <v>694</v>
+        <v>697</v>
       </c>
       <c r="F1028" s="27" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="G1028" s="16" t="s">
         <v>58</v>
@@ -28042,22 +28071,22 @@
     </row>
     <row r="1034" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1034" s="53" t="s">
-        <v>675</v>
+        <v>678</v>
       </c>
       <c r="B1034" s="30" t="s">
         <v>89</v>
       </c>
       <c r="C1034" s="14" t="s">
-        <v>696</v>
+        <v>699</v>
       </c>
       <c r="D1034" s="15" t="s">
-        <v>697</v>
+        <v>700</v>
       </c>
       <c r="E1034" s="15" t="s">
-        <v>698</v>
+        <v>701</v>
       </c>
       <c r="F1034" s="15" t="s">
-        <v>699</v>
+        <v>702</v>
       </c>
       <c r="G1034" s="16" t="s">
         <v>58</v>
@@ -28186,22 +28215,22 @@
     </row>
     <row r="1040" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1040" s="54" t="s">
-        <v>700</v>
+        <v>703</v>
       </c>
       <c r="B1040" s="30" t="s">
         <v>89</v>
       </c>
       <c r="C1040" s="26" t="s">
-        <v>701</v>
+        <v>704</v>
       </c>
       <c r="D1040" s="27" t="s">
-        <v>689</v>
+        <v>692</v>
       </c>
       <c r="E1040" s="27" t="s">
-        <v>702</v>
+        <v>705</v>
       </c>
       <c r="F1040" s="27" t="s">
-        <v>703</v>
+        <v>706</v>
       </c>
       <c r="G1040" s="16" t="s">
         <v>58</v>
@@ -28330,22 +28359,22 @@
     </row>
     <row r="1046" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1046" s="54" t="s">
-        <v>700</v>
+        <v>703</v>
       </c>
       <c r="B1046" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1046" s="14" t="s">
-        <v>704</v>
+        <v>707</v>
       </c>
       <c r="D1046" s="15" t="s">
-        <v>681</v>
+        <v>684</v>
       </c>
       <c r="E1046" s="15" t="s">
-        <v>705</v>
+        <v>708</v>
       </c>
       <c r="F1046" s="15" t="s">
-        <v>706</v>
+        <v>709</v>
       </c>
       <c r="G1046" s="16" t="s">
         <v>58</v>
@@ -28480,16 +28509,16 @@
         <v>53</v>
       </c>
       <c r="C1052" s="26" t="s">
-        <v>707</v>
+        <v>710</v>
       </c>
       <c r="D1052" s="27" t="s">
-        <v>708</v>
+        <v>711</v>
       </c>
       <c r="E1052" s="27" t="s">
-        <v>709</v>
+        <v>712</v>
       </c>
       <c r="F1052" s="27" t="s">
-        <v>710</v>
+        <v>713</v>
       </c>
       <c r="G1052" s="16" t="s">
         <v>58</v>
@@ -28624,16 +28653,16 @@
         <v>53</v>
       </c>
       <c r="C1058" s="14" t="s">
-        <v>711</v>
+        <v>714</v>
       </c>
       <c r="D1058" s="15" t="s">
-        <v>712</v>
+        <v>715</v>
       </c>
       <c r="E1058" s="15" t="s">
-        <v>713</v>
+        <v>716</v>
       </c>
       <c r="F1058" s="15" t="s">
-        <v>714</v>
+        <v>717</v>
       </c>
       <c r="G1058" s="16" t="s">
         <v>58</v>
@@ -29719,10 +29748,10 @@
         <v>39</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>715</v>
+        <v>718</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>716</v>
+        <v>719</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>53</v>
@@ -29740,7 +29769,7 @@
         <v>86</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>717</v>
+        <v>720</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -29919,7 +29948,7 @@
     </row>
     <row r="8" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="61" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="B8" s="1">
         <v>10</v>
@@ -29948,7 +29977,7 @@
     </row>
     <row r="9" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="62" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="B9" s="1">
         <v>11</v>
@@ -29977,7 +30006,7 @@
     </row>
     <row r="10" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="63" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
       <c r="B10" s="1">
         <v>9</v>
@@ -30006,7 +30035,7 @@
     </row>
     <row r="11" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="64" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
       <c r="B11" s="1">
         <v>5</v>
@@ -30035,7 +30064,7 @@
     </row>
     <row r="12" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="65" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="B12" s="1">
         <v>5</v>
@@ -30064,7 +30093,7 @@
     </row>
     <row r="13" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="66" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="B13" s="1">
         <v>4</v>
@@ -30093,7 +30122,7 @@
     </row>
     <row r="14" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="67" t="s">
-        <v>491</v>
+        <v>494</v>
       </c>
       <c r="B14" s="1">
         <v>5</v>
@@ -30122,7 +30151,7 @@
     </row>
     <row r="15" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="68" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
       <c r="B15" s="1">
         <v>12</v>
@@ -30151,7 +30180,7 @@
     </row>
     <row r="16" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="69" t="s">
-        <v>560</v>
+        <v>563</v>
       </c>
       <c r="B16" s="1">
         <v>4</v>
@@ -30180,7 +30209,7 @@
     </row>
     <row r="17" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="70" t="s">
-        <v>576</v>
+        <v>579</v>
       </c>
       <c r="B17" s="1">
         <v>7</v>
@@ -30209,7 +30238,7 @@
     </row>
     <row r="18" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="71" t="s">
-        <v>605</v>
+        <v>608</v>
       </c>
       <c r="B18" s="1">
         <v>6</v>
@@ -30238,7 +30267,7 @@
     </row>
     <row r="19" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="72" t="s">
-        <v>630</v>
+        <v>633</v>
       </c>
       <c r="B19" s="1">
         <v>6</v>
@@ -30267,7 +30296,7 @@
     </row>
     <row r="20" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="73" t="s">
-        <v>654</v>
+        <v>657</v>
       </c>
       <c r="B20" s="1">
         <v>5</v>
@@ -30296,7 +30325,7 @@
     </row>
     <row r="21" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="74" t="s">
-        <v>675</v>
+        <v>678</v>
       </c>
       <c r="B21" s="1">
         <v>6</v>
@@ -30325,7 +30354,7 @@
     </row>
     <row r="22" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="75" t="s">
-        <v>700</v>
+        <v>703</v>
       </c>
       <c r="B22" s="1">
         <v>2</v>
@@ -30354,7 +30383,7 @@
     </row>
     <row r="23" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="76" t="s">
-        <v>718</v>
+        <v>721</v>
       </c>
       <c r="B23" s="76">
         <v>153</v>
@@ -30405,7 +30434,7 @@
         <v>44</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>716</v>
+        <v>719</v>
       </c>
       <c r="C1" s="10" t="s">
         <v>71</v>
@@ -30414,7 +30443,7 @@
         <v>86</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>717</v>
+        <v>720</v>
       </c>
       <c r="F1" s="10" t="s">
         <v>94</v>
@@ -30565,10 +30594,10 @@
         <v>45</v>
       </c>
       <c r="B1" s="10" t="s">
+        <v>722</v>
+      </c>
+      <c r="C1" s="10" t="s">
         <v>719</v>
-      </c>
-      <c r="C1" s="10" t="s">
-        <v>716</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>71</v>
@@ -30577,7 +30606,7 @@
         <v>86</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>717</v>
+        <v>720</v>
       </c>
       <c r="G1" s="10" t="s">
         <v>94</v>
@@ -30588,7 +30617,7 @@
         <v>59</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>720</v>
+        <v>723</v>
       </c>
       <c r="C2" s="1">
         <v>18</v>

</xml_diff>

<commit_message>
081 => fase IV => ZUP-055 OK (Chrome/USER), placeholder Imatge no disponible al detall i millora FET
</commit_message>
<xml_diff>
--- a/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
+++ b/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4307" uniqueCount="724">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4309" uniqueCount="726">
   <si>
     <t>Zuppeto — Joc de probes manual (totes les pantalles)</t>
   </si>
@@ -991,6 +991,12 @@
   </si>
   <si>
     <t>H1 amb nom, imatge, descripció i mètriques</t>
+  </si>
+  <si>
+    <t>29-08-2026</t>
+  </si>
+  <si>
+    <t>Fitxa OK (nom, descripció, mètriques). Sense foto de portada: placeholder «Imatge no disponible» (millora FET; implementada per error durant proves).</t>
   </si>
   <si>
     <t>ZUP-056</t>
@@ -2241,6 +2247,8 @@
     <font>
       <b/>
       <color rgb="FF006100"/>
+      <sz val="10"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
@@ -2749,7 +2757,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -13092,11 +13100,15 @@
       <c r="H404" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="I404" s="18"/>
+      <c r="I404" s="18" t="s">
+        <v>320</v>
+      </c>
       <c r="J404" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="K404" s="19"/>
+        <v>71</v>
+      </c>
+      <c r="K404" s="19" t="s">
+        <v>321</v>
+      </c>
       <c r="L404" s="18"/>
       <c r="M404" s="1"/>
       <c r="N404" s="19"/>
@@ -13483,16 +13495,16 @@
         <v>53</v>
       </c>
       <c r="C422" s="25" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="D422" s="26" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="E422" s="26" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="F422" s="26" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="G422" s="16" t="s">
         <v>58</v>
@@ -13627,16 +13639,16 @@
         <v>89</v>
       </c>
       <c r="C428" s="14" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="D428" s="15" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="E428" s="15" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="F428" s="15" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="G428" s="16" t="s">
         <v>58</v>
@@ -13771,16 +13783,16 @@
         <v>89</v>
       </c>
       <c r="C434" s="25" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="D434" s="26" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="E434" s="26" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="F434" s="26" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="G434" s="16" t="s">
         <v>58</v>
@@ -13915,16 +13927,16 @@
         <v>89</v>
       </c>
       <c r="C440" s="14" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="D440" s="15" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="E440" s="15" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="F440" s="15" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="G440" s="16" t="s">
         <v>58</v>
@@ -14059,16 +14071,16 @@
         <v>53</v>
       </c>
       <c r="C446" s="25" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="D446" s="26" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="E446" s="26" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="F446" s="26" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="G446" s="16" t="s">
         <v>58</v>
@@ -14083,7 +14095,7 @@
         <v>86</v>
       </c>
       <c r="K446" s="19" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="L446" s="18" t="s">
         <v>209</v>
@@ -14092,7 +14104,7 @@
         <v>71</v>
       </c>
       <c r="N446" s="19" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
     </row>
     <row r="447" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -14213,16 +14225,16 @@
         <v>89</v>
       </c>
       <c r="C452" s="14" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="D452" s="15" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="E452" s="15" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="F452" s="15" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="G452" s="16" t="s">
         <v>58</v>
@@ -14357,16 +14369,16 @@
         <v>89</v>
       </c>
       <c r="C458" s="25" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="D458" s="26" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="E458" s="26" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="F458" s="26" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="G458" s="16" t="s">
         <v>58</v>
@@ -14501,16 +14513,16 @@
         <v>89</v>
       </c>
       <c r="C464" s="14" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="D464" s="15" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="E464" s="15" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="F464" s="15" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="G464" s="16" t="s">
         <v>58</v>
@@ -14645,16 +14657,16 @@
         <v>53</v>
       </c>
       <c r="C470" s="25" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="D470" s="26" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="E470" s="26" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="F470" s="26" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="G470" s="16" t="s">
         <v>58</v>
@@ -14783,22 +14795,22 @@
     </row>
     <row r="476" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A476" s="40" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B476" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C476" s="14" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="D476" s="15" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="E476" s="15" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="F476" s="15" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="G476" s="16" t="s">
         <v>58</v>
@@ -14927,22 +14939,22 @@
     </row>
     <row r="482" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A482" s="40" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B482" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C482" s="25" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="D482" s="26" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="E482" s="26" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="F482" s="26" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="G482" s="16" t="s">
         <v>58</v>
@@ -15071,22 +15083,22 @@
     </row>
     <row r="488" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A488" s="40" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B488" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C488" s="14" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="D488" s="15" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="E488" s="15" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="F488" s="15" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="G488" s="16" t="s">
         <v>58</v>
@@ -15215,22 +15227,22 @@
     </row>
     <row r="494" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A494" s="40" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B494" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C494" s="25" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="D494" s="26" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="E494" s="26" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="F494" s="26" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="G494" s="16" t="s">
         <v>58</v>
@@ -15359,22 +15371,22 @@
     </row>
     <row r="500" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A500" s="40" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B500" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C500" s="14" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="D500" s="15" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="E500" s="15" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="F500" s="15" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="G500" s="16" t="s">
         <v>58</v>
@@ -15503,22 +15515,22 @@
     </row>
     <row r="506" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A506" s="40" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B506" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C506" s="25" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="D506" s="26" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="E506" s="26" t="s">
         <v>251</v>
       </c>
       <c r="F506" s="26" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="G506" s="16" t="s">
         <v>58</v>
@@ -15647,22 +15659,22 @@
     </row>
     <row r="512" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A512" s="40" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B512" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C512" s="14" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="D512" s="15" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="E512" s="15" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="F512" s="15" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="G512" s="16" t="s">
         <v>58</v>
@@ -15791,22 +15803,22 @@
     </row>
     <row r="518" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A518" s="40" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B518" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C518" s="25" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="D518" s="26" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="E518" s="26" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="F518" s="26" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="G518" s="16" t="s">
         <v>58</v>
@@ -15935,22 +15947,22 @@
     </row>
     <row r="524" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A524" s="40" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B524" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C524" s="14" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="D524" s="15" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="E524" s="15" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="F524" s="15" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="G524" s="16" t="s">
         <v>58</v>
@@ -16079,22 +16091,22 @@
     </row>
     <row r="530" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A530" s="40" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B530" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C530" s="25" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="D530" s="26" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="E530" s="26" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="F530" s="26" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="G530" s="16" t="s">
         <v>58</v>
@@ -16223,22 +16235,22 @@
     </row>
     <row r="536" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A536" s="40" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B536" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C536" s="14" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="D536" s="15" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="E536" s="15" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="F536" s="15" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="G536" s="16" t="s">
         <v>58</v>
@@ -16367,22 +16379,22 @@
     </row>
     <row r="542" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A542" s="41" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="B542" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C542" s="25" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="D542" s="26" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="E542" s="26" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="F542" s="26" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="G542" s="16" t="s">
         <v>58</v>
@@ -16511,22 +16523,22 @@
     </row>
     <row r="548" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A548" s="41" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="B548" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C548" s="14" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="D548" s="15" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="E548" s="15" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="F548" s="15" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="G548" s="16" t="s">
         <v>58</v>
@@ -16655,22 +16667,22 @@
     </row>
     <row r="554" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A554" s="41" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="B554" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C554" s="25" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="D554" s="26" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="E554" s="26" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="F554" s="26" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="G554" s="16" t="s">
         <v>58</v>
@@ -16799,22 +16811,22 @@
     </row>
     <row r="560" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A560" s="41" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="B560" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C560" s="14" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="D560" s="15" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="E560" s="15" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="F560" s="15" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="G560" s="16" t="s">
         <v>58</v>
@@ -16943,22 +16955,22 @@
     </row>
     <row r="566" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A566" s="41" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="B566" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C566" s="25" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="D566" s="26" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="E566" s="26" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="F566" s="26" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="G566" s="16" t="s">
         <v>58</v>
@@ -17087,22 +17099,22 @@
     </row>
     <row r="572" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A572" s="41" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="B572" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C572" s="14" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="D572" s="15" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="E572" s="15" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="F572" s="15" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="G572" s="16" t="s">
         <v>58</v>
@@ -17231,22 +17243,22 @@
     </row>
     <row r="578" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A578" s="41" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="B578" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C578" s="25" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="D578" s="26" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="E578" s="26" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="F578" s="26" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="G578" s="16" t="s">
         <v>58</v>
@@ -17375,22 +17387,22 @@
     </row>
     <row r="584" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A584" s="41" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="B584" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C584" s="14" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="D584" s="15" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="E584" s="15" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="F584" s="15" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="G584" s="16" t="s">
         <v>58</v>
@@ -17519,22 +17531,22 @@
     </row>
     <row r="590" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A590" s="41" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="B590" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C590" s="25" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="D590" s="26" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="E590" s="26" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="F590" s="26" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="G590" s="16" t="s">
         <v>58</v>
@@ -17663,22 +17675,22 @@
     </row>
     <row r="596" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A596" s="42" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="B596" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C596" s="14" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="D596" s="15" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="E596" s="15" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="F596" s="15" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="G596" s="16" t="s">
         <v>58</v>
@@ -18203,22 +18215,22 @@
     </row>
     <row r="620" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A620" s="42" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="B620" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C620" s="25" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="D620" s="26" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="E620" s="26" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="F620" s="26" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="G620" s="16" t="s">
         <v>58</v>
@@ -18347,22 +18359,22 @@
     </row>
     <row r="626" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A626" s="42" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="B626" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C626" s="14" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="D626" s="15" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="E626" s="15" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="F626" s="15" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="G626" s="16" t="s">
         <v>58</v>
@@ -18491,22 +18503,22 @@
     </row>
     <row r="632" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A632" s="42" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="B632" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C632" s="25" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="D632" s="26" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="E632" s="26" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="F632" s="26" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="G632" s="16" t="s">
         <v>58</v>
@@ -18635,22 +18647,22 @@
     </row>
     <row r="638" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A638" s="42" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="B638" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C638" s="14" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="D638" s="15" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="E638" s="15" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="F638" s="15" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="G638" s="16" t="s">
         <v>58</v>
@@ -18779,22 +18791,22 @@
     </row>
     <row r="644" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A644" s="43" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="B644" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C644" s="25" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="D644" s="26" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="E644" s="26" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="F644" s="26" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="G644" s="16" t="s">
         <v>58</v>
@@ -19319,22 +19331,22 @@
     </row>
     <row r="668" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A668" s="43" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="B668" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C668" s="14" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="D668" s="15" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="E668" s="15" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="F668" s="15" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="G668" s="16" t="s">
         <v>58</v>
@@ -19463,22 +19475,22 @@
     </row>
     <row r="674" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A674" s="43" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="B674" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C674" s="25" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="D674" s="26" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="E674" s="26" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="F674" s="26" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="G674" s="16" t="s">
         <v>58</v>
@@ -19607,22 +19619,22 @@
     </row>
     <row r="680" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A680" s="43" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="B680" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C680" s="14" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="D680" s="15" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="E680" s="15" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="F680" s="15" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="G680" s="16" t="s">
         <v>58</v>
@@ -19751,22 +19763,22 @@
     </row>
     <row r="686" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A686" s="43" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="B686" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C686" s="25" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="D686" s="26" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="E686" s="26" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="F686" s="26" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="G686" s="16" t="s">
         <v>58</v>
@@ -19895,22 +19907,22 @@
     </row>
     <row r="692" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A692" s="44" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="B692" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C692" s="14" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="D692" s="15" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="E692" s="15" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="F692" s="15" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="G692" s="16" t="s">
         <v>58</v>
@@ -20435,22 +20447,22 @@
     </row>
     <row r="716" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A716" s="44" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="B716" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C716" s="25" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="D716" s="26" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="E716" s="26" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="F716" s="26" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="G716" s="16" t="s">
         <v>58</v>
@@ -20579,22 +20591,22 @@
     </row>
     <row r="722" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A722" s="44" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="B722" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C722" s="14" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="D722" s="15" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="E722" s="15" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="F722" s="15" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="G722" s="16" t="s">
         <v>58</v>
@@ -20723,19 +20735,19 @@
     </row>
     <row r="728" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A728" s="44" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="B728" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C728" s="25" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="D728" s="26" t="s">
         <v>215</v>
       </c>
       <c r="E728" s="26" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="F728" s="26" t="s">
         <v>217</v>
@@ -20867,22 +20879,22 @@
     </row>
     <row r="734" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A734" s="45" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="B734" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C734" s="14" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="D734" s="15" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="E734" s="15" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="F734" s="15" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="G734" s="16" t="s">
         <v>58</v>
@@ -21011,22 +21023,22 @@
     </row>
     <row r="740" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A740" s="45" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="B740" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C740" s="25" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="D740" s="26" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="E740" s="26" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="F740" s="26" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="G740" s="16" t="s">
         <v>58</v>
@@ -21155,22 +21167,22 @@
     </row>
     <row r="746" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A746" s="45" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="B746" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C746" s="14" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="D746" s="15" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="E746" s="15" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="F746" s="15" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="G746" s="16" t="s">
         <v>58</v>
@@ -21299,22 +21311,22 @@
     </row>
     <row r="752" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A752" s="45" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="B752" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C752" s="25" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="D752" s="26" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="E752" s="26" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="F752" s="26" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="G752" s="16" t="s">
         <v>58</v>
@@ -21443,22 +21455,22 @@
     </row>
     <row r="758" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A758" s="45" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="B758" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C758" s="14" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="D758" s="15" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="E758" s="15" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="F758" s="15" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="G758" s="16" t="s">
         <v>58</v>
@@ -21587,22 +21599,22 @@
     </row>
     <row r="764" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A764" s="46" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="B764" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C764" s="25" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="D764" s="26" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="E764" s="26" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="F764" s="26" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="G764" s="16" t="s">
         <v>58</v>
@@ -21731,22 +21743,22 @@
     </row>
     <row r="770" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A770" s="46" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="B770" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C770" s="14" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="D770" s="15" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="E770" s="15" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="F770" s="15" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="G770" s="16" t="s">
         <v>58</v>
@@ -21875,22 +21887,22 @@
     </row>
     <row r="776" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A776" s="46" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="B776" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C776" s="25" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="D776" s="26" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="E776" s="26" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="F776" s="26" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="G776" s="16" t="s">
         <v>58</v>
@@ -22019,22 +22031,22 @@
     </row>
     <row r="782" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A782" s="46" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="B782" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C782" s="14" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="D782" s="15" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="E782" s="15" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="F782" s="15" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="G782" s="16" t="s">
         <v>58</v>
@@ -22163,22 +22175,22 @@
     </row>
     <row r="788" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A788" s="46" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="B788" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C788" s="25" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="D788" s="26" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="E788" s="26" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="F788" s="26" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="G788" s="16" t="s">
         <v>58</v>
@@ -22307,22 +22319,22 @@
     </row>
     <row r="794" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A794" s="46" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="B794" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C794" s="14" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="D794" s="15" t="s">
+        <v>539</v>
+      </c>
+      <c r="E794" s="15" t="s">
+        <v>540</v>
+      </c>
+      <c r="F794" s="15" t="s">
         <v>537</v>
-      </c>
-      <c r="E794" s="15" t="s">
-        <v>538</v>
-      </c>
-      <c r="F794" s="15" t="s">
-        <v>535</v>
       </c>
       <c r="G794" s="16" t="s">
         <v>58</v>
@@ -22451,22 +22463,22 @@
     </row>
     <row r="800" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A800" s="46" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="B800" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C800" s="25" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="D800" s="26" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="E800" s="26" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="F800" s="26" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="G800" s="16" t="s">
         <v>58</v>
@@ -22595,22 +22607,22 @@
     </row>
     <row r="806" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A806" s="46" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="B806" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C806" s="14" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D806" s="15" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="E806" s="15" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="F806" s="15" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="G806" s="16" t="s">
         <v>58</v>
@@ -22739,22 +22751,22 @@
     </row>
     <row r="812" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A812" s="46" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="B812" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C812" s="25" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="D812" s="26" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="E812" s="26" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="F812" s="26" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="G812" s="16" t="s">
         <v>58</v>
@@ -22883,22 +22895,22 @@
     </row>
     <row r="818" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A818" s="46" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="B818" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C818" s="14" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="D818" s="15" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="E818" s="15" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="F818" s="15" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="G818" s="16" t="s">
         <v>58</v>
@@ -23027,22 +23039,22 @@
     </row>
     <row r="824" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A824" s="46" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="B824" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C824" s="25" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="D824" s="26" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="E824" s="26" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
       <c r="F824" s="26" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="G824" s="16" t="s">
         <v>58</v>
@@ -23171,22 +23183,22 @@
     </row>
     <row r="830" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A830" s="46" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="B830" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C830" s="14" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="D830" s="15" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="E830" s="15" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
       <c r="F830" s="15" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
       <c r="G830" s="16" t="s">
         <v>58</v>
@@ -23315,22 +23327,22 @@
     </row>
     <row r="836" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A836" s="47" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
       <c r="B836" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C836" s="25" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="D836" s="26" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="E836" s="26" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="F836" s="26" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
       <c r="G836" s="16" t="s">
         <v>58</v>
@@ -23459,22 +23471,22 @@
     </row>
     <row r="842" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A842" s="47" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
       <c r="B842" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C842" s="14" t="s">
-        <v>568</v>
+        <v>570</v>
       </c>
       <c r="D842" s="15" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="E842" s="15" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
       <c r="F842" s="15" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="G842" s="16" t="s">
         <v>58</v>
@@ -23603,22 +23615,22 @@
     </row>
     <row r="848" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A848" s="47" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
       <c r="B848" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C848" s="25" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
       <c r="D848" s="26" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
       <c r="E848" s="26" t="s">
-        <v>573</v>
+        <v>575</v>
       </c>
       <c r="F848" s="26" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="G848" s="16" t="s">
         <v>58</v>
@@ -23747,22 +23759,22 @@
     </row>
     <row r="854" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A854" s="47" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
       <c r="B854" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C854" s="14" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="D854" s="15" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="E854" s="15" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="F854" s="15" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="G854" s="16" t="s">
         <v>58</v>
@@ -23891,22 +23903,22 @@
     </row>
     <row r="860" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A860" s="48" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="B860" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C860" s="25" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="D860" s="26" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="E860" s="26" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="F860" s="26" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="G860" s="16" t="s">
         <v>58</v>
@@ -24035,22 +24047,22 @@
     </row>
     <row r="866" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A866" s="48" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="B866" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C866" s="14" t="s">
-        <v>584</v>
+        <v>586</v>
       </c>
       <c r="D866" s="15" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
       <c r="E866" s="15" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
       <c r="F866" s="15" t="s">
-        <v>587</v>
+        <v>589</v>
       </c>
       <c r="G866" s="16" t="s">
         <v>58</v>
@@ -24179,22 +24191,22 @@
     </row>
     <row r="872" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A872" s="48" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="B872" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C872" s="25" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="D872" s="26" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="E872" s="26" t="s">
-        <v>590</v>
+        <v>592</v>
       </c>
       <c r="F872" s="26" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="G872" s="16" t="s">
         <v>58</v>
@@ -24323,22 +24335,22 @@
     </row>
     <row r="878" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A878" s="48" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="B878" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C878" s="14" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
       <c r="D878" s="15" t="s">
-        <v>593</v>
+        <v>595</v>
       </c>
       <c r="E878" s="15" t="s">
-        <v>594</v>
+        <v>596</v>
       </c>
       <c r="F878" s="15" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
       <c r="G878" s="16" t="s">
         <v>58</v>
@@ -24467,22 +24479,22 @@
     </row>
     <row r="884" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A884" s="48" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="B884" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C884" s="25" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
       <c r="D884" s="26" t="s">
-        <v>597</v>
+        <v>599</v>
       </c>
       <c r="E884" s="26" t="s">
-        <v>598</v>
+        <v>600</v>
       </c>
       <c r="F884" s="26" t="s">
-        <v>599</v>
+        <v>601</v>
       </c>
       <c r="G884" s="16" t="s">
         <v>58</v>
@@ -24611,22 +24623,22 @@
     </row>
     <row r="890" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A890" s="48" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="B890" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C890" s="14" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
       <c r="D890" s="15" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="E890" s="15" t="s">
-        <v>602</v>
+        <v>604</v>
       </c>
       <c r="F890" s="15" t="s">
-        <v>603</v>
+        <v>605</v>
       </c>
       <c r="G890" s="16" t="s">
         <v>58</v>
@@ -24755,22 +24767,22 @@
     </row>
     <row r="896" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A896" s="48" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="B896" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C896" s="25" t="s">
-        <v>604</v>
+        <v>606</v>
       </c>
       <c r="D896" s="26" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
       <c r="E896" s="26" t="s">
-        <v>606</v>
+        <v>608</v>
       </c>
       <c r="F896" s="26" t="s">
-        <v>607</v>
+        <v>609</v>
       </c>
       <c r="G896" s="16" t="s">
         <v>58</v>
@@ -24899,22 +24911,22 @@
     </row>
     <row r="902" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A902" s="49" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
       <c r="B902" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C902" s="14" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="D902" s="15" t="s">
-        <v>610</v>
+        <v>612</v>
       </c>
       <c r="E902" s="15" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
       <c r="F902" s="15" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="G902" s="16" t="s">
         <v>58</v>
@@ -25043,22 +25055,22 @@
     </row>
     <row r="908" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A908" s="49" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
       <c r="B908" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C908" s="25" t="s">
-        <v>613</v>
+        <v>615</v>
       </c>
       <c r="D908" s="26" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
       <c r="E908" s="26" t="s">
-        <v>615</v>
+        <v>617</v>
       </c>
       <c r="F908" s="26" t="s">
-        <v>616</v>
+        <v>618</v>
       </c>
       <c r="G908" s="16" t="s">
         <v>58</v>
@@ -25187,22 +25199,22 @@
     </row>
     <row r="914" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A914" s="49" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
       <c r="B914" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C914" s="14" t="s">
-        <v>617</v>
+        <v>619</v>
       </c>
       <c r="D914" s="15" t="s">
-        <v>618</v>
+        <v>620</v>
       </c>
       <c r="E914" s="15" t="s">
-        <v>619</v>
+        <v>621</v>
       </c>
       <c r="F914" s="15" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="G914" s="16" t="s">
         <v>58</v>
@@ -25331,22 +25343,22 @@
     </row>
     <row r="920" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A920" s="49" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
       <c r="B920" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C920" s="25" t="s">
-        <v>621</v>
+        <v>623</v>
       </c>
       <c r="D920" s="26" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
       <c r="E920" s="26" t="s">
-        <v>623</v>
+        <v>625</v>
       </c>
       <c r="F920" s="26" t="s">
-        <v>624</v>
+        <v>626</v>
       </c>
       <c r="G920" s="16" t="s">
         <v>58</v>
@@ -25475,22 +25487,22 @@
     </row>
     <row r="926" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A926" s="49" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
       <c r="B926" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C926" s="14" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
       <c r="D926" s="15" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
       <c r="E926" s="15" t="s">
-        <v>627</v>
+        <v>629</v>
       </c>
       <c r="F926" s="15" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
       <c r="G926" s="16" t="s">
         <v>58</v>
@@ -25619,22 +25631,22 @@
     </row>
     <row r="932" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A932" s="49" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
       <c r="B932" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C932" s="25" t="s">
-        <v>629</v>
+        <v>631</v>
       </c>
       <c r="D932" s="26" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
       <c r="E932" s="26" t="s">
-        <v>631</v>
+        <v>633</v>
       </c>
       <c r="F932" s="26" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
       <c r="G932" s="16" t="s">
         <v>58</v>
@@ -25763,22 +25775,22 @@
     </row>
     <row r="938" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A938" s="50" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="B938" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C938" s="14" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
       <c r="D938" s="15" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="E938" s="15" t="s">
-        <v>636</v>
+        <v>638</v>
       </c>
       <c r="F938" s="15" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="G938" s="16" t="s">
         <v>58</v>
@@ -25907,22 +25919,22 @@
     </row>
     <row r="944" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A944" s="50" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="B944" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C944" s="25" t="s">
-        <v>638</v>
+        <v>640</v>
       </c>
       <c r="D944" s="26" t="s">
-        <v>639</v>
+        <v>641</v>
       </c>
       <c r="E944" s="26" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
       <c r="F944" s="26" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
       <c r="G944" s="16" t="s">
         <v>58</v>
@@ -26051,22 +26063,22 @@
     </row>
     <row r="950" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A950" s="50" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="B950" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C950" s="14" t="s">
-        <v>642</v>
+        <v>644</v>
       </c>
       <c r="D950" s="15" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
       <c r="E950" s="15" t="s">
-        <v>644</v>
+        <v>646</v>
       </c>
       <c r="F950" s="15" t="s">
-        <v>645</v>
+        <v>647</v>
       </c>
       <c r="G950" s="16" t="s">
         <v>58</v>
@@ -26195,22 +26207,22 @@
     </row>
     <row r="956" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A956" s="50" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="B956" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C956" s="25" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
       <c r="D956" s="26" t="s">
-        <v>647</v>
+        <v>649</v>
       </c>
       <c r="E956" s="26" t="s">
-        <v>648</v>
+        <v>650</v>
       </c>
       <c r="F956" s="26" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="G956" s="16" t="s">
         <v>58</v>
@@ -26339,22 +26351,22 @@
     </row>
     <row r="962" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A962" s="50" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="B962" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C962" s="14" t="s">
-        <v>649</v>
+        <v>651</v>
       </c>
       <c r="D962" s="15" t="s">
-        <v>650</v>
+        <v>652</v>
       </c>
       <c r="E962" s="15" t="s">
-        <v>651</v>
+        <v>653</v>
       </c>
       <c r="F962" s="15" t="s">
-        <v>652</v>
+        <v>654</v>
       </c>
       <c r="G962" s="16" t="s">
         <v>58</v>
@@ -26483,22 +26495,22 @@
     </row>
     <row r="968" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A968" s="50" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="B968" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C968" s="25" t="s">
-        <v>653</v>
+        <v>655</v>
       </c>
       <c r="D968" s="26" t="s">
-        <v>654</v>
+        <v>656</v>
       </c>
       <c r="E968" s="26" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
       <c r="F968" s="26" t="s">
-        <v>656</v>
+        <v>658</v>
       </c>
       <c r="G968" s="16" t="s">
         <v>58</v>
@@ -26627,22 +26639,22 @@
     </row>
     <row r="974" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A974" s="51" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
       <c r="B974" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C974" s="14" t="s">
-        <v>658</v>
+        <v>660</v>
       </c>
       <c r="D974" s="15" t="s">
-        <v>659</v>
+        <v>661</v>
       </c>
       <c r="E974" s="15" t="s">
-        <v>660</v>
+        <v>662</v>
       </c>
       <c r="F974" s="15" t="s">
-        <v>661</v>
+        <v>663</v>
       </c>
       <c r="G974" s="16" t="s">
         <v>58</v>
@@ -26771,22 +26783,22 @@
     </row>
     <row r="980" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A980" s="51" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
       <c r="B980" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C980" s="25" t="s">
-        <v>662</v>
+        <v>664</v>
       </c>
       <c r="D980" s="26" t="s">
-        <v>663</v>
+        <v>665</v>
       </c>
       <c r="E980" s="26" t="s">
-        <v>664</v>
+        <v>666</v>
       </c>
       <c r="F980" s="26" t="s">
-        <v>665</v>
+        <v>667</v>
       </c>
       <c r="G980" s="16" t="s">
         <v>58</v>
@@ -26915,22 +26927,22 @@
     </row>
     <row r="986" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A986" s="51" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
       <c r="B986" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C986" s="14" t="s">
-        <v>666</v>
+        <v>668</v>
       </c>
       <c r="D986" s="15" t="s">
-        <v>667</v>
+        <v>669</v>
       </c>
       <c r="E986" s="15" t="s">
-        <v>668</v>
+        <v>670</v>
       </c>
       <c r="F986" s="15" t="s">
-        <v>669</v>
+        <v>671</v>
       </c>
       <c r="G986" s="16" t="s">
         <v>58</v>
@@ -27059,22 +27071,22 @@
     </row>
     <row r="992" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A992" s="51" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
       <c r="B992" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C992" s="25" t="s">
-        <v>670</v>
+        <v>672</v>
       </c>
       <c r="D992" s="26" t="s">
-        <v>671</v>
+        <v>673</v>
       </c>
       <c r="E992" s="26" t="s">
-        <v>672</v>
+        <v>674</v>
       </c>
       <c r="F992" s="26" t="s">
-        <v>673</v>
+        <v>675</v>
       </c>
       <c r="G992" s="16" t="s">
         <v>58</v>
@@ -27203,22 +27215,22 @@
     </row>
     <row r="998" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A998" s="51" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
       <c r="B998" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C998" s="14" t="s">
-        <v>674</v>
+        <v>676</v>
       </c>
       <c r="D998" s="15" t="s">
-        <v>675</v>
+        <v>677</v>
       </c>
       <c r="E998" s="15" t="s">
-        <v>676</v>
+        <v>678</v>
       </c>
       <c r="F998" s="15" t="s">
-        <v>677</v>
+        <v>679</v>
       </c>
       <c r="G998" s="16" t="s">
         <v>58</v>
@@ -27347,22 +27359,22 @@
     </row>
     <row r="1004" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1004" s="52" t="s">
-        <v>678</v>
+        <v>680</v>
       </c>
       <c r="B1004" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1004" s="25" t="s">
-        <v>679</v>
+        <v>681</v>
       </c>
       <c r="D1004" s="26" t="s">
-        <v>680</v>
+        <v>682</v>
       </c>
       <c r="E1004" s="26" t="s">
-        <v>681</v>
+        <v>683</v>
       </c>
       <c r="F1004" s="26" t="s">
-        <v>682</v>
+        <v>684</v>
       </c>
       <c r="G1004" s="16" t="s">
         <v>58</v>
@@ -27491,22 +27503,22 @@
     </row>
     <row r="1010" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1010" s="52" t="s">
-        <v>678</v>
+        <v>680</v>
       </c>
       <c r="B1010" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1010" s="14" t="s">
-        <v>683</v>
+        <v>685</v>
       </c>
       <c r="D1010" s="15" t="s">
-        <v>684</v>
+        <v>686</v>
       </c>
       <c r="E1010" s="15" t="s">
-        <v>685</v>
+        <v>687</v>
       </c>
       <c r="F1010" s="15" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
       <c r="G1010" s="16" t="s">
         <v>58</v>
@@ -27635,22 +27647,22 @@
     </row>
     <row r="1016" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1016" s="52" t="s">
-        <v>678</v>
+        <v>680</v>
       </c>
       <c r="B1016" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1016" s="25" t="s">
-        <v>687</v>
+        <v>689</v>
       </c>
       <c r="D1016" s="26" t="s">
-        <v>688</v>
+        <v>690</v>
       </c>
       <c r="E1016" s="26" t="s">
-        <v>689</v>
+        <v>691</v>
       </c>
       <c r="F1016" s="26" t="s">
-        <v>690</v>
+        <v>692</v>
       </c>
       <c r="G1016" s="16" t="s">
         <v>58</v>
@@ -27779,22 +27791,22 @@
     </row>
     <row r="1022" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1022" s="52" t="s">
-        <v>678</v>
+        <v>680</v>
       </c>
       <c r="B1022" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1022" s="14" t="s">
-        <v>691</v>
+        <v>693</v>
       </c>
       <c r="D1022" s="15" t="s">
-        <v>692</v>
+        <v>694</v>
       </c>
       <c r="E1022" s="15" t="s">
-        <v>693</v>
+        <v>695</v>
       </c>
       <c r="F1022" s="15" t="s">
-        <v>694</v>
+        <v>696</v>
       </c>
       <c r="G1022" s="16" t="s">
         <v>58</v>
@@ -27923,22 +27935,22 @@
     </row>
     <row r="1028" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1028" s="52" t="s">
-        <v>678</v>
+        <v>680</v>
       </c>
       <c r="B1028" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C1028" s="25" t="s">
-        <v>695</v>
+        <v>697</v>
       </c>
       <c r="D1028" s="26" t="s">
-        <v>696</v>
+        <v>698</v>
       </c>
       <c r="E1028" s="26" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
       <c r="F1028" s="26" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
       <c r="G1028" s="16" t="s">
         <v>58</v>
@@ -28067,22 +28079,22 @@
     </row>
     <row r="1034" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1034" s="52" t="s">
-        <v>678</v>
+        <v>680</v>
       </c>
       <c r="B1034" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C1034" s="14" t="s">
-        <v>699</v>
+        <v>701</v>
       </c>
       <c r="D1034" s="15" t="s">
-        <v>700</v>
+        <v>702</v>
       </c>
       <c r="E1034" s="15" t="s">
-        <v>701</v>
+        <v>703</v>
       </c>
       <c r="F1034" s="15" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="G1034" s="16" t="s">
         <v>58</v>
@@ -28211,22 +28223,22 @@
     </row>
     <row r="1040" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1040" s="53" t="s">
-        <v>703</v>
+        <v>705</v>
       </c>
       <c r="B1040" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C1040" s="25" t="s">
-        <v>704</v>
+        <v>706</v>
       </c>
       <c r="D1040" s="26" t="s">
-        <v>692</v>
+        <v>694</v>
       </c>
       <c r="E1040" s="26" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
       <c r="F1040" s="26" t="s">
-        <v>706</v>
+        <v>708</v>
       </c>
       <c r="G1040" s="16" t="s">
         <v>58</v>
@@ -28355,22 +28367,22 @@
     </row>
     <row r="1046" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1046" s="53" t="s">
-        <v>703</v>
+        <v>705</v>
       </c>
       <c r="B1046" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1046" s="14" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
       <c r="D1046" s="15" t="s">
-        <v>684</v>
+        <v>686</v>
       </c>
       <c r="E1046" s="15" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="F1046" s="15" t="s">
-        <v>709</v>
+        <v>711</v>
       </c>
       <c r="G1046" s="16" t="s">
         <v>58</v>
@@ -28505,16 +28517,16 @@
         <v>53</v>
       </c>
       <c r="C1052" s="25" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="D1052" s="26" t="s">
-        <v>711</v>
+        <v>713</v>
       </c>
       <c r="E1052" s="26" t="s">
-        <v>712</v>
+        <v>714</v>
       </c>
       <c r="F1052" s="26" t="s">
-        <v>713</v>
+        <v>715</v>
       </c>
       <c r="G1052" s="16" t="s">
         <v>58</v>
@@ -28649,16 +28661,16 @@
         <v>53</v>
       </c>
       <c r="C1058" s="14" t="s">
-        <v>714</v>
+        <v>716</v>
       </c>
       <c r="D1058" s="15" t="s">
-        <v>715</v>
+        <v>717</v>
       </c>
       <c r="E1058" s="15" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
       <c r="F1058" s="15" t="s">
-        <v>717</v>
+        <v>719</v>
       </c>
       <c r="G1058" s="16" t="s">
         <v>58</v>
@@ -29744,10 +29756,10 @@
         <v>39</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>718</v>
+        <v>720</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>53</v>
@@ -29765,7 +29777,7 @@
         <v>86</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -29973,7 +29985,7 @@
     </row>
     <row r="9" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="61" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="B9" s="1">
         <v>11</v>
@@ -30002,7 +30014,7 @@
     </row>
     <row r="10" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="62" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="B10" s="1">
         <v>9</v>
@@ -30031,7 +30043,7 @@
     </row>
     <row r="11" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="63" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="B11" s="1">
         <v>5</v>
@@ -30060,7 +30072,7 @@
     </row>
     <row r="12" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="64" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="B12" s="1">
         <v>5</v>
@@ -30089,7 +30101,7 @@
     </row>
     <row r="13" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="65" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="B13" s="1">
         <v>4</v>
@@ -30118,7 +30130,7 @@
     </row>
     <row r="14" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="66" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="B14" s="1">
         <v>5</v>
@@ -30147,7 +30159,7 @@
     </row>
     <row r="15" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="67" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="B15" s="1">
         <v>12</v>
@@ -30176,7 +30188,7 @@
     </row>
     <row r="16" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="68" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
       <c r="B16" s="1">
         <v>4</v>
@@ -30205,7 +30217,7 @@
     </row>
     <row r="17" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="69" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="B17" s="1">
         <v>7</v>
@@ -30234,7 +30246,7 @@
     </row>
     <row r="18" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="70" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
       <c r="B18" s="1">
         <v>6</v>
@@ -30263,7 +30275,7 @@
     </row>
     <row r="19" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="71" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="B19" s="1">
         <v>6</v>
@@ -30292,7 +30304,7 @@
     </row>
     <row r="20" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="72" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
       <c r="B20" s="1">
         <v>5</v>
@@ -30321,7 +30333,7 @@
     </row>
     <row r="21" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="73" t="s">
-        <v>678</v>
+        <v>680</v>
       </c>
       <c r="B21" s="1">
         <v>6</v>
@@ -30350,7 +30362,7 @@
     </row>
     <row r="22" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="74" t="s">
-        <v>703</v>
+        <v>705</v>
       </c>
       <c r="B22" s="1">
         <v>2</v>
@@ -30379,7 +30391,7 @@
     </row>
     <row r="23" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="75" t="s">
-        <v>721</v>
+        <v>723</v>
       </c>
       <c r="B23" s="75">
         <v>153</v>
@@ -30430,7 +30442,7 @@
         <v>44</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
       <c r="C1" s="10" t="s">
         <v>71</v>
@@ -30439,7 +30451,7 @@
         <v>86</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
       <c r="F1" s="10" t="s">
         <v>94</v>
@@ -30590,10 +30602,10 @@
         <v>45</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>722</v>
+        <v>724</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>71</v>
@@ -30602,7 +30614,7 @@
         <v>86</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
       <c r="G1" s="10" t="s">
         <v>94</v>
@@ -30613,7 +30625,7 @@
         <v>59</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>723</v>
+        <v>725</v>
       </c>
       <c r="C2" s="1">
         <v>18</v>

</xml_diff>

<commit_message>
082 => fase IV => ZUP-056 ZUP-064 OK (Chrome/USER) i regla xat proves (codi + pas a pas)
</commit_message>
<xml_diff>
--- a/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
+++ b/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4309" uniqueCount="726">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4311" uniqueCount="727">
   <si>
     <t>Zuppeto — Joc de probes manual (totes les pantalles)</t>
   </si>
@@ -1009,6 +1009,9 @@
   </si>
   <si>
     <t>Enllaços funcionals a / i /places</t>
+  </si>
+  <si>
+    <t>30-08-2026</t>
   </si>
   <si>
     <t>ZUP-057</t>
@@ -13512,9 +13515,11 @@
       <c r="H422" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="I422" s="18"/>
+      <c r="I422" s="18" t="s">
+        <v>326</v>
+      </c>
       <c r="J422" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K422" s="19"/>
       <c r="L422" s="18"/>
@@ -13639,16 +13644,16 @@
         <v>89</v>
       </c>
       <c r="C428" s="14" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="D428" s="15" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="E428" s="15" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="F428" s="15" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="G428" s="16" t="s">
         <v>58</v>
@@ -13783,16 +13788,16 @@
         <v>89</v>
       </c>
       <c r="C434" s="25" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D434" s="26" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="E434" s="26" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="F434" s="26" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G434" s="16" t="s">
         <v>58</v>
@@ -13927,16 +13932,16 @@
         <v>89</v>
       </c>
       <c r="C440" s="14" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="D440" s="15" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="E440" s="15" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="F440" s="15" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="G440" s="16" t="s">
         <v>58</v>
@@ -14071,16 +14076,16 @@
         <v>53</v>
       </c>
       <c r="C446" s="25" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="D446" s="26" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="E446" s="26" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="F446" s="26" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="G446" s="16" t="s">
         <v>58</v>
@@ -14095,7 +14100,7 @@
         <v>86</v>
       </c>
       <c r="K446" s="19" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="L446" s="18" t="s">
         <v>209</v>
@@ -14104,7 +14109,7 @@
         <v>71</v>
       </c>
       <c r="N446" s="19" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
     </row>
     <row r="447" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -14225,16 +14230,16 @@
         <v>89</v>
       </c>
       <c r="C452" s="14" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="D452" s="15" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="E452" s="15" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="F452" s="15" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="G452" s="16" t="s">
         <v>58</v>
@@ -14369,16 +14374,16 @@
         <v>89</v>
       </c>
       <c r="C458" s="25" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="D458" s="26" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="E458" s="26" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="F458" s="26" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="G458" s="16" t="s">
         <v>58</v>
@@ -14513,16 +14518,16 @@
         <v>89</v>
       </c>
       <c r="C464" s="14" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="D464" s="15" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="E464" s="15" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="F464" s="15" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="G464" s="16" t="s">
         <v>58</v>
@@ -14657,16 +14662,16 @@
         <v>53</v>
       </c>
       <c r="C470" s="25" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="D470" s="26" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="E470" s="26" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="F470" s="26" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="G470" s="16" t="s">
         <v>58</v>
@@ -14674,9 +14679,11 @@
       <c r="H470" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="I470" s="18"/>
+      <c r="I470" s="18" t="s">
+        <v>326</v>
+      </c>
       <c r="J470" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K470" s="19"/>
       <c r="L470" s="18"/>
@@ -14795,22 +14802,22 @@
     </row>
     <row r="476" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A476" s="40" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="B476" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C476" s="14" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="D476" s="15" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="E476" s="15" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="F476" s="15" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="G476" s="16" t="s">
         <v>58</v>
@@ -14939,22 +14946,22 @@
     </row>
     <row r="482" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A482" s="40" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="B482" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C482" s="25" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="D482" s="26" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="E482" s="26" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="F482" s="26" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="G482" s="16" t="s">
         <v>58</v>
@@ -15083,22 +15090,22 @@
     </row>
     <row r="488" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A488" s="40" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="B488" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C488" s="14" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="D488" s="15" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="E488" s="15" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="F488" s="15" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="G488" s="16" t="s">
         <v>58</v>
@@ -15227,22 +15234,22 @@
     </row>
     <row r="494" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A494" s="40" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="B494" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C494" s="25" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="D494" s="26" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="E494" s="26" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="F494" s="26" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="G494" s="16" t="s">
         <v>58</v>
@@ -15371,22 +15378,22 @@
     </row>
     <row r="500" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A500" s="40" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="B500" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C500" s="14" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="D500" s="15" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="E500" s="15" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="F500" s="15" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="G500" s="16" t="s">
         <v>58</v>
@@ -15515,22 +15522,22 @@
     </row>
     <row r="506" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A506" s="40" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="B506" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C506" s="25" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="D506" s="26" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="E506" s="26" t="s">
         <v>251</v>
       </c>
       <c r="F506" s="26" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="G506" s="16" t="s">
         <v>58</v>
@@ -15659,22 +15666,22 @@
     </row>
     <row r="512" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A512" s="40" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="B512" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C512" s="14" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="D512" s="15" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="E512" s="15" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="F512" s="15" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="G512" s="16" t="s">
         <v>58</v>
@@ -15803,22 +15810,22 @@
     </row>
     <row r="518" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A518" s="40" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="B518" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C518" s="25" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="D518" s="26" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="E518" s="26" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="F518" s="26" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="G518" s="16" t="s">
         <v>58</v>
@@ -15947,22 +15954,22 @@
     </row>
     <row r="524" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A524" s="40" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="B524" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C524" s="14" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="D524" s="15" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="E524" s="15" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="F524" s="15" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="G524" s="16" t="s">
         <v>58</v>
@@ -16091,22 +16098,22 @@
     </row>
     <row r="530" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A530" s="40" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="B530" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C530" s="25" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="D530" s="26" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="E530" s="26" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="F530" s="26" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="G530" s="16" t="s">
         <v>58</v>
@@ -16235,22 +16242,22 @@
     </row>
     <row r="536" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A536" s="40" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="B536" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C536" s="14" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="D536" s="15" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="E536" s="15" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="F536" s="15" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="G536" s="16" t="s">
         <v>58</v>
@@ -16379,22 +16386,22 @@
     </row>
     <row r="542" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A542" s="41" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="B542" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C542" s="25" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="D542" s="26" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="E542" s="26" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="F542" s="26" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="G542" s="16" t="s">
         <v>58</v>
@@ -16523,22 +16530,22 @@
     </row>
     <row r="548" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A548" s="41" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="B548" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C548" s="14" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="D548" s="15" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="E548" s="15" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="F548" s="15" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="G548" s="16" t="s">
         <v>58</v>
@@ -16667,22 +16674,22 @@
     </row>
     <row r="554" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A554" s="41" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="B554" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C554" s="25" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="D554" s="26" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="E554" s="26" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="F554" s="26" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="G554" s="16" t="s">
         <v>58</v>
@@ -16811,22 +16818,22 @@
     </row>
     <row r="560" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A560" s="41" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="B560" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C560" s="14" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="D560" s="15" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="E560" s="15" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="F560" s="15" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="G560" s="16" t="s">
         <v>58</v>
@@ -16955,22 +16962,22 @@
     </row>
     <row r="566" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A566" s="41" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="B566" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C566" s="25" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="D566" s="26" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="E566" s="26" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="F566" s="26" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="G566" s="16" t="s">
         <v>58</v>
@@ -17099,22 +17106,22 @@
     </row>
     <row r="572" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A572" s="41" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="B572" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C572" s="14" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="D572" s="15" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="E572" s="15" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="F572" s="15" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="G572" s="16" t="s">
         <v>58</v>
@@ -17243,22 +17250,22 @@
     </row>
     <row r="578" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A578" s="41" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="B578" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C578" s="25" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="D578" s="26" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="E578" s="26" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="F578" s="26" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="G578" s="16" t="s">
         <v>58</v>
@@ -17387,22 +17394,22 @@
     </row>
     <row r="584" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A584" s="41" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="B584" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C584" s="14" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="D584" s="15" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="E584" s="15" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="F584" s="15" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="G584" s="16" t="s">
         <v>58</v>
@@ -17531,22 +17538,22 @@
     </row>
     <row r="590" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A590" s="41" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="B590" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C590" s="25" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="D590" s="26" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="E590" s="26" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="F590" s="26" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="G590" s="16" t="s">
         <v>58</v>
@@ -17675,22 +17682,22 @@
     </row>
     <row r="596" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A596" s="42" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="B596" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C596" s="14" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="D596" s="15" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="E596" s="15" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="F596" s="15" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="G596" s="16" t="s">
         <v>58</v>
@@ -18215,22 +18222,22 @@
     </row>
     <row r="620" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A620" s="42" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="B620" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C620" s="25" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="D620" s="26" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="E620" s="26" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="F620" s="26" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="G620" s="16" t="s">
         <v>58</v>
@@ -18359,22 +18366,22 @@
     </row>
     <row r="626" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A626" s="42" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="B626" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C626" s="14" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="D626" s="15" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="E626" s="15" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="F626" s="15" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="G626" s="16" t="s">
         <v>58</v>
@@ -18503,22 +18510,22 @@
     </row>
     <row r="632" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A632" s="42" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="B632" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C632" s="25" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="D632" s="26" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="E632" s="26" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="F632" s="26" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="G632" s="16" t="s">
         <v>58</v>
@@ -18647,22 +18654,22 @@
     </row>
     <row r="638" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A638" s="42" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="B638" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C638" s="14" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="D638" s="15" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="E638" s="15" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="F638" s="15" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="G638" s="16" t="s">
         <v>58</v>
@@ -18791,22 +18798,22 @@
     </row>
     <row r="644" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A644" s="43" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="B644" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C644" s="25" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="D644" s="26" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="E644" s="26" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="F644" s="26" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="G644" s="16" t="s">
         <v>58</v>
@@ -19331,22 +19338,22 @@
     </row>
     <row r="668" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A668" s="43" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="B668" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C668" s="14" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="D668" s="15" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="E668" s="15" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="F668" s="15" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="G668" s="16" t="s">
         <v>58</v>
@@ -19475,22 +19482,22 @@
     </row>
     <row r="674" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A674" s="43" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="B674" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C674" s="25" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="D674" s="26" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="E674" s="26" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="F674" s="26" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="G674" s="16" t="s">
         <v>58</v>
@@ -19619,22 +19626,22 @@
     </row>
     <row r="680" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A680" s="43" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="B680" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C680" s="14" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="D680" s="15" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="E680" s="15" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="F680" s="15" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="G680" s="16" t="s">
         <v>58</v>
@@ -19763,22 +19770,22 @@
     </row>
     <row r="686" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A686" s="43" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="B686" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C686" s="25" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="D686" s="26" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="E686" s="26" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="F686" s="26" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="G686" s="16" t="s">
         <v>58</v>
@@ -19907,22 +19914,22 @@
     </row>
     <row r="692" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A692" s="44" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="B692" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C692" s="14" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="D692" s="15" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="E692" s="15" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="F692" s="15" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="G692" s="16" t="s">
         <v>58</v>
@@ -20447,22 +20454,22 @@
     </row>
     <row r="716" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A716" s="44" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="B716" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C716" s="25" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="D716" s="26" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="E716" s="26" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="F716" s="26" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="G716" s="16" t="s">
         <v>58</v>
@@ -20591,22 +20598,22 @@
     </row>
     <row r="722" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A722" s="44" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="B722" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C722" s="14" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="D722" s="15" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="E722" s="15" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="F722" s="15" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="G722" s="16" t="s">
         <v>58</v>
@@ -20735,19 +20742,19 @@
     </row>
     <row r="728" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A728" s="44" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="B728" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C728" s="25" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="D728" s="26" t="s">
         <v>215</v>
       </c>
       <c r="E728" s="26" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="F728" s="26" t="s">
         <v>217</v>
@@ -20879,22 +20886,22 @@
     </row>
     <row r="734" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A734" s="45" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="B734" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C734" s="14" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="D734" s="15" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="E734" s="15" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="F734" s="15" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="G734" s="16" t="s">
         <v>58</v>
@@ -21023,22 +21030,22 @@
     </row>
     <row r="740" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A740" s="45" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="B740" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C740" s="25" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="D740" s="26" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="E740" s="26" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="F740" s="26" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="G740" s="16" t="s">
         <v>58</v>
@@ -21167,22 +21174,22 @@
     </row>
     <row r="746" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A746" s="45" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="B746" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C746" s="14" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="D746" s="15" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="E746" s="15" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="F746" s="15" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="G746" s="16" t="s">
         <v>58</v>
@@ -21311,22 +21318,22 @@
     </row>
     <row r="752" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A752" s="45" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="B752" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C752" s="25" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="D752" s="26" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="E752" s="26" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="F752" s="26" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="G752" s="16" t="s">
         <v>58</v>
@@ -21455,22 +21462,22 @@
     </row>
     <row r="758" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A758" s="45" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="B758" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C758" s="14" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="D758" s="15" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="E758" s="15" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="F758" s="15" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="G758" s="16" t="s">
         <v>58</v>
@@ -21599,22 +21606,22 @@
     </row>
     <row r="764" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A764" s="46" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="B764" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C764" s="25" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="D764" s="26" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="E764" s="26" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="F764" s="26" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="G764" s="16" t="s">
         <v>58</v>
@@ -21743,22 +21750,22 @@
     </row>
     <row r="770" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A770" s="46" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="B770" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C770" s="14" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="D770" s="15" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="E770" s="15" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="F770" s="15" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="G770" s="16" t="s">
         <v>58</v>
@@ -21887,22 +21894,22 @@
     </row>
     <row r="776" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A776" s="46" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="B776" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C776" s="25" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="D776" s="26" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="E776" s="26" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="F776" s="26" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="G776" s="16" t="s">
         <v>58</v>
@@ -22031,22 +22038,22 @@
     </row>
     <row r="782" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A782" s="46" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="B782" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C782" s="14" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="D782" s="15" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="E782" s="15" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="F782" s="15" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="G782" s="16" t="s">
         <v>58</v>
@@ -22175,22 +22182,22 @@
     </row>
     <row r="788" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A788" s="46" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="B788" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C788" s="25" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="D788" s="26" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="E788" s="26" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="F788" s="26" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="G788" s="16" t="s">
         <v>58</v>
@@ -22319,22 +22326,22 @@
     </row>
     <row r="794" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A794" s="46" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="B794" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C794" s="14" t="s">
+        <v>539</v>
+      </c>
+      <c r="D794" s="15" t="s">
+        <v>540</v>
+      </c>
+      <c r="E794" s="15" t="s">
+        <v>541</v>
+      </c>
+      <c r="F794" s="15" t="s">
         <v>538</v>
-      </c>
-      <c r="D794" s="15" t="s">
-        <v>539</v>
-      </c>
-      <c r="E794" s="15" t="s">
-        <v>540</v>
-      </c>
-      <c r="F794" s="15" t="s">
-        <v>537</v>
       </c>
       <c r="G794" s="16" t="s">
         <v>58</v>
@@ -22463,22 +22470,22 @@
     </row>
     <row r="800" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A800" s="46" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="B800" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C800" s="25" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="D800" s="26" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="E800" s="26" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="F800" s="26" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="G800" s="16" t="s">
         <v>58</v>
@@ -22607,22 +22614,22 @@
     </row>
     <row r="806" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A806" s="46" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="B806" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C806" s="14" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="D806" s="15" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="E806" s="15" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="F806" s="15" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="G806" s="16" t="s">
         <v>58</v>
@@ -22751,22 +22758,22 @@
     </row>
     <row r="812" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A812" s="46" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="B812" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C812" s="25" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="D812" s="26" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="E812" s="26" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="F812" s="26" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="G812" s="16" t="s">
         <v>58</v>
@@ -22895,22 +22902,22 @@
     </row>
     <row r="818" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A818" s="46" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="B818" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C818" s="14" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="D818" s="15" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="E818" s="15" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="F818" s="15" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="G818" s="16" t="s">
         <v>58</v>
@@ -23039,22 +23046,22 @@
     </row>
     <row r="824" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A824" s="46" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="B824" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C824" s="25" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="D824" s="26" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="E824" s="26" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="F824" s="26" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="G824" s="16" t="s">
         <v>58</v>
@@ -23183,22 +23190,22 @@
     </row>
     <row r="830" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A830" s="46" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="B830" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C830" s="14" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="D830" s="15" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="E830" s="15" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="F830" s="15" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="G830" s="16" t="s">
         <v>58</v>
@@ -23327,22 +23334,22 @@
     </row>
     <row r="836" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A836" s="47" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="B836" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C836" s="25" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="D836" s="26" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="E836" s="26" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="F836" s="26" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="G836" s="16" t="s">
         <v>58</v>
@@ -23471,22 +23478,22 @@
     </row>
     <row r="842" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A842" s="47" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="B842" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C842" s="14" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="D842" s="15" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="E842" s="15" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="F842" s="15" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="G842" s="16" t="s">
         <v>58</v>
@@ -23615,22 +23622,22 @@
     </row>
     <row r="848" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A848" s="47" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="B848" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C848" s="25" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="D848" s="26" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="E848" s="26" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="F848" s="26" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="G848" s="16" t="s">
         <v>58</v>
@@ -23759,22 +23766,22 @@
     </row>
     <row r="854" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A854" s="47" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="B854" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C854" s="14" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="D854" s="15" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="E854" s="15" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="F854" s="15" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="G854" s="16" t="s">
         <v>58</v>
@@ -23903,22 +23910,22 @@
     </row>
     <row r="860" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A860" s="48" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="B860" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C860" s="25" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="D860" s="26" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="E860" s="26" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="F860" s="26" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="G860" s="16" t="s">
         <v>58</v>
@@ -24047,22 +24054,22 @@
     </row>
     <row r="866" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A866" s="48" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="B866" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C866" s="14" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="D866" s="15" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="E866" s="15" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="F866" s="15" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="G866" s="16" t="s">
         <v>58</v>
@@ -24191,22 +24198,22 @@
     </row>
     <row r="872" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A872" s="48" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="B872" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C872" s="25" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="D872" s="26" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="E872" s="26" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="F872" s="26" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="G872" s="16" t="s">
         <v>58</v>
@@ -24335,22 +24342,22 @@
     </row>
     <row r="878" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A878" s="48" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="B878" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C878" s="14" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="D878" s="15" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="E878" s="15" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="F878" s="15" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="G878" s="16" t="s">
         <v>58</v>
@@ -24479,22 +24486,22 @@
     </row>
     <row r="884" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A884" s="48" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="B884" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C884" s="25" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="D884" s="26" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="E884" s="26" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="F884" s="26" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="G884" s="16" t="s">
         <v>58</v>
@@ -24623,22 +24630,22 @@
     </row>
     <row r="890" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A890" s="48" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="B890" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C890" s="14" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="D890" s="15" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="E890" s="15" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="F890" s="15" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="G890" s="16" t="s">
         <v>58</v>
@@ -24767,22 +24774,22 @@
     </row>
     <row r="896" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A896" s="48" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="B896" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C896" s="25" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="D896" s="26" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="E896" s="26" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="F896" s="26" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="G896" s="16" t="s">
         <v>58</v>
@@ -24911,22 +24918,22 @@
     </row>
     <row r="902" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A902" s="49" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="B902" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C902" s="14" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="D902" s="15" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="E902" s="15" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="F902" s="15" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="G902" s="16" t="s">
         <v>58</v>
@@ -25055,22 +25062,22 @@
     </row>
     <row r="908" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A908" s="49" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="B908" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C908" s="25" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="D908" s="26" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="E908" s="26" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="F908" s="26" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="G908" s="16" t="s">
         <v>58</v>
@@ -25199,22 +25206,22 @@
     </row>
     <row r="914" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A914" s="49" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="B914" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C914" s="14" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="D914" s="15" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="E914" s="15" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="F914" s="15" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="G914" s="16" t="s">
         <v>58</v>
@@ -25343,22 +25350,22 @@
     </row>
     <row r="920" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A920" s="49" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="B920" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C920" s="25" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="D920" s="26" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="E920" s="26" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="F920" s="26" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="G920" s="16" t="s">
         <v>58</v>
@@ -25487,22 +25494,22 @@
     </row>
     <row r="926" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A926" s="49" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="B926" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C926" s="14" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="D926" s="15" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="E926" s="15" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="F926" s="15" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="G926" s="16" t="s">
         <v>58</v>
@@ -25631,22 +25638,22 @@
     </row>
     <row r="932" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A932" s="49" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="B932" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C932" s="25" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="D932" s="26" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="E932" s="26" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="F932" s="26" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="G932" s="16" t="s">
         <v>58</v>
@@ -25775,22 +25782,22 @@
     </row>
     <row r="938" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A938" s="50" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="B938" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C938" s="14" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="D938" s="15" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="E938" s="15" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="F938" s="15" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="G938" s="16" t="s">
         <v>58</v>
@@ -25919,22 +25926,22 @@
     </row>
     <row r="944" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A944" s="50" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="B944" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C944" s="25" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="D944" s="26" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="E944" s="26" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="F944" s="26" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="G944" s="16" t="s">
         <v>58</v>
@@ -26063,22 +26070,22 @@
     </row>
     <row r="950" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A950" s="50" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="B950" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C950" s="14" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="D950" s="15" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="E950" s="15" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="F950" s="15" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="G950" s="16" t="s">
         <v>58</v>
@@ -26207,22 +26214,22 @@
     </row>
     <row r="956" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A956" s="50" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="B956" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C956" s="25" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="D956" s="26" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="E956" s="26" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="F956" s="26" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="G956" s="16" t="s">
         <v>58</v>
@@ -26351,22 +26358,22 @@
     </row>
     <row r="962" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A962" s="50" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="B962" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C962" s="14" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="D962" s="15" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="E962" s="15" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="F962" s="15" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="G962" s="16" t="s">
         <v>58</v>
@@ -26495,22 +26502,22 @@
     </row>
     <row r="968" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A968" s="50" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="B968" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C968" s="25" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="D968" s="26" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="E968" s="26" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="F968" s="26" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="G968" s="16" t="s">
         <v>58</v>
@@ -26639,22 +26646,22 @@
     </row>
     <row r="974" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A974" s="51" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="B974" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C974" s="14" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="D974" s="15" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="E974" s="15" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="F974" s="15" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="G974" s="16" t="s">
         <v>58</v>
@@ -26783,22 +26790,22 @@
     </row>
     <row r="980" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A980" s="51" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="B980" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C980" s="25" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="D980" s="26" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="E980" s="26" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="F980" s="26" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="G980" s="16" t="s">
         <v>58</v>
@@ -26927,22 +26934,22 @@
     </row>
     <row r="986" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A986" s="51" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="B986" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C986" s="14" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="D986" s="15" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="E986" s="15" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="F986" s="15" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="G986" s="16" t="s">
         <v>58</v>
@@ -27071,22 +27078,22 @@
     </row>
     <row r="992" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A992" s="51" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="B992" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C992" s="25" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="D992" s="26" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="E992" s="26" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="F992" s="26" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="G992" s="16" t="s">
         <v>58</v>
@@ -27215,22 +27222,22 @@
     </row>
     <row r="998" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A998" s="51" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="B998" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C998" s="14" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="D998" s="15" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="E998" s="15" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="F998" s="15" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="G998" s="16" t="s">
         <v>58</v>
@@ -27359,22 +27366,22 @@
     </row>
     <row r="1004" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1004" s="52" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="B1004" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1004" s="25" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="D1004" s="26" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="E1004" s="26" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="F1004" s="26" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="G1004" s="16" t="s">
         <v>58</v>
@@ -27503,22 +27510,22 @@
     </row>
     <row r="1010" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1010" s="52" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="B1010" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1010" s="14" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="D1010" s="15" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="E1010" s="15" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="F1010" s="15" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="G1010" s="16" t="s">
         <v>58</v>
@@ -27647,22 +27654,22 @@
     </row>
     <row r="1016" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1016" s="52" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="B1016" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1016" s="25" t="s">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="D1016" s="26" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="E1016" s="26" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="F1016" s="26" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="G1016" s="16" t="s">
         <v>58</v>
@@ -27791,22 +27798,22 @@
     </row>
     <row r="1022" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1022" s="52" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="B1022" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1022" s="14" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="D1022" s="15" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="E1022" s="15" t="s">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="F1022" s="15" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="G1022" s="16" t="s">
         <v>58</v>
@@ -27935,22 +27942,22 @@
     </row>
     <row r="1028" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1028" s="52" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="B1028" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C1028" s="25" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="D1028" s="26" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="E1028" s="26" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="F1028" s="26" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="G1028" s="16" t="s">
         <v>58</v>
@@ -28079,22 +28086,22 @@
     </row>
     <row r="1034" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1034" s="52" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="B1034" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C1034" s="14" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="D1034" s="15" t="s">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="E1034" s="15" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="F1034" s="15" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="G1034" s="16" t="s">
         <v>58</v>
@@ -28223,22 +28230,22 @@
     </row>
     <row r="1040" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1040" s="53" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="B1040" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C1040" s="25" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="D1040" s="26" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="E1040" s="26" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="F1040" s="26" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="G1040" s="16" t="s">
         <v>58</v>
@@ -28367,22 +28374,22 @@
     </row>
     <row r="1046" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1046" s="53" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="B1046" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1046" s="14" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="D1046" s="15" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="E1046" s="15" t="s">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="F1046" s="15" t="s">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="G1046" s="16" t="s">
         <v>58</v>
@@ -28517,16 +28524,16 @@
         <v>53</v>
       </c>
       <c r="C1052" s="25" t="s">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="D1052" s="26" t="s">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="E1052" s="26" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="F1052" s="26" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="G1052" s="16" t="s">
         <v>58</v>
@@ -28661,16 +28668,16 @@
         <v>53</v>
       </c>
       <c r="C1058" s="14" t="s">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="D1058" s="15" t="s">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="E1058" s="15" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="F1058" s="15" t="s">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="G1058" s="16" t="s">
         <v>58</v>
@@ -29756,10 +29763,10 @@
         <v>39</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>53</v>
@@ -29777,7 +29784,7 @@
         <v>86</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -29985,7 +29992,7 @@
     </row>
     <row r="9" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="61" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="B9" s="1">
         <v>11</v>
@@ -30014,7 +30021,7 @@
     </row>
     <row r="10" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="62" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="B10" s="1">
         <v>9</v>
@@ -30043,7 +30050,7 @@
     </row>
     <row r="11" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="63" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="B11" s="1">
         <v>5</v>
@@ -30072,7 +30079,7 @@
     </row>
     <row r="12" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="64" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="B12" s="1">
         <v>5</v>
@@ -30101,7 +30108,7 @@
     </row>
     <row r="13" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="65" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="B13" s="1">
         <v>4</v>
@@ -30130,7 +30137,7 @@
     </row>
     <row r="14" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="66" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="B14" s="1">
         <v>5</v>
@@ -30159,7 +30166,7 @@
     </row>
     <row r="15" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="67" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="B15" s="1">
         <v>12</v>
@@ -30188,7 +30195,7 @@
     </row>
     <row r="16" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="68" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="B16" s="1">
         <v>4</v>
@@ -30217,7 +30224,7 @@
     </row>
     <row r="17" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="69" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="B17" s="1">
         <v>7</v>
@@ -30246,7 +30253,7 @@
     </row>
     <row r="18" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="70" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="B18" s="1">
         <v>6</v>
@@ -30275,7 +30282,7 @@
     </row>
     <row r="19" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="71" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="B19" s="1">
         <v>6</v>
@@ -30304,7 +30311,7 @@
     </row>
     <row r="20" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="72" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="B20" s="1">
         <v>5</v>
@@ -30333,7 +30340,7 @@
     </row>
     <row r="21" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="73" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="B21" s="1">
         <v>6</v>
@@ -30362,7 +30369,7 @@
     </row>
     <row r="22" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="74" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="B22" s="1">
         <v>2</v>
@@ -30391,7 +30398,7 @@
     </row>
     <row r="23" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="75" t="s">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="B23" s="75">
         <v>153</v>
@@ -30442,7 +30449,7 @@
         <v>44</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="C1" s="10" t="s">
         <v>71</v>
@@ -30451,7 +30458,7 @@
         <v>86</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="F1" s="10" t="s">
         <v>94</v>
@@ -30602,10 +30609,10 @@
         <v>45</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>71</v>
@@ -30614,7 +30621,7 @@
         <v>86</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="G1" s="10" t="s">
         <v>94</v>
@@ -30625,7 +30632,7 @@
         <v>59</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="C2" s="1">
         <v>18</v>

</xml_diff>

<commit_message>
083 => fase IV => ZUP-065–075 OK (Chrome/USER), ZUP-076 KO perfil sense email/contrasenya i millores anotades
</commit_message>
<xml_diff>
--- a/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
+++ b/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4311" uniqueCount="727">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4321" uniqueCount="730">
   <si>
     <t>Zuppeto — Joc de probes manual (totes les pantalles)</t>
   </si>
@@ -1148,6 +1148,9 @@
     <t>Pantalla buida «Encara no tens favorits» + enllaç Explorar</t>
   </si>
   <si>
+    <t>Empty state OK. Millora (no bloqueja): a Favorits el botó de targeta diu «Guardat» i hauria de dir «Treure».</t>
+  </si>
+  <si>
     <t>ZUP-066</t>
   </si>
   <si>
@@ -1160,6 +1163,9 @@
     <t>Lloc apareix a la graella</t>
   </si>
   <si>
+    <t>El lloc apareix a Favorits. El botó de la targeta diu «Guardat» (millora: hauria de dir «Treure») però l’acció funciona.</t>
+  </si>
+  <si>
     <t>ZUP-067</t>
   </si>
   <si>
@@ -1278,6 +1284,10 @@
   </si>
   <si>
     <t>Heading perfil, avatar, email, rol, formulari</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La fitxa carrega (avatar NONE, email, rol User, formulari nom/ciutat/país/bio).
+KO de producte: no es pot canviar l’email ni la contrasenya. Cal afegir-ho al perfil.</t>
   </si>
   <si>
     <t>ZUP-077</t>
@@ -2249,7 +2259,7 @@
     </font>
     <font>
       <b/>
-      <color rgb="FF006100"/>
+      <color rgb="FF9C0006"/>
       <sz val="10"/>
       <name val="Calibri"/>
     </font>
@@ -2427,7 +2437,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
+        <fgColor rgb="FFFFC7CE"/>
       </patternFill>
     </fill>
     <fill>
@@ -14825,11 +14835,15 @@
       <c r="H476" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="I476" s="18"/>
+      <c r="I476" s="18" t="s">
+        <v>326</v>
+      </c>
       <c r="J476" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="K476" s="19"/>
+        <v>71</v>
+      </c>
+      <c r="K476" s="19" t="s">
+        <v>366</v>
+      </c>
       <c r="L476" s="18"/>
       <c r="M476" s="1"/>
       <c r="N476" s="19"/>
@@ -14952,16 +14966,16 @@
         <v>53</v>
       </c>
       <c r="C482" s="25" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="D482" s="26" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="E482" s="26" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="F482" s="26" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="G482" s="16" t="s">
         <v>58</v>
@@ -14969,11 +14983,15 @@
       <c r="H482" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="I482" s="18"/>
+      <c r="I482" s="18" t="s">
+        <v>326</v>
+      </c>
       <c r="J482" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="K482" s="19"/>
+        <v>71</v>
+      </c>
+      <c r="K482" s="19" t="s">
+        <v>371</v>
+      </c>
       <c r="L482" s="18"/>
       <c r="M482" s="1"/>
       <c r="N482" s="19"/>
@@ -15096,16 +15114,16 @@
         <v>53</v>
       </c>
       <c r="C488" s="14" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="D488" s="15" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="E488" s="15" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="F488" s="15" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="G488" s="16" t="s">
         <v>58</v>
@@ -15113,9 +15131,11 @@
       <c r="H488" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="I488" s="18"/>
+      <c r="I488" s="18" t="s">
+        <v>326</v>
+      </c>
       <c r="J488" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K488" s="19"/>
       <c r="L488" s="18"/>
@@ -15240,16 +15260,16 @@
         <v>89</v>
       </c>
       <c r="C494" s="25" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="D494" s="26" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="E494" s="26" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="F494" s="26" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="G494" s="16" t="s">
         <v>58</v>
@@ -15384,16 +15404,16 @@
         <v>89</v>
       </c>
       <c r="C500" s="14" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="D500" s="15" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="E500" s="15" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="F500" s="15" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="G500" s="16" t="s">
         <v>58</v>
@@ -15528,16 +15548,16 @@
         <v>89</v>
       </c>
       <c r="C506" s="25" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="D506" s="26" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="E506" s="26" t="s">
         <v>251</v>
       </c>
       <c r="F506" s="26" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="G506" s="16" t="s">
         <v>58</v>
@@ -15672,16 +15692,16 @@
         <v>89</v>
       </c>
       <c r="C512" s="14" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="D512" s="15" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="E512" s="15" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="F512" s="15" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="G512" s="16" t="s">
         <v>58</v>
@@ -15816,16 +15836,16 @@
         <v>89</v>
       </c>
       <c r="C518" s="25" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="D518" s="26" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="E518" s="26" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="F518" s="26" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="G518" s="16" t="s">
         <v>58</v>
@@ -15960,16 +15980,16 @@
         <v>53</v>
       </c>
       <c r="C524" s="14" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="D524" s="15" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="E524" s="15" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="F524" s="15" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="G524" s="16" t="s">
         <v>58</v>
@@ -15977,9 +15997,11 @@
       <c r="H524" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="I524" s="18"/>
+      <c r="I524" s="18" t="s">
+        <v>326</v>
+      </c>
       <c r="J524" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K524" s="19"/>
       <c r="L524" s="18"/>
@@ -16104,16 +16126,16 @@
         <v>53</v>
       </c>
       <c r="C530" s="25" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="D530" s="26" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="E530" s="26" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="F530" s="26" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="G530" s="16" t="s">
         <v>58</v>
@@ -16121,9 +16143,11 @@
       <c r="H530" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="I530" s="18"/>
+      <c r="I530" s="18" t="s">
+        <v>326</v>
+      </c>
       <c r="J530" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K530" s="19"/>
       <c r="L530" s="18"/>
@@ -16248,16 +16272,16 @@
         <v>53</v>
       </c>
       <c r="C536" s="14" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="D536" s="15" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="E536" s="15" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="F536" s="15" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="G536" s="16" t="s">
         <v>58</v>
@@ -16265,9 +16289,11 @@
       <c r="H536" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="I536" s="18"/>
+      <c r="I536" s="18" t="s">
+        <v>326</v>
+      </c>
       <c r="J536" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K536" s="19"/>
       <c r="L536" s="18"/>
@@ -16386,22 +16412,22 @@
     </row>
     <row r="542" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A542" s="41" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B542" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C542" s="25" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="D542" s="26" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="E542" s="26" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="F542" s="26" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="G542" s="16" t="s">
         <v>58</v>
@@ -16409,11 +16435,15 @@
       <c r="H542" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="I542" s="18"/>
+      <c r="I542" s="18" t="s">
+        <v>326</v>
+      </c>
       <c r="J542" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="K542" s="19"/>
+        <v>86</v>
+      </c>
+      <c r="K542" s="19" t="s">
+        <v>412</v>
+      </c>
       <c r="L542" s="18"/>
       <c r="M542" s="1"/>
       <c r="N542" s="19"/>
@@ -16530,22 +16560,22 @@
     </row>
     <row r="548" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A548" s="41" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B548" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C548" s="14" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="D548" s="15" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
       <c r="E548" s="15" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
       <c r="F548" s="15" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="G548" s="16" t="s">
         <v>58</v>
@@ -16674,22 +16704,22 @@
     </row>
     <row r="554" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A554" s="41" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B554" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C554" s="25" t="s">
-        <v>414</v>
+        <v>417</v>
       </c>
       <c r="D554" s="26" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
       <c r="E554" s="26" t="s">
-        <v>416</v>
+        <v>419</v>
       </c>
       <c r="F554" s="26" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="G554" s="16" t="s">
         <v>58</v>
@@ -16818,22 +16848,22 @@
     </row>
     <row r="560" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A560" s="41" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B560" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C560" s="14" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
       <c r="D560" s="15" t="s">
-        <v>419</v>
+        <v>422</v>
       </c>
       <c r="E560" s="15" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
       <c r="F560" s="15" t="s">
-        <v>421</v>
+        <v>424</v>
       </c>
       <c r="G560" s="16" t="s">
         <v>58</v>
@@ -16962,22 +16992,22 @@
     </row>
     <row r="566" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A566" s="41" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B566" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C566" s="25" t="s">
-        <v>422</v>
+        <v>425</v>
       </c>
       <c r="D566" s="26" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="E566" s="26" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="F566" s="26" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
       <c r="G566" s="16" t="s">
         <v>58</v>
@@ -17106,22 +17136,22 @@
     </row>
     <row r="572" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A572" s="41" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B572" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C572" s="14" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="D572" s="15" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="E572" s="15" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="F572" s="15" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="G572" s="16" t="s">
         <v>58</v>
@@ -17250,22 +17280,22 @@
     </row>
     <row r="578" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A578" s="41" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B578" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C578" s="25" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="D578" s="26" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="E578" s="26" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="F578" s="26" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
       <c r="G578" s="16" t="s">
         <v>58</v>
@@ -17394,22 +17424,22 @@
     </row>
     <row r="584" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A584" s="41" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B584" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C584" s="14" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="D584" s="15" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="E584" s="15" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
       <c r="F584" s="15" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="G584" s="16" t="s">
         <v>58</v>
@@ -17538,22 +17568,22 @@
     </row>
     <row r="590" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A590" s="41" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B590" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C590" s="25" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="D590" s="26" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
       <c r="E590" s="26" t="s">
-        <v>440</v>
+        <v>443</v>
       </c>
       <c r="F590" s="26" t="s">
-        <v>441</v>
+        <v>444</v>
       </c>
       <c r="G590" s="16" t="s">
         <v>58</v>
@@ -17682,22 +17712,22 @@
     </row>
     <row r="596" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A596" s="42" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="B596" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C596" s="14" t="s">
-        <v>443</v>
+        <v>446</v>
       </c>
       <c r="D596" s="15" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
       <c r="E596" s="15" t="s">
-        <v>445</v>
+        <v>448</v>
       </c>
       <c r="F596" s="15" t="s">
-        <v>446</v>
+        <v>449</v>
       </c>
       <c r="G596" s="16" t="s">
         <v>58</v>
@@ -18222,22 +18252,22 @@
     </row>
     <row r="620" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A620" s="42" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="B620" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C620" s="25" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="D620" s="26" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="E620" s="26" t="s">
-        <v>449</v>
+        <v>452</v>
       </c>
       <c r="F620" s="26" t="s">
-        <v>450</v>
+        <v>453</v>
       </c>
       <c r="G620" s="16" t="s">
         <v>58</v>
@@ -18366,22 +18396,22 @@
     </row>
     <row r="626" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A626" s="42" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="B626" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C626" s="14" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="D626" s="15" t="s">
-        <v>452</v>
+        <v>455</v>
       </c>
       <c r="E626" s="15" t="s">
-        <v>453</v>
+        <v>456</v>
       </c>
       <c r="F626" s="15" t="s">
-        <v>454</v>
+        <v>457</v>
       </c>
       <c r="G626" s="16" t="s">
         <v>58</v>
@@ -18510,22 +18540,22 @@
     </row>
     <row r="632" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A632" s="42" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="B632" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C632" s="25" t="s">
-        <v>455</v>
+        <v>458</v>
       </c>
       <c r="D632" s="26" t="s">
-        <v>456</v>
+        <v>459</v>
       </c>
       <c r="E632" s="26" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="F632" s="26" t="s">
-        <v>458</v>
+        <v>461</v>
       </c>
       <c r="G632" s="16" t="s">
         <v>58</v>
@@ -18654,22 +18684,22 @@
     </row>
     <row r="638" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A638" s="42" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="B638" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C638" s="14" t="s">
-        <v>459</v>
+        <v>462</v>
       </c>
       <c r="D638" s="15" t="s">
-        <v>460</v>
+        <v>463</v>
       </c>
       <c r="E638" s="15" t="s">
-        <v>461</v>
+        <v>464</v>
       </c>
       <c r="F638" s="15" t="s">
-        <v>462</v>
+        <v>465</v>
       </c>
       <c r="G638" s="16" t="s">
         <v>58</v>
@@ -18798,22 +18828,22 @@
     </row>
     <row r="644" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A644" s="43" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="B644" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C644" s="25" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="D644" s="26" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
       <c r="E644" s="26" t="s">
-        <v>466</v>
+        <v>469</v>
       </c>
       <c r="F644" s="26" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="G644" s="16" t="s">
         <v>58</v>
@@ -19338,22 +19368,22 @@
     </row>
     <row r="668" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A668" s="43" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="B668" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C668" s="14" t="s">
-        <v>468</v>
+        <v>471</v>
       </c>
       <c r="D668" s="15" t="s">
-        <v>469</v>
+        <v>472</v>
       </c>
       <c r="E668" s="15" t="s">
-        <v>470</v>
+        <v>473</v>
       </c>
       <c r="F668" s="15" t="s">
-        <v>471</v>
+        <v>474</v>
       </c>
       <c r="G668" s="16" t="s">
         <v>58</v>
@@ -19482,22 +19512,22 @@
     </row>
     <row r="674" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A674" s="43" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="B674" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C674" s="25" t="s">
-        <v>472</v>
+        <v>475</v>
       </c>
       <c r="D674" s="26" t="s">
-        <v>473</v>
+        <v>476</v>
       </c>
       <c r="E674" s="26" t="s">
-        <v>474</v>
+        <v>477</v>
       </c>
       <c r="F674" s="26" t="s">
-        <v>475</v>
+        <v>478</v>
       </c>
       <c r="G674" s="16" t="s">
         <v>58</v>
@@ -19626,22 +19656,22 @@
     </row>
     <row r="680" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A680" s="43" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="B680" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C680" s="14" t="s">
-        <v>476</v>
+        <v>479</v>
       </c>
       <c r="D680" s="15" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="E680" s="15" t="s">
-        <v>478</v>
+        <v>481</v>
       </c>
       <c r="F680" s="15" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="G680" s="16" t="s">
         <v>58</v>
@@ -19770,22 +19800,22 @@
     </row>
     <row r="686" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A686" s="43" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="B686" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C686" s="25" t="s">
-        <v>479</v>
+        <v>482</v>
       </c>
       <c r="D686" s="26" t="s">
-        <v>480</v>
+        <v>483</v>
       </c>
       <c r="E686" s="26" t="s">
-        <v>481</v>
+        <v>484</v>
       </c>
       <c r="F686" s="26" t="s">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="G686" s="16" t="s">
         <v>58</v>
@@ -19914,22 +19944,22 @@
     </row>
     <row r="692" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A692" s="44" t="s">
-        <v>483</v>
+        <v>486</v>
       </c>
       <c r="B692" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C692" s="14" t="s">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="D692" s="15" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="E692" s="15" t="s">
-        <v>486</v>
+        <v>489</v>
       </c>
       <c r="F692" s="15" t="s">
-        <v>487</v>
+        <v>490</v>
       </c>
       <c r="G692" s="16" t="s">
         <v>58</v>
@@ -20454,22 +20484,22 @@
     </row>
     <row r="716" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A716" s="44" t="s">
-        <v>483</v>
+        <v>486</v>
       </c>
       <c r="B716" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C716" s="25" t="s">
-        <v>488</v>
+        <v>491</v>
       </c>
       <c r="D716" s="26" t="s">
-        <v>489</v>
+        <v>492</v>
       </c>
       <c r="E716" s="26" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="F716" s="26" t="s">
-        <v>491</v>
+        <v>494</v>
       </c>
       <c r="G716" s="16" t="s">
         <v>58</v>
@@ -20598,22 +20628,22 @@
     </row>
     <row r="722" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A722" s="44" t="s">
-        <v>483</v>
+        <v>486</v>
       </c>
       <c r="B722" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C722" s="14" t="s">
-        <v>492</v>
+        <v>495</v>
       </c>
       <c r="D722" s="15" t="s">
-        <v>493</v>
+        <v>496</v>
       </c>
       <c r="E722" s="15" t="s">
-        <v>494</v>
+        <v>497</v>
       </c>
       <c r="F722" s="15" t="s">
-        <v>495</v>
+        <v>498</v>
       </c>
       <c r="G722" s="16" t="s">
         <v>58</v>
@@ -20742,19 +20772,19 @@
     </row>
     <row r="728" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A728" s="44" t="s">
-        <v>483</v>
+        <v>486</v>
       </c>
       <c r="B728" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C728" s="25" t="s">
-        <v>496</v>
+        <v>499</v>
       </c>
       <c r="D728" s="26" t="s">
         <v>215</v>
       </c>
       <c r="E728" s="26" t="s">
-        <v>494</v>
+        <v>497</v>
       </c>
       <c r="F728" s="26" t="s">
         <v>217</v>
@@ -20886,22 +20916,22 @@
     </row>
     <row r="734" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A734" s="45" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="B734" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C734" s="14" t="s">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="D734" s="15" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
       <c r="E734" s="15" t="s">
-        <v>500</v>
+        <v>503</v>
       </c>
       <c r="F734" s="15" t="s">
-        <v>501</v>
+        <v>504</v>
       </c>
       <c r="G734" s="16" t="s">
         <v>58</v>
@@ -21030,22 +21060,22 @@
     </row>
     <row r="740" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A740" s="45" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="B740" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C740" s="25" t="s">
-        <v>502</v>
+        <v>505</v>
       </c>
       <c r="D740" s="26" t="s">
-        <v>503</v>
+        <v>506</v>
       </c>
       <c r="E740" s="26" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
       <c r="F740" s="26" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="G740" s="16" t="s">
         <v>58</v>
@@ -21174,22 +21204,22 @@
     </row>
     <row r="746" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A746" s="45" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="B746" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C746" s="14" t="s">
-        <v>506</v>
+        <v>509</v>
       </c>
       <c r="D746" s="15" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="E746" s="15" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="F746" s="15" t="s">
-        <v>509</v>
+        <v>512</v>
       </c>
       <c r="G746" s="16" t="s">
         <v>58</v>
@@ -21318,22 +21348,22 @@
     </row>
     <row r="752" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A752" s="45" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="B752" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C752" s="25" t="s">
-        <v>510</v>
+        <v>513</v>
       </c>
       <c r="D752" s="26" t="s">
-        <v>511</v>
+        <v>514</v>
       </c>
       <c r="E752" s="26" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
       <c r="F752" s="26" t="s">
-        <v>513</v>
+        <v>516</v>
       </c>
       <c r="G752" s="16" t="s">
         <v>58</v>
@@ -21462,22 +21492,22 @@
     </row>
     <row r="758" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A758" s="45" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="B758" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C758" s="14" t="s">
-        <v>514</v>
+        <v>517</v>
       </c>
       <c r="D758" s="15" t="s">
-        <v>515</v>
+        <v>518</v>
       </c>
       <c r="E758" s="15" t="s">
-        <v>516</v>
+        <v>519</v>
       </c>
       <c r="F758" s="15" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
       <c r="G758" s="16" t="s">
         <v>58</v>
@@ -21606,22 +21636,22 @@
     </row>
     <row r="764" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A764" s="46" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="B764" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C764" s="25" t="s">
-        <v>519</v>
+        <v>522</v>
       </c>
       <c r="D764" s="26" t="s">
-        <v>520</v>
+        <v>523</v>
       </c>
       <c r="E764" s="26" t="s">
-        <v>521</v>
+        <v>524</v>
       </c>
       <c r="F764" s="26" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="G764" s="16" t="s">
         <v>58</v>
@@ -21750,22 +21780,22 @@
     </row>
     <row r="770" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A770" s="46" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="B770" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C770" s="14" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="D770" s="15" t="s">
-        <v>524</v>
+        <v>527</v>
       </c>
       <c r="E770" s="15" t="s">
-        <v>525</v>
+        <v>528</v>
       </c>
       <c r="F770" s="15" t="s">
-        <v>526</v>
+        <v>529</v>
       </c>
       <c r="G770" s="16" t="s">
         <v>58</v>
@@ -21894,22 +21924,22 @@
     </row>
     <row r="776" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A776" s="46" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="B776" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C776" s="25" t="s">
-        <v>527</v>
+        <v>530</v>
       </c>
       <c r="D776" s="26" t="s">
-        <v>528</v>
+        <v>531</v>
       </c>
       <c r="E776" s="26" t="s">
-        <v>529</v>
+        <v>532</v>
       </c>
       <c r="F776" s="26" t="s">
-        <v>530</v>
+        <v>533</v>
       </c>
       <c r="G776" s="16" t="s">
         <v>58</v>
@@ -22038,22 +22068,22 @@
     </row>
     <row r="782" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A782" s="46" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="B782" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C782" s="14" t="s">
-        <v>531</v>
+        <v>534</v>
       </c>
       <c r="D782" s="15" t="s">
-        <v>532</v>
+        <v>535</v>
       </c>
       <c r="E782" s="15" t="s">
-        <v>533</v>
+        <v>536</v>
       </c>
       <c r="F782" s="15" t="s">
-        <v>534</v>
+        <v>537</v>
       </c>
       <c r="G782" s="16" t="s">
         <v>58</v>
@@ -22182,22 +22212,22 @@
     </row>
     <row r="788" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A788" s="46" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="B788" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C788" s="25" t="s">
-        <v>535</v>
+        <v>538</v>
       </c>
       <c r="D788" s="26" t="s">
-        <v>536</v>
+        <v>539</v>
       </c>
       <c r="E788" s="26" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
       <c r="F788" s="26" t="s">
-        <v>538</v>
+        <v>541</v>
       </c>
       <c r="G788" s="16" t="s">
         <v>58</v>
@@ -22326,22 +22356,22 @@
     </row>
     <row r="794" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A794" s="46" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="B794" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C794" s="14" t="s">
-        <v>539</v>
+        <v>542</v>
       </c>
       <c r="D794" s="15" t="s">
-        <v>540</v>
+        <v>543</v>
       </c>
       <c r="E794" s="15" t="s">
+        <v>544</v>
+      </c>
+      <c r="F794" s="15" t="s">
         <v>541</v>
-      </c>
-      <c r="F794" s="15" t="s">
-        <v>538</v>
       </c>
       <c r="G794" s="16" t="s">
         <v>58</v>
@@ -22470,22 +22500,22 @@
     </row>
     <row r="800" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A800" s="46" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="B800" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C800" s="25" t="s">
-        <v>542</v>
+        <v>545</v>
       </c>
       <c r="D800" s="26" t="s">
-        <v>543</v>
+        <v>546</v>
       </c>
       <c r="E800" s="26" t="s">
-        <v>544</v>
+        <v>547</v>
       </c>
       <c r="F800" s="26" t="s">
-        <v>545</v>
+        <v>548</v>
       </c>
       <c r="G800" s="16" t="s">
         <v>58</v>
@@ -22614,22 +22644,22 @@
     </row>
     <row r="806" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A806" s="46" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="B806" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C806" s="14" t="s">
-        <v>546</v>
+        <v>549</v>
       </c>
       <c r="D806" s="15" t="s">
-        <v>547</v>
+        <v>550</v>
       </c>
       <c r="E806" s="15" t="s">
-        <v>548</v>
+        <v>551</v>
       </c>
       <c r="F806" s="15" t="s">
-        <v>549</v>
+        <v>552</v>
       </c>
       <c r="G806" s="16" t="s">
         <v>58</v>
@@ -22758,22 +22788,22 @@
     </row>
     <row r="812" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A812" s="46" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="B812" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C812" s="25" t="s">
-        <v>550</v>
+        <v>553</v>
       </c>
       <c r="D812" s="26" t="s">
-        <v>551</v>
+        <v>554</v>
       </c>
       <c r="E812" s="26" t="s">
-        <v>552</v>
+        <v>555</v>
       </c>
       <c r="F812" s="26" t="s">
-        <v>553</v>
+        <v>556</v>
       </c>
       <c r="G812" s="16" t="s">
         <v>58</v>
@@ -22902,22 +22932,22 @@
     </row>
     <row r="818" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A818" s="46" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="B818" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C818" s="14" t="s">
-        <v>554</v>
+        <v>557</v>
       </c>
       <c r="D818" s="15" t="s">
-        <v>555</v>
+        <v>558</v>
       </c>
       <c r="E818" s="15" t="s">
-        <v>556</v>
+        <v>559</v>
       </c>
       <c r="F818" s="15" t="s">
-        <v>557</v>
+        <v>560</v>
       </c>
       <c r="G818" s="16" t="s">
         <v>58</v>
@@ -23046,22 +23076,22 @@
     </row>
     <row r="824" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A824" s="46" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="B824" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C824" s="25" t="s">
-        <v>558</v>
+        <v>561</v>
       </c>
       <c r="D824" s="26" t="s">
-        <v>559</v>
+        <v>562</v>
       </c>
       <c r="E824" s="26" t="s">
-        <v>560</v>
+        <v>563</v>
       </c>
       <c r="F824" s="26" t="s">
-        <v>561</v>
+        <v>564</v>
       </c>
       <c r="G824" s="16" t="s">
         <v>58</v>
@@ -23190,22 +23220,22 @@
     </row>
     <row r="830" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A830" s="46" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="B830" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C830" s="14" t="s">
-        <v>562</v>
+        <v>565</v>
       </c>
       <c r="D830" s="15" t="s">
-        <v>563</v>
+        <v>566</v>
       </c>
       <c r="E830" s="15" t="s">
-        <v>564</v>
+        <v>567</v>
       </c>
       <c r="F830" s="15" t="s">
-        <v>565</v>
+        <v>568</v>
       </c>
       <c r="G830" s="16" t="s">
         <v>58</v>
@@ -23334,22 +23364,22 @@
     </row>
     <row r="836" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A836" s="47" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="B836" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C836" s="25" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="D836" s="26" t="s">
-        <v>568</v>
+        <v>571</v>
       </c>
       <c r="E836" s="26" t="s">
-        <v>569</v>
+        <v>572</v>
       </c>
       <c r="F836" s="26" t="s">
-        <v>570</v>
+        <v>573</v>
       </c>
       <c r="G836" s="16" t="s">
         <v>58</v>
@@ -23478,22 +23508,22 @@
     </row>
     <row r="842" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A842" s="47" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="B842" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C842" s="14" t="s">
-        <v>571</v>
+        <v>574</v>
       </c>
       <c r="D842" s="15" t="s">
-        <v>572</v>
+        <v>575</v>
       </c>
       <c r="E842" s="15" t="s">
-        <v>573</v>
+        <v>576</v>
       </c>
       <c r="F842" s="15" t="s">
-        <v>509</v>
+        <v>512</v>
       </c>
       <c r="G842" s="16" t="s">
         <v>58</v>
@@ -23622,22 +23652,22 @@
     </row>
     <row r="848" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A848" s="47" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="B848" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C848" s="25" t="s">
-        <v>574</v>
+        <v>577</v>
       </c>
       <c r="D848" s="26" t="s">
-        <v>575</v>
+        <v>578</v>
       </c>
       <c r="E848" s="26" t="s">
-        <v>576</v>
+        <v>579</v>
       </c>
       <c r="F848" s="26" t="s">
-        <v>577</v>
+        <v>580</v>
       </c>
       <c r="G848" s="16" t="s">
         <v>58</v>
@@ -23766,22 +23796,22 @@
     </row>
     <row r="854" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A854" s="47" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="B854" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C854" s="14" t="s">
-        <v>578</v>
+        <v>581</v>
       </c>
       <c r="D854" s="15" t="s">
-        <v>579</v>
+        <v>582</v>
       </c>
       <c r="E854" s="15" t="s">
-        <v>580</v>
+        <v>583</v>
       </c>
       <c r="F854" s="15" t="s">
-        <v>581</v>
+        <v>584</v>
       </c>
       <c r="G854" s="16" t="s">
         <v>58</v>
@@ -23910,22 +23940,22 @@
     </row>
     <row r="860" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A860" s="48" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="B860" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C860" s="25" t="s">
-        <v>583</v>
+        <v>586</v>
       </c>
       <c r="D860" s="26" t="s">
-        <v>584</v>
+        <v>587</v>
       </c>
       <c r="E860" s="26" t="s">
-        <v>585</v>
+        <v>588</v>
       </c>
       <c r="F860" s="26" t="s">
-        <v>586</v>
+        <v>589</v>
       </c>
       <c r="G860" s="16" t="s">
         <v>58</v>
@@ -24054,22 +24084,22 @@
     </row>
     <row r="866" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A866" s="48" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="B866" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C866" s="14" t="s">
-        <v>587</v>
+        <v>590</v>
       </c>
       <c r="D866" s="15" t="s">
-        <v>588</v>
+        <v>591</v>
       </c>
       <c r="E866" s="15" t="s">
-        <v>589</v>
+        <v>592</v>
       </c>
       <c r="F866" s="15" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="G866" s="16" t="s">
         <v>58</v>
@@ -24198,22 +24228,22 @@
     </row>
     <row r="872" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A872" s="48" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="B872" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C872" s="25" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
       <c r="D872" s="26" t="s">
-        <v>592</v>
+        <v>595</v>
       </c>
       <c r="E872" s="26" t="s">
-        <v>593</v>
+        <v>596</v>
       </c>
       <c r="F872" s="26" t="s">
-        <v>594</v>
+        <v>597</v>
       </c>
       <c r="G872" s="16" t="s">
         <v>58</v>
@@ -24342,22 +24372,22 @@
     </row>
     <row r="878" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A878" s="48" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="B878" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C878" s="14" t="s">
-        <v>595</v>
+        <v>598</v>
       </c>
       <c r="D878" s="15" t="s">
-        <v>596</v>
+        <v>599</v>
       </c>
       <c r="E878" s="15" t="s">
-        <v>597</v>
+        <v>600</v>
       </c>
       <c r="F878" s="15" t="s">
-        <v>598</v>
+        <v>601</v>
       </c>
       <c r="G878" s="16" t="s">
         <v>58</v>
@@ -24486,22 +24516,22 @@
     </row>
     <row r="884" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A884" s="48" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="B884" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C884" s="25" t="s">
-        <v>599</v>
+        <v>602</v>
       </c>
       <c r="D884" s="26" t="s">
-        <v>600</v>
+        <v>603</v>
       </c>
       <c r="E884" s="26" t="s">
-        <v>601</v>
+        <v>604</v>
       </c>
       <c r="F884" s="26" t="s">
-        <v>602</v>
+        <v>605</v>
       </c>
       <c r="G884" s="16" t="s">
         <v>58</v>
@@ -24630,22 +24660,22 @@
     </row>
     <row r="890" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A890" s="48" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="B890" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C890" s="14" t="s">
-        <v>603</v>
+        <v>606</v>
       </c>
       <c r="D890" s="15" t="s">
-        <v>604</v>
+        <v>607</v>
       </c>
       <c r="E890" s="15" t="s">
-        <v>605</v>
+        <v>608</v>
       </c>
       <c r="F890" s="15" t="s">
-        <v>606</v>
+        <v>609</v>
       </c>
       <c r="G890" s="16" t="s">
         <v>58</v>
@@ -24774,22 +24804,22 @@
     </row>
     <row r="896" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A896" s="48" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="B896" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C896" s="25" t="s">
-        <v>607</v>
+        <v>610</v>
       </c>
       <c r="D896" s="26" t="s">
-        <v>608</v>
+        <v>611</v>
       </c>
       <c r="E896" s="26" t="s">
-        <v>609</v>
+        <v>612</v>
       </c>
       <c r="F896" s="26" t="s">
-        <v>610</v>
+        <v>613</v>
       </c>
       <c r="G896" s="16" t="s">
         <v>58</v>
@@ -24918,22 +24948,22 @@
     </row>
     <row r="902" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A902" s="49" t="s">
-        <v>611</v>
+        <v>614</v>
       </c>
       <c r="B902" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C902" s="14" t="s">
-        <v>612</v>
+        <v>615</v>
       </c>
       <c r="D902" s="15" t="s">
-        <v>613</v>
+        <v>616</v>
       </c>
       <c r="E902" s="15" t="s">
-        <v>614</v>
+        <v>617</v>
       </c>
       <c r="F902" s="15" t="s">
-        <v>615</v>
+        <v>618</v>
       </c>
       <c r="G902" s="16" t="s">
         <v>58</v>
@@ -25062,22 +25092,22 @@
     </row>
     <row r="908" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A908" s="49" t="s">
-        <v>611</v>
+        <v>614</v>
       </c>
       <c r="B908" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C908" s="25" t="s">
-        <v>616</v>
+        <v>619</v>
       </c>
       <c r="D908" s="26" t="s">
-        <v>617</v>
+        <v>620</v>
       </c>
       <c r="E908" s="26" t="s">
-        <v>618</v>
+        <v>621</v>
       </c>
       <c r="F908" s="26" t="s">
-        <v>619</v>
+        <v>622</v>
       </c>
       <c r="G908" s="16" t="s">
         <v>58</v>
@@ -25206,22 +25236,22 @@
     </row>
     <row r="914" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A914" s="49" t="s">
-        <v>611</v>
+        <v>614</v>
       </c>
       <c r="B914" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C914" s="14" t="s">
-        <v>620</v>
+        <v>623</v>
       </c>
       <c r="D914" s="15" t="s">
-        <v>621</v>
+        <v>624</v>
       </c>
       <c r="E914" s="15" t="s">
-        <v>622</v>
+        <v>625</v>
       </c>
       <c r="F914" s="15" t="s">
-        <v>623</v>
+        <v>626</v>
       </c>
       <c r="G914" s="16" t="s">
         <v>58</v>
@@ -25350,22 +25380,22 @@
     </row>
     <row r="920" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A920" s="49" t="s">
-        <v>611</v>
+        <v>614</v>
       </c>
       <c r="B920" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C920" s="25" t="s">
-        <v>624</v>
+        <v>627</v>
       </c>
       <c r="D920" s="26" t="s">
-        <v>625</v>
+        <v>628</v>
       </c>
       <c r="E920" s="26" t="s">
-        <v>626</v>
+        <v>629</v>
       </c>
       <c r="F920" s="26" t="s">
-        <v>627</v>
+        <v>630</v>
       </c>
       <c r="G920" s="16" t="s">
         <v>58</v>
@@ -25494,22 +25524,22 @@
     </row>
     <row r="926" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A926" s="49" t="s">
-        <v>611</v>
+        <v>614</v>
       </c>
       <c r="B926" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C926" s="14" t="s">
-        <v>628</v>
+        <v>631</v>
       </c>
       <c r="D926" s="15" t="s">
-        <v>629</v>
+        <v>632</v>
       </c>
       <c r="E926" s="15" t="s">
-        <v>630</v>
+        <v>633</v>
       </c>
       <c r="F926" s="15" t="s">
-        <v>631</v>
+        <v>634</v>
       </c>
       <c r="G926" s="16" t="s">
         <v>58</v>
@@ -25638,22 +25668,22 @@
     </row>
     <row r="932" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A932" s="49" t="s">
-        <v>611</v>
+        <v>614</v>
       </c>
       <c r="B932" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C932" s="25" t="s">
-        <v>632</v>
+        <v>635</v>
       </c>
       <c r="D932" s="26" t="s">
-        <v>633</v>
+        <v>636</v>
       </c>
       <c r="E932" s="26" t="s">
-        <v>634</v>
+        <v>637</v>
       </c>
       <c r="F932" s="26" t="s">
-        <v>635</v>
+        <v>638</v>
       </c>
       <c r="G932" s="16" t="s">
         <v>58</v>
@@ -25782,22 +25812,22 @@
     </row>
     <row r="938" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A938" s="50" t="s">
-        <v>636</v>
+        <v>639</v>
       </c>
       <c r="B938" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C938" s="14" t="s">
-        <v>637</v>
+        <v>640</v>
       </c>
       <c r="D938" s="15" t="s">
-        <v>638</v>
+        <v>641</v>
       </c>
       <c r="E938" s="15" t="s">
-        <v>639</v>
+        <v>642</v>
       </c>
       <c r="F938" s="15" t="s">
-        <v>640</v>
+        <v>643</v>
       </c>
       <c r="G938" s="16" t="s">
         <v>58</v>
@@ -25926,22 +25956,22 @@
     </row>
     <row r="944" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A944" s="50" t="s">
-        <v>636</v>
+        <v>639</v>
       </c>
       <c r="B944" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C944" s="25" t="s">
-        <v>641</v>
+        <v>644</v>
       </c>
       <c r="D944" s="26" t="s">
-        <v>642</v>
+        <v>645</v>
       </c>
       <c r="E944" s="26" t="s">
-        <v>643</v>
+        <v>646</v>
       </c>
       <c r="F944" s="26" t="s">
-        <v>644</v>
+        <v>647</v>
       </c>
       <c r="G944" s="16" t="s">
         <v>58</v>
@@ -26070,22 +26100,22 @@
     </row>
     <row r="950" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A950" s="50" t="s">
-        <v>636</v>
+        <v>639</v>
       </c>
       <c r="B950" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C950" s="14" t="s">
-        <v>645</v>
+        <v>648</v>
       </c>
       <c r="D950" s="15" t="s">
-        <v>646</v>
+        <v>649</v>
       </c>
       <c r="E950" s="15" t="s">
-        <v>647</v>
+        <v>650</v>
       </c>
       <c r="F950" s="15" t="s">
-        <v>648</v>
+        <v>651</v>
       </c>
       <c r="G950" s="16" t="s">
         <v>58</v>
@@ -26214,22 +26244,22 @@
     </row>
     <row r="956" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A956" s="50" t="s">
-        <v>636</v>
+        <v>639</v>
       </c>
       <c r="B956" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C956" s="25" t="s">
-        <v>649</v>
+        <v>652</v>
       </c>
       <c r="D956" s="26" t="s">
-        <v>650</v>
+        <v>653</v>
       </c>
       <c r="E956" s="26" t="s">
-        <v>651</v>
+        <v>654</v>
       </c>
       <c r="F956" s="26" t="s">
-        <v>623</v>
+        <v>626</v>
       </c>
       <c r="G956" s="16" t="s">
         <v>58</v>
@@ -26358,22 +26388,22 @@
     </row>
     <row r="962" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A962" s="50" t="s">
-        <v>636</v>
+        <v>639</v>
       </c>
       <c r="B962" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C962" s="14" t="s">
-        <v>652</v>
+        <v>655</v>
       </c>
       <c r="D962" s="15" t="s">
-        <v>653</v>
+        <v>656</v>
       </c>
       <c r="E962" s="15" t="s">
-        <v>654</v>
+        <v>657</v>
       </c>
       <c r="F962" s="15" t="s">
-        <v>655</v>
+        <v>658</v>
       </c>
       <c r="G962" s="16" t="s">
         <v>58</v>
@@ -26502,22 +26532,22 @@
     </row>
     <row r="968" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A968" s="50" t="s">
-        <v>636</v>
+        <v>639</v>
       </c>
       <c r="B968" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C968" s="25" t="s">
-        <v>656</v>
+        <v>659</v>
       </c>
       <c r="D968" s="26" t="s">
-        <v>657</v>
+        <v>660</v>
       </c>
       <c r="E968" s="26" t="s">
-        <v>658</v>
+        <v>661</v>
       </c>
       <c r="F968" s="26" t="s">
-        <v>659</v>
+        <v>662</v>
       </c>
       <c r="G968" s="16" t="s">
         <v>58</v>
@@ -26646,22 +26676,22 @@
     </row>
     <row r="974" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A974" s="51" t="s">
-        <v>660</v>
+        <v>663</v>
       </c>
       <c r="B974" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C974" s="14" t="s">
-        <v>661</v>
+        <v>664</v>
       </c>
       <c r="D974" s="15" t="s">
-        <v>662</v>
+        <v>665</v>
       </c>
       <c r="E974" s="15" t="s">
-        <v>663</v>
+        <v>666</v>
       </c>
       <c r="F974" s="15" t="s">
-        <v>664</v>
+        <v>667</v>
       </c>
       <c r="G974" s="16" t="s">
         <v>58</v>
@@ -26790,22 +26820,22 @@
     </row>
     <row r="980" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A980" s="51" t="s">
-        <v>660</v>
+        <v>663</v>
       </c>
       <c r="B980" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C980" s="25" t="s">
-        <v>665</v>
+        <v>668</v>
       </c>
       <c r="D980" s="26" t="s">
-        <v>666</v>
+        <v>669</v>
       </c>
       <c r="E980" s="26" t="s">
-        <v>667</v>
+        <v>670</v>
       </c>
       <c r="F980" s="26" t="s">
-        <v>668</v>
+        <v>671</v>
       </c>
       <c r="G980" s="16" t="s">
         <v>58</v>
@@ -26934,22 +26964,22 @@
     </row>
     <row r="986" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A986" s="51" t="s">
-        <v>660</v>
+        <v>663</v>
       </c>
       <c r="B986" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C986" s="14" t="s">
-        <v>669</v>
+        <v>672</v>
       </c>
       <c r="D986" s="15" t="s">
-        <v>670</v>
+        <v>673</v>
       </c>
       <c r="E986" s="15" t="s">
-        <v>671</v>
+        <v>674</v>
       </c>
       <c r="F986" s="15" t="s">
-        <v>672</v>
+        <v>675</v>
       </c>
       <c r="G986" s="16" t="s">
         <v>58</v>
@@ -27078,22 +27108,22 @@
     </row>
     <row r="992" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A992" s="51" t="s">
-        <v>660</v>
+        <v>663</v>
       </c>
       <c r="B992" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C992" s="25" t="s">
-        <v>673</v>
+        <v>676</v>
       </c>
       <c r="D992" s="26" t="s">
-        <v>674</v>
+        <v>677</v>
       </c>
       <c r="E992" s="26" t="s">
-        <v>675</v>
+        <v>678</v>
       </c>
       <c r="F992" s="26" t="s">
-        <v>676</v>
+        <v>679</v>
       </c>
       <c r="G992" s="16" t="s">
         <v>58</v>
@@ -27222,22 +27252,22 @@
     </row>
     <row r="998" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A998" s="51" t="s">
-        <v>660</v>
+        <v>663</v>
       </c>
       <c r="B998" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C998" s="14" t="s">
-        <v>677</v>
+        <v>680</v>
       </c>
       <c r="D998" s="15" t="s">
-        <v>678</v>
+        <v>681</v>
       </c>
       <c r="E998" s="15" t="s">
-        <v>679</v>
+        <v>682</v>
       </c>
       <c r="F998" s="15" t="s">
-        <v>680</v>
+        <v>683</v>
       </c>
       <c r="G998" s="16" t="s">
         <v>58</v>
@@ -27366,22 +27396,22 @@
     </row>
     <row r="1004" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1004" s="52" t="s">
-        <v>681</v>
+        <v>684</v>
       </c>
       <c r="B1004" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1004" s="25" t="s">
-        <v>682</v>
+        <v>685</v>
       </c>
       <c r="D1004" s="26" t="s">
-        <v>683</v>
+        <v>686</v>
       </c>
       <c r="E1004" s="26" t="s">
-        <v>684</v>
+        <v>687</v>
       </c>
       <c r="F1004" s="26" t="s">
-        <v>685</v>
+        <v>688</v>
       </c>
       <c r="G1004" s="16" t="s">
         <v>58</v>
@@ -27510,22 +27540,22 @@
     </row>
     <row r="1010" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1010" s="52" t="s">
-        <v>681</v>
+        <v>684</v>
       </c>
       <c r="B1010" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1010" s="14" t="s">
-        <v>686</v>
+        <v>689</v>
       </c>
       <c r="D1010" s="15" t="s">
-        <v>687</v>
+        <v>690</v>
       </c>
       <c r="E1010" s="15" t="s">
-        <v>688</v>
+        <v>691</v>
       </c>
       <c r="F1010" s="15" t="s">
-        <v>689</v>
+        <v>692</v>
       </c>
       <c r="G1010" s="16" t="s">
         <v>58</v>
@@ -27654,22 +27684,22 @@
     </row>
     <row r="1016" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1016" s="52" t="s">
-        <v>681</v>
+        <v>684</v>
       </c>
       <c r="B1016" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1016" s="25" t="s">
-        <v>690</v>
+        <v>693</v>
       </c>
       <c r="D1016" s="26" t="s">
-        <v>691</v>
+        <v>694</v>
       </c>
       <c r="E1016" s="26" t="s">
-        <v>692</v>
+        <v>695</v>
       </c>
       <c r="F1016" s="26" t="s">
-        <v>693</v>
+        <v>696</v>
       </c>
       <c r="G1016" s="16" t="s">
         <v>58</v>
@@ -27798,22 +27828,22 @@
     </row>
     <row r="1022" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1022" s="52" t="s">
-        <v>681</v>
+        <v>684</v>
       </c>
       <c r="B1022" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1022" s="14" t="s">
-        <v>694</v>
+        <v>697</v>
       </c>
       <c r="D1022" s="15" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="E1022" s="15" t="s">
-        <v>696</v>
+        <v>699</v>
       </c>
       <c r="F1022" s="15" t="s">
-        <v>697</v>
+        <v>700</v>
       </c>
       <c r="G1022" s="16" t="s">
         <v>58</v>
@@ -27942,22 +27972,22 @@
     </row>
     <row r="1028" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1028" s="52" t="s">
-        <v>681</v>
+        <v>684</v>
       </c>
       <c r="B1028" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C1028" s="25" t="s">
-        <v>698</v>
+        <v>701</v>
       </c>
       <c r="D1028" s="26" t="s">
-        <v>699</v>
+        <v>702</v>
       </c>
       <c r="E1028" s="26" t="s">
-        <v>700</v>
+        <v>703</v>
       </c>
       <c r="F1028" s="26" t="s">
-        <v>701</v>
+        <v>704</v>
       </c>
       <c r="G1028" s="16" t="s">
         <v>58</v>
@@ -28086,22 +28116,22 @@
     </row>
     <row r="1034" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1034" s="52" t="s">
-        <v>681</v>
+        <v>684</v>
       </c>
       <c r="B1034" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C1034" s="14" t="s">
-        <v>702</v>
+        <v>705</v>
       </c>
       <c r="D1034" s="15" t="s">
-        <v>703</v>
+        <v>706</v>
       </c>
       <c r="E1034" s="15" t="s">
-        <v>704</v>
+        <v>707</v>
       </c>
       <c r="F1034" s="15" t="s">
-        <v>705</v>
+        <v>708</v>
       </c>
       <c r="G1034" s="16" t="s">
         <v>58</v>
@@ -28230,22 +28260,22 @@
     </row>
     <row r="1040" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1040" s="53" t="s">
-        <v>706</v>
+        <v>709</v>
       </c>
       <c r="B1040" s="29" t="s">
         <v>89</v>
       </c>
       <c r="C1040" s="25" t="s">
-        <v>707</v>
+        <v>710</v>
       </c>
       <c r="D1040" s="26" t="s">
-        <v>695</v>
+        <v>698</v>
       </c>
       <c r="E1040" s="26" t="s">
-        <v>708</v>
+        <v>711</v>
       </c>
       <c r="F1040" s="26" t="s">
-        <v>709</v>
+        <v>712</v>
       </c>
       <c r="G1040" s="16" t="s">
         <v>58</v>
@@ -28374,22 +28404,22 @@
     </row>
     <row r="1046" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1046" s="53" t="s">
-        <v>706</v>
+        <v>709</v>
       </c>
       <c r="B1046" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1046" s="14" t="s">
-        <v>710</v>
+        <v>713</v>
       </c>
       <c r="D1046" s="15" t="s">
-        <v>687</v>
+        <v>690</v>
       </c>
       <c r="E1046" s="15" t="s">
-        <v>711</v>
+        <v>714</v>
       </c>
       <c r="F1046" s="15" t="s">
-        <v>712</v>
+        <v>715</v>
       </c>
       <c r="G1046" s="16" t="s">
         <v>58</v>
@@ -28524,16 +28554,16 @@
         <v>53</v>
       </c>
       <c r="C1052" s="25" t="s">
-        <v>713</v>
+        <v>716</v>
       </c>
       <c r="D1052" s="26" t="s">
-        <v>714</v>
+        <v>717</v>
       </c>
       <c r="E1052" s="26" t="s">
-        <v>715</v>
+        <v>718</v>
       </c>
       <c r="F1052" s="26" t="s">
-        <v>716</v>
+        <v>719</v>
       </c>
       <c r="G1052" s="16" t="s">
         <v>58</v>
@@ -28668,16 +28698,16 @@
         <v>53</v>
       </c>
       <c r="C1058" s="14" t="s">
-        <v>717</v>
+        <v>720</v>
       </c>
       <c r="D1058" s="15" t="s">
-        <v>718</v>
+        <v>721</v>
       </c>
       <c r="E1058" s="15" t="s">
-        <v>719</v>
+        <v>722</v>
       </c>
       <c r="F1058" s="15" t="s">
-        <v>720</v>
+        <v>723</v>
       </c>
       <c r="G1058" s="16" t="s">
         <v>58</v>
@@ -29763,10 +29793,10 @@
         <v>39</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>721</v>
+        <v>724</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>53</v>
@@ -29784,7 +29814,7 @@
         <v>86</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>723</v>
+        <v>726</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -30021,7 +30051,7 @@
     </row>
     <row r="10" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="62" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="B10" s="1">
         <v>9</v>
@@ -30050,7 +30080,7 @@
     </row>
     <row r="11" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="63" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="B11" s="1">
         <v>5</v>
@@ -30079,7 +30109,7 @@
     </row>
     <row r="12" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="64" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="B12" s="1">
         <v>5</v>
@@ -30108,7 +30138,7 @@
     </row>
     <row r="13" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="65" t="s">
-        <v>483</v>
+        <v>486</v>
       </c>
       <c r="B13" s="1">
         <v>4</v>
@@ -30137,7 +30167,7 @@
     </row>
     <row r="14" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="66" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="B14" s="1">
         <v>5</v>
@@ -30166,7 +30196,7 @@
     </row>
     <row r="15" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="67" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="B15" s="1">
         <v>12</v>
@@ -30195,7 +30225,7 @@
     </row>
     <row r="16" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="68" t="s">
-        <v>566</v>
+        <v>569</v>
       </c>
       <c r="B16" s="1">
         <v>4</v>
@@ -30224,7 +30254,7 @@
     </row>
     <row r="17" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="69" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="B17" s="1">
         <v>7</v>
@@ -30253,7 +30283,7 @@
     </row>
     <row r="18" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="70" t="s">
-        <v>611</v>
+        <v>614</v>
       </c>
       <c r="B18" s="1">
         <v>6</v>
@@ -30282,7 +30312,7 @@
     </row>
     <row r="19" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="71" t="s">
-        <v>636</v>
+        <v>639</v>
       </c>
       <c r="B19" s="1">
         <v>6</v>
@@ -30311,7 +30341,7 @@
     </row>
     <row r="20" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="72" t="s">
-        <v>660</v>
+        <v>663</v>
       </c>
       <c r="B20" s="1">
         <v>5</v>
@@ -30340,7 +30370,7 @@
     </row>
     <row r="21" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="73" t="s">
-        <v>681</v>
+        <v>684</v>
       </c>
       <c r="B21" s="1">
         <v>6</v>
@@ -30369,7 +30399,7 @@
     </row>
     <row r="22" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="74" t="s">
-        <v>706</v>
+        <v>709</v>
       </c>
       <c r="B22" s="1">
         <v>2</v>
@@ -30398,7 +30428,7 @@
     </row>
     <row r="23" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="75" t="s">
-        <v>724</v>
+        <v>727</v>
       </c>
       <c r="B23" s="75">
         <v>153</v>
@@ -30449,7 +30479,7 @@
         <v>44</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="C1" s="10" t="s">
         <v>71</v>
@@ -30458,7 +30488,7 @@
         <v>86</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>723</v>
+        <v>726</v>
       </c>
       <c r="F1" s="10" t="s">
         <v>94</v>
@@ -30609,10 +30639,10 @@
         <v>45</v>
       </c>
       <c r="B1" s="10" t="s">
+        <v>728</v>
+      </c>
+      <c r="C1" s="10" t="s">
         <v>725</v>
-      </c>
-      <c r="C1" s="10" t="s">
-        <v>722</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>71</v>
@@ -30621,7 +30651,7 @@
         <v>86</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>723</v>
+        <v>726</v>
       </c>
       <c r="G1" s="10" t="s">
         <v>94</v>
@@ -30632,7 +30662,7 @@
         <v>59</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>726</v>
+        <v>729</v>
       </c>
       <c r="C2" s="1">
         <v>18</v>

</xml_diff>

<commit_message>
085 => fase IV => ZUP-078 OK (Chrome/USER) i perfil no desa amb Enter
</commit_message>
<xml_diff>
--- a/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
+++ b/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
@@ -16748,9 +16748,11 @@
       <c r="H554" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="I554" s="18"/>
+      <c r="I554" s="18">
+        <v>46264.91666666667</v>
+      </c>
       <c r="J554" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K554" s="19"/>
       <c r="L554" s="18"/>

</xml_diff>

<commit_message>
086 => fase IV => ZUP-082 ZUP-084–087 OK (Chrome/USER), notificacions persistides i noves no llegides
</commit_message>
<xml_diff>
--- a/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
+++ b/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4323" uniqueCount="731">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4326" uniqueCount="733">
   <si>
     <t>Zuppeto — Joc de probes manual (totes les pantalles)</t>
   </si>
@@ -1428,6 +1428,19 @@
   </si>
   <si>
     <t>Pantalla buida «No hi ha notificacions»</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La safata tenia avisos (perfil, sessió tancada) amb l’usuari ja logat.
+Després de recarregar, la llista quedava buida (les notificacions són només memòria, no el login).
+KO: després de tancar sessió i tornar a entrar, seguia sortint «Sessió tancada» tot i estar autenticat.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Què s'ha fet:
+- src/Web/src/app/core/services/error-notifications.service.ts — safata per compte a localStorage; nova sempre No llegida; no es desa «Sessió tancada»
+- src/Web/src/app/features/auth/services/auth.service.ts — loadForUser al login / unload al logout
+- src/Web/src/app/core/layout/components/app-toast-stack/app-toast-stack.component.ts — el toast no marca com a llegida
+- src/Web/src/app/features/auth/pages/profile-page/profile-page.component.ts — logout sense avís «Sessió tancada»
+- docs/ca/funcional-ca.md, docs/ca/tecnic-ca.md</t>
   </si>
   <si>
     <t>ZUP-086</t>
@@ -2788,7 +2801,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -17326,9 +17339,11 @@
       <c r="H578" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="I578" s="18"/>
+      <c r="I578" s="18">
+        <v>46264.91666666667</v>
+      </c>
       <c r="J578" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K578" s="19"/>
       <c r="L578" s="18"/>
@@ -17614,9 +17629,11 @@
       <c r="H590" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="I590" s="18"/>
+      <c r="I590" s="18">
+        <v>46264.91666666667</v>
+      </c>
       <c r="J590" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K590" s="19"/>
       <c r="L590" s="18"/>
@@ -17877,7 +17894,7 @@
       <c r="M601" s="1"/>
       <c r="N601" s="19"/>
     </row>
-    <row r="602" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="602" ht="110" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A602" s="41"/>
       <c r="B602" s="13"/>
       <c r="C602" s="14"/>
@@ -17890,14 +17907,24 @@
       <c r="H602" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="I602" s="18"/>
+      <c r="I602" s="18">
+        <v>46264.91666666667</v>
+      </c>
       <c r="J602" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="K602" s="19"/>
-      <c r="L602" s="18"/>
-      <c r="M602" s="1"/>
-      <c r="N602" s="19"/>
+        <v>86</v>
+      </c>
+      <c r="K602" s="19" t="s">
+        <v>451</v>
+      </c>
+      <c r="L602" s="18">
+        <v>46264.91666666667</v>
+      </c>
+      <c r="M602" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="N602" s="19" t="s">
+        <v>452</v>
+      </c>
     </row>
     <row r="603" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A603" s="41"/>
@@ -18281,16 +18308,16 @@
         <v>53</v>
       </c>
       <c r="C620" s="25" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="D620" s="26" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="E620" s="26" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="F620" s="26" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="G620" s="16" t="s">
         <v>58</v>
@@ -18298,9 +18325,11 @@
       <c r="H620" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="I620" s="18"/>
+      <c r="I620" s="18">
+        <v>46264.91666666667</v>
+      </c>
       <c r="J620" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K620" s="19"/>
       <c r="L620" s="18"/>
@@ -18425,16 +18454,16 @@
         <v>53</v>
       </c>
       <c r="C626" s="14" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="D626" s="15" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="E626" s="15" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="F626" s="15" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="G626" s="16" t="s">
         <v>58</v>
@@ -18442,9 +18471,11 @@
       <c r="H626" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="I626" s="18"/>
+      <c r="I626" s="18">
+        <v>46264.91666666667</v>
+      </c>
       <c r="J626" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K626" s="19"/>
       <c r="L626" s="18"/>
@@ -18569,16 +18600,16 @@
         <v>89</v>
       </c>
       <c r="C632" s="25" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="D632" s="26" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="E632" s="26" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="F632" s="26" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="G632" s="16" t="s">
         <v>58</v>
@@ -18713,16 +18744,16 @@
         <v>53</v>
       </c>
       <c r="C638" s="14" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="D638" s="15" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="E638" s="15" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="F638" s="15" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="G638" s="16" t="s">
         <v>58</v>
@@ -18851,22 +18882,22 @@
     </row>
     <row r="644" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A644" s="42" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="B644" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C644" s="25" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="D644" s="26" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="E644" s="26" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="F644" s="26" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="G644" s="16" t="s">
         <v>58</v>
@@ -19391,22 +19422,22 @@
     </row>
     <row r="668" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A668" s="42" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="B668" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C668" s="14" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="D668" s="15" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="E668" s="15" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="F668" s="15" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="G668" s="16" t="s">
         <v>58</v>
@@ -19535,22 +19566,22 @@
     </row>
     <row r="674" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A674" s="42" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="B674" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C674" s="25" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="D674" s="26" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="E674" s="26" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="F674" s="26" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="G674" s="16" t="s">
         <v>58</v>
@@ -19679,19 +19710,19 @@
     </row>
     <row r="680" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A680" s="42" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="B680" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C680" s="14" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="D680" s="15" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="E680" s="15" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="F680" s="15" t="s">
         <v>406</v>
@@ -19823,22 +19854,22 @@
     </row>
     <row r="686" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A686" s="42" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="B686" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C686" s="25" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="D686" s="26" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="E686" s="26" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="F686" s="26" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="G686" s="16" t="s">
         <v>58</v>
@@ -19967,22 +19998,22 @@
     </row>
     <row r="692" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A692" s="43" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="B692" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C692" s="14" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="D692" s="15" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="E692" s="15" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="F692" s="15" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="G692" s="16" t="s">
         <v>58</v>
@@ -20507,22 +20538,22 @@
     </row>
     <row r="716" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A716" s="43" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="B716" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C716" s="25" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="D716" s="26" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="E716" s="26" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="F716" s="26" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="G716" s="16" t="s">
         <v>58</v>
@@ -20651,22 +20682,22 @@
     </row>
     <row r="722" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A722" s="43" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="B722" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C722" s="14" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="D722" s="15" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="E722" s="15" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="F722" s="15" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="G722" s="16" t="s">
         <v>58</v>
@@ -20795,19 +20826,19 @@
     </row>
     <row r="728" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A728" s="43" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="B728" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C728" s="25" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="D728" s="26" t="s">
         <v>215</v>
       </c>
       <c r="E728" s="26" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="F728" s="26" t="s">
         <v>217</v>
@@ -20939,22 +20970,22 @@
     </row>
     <row r="734" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A734" s="44" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="B734" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C734" s="14" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="D734" s="15" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="E734" s="15" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="F734" s="15" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="G734" s="16" t="s">
         <v>58</v>
@@ -21083,22 +21114,22 @@
     </row>
     <row r="740" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A740" s="44" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="B740" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C740" s="25" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="D740" s="26" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="E740" s="26" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="F740" s="26" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="G740" s="16" t="s">
         <v>58</v>
@@ -21227,22 +21258,22 @@
     </row>
     <row r="746" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A746" s="44" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="B746" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C746" s="14" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="D746" s="15" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="E746" s="15" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="F746" s="15" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="G746" s="16" t="s">
         <v>58</v>
@@ -21371,22 +21402,22 @@
     </row>
     <row r="752" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A752" s="44" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="B752" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C752" s="25" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="D752" s="26" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="E752" s="26" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="F752" s="26" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="G752" s="16" t="s">
         <v>58</v>
@@ -21515,22 +21546,22 @@
     </row>
     <row r="758" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A758" s="44" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="B758" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C758" s="14" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="D758" s="15" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="E758" s="15" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="F758" s="15" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="G758" s="16" t="s">
         <v>58</v>
@@ -21659,22 +21690,22 @@
     </row>
     <row r="764" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A764" s="45" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="B764" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C764" s="25" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="D764" s="26" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="E764" s="26" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="F764" s="26" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="G764" s="16" t="s">
         <v>58</v>
@@ -21803,22 +21834,22 @@
     </row>
     <row r="770" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A770" s="45" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="B770" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C770" s="14" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="D770" s="15" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="E770" s="15" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="F770" s="15" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="G770" s="16" t="s">
         <v>58</v>
@@ -21947,22 +21978,22 @@
     </row>
     <row r="776" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A776" s="45" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="B776" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C776" s="25" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="D776" s="26" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="E776" s="26" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="F776" s="26" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="G776" s="16" t="s">
         <v>58</v>
@@ -22091,22 +22122,22 @@
     </row>
     <row r="782" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A782" s="45" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="B782" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C782" s="14" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="D782" s="15" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="E782" s="15" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="F782" s="15" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="G782" s="16" t="s">
         <v>58</v>
@@ -22235,22 +22266,22 @@
     </row>
     <row r="788" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A788" s="45" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="B788" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C788" s="25" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="D788" s="26" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="E788" s="26" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="F788" s="26" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="G788" s="16" t="s">
         <v>58</v>
@@ -22379,22 +22410,22 @@
     </row>
     <row r="794" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A794" s="45" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="B794" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C794" s="14" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="D794" s="15" t="s">
+        <v>546</v>
+      </c>
+      <c r="E794" s="15" t="s">
+        <v>547</v>
+      </c>
+      <c r="F794" s="15" t="s">
         <v>544</v>
-      </c>
-      <c r="E794" s="15" t="s">
-        <v>545</v>
-      </c>
-      <c r="F794" s="15" t="s">
-        <v>542</v>
       </c>
       <c r="G794" s="16" t="s">
         <v>58</v>
@@ -22523,22 +22554,22 @@
     </row>
     <row r="800" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A800" s="45" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="B800" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C800" s="25" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="D800" s="26" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="E800" s="26" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="F800" s="26" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="G800" s="16" t="s">
         <v>58</v>
@@ -22667,22 +22698,22 @@
     </row>
     <row r="806" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A806" s="45" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="B806" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C806" s="14" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="D806" s="15" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="E806" s="15" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="F806" s="15" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="G806" s="16" t="s">
         <v>58</v>
@@ -22811,22 +22842,22 @@
     </row>
     <row r="812" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A812" s="45" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="B812" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C812" s="25" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="D812" s="26" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="E812" s="26" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="F812" s="26" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
       <c r="G812" s="16" t="s">
         <v>58</v>
@@ -22955,22 +22986,22 @@
     </row>
     <row r="818" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A818" s="45" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="B818" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C818" s="14" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="D818" s="15" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="E818" s="15" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="F818" s="15" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
       <c r="G818" s="16" t="s">
         <v>58</v>
@@ -23099,22 +23130,22 @@
     </row>
     <row r="824" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A824" s="45" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="B824" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C824" s="25" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
       <c r="D824" s="26" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
       <c r="E824" s="26" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="F824" s="26" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="G824" s="16" t="s">
         <v>58</v>
@@ -23243,22 +23274,22 @@
     </row>
     <row r="830" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A830" s="45" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="B830" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C830" s="14" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="D830" s="15" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
       <c r="E830" s="15" t="s">
-        <v>568</v>
+        <v>570</v>
       </c>
       <c r="F830" s="15" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="G830" s="16" t="s">
         <v>58</v>
@@ -23387,22 +23418,22 @@
     </row>
     <row r="836" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A836" s="46" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
       <c r="B836" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C836" s="25" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
       <c r="D836" s="26" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
       <c r="E836" s="26" t="s">
-        <v>573</v>
+        <v>575</v>
       </c>
       <c r="F836" s="26" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="G836" s="16" t="s">
         <v>58</v>
@@ -23531,22 +23562,22 @@
     </row>
     <row r="842" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A842" s="46" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
       <c r="B842" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C842" s="14" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="D842" s="15" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="E842" s="15" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="F842" s="15" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="G842" s="16" t="s">
         <v>58</v>
@@ -23675,22 +23706,22 @@
     </row>
     <row r="848" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A848" s="46" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
       <c r="B848" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C848" s="25" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D848" s="26" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E848" s="26" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="F848" s="26" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G848" s="16" t="s">
         <v>58</v>
@@ -23819,22 +23850,22 @@
     </row>
     <row r="854" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A854" s="46" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
       <c r="B854" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C854" s="14" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="D854" s="15" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="E854" s="15" t="s">
-        <v>584</v>
+        <v>586</v>
       </c>
       <c r="F854" s="15" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
       <c r="G854" s="16" t="s">
         <v>58</v>
@@ -23963,22 +23994,22 @@
     </row>
     <row r="860" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A860" s="47" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
       <c r="B860" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C860" s="25" t="s">
-        <v>587</v>
+        <v>589</v>
       </c>
       <c r="D860" s="26" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="E860" s="26" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="F860" s="26" t="s">
-        <v>590</v>
+        <v>592</v>
       </c>
       <c r="G860" s="16" t="s">
         <v>58</v>
@@ -24107,22 +24138,22 @@
     </row>
     <row r="866" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A866" s="47" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
       <c r="B866" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C866" s="14" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="D866" s="15" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
       <c r="E866" s="15" t="s">
-        <v>593</v>
+        <v>595</v>
       </c>
       <c r="F866" s="15" t="s">
-        <v>594</v>
+        <v>596</v>
       </c>
       <c r="G866" s="16" t="s">
         <v>58</v>
@@ -24251,22 +24282,22 @@
     </row>
     <row r="872" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A872" s="47" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
       <c r="B872" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C872" s="25" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
       <c r="D872" s="26" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
       <c r="E872" s="26" t="s">
-        <v>597</v>
+        <v>599</v>
       </c>
       <c r="F872" s="26" t="s">
-        <v>598</v>
+        <v>600</v>
       </c>
       <c r="G872" s="16" t="s">
         <v>58</v>
@@ -24395,22 +24426,22 @@
     </row>
     <row r="878" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A878" s="47" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
       <c r="B878" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C878" s="14" t="s">
-        <v>599</v>
+        <v>601</v>
       </c>
       <c r="D878" s="15" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
       <c r="E878" s="15" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="F878" s="15" t="s">
-        <v>602</v>
+        <v>604</v>
       </c>
       <c r="G878" s="16" t="s">
         <v>58</v>
@@ -24539,22 +24570,22 @@
     </row>
     <row r="884" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A884" s="47" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
       <c r="B884" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C884" s="25" t="s">
-        <v>603</v>
+        <v>605</v>
       </c>
       <c r="D884" s="26" t="s">
-        <v>604</v>
+        <v>606</v>
       </c>
       <c r="E884" s="26" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
       <c r="F884" s="26" t="s">
-        <v>606</v>
+        <v>608</v>
       </c>
       <c r="G884" s="16" t="s">
         <v>58</v>
@@ -24683,22 +24714,22 @@
     </row>
     <row r="890" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A890" s="47" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
       <c r="B890" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C890" s="14" t="s">
-        <v>607</v>
+        <v>609</v>
       </c>
       <c r="D890" s="15" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
       <c r="E890" s="15" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="F890" s="15" t="s">
-        <v>610</v>
+        <v>612</v>
       </c>
       <c r="G890" s="16" t="s">
         <v>58</v>
@@ -24827,22 +24858,22 @@
     </row>
     <row r="896" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A896" s="47" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
       <c r="B896" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C896" s="25" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
       <c r="D896" s="26" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="E896" s="26" t="s">
-        <v>613</v>
+        <v>615</v>
       </c>
       <c r="F896" s="26" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
       <c r="G896" s="16" t="s">
         <v>58</v>
@@ -24971,22 +25002,22 @@
     </row>
     <row r="902" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A902" s="48" t="s">
-        <v>615</v>
+        <v>617</v>
       </c>
       <c r="B902" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C902" s="14" t="s">
-        <v>616</v>
+        <v>618</v>
       </c>
       <c r="D902" s="15" t="s">
-        <v>617</v>
+        <v>619</v>
       </c>
       <c r="E902" s="15" t="s">
-        <v>618</v>
+        <v>620</v>
       </c>
       <c r="F902" s="15" t="s">
-        <v>619</v>
+        <v>621</v>
       </c>
       <c r="G902" s="16" t="s">
         <v>58</v>
@@ -25115,22 +25146,22 @@
     </row>
     <row r="908" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A908" s="48" t="s">
-        <v>615</v>
+        <v>617</v>
       </c>
       <c r="B908" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C908" s="25" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="D908" s="26" t="s">
-        <v>621</v>
+        <v>623</v>
       </c>
       <c r="E908" s="26" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
       <c r="F908" s="26" t="s">
-        <v>623</v>
+        <v>625</v>
       </c>
       <c r="G908" s="16" t="s">
         <v>58</v>
@@ -25259,22 +25290,22 @@
     </row>
     <row r="914" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A914" s="48" t="s">
-        <v>615</v>
+        <v>617</v>
       </c>
       <c r="B914" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C914" s="14" t="s">
-        <v>624</v>
+        <v>626</v>
       </c>
       <c r="D914" s="15" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
       <c r="E914" s="15" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
       <c r="F914" s="15" t="s">
-        <v>627</v>
+        <v>629</v>
       </c>
       <c r="G914" s="16" t="s">
         <v>58</v>
@@ -25403,22 +25434,22 @@
     </row>
     <row r="920" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A920" s="48" t="s">
-        <v>615</v>
+        <v>617</v>
       </c>
       <c r="B920" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C920" s="25" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
       <c r="D920" s="26" t="s">
-        <v>629</v>
+        <v>631</v>
       </c>
       <c r="E920" s="26" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
       <c r="F920" s="26" t="s">
-        <v>631</v>
+        <v>633</v>
       </c>
       <c r="G920" s="16" t="s">
         <v>58</v>
@@ -25547,22 +25578,22 @@
     </row>
     <row r="926" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A926" s="48" t="s">
-        <v>615</v>
+        <v>617</v>
       </c>
       <c r="B926" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C926" s="14" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
       <c r="D926" s="15" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="E926" s="15" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
       <c r="F926" s="15" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="G926" s="16" t="s">
         <v>58</v>
@@ -25691,22 +25722,22 @@
     </row>
     <row r="932" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A932" s="48" t="s">
-        <v>615</v>
+        <v>617</v>
       </c>
       <c r="B932" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C932" s="25" t="s">
-        <v>636</v>
+        <v>638</v>
       </c>
       <c r="D932" s="26" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="E932" s="26" t="s">
-        <v>638</v>
+        <v>640</v>
       </c>
       <c r="F932" s="26" t="s">
-        <v>639</v>
+        <v>641</v>
       </c>
       <c r="G932" s="16" t="s">
         <v>58</v>
@@ -25835,22 +25866,22 @@
     </row>
     <row r="938" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A938" s="49" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
       <c r="B938" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C938" s="14" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
       <c r="D938" s="15" t="s">
-        <v>642</v>
+        <v>644</v>
       </c>
       <c r="E938" s="15" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
       <c r="F938" s="15" t="s">
-        <v>644</v>
+        <v>646</v>
       </c>
       <c r="G938" s="16" t="s">
         <v>58</v>
@@ -25979,22 +26010,22 @@
     </row>
     <row r="944" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A944" s="49" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
       <c r="B944" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C944" s="25" t="s">
-        <v>645</v>
+        <v>647</v>
       </c>
       <c r="D944" s="26" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
       <c r="E944" s="26" t="s">
-        <v>647</v>
+        <v>649</v>
       </c>
       <c r="F944" s="26" t="s">
-        <v>648</v>
+        <v>650</v>
       </c>
       <c r="G944" s="16" t="s">
         <v>58</v>
@@ -26123,22 +26154,22 @@
     </row>
     <row r="950" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A950" s="49" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
       <c r="B950" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C950" s="14" t="s">
-        <v>649</v>
+        <v>651</v>
       </c>
       <c r="D950" s="15" t="s">
-        <v>650</v>
+        <v>652</v>
       </c>
       <c r="E950" s="15" t="s">
-        <v>651</v>
+        <v>653</v>
       </c>
       <c r="F950" s="15" t="s">
-        <v>652</v>
+        <v>654</v>
       </c>
       <c r="G950" s="16" t="s">
         <v>58</v>
@@ -26267,22 +26298,22 @@
     </row>
     <row r="956" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A956" s="49" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
       <c r="B956" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C956" s="25" t="s">
-        <v>653</v>
+        <v>655</v>
       </c>
       <c r="D956" s="26" t="s">
-        <v>654</v>
+        <v>656</v>
       </c>
       <c r="E956" s="26" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
       <c r="F956" s="26" t="s">
-        <v>627</v>
+        <v>629</v>
       </c>
       <c r="G956" s="16" t="s">
         <v>58</v>
@@ -26411,22 +26442,22 @@
     </row>
     <row r="962" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A962" s="49" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
       <c r="B962" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C962" s="14" t="s">
-        <v>656</v>
+        <v>658</v>
       </c>
       <c r="D962" s="15" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
       <c r="E962" s="15" t="s">
-        <v>658</v>
+        <v>660</v>
       </c>
       <c r="F962" s="15" t="s">
-        <v>659</v>
+        <v>661</v>
       </c>
       <c r="G962" s="16" t="s">
         <v>58</v>
@@ -26555,22 +26586,22 @@
     </row>
     <row r="968" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A968" s="49" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
       <c r="B968" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C968" s="25" t="s">
-        <v>660</v>
+        <v>662</v>
       </c>
       <c r="D968" s="26" t="s">
-        <v>661</v>
+        <v>663</v>
       </c>
       <c r="E968" s="26" t="s">
-        <v>662</v>
+        <v>664</v>
       </c>
       <c r="F968" s="26" t="s">
-        <v>663</v>
+        <v>665</v>
       </c>
       <c r="G968" s="16" t="s">
         <v>58</v>
@@ -26699,22 +26730,22 @@
     </row>
     <row r="974" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A974" s="50" t="s">
-        <v>664</v>
+        <v>666</v>
       </c>
       <c r="B974" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C974" s="14" t="s">
-        <v>665</v>
+        <v>667</v>
       </c>
       <c r="D974" s="15" t="s">
-        <v>666</v>
+        <v>668</v>
       </c>
       <c r="E974" s="15" t="s">
-        <v>667</v>
+        <v>669</v>
       </c>
       <c r="F974" s="15" t="s">
-        <v>668</v>
+        <v>670</v>
       </c>
       <c r="G974" s="16" t="s">
         <v>58</v>
@@ -26843,22 +26874,22 @@
     </row>
     <row r="980" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A980" s="50" t="s">
-        <v>664</v>
+        <v>666</v>
       </c>
       <c r="B980" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C980" s="25" t="s">
-        <v>669</v>
+        <v>671</v>
       </c>
       <c r="D980" s="26" t="s">
-        <v>670</v>
+        <v>672</v>
       </c>
       <c r="E980" s="26" t="s">
-        <v>671</v>
+        <v>673</v>
       </c>
       <c r="F980" s="26" t="s">
-        <v>672</v>
+        <v>674</v>
       </c>
       <c r="G980" s="16" t="s">
         <v>58</v>
@@ -26987,22 +27018,22 @@
     </row>
     <row r="986" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A986" s="50" t="s">
-        <v>664</v>
+        <v>666</v>
       </c>
       <c r="B986" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C986" s="14" t="s">
-        <v>673</v>
+        <v>675</v>
       </c>
       <c r="D986" s="15" t="s">
-        <v>674</v>
+        <v>676</v>
       </c>
       <c r="E986" s="15" t="s">
-        <v>675</v>
+        <v>677</v>
       </c>
       <c r="F986" s="15" t="s">
-        <v>676</v>
+        <v>678</v>
       </c>
       <c r="G986" s="16" t="s">
         <v>58</v>
@@ -27131,22 +27162,22 @@
     </row>
     <row r="992" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A992" s="50" t="s">
-        <v>664</v>
+        <v>666</v>
       </c>
       <c r="B992" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C992" s="25" t="s">
-        <v>677</v>
+        <v>679</v>
       </c>
       <c r="D992" s="26" t="s">
-        <v>678</v>
+        <v>680</v>
       </c>
       <c r="E992" s="26" t="s">
-        <v>679</v>
+        <v>681</v>
       </c>
       <c r="F992" s="26" t="s">
-        <v>680</v>
+        <v>682</v>
       </c>
       <c r="G992" s="16" t="s">
         <v>58</v>
@@ -27275,22 +27306,22 @@
     </row>
     <row r="998" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A998" s="50" t="s">
-        <v>664</v>
+        <v>666</v>
       </c>
       <c r="B998" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C998" s="14" t="s">
-        <v>681</v>
+        <v>683</v>
       </c>
       <c r="D998" s="15" t="s">
-        <v>682</v>
+        <v>684</v>
       </c>
       <c r="E998" s="15" t="s">
-        <v>683</v>
+        <v>685</v>
       </c>
       <c r="F998" s="15" t="s">
-        <v>684</v>
+        <v>686</v>
       </c>
       <c r="G998" s="16" t="s">
         <v>58</v>
@@ -27419,22 +27450,22 @@
     </row>
     <row r="1004" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1004" s="51" t="s">
-        <v>685</v>
+        <v>687</v>
       </c>
       <c r="B1004" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1004" s="25" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
       <c r="D1004" s="26" t="s">
-        <v>687</v>
+        <v>689</v>
       </c>
       <c r="E1004" s="26" t="s">
-        <v>688</v>
+        <v>690</v>
       </c>
       <c r="F1004" s="26" t="s">
-        <v>689</v>
+        <v>691</v>
       </c>
       <c r="G1004" s="16" t="s">
         <v>58</v>
@@ -27563,22 +27594,22 @@
     </row>
     <row r="1010" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1010" s="51" t="s">
-        <v>685</v>
+        <v>687</v>
       </c>
       <c r="B1010" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1010" s="14" t="s">
-        <v>690</v>
+        <v>692</v>
       </c>
       <c r="D1010" s="15" t="s">
-        <v>691</v>
+        <v>693</v>
       </c>
       <c r="E1010" s="15" t="s">
-        <v>692</v>
+        <v>694</v>
       </c>
       <c r="F1010" s="15" t="s">
-        <v>693</v>
+        <v>695</v>
       </c>
       <c r="G1010" s="16" t="s">
         <v>58</v>
@@ -27707,22 +27738,22 @@
     </row>
     <row r="1016" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1016" s="51" t="s">
-        <v>685</v>
+        <v>687</v>
       </c>
       <c r="B1016" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1016" s="25" t="s">
-        <v>694</v>
+        <v>696</v>
       </c>
       <c r="D1016" s="26" t="s">
-        <v>695</v>
+        <v>697</v>
       </c>
       <c r="E1016" s="26" t="s">
-        <v>696</v>
+        <v>698</v>
       </c>
       <c r="F1016" s="26" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
       <c r="G1016" s="16" t="s">
         <v>58</v>
@@ -27851,22 +27882,22 @@
     </row>
     <row r="1022" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1022" s="51" t="s">
-        <v>685</v>
+        <v>687</v>
       </c>
       <c r="B1022" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1022" s="14" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
       <c r="D1022" s="15" t="s">
-        <v>699</v>
+        <v>701</v>
       </c>
       <c r="E1022" s="15" t="s">
-        <v>700</v>
+        <v>702</v>
       </c>
       <c r="F1022" s="15" t="s">
-        <v>701</v>
+        <v>703</v>
       </c>
       <c r="G1022" s="16" t="s">
         <v>58</v>
@@ -27995,22 +28026,22 @@
     </row>
     <row r="1028" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1028" s="51" t="s">
-        <v>685</v>
+        <v>687</v>
       </c>
       <c r="B1028" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C1028" s="25" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="D1028" s="26" t="s">
-        <v>703</v>
+        <v>705</v>
       </c>
       <c r="E1028" s="26" t="s">
-        <v>704</v>
+        <v>706</v>
       </c>
       <c r="F1028" s="26" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
       <c r="G1028" s="16" t="s">
         <v>58</v>
@@ -28139,22 +28170,22 @@
     </row>
     <row r="1034" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1034" s="51" t="s">
-        <v>685</v>
+        <v>687</v>
       </c>
       <c r="B1034" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C1034" s="14" t="s">
-        <v>706</v>
+        <v>708</v>
       </c>
       <c r="D1034" s="15" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
       <c r="E1034" s="15" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="F1034" s="15" t="s">
-        <v>709</v>
+        <v>711</v>
       </c>
       <c r="G1034" s="16" t="s">
         <v>58</v>
@@ -28283,22 +28314,22 @@
     </row>
     <row r="1040" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1040" s="52" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="B1040" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C1040" s="25" t="s">
-        <v>711</v>
+        <v>713</v>
       </c>
       <c r="D1040" s="26" t="s">
-        <v>699</v>
+        <v>701</v>
       </c>
       <c r="E1040" s="26" t="s">
-        <v>712</v>
+        <v>714</v>
       </c>
       <c r="F1040" s="26" t="s">
-        <v>713</v>
+        <v>715</v>
       </c>
       <c r="G1040" s="16" t="s">
         <v>58</v>
@@ -28427,22 +28458,22 @@
     </row>
     <row r="1046" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1046" s="52" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="B1046" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1046" s="14" t="s">
-        <v>714</v>
+        <v>716</v>
       </c>
       <c r="D1046" s="15" t="s">
-        <v>691</v>
+        <v>693</v>
       </c>
       <c r="E1046" s="15" t="s">
-        <v>715</v>
+        <v>717</v>
       </c>
       <c r="F1046" s="15" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
       <c r="G1046" s="16" t="s">
         <v>58</v>
@@ -28577,16 +28608,16 @@
         <v>53</v>
       </c>
       <c r="C1052" s="25" t="s">
-        <v>717</v>
+        <v>719</v>
       </c>
       <c r="D1052" s="26" t="s">
-        <v>718</v>
+        <v>720</v>
       </c>
       <c r="E1052" s="26" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
       <c r="F1052" s="26" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
       <c r="G1052" s="16" t="s">
         <v>58</v>
@@ -28721,16 +28752,16 @@
         <v>53</v>
       </c>
       <c r="C1058" s="14" t="s">
-        <v>721</v>
+        <v>723</v>
       </c>
       <c r="D1058" s="15" t="s">
-        <v>722</v>
+        <v>724</v>
       </c>
       <c r="E1058" s="15" t="s">
-        <v>723</v>
+        <v>725</v>
       </c>
       <c r="F1058" s="15" t="s">
-        <v>724</v>
+        <v>726</v>
       </c>
       <c r="G1058" s="16" t="s">
         <v>58</v>
@@ -29816,10 +29847,10 @@
         <v>39</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>725</v>
+        <v>727</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>726</v>
+        <v>728</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>53</v>
@@ -29837,7 +29868,7 @@
         <v>86</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -30132,7 +30163,7 @@
     </row>
     <row r="12" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="63" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="B12" s="1">
         <v>5</v>
@@ -30161,7 +30192,7 @@
     </row>
     <row r="13" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="64" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="B13" s="1">
         <v>4</v>
@@ -30190,7 +30221,7 @@
     </row>
     <row r="14" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="65" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="B14" s="1">
         <v>5</v>
@@ -30219,7 +30250,7 @@
     </row>
     <row r="15" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="66" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="B15" s="1">
         <v>12</v>
@@ -30248,7 +30279,7 @@
     </row>
     <row r="16" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="67" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
       <c r="B16" s="1">
         <v>4</v>
@@ -30277,7 +30308,7 @@
     </row>
     <row r="17" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="68" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
       <c r="B17" s="1">
         <v>7</v>
@@ -30306,7 +30337,7 @@
     </row>
     <row r="18" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="69" t="s">
-        <v>615</v>
+        <v>617</v>
       </c>
       <c r="B18" s="1">
         <v>6</v>
@@ -30335,7 +30366,7 @@
     </row>
     <row r="19" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="70" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
       <c r="B19" s="1">
         <v>6</v>
@@ -30364,7 +30395,7 @@
     </row>
     <row r="20" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="71" t="s">
-        <v>664</v>
+        <v>666</v>
       </c>
       <c r="B20" s="1">
         <v>5</v>
@@ -30393,7 +30424,7 @@
     </row>
     <row r="21" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="72" t="s">
-        <v>685</v>
+        <v>687</v>
       </c>
       <c r="B21" s="1">
         <v>6</v>
@@ -30422,7 +30453,7 @@
     </row>
     <row r="22" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="73" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="B22" s="1">
         <v>2</v>
@@ -30451,7 +30482,7 @@
     </row>
     <row r="23" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="74" t="s">
-        <v>728</v>
+        <v>730</v>
       </c>
       <c r="B23" s="74">
         <v>153</v>
@@ -30502,7 +30533,7 @@
         <v>44</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>726</v>
+        <v>728</v>
       </c>
       <c r="C1" s="10" t="s">
         <v>71</v>
@@ -30511,7 +30542,7 @@
         <v>86</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
       <c r="F1" s="10" t="s">
         <v>94</v>
@@ -30662,10 +30693,10 @@
         <v>45</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>726</v>
+        <v>728</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>71</v>
@@ -30674,7 +30705,7 @@
         <v>86</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
       <c r="G1" s="10" t="s">
         <v>94</v>
@@ -30685,7 +30716,7 @@
         <v>59</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="C2" s="1">
         <v>18</v>

</xml_diff>

<commit_message>
088 => fase IV => ZUP-037 ZUP-049 ZUP-051 ZUP-057 OK (Chrome/USER), ZUP-054 ZUP-058 KO i millores anotades
</commit_message>
<xml_diff>
--- a/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
+++ b/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4342" uniqueCount="736">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4354" uniqueCount="740">
   <si>
     <t>Zuppeto — Joc de probes manual (totes les pantalles)</t>
   </si>
@@ -992,6 +992,14 @@
     <t>Estat buit «Sense selecció activa»</t>
   </si>
   <si>
+    <t>Amb un pin seleccionat (popup + targeta «Seleccionat al mapa»), Treure selecció no deixa l’estat «Sense selecció activa»: el globus o la targeta es queden, o el mapa salta a tots els pins.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Què s'ha fet:
+- src/Web/src/app/features/places/components/place-map/place-map.component.ts — Treure selecció tanca el globus; tancar el globus també treu la selecció; el mapa ja no salta a tots els pins; sincronia amb effect
+- docs/ca/funcional-ca.md, docs/ca/tecnic-ca.md</t>
+  </si>
+  <si>
     <t>Detall lloc (/places/:id)</t>
   </si>
   <si>
@@ -1040,6 +1048,9 @@
     <t>Dades completes del lloc</t>
   </si>
   <si>
+    <t>Secció visible (adreça, barri, valoració…). Millora: Política pet no ha de mostrar «Google Places (cache)» ni informació tècnica.</t>
+  </si>
+  <si>
     <t>ZUP-058</t>
   </si>
   <si>
@@ -1050,6 +1061,10 @@
   </si>
   <si>
     <t>Llista de característiques visible</t>
+  </si>
+  <si>
+    <t xml:space="preserve">«Què hi trobaràs» buit (caixa blanca, sense etiquetes).
+Cal omplir característiques útils (gos dins / només terrassa / no es permet, etc.). Si no hi són a la BD, consultar web/detall del local. No deixar la targeta buida.</t>
   </si>
   <si>
     <t>ZUP-059</t>
@@ -2315,7 +2330,7 @@
     </font>
     <font>
       <b/>
-      <color rgb="FF006100"/>
+      <color rgb="FF9C0006"/>
       <sz val="10"/>
       <name val="Calibri"/>
     </font>
@@ -2487,7 +2502,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
+        <fgColor rgb="FFFFC7CE"/>
       </patternFill>
     </fill>
     <fill>
@@ -10011,9 +10026,11 @@
       <c r="H272" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="I272" s="18"/>
+      <c r="I272" s="18" t="s">
+        <v>132</v>
+      </c>
       <c r="J272" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K272" s="19"/>
       <c r="L272" s="18"/>
@@ -12175,9 +12192,11 @@
       <c r="H362" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="I362" s="18"/>
+      <c r="I362" s="18" t="s">
+        <v>132</v>
+      </c>
       <c r="J362" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K362" s="19"/>
       <c r="L362" s="18"/>
@@ -12465,9 +12484,11 @@
       <c r="H374" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="I374" s="18"/>
+      <c r="I374" s="18" t="s">
+        <v>132</v>
+      </c>
       <c r="J374" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K374" s="19"/>
       <c r="L374" s="18"/>
@@ -12901,14 +12922,24 @@
       <c r="H392" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="I392" s="18"/>
+      <c r="I392" s="18" t="s">
+        <v>132</v>
+      </c>
       <c r="J392" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="K392" s="19"/>
-      <c r="L392" s="18"/>
-      <c r="M392" s="1"/>
-      <c r="N392" s="19"/>
+        <v>86</v>
+      </c>
+      <c r="K392" s="19" t="s">
+        <v>318</v>
+      </c>
+      <c r="L392" s="18" t="s">
+        <v>132</v>
+      </c>
+      <c r="M392" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="N392" s="19" t="s">
+        <v>319</v>
+      </c>
     </row>
     <row r="393" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A393" s="37"/>
@@ -13022,22 +13053,22 @@
     </row>
     <row r="398" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A398" s="38" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B398" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C398" s="14" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="D398" s="15" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="E398" s="15" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="F398" s="15" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="G398" s="16" t="s">
         <v>58</v>
@@ -13178,13 +13209,13 @@
         <v>34</v>
       </c>
       <c r="I404" s="18" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="J404" s="1" t="s">
         <v>71</v>
       </c>
       <c r="K404" s="19" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="L404" s="18"/>
       <c r="M404" s="1"/>
@@ -13566,22 +13597,22 @@
     </row>
     <row r="422" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A422" s="38" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B422" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C422" s="25" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="D422" s="26" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="E422" s="26" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="F422" s="26" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="G422" s="16" t="s">
         <v>58</v>
@@ -13590,7 +13621,7 @@
         <v>34</v>
       </c>
       <c r="I422" s="18" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="J422" s="1" t="s">
         <v>71</v>
@@ -13712,22 +13743,22 @@
     </row>
     <row r="428" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A428" s="38" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B428" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C428" s="14" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="D428" s="15" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="E428" s="15" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="F428" s="15" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="G428" s="16" t="s">
         <v>58</v>
@@ -13735,11 +13766,15 @@
       <c r="H428" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="I428" s="18"/>
+      <c r="I428" s="18" t="s">
+        <v>132</v>
+      </c>
       <c r="J428" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="K428" s="19"/>
+        <v>71</v>
+      </c>
+      <c r="K428" s="19" t="s">
+        <v>336</v>
+      </c>
       <c r="L428" s="18"/>
       <c r="M428" s="1"/>
       <c r="N428" s="19"/>
@@ -13856,22 +13891,22 @@
     </row>
     <row r="434" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A434" s="38" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B434" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C434" s="25" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="D434" s="26" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="E434" s="26" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="F434" s="26" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="G434" s="16" t="s">
         <v>58</v>
@@ -13879,11 +13914,15 @@
       <c r="H434" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="I434" s="18"/>
+      <c r="I434" s="18" t="s">
+        <v>132</v>
+      </c>
       <c r="J434" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="K434" s="19"/>
+        <v>86</v>
+      </c>
+      <c r="K434" s="19" t="s">
+        <v>341</v>
+      </c>
       <c r="L434" s="18"/>
       <c r="M434" s="1"/>
       <c r="N434" s="19"/>
@@ -14000,22 +14039,22 @@
     </row>
     <row r="440" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A440" s="38" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B440" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C440" s="14" t="s">
-        <v>338</v>
+        <v>342</v>
       </c>
       <c r="D440" s="15" t="s">
-        <v>339</v>
+        <v>343</v>
       </c>
       <c r="E440" s="15" t="s">
-        <v>340</v>
+        <v>344</v>
       </c>
       <c r="F440" s="15" t="s">
-        <v>341</v>
+        <v>345</v>
       </c>
       <c r="G440" s="16" t="s">
         <v>58</v>
@@ -14144,22 +14183,22 @@
     </row>
     <row r="446" ht="77" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A446" s="38" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B446" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C446" s="25" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="D446" s="26" t="s">
-        <v>343</v>
+        <v>347</v>
       </c>
       <c r="E446" s="26" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
       <c r="F446" s="26" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
       <c r="G446" s="16" t="s">
         <v>58</v>
@@ -14174,7 +14213,7 @@
         <v>86</v>
       </c>
       <c r="K446" s="19" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="L446" s="18" t="s">
         <v>210</v>
@@ -14183,7 +14222,7 @@
         <v>71</v>
       </c>
       <c r="N446" s="19" t="s">
-        <v>347</v>
+        <v>351</v>
       </c>
     </row>
     <row r="447" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -14298,22 +14337,22 @@
     </row>
     <row r="452" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A452" s="38" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B452" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C452" s="14" t="s">
-        <v>348</v>
+        <v>352</v>
       </c>
       <c r="D452" s="15" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
       <c r="E452" s="15" t="s">
-        <v>350</v>
+        <v>354</v>
       </c>
       <c r="F452" s="15" t="s">
-        <v>351</v>
+        <v>355</v>
       </c>
       <c r="G452" s="16" t="s">
         <v>58</v>
@@ -14442,22 +14481,22 @@
     </row>
     <row r="458" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A458" s="38" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B458" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C458" s="25" t="s">
-        <v>352</v>
+        <v>356</v>
       </c>
       <c r="D458" s="26" t="s">
-        <v>353</v>
+        <v>357</v>
       </c>
       <c r="E458" s="26" t="s">
-        <v>354</v>
+        <v>358</v>
       </c>
       <c r="F458" s="26" t="s">
-        <v>355</v>
+        <v>359</v>
       </c>
       <c r="G458" s="16" t="s">
         <v>58</v>
@@ -14586,22 +14625,22 @@
     </row>
     <row r="464" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A464" s="38" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B464" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C464" s="14" t="s">
-        <v>356</v>
+        <v>360</v>
       </c>
       <c r="D464" s="15" t="s">
-        <v>357</v>
+        <v>361</v>
       </c>
       <c r="E464" s="15" t="s">
-        <v>358</v>
+        <v>362</v>
       </c>
       <c r="F464" s="15" t="s">
-        <v>359</v>
+        <v>363</v>
       </c>
       <c r="G464" s="16" t="s">
         <v>58</v>
@@ -14730,22 +14769,22 @@
     </row>
     <row r="470" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A470" s="38" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B470" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C470" s="25" t="s">
-        <v>360</v>
+        <v>364</v>
       </c>
       <c r="D470" s="26" t="s">
-        <v>361</v>
+        <v>365</v>
       </c>
       <c r="E470" s="26" t="s">
-        <v>362</v>
+        <v>366</v>
       </c>
       <c r="F470" s="26" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="G470" s="16" t="s">
         <v>58</v>
@@ -14754,7 +14793,7 @@
         <v>34</v>
       </c>
       <c r="I470" s="18" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="J470" s="1" t="s">
         <v>71</v>
@@ -14876,22 +14915,22 @@
     </row>
     <row r="476" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A476" s="39" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="B476" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C476" s="14" t="s">
-        <v>365</v>
+        <v>369</v>
       </c>
       <c r="D476" s="15" t="s">
-        <v>366</v>
+        <v>370</v>
       </c>
       <c r="E476" s="15" t="s">
-        <v>367</v>
+        <v>371</v>
       </c>
       <c r="F476" s="15" t="s">
-        <v>368</v>
+        <v>372</v>
       </c>
       <c r="G476" s="16" t="s">
         <v>58</v>
@@ -14900,13 +14939,13 @@
         <v>34</v>
       </c>
       <c r="I476" s="18" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="J476" s="1" t="s">
         <v>71</v>
       </c>
       <c r="K476" s="19" t="s">
-        <v>369</v>
+        <v>373</v>
       </c>
       <c r="L476" s="18"/>
       <c r="M476" s="1"/>
@@ -15024,22 +15063,22 @@
     </row>
     <row r="482" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A482" s="39" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="B482" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C482" s="25" t="s">
-        <v>370</v>
+        <v>374</v>
       </c>
       <c r="D482" s="26" t="s">
-        <v>371</v>
+        <v>375</v>
       </c>
       <c r="E482" s="26" t="s">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="F482" s="26" t="s">
-        <v>373</v>
+        <v>377</v>
       </c>
       <c r="G482" s="16" t="s">
         <v>58</v>
@@ -15048,13 +15087,13 @@
         <v>34</v>
       </c>
       <c r="I482" s="18" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="J482" s="1" t="s">
         <v>71</v>
       </c>
       <c r="K482" s="19" t="s">
-        <v>374</v>
+        <v>378</v>
       </c>
       <c r="L482" s="18"/>
       <c r="M482" s="1"/>
@@ -15172,22 +15211,22 @@
     </row>
     <row r="488" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A488" s="39" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="B488" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C488" s="14" t="s">
-        <v>375</v>
+        <v>379</v>
       </c>
       <c r="D488" s="15" t="s">
-        <v>376</v>
+        <v>380</v>
       </c>
       <c r="E488" s="15" t="s">
-        <v>377</v>
+        <v>381</v>
       </c>
       <c r="F488" s="15" t="s">
-        <v>378</v>
+        <v>382</v>
       </c>
       <c r="G488" s="16" t="s">
         <v>58</v>
@@ -15196,7 +15235,7 @@
         <v>34</v>
       </c>
       <c r="I488" s="18" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="J488" s="1" t="s">
         <v>71</v>
@@ -15318,22 +15357,22 @@
     </row>
     <row r="494" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A494" s="39" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="B494" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C494" s="25" t="s">
-        <v>379</v>
+        <v>383</v>
       </c>
       <c r="D494" s="26" t="s">
-        <v>380</v>
+        <v>384</v>
       </c>
       <c r="E494" s="26" t="s">
-        <v>381</v>
+        <v>385</v>
       </c>
       <c r="F494" s="26" t="s">
-        <v>382</v>
+        <v>386</v>
       </c>
       <c r="G494" s="16" t="s">
         <v>58</v>
@@ -15462,22 +15501,22 @@
     </row>
     <row r="500" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A500" s="39" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="B500" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C500" s="14" t="s">
-        <v>383</v>
+        <v>387</v>
       </c>
       <c r="D500" s="15" t="s">
-        <v>384</v>
+        <v>388</v>
       </c>
       <c r="E500" s="15" t="s">
-        <v>385</v>
+        <v>389</v>
       </c>
       <c r="F500" s="15" t="s">
-        <v>386</v>
+        <v>390</v>
       </c>
       <c r="G500" s="16" t="s">
         <v>58</v>
@@ -15606,22 +15645,22 @@
     </row>
     <row r="506" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A506" s="39" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="B506" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C506" s="25" t="s">
-        <v>387</v>
+        <v>391</v>
       </c>
       <c r="D506" s="26" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="E506" s="26" t="s">
         <v>254</v>
       </c>
       <c r="F506" s="26" t="s">
-        <v>389</v>
+        <v>393</v>
       </c>
       <c r="G506" s="16" t="s">
         <v>58</v>
@@ -15750,22 +15789,22 @@
     </row>
     <row r="512" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A512" s="39" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="B512" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C512" s="14" t="s">
-        <v>390</v>
+        <v>394</v>
       </c>
       <c r="D512" s="15" t="s">
-        <v>391</v>
+        <v>395</v>
       </c>
       <c r="E512" s="15" t="s">
-        <v>392</v>
+        <v>396</v>
       </c>
       <c r="F512" s="15" t="s">
-        <v>393</v>
+        <v>397</v>
       </c>
       <c r="G512" s="16" t="s">
         <v>58</v>
@@ -15894,22 +15933,22 @@
     </row>
     <row r="518" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A518" s="39" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="B518" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C518" s="25" t="s">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="D518" s="26" t="s">
-        <v>395</v>
+        <v>399</v>
       </c>
       <c r="E518" s="26" t="s">
-        <v>396</v>
+        <v>400</v>
       </c>
       <c r="F518" s="26" t="s">
-        <v>397</v>
+        <v>401</v>
       </c>
       <c r="G518" s="16" t="s">
         <v>58</v>
@@ -16038,22 +16077,22 @@
     </row>
     <row r="524" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A524" s="39" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="B524" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C524" s="14" t="s">
-        <v>398</v>
+        <v>402</v>
       </c>
       <c r="D524" s="15" t="s">
-        <v>399</v>
+        <v>403</v>
       </c>
       <c r="E524" s="15" t="s">
-        <v>400</v>
+        <v>404</v>
       </c>
       <c r="F524" s="15" t="s">
-        <v>401</v>
+        <v>405</v>
       </c>
       <c r="G524" s="16" t="s">
         <v>58</v>
@@ -16062,7 +16101,7 @@
         <v>34</v>
       </c>
       <c r="I524" s="18" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="J524" s="1" t="s">
         <v>71</v>
@@ -16184,22 +16223,22 @@
     </row>
     <row r="530" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A530" s="39" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="B530" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C530" s="25" t="s">
-        <v>402</v>
+        <v>406</v>
       </c>
       <c r="D530" s="26" t="s">
-        <v>403</v>
+        <v>407</v>
       </c>
       <c r="E530" s="26" t="s">
-        <v>404</v>
+        <v>408</v>
       </c>
       <c r="F530" s="26" t="s">
-        <v>405</v>
+        <v>409</v>
       </c>
       <c r="G530" s="16" t="s">
         <v>58</v>
@@ -16208,7 +16247,7 @@
         <v>34</v>
       </c>
       <c r="I530" s="18" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="J530" s="1" t="s">
         <v>71</v>
@@ -16330,22 +16369,22 @@
     </row>
     <row r="536" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A536" s="39" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="B536" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C536" s="14" t="s">
-        <v>406</v>
+        <v>410</v>
       </c>
       <c r="D536" s="15" t="s">
-        <v>407</v>
+        <v>411</v>
       </c>
       <c r="E536" s="15" t="s">
-        <v>408</v>
+        <v>412</v>
       </c>
       <c r="F536" s="15" t="s">
-        <v>409</v>
+        <v>413</v>
       </c>
       <c r="G536" s="16" t="s">
         <v>58</v>
@@ -16354,7 +16393,7 @@
         <v>34</v>
       </c>
       <c r="I536" s="18" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="J536" s="1" t="s">
         <v>71</v>
@@ -16476,22 +16515,22 @@
     </row>
     <row r="542" ht="180" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A542" s="40" t="s">
-        <v>410</v>
+        <v>414</v>
       </c>
       <c r="B542" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C542" s="25" t="s">
-        <v>411</v>
+        <v>415</v>
       </c>
       <c r="D542" s="26" t="s">
-        <v>412</v>
+        <v>416</v>
       </c>
       <c r="E542" s="26" t="s">
-        <v>413</v>
+        <v>417</v>
       </c>
       <c r="F542" s="26" t="s">
-        <v>414</v>
+        <v>418</v>
       </c>
       <c r="G542" s="16" t="s">
         <v>58</v>
@@ -16500,13 +16539,13 @@
         <v>34</v>
       </c>
       <c r="I542" s="18" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="J542" s="1" t="s">
         <v>86</v>
       </c>
       <c r="K542" s="19" t="s">
-        <v>415</v>
+        <v>419</v>
       </c>
       <c r="L542" s="18">
         <v>46264.91666666667</v>
@@ -16515,7 +16554,7 @@
         <v>71</v>
       </c>
       <c r="N542" s="19" t="s">
-        <v>416</v>
+        <v>420</v>
       </c>
     </row>
     <row r="543" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -16630,22 +16669,22 @@
     </row>
     <row r="548" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A548" s="40" t="s">
-        <v>410</v>
+        <v>414</v>
       </c>
       <c r="B548" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C548" s="14" t="s">
-        <v>417</v>
+        <v>421</v>
       </c>
       <c r="D548" s="15" t="s">
-        <v>418</v>
+        <v>422</v>
       </c>
       <c r="E548" s="15" t="s">
-        <v>419</v>
+        <v>423</v>
       </c>
       <c r="F548" s="15" t="s">
-        <v>420</v>
+        <v>424</v>
       </c>
       <c r="G548" s="16" t="s">
         <v>58</v>
@@ -16774,22 +16813,22 @@
     </row>
     <row r="554" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A554" s="40" t="s">
-        <v>410</v>
+        <v>414</v>
       </c>
       <c r="B554" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C554" s="25" t="s">
-        <v>421</v>
+        <v>425</v>
       </c>
       <c r="D554" s="26" t="s">
-        <v>422</v>
+        <v>426</v>
       </c>
       <c r="E554" s="26" t="s">
-        <v>423</v>
+        <v>427</v>
       </c>
       <c r="F554" s="26" t="s">
-        <v>424</v>
+        <v>428</v>
       </c>
       <c r="G554" s="16" t="s">
         <v>58</v>
@@ -16920,22 +16959,22 @@
     </row>
     <row r="560" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A560" s="40" t="s">
-        <v>410</v>
+        <v>414</v>
       </c>
       <c r="B560" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C560" s="14" t="s">
-        <v>425</v>
+        <v>429</v>
       </c>
       <c r="D560" s="15" t="s">
-        <v>426</v>
+        <v>430</v>
       </c>
       <c r="E560" s="15" t="s">
-        <v>427</v>
+        <v>431</v>
       </c>
       <c r="F560" s="15" t="s">
-        <v>428</v>
+        <v>432</v>
       </c>
       <c r="G560" s="16" t="s">
         <v>58</v>
@@ -17064,22 +17103,22 @@
     </row>
     <row r="566" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A566" s="40" t="s">
-        <v>410</v>
+        <v>414</v>
       </c>
       <c r="B566" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C566" s="25" t="s">
-        <v>429</v>
+        <v>433</v>
       </c>
       <c r="D566" s="26" t="s">
-        <v>430</v>
+        <v>434</v>
       </c>
       <c r="E566" s="26" t="s">
-        <v>431</v>
+        <v>435</v>
       </c>
       <c r="F566" s="26" t="s">
-        <v>432</v>
+        <v>436</v>
       </c>
       <c r="G566" s="16" t="s">
         <v>58</v>
@@ -17208,22 +17247,22 @@
     </row>
     <row r="572" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A572" s="40" t="s">
-        <v>410</v>
+        <v>414</v>
       </c>
       <c r="B572" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C572" s="14" t="s">
-        <v>433</v>
+        <v>437</v>
       </c>
       <c r="D572" s="15" t="s">
-        <v>434</v>
+        <v>438</v>
       </c>
       <c r="E572" s="15" t="s">
-        <v>435</v>
+        <v>439</v>
       </c>
       <c r="F572" s="15" t="s">
-        <v>436</v>
+        <v>440</v>
       </c>
       <c r="G572" s="16" t="s">
         <v>58</v>
@@ -17352,22 +17391,22 @@
     </row>
     <row r="578" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A578" s="40" t="s">
-        <v>410</v>
+        <v>414</v>
       </c>
       <c r="B578" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C578" s="25" t="s">
-        <v>437</v>
+        <v>441</v>
       </c>
       <c r="D578" s="26" t="s">
-        <v>438</v>
+        <v>442</v>
       </c>
       <c r="E578" s="26" t="s">
-        <v>439</v>
+        <v>443</v>
       </c>
       <c r="F578" s="26" t="s">
-        <v>440</v>
+        <v>444</v>
       </c>
       <c r="G578" s="16" t="s">
         <v>58</v>
@@ -17498,22 +17537,22 @@
     </row>
     <row r="584" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A584" s="40" t="s">
-        <v>410</v>
+        <v>414</v>
       </c>
       <c r="B584" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C584" s="14" t="s">
-        <v>441</v>
+        <v>445</v>
       </c>
       <c r="D584" s="15" t="s">
-        <v>442</v>
+        <v>446</v>
       </c>
       <c r="E584" s="15" t="s">
-        <v>443</v>
+        <v>447</v>
       </c>
       <c r="F584" s="15" t="s">
-        <v>444</v>
+        <v>448</v>
       </c>
       <c r="G584" s="16" t="s">
         <v>58</v>
@@ -17642,22 +17681,22 @@
     </row>
     <row r="590" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A590" s="40" t="s">
-        <v>410</v>
+        <v>414</v>
       </c>
       <c r="B590" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C590" s="25" t="s">
-        <v>445</v>
+        <v>449</v>
       </c>
       <c r="D590" s="26" t="s">
-        <v>446</v>
+        <v>450</v>
       </c>
       <c r="E590" s="26" t="s">
-        <v>447</v>
+        <v>451</v>
       </c>
       <c r="F590" s="26" t="s">
-        <v>448</v>
+        <v>452</v>
       </c>
       <c r="G590" s="16" t="s">
         <v>58</v>
@@ -17788,22 +17827,22 @@
     </row>
     <row r="596" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A596" s="41" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="B596" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C596" s="14" t="s">
-        <v>450</v>
+        <v>454</v>
       </c>
       <c r="D596" s="15" t="s">
-        <v>451</v>
+        <v>455</v>
       </c>
       <c r="E596" s="15" t="s">
-        <v>452</v>
+        <v>456</v>
       </c>
       <c r="F596" s="15" t="s">
-        <v>453</v>
+        <v>457</v>
       </c>
       <c r="G596" s="16" t="s">
         <v>58</v>
@@ -17950,7 +17989,7 @@
         <v>86</v>
       </c>
       <c r="K602" s="19" t="s">
-        <v>454</v>
+        <v>458</v>
       </c>
       <c r="L602" s="18">
         <v>46264.91666666667</v>
@@ -17959,7 +17998,7 @@
         <v>71</v>
       </c>
       <c r="N602" s="19" t="s">
-        <v>455</v>
+        <v>459</v>
       </c>
     </row>
     <row r="603" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -18338,22 +18377,22 @@
     </row>
     <row r="620" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A620" s="41" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="B620" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C620" s="25" t="s">
-        <v>456</v>
+        <v>460</v>
       </c>
       <c r="D620" s="26" t="s">
-        <v>457</v>
+        <v>461</v>
       </c>
       <c r="E620" s="26" t="s">
-        <v>458</v>
+        <v>462</v>
       </c>
       <c r="F620" s="26" t="s">
-        <v>459</v>
+        <v>463</v>
       </c>
       <c r="G620" s="16" t="s">
         <v>58</v>
@@ -18484,22 +18523,22 @@
     </row>
     <row r="626" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A626" s="41" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="B626" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C626" s="14" t="s">
-        <v>460</v>
+        <v>464</v>
       </c>
       <c r="D626" s="15" t="s">
-        <v>461</v>
+        <v>465</v>
       </c>
       <c r="E626" s="15" t="s">
-        <v>462</v>
+        <v>466</v>
       </c>
       <c r="F626" s="15" t="s">
-        <v>463</v>
+        <v>467</v>
       </c>
       <c r="G626" s="16" t="s">
         <v>58</v>
@@ -18630,22 +18669,22 @@
     </row>
     <row r="632" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A632" s="41" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="B632" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C632" s="25" t="s">
-        <v>464</v>
+        <v>468</v>
       </c>
       <c r="D632" s="26" t="s">
-        <v>465</v>
+        <v>469</v>
       </c>
       <c r="E632" s="26" t="s">
-        <v>466</v>
+        <v>470</v>
       </c>
       <c r="F632" s="26" t="s">
-        <v>467</v>
+        <v>471</v>
       </c>
       <c r="G632" s="16" t="s">
         <v>58</v>
@@ -18774,22 +18813,22 @@
     </row>
     <row r="638" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A638" s="41" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="B638" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C638" s="14" t="s">
-        <v>468</v>
+        <v>472</v>
       </c>
       <c r="D638" s="15" t="s">
-        <v>469</v>
+        <v>473</v>
       </c>
       <c r="E638" s="15" t="s">
-        <v>470</v>
+        <v>474</v>
       </c>
       <c r="F638" s="15" t="s">
-        <v>471</v>
+        <v>475</v>
       </c>
       <c r="G638" s="16" t="s">
         <v>58</v>
@@ -18920,22 +18959,22 @@
     </row>
     <row r="644" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A644" s="42" t="s">
-        <v>472</v>
+        <v>476</v>
       </c>
       <c r="B644" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C644" s="25" t="s">
-        <v>473</v>
+        <v>477</v>
       </c>
       <c r="D644" s="26" t="s">
-        <v>474</v>
+        <v>478</v>
       </c>
       <c r="E644" s="26" t="s">
-        <v>475</v>
+        <v>479</v>
       </c>
       <c r="F644" s="26" t="s">
-        <v>476</v>
+        <v>480</v>
       </c>
       <c r="G644" s="16" t="s">
         <v>58</v>
@@ -19462,22 +19501,22 @@
     </row>
     <row r="668" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A668" s="42" t="s">
-        <v>472</v>
+        <v>476</v>
       </c>
       <c r="B668" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C668" s="14" t="s">
-        <v>477</v>
+        <v>481</v>
       </c>
       <c r="D668" s="15" t="s">
-        <v>478</v>
+        <v>482</v>
       </c>
       <c r="E668" s="15" t="s">
-        <v>479</v>
+        <v>483</v>
       </c>
       <c r="F668" s="15" t="s">
-        <v>480</v>
+        <v>484</v>
       </c>
       <c r="G668" s="16" t="s">
         <v>58</v>
@@ -19606,22 +19645,22 @@
     </row>
     <row r="674" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A674" s="42" t="s">
-        <v>472</v>
+        <v>476</v>
       </c>
       <c r="B674" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C674" s="25" t="s">
-        <v>481</v>
+        <v>485</v>
       </c>
       <c r="D674" s="26" t="s">
-        <v>482</v>
+        <v>486</v>
       </c>
       <c r="E674" s="26" t="s">
-        <v>483</v>
+        <v>487</v>
       </c>
       <c r="F674" s="26" t="s">
-        <v>484</v>
+        <v>488</v>
       </c>
       <c r="G674" s="16" t="s">
         <v>58</v>
@@ -19750,22 +19789,22 @@
     </row>
     <row r="680" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A680" s="42" t="s">
-        <v>472</v>
+        <v>476</v>
       </c>
       <c r="B680" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C680" s="14" t="s">
-        <v>485</v>
+        <v>489</v>
       </c>
       <c r="D680" s="15" t="s">
-        <v>486</v>
+        <v>490</v>
       </c>
       <c r="E680" s="15" t="s">
-        <v>487</v>
+        <v>491</v>
       </c>
       <c r="F680" s="15" t="s">
-        <v>409</v>
+        <v>413</v>
       </c>
       <c r="G680" s="16" t="s">
         <v>58</v>
@@ -19894,22 +19933,22 @@
     </row>
     <row r="686" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A686" s="42" t="s">
-        <v>472</v>
+        <v>476</v>
       </c>
       <c r="B686" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C686" s="25" t="s">
-        <v>488</v>
+        <v>492</v>
       </c>
       <c r="D686" s="26" t="s">
-        <v>489</v>
+        <v>493</v>
       </c>
       <c r="E686" s="26" t="s">
-        <v>490</v>
+        <v>494</v>
       </c>
       <c r="F686" s="26" t="s">
-        <v>491</v>
+        <v>495</v>
       </c>
       <c r="G686" s="16" t="s">
         <v>58</v>
@@ -20038,22 +20077,22 @@
     </row>
     <row r="692" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A692" s="43" t="s">
-        <v>492</v>
+        <v>496</v>
       </c>
       <c r="B692" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C692" s="14" t="s">
-        <v>493</v>
+        <v>497</v>
       </c>
       <c r="D692" s="15" t="s">
-        <v>494</v>
+        <v>498</v>
       </c>
       <c r="E692" s="15" t="s">
-        <v>495</v>
+        <v>499</v>
       </c>
       <c r="F692" s="15" t="s">
-        <v>496</v>
+        <v>500</v>
       </c>
       <c r="G692" s="16" t="s">
         <v>58</v>
@@ -20580,22 +20619,22 @@
     </row>
     <row r="716" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A716" s="43" t="s">
-        <v>492</v>
+        <v>496</v>
       </c>
       <c r="B716" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C716" s="25" t="s">
-        <v>497</v>
+        <v>501</v>
       </c>
       <c r="D716" s="26" t="s">
-        <v>498</v>
+        <v>502</v>
       </c>
       <c r="E716" s="26" t="s">
-        <v>499</v>
+        <v>503</v>
       </c>
       <c r="F716" s="26" t="s">
-        <v>500</v>
+        <v>504</v>
       </c>
       <c r="G716" s="16" t="s">
         <v>58</v>
@@ -20724,22 +20763,22 @@
     </row>
     <row r="722" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A722" s="43" t="s">
-        <v>492</v>
+        <v>496</v>
       </c>
       <c r="B722" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C722" s="14" t="s">
-        <v>501</v>
+        <v>505</v>
       </c>
       <c r="D722" s="15" t="s">
-        <v>502</v>
+        <v>506</v>
       </c>
       <c r="E722" s="15" t="s">
-        <v>503</v>
+        <v>507</v>
       </c>
       <c r="F722" s="15" t="s">
-        <v>504</v>
+        <v>508</v>
       </c>
       <c r="G722" s="16" t="s">
         <v>58</v>
@@ -20868,19 +20907,19 @@
     </row>
     <row r="728" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A728" s="43" t="s">
-        <v>492</v>
+        <v>496</v>
       </c>
       <c r="B728" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C728" s="25" t="s">
-        <v>505</v>
+        <v>509</v>
       </c>
       <c r="D728" s="26" t="s">
         <v>216</v>
       </c>
       <c r="E728" s="26" t="s">
-        <v>503</v>
+        <v>507</v>
       </c>
       <c r="F728" s="26" t="s">
         <v>218</v>
@@ -21012,22 +21051,22 @@
     </row>
     <row r="734" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A734" s="44" t="s">
-        <v>506</v>
+        <v>510</v>
       </c>
       <c r="B734" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C734" s="14" t="s">
-        <v>507</v>
+        <v>511</v>
       </c>
       <c r="D734" s="15" t="s">
-        <v>508</v>
+        <v>512</v>
       </c>
       <c r="E734" s="15" t="s">
-        <v>509</v>
+        <v>513</v>
       </c>
       <c r="F734" s="15" t="s">
-        <v>510</v>
+        <v>514</v>
       </c>
       <c r="G734" s="16" t="s">
         <v>58</v>
@@ -21156,22 +21195,22 @@
     </row>
     <row r="740" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A740" s="44" t="s">
-        <v>506</v>
+        <v>510</v>
       </c>
       <c r="B740" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C740" s="25" t="s">
-        <v>511</v>
+        <v>515</v>
       </c>
       <c r="D740" s="26" t="s">
-        <v>512</v>
+        <v>516</v>
       </c>
       <c r="E740" s="26" t="s">
-        <v>513</v>
+        <v>517</v>
       </c>
       <c r="F740" s="26" t="s">
-        <v>514</v>
+        <v>518</v>
       </c>
       <c r="G740" s="16" t="s">
         <v>58</v>
@@ -21300,22 +21339,22 @@
     </row>
     <row r="746" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A746" s="44" t="s">
-        <v>506</v>
+        <v>510</v>
       </c>
       <c r="B746" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C746" s="14" t="s">
-        <v>515</v>
+        <v>519</v>
       </c>
       <c r="D746" s="15" t="s">
-        <v>516</v>
+        <v>520</v>
       </c>
       <c r="E746" s="15" t="s">
-        <v>517</v>
+        <v>521</v>
       </c>
       <c r="F746" s="15" t="s">
-        <v>518</v>
+        <v>522</v>
       </c>
       <c r="G746" s="16" t="s">
         <v>58</v>
@@ -21444,22 +21483,22 @@
     </row>
     <row r="752" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A752" s="44" t="s">
-        <v>506</v>
+        <v>510</v>
       </c>
       <c r="B752" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C752" s="25" t="s">
-        <v>519</v>
+        <v>523</v>
       </c>
       <c r="D752" s="26" t="s">
-        <v>520</v>
+        <v>524</v>
       </c>
       <c r="E752" s="26" t="s">
-        <v>521</v>
+        <v>525</v>
       </c>
       <c r="F752" s="26" t="s">
-        <v>522</v>
+        <v>526</v>
       </c>
       <c r="G752" s="16" t="s">
         <v>58</v>
@@ -21588,22 +21627,22 @@
     </row>
     <row r="758" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A758" s="44" t="s">
-        <v>506</v>
+        <v>510</v>
       </c>
       <c r="B758" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C758" s="14" t="s">
-        <v>523</v>
+        <v>527</v>
       </c>
       <c r="D758" s="15" t="s">
-        <v>524</v>
+        <v>528</v>
       </c>
       <c r="E758" s="15" t="s">
-        <v>525</v>
+        <v>529</v>
       </c>
       <c r="F758" s="15" t="s">
-        <v>526</v>
+        <v>530</v>
       </c>
       <c r="G758" s="16" t="s">
         <v>58</v>
@@ -21732,22 +21771,22 @@
     </row>
     <row r="764" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A764" s="45" t="s">
-        <v>527</v>
+        <v>531</v>
       </c>
       <c r="B764" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C764" s="25" t="s">
-        <v>528</v>
+        <v>532</v>
       </c>
       <c r="D764" s="26" t="s">
-        <v>529</v>
+        <v>533</v>
       </c>
       <c r="E764" s="26" t="s">
-        <v>530</v>
+        <v>534</v>
       </c>
       <c r="F764" s="26" t="s">
-        <v>531</v>
+        <v>535</v>
       </c>
       <c r="G764" s="16" t="s">
         <v>58</v>
@@ -21876,22 +21915,22 @@
     </row>
     <row r="770" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A770" s="45" t="s">
-        <v>527</v>
+        <v>531</v>
       </c>
       <c r="B770" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C770" s="14" t="s">
-        <v>532</v>
+        <v>536</v>
       </c>
       <c r="D770" s="15" t="s">
-        <v>533</v>
+        <v>537</v>
       </c>
       <c r="E770" s="15" t="s">
-        <v>534</v>
+        <v>538</v>
       </c>
       <c r="F770" s="15" t="s">
-        <v>535</v>
+        <v>539</v>
       </c>
       <c r="G770" s="16" t="s">
         <v>58</v>
@@ -22020,22 +22059,22 @@
     </row>
     <row r="776" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A776" s="45" t="s">
-        <v>527</v>
+        <v>531</v>
       </c>
       <c r="B776" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C776" s="25" t="s">
-        <v>536</v>
+        <v>540</v>
       </c>
       <c r="D776" s="26" t="s">
-        <v>537</v>
+        <v>541</v>
       </c>
       <c r="E776" s="26" t="s">
-        <v>538</v>
+        <v>542</v>
       </c>
       <c r="F776" s="26" t="s">
-        <v>539</v>
+        <v>543</v>
       </c>
       <c r="G776" s="16" t="s">
         <v>58</v>
@@ -22164,22 +22203,22 @@
     </row>
     <row r="782" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A782" s="45" t="s">
-        <v>527</v>
+        <v>531</v>
       </c>
       <c r="B782" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C782" s="14" t="s">
-        <v>540</v>
+        <v>544</v>
       </c>
       <c r="D782" s="15" t="s">
-        <v>541</v>
+        <v>545</v>
       </c>
       <c r="E782" s="15" t="s">
-        <v>542</v>
+        <v>546</v>
       </c>
       <c r="F782" s="15" t="s">
-        <v>543</v>
+        <v>547</v>
       </c>
       <c r="G782" s="16" t="s">
         <v>58</v>
@@ -22308,22 +22347,22 @@
     </row>
     <row r="788" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A788" s="45" t="s">
-        <v>527</v>
+        <v>531</v>
       </c>
       <c r="B788" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C788" s="25" t="s">
-        <v>544</v>
+        <v>548</v>
       </c>
       <c r="D788" s="26" t="s">
-        <v>545</v>
+        <v>549</v>
       </c>
       <c r="E788" s="26" t="s">
-        <v>546</v>
+        <v>550</v>
       </c>
       <c r="F788" s="26" t="s">
-        <v>547</v>
+        <v>551</v>
       </c>
       <c r="G788" s="16" t="s">
         <v>58</v>
@@ -22452,22 +22491,22 @@
     </row>
     <row r="794" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A794" s="45" t="s">
-        <v>527</v>
+        <v>531</v>
       </c>
       <c r="B794" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C794" s="14" t="s">
-        <v>548</v>
+        <v>552</v>
       </c>
       <c r="D794" s="15" t="s">
-        <v>549</v>
+        <v>553</v>
       </c>
       <c r="E794" s="15" t="s">
-        <v>550</v>
+        <v>554</v>
       </c>
       <c r="F794" s="15" t="s">
-        <v>547</v>
+        <v>551</v>
       </c>
       <c r="G794" s="16" t="s">
         <v>58</v>
@@ -22596,22 +22635,22 @@
     </row>
     <row r="800" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A800" s="45" t="s">
-        <v>527</v>
+        <v>531</v>
       </c>
       <c r="B800" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C800" s="25" t="s">
-        <v>551</v>
+        <v>555</v>
       </c>
       <c r="D800" s="26" t="s">
-        <v>552</v>
+        <v>556</v>
       </c>
       <c r="E800" s="26" t="s">
-        <v>553</v>
+        <v>557</v>
       </c>
       <c r="F800" s="26" t="s">
-        <v>554</v>
+        <v>558</v>
       </c>
       <c r="G800" s="16" t="s">
         <v>58</v>
@@ -22740,22 +22779,22 @@
     </row>
     <row r="806" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A806" s="45" t="s">
-        <v>527</v>
+        <v>531</v>
       </c>
       <c r="B806" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C806" s="14" t="s">
-        <v>555</v>
+        <v>559</v>
       </c>
       <c r="D806" s="15" t="s">
-        <v>556</v>
+        <v>560</v>
       </c>
       <c r="E806" s="15" t="s">
-        <v>557</v>
+        <v>561</v>
       </c>
       <c r="F806" s="15" t="s">
-        <v>558</v>
+        <v>562</v>
       </c>
       <c r="G806" s="16" t="s">
         <v>58</v>
@@ -22884,22 +22923,22 @@
     </row>
     <row r="812" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A812" s="45" t="s">
-        <v>527</v>
+        <v>531</v>
       </c>
       <c r="B812" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C812" s="25" t="s">
-        <v>559</v>
+        <v>563</v>
       </c>
       <c r="D812" s="26" t="s">
-        <v>560</v>
+        <v>564</v>
       </c>
       <c r="E812" s="26" t="s">
-        <v>561</v>
+        <v>565</v>
       </c>
       <c r="F812" s="26" t="s">
-        <v>562</v>
+        <v>566</v>
       </c>
       <c r="G812" s="16" t="s">
         <v>58</v>
@@ -23028,22 +23067,22 @@
     </row>
     <row r="818" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A818" s="45" t="s">
-        <v>527</v>
+        <v>531</v>
       </c>
       <c r="B818" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C818" s="14" t="s">
-        <v>563</v>
+        <v>567</v>
       </c>
       <c r="D818" s="15" t="s">
-        <v>564</v>
+        <v>568</v>
       </c>
       <c r="E818" s="15" t="s">
-        <v>565</v>
+        <v>569</v>
       </c>
       <c r="F818" s="15" t="s">
-        <v>566</v>
+        <v>570</v>
       </c>
       <c r="G818" s="16" t="s">
         <v>58</v>
@@ -23172,22 +23211,22 @@
     </row>
     <row r="824" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A824" s="45" t="s">
-        <v>527</v>
+        <v>531</v>
       </c>
       <c r="B824" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C824" s="25" t="s">
-        <v>567</v>
+        <v>571</v>
       </c>
       <c r="D824" s="26" t="s">
-        <v>568</v>
+        <v>572</v>
       </c>
       <c r="E824" s="26" t="s">
-        <v>569</v>
+        <v>573</v>
       </c>
       <c r="F824" s="26" t="s">
-        <v>570</v>
+        <v>574</v>
       </c>
       <c r="G824" s="16" t="s">
         <v>58</v>
@@ -23316,22 +23355,22 @@
     </row>
     <row r="830" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A830" s="45" t="s">
-        <v>527</v>
+        <v>531</v>
       </c>
       <c r="B830" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C830" s="14" t="s">
-        <v>571</v>
+        <v>575</v>
       </c>
       <c r="D830" s="15" t="s">
-        <v>572</v>
+        <v>576</v>
       </c>
       <c r="E830" s="15" t="s">
-        <v>573</v>
+        <v>577</v>
       </c>
       <c r="F830" s="15" t="s">
-        <v>574</v>
+        <v>578</v>
       </c>
       <c r="G830" s="16" t="s">
         <v>58</v>
@@ -23460,22 +23499,22 @@
     </row>
     <row r="836" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A836" s="46" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="B836" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C836" s="25" t="s">
-        <v>576</v>
+        <v>580</v>
       </c>
       <c r="D836" s="26" t="s">
-        <v>577</v>
+        <v>581</v>
       </c>
       <c r="E836" s="26" t="s">
-        <v>578</v>
+        <v>582</v>
       </c>
       <c r="F836" s="26" t="s">
-        <v>579</v>
+        <v>583</v>
       </c>
       <c r="G836" s="16" t="s">
         <v>58</v>
@@ -23604,22 +23643,22 @@
     </row>
     <row r="842" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A842" s="46" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="B842" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C842" s="14" t="s">
-        <v>580</v>
+        <v>584</v>
       </c>
       <c r="D842" s="15" t="s">
-        <v>581</v>
+        <v>585</v>
       </c>
       <c r="E842" s="15" t="s">
-        <v>582</v>
+        <v>586</v>
       </c>
       <c r="F842" s="15" t="s">
-        <v>518</v>
+        <v>522</v>
       </c>
       <c r="G842" s="16" t="s">
         <v>58</v>
@@ -23748,22 +23787,22 @@
     </row>
     <row r="848" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A848" s="46" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="B848" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C848" s="25" t="s">
-        <v>583</v>
+        <v>587</v>
       </c>
       <c r="D848" s="26" t="s">
-        <v>584</v>
+        <v>588</v>
       </c>
       <c r="E848" s="26" t="s">
-        <v>585</v>
+        <v>589</v>
       </c>
       <c r="F848" s="26" t="s">
-        <v>586</v>
+        <v>590</v>
       </c>
       <c r="G848" s="16" t="s">
         <v>58</v>
@@ -23892,22 +23931,22 @@
     </row>
     <row r="854" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A854" s="46" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="B854" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C854" s="14" t="s">
-        <v>587</v>
+        <v>591</v>
       </c>
       <c r="D854" s="15" t="s">
-        <v>588</v>
+        <v>592</v>
       </c>
       <c r="E854" s="15" t="s">
-        <v>589</v>
+        <v>593</v>
       </c>
       <c r="F854" s="15" t="s">
-        <v>590</v>
+        <v>594</v>
       </c>
       <c r="G854" s="16" t="s">
         <v>58</v>
@@ -24036,22 +24075,22 @@
     </row>
     <row r="860" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A860" s="47" t="s">
-        <v>591</v>
+        <v>595</v>
       </c>
       <c r="B860" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C860" s="25" t="s">
-        <v>592</v>
+        <v>596</v>
       </c>
       <c r="D860" s="26" t="s">
-        <v>593</v>
+        <v>597</v>
       </c>
       <c r="E860" s="26" t="s">
-        <v>594</v>
+        <v>598</v>
       </c>
       <c r="F860" s="26" t="s">
-        <v>595</v>
+        <v>599</v>
       </c>
       <c r="G860" s="16" t="s">
         <v>58</v>
@@ -24180,22 +24219,22 @@
     </row>
     <row r="866" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A866" s="47" t="s">
-        <v>591</v>
+        <v>595</v>
       </c>
       <c r="B866" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C866" s="14" t="s">
-        <v>596</v>
+        <v>600</v>
       </c>
       <c r="D866" s="15" t="s">
-        <v>597</v>
+        <v>601</v>
       </c>
       <c r="E866" s="15" t="s">
-        <v>598</v>
+        <v>602</v>
       </c>
       <c r="F866" s="15" t="s">
-        <v>599</v>
+        <v>603</v>
       </c>
       <c r="G866" s="16" t="s">
         <v>58</v>
@@ -24324,22 +24363,22 @@
     </row>
     <row r="872" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A872" s="47" t="s">
-        <v>591</v>
+        <v>595</v>
       </c>
       <c r="B872" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C872" s="25" t="s">
-        <v>600</v>
+        <v>604</v>
       </c>
       <c r="D872" s="26" t="s">
-        <v>601</v>
+        <v>605</v>
       </c>
       <c r="E872" s="26" t="s">
-        <v>602</v>
+        <v>606</v>
       </c>
       <c r="F872" s="26" t="s">
-        <v>603</v>
+        <v>607</v>
       </c>
       <c r="G872" s="16" t="s">
         <v>58</v>
@@ -24468,22 +24507,22 @@
     </row>
     <row r="878" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A878" s="47" t="s">
-        <v>591</v>
+        <v>595</v>
       </c>
       <c r="B878" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C878" s="14" t="s">
-        <v>604</v>
+        <v>608</v>
       </c>
       <c r="D878" s="15" t="s">
-        <v>605</v>
+        <v>609</v>
       </c>
       <c r="E878" s="15" t="s">
-        <v>606</v>
+        <v>610</v>
       </c>
       <c r="F878" s="15" t="s">
-        <v>607</v>
+        <v>611</v>
       </c>
       <c r="G878" s="16" t="s">
         <v>58</v>
@@ -24612,22 +24651,22 @@
     </row>
     <row r="884" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A884" s="47" t="s">
-        <v>591</v>
+        <v>595</v>
       </c>
       <c r="B884" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C884" s="25" t="s">
-        <v>608</v>
+        <v>612</v>
       </c>
       <c r="D884" s="26" t="s">
-        <v>609</v>
+        <v>613</v>
       </c>
       <c r="E884" s="26" t="s">
-        <v>610</v>
+        <v>614</v>
       </c>
       <c r="F884" s="26" t="s">
-        <v>611</v>
+        <v>615</v>
       </c>
       <c r="G884" s="16" t="s">
         <v>58</v>
@@ -24756,22 +24795,22 @@
     </row>
     <row r="890" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A890" s="47" t="s">
-        <v>591</v>
+        <v>595</v>
       </c>
       <c r="B890" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C890" s="14" t="s">
-        <v>612</v>
+        <v>616</v>
       </c>
       <c r="D890" s="15" t="s">
-        <v>613</v>
+        <v>617</v>
       </c>
       <c r="E890" s="15" t="s">
-        <v>614</v>
+        <v>618</v>
       </c>
       <c r="F890" s="15" t="s">
-        <v>615</v>
+        <v>619</v>
       </c>
       <c r="G890" s="16" t="s">
         <v>58</v>
@@ -24900,22 +24939,22 @@
     </row>
     <row r="896" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A896" s="47" t="s">
-        <v>591</v>
+        <v>595</v>
       </c>
       <c r="B896" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C896" s="25" t="s">
-        <v>616</v>
+        <v>620</v>
       </c>
       <c r="D896" s="26" t="s">
-        <v>617</v>
+        <v>621</v>
       </c>
       <c r="E896" s="26" t="s">
-        <v>618</v>
+        <v>622</v>
       </c>
       <c r="F896" s="26" t="s">
-        <v>619</v>
+        <v>623</v>
       </c>
       <c r="G896" s="16" t="s">
         <v>58</v>
@@ -25044,22 +25083,22 @@
     </row>
     <row r="902" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A902" s="48" t="s">
-        <v>620</v>
+        <v>624</v>
       </c>
       <c r="B902" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C902" s="14" t="s">
-        <v>621</v>
+        <v>625</v>
       </c>
       <c r="D902" s="15" t="s">
-        <v>622</v>
+        <v>626</v>
       </c>
       <c r="E902" s="15" t="s">
-        <v>623</v>
+        <v>627</v>
       </c>
       <c r="F902" s="15" t="s">
-        <v>624</v>
+        <v>628</v>
       </c>
       <c r="G902" s="16" t="s">
         <v>58</v>
@@ -25188,22 +25227,22 @@
     </row>
     <row r="908" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A908" s="48" t="s">
-        <v>620</v>
+        <v>624</v>
       </c>
       <c r="B908" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C908" s="25" t="s">
-        <v>625</v>
+        <v>629</v>
       </c>
       <c r="D908" s="26" t="s">
-        <v>626</v>
+        <v>630</v>
       </c>
       <c r="E908" s="26" t="s">
-        <v>627</v>
+        <v>631</v>
       </c>
       <c r="F908" s="26" t="s">
-        <v>628</v>
+        <v>632</v>
       </c>
       <c r="G908" s="16" t="s">
         <v>58</v>
@@ -25332,22 +25371,22 @@
     </row>
     <row r="914" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A914" s="48" t="s">
-        <v>620</v>
+        <v>624</v>
       </c>
       <c r="B914" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C914" s="14" t="s">
-        <v>629</v>
+        <v>633</v>
       </c>
       <c r="D914" s="15" t="s">
-        <v>630</v>
+        <v>634</v>
       </c>
       <c r="E914" s="15" t="s">
-        <v>631</v>
+        <v>635</v>
       </c>
       <c r="F914" s="15" t="s">
-        <v>632</v>
+        <v>636</v>
       </c>
       <c r="G914" s="16" t="s">
         <v>58</v>
@@ -25476,22 +25515,22 @@
     </row>
     <row r="920" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A920" s="48" t="s">
-        <v>620</v>
+        <v>624</v>
       </c>
       <c r="B920" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C920" s="25" t="s">
-        <v>633</v>
+        <v>637</v>
       </c>
       <c r="D920" s="26" t="s">
-        <v>634</v>
+        <v>638</v>
       </c>
       <c r="E920" s="26" t="s">
-        <v>635</v>
+        <v>639</v>
       </c>
       <c r="F920" s="26" t="s">
-        <v>636</v>
+        <v>640</v>
       </c>
       <c r="G920" s="16" t="s">
         <v>58</v>
@@ -25620,22 +25659,22 @@
     </row>
     <row r="926" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A926" s="48" t="s">
-        <v>620</v>
+        <v>624</v>
       </c>
       <c r="B926" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C926" s="14" t="s">
-        <v>637</v>
+        <v>641</v>
       </c>
       <c r="D926" s="15" t="s">
-        <v>638</v>
+        <v>642</v>
       </c>
       <c r="E926" s="15" t="s">
-        <v>639</v>
+        <v>643</v>
       </c>
       <c r="F926" s="15" t="s">
-        <v>640</v>
+        <v>644</v>
       </c>
       <c r="G926" s="16" t="s">
         <v>58</v>
@@ -25764,22 +25803,22 @@
     </row>
     <row r="932" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A932" s="48" t="s">
-        <v>620</v>
+        <v>624</v>
       </c>
       <c r="B932" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C932" s="25" t="s">
-        <v>641</v>
+        <v>645</v>
       </c>
       <c r="D932" s="26" t="s">
-        <v>642</v>
+        <v>646</v>
       </c>
       <c r="E932" s="26" t="s">
-        <v>643</v>
+        <v>647</v>
       </c>
       <c r="F932" s="26" t="s">
-        <v>644</v>
+        <v>648</v>
       </c>
       <c r="G932" s="16" t="s">
         <v>58</v>
@@ -25908,22 +25947,22 @@
     </row>
     <row r="938" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A938" s="49" t="s">
-        <v>645</v>
+        <v>649</v>
       </c>
       <c r="B938" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C938" s="14" t="s">
-        <v>646</v>
+        <v>650</v>
       </c>
       <c r="D938" s="15" t="s">
-        <v>647</v>
+        <v>651</v>
       </c>
       <c r="E938" s="15" t="s">
-        <v>648</v>
+        <v>652</v>
       </c>
       <c r="F938" s="15" t="s">
-        <v>649</v>
+        <v>653</v>
       </c>
       <c r="G938" s="16" t="s">
         <v>58</v>
@@ -26052,22 +26091,22 @@
     </row>
     <row r="944" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A944" s="49" t="s">
-        <v>645</v>
+        <v>649</v>
       </c>
       <c r="B944" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C944" s="25" t="s">
-        <v>650</v>
+        <v>654</v>
       </c>
       <c r="D944" s="26" t="s">
-        <v>651</v>
+        <v>655</v>
       </c>
       <c r="E944" s="26" t="s">
-        <v>652</v>
+        <v>656</v>
       </c>
       <c r="F944" s="26" t="s">
-        <v>653</v>
+        <v>657</v>
       </c>
       <c r="G944" s="16" t="s">
         <v>58</v>
@@ -26196,22 +26235,22 @@
     </row>
     <row r="950" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A950" s="49" t="s">
-        <v>645</v>
+        <v>649</v>
       </c>
       <c r="B950" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C950" s="14" t="s">
-        <v>654</v>
+        <v>658</v>
       </c>
       <c r="D950" s="15" t="s">
-        <v>655</v>
+        <v>659</v>
       </c>
       <c r="E950" s="15" t="s">
-        <v>656</v>
+        <v>660</v>
       </c>
       <c r="F950" s="15" t="s">
-        <v>657</v>
+        <v>661</v>
       </c>
       <c r="G950" s="16" t="s">
         <v>58</v>
@@ -26340,22 +26379,22 @@
     </row>
     <row r="956" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A956" s="49" t="s">
-        <v>645</v>
+        <v>649</v>
       </c>
       <c r="B956" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C956" s="25" t="s">
-        <v>658</v>
+        <v>662</v>
       </c>
       <c r="D956" s="26" t="s">
-        <v>659</v>
+        <v>663</v>
       </c>
       <c r="E956" s="26" t="s">
-        <v>660</v>
+        <v>664</v>
       </c>
       <c r="F956" s="26" t="s">
-        <v>632</v>
+        <v>636</v>
       </c>
       <c r="G956" s="16" t="s">
         <v>58</v>
@@ -26484,22 +26523,22 @@
     </row>
     <row r="962" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A962" s="49" t="s">
-        <v>645</v>
+        <v>649</v>
       </c>
       <c r="B962" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C962" s="14" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="D962" s="15" t="s">
-        <v>662</v>
+        <v>666</v>
       </c>
       <c r="E962" s="15" t="s">
-        <v>663</v>
+        <v>667</v>
       </c>
       <c r="F962" s="15" t="s">
-        <v>664</v>
+        <v>668</v>
       </c>
       <c r="G962" s="16" t="s">
         <v>58</v>
@@ -26628,22 +26667,22 @@
     </row>
     <row r="968" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A968" s="49" t="s">
-        <v>645</v>
+        <v>649</v>
       </c>
       <c r="B968" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C968" s="25" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="D968" s="26" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="E968" s="26" t="s">
-        <v>667</v>
+        <v>671</v>
       </c>
       <c r="F968" s="26" t="s">
-        <v>668</v>
+        <v>672</v>
       </c>
       <c r="G968" s="16" t="s">
         <v>58</v>
@@ -26772,22 +26811,22 @@
     </row>
     <row r="974" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A974" s="50" t="s">
-        <v>669</v>
+        <v>673</v>
       </c>
       <c r="B974" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C974" s="14" t="s">
-        <v>670</v>
+        <v>674</v>
       </c>
       <c r="D974" s="15" t="s">
-        <v>671</v>
+        <v>675</v>
       </c>
       <c r="E974" s="15" t="s">
-        <v>672</v>
+        <v>676</v>
       </c>
       <c r="F974" s="15" t="s">
-        <v>673</v>
+        <v>677</v>
       </c>
       <c r="G974" s="16" t="s">
         <v>58</v>
@@ -26916,22 +26955,22 @@
     </row>
     <row r="980" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A980" s="50" t="s">
-        <v>669</v>
+        <v>673</v>
       </c>
       <c r="B980" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C980" s="25" t="s">
-        <v>674</v>
+        <v>678</v>
       </c>
       <c r="D980" s="26" t="s">
-        <v>675</v>
+        <v>679</v>
       </c>
       <c r="E980" s="26" t="s">
-        <v>676</v>
+        <v>680</v>
       </c>
       <c r="F980" s="26" t="s">
-        <v>677</v>
+        <v>681</v>
       </c>
       <c r="G980" s="16" t="s">
         <v>58</v>
@@ -27060,22 +27099,22 @@
     </row>
     <row r="986" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A986" s="50" t="s">
-        <v>669</v>
+        <v>673</v>
       </c>
       <c r="B986" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C986" s="14" t="s">
-        <v>678</v>
+        <v>682</v>
       </c>
       <c r="D986" s="15" t="s">
-        <v>679</v>
+        <v>683</v>
       </c>
       <c r="E986" s="15" t="s">
-        <v>680</v>
+        <v>684</v>
       </c>
       <c r="F986" s="15" t="s">
-        <v>681</v>
+        <v>685</v>
       </c>
       <c r="G986" s="16" t="s">
         <v>58</v>
@@ -27204,22 +27243,22 @@
     </row>
     <row r="992" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A992" s="50" t="s">
-        <v>669</v>
+        <v>673</v>
       </c>
       <c r="B992" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C992" s="25" t="s">
-        <v>682</v>
+        <v>686</v>
       </c>
       <c r="D992" s="26" t="s">
-        <v>683</v>
+        <v>687</v>
       </c>
       <c r="E992" s="26" t="s">
-        <v>684</v>
+        <v>688</v>
       </c>
       <c r="F992" s="26" t="s">
-        <v>685</v>
+        <v>689</v>
       </c>
       <c r="G992" s="16" t="s">
         <v>58</v>
@@ -27348,22 +27387,22 @@
     </row>
     <row r="998" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A998" s="50" t="s">
-        <v>669</v>
+        <v>673</v>
       </c>
       <c r="B998" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C998" s="14" t="s">
-        <v>686</v>
+        <v>690</v>
       </c>
       <c r="D998" s="15" t="s">
-        <v>687</v>
+        <v>691</v>
       </c>
       <c r="E998" s="15" t="s">
-        <v>688</v>
+        <v>692</v>
       </c>
       <c r="F998" s="15" t="s">
-        <v>689</v>
+        <v>693</v>
       </c>
       <c r="G998" s="16" t="s">
         <v>58</v>
@@ -27492,22 +27531,22 @@
     </row>
     <row r="1004" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1004" s="51" t="s">
-        <v>690</v>
+        <v>694</v>
       </c>
       <c r="B1004" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1004" s="25" t="s">
-        <v>691</v>
+        <v>695</v>
       </c>
       <c r="D1004" s="26" t="s">
-        <v>692</v>
+        <v>696</v>
       </c>
       <c r="E1004" s="26" t="s">
-        <v>693</v>
+        <v>697</v>
       </c>
       <c r="F1004" s="26" t="s">
-        <v>694</v>
+        <v>698</v>
       </c>
       <c r="G1004" s="16" t="s">
         <v>58</v>
@@ -27636,22 +27675,22 @@
     </row>
     <row r="1010" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1010" s="51" t="s">
-        <v>690</v>
+        <v>694</v>
       </c>
       <c r="B1010" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1010" s="14" t="s">
-        <v>695</v>
+        <v>699</v>
       </c>
       <c r="D1010" s="15" t="s">
-        <v>696</v>
+        <v>700</v>
       </c>
       <c r="E1010" s="15" t="s">
-        <v>697</v>
+        <v>701</v>
       </c>
       <c r="F1010" s="15" t="s">
-        <v>698</v>
+        <v>702</v>
       </c>
       <c r="G1010" s="16" t="s">
         <v>58</v>
@@ -27780,22 +27819,22 @@
     </row>
     <row r="1016" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1016" s="51" t="s">
-        <v>690</v>
+        <v>694</v>
       </c>
       <c r="B1016" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1016" s="25" t="s">
-        <v>699</v>
+        <v>703</v>
       </c>
       <c r="D1016" s="26" t="s">
-        <v>700</v>
+        <v>704</v>
       </c>
       <c r="E1016" s="26" t="s">
-        <v>701</v>
+        <v>705</v>
       </c>
       <c r="F1016" s="26" t="s">
-        <v>702</v>
+        <v>706</v>
       </c>
       <c r="G1016" s="16" t="s">
         <v>58</v>
@@ -27924,22 +27963,22 @@
     </row>
     <row r="1022" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1022" s="51" t="s">
-        <v>690</v>
+        <v>694</v>
       </c>
       <c r="B1022" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1022" s="14" t="s">
-        <v>703</v>
+        <v>707</v>
       </c>
       <c r="D1022" s="15" t="s">
-        <v>704</v>
+        <v>708</v>
       </c>
       <c r="E1022" s="15" t="s">
-        <v>705</v>
+        <v>709</v>
       </c>
       <c r="F1022" s="15" t="s">
-        <v>706</v>
+        <v>710</v>
       </c>
       <c r="G1022" s="16" t="s">
         <v>58</v>
@@ -28068,22 +28107,22 @@
     </row>
     <row r="1028" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1028" s="51" t="s">
-        <v>690</v>
+        <v>694</v>
       </c>
       <c r="B1028" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C1028" s="25" t="s">
-        <v>707</v>
+        <v>711</v>
       </c>
       <c r="D1028" s="26" t="s">
-        <v>708</v>
+        <v>712</v>
       </c>
       <c r="E1028" s="26" t="s">
-        <v>709</v>
+        <v>713</v>
       </c>
       <c r="F1028" s="26" t="s">
-        <v>710</v>
+        <v>714</v>
       </c>
       <c r="G1028" s="16" t="s">
         <v>58</v>
@@ -28212,22 +28251,22 @@
     </row>
     <row r="1034" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1034" s="51" t="s">
-        <v>690</v>
+        <v>694</v>
       </c>
       <c r="B1034" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C1034" s="14" t="s">
-        <v>711</v>
+        <v>715</v>
       </c>
       <c r="D1034" s="15" t="s">
-        <v>712</v>
+        <v>716</v>
       </c>
       <c r="E1034" s="15" t="s">
-        <v>713</v>
+        <v>717</v>
       </c>
       <c r="F1034" s="15" t="s">
-        <v>714</v>
+        <v>718</v>
       </c>
       <c r="G1034" s="16" t="s">
         <v>58</v>
@@ -28356,22 +28395,22 @@
     </row>
     <row r="1040" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1040" s="52" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="B1040" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C1040" s="25" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="D1040" s="26" t="s">
-        <v>704</v>
+        <v>708</v>
       </c>
       <c r="E1040" s="26" t="s">
-        <v>717</v>
+        <v>721</v>
       </c>
       <c r="F1040" s="26" t="s">
-        <v>718</v>
+        <v>722</v>
       </c>
       <c r="G1040" s="16" t="s">
         <v>58</v>
@@ -28500,22 +28539,22 @@
     </row>
     <row r="1046" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1046" s="52" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="B1046" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1046" s="14" t="s">
-        <v>719</v>
+        <v>723</v>
       </c>
       <c r="D1046" s="15" t="s">
-        <v>696</v>
+        <v>700</v>
       </c>
       <c r="E1046" s="15" t="s">
-        <v>720</v>
+        <v>724</v>
       </c>
       <c r="F1046" s="15" t="s">
-        <v>721</v>
+        <v>725</v>
       </c>
       <c r="G1046" s="16" t="s">
         <v>58</v>
@@ -28652,16 +28691,16 @@
         <v>53</v>
       </c>
       <c r="C1052" s="25" t="s">
-        <v>722</v>
+        <v>726</v>
       </c>
       <c r="D1052" s="26" t="s">
-        <v>723</v>
+        <v>727</v>
       </c>
       <c r="E1052" s="26" t="s">
-        <v>724</v>
+        <v>728</v>
       </c>
       <c r="F1052" s="26" t="s">
-        <v>725</v>
+        <v>729</v>
       </c>
       <c r="G1052" s="16" t="s">
         <v>58</v>
@@ -28798,16 +28837,16 @@
         <v>53</v>
       </c>
       <c r="C1058" s="14" t="s">
-        <v>726</v>
+        <v>730</v>
       </c>
       <c r="D1058" s="15" t="s">
-        <v>727</v>
+        <v>731</v>
       </c>
       <c r="E1058" s="15" t="s">
-        <v>728</v>
+        <v>732</v>
       </c>
       <c r="F1058" s="15" t="s">
-        <v>729</v>
+        <v>733</v>
       </c>
       <c r="G1058" s="16" t="s">
         <v>58</v>
@@ -29893,10 +29932,10 @@
         <v>39</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>730</v>
+        <v>734</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>731</v>
+        <v>735</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>53</v>
@@ -29914,7 +29953,7 @@
         <v>86</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>732</v>
+        <v>736</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -30093,7 +30132,7 @@
     </row>
     <row r="8" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="59" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="B8" s="1">
         <v>10</v>
@@ -30122,7 +30161,7 @@
     </row>
     <row r="9" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="60" t="s">
-        <v>364</v>
+        <v>368</v>
       </c>
       <c r="B9" s="1">
         <v>11</v>
@@ -30151,7 +30190,7 @@
     </row>
     <row r="10" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="61" t="s">
-        <v>410</v>
+        <v>414</v>
       </c>
       <c r="B10" s="1">
         <v>9</v>
@@ -30180,7 +30219,7 @@
     </row>
     <row r="11" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="62" t="s">
-        <v>449</v>
+        <v>453</v>
       </c>
       <c r="B11" s="1">
         <v>5</v>
@@ -30209,7 +30248,7 @@
     </row>
     <row r="12" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="63" t="s">
-        <v>472</v>
+        <v>476</v>
       </c>
       <c r="B12" s="1">
         <v>5</v>
@@ -30238,7 +30277,7 @@
     </row>
     <row r="13" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="64" t="s">
-        <v>492</v>
+        <v>496</v>
       </c>
       <c r="B13" s="1">
         <v>4</v>
@@ -30267,7 +30306,7 @@
     </row>
     <row r="14" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="65" t="s">
-        <v>506</v>
+        <v>510</v>
       </c>
       <c r="B14" s="1">
         <v>5</v>
@@ -30296,7 +30335,7 @@
     </row>
     <row r="15" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="66" t="s">
-        <v>527</v>
+        <v>531</v>
       </c>
       <c r="B15" s="1">
         <v>12</v>
@@ -30325,7 +30364,7 @@
     </row>
     <row r="16" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="67" t="s">
-        <v>575</v>
+        <v>579</v>
       </c>
       <c r="B16" s="1">
         <v>4</v>
@@ -30354,7 +30393,7 @@
     </row>
     <row r="17" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="68" t="s">
-        <v>591</v>
+        <v>595</v>
       </c>
       <c r="B17" s="1">
         <v>7</v>
@@ -30383,7 +30422,7 @@
     </row>
     <row r="18" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="69" t="s">
-        <v>620</v>
+        <v>624</v>
       </c>
       <c r="B18" s="1">
         <v>6</v>
@@ -30412,7 +30451,7 @@
     </row>
     <row r="19" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="70" t="s">
-        <v>645</v>
+        <v>649</v>
       </c>
       <c r="B19" s="1">
         <v>6</v>
@@ -30441,7 +30480,7 @@
     </row>
     <row r="20" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="71" t="s">
-        <v>669</v>
+        <v>673</v>
       </c>
       <c r="B20" s="1">
         <v>5</v>
@@ -30470,7 +30509,7 @@
     </row>
     <row r="21" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="72" t="s">
-        <v>690</v>
+        <v>694</v>
       </c>
       <c r="B21" s="1">
         <v>6</v>
@@ -30499,7 +30538,7 @@
     </row>
     <row r="22" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="73" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="B22" s="1">
         <v>2</v>
@@ -30528,7 +30567,7 @@
     </row>
     <row r="23" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="74" t="s">
-        <v>733</v>
+        <v>737</v>
       </c>
       <c r="B23" s="74">
         <v>153</v>
@@ -30579,7 +30618,7 @@
         <v>44</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>731</v>
+        <v>735</v>
       </c>
       <c r="C1" s="10" t="s">
         <v>71</v>
@@ -30588,7 +30627,7 @@
         <v>86</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>732</v>
+        <v>736</v>
       </c>
       <c r="F1" s="10" t="s">
         <v>94</v>
@@ -30739,10 +30778,10 @@
         <v>45</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>734</v>
+        <v>738</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>731</v>
+        <v>735</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>71</v>
@@ -30751,7 +30790,7 @@
         <v>86</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>732</v>
+        <v>736</v>
       </c>
       <c r="G1" s="10" t="s">
         <v>94</v>
@@ -30762,7 +30801,7 @@
         <v>59</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>735</v>
+        <v>739</v>
       </c>
       <c r="C2" s="1">
         <f>COUNTIF(Proves!$H:$H,A2)</f>

</xml_diff>

<commit_message>
`090 => fase IV => xips fitxa (web/Google, botiga vs fleca), combo Excel EN CURS, ZUP-059 ZUP-061 OK (Chrome/USER) i millora llistat editorial anotada`
</commit_message>
<xml_diff>
--- a/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
+++ b/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
@@ -12,6 +12,7 @@
     <sheet sheetId="3" name="Resum" state="visible" r:id="rId6"/>
     <sheet sheetId="4" name="Resum navegadors" state="visible" r:id="rId7"/>
     <sheet sheetId="5" name="Resum rols" state="visible" r:id="rId8"/>
+    <sheet sheetId="6" name="Llistes" state="hidden" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase">Proves!$A$1:$K$1063</definedName>
@@ -21,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4354" uniqueCount="740">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4361" uniqueCount="743">
   <si>
     <t>Zuppeto — Joc de probes manual (totes les pantalles)</t>
   </si>
@@ -89,7 +90,7 @@
     <t>Columna Resultat</t>
   </si>
   <si>
-    <t>Omplir amb: OK · KO · PENDENT · N/A (per cada rol i navegador)</t>
+    <t>Combo: OK · KO · PENDENT · N/A · EN CURS. Cicle: PENDENT → EN CURS → OK / KO.</t>
   </si>
   <si>
     <t>Columna Data</t>
@@ -1136,6 +1137,9 @@
   </si>
   <si>
     <t>Indicador visible si escau</t>
+  </si>
+  <si>
+    <t>EN CURS</t>
   </si>
   <si>
     <t>ZUP-063</t>
@@ -2311,6 +2315,12 @@
   <si>
     <t>— (sense login)</t>
   </si>
+  <si>
+    <t>Estat</t>
+  </si>
+  <si>
+    <t>Combo de Resultat i Resultat Correcció (un valor per cel·la; EN CURS no es pot posar en una llista amb comes).</t>
+  </si>
 </sst>
 </file>
 
@@ -2318,9 +2328,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="dd/mm/yy"/>
-    <numFmt numFmtId="165" formatCode="dd-mm-yyyy"/>
+    <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="28" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -2330,8 +2340,8 @@
     </font>
     <font>
       <b/>
-      <color rgb="FF9C0006"/>
-      <sz val="10"/>
+      <color rgb="FF1D4ED8"/>
+      <sz val="11"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -2492,8 +2502,17 @@
       <sz val="11"/>
       <name val="Cambria"/>
     </font>
+    <font>
+      <b/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF166534"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
-  <fills count="41">
+  <fills count="42">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2502,7 +2521,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
+        <fgColor rgb="FFDBEAFE"/>
       </patternFill>
     </fill>
     <fill>
@@ -2730,6 +2749,11 @@
         <bgColor rgb="FFEFF6FF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDCFCE7"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -2773,7 +2797,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="84">
+  <cellXfs count="88">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3024,6 +3048,16 @@
     <xf numFmtId="0" fontId="23" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="bottom"/>
     </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="27" fillId="41" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -14062,9 +14096,11 @@
       <c r="H440" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="I440" s="18"/>
+      <c r="I440" s="18">
+        <v>46266.91666666667</v>
+      </c>
       <c r="J440" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K440" s="19"/>
       <c r="L440" s="18"/>
@@ -14360,9 +14396,11 @@
       <c r="H452" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="I452" s="18"/>
+      <c r="I452" s="18">
+        <v>46266.91666666667</v>
+      </c>
       <c r="J452" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K452" s="19"/>
       <c r="L452" s="18"/>
@@ -14506,7 +14544,7 @@
       </c>
       <c r="I458" s="18"/>
       <c r="J458" s="1" t="s">
-        <v>60</v>
+        <v>360</v>
       </c>
       <c r="K458" s="19"/>
       <c r="L458" s="18"/>
@@ -14631,16 +14669,16 @@
         <v>89</v>
       </c>
       <c r="C464" s="14" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="D464" s="15" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="E464" s="15" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="F464" s="15" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="G464" s="16" t="s">
         <v>58</v>
@@ -14775,16 +14813,16 @@
         <v>53</v>
       </c>
       <c r="C470" s="25" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="D470" s="26" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="E470" s="26" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="F470" s="26" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="G470" s="16" t="s">
         <v>58</v>
@@ -14915,22 +14953,22 @@
     </row>
     <row r="476" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A476" s="39" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="B476" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C476" s="14" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="D476" s="15" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="E476" s="15" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="F476" s="15" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="G476" s="16" t="s">
         <v>58</v>
@@ -14945,7 +14983,7 @@
         <v>71</v>
       </c>
       <c r="K476" s="19" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="L476" s="18"/>
       <c r="M476" s="1"/>
@@ -15063,22 +15101,22 @@
     </row>
     <row r="482" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A482" s="39" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="B482" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C482" s="25" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="D482" s="26" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="E482" s="26" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="F482" s="26" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="G482" s="16" t="s">
         <v>58</v>
@@ -15093,7 +15131,7 @@
         <v>71</v>
       </c>
       <c r="K482" s="19" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="L482" s="18"/>
       <c r="M482" s="1"/>
@@ -15211,22 +15249,22 @@
     </row>
     <row r="488" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A488" s="39" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="B488" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C488" s="14" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="D488" s="15" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="E488" s="15" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="F488" s="15" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="G488" s="16" t="s">
         <v>58</v>
@@ -15357,22 +15395,22 @@
     </row>
     <row r="494" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A494" s="39" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="B494" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C494" s="25" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="D494" s="26" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="E494" s="26" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="F494" s="26" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="G494" s="16" t="s">
         <v>58</v>
@@ -15501,22 +15539,22 @@
     </row>
     <row r="500" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A500" s="39" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="B500" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C500" s="14" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="D500" s="15" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="E500" s="15" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="F500" s="15" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="G500" s="16" t="s">
         <v>58</v>
@@ -15645,22 +15683,22 @@
     </row>
     <row r="506" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A506" s="39" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="B506" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C506" s="25" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="D506" s="26" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="E506" s="26" t="s">
         <v>254</v>
       </c>
       <c r="F506" s="26" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="G506" s="16" t="s">
         <v>58</v>
@@ -15789,22 +15827,22 @@
     </row>
     <row r="512" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A512" s="39" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="B512" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C512" s="14" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="D512" s="15" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="E512" s="15" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="F512" s="15" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="G512" s="16" t="s">
         <v>58</v>
@@ -15933,22 +15971,22 @@
     </row>
     <row r="518" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A518" s="39" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="B518" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C518" s="25" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="D518" s="26" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="E518" s="26" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="F518" s="26" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="G518" s="16" t="s">
         <v>58</v>
@@ -16077,22 +16115,22 @@
     </row>
     <row r="524" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A524" s="39" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="B524" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C524" s="14" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="D524" s="15" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="E524" s="15" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="F524" s="15" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="G524" s="16" t="s">
         <v>58</v>
@@ -16223,22 +16261,22 @@
     </row>
     <row r="530" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A530" s="39" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="B530" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C530" s="25" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="D530" s="26" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="E530" s="26" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="F530" s="26" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="G530" s="16" t="s">
         <v>58</v>
@@ -16369,22 +16407,22 @@
     </row>
     <row r="536" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A536" s="39" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="B536" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C536" s="14" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="D536" s="15" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="E536" s="15" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="F536" s="15" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="G536" s="16" t="s">
         <v>58</v>
@@ -16515,22 +16553,22 @@
     </row>
     <row r="542" ht="180" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A542" s="40" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="B542" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C542" s="25" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="D542" s="26" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="E542" s="26" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="F542" s="26" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="G542" s="16" t="s">
         <v>58</v>
@@ -16545,7 +16583,7 @@
         <v>86</v>
       </c>
       <c r="K542" s="19" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="L542" s="18">
         <v>46264.91666666667</v>
@@ -16554,7 +16592,7 @@
         <v>71</v>
       </c>
       <c r="N542" s="19" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
     </row>
     <row r="543" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -16669,22 +16707,22 @@
     </row>
     <row r="548" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A548" s="40" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="B548" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C548" s="14" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="D548" s="15" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="E548" s="15" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="F548" s="15" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="G548" s="16" t="s">
         <v>58</v>
@@ -16813,22 +16851,22 @@
     </row>
     <row r="554" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A554" s="40" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="B554" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C554" s="25" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="D554" s="26" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="E554" s="26" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="F554" s="26" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="G554" s="16" t="s">
         <v>58</v>
@@ -16959,22 +16997,22 @@
     </row>
     <row r="560" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A560" s="40" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="B560" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C560" s="14" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="D560" s="15" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="E560" s="15" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="F560" s="15" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="G560" s="16" t="s">
         <v>58</v>
@@ -17103,22 +17141,22 @@
     </row>
     <row r="566" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A566" s="40" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="B566" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C566" s="25" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="D566" s="26" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="E566" s="26" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="F566" s="26" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="G566" s="16" t="s">
         <v>58</v>
@@ -17247,22 +17285,22 @@
     </row>
     <row r="572" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A572" s="40" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="B572" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C572" s="14" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="D572" s="15" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="E572" s="15" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="F572" s="15" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="G572" s="16" t="s">
         <v>58</v>
@@ -17391,22 +17429,22 @@
     </row>
     <row r="578" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A578" s="40" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="B578" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C578" s="25" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="D578" s="26" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="E578" s="26" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="F578" s="26" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="G578" s="16" t="s">
         <v>58</v>
@@ -17537,22 +17575,22 @@
     </row>
     <row r="584" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A584" s="40" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="B584" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C584" s="14" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="D584" s="15" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="E584" s="15" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="F584" s="15" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="G584" s="16" t="s">
         <v>58</v>
@@ -17681,22 +17719,22 @@
     </row>
     <row r="590" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A590" s="40" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="B590" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C590" s="25" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="D590" s="26" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="E590" s="26" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="F590" s="26" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="G590" s="16" t="s">
         <v>58</v>
@@ -17827,22 +17865,22 @@
     </row>
     <row r="596" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A596" s="41" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="B596" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C596" s="14" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="D596" s="15" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="E596" s="15" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="F596" s="15" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="G596" s="16" t="s">
         <v>58</v>
@@ -17989,7 +18027,7 @@
         <v>86</v>
       </c>
       <c r="K602" s="19" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="L602" s="18">
         <v>46264.91666666667</v>
@@ -17998,7 +18036,7 @@
         <v>71</v>
       </c>
       <c r="N602" s="19" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
     </row>
     <row r="603" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -18377,22 +18415,22 @@
     </row>
     <row r="620" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A620" s="41" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="B620" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C620" s="25" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="D620" s="26" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="E620" s="26" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="F620" s="26" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="G620" s="16" t="s">
         <v>58</v>
@@ -18523,22 +18561,22 @@
     </row>
     <row r="626" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A626" s="41" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="B626" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C626" s="14" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="D626" s="15" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="E626" s="15" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="F626" s="15" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="G626" s="16" t="s">
         <v>58</v>
@@ -18669,22 +18707,22 @@
     </row>
     <row r="632" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A632" s="41" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="B632" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C632" s="25" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="D632" s="26" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="E632" s="26" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="F632" s="26" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="G632" s="16" t="s">
         <v>58</v>
@@ -18813,22 +18851,22 @@
     </row>
     <row r="638" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A638" s="41" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="B638" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C638" s="14" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="D638" s="15" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="E638" s="15" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="F638" s="15" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="G638" s="16" t="s">
         <v>58</v>
@@ -18959,22 +18997,22 @@
     </row>
     <row r="644" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A644" s="42" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="B644" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C644" s="25" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="D644" s="26" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="E644" s="26" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="F644" s="26" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="G644" s="16" t="s">
         <v>58</v>
@@ -19501,22 +19539,22 @@
     </row>
     <row r="668" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A668" s="42" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="B668" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C668" s="14" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="D668" s="15" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="E668" s="15" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="F668" s="15" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="G668" s="16" t="s">
         <v>58</v>
@@ -19645,22 +19683,22 @@
     </row>
     <row r="674" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A674" s="42" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="B674" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C674" s="25" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="D674" s="26" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="E674" s="26" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="F674" s="26" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="G674" s="16" t="s">
         <v>58</v>
@@ -19789,22 +19827,22 @@
     </row>
     <row r="680" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A680" s="42" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="B680" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C680" s="14" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="D680" s="15" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="E680" s="15" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="F680" s="15" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="G680" s="16" t="s">
         <v>58</v>
@@ -19933,22 +19971,22 @@
     </row>
     <row r="686" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A686" s="42" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="B686" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C686" s="25" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="D686" s="26" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="E686" s="26" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="F686" s="26" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="G686" s="16" t="s">
         <v>58</v>
@@ -20077,22 +20115,22 @@
     </row>
     <row r="692" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A692" s="43" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="B692" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C692" s="14" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="D692" s="15" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="E692" s="15" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="F692" s="15" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="G692" s="16" t="s">
         <v>58</v>
@@ -20619,22 +20657,22 @@
     </row>
     <row r="716" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A716" s="43" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="B716" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C716" s="25" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="D716" s="26" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="E716" s="26" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="F716" s="26" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="G716" s="16" t="s">
         <v>58</v>
@@ -20763,22 +20801,22 @@
     </row>
     <row r="722" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A722" s="43" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="B722" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C722" s="14" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="D722" s="15" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="E722" s="15" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="F722" s="15" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="G722" s="16" t="s">
         <v>58</v>
@@ -20907,19 +20945,19 @@
     </row>
     <row r="728" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A728" s="43" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="B728" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C728" s="25" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="D728" s="26" t="s">
         <v>216</v>
       </c>
       <c r="E728" s="26" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="F728" s="26" t="s">
         <v>218</v>
@@ -21051,22 +21089,22 @@
     </row>
     <row r="734" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A734" s="44" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="B734" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C734" s="14" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="D734" s="15" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="E734" s="15" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="F734" s="15" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="G734" s="16" t="s">
         <v>58</v>
@@ -21195,22 +21233,22 @@
     </row>
     <row r="740" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A740" s="44" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="B740" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C740" s="25" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="D740" s="26" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="E740" s="26" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="F740" s="26" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="G740" s="16" t="s">
         <v>58</v>
@@ -21339,22 +21377,22 @@
     </row>
     <row r="746" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A746" s="44" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="B746" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C746" s="14" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="D746" s="15" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="E746" s="15" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="F746" s="15" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="G746" s="16" t="s">
         <v>58</v>
@@ -21483,22 +21521,22 @@
     </row>
     <row r="752" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A752" s="44" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="B752" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C752" s="25" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="D752" s="26" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="E752" s="26" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="F752" s="26" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="G752" s="16" t="s">
         <v>58</v>
@@ -21627,22 +21665,22 @@
     </row>
     <row r="758" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A758" s="44" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="B758" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C758" s="14" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="D758" s="15" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="E758" s="15" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="F758" s="15" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="G758" s="16" t="s">
         <v>58</v>
@@ -21771,22 +21809,22 @@
     </row>
     <row r="764" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A764" s="45" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="B764" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C764" s="25" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="D764" s="26" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="E764" s="26" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="F764" s="26" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="G764" s="16" t="s">
         <v>58</v>
@@ -21915,22 +21953,22 @@
     </row>
     <row r="770" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A770" s="45" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="B770" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C770" s="14" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="D770" s="15" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="E770" s="15" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="F770" s="15" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="G770" s="16" t="s">
         <v>58</v>
@@ -22059,22 +22097,22 @@
     </row>
     <row r="776" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A776" s="45" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="B776" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C776" s="25" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="D776" s="26" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="E776" s="26" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="F776" s="26" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="G776" s="16" t="s">
         <v>58</v>
@@ -22203,22 +22241,22 @@
     </row>
     <row r="782" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A782" s="45" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="B782" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C782" s="14" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="D782" s="15" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="E782" s="15" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="F782" s="15" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="G782" s="16" t="s">
         <v>58</v>
@@ -22347,22 +22385,22 @@
     </row>
     <row r="788" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A788" s="45" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="B788" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C788" s="25" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="D788" s="26" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="E788" s="26" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="F788" s="26" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="G788" s="16" t="s">
         <v>58</v>
@@ -22491,22 +22529,22 @@
     </row>
     <row r="794" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A794" s="45" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="B794" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C794" s="14" t="s">
+        <v>553</v>
+      </c>
+      <c r="D794" s="15" t="s">
+        <v>554</v>
+      </c>
+      <c r="E794" s="15" t="s">
+        <v>555</v>
+      </c>
+      <c r="F794" s="15" t="s">
         <v>552</v>
-      </c>
-      <c r="D794" s="15" t="s">
-        <v>553</v>
-      </c>
-      <c r="E794" s="15" t="s">
-        <v>554</v>
-      </c>
-      <c r="F794" s="15" t="s">
-        <v>551</v>
       </c>
       <c r="G794" s="16" t="s">
         <v>58</v>
@@ -22635,22 +22673,22 @@
     </row>
     <row r="800" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A800" s="45" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="B800" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C800" s="25" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="D800" s="26" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="E800" s="26" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="F800" s="26" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="G800" s="16" t="s">
         <v>58</v>
@@ -22779,22 +22817,22 @@
     </row>
     <row r="806" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A806" s="45" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="B806" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C806" s="14" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="D806" s="15" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="E806" s="15" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="F806" s="15" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="G806" s="16" t="s">
         <v>58</v>
@@ -22923,22 +22961,22 @@
     </row>
     <row r="812" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A812" s="45" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="B812" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C812" s="25" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="D812" s="26" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="E812" s="26" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="F812" s="26" t="s">
-        <v>566</v>
+        <v>567</v>
       </c>
       <c r="G812" s="16" t="s">
         <v>58</v>
@@ -23067,22 +23105,22 @@
     </row>
     <row r="818" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A818" s="45" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="B818" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C818" s="14" t="s">
-        <v>567</v>
+        <v>568</v>
       </c>
       <c r="D818" s="15" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="E818" s="15" t="s">
-        <v>569</v>
+        <v>570</v>
       </c>
       <c r="F818" s="15" t="s">
-        <v>570</v>
+        <v>571</v>
       </c>
       <c r="G818" s="16" t="s">
         <v>58</v>
@@ -23211,22 +23249,22 @@
     </row>
     <row r="824" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A824" s="45" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="B824" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C824" s="25" t="s">
-        <v>571</v>
+        <v>572</v>
       </c>
       <c r="D824" s="26" t="s">
-        <v>572</v>
+        <v>573</v>
       </c>
       <c r="E824" s="26" t="s">
-        <v>573</v>
+        <v>574</v>
       </c>
       <c r="F824" s="26" t="s">
-        <v>574</v>
+        <v>575</v>
       </c>
       <c r="G824" s="16" t="s">
         <v>58</v>
@@ -23355,22 +23393,22 @@
     </row>
     <row r="830" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A830" s="45" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="B830" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C830" s="14" t="s">
-        <v>575</v>
+        <v>576</v>
       </c>
       <c r="D830" s="15" t="s">
-        <v>576</v>
+        <v>577</v>
       </c>
       <c r="E830" s="15" t="s">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="F830" s="15" t="s">
-        <v>578</v>
+        <v>579</v>
       </c>
       <c r="G830" s="16" t="s">
         <v>58</v>
@@ -23499,22 +23537,22 @@
     </row>
     <row r="836" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A836" s="46" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="B836" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C836" s="25" t="s">
-        <v>580</v>
+        <v>581</v>
       </c>
       <c r="D836" s="26" t="s">
-        <v>581</v>
+        <v>582</v>
       </c>
       <c r="E836" s="26" t="s">
-        <v>582</v>
+        <v>583</v>
       </c>
       <c r="F836" s="26" t="s">
-        <v>583</v>
+        <v>584</v>
       </c>
       <c r="G836" s="16" t="s">
         <v>58</v>
@@ -23643,22 +23681,22 @@
     </row>
     <row r="842" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A842" s="46" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="B842" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C842" s="14" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
       <c r="D842" s="15" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="E842" s="15" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="F842" s="15" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="G842" s="16" t="s">
         <v>58</v>
@@ -23787,22 +23825,22 @@
     </row>
     <row r="848" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A848" s="46" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="B848" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C848" s="25" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="D848" s="26" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="E848" s="26" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="F848" s="26" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="G848" s="16" t="s">
         <v>58</v>
@@ -23931,22 +23969,22 @@
     </row>
     <row r="854" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A854" s="46" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="B854" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C854" s="14" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="D854" s="15" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="E854" s="15" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="F854" s="15" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="G854" s="16" t="s">
         <v>58</v>
@@ -24075,22 +24113,22 @@
     </row>
     <row r="860" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A860" s="47" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="B860" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C860" s="25" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="D860" s="26" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="E860" s="26" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="F860" s="26" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="G860" s="16" t="s">
         <v>58</v>
@@ -24219,22 +24257,22 @@
     </row>
     <row r="866" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A866" s="47" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="B866" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C866" s="14" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="D866" s="15" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="E866" s="15" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="F866" s="15" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="G866" s="16" t="s">
         <v>58</v>
@@ -24363,22 +24401,22 @@
     </row>
     <row r="872" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A872" s="47" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="B872" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C872" s="25" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="D872" s="26" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="E872" s="26" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="F872" s="26" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="G872" s="16" t="s">
         <v>58</v>
@@ -24507,22 +24545,22 @@
     </row>
     <row r="878" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A878" s="47" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="B878" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C878" s="14" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="D878" s="15" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="E878" s="15" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="F878" s="15" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="G878" s="16" t="s">
         <v>58</v>
@@ -24651,22 +24689,22 @@
     </row>
     <row r="884" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A884" s="47" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="B884" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C884" s="25" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="D884" s="26" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="E884" s="26" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="F884" s="26" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="G884" s="16" t="s">
         <v>58</v>
@@ -24795,22 +24833,22 @@
     </row>
     <row r="890" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A890" s="47" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="B890" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C890" s="14" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="D890" s="15" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="E890" s="15" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="F890" s="15" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="G890" s="16" t="s">
         <v>58</v>
@@ -24939,22 +24977,22 @@
     </row>
     <row r="896" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A896" s="47" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="B896" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C896" s="25" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="D896" s="26" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="E896" s="26" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="F896" s="26" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="G896" s="16" t="s">
         <v>58</v>
@@ -25083,22 +25121,22 @@
     </row>
     <row r="902" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A902" s="48" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="B902" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C902" s="14" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="D902" s="15" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="E902" s="15" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="F902" s="15" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="G902" s="16" t="s">
         <v>58</v>
@@ -25227,22 +25265,22 @@
     </row>
     <row r="908" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A908" s="48" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="B908" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C908" s="25" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="D908" s="26" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="E908" s="26" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="F908" s="26" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="G908" s="16" t="s">
         <v>58</v>
@@ -25371,22 +25409,22 @@
     </row>
     <row r="914" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A914" s="48" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="B914" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C914" s="14" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="D914" s="15" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="E914" s="15" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="F914" s="15" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="G914" s="16" t="s">
         <v>58</v>
@@ -25515,22 +25553,22 @@
     </row>
     <row r="920" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A920" s="48" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="B920" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C920" s="25" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="D920" s="26" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="E920" s="26" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="F920" s="26" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="G920" s="16" t="s">
         <v>58</v>
@@ -25659,22 +25697,22 @@
     </row>
     <row r="926" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A926" s="48" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="B926" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C926" s="14" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="D926" s="15" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="E926" s="15" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="F926" s="15" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="G926" s="16" t="s">
         <v>58</v>
@@ -25803,22 +25841,22 @@
     </row>
     <row r="932" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A932" s="48" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="B932" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C932" s="25" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="D932" s="26" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="E932" s="26" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="F932" s="26" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="G932" s="16" t="s">
         <v>58</v>
@@ -25947,22 +25985,22 @@
     </row>
     <row r="938" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A938" s="49" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="B938" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C938" s="14" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="D938" s="15" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="E938" s="15" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="F938" s="15" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="G938" s="16" t="s">
         <v>58</v>
@@ -26091,22 +26129,22 @@
     </row>
     <row r="944" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A944" s="49" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="B944" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C944" s="25" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="D944" s="26" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="E944" s="26" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="F944" s="26" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="G944" s="16" t="s">
         <v>58</v>
@@ -26235,22 +26273,22 @@
     </row>
     <row r="950" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A950" s="49" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="B950" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C950" s="14" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="D950" s="15" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="E950" s="15" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="F950" s="15" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="G950" s="16" t="s">
         <v>58</v>
@@ -26379,22 +26417,22 @@
     </row>
     <row r="956" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A956" s="49" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="B956" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C956" s="25" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="D956" s="26" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="E956" s="26" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="F956" s="26" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="G956" s="16" t="s">
         <v>58</v>
@@ -26523,22 +26561,22 @@
     </row>
     <row r="962" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A962" s="49" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="B962" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C962" s="14" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="D962" s="15" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="E962" s="15" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="F962" s="15" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="G962" s="16" t="s">
         <v>58</v>
@@ -26667,22 +26705,22 @@
     </row>
     <row r="968" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A968" s="49" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="B968" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C968" s="25" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="D968" s="26" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="E968" s="26" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="F968" s="26" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="G968" s="16" t="s">
         <v>58</v>
@@ -26811,22 +26849,22 @@
     </row>
     <row r="974" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A974" s="50" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="B974" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C974" s="14" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="D974" s="15" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="E974" s="15" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="F974" s="15" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="G974" s="16" t="s">
         <v>58</v>
@@ -26955,22 +26993,22 @@
     </row>
     <row r="980" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A980" s="50" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="B980" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C980" s="25" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="D980" s="26" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="E980" s="26" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="F980" s="26" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="G980" s="16" t="s">
         <v>58</v>
@@ -27099,22 +27137,22 @@
     </row>
     <row r="986" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A986" s="50" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="B986" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C986" s="14" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="D986" s="15" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="E986" s="15" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="F986" s="15" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="G986" s="16" t="s">
         <v>58</v>
@@ -27243,22 +27281,22 @@
     </row>
     <row r="992" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A992" s="50" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="B992" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C992" s="25" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="D992" s="26" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="E992" s="26" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="F992" s="26" t="s">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="G992" s="16" t="s">
         <v>58</v>
@@ -27387,22 +27425,22 @@
     </row>
     <row r="998" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A998" s="50" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="B998" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C998" s="14" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="D998" s="15" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="E998" s="15" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="F998" s="15" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="G998" s="16" t="s">
         <v>58</v>
@@ -27531,22 +27569,22 @@
     </row>
     <row r="1004" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1004" s="51" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="B1004" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1004" s="25" t="s">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="D1004" s="26" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="E1004" s="26" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="F1004" s="26" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="G1004" s="16" t="s">
         <v>58</v>
@@ -27675,22 +27713,22 @@
     </row>
     <row r="1010" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1010" s="51" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="B1010" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1010" s="14" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="D1010" s="15" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="E1010" s="15" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="F1010" s="15" t="s">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="G1010" s="16" t="s">
         <v>58</v>
@@ -27819,22 +27857,22 @@
     </row>
     <row r="1016" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1016" s="51" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="B1016" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1016" s="25" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="D1016" s="26" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="E1016" s="26" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="F1016" s="26" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="G1016" s="16" t="s">
         <v>58</v>
@@ -27963,22 +28001,22 @@
     </row>
     <row r="1022" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1022" s="51" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="B1022" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1022" s="14" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="D1022" s="15" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="E1022" s="15" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="F1022" s="15" t="s">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="G1022" s="16" t="s">
         <v>58</v>
@@ -28107,22 +28145,22 @@
     </row>
     <row r="1028" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1028" s="51" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="B1028" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C1028" s="25" t="s">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="D1028" s="26" t="s">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="E1028" s="26" t="s">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="F1028" s="26" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="G1028" s="16" t="s">
         <v>58</v>
@@ -28251,22 +28289,22 @@
     </row>
     <row r="1034" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1034" s="51" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="B1034" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C1034" s="14" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="D1034" s="15" t="s">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="E1034" s="15" t="s">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="F1034" s="15" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="G1034" s="16" t="s">
         <v>58</v>
@@ -28395,22 +28433,22 @@
     </row>
     <row r="1040" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1040" s="52" t="s">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="B1040" s="28" t="s">
         <v>89</v>
       </c>
       <c r="C1040" s="25" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="D1040" s="26" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="E1040" s="26" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="F1040" s="26" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="G1040" s="16" t="s">
         <v>58</v>
@@ -28539,22 +28577,22 @@
     </row>
     <row r="1046" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1046" s="52" t="s">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="B1046" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1046" s="14" t="s">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="D1046" s="15" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="E1046" s="15" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="F1046" s="15" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="G1046" s="16" t="s">
         <v>58</v>
@@ -28691,16 +28729,16 @@
         <v>53</v>
       </c>
       <c r="C1052" s="25" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="D1052" s="26" t="s">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="E1052" s="26" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="F1052" s="26" t="s">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="G1052" s="16" t="s">
         <v>58</v>
@@ -28837,16 +28875,16 @@
         <v>53</v>
       </c>
       <c r="C1058" s="14" t="s">
-        <v>730</v>
+        <v>731</v>
       </c>
       <c r="D1058" s="15" t="s">
-        <v>731</v>
+        <v>732</v>
       </c>
       <c r="E1058" s="15" t="s">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="F1058" s="15" t="s">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="G1058" s="16" t="s">
         <v>58</v>
@@ -29896,17 +29934,17 @@
     <mergeCell ref="F1058:F1063"/>
   </mergeCells>
   <dataValidations count="4">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Valor invàlid" error="Escull OK, KO, PENDENT o N/A" sqref="J10:J1063">
-      <formula1>"OK,KO,PENDENT,N/A"</formula1>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Valor invàlid" error="Escull OK, KO, PENDENT, N/A o EN CURS" sqref="J10:J1063">
+      <formula1>EstatsProva</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Valor invàlid" error="Escull OK, KO, PENDENT o N/A" sqref="J2:J1063">
-      <formula1>"OK,KO,PENDENT,N/A"</formula1>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Valor invàlid" error="Escull OK, KO, PENDENT, N/A o EN CURS" sqref="J2:J1063">
+      <formula1>EstatsProva</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Valor invàlid" error="Escull OK, KO, PENDENT o N/A" sqref="M10:M1063">
-      <formula1>"OK,KO,PENDENT,N/A"</formula1>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Valor invàlid" error="Escull OK, KO, PENDENT, N/A o EN CURS" sqref="M10:M1063">
+      <formula1>EstatsProva</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Valor invàlid" error="Escull OK, KO, PENDENT o N/A" sqref="M2:M1063">
-      <formula1>"OK,KO,PENDENT,N/A"</formula1>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="stop" errorTitle="Valor invàlid" error="Escull OK, KO, PENDENT, N/A o EN CURS" sqref="M2:M1063">
+      <formula1>EstatsProva</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -29932,10 +29970,10 @@
         <v>39</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>53</v>
@@ -29953,7 +29991,7 @@
         <v>86</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -30161,7 +30199,7 @@
     </row>
     <row r="9" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="60" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="B9" s="1">
         <v>11</v>
@@ -30190,7 +30228,7 @@
     </row>
     <row r="10" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="61" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="B10" s="1">
         <v>9</v>
@@ -30219,7 +30257,7 @@
     </row>
     <row r="11" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="62" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="B11" s="1">
         <v>5</v>
@@ -30248,7 +30286,7 @@
     </row>
     <row r="12" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="63" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="B12" s="1">
         <v>5</v>
@@ -30277,7 +30315,7 @@
     </row>
     <row r="13" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="64" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="B13" s="1">
         <v>4</v>
@@ -30306,7 +30344,7 @@
     </row>
     <row r="14" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="65" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="B14" s="1">
         <v>5</v>
@@ -30335,7 +30373,7 @@
     </row>
     <row r="15" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="66" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="B15" s="1">
         <v>12</v>
@@ -30364,7 +30402,7 @@
     </row>
     <row r="16" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="67" t="s">
-        <v>579</v>
+        <v>580</v>
       </c>
       <c r="B16" s="1">
         <v>4</v>
@@ -30393,7 +30431,7 @@
     </row>
     <row r="17" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="68" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="B17" s="1">
         <v>7</v>
@@ -30422,7 +30460,7 @@
     </row>
     <row r="18" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="69" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="B18" s="1">
         <v>6</v>
@@ -30451,7 +30489,7 @@
     </row>
     <row r="19" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="70" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="B19" s="1">
         <v>6</v>
@@ -30480,7 +30518,7 @@
     </row>
     <row r="20" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="71" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="B20" s="1">
         <v>5</v>
@@ -30509,7 +30547,7 @@
     </row>
     <row r="21" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="72" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="B21" s="1">
         <v>6</v>
@@ -30538,7 +30576,7 @@
     </row>
     <row r="22" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="73" t="s">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="B22" s="1">
         <v>2</v>
@@ -30567,7 +30605,7 @@
     </row>
     <row r="23" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="74" t="s">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="B23" s="74">
         <v>153</v>
@@ -30618,7 +30656,7 @@
         <v>44</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="C1" s="10" t="s">
         <v>71</v>
@@ -30627,7 +30665,7 @@
         <v>86</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="F1" s="10" t="s">
         <v>94</v>
@@ -30778,10 +30816,10 @@
         <v>45</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>71</v>
@@ -30790,7 +30828,7 @@
         <v>86</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="G1" s="10" t="s">
         <v>94</v>
@@ -30801,7 +30839,7 @@
         <v>59</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="C2" s="1">
         <f>COUNTIF(Proves!$H:$H,A2)</f>
@@ -30915,4 +30953,55 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" orientation="portrait" horizontalDpi="300" verticalDpi="300" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <tabColor rgb="FF64748B"/>
+  </sheetPr>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="52" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" s="84" t="s">
+        <v>741</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="85" t="s">
+        <v>71</v>
+      </c>
+      <c r="B2" s="86" t="s">
+        <v>742</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" s="27" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" s="87" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" s="29" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>360</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
093 => fase IV => Ordre (Nom A-Z) a la fila de filtres de favorits, ZUP-070–072 ZUP-079–081 ZUP-088 ZUP-091 OK i ZUP-071 KO/corr (Chrome/USER)
</commit_message>
<xml_diff>
--- a/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
+++ b/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4373" uniqueCount="748">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4385" uniqueCount="750">
   <si>
     <t>Zuppeto — Joc de probes manual (totes les pantalles)</t>
   </si>
@@ -1249,9 +1249,6 @@
 De moment sense correcció.</t>
   </si>
   <si>
-    <t>EN CURS</t>
-  </si>
-  <si>
     <t>Què s'ha fet: A Favorits, Cercar i Netejar funcionen igual que a Llocs (els combos no filtren sols). El filtre s'aplica només als favorits de BD, sense Text Search. Si el place_id / caché Google ha caducat (~30 dies) o falta portada, es refresca amb GET /api/places/{id} (Place Details). Fitxers: favorites-page.component.html/.ts/.scss, place-filters (enableRemoteCitySearch), place-list-filter.ts, place-google-cache.ts, place-google-details-refresh.service.ts, place.service.ts, docs/ca/funcional-ca.md, docs/ca/tecnic-ca.md.</t>
   </si>
   <si>
@@ -1274,6 +1271,13 @@
   </si>
   <si>
     <t>Ordre de la graella canvia correctament</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No es veia Nom A-Z al llistat de filtres: Ordre anava sota la fila (Cerca/Ciutat/Tipus/Mascota), no al costat.
+El llistat de targetes queda sota el mapa; cal Cercar i mirar les targetes, no el mapa.</t>
+  </si>
+  <si>
+    <t>Què s'ha fet: Ordre (Més recents / Millor valorats / Nom A-Z) passa a la mateixa fila de filtres que Llocs. L'A-Z ordena per nom amb locale català. Fitxers: place-filters.component.html/.ts, favorites-page.component.html/.ts/.scss, favorite-places-sort.ts.</t>
   </si>
   <si>
     <t>ZUP-072</t>
@@ -1581,6 +1585,9 @@
   </si>
   <si>
     <t>Cards amb respostes validades</t>
+  </si>
+  <si>
+    <t>EN CURS</t>
   </si>
   <si>
     <t>ZUP-093</t>
@@ -15594,10 +15601,10 @@
         <v>360</v>
       </c>
       <c r="M500" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="N500" s="19" t="s">
         <v>395</v>
-      </c>
-      <c r="N500" s="19" t="s">
-        <v>396</v>
       </c>
     </row>
     <row r="501" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -15718,16 +15725,16 @@
         <v>89</v>
       </c>
       <c r="C506" s="25" t="s">
+        <v>396</v>
+      </c>
+      <c r="D506" s="26" t="s">
         <v>397</v>
-      </c>
-      <c r="D506" s="26" t="s">
-        <v>398</v>
       </c>
       <c r="E506" s="26" t="s">
         <v>254</v>
       </c>
       <c r="F506" s="26" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="G506" s="16" t="s">
         <v>58</v>
@@ -15735,9 +15742,11 @@
       <c r="H506" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="I506" s="18"/>
+      <c r="I506" s="18" t="s">
+        <v>360</v>
+      </c>
       <c r="J506" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K506" s="19"/>
       <c r="L506" s="18"/>
@@ -15854,7 +15863,7 @@
       <c r="M511" s="1"/>
       <c r="N511" s="19"/>
     </row>
-    <row r="512" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="512" ht="80" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A512" s="38" t="s">
         <v>369</v>
       </c>
@@ -15862,16 +15871,16 @@
         <v>89</v>
       </c>
       <c r="C512" s="14" t="s">
+        <v>399</v>
+      </c>
+      <c r="D512" s="15" t="s">
         <v>400</v>
       </c>
-      <c r="D512" s="15" t="s">
+      <c r="E512" s="15" t="s">
         <v>401</v>
       </c>
-      <c r="E512" s="15" t="s">
+      <c r="F512" s="15" t="s">
         <v>402</v>
-      </c>
-      <c r="F512" s="15" t="s">
-        <v>403</v>
       </c>
       <c r="G512" s="16" t="s">
         <v>58</v>
@@ -15879,14 +15888,24 @@
       <c r="H512" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="I512" s="18"/>
+      <c r="I512" s="18" t="s">
+        <v>360</v>
+      </c>
       <c r="J512" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="K512" s="19"/>
-      <c r="L512" s="18"/>
-      <c r="M512" s="1"/>
-      <c r="N512" s="19"/>
+        <v>86</v>
+      </c>
+      <c r="K512" s="19" t="s">
+        <v>403</v>
+      </c>
+      <c r="L512" s="18" t="s">
+        <v>360</v>
+      </c>
+      <c r="M512" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="N512" s="19" t="s">
+        <v>404</v>
+      </c>
     </row>
     <row r="513" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A513" s="38"/>
@@ -16006,16 +16025,16 @@
         <v>89</v>
       </c>
       <c r="C518" s="25" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D518" s="26" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="E518" s="26" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="F518" s="26" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="G518" s="16" t="s">
         <v>58</v>
@@ -16023,9 +16042,11 @@
       <c r="H518" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="I518" s="18"/>
+      <c r="I518" s="18" t="s">
+        <v>360</v>
+      </c>
       <c r="J518" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K518" s="19"/>
       <c r="L518" s="18"/>
@@ -16150,16 +16171,16 @@
         <v>53</v>
       </c>
       <c r="C524" s="14" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="D524" s="15" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="E524" s="15" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="F524" s="15" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="G524" s="16" t="s">
         <v>58</v>
@@ -16296,16 +16317,16 @@
         <v>53</v>
       </c>
       <c r="C530" s="25" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="D530" s="26" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="E530" s="26" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="F530" s="26" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="G530" s="16" t="s">
         <v>58</v>
@@ -16442,16 +16463,16 @@
         <v>53</v>
       </c>
       <c r="C536" s="14" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="D536" s="15" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="E536" s="15" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="F536" s="15" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="G536" s="16" t="s">
         <v>58</v>
@@ -16582,22 +16603,22 @@
     </row>
     <row r="542" ht="180" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A542" s="39" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B542" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C542" s="25" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="D542" s="26" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="E542" s="26" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="F542" s="26" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="G542" s="16" t="s">
         <v>58</v>
@@ -16612,7 +16633,7 @@
         <v>86</v>
       </c>
       <c r="K542" s="19" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="L542" s="18">
         <v>46264.91666666667</v>
@@ -16621,7 +16642,7 @@
         <v>71</v>
       </c>
       <c r="N542" s="19" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
     </row>
     <row r="543" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -16736,22 +16757,22 @@
     </row>
     <row r="548" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A548" s="39" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B548" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C548" s="14" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="D548" s="15" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="E548" s="15" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="F548" s="15" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="G548" s="16" t="s">
         <v>58</v>
@@ -16880,22 +16901,22 @@
     </row>
     <row r="554" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A554" s="39" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B554" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C554" s="25" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="D554" s="26" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="E554" s="26" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="F554" s="26" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="G554" s="16" t="s">
         <v>58</v>
@@ -17026,22 +17047,22 @@
     </row>
     <row r="560" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A560" s="39" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B560" s="27" t="s">
         <v>89</v>
       </c>
       <c r="C560" s="14" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="D560" s="15" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="E560" s="15" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="F560" s="15" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="G560" s="16" t="s">
         <v>58</v>
@@ -17049,9 +17070,11 @@
       <c r="H560" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="I560" s="18"/>
+      <c r="I560" s="18" t="s">
+        <v>360</v>
+      </c>
       <c r="J560" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K560" s="19"/>
       <c r="L560" s="18"/>
@@ -17170,22 +17193,22 @@
     </row>
     <row r="566" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A566" s="39" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B566" s="27" t="s">
         <v>89</v>
       </c>
       <c r="C566" s="25" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="D566" s="26" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="E566" s="26" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="F566" s="26" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="G566" s="16" t="s">
         <v>58</v>
@@ -17193,9 +17216,11 @@
       <c r="H566" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="I566" s="18"/>
+      <c r="I566" s="18" t="s">
+        <v>360</v>
+      </c>
       <c r="J566" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K566" s="19"/>
       <c r="L566" s="18"/>
@@ -17314,22 +17339,22 @@
     </row>
     <row r="572" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A572" s="39" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B572" s="27" t="s">
         <v>89</v>
       </c>
       <c r="C572" s="14" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="D572" s="15" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="E572" s="15" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="F572" s="15" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="G572" s="16" t="s">
         <v>58</v>
@@ -17337,9 +17362,11 @@
       <c r="H572" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="I572" s="18"/>
+      <c r="I572" s="18" t="s">
+        <v>360</v>
+      </c>
       <c r="J572" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K572" s="19"/>
       <c r="L572" s="18"/>
@@ -17458,22 +17485,22 @@
     </row>
     <row r="578" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A578" s="39" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B578" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C578" s="25" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="D578" s="26" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="E578" s="26" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="F578" s="26" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="G578" s="16" t="s">
         <v>58</v>
@@ -17604,22 +17631,22 @@
     </row>
     <row r="584" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A584" s="39" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B584" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C584" s="14" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="D584" s="15" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="E584" s="15" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="F584" s="15" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="G584" s="16" t="s">
         <v>58</v>
@@ -17748,22 +17775,22 @@
     </row>
     <row r="590" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A590" s="39" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B590" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C590" s="25" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="D590" s="26" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="E590" s="26" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="F590" s="26" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="G590" s="16" t="s">
         <v>58</v>
@@ -17894,22 +17921,22 @@
     </row>
     <row r="596" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A596" s="40" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="B596" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C596" s="14" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="D596" s="15" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="E596" s="15" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="F596" s="15" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="G596" s="16" t="s">
         <v>58</v>
@@ -18056,7 +18083,7 @@
         <v>86</v>
       </c>
       <c r="K602" s="19" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="L602" s="18">
         <v>46264.91666666667</v>
@@ -18065,7 +18092,7 @@
         <v>71</v>
       </c>
       <c r="N602" s="19" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
     </row>
     <row r="603" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -18444,22 +18471,22 @@
     </row>
     <row r="620" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A620" s="40" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="B620" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C620" s="25" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="D620" s="26" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="E620" s="26" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="F620" s="26" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="G620" s="16" t="s">
         <v>58</v>
@@ -18590,22 +18617,22 @@
     </row>
     <row r="626" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A626" s="40" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="B626" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C626" s="14" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="D626" s="15" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="E626" s="15" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="F626" s="15" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="G626" s="16" t="s">
         <v>58</v>
@@ -18736,22 +18763,22 @@
     </row>
     <row r="632" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A632" s="40" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="B632" s="27" t="s">
         <v>89</v>
       </c>
       <c r="C632" s="25" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="D632" s="26" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="E632" s="26" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="F632" s="26" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="G632" s="16" t="s">
         <v>58</v>
@@ -18759,9 +18786,11 @@
       <c r="H632" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="I632" s="18"/>
+      <c r="I632" s="18" t="s">
+        <v>360</v>
+      </c>
       <c r="J632" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K632" s="19"/>
       <c r="L632" s="18"/>
@@ -18880,22 +18909,22 @@
     </row>
     <row r="638" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A638" s="40" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="B638" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C638" s="14" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="D638" s="15" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="E638" s="15" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="F638" s="15" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="G638" s="16" t="s">
         <v>58</v>
@@ -19026,22 +19055,22 @@
     </row>
     <row r="644" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A644" s="41" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="B644" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C644" s="25" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="D644" s="26" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="E644" s="26" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="F644" s="26" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="G644" s="16" t="s">
         <v>58</v>
@@ -19568,22 +19597,22 @@
     </row>
     <row r="668" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A668" s="41" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="B668" s="27" t="s">
         <v>89</v>
       </c>
       <c r="C668" s="14" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="D668" s="15" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="E668" s="15" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="F668" s="15" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="G668" s="16" t="s">
         <v>58</v>
@@ -19591,9 +19620,11 @@
       <c r="H668" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="I668" s="18"/>
+      <c r="I668" s="18" t="s">
+        <v>360</v>
+      </c>
       <c r="J668" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K668" s="19"/>
       <c r="L668" s="18"/>
@@ -19712,22 +19743,22 @@
     </row>
     <row r="674" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A674" s="41" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="B674" s="27" t="s">
         <v>89</v>
       </c>
       <c r="C674" s="25" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="D674" s="26" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="E674" s="26" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="F674" s="26" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="G674" s="16" t="s">
         <v>58</v>
@@ -19737,7 +19768,7 @@
       </c>
       <c r="I674" s="18"/>
       <c r="J674" s="1" t="s">
-        <v>60</v>
+        <v>496</v>
       </c>
       <c r="K674" s="19"/>
       <c r="L674" s="18"/>
@@ -19856,22 +19887,22 @@
     </row>
     <row r="680" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A680" s="41" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="B680" s="27" t="s">
         <v>89</v>
       </c>
       <c r="C680" s="14" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="D680" s="15" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="E680" s="15" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="F680" s="15" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="G680" s="16" t="s">
         <v>58</v>
@@ -20000,22 +20031,22 @@
     </row>
     <row r="686" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A686" s="41" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="B686" s="27" t="s">
         <v>89</v>
       </c>
       <c r="C686" s="25" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="D686" s="26" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="E686" s="26" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="F686" s="26" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="G686" s="16" t="s">
         <v>58</v>
@@ -20144,22 +20175,22 @@
     </row>
     <row r="692" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A692" s="42" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="B692" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C692" s="14" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="D692" s="15" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="E692" s="15" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="F692" s="15" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="G692" s="16" t="s">
         <v>58</v>
@@ -20686,22 +20717,22 @@
     </row>
     <row r="716" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A716" s="42" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="B716" s="27" t="s">
         <v>89</v>
       </c>
       <c r="C716" s="25" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="D716" s="26" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="E716" s="26" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="F716" s="26" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="G716" s="16" t="s">
         <v>58</v>
@@ -20830,22 +20861,22 @@
     </row>
     <row r="722" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A722" s="42" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="B722" s="27" t="s">
         <v>89</v>
       </c>
       <c r="C722" s="14" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="D722" s="15" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="E722" s="15" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="F722" s="15" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="G722" s="16" t="s">
         <v>58</v>
@@ -20974,19 +21005,19 @@
     </row>
     <row r="728" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A728" s="42" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="B728" s="27" t="s">
         <v>89</v>
       </c>
       <c r="C728" s="25" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="D728" s="26" t="s">
         <v>216</v>
       </c>
       <c r="E728" s="26" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="F728" s="26" t="s">
         <v>218</v>
@@ -21118,22 +21149,22 @@
     </row>
     <row r="734" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A734" s="43" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="B734" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C734" s="14" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="D734" s="15" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="E734" s="15" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="F734" s="15" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="G734" s="16" t="s">
         <v>58</v>
@@ -21262,22 +21293,22 @@
     </row>
     <row r="740" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A740" s="43" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="B740" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C740" s="25" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="D740" s="26" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="E740" s="26" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="F740" s="26" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="G740" s="16" t="s">
         <v>58</v>
@@ -21406,22 +21437,22 @@
     </row>
     <row r="746" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A746" s="43" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="B746" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C746" s="14" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="D746" s="15" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="E746" s="15" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="F746" s="15" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="G746" s="16" t="s">
         <v>58</v>
@@ -21550,22 +21581,22 @@
     </row>
     <row r="752" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A752" s="43" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="B752" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C752" s="25" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="D752" s="26" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="E752" s="26" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="F752" s="26" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="G752" s="16" t="s">
         <v>58</v>
@@ -21694,22 +21725,22 @@
     </row>
     <row r="758" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A758" s="43" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="B758" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C758" s="14" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="D758" s="15" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="E758" s="15" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="F758" s="15" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="G758" s="16" t="s">
         <v>58</v>
@@ -21838,22 +21869,22 @@
     </row>
     <row r="764" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A764" s="44" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="B764" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C764" s="25" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="D764" s="26" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="E764" s="26" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="F764" s="26" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="G764" s="16" t="s">
         <v>58</v>
@@ -21982,22 +22013,22 @@
     </row>
     <row r="770" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A770" s="44" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="B770" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C770" s="14" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="D770" s="15" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="E770" s="15" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="F770" s="15" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="G770" s="16" t="s">
         <v>58</v>
@@ -22126,22 +22157,22 @@
     </row>
     <row r="776" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A776" s="44" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="B776" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C776" s="25" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="D776" s="26" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="E776" s="26" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="F776" s="26" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="G776" s="16" t="s">
         <v>58</v>
@@ -22270,22 +22301,22 @@
     </row>
     <row r="782" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A782" s="44" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="B782" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C782" s="14" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="D782" s="15" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="E782" s="15" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="F782" s="15" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="G782" s="16" t="s">
         <v>58</v>
@@ -22414,22 +22445,22 @@
     </row>
     <row r="788" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A788" s="44" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="B788" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C788" s="25" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="D788" s="26" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="E788" s="26" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="F788" s="26" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
       <c r="G788" s="16" t="s">
         <v>58</v>
@@ -22558,22 +22589,22 @@
     </row>
     <row r="794" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A794" s="44" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="B794" s="27" t="s">
         <v>89</v>
       </c>
       <c r="C794" s="14" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="D794" s="15" t="s">
+        <v>561</v>
+      </c>
+      <c r="E794" s="15" t="s">
+        <v>562</v>
+      </c>
+      <c r="F794" s="15" t="s">
         <v>559</v>
-      </c>
-      <c r="E794" s="15" t="s">
-        <v>560</v>
-      </c>
-      <c r="F794" s="15" t="s">
-        <v>557</v>
       </c>
       <c r="G794" s="16" t="s">
         <v>58</v>
@@ -22702,22 +22733,22 @@
     </row>
     <row r="800" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A800" s="44" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="B800" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C800" s="25" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
       <c r="D800" s="26" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
       <c r="E800" s="26" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
       <c r="F800" s="26" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="G800" s="16" t="s">
         <v>58</v>
@@ -22846,22 +22877,22 @@
     </row>
     <row r="806" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A806" s="44" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="B806" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C806" s="14" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="D806" s="15" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="E806" s="15" t="s">
-        <v>567</v>
+        <v>569</v>
       </c>
       <c r="F806" s="15" t="s">
-        <v>568</v>
+        <v>570</v>
       </c>
       <c r="G806" s="16" t="s">
         <v>58</v>
@@ -22990,22 +23021,22 @@
     </row>
     <row r="812" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A812" s="44" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="B812" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C812" s="25" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="D812" s="26" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
       <c r="E812" s="26" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
       <c r="F812" s="26" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
       <c r="G812" s="16" t="s">
         <v>58</v>
@@ -23134,22 +23165,22 @@
     </row>
     <row r="818" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A818" s="44" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="B818" s="27" t="s">
         <v>89</v>
       </c>
       <c r="C818" s="14" t="s">
-        <v>573</v>
+        <v>575</v>
       </c>
       <c r="D818" s="15" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="E818" s="15" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="F818" s="15" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="G818" s="16" t="s">
         <v>58</v>
@@ -23278,22 +23309,22 @@
     </row>
     <row r="824" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A824" s="44" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="B824" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C824" s="25" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="D824" s="26" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="E824" s="26" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="F824" s="26" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="G824" s="16" t="s">
         <v>58</v>
@@ -23422,22 +23453,22 @@
     </row>
     <row r="830" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A830" s="44" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="B830" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C830" s="14" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="D830" s="15" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="E830" s="15" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="F830" s="15" t="s">
-        <v>584</v>
+        <v>586</v>
       </c>
       <c r="G830" s="16" t="s">
         <v>58</v>
@@ -23566,22 +23597,22 @@
     </row>
     <row r="836" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A836" s="45" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
       <c r="B836" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C836" s="25" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
       <c r="D836" s="26" t="s">
-        <v>587</v>
+        <v>589</v>
       </c>
       <c r="E836" s="26" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="F836" s="26" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="G836" s="16" t="s">
         <v>58</v>
@@ -23710,22 +23741,22 @@
     </row>
     <row r="842" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A842" s="45" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
       <c r="B842" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C842" s="14" t="s">
-        <v>590</v>
+        <v>592</v>
       </c>
       <c r="D842" s="15" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="E842" s="15" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
       <c r="F842" s="15" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="G842" s="16" t="s">
         <v>58</v>
@@ -23854,22 +23885,22 @@
     </row>
     <row r="848" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A848" s="45" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
       <c r="B848" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C848" s="25" t="s">
-        <v>593</v>
+        <v>595</v>
       </c>
       <c r="D848" s="26" t="s">
-        <v>594</v>
+        <v>596</v>
       </c>
       <c r="E848" s="26" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
       <c r="F848" s="26" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
       <c r="G848" s="16" t="s">
         <v>58</v>
@@ -23998,22 +24029,22 @@
     </row>
     <row r="854" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A854" s="45" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
       <c r="B854" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C854" s="14" t="s">
-        <v>597</v>
+        <v>599</v>
       </c>
       <c r="D854" s="15" t="s">
-        <v>598</v>
+        <v>600</v>
       </c>
       <c r="E854" s="15" t="s">
-        <v>599</v>
+        <v>601</v>
       </c>
       <c r="F854" s="15" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
       <c r="G854" s="16" t="s">
         <v>58</v>
@@ -24142,22 +24173,22 @@
     </row>
     <row r="860" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A860" s="46" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="B860" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C860" s="25" t="s">
-        <v>602</v>
+        <v>604</v>
       </c>
       <c r="D860" s="26" t="s">
-        <v>603</v>
+        <v>605</v>
       </c>
       <c r="E860" s="26" t="s">
-        <v>604</v>
+        <v>606</v>
       </c>
       <c r="F860" s="26" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
       <c r="G860" s="16" t="s">
         <v>58</v>
@@ -24286,22 +24317,22 @@
     </row>
     <row r="866" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A866" s="46" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="B866" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C866" s="14" t="s">
-        <v>606</v>
+        <v>608</v>
       </c>
       <c r="D866" s="15" t="s">
-        <v>607</v>
+        <v>609</v>
       </c>
       <c r="E866" s="15" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
       <c r="F866" s="15" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="G866" s="16" t="s">
         <v>58</v>
@@ -24430,22 +24461,22 @@
     </row>
     <row r="872" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A872" s="46" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="B872" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C872" s="25" t="s">
-        <v>610</v>
+        <v>612</v>
       </c>
       <c r="D872" s="26" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
       <c r="E872" s="26" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="F872" s="26" t="s">
-        <v>613</v>
+        <v>615</v>
       </c>
       <c r="G872" s="16" t="s">
         <v>58</v>
@@ -24574,22 +24605,22 @@
     </row>
     <row r="878" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A878" s="46" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="B878" s="27" t="s">
         <v>89</v>
       </c>
       <c r="C878" s="14" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
       <c r="D878" s="15" t="s">
-        <v>615</v>
+        <v>617</v>
       </c>
       <c r="E878" s="15" t="s">
-        <v>616</v>
+        <v>618</v>
       </c>
       <c r="F878" s="15" t="s">
-        <v>617</v>
+        <v>619</v>
       </c>
       <c r="G878" s="16" t="s">
         <v>58</v>
@@ -24718,22 +24749,22 @@
     </row>
     <row r="884" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A884" s="46" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="B884" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C884" s="25" t="s">
-        <v>618</v>
+        <v>620</v>
       </c>
       <c r="D884" s="26" t="s">
-        <v>619</v>
+        <v>621</v>
       </c>
       <c r="E884" s="26" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="F884" s="26" t="s">
-        <v>621</v>
+        <v>623</v>
       </c>
       <c r="G884" s="16" t="s">
         <v>58</v>
@@ -24862,22 +24893,22 @@
     </row>
     <row r="890" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A890" s="46" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="B890" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C890" s="14" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
       <c r="D890" s="15" t="s">
-        <v>623</v>
+        <v>625</v>
       </c>
       <c r="E890" s="15" t="s">
-        <v>624</v>
+        <v>626</v>
       </c>
       <c r="F890" s="15" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
       <c r="G890" s="16" t="s">
         <v>58</v>
@@ -25006,22 +25037,22 @@
     </row>
     <row r="896" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A896" s="46" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="B896" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C896" s="25" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
       <c r="D896" s="26" t="s">
-        <v>627</v>
+        <v>629</v>
       </c>
       <c r="E896" s="26" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
       <c r="F896" s="26" t="s">
-        <v>629</v>
+        <v>631</v>
       </c>
       <c r="G896" s="16" t="s">
         <v>58</v>
@@ -25150,22 +25181,22 @@
     </row>
     <row r="902" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A902" s="47" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
       <c r="B902" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C902" s="14" t="s">
-        <v>631</v>
+        <v>633</v>
       </c>
       <c r="D902" s="15" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
       <c r="E902" s="15" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="F902" s="15" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
       <c r="G902" s="16" t="s">
         <v>58</v>
@@ -25294,22 +25325,22 @@
     </row>
     <row r="908" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A908" s="47" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
       <c r="B908" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C908" s="25" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="D908" s="26" t="s">
-        <v>636</v>
+        <v>638</v>
       </c>
       <c r="E908" s="26" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="F908" s="26" t="s">
-        <v>638</v>
+        <v>640</v>
       </c>
       <c r="G908" s="16" t="s">
         <v>58</v>
@@ -25438,22 +25469,22 @@
     </row>
     <row r="914" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A914" s="47" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
       <c r="B914" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C914" s="14" t="s">
-        <v>639</v>
+        <v>641</v>
       </c>
       <c r="D914" s="15" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
       <c r="E914" s="15" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
       <c r="F914" s="15" t="s">
-        <v>642</v>
+        <v>644</v>
       </c>
       <c r="G914" s="16" t="s">
         <v>58</v>
@@ -25582,22 +25613,22 @@
     </row>
     <row r="920" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A920" s="47" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
       <c r="B920" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C920" s="25" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
       <c r="D920" s="26" t="s">
-        <v>644</v>
+        <v>646</v>
       </c>
       <c r="E920" s="26" t="s">
-        <v>645</v>
+        <v>647</v>
       </c>
       <c r="F920" s="26" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
       <c r="G920" s="16" t="s">
         <v>58</v>
@@ -25726,22 +25757,22 @@
     </row>
     <row r="926" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A926" s="47" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
       <c r="B926" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C926" s="14" t="s">
-        <v>647</v>
+        <v>649</v>
       </c>
       <c r="D926" s="15" t="s">
-        <v>648</v>
+        <v>650</v>
       </c>
       <c r="E926" s="15" t="s">
-        <v>649</v>
+        <v>651</v>
       </c>
       <c r="F926" s="15" t="s">
-        <v>650</v>
+        <v>652</v>
       </c>
       <c r="G926" s="16" t="s">
         <v>58</v>
@@ -25870,22 +25901,22 @@
     </row>
     <row r="932" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A932" s="47" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
       <c r="B932" s="27" t="s">
         <v>89</v>
       </c>
       <c r="C932" s="25" t="s">
-        <v>651</v>
+        <v>653</v>
       </c>
       <c r="D932" s="26" t="s">
-        <v>652</v>
+        <v>654</v>
       </c>
       <c r="E932" s="26" t="s">
-        <v>653</v>
+        <v>655</v>
       </c>
       <c r="F932" s="26" t="s">
-        <v>654</v>
+        <v>656</v>
       </c>
       <c r="G932" s="16" t="s">
         <v>58</v>
@@ -26014,22 +26045,22 @@
     </row>
     <row r="938" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A938" s="48" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
       <c r="B938" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C938" s="14" t="s">
-        <v>656</v>
+        <v>658</v>
       </c>
       <c r="D938" s="15" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
       <c r="E938" s="15" t="s">
-        <v>658</v>
+        <v>660</v>
       </c>
       <c r="F938" s="15" t="s">
-        <v>659</v>
+        <v>661</v>
       </c>
       <c r="G938" s="16" t="s">
         <v>58</v>
@@ -26158,22 +26189,22 @@
     </row>
     <row r="944" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A944" s="48" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
       <c r="B944" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C944" s="25" t="s">
-        <v>660</v>
+        <v>662</v>
       </c>
       <c r="D944" s="26" t="s">
-        <v>661</v>
+        <v>663</v>
       </c>
       <c r="E944" s="26" t="s">
-        <v>662</v>
+        <v>664</v>
       </c>
       <c r="F944" s="26" t="s">
-        <v>663</v>
+        <v>665</v>
       </c>
       <c r="G944" s="16" t="s">
         <v>58</v>
@@ -26302,22 +26333,22 @@
     </row>
     <row r="950" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A950" s="48" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
       <c r="B950" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C950" s="14" t="s">
-        <v>664</v>
+        <v>666</v>
       </c>
       <c r="D950" s="15" t="s">
-        <v>665</v>
+        <v>667</v>
       </c>
       <c r="E950" s="15" t="s">
-        <v>666</v>
+        <v>668</v>
       </c>
       <c r="F950" s="15" t="s">
-        <v>667</v>
+        <v>669</v>
       </c>
       <c r="G950" s="16" t="s">
         <v>58</v>
@@ -26446,22 +26477,22 @@
     </row>
     <row r="956" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A956" s="48" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
       <c r="B956" s="27" t="s">
         <v>89</v>
       </c>
       <c r="C956" s="25" t="s">
-        <v>668</v>
+        <v>670</v>
       </c>
       <c r="D956" s="26" t="s">
-        <v>669</v>
+        <v>671</v>
       </c>
       <c r="E956" s="26" t="s">
-        <v>670</v>
+        <v>672</v>
       </c>
       <c r="F956" s="26" t="s">
-        <v>642</v>
+        <v>644</v>
       </c>
       <c r="G956" s="16" t="s">
         <v>58</v>
@@ -26590,22 +26621,22 @@
     </row>
     <row r="962" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A962" s="48" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
       <c r="B962" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C962" s="14" t="s">
-        <v>671</v>
+        <v>673</v>
       </c>
       <c r="D962" s="15" t="s">
-        <v>672</v>
+        <v>674</v>
       </c>
       <c r="E962" s="15" t="s">
-        <v>673</v>
+        <v>675</v>
       </c>
       <c r="F962" s="15" t="s">
-        <v>674</v>
+        <v>676</v>
       </c>
       <c r="G962" s="16" t="s">
         <v>58</v>
@@ -26734,22 +26765,22 @@
     </row>
     <row r="968" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A968" s="48" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
       <c r="B968" s="27" t="s">
         <v>89</v>
       </c>
       <c r="C968" s="25" t="s">
-        <v>675</v>
+        <v>677</v>
       </c>
       <c r="D968" s="26" t="s">
-        <v>676</v>
+        <v>678</v>
       </c>
       <c r="E968" s="26" t="s">
-        <v>677</v>
+        <v>679</v>
       </c>
       <c r="F968" s="26" t="s">
-        <v>678</v>
+        <v>680</v>
       </c>
       <c r="G968" s="16" t="s">
         <v>58</v>
@@ -26878,22 +26909,22 @@
     </row>
     <row r="974" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A974" s="49" t="s">
-        <v>679</v>
+        <v>681</v>
       </c>
       <c r="B974" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C974" s="14" t="s">
-        <v>680</v>
+        <v>682</v>
       </c>
       <c r="D974" s="15" t="s">
-        <v>681</v>
+        <v>683</v>
       </c>
       <c r="E974" s="15" t="s">
-        <v>682</v>
+        <v>684</v>
       </c>
       <c r="F974" s="15" t="s">
-        <v>683</v>
+        <v>685</v>
       </c>
       <c r="G974" s="16" t="s">
         <v>58</v>
@@ -27022,22 +27053,22 @@
     </row>
     <row r="980" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A980" s="49" t="s">
-        <v>679</v>
+        <v>681</v>
       </c>
       <c r="B980" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C980" s="25" t="s">
-        <v>684</v>
+        <v>686</v>
       </c>
       <c r="D980" s="26" t="s">
-        <v>685</v>
+        <v>687</v>
       </c>
       <c r="E980" s="26" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
       <c r="F980" s="26" t="s">
-        <v>687</v>
+        <v>689</v>
       </c>
       <c r="G980" s="16" t="s">
         <v>58</v>
@@ -27166,22 +27197,22 @@
     </row>
     <row r="986" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A986" s="49" t="s">
-        <v>679</v>
+        <v>681</v>
       </c>
       <c r="B986" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C986" s="14" t="s">
-        <v>688</v>
+        <v>690</v>
       </c>
       <c r="D986" s="15" t="s">
-        <v>689</v>
+        <v>691</v>
       </c>
       <c r="E986" s="15" t="s">
-        <v>690</v>
+        <v>692</v>
       </c>
       <c r="F986" s="15" t="s">
-        <v>691</v>
+        <v>693</v>
       </c>
       <c r="G986" s="16" t="s">
         <v>58</v>
@@ -27310,22 +27341,22 @@
     </row>
     <row r="992" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A992" s="49" t="s">
-        <v>679</v>
+        <v>681</v>
       </c>
       <c r="B992" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C992" s="25" t="s">
-        <v>692</v>
+        <v>694</v>
       </c>
       <c r="D992" s="26" t="s">
-        <v>693</v>
+        <v>695</v>
       </c>
       <c r="E992" s="26" t="s">
-        <v>694</v>
+        <v>696</v>
       </c>
       <c r="F992" s="26" t="s">
-        <v>695</v>
+        <v>697</v>
       </c>
       <c r="G992" s="16" t="s">
         <v>58</v>
@@ -27454,22 +27485,22 @@
     </row>
     <row r="998" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A998" s="49" t="s">
-        <v>679</v>
+        <v>681</v>
       </c>
       <c r="B998" s="27" t="s">
         <v>89</v>
       </c>
       <c r="C998" s="14" t="s">
-        <v>696</v>
+        <v>698</v>
       </c>
       <c r="D998" s="15" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
       <c r="E998" s="15" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
       <c r="F998" s="15" t="s">
-        <v>699</v>
+        <v>701</v>
       </c>
       <c r="G998" s="16" t="s">
         <v>58</v>
@@ -27598,22 +27629,22 @@
     </row>
     <row r="1004" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1004" s="50" t="s">
-        <v>700</v>
+        <v>702</v>
       </c>
       <c r="B1004" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1004" s="25" t="s">
-        <v>701</v>
+        <v>703</v>
       </c>
       <c r="D1004" s="26" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="E1004" s="26" t="s">
-        <v>703</v>
+        <v>705</v>
       </c>
       <c r="F1004" s="26" t="s">
-        <v>704</v>
+        <v>706</v>
       </c>
       <c r="G1004" s="16" t="s">
         <v>58</v>
@@ -27742,22 +27773,22 @@
     </row>
     <row r="1010" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1010" s="50" t="s">
-        <v>700</v>
+        <v>702</v>
       </c>
       <c r="B1010" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1010" s="14" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
       <c r="D1010" s="15" t="s">
-        <v>706</v>
+        <v>708</v>
       </c>
       <c r="E1010" s="15" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
       <c r="F1010" s="15" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="G1010" s="16" t="s">
         <v>58</v>
@@ -27886,22 +27917,22 @@
     </row>
     <row r="1016" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1016" s="50" t="s">
-        <v>700</v>
+        <v>702</v>
       </c>
       <c r="B1016" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1016" s="25" t="s">
-        <v>709</v>
+        <v>711</v>
       </c>
       <c r="D1016" s="26" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="E1016" s="26" t="s">
-        <v>711</v>
+        <v>713</v>
       </c>
       <c r="F1016" s="26" t="s">
-        <v>712</v>
+        <v>714</v>
       </c>
       <c r="G1016" s="16" t="s">
         <v>58</v>
@@ -28030,22 +28061,22 @@
     </row>
     <row r="1022" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1022" s="50" t="s">
-        <v>700</v>
+        <v>702</v>
       </c>
       <c r="B1022" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1022" s="14" t="s">
-        <v>713</v>
+        <v>715</v>
       </c>
       <c r="D1022" s="15" t="s">
-        <v>714</v>
+        <v>716</v>
       </c>
       <c r="E1022" s="15" t="s">
-        <v>715</v>
+        <v>717</v>
       </c>
       <c r="F1022" s="15" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
       <c r="G1022" s="16" t="s">
         <v>58</v>
@@ -28174,22 +28205,22 @@
     </row>
     <row r="1028" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1028" s="50" t="s">
-        <v>700</v>
+        <v>702</v>
       </c>
       <c r="B1028" s="27" t="s">
         <v>89</v>
       </c>
       <c r="C1028" s="25" t="s">
-        <v>717</v>
+        <v>719</v>
       </c>
       <c r="D1028" s="26" t="s">
-        <v>718</v>
+        <v>720</v>
       </c>
       <c r="E1028" s="26" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
       <c r="F1028" s="26" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
       <c r="G1028" s="16" t="s">
         <v>58</v>
@@ -28318,22 +28349,22 @@
     </row>
     <row r="1034" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1034" s="50" t="s">
-        <v>700</v>
+        <v>702</v>
       </c>
       <c r="B1034" s="27" t="s">
         <v>89</v>
       </c>
       <c r="C1034" s="14" t="s">
-        <v>721</v>
+        <v>723</v>
       </c>
       <c r="D1034" s="15" t="s">
-        <v>722</v>
+        <v>724</v>
       </c>
       <c r="E1034" s="15" t="s">
-        <v>723</v>
+        <v>725</v>
       </c>
       <c r="F1034" s="15" t="s">
-        <v>724</v>
+        <v>726</v>
       </c>
       <c r="G1034" s="16" t="s">
         <v>58</v>
@@ -28462,22 +28493,22 @@
     </row>
     <row r="1040" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1040" s="51" t="s">
-        <v>725</v>
+        <v>727</v>
       </c>
       <c r="B1040" s="27" t="s">
         <v>89</v>
       </c>
       <c r="C1040" s="25" t="s">
-        <v>726</v>
+        <v>728</v>
       </c>
       <c r="D1040" s="26" t="s">
-        <v>714</v>
+        <v>716</v>
       </c>
       <c r="E1040" s="26" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
       <c r="F1040" s="26" t="s">
-        <v>728</v>
+        <v>730</v>
       </c>
       <c r="G1040" s="16" t="s">
         <v>58</v>
@@ -28606,22 +28637,22 @@
     </row>
     <row r="1046" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1046" s="51" t="s">
-        <v>725</v>
+        <v>727</v>
       </c>
       <c r="B1046" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1046" s="14" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
       <c r="D1046" s="15" t="s">
-        <v>706</v>
+        <v>708</v>
       </c>
       <c r="E1046" s="15" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="F1046" s="15" t="s">
-        <v>731</v>
+        <v>733</v>
       </c>
       <c r="G1046" s="16" t="s">
         <v>58</v>
@@ -28758,16 +28789,16 @@
         <v>53</v>
       </c>
       <c r="C1052" s="25" t="s">
-        <v>732</v>
+        <v>734</v>
       </c>
       <c r="D1052" s="26" t="s">
-        <v>733</v>
+        <v>735</v>
       </c>
       <c r="E1052" s="26" t="s">
-        <v>734</v>
+        <v>736</v>
       </c>
       <c r="F1052" s="26" t="s">
-        <v>735</v>
+        <v>737</v>
       </c>
       <c r="G1052" s="16" t="s">
         <v>58</v>
@@ -28904,16 +28935,16 @@
         <v>53</v>
       </c>
       <c r="C1058" s="14" t="s">
-        <v>736</v>
+        <v>738</v>
       </c>
       <c r="D1058" s="15" t="s">
-        <v>737</v>
+        <v>739</v>
       </c>
       <c r="E1058" s="15" t="s">
-        <v>738</v>
+        <v>740</v>
       </c>
       <c r="F1058" s="15" t="s">
-        <v>739</v>
+        <v>741</v>
       </c>
       <c r="G1058" s="16" t="s">
         <v>58</v>
@@ -29999,10 +30030,10 @@
         <v>39</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>740</v>
+        <v>742</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>741</v>
+        <v>743</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>53</v>
@@ -30020,7 +30051,7 @@
         <v>86</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>742</v>
+        <v>744</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -30257,7 +30288,7 @@
     </row>
     <row r="10" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="60" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B10" s="1">
         <v>9</v>
@@ -30286,7 +30317,7 @@
     </row>
     <row r="11" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="61" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="B11" s="1">
         <v>5</v>
@@ -30315,7 +30346,7 @@
     </row>
     <row r="12" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="62" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="B12" s="1">
         <v>5</v>
@@ -30344,7 +30375,7 @@
     </row>
     <row r="13" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="63" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="B13" s="1">
         <v>4</v>
@@ -30373,7 +30404,7 @@
     </row>
     <row r="14" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="64" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="B14" s="1">
         <v>5</v>
@@ -30402,7 +30433,7 @@
     </row>
     <row r="15" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="65" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="B15" s="1">
         <v>12</v>
@@ -30431,7 +30462,7 @@
     </row>
     <row r="16" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="66" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
       <c r="B16" s="1">
         <v>4</v>
@@ -30460,7 +30491,7 @@
     </row>
     <row r="17" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="67" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="B17" s="1">
         <v>7</v>
@@ -30489,7 +30520,7 @@
     </row>
     <row r="18" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="68" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
       <c r="B18" s="1">
         <v>6</v>
@@ -30518,7 +30549,7 @@
     </row>
     <row r="19" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="69" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
       <c r="B19" s="1">
         <v>6</v>
@@ -30547,7 +30578,7 @@
     </row>
     <row r="20" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="70" t="s">
-        <v>679</v>
+        <v>681</v>
       </c>
       <c r="B20" s="1">
         <v>5</v>
@@ -30576,7 +30607,7 @@
     </row>
     <row r="21" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="71" t="s">
-        <v>700</v>
+        <v>702</v>
       </c>
       <c r="B21" s="1">
         <v>6</v>
@@ -30605,7 +30636,7 @@
     </row>
     <row r="22" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="72" t="s">
-        <v>725</v>
+        <v>727</v>
       </c>
       <c r="B22" s="1">
         <v>2</v>
@@ -30634,7 +30665,7 @@
     </row>
     <row r="23" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="73" t="s">
-        <v>743</v>
+        <v>745</v>
       </c>
       <c r="B23" s="73">
         <v>153</v>
@@ -30685,7 +30716,7 @@
         <v>44</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>741</v>
+        <v>743</v>
       </c>
       <c r="C1" s="10" t="s">
         <v>71</v>
@@ -30694,7 +30725,7 @@
         <v>86</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>742</v>
+        <v>744</v>
       </c>
       <c r="F1" s="10" t="s">
         <v>94</v>
@@ -30845,10 +30876,10 @@
         <v>45</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>744</v>
+        <v>746</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>741</v>
+        <v>743</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>71</v>
@@ -30857,7 +30888,7 @@
         <v>86</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>742</v>
+        <v>744</v>
       </c>
       <c r="G1" s="10" t="s">
         <v>94</v>
@@ -30868,7 +30899,7 @@
         <v>59</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>745</v>
+        <v>747</v>
       </c>
       <c r="C2" s="1">
         <f>COUNTIF(Proves!$H:$H,A2)</f>
@@ -30998,7 +31029,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="83" t="s">
-        <v>746</v>
+        <v>748</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -31006,7 +31037,7 @@
         <v>71</v>
       </c>
       <c r="B2" s="85" t="s">
-        <v>747</v>
+        <v>749</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
@@ -31026,7 +31057,7 @@
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>395</v>
+        <v>496</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
096 => fase IV => xips Inici marquen mascota a Llocs, filtre gats sense llocs de gos, paraules prohibides (Factory, ca), ZUP-030 ZUP-038 ZUP-055 ZUP-077 ZUP-085 ZUP-090 OK (Chrome/ADMIN)
</commit_message>
<xml_diff>
--- a/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
+++ b/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4406" uniqueCount="755">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4412" uniqueCount="755">
   <si>
     <t>Zuppeto — Joc de probes manual (totes les pantalles)</t>
   </si>
@@ -665,9 +665,6 @@
   </si>
   <si>
     <t>Títol de la portada, etiquetes pet-friendly i botons «Explora llocs» / «Entén el flux»</t>
-  </si>
-  <si>
-    <t>EN CURS</t>
   </si>
   <si>
     <t>24-08-2026</t>
@@ -1639,6 +1636,9 @@
   </si>
   <si>
     <t>Heading contacte, etiquetes i canal suport@zuppeto.fake</t>
+  </si>
+  <si>
+    <t>EN CURS</t>
   </si>
   <si>
     <t>ZUP-096</t>
@@ -8668,9 +8668,11 @@
       <c r="H212" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="I212" s="18"/>
+      <c r="I212" s="18" t="s">
+        <v>82</v>
+      </c>
       <c r="J212" s="1" t="s">
-        <v>213</v>
+        <v>71</v>
       </c>
       <c r="K212" s="19"/>
       <c r="L212" s="18"/>
@@ -8801,7 +8803,7 @@
         <v>34</v>
       </c>
       <c r="I218" s="18" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="J218" s="1" t="s">
         <v>71</v>
@@ -9193,16 +9195,16 @@
         <v>92</v>
       </c>
       <c r="C236" s="14" t="s">
+        <v>214</v>
+      </c>
+      <c r="D236" s="15" t="s">
         <v>215</v>
       </c>
-      <c r="D236" s="15" t="s">
+      <c r="E236" s="15" t="s">
         <v>216</v>
       </c>
-      <c r="E236" s="15" t="s">
+      <c r="F236" s="15" t="s">
         <v>217</v>
-      </c>
-      <c r="F236" s="15" t="s">
-        <v>218</v>
       </c>
       <c r="G236" s="16" t="s">
         <v>58</v>
@@ -9339,16 +9341,16 @@
         <v>53</v>
       </c>
       <c r="C242" s="25" t="s">
+        <v>218</v>
+      </c>
+      <c r="D242" s="26" t="s">
         <v>219</v>
       </c>
-      <c r="D242" s="26" t="s">
+      <c r="E242" s="26" t="s">
         <v>220</v>
       </c>
-      <c r="E242" s="26" t="s">
+      <c r="F242" s="26" t="s">
         <v>221</v>
-      </c>
-      <c r="F242" s="26" t="s">
-        <v>222</v>
       </c>
       <c r="G242" s="16" t="s">
         <v>58</v>
@@ -9357,7 +9359,7 @@
         <v>34</v>
       </c>
       <c r="I242" s="18" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="J242" s="1" t="s">
         <v>71</v>
@@ -9485,16 +9487,16 @@
         <v>53</v>
       </c>
       <c r="C248" s="14" t="s">
+        <v>222</v>
+      </c>
+      <c r="D248" s="15" t="s">
         <v>223</v>
       </c>
-      <c r="D248" s="15" t="s">
+      <c r="E248" s="15" t="s">
         <v>224</v>
       </c>
-      <c r="E248" s="15" t="s">
+      <c r="F248" s="15" t="s">
         <v>225</v>
-      </c>
-      <c r="F248" s="15" t="s">
-        <v>226</v>
       </c>
       <c r="G248" s="16" t="s">
         <v>58</v>
@@ -9503,7 +9505,7 @@
         <v>34</v>
       </c>
       <c r="I248" s="18" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="J248" s="1" t="s">
         <v>71</v>
@@ -9631,16 +9633,16 @@
         <v>53</v>
       </c>
       <c r="C254" s="25" t="s">
+        <v>226</v>
+      </c>
+      <c r="D254" s="26" t="s">
         <v>227</v>
       </c>
-      <c r="D254" s="26" t="s">
+      <c r="E254" s="26" t="s">
         <v>228</v>
       </c>
-      <c r="E254" s="26" t="s">
+      <c r="F254" s="26" t="s">
         <v>229</v>
-      </c>
-      <c r="F254" s="26" t="s">
-        <v>230</v>
       </c>
       <c r="G254" s="16" t="s">
         <v>58</v>
@@ -9649,13 +9651,13 @@
         <v>34</v>
       </c>
       <c r="I254" s="18" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="J254" s="1" t="s">
         <v>71</v>
       </c>
       <c r="K254" s="19" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="L254" s="18"/>
       <c r="M254" s="1"/>
@@ -9779,16 +9781,16 @@
         <v>92</v>
       </c>
       <c r="C260" s="14" t="s">
+        <v>231</v>
+      </c>
+      <c r="D260" s="15" t="s">
         <v>232</v>
       </c>
-      <c r="D260" s="15" t="s">
+      <c r="E260" s="15" t="s">
         <v>233</v>
       </c>
-      <c r="E260" s="15" t="s">
+      <c r="F260" s="15" t="s">
         <v>234</v>
-      </c>
-      <c r="F260" s="15" t="s">
-        <v>235</v>
       </c>
       <c r="G260" s="16" t="s">
         <v>58</v>
@@ -9803,7 +9805,7 @@
         <v>83</v>
       </c>
       <c r="K260" s="19" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="L260" s="18" t="s">
         <v>135</v>
@@ -9812,7 +9814,7 @@
         <v>71</v>
       </c>
       <c r="N260" s="19" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="261" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -9933,16 +9935,16 @@
         <v>92</v>
       </c>
       <c r="C266" s="25" t="s">
+        <v>237</v>
+      </c>
+      <c r="D266" s="26" t="s">
         <v>238</v>
       </c>
-      <c r="D266" s="26" t="s">
+      <c r="E266" s="26" t="s">
         <v>239</v>
       </c>
-      <c r="E266" s="26" t="s">
+      <c r="F266" s="26" t="s">
         <v>240</v>
-      </c>
-      <c r="F266" s="26" t="s">
-        <v>241</v>
       </c>
       <c r="G266" s="16" t="s">
         <v>58</v>
@@ -10079,16 +10081,16 @@
         <v>92</v>
       </c>
       <c r="C272" s="14" t="s">
+        <v>241</v>
+      </c>
+      <c r="D272" s="15" t="s">
         <v>242</v>
       </c>
-      <c r="D272" s="15" t="s">
+      <c r="E272" s="15" t="s">
         <v>243</v>
       </c>
-      <c r="E272" s="15" t="s">
+      <c r="F272" s="15" t="s">
         <v>244</v>
-      </c>
-      <c r="F272" s="15" t="s">
-        <v>245</v>
       </c>
       <c r="G272" s="16" t="s">
         <v>58</v>
@@ -10219,22 +10221,22 @@
     </row>
     <row r="278" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A278" s="36" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B278" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C278" s="25" t="s">
+        <v>246</v>
+      </c>
+      <c r="D278" s="26" t="s">
         <v>247</v>
       </c>
-      <c r="D278" s="26" t="s">
+      <c r="E278" s="26" t="s">
         <v>248</v>
       </c>
-      <c r="E278" s="26" t="s">
+      <c r="F278" s="26" t="s">
         <v>249</v>
-      </c>
-      <c r="F278" s="26" t="s">
-        <v>250</v>
       </c>
       <c r="G278" s="16" t="s">
         <v>58</v>
@@ -10242,9 +10244,11 @@
       <c r="H278" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="I278" s="18"/>
+      <c r="I278" s="18" t="s">
+        <v>82</v>
+      </c>
       <c r="J278" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K278" s="19"/>
       <c r="L278" s="18"/>
@@ -10375,13 +10379,13 @@
         <v>34</v>
       </c>
       <c r="I284" s="18" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="J284" s="1" t="s">
         <v>71</v>
       </c>
       <c r="K284" s="19" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="L284" s="18"/>
       <c r="M284" s="1"/>
@@ -10763,22 +10767,22 @@
     </row>
     <row r="302" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A302" s="36" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B302" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C302" s="14" t="s">
+        <v>251</v>
+      </c>
+      <c r="D302" s="15" t="s">
         <v>252</v>
       </c>
-      <c r="D302" s="15" t="s">
+      <c r="E302" s="15" t="s">
         <v>253</v>
       </c>
-      <c r="E302" s="15" t="s">
+      <c r="F302" s="15" t="s">
         <v>254</v>
-      </c>
-      <c r="F302" s="15" t="s">
-        <v>255</v>
       </c>
       <c r="G302" s="16" t="s">
         <v>58</v>
@@ -10787,7 +10791,7 @@
         <v>34</v>
       </c>
       <c r="I302" s="18" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="J302" s="1" t="s">
         <v>71</v>
@@ -10909,22 +10913,22 @@
     </row>
     <row r="308" ht="56" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A308" s="36" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B308" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C308" s="25" t="s">
+        <v>255</v>
+      </c>
+      <c r="D308" s="26" t="s">
         <v>256</v>
       </c>
-      <c r="D308" s="26" t="s">
+      <c r="E308" s="26" t="s">
         <v>257</v>
       </c>
-      <c r="E308" s="26" t="s">
+      <c r="F308" s="26" t="s">
         <v>258</v>
-      </c>
-      <c r="F308" s="26" t="s">
-        <v>259</v>
       </c>
       <c r="G308" s="16" t="s">
         <v>58</v>
@@ -10933,22 +10937,22 @@
         <v>34</v>
       </c>
       <c r="I308" s="18" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="J308" s="1" t="s">
         <v>83</v>
       </c>
       <c r="K308" s="19" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="L308" s="18" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="M308" s="1" t="s">
         <v>71</v>
       </c>
       <c r="N308" s="19" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="309" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -11063,22 +11067,22 @@
     </row>
     <row r="314" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A314" s="36" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B314" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C314" s="14" t="s">
+        <v>261</v>
+      </c>
+      <c r="D314" s="15" t="s">
         <v>262</v>
       </c>
-      <c r="D314" s="15" t="s">
+      <c r="E314" s="15" t="s">
         <v>263</v>
       </c>
-      <c r="E314" s="15" t="s">
+      <c r="F314" s="15" t="s">
         <v>264</v>
-      </c>
-      <c r="F314" s="15" t="s">
-        <v>265</v>
       </c>
       <c r="G314" s="16" t="s">
         <v>58</v>
@@ -11087,7 +11091,7 @@
         <v>34</v>
       </c>
       <c r="I314" s="18" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="J314" s="1" t="s">
         <v>71</v>
@@ -11209,22 +11213,22 @@
     </row>
     <row r="320" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A320" s="36" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B320" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C320" s="25" t="s">
+        <v>265</v>
+      </c>
+      <c r="D320" s="26" t="s">
         <v>266</v>
       </c>
-      <c r="D320" s="26" t="s">
+      <c r="E320" s="26" t="s">
         <v>267</v>
       </c>
-      <c r="E320" s="26" t="s">
+      <c r="F320" s="26" t="s">
         <v>268</v>
-      </c>
-      <c r="F320" s="26" t="s">
-        <v>269</v>
       </c>
       <c r="G320" s="16" t="s">
         <v>58</v>
@@ -11233,7 +11237,7 @@
         <v>34</v>
       </c>
       <c r="I320" s="18" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="J320" s="1" t="s">
         <v>71</v>
@@ -11355,22 +11359,22 @@
     </row>
     <row r="326" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A326" s="36" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B326" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C326" s="14" t="s">
+        <v>270</v>
+      </c>
+      <c r="D326" s="15" t="s">
         <v>271</v>
       </c>
-      <c r="D326" s="15" t="s">
+      <c r="E326" s="15" t="s">
         <v>272</v>
       </c>
-      <c r="E326" s="15" t="s">
+      <c r="F326" s="15" t="s">
         <v>273</v>
-      </c>
-      <c r="F326" s="15" t="s">
-        <v>274</v>
       </c>
       <c r="G326" s="16" t="s">
         <v>58</v>
@@ -11379,13 +11383,13 @@
         <v>34</v>
       </c>
       <c r="I326" s="18" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="J326" s="1" t="s">
         <v>71</v>
       </c>
       <c r="K326" s="19" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="L326" s="18"/>
       <c r="M326" s="1"/>
@@ -11503,22 +11507,22 @@
     </row>
     <row r="332" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A332" s="36" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B332" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C332" s="25" t="s">
+        <v>275</v>
+      </c>
+      <c r="D332" s="26" t="s">
         <v>276</v>
       </c>
-      <c r="D332" s="26" t="s">
+      <c r="E332" s="26" t="s">
         <v>277</v>
       </c>
-      <c r="E332" s="26" t="s">
+      <c r="F332" s="26" t="s">
         <v>278</v>
-      </c>
-      <c r="F332" s="26" t="s">
-        <v>279</v>
       </c>
       <c r="G332" s="16" t="s">
         <v>58</v>
@@ -11527,7 +11531,7 @@
         <v>34</v>
       </c>
       <c r="I332" s="18" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="J332" s="1" t="s">
         <v>71</v>
@@ -11649,22 +11653,22 @@
     </row>
     <row r="338" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A338" s="36" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B338" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C338" s="14" t="s">
+        <v>279</v>
+      </c>
+      <c r="D338" s="15" t="s">
         <v>280</v>
       </c>
-      <c r="D338" s="15" t="s">
+      <c r="E338" s="15" t="s">
         <v>281</v>
       </c>
-      <c r="E338" s="15" t="s">
+      <c r="F338" s="15" t="s">
         <v>282</v>
-      </c>
-      <c r="F338" s="15" t="s">
-        <v>283</v>
       </c>
       <c r="G338" s="16" t="s">
         <v>58</v>
@@ -11673,7 +11677,7 @@
         <v>34</v>
       </c>
       <c r="I338" s="18" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="J338" s="1" t="s">
         <v>71</v>
@@ -11795,22 +11799,22 @@
     </row>
     <row r="344" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A344" s="36" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B344" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C344" s="25" t="s">
+        <v>284</v>
+      </c>
+      <c r="D344" s="26" t="s">
         <v>285</v>
       </c>
-      <c r="D344" s="26" t="s">
+      <c r="E344" s="26" t="s">
         <v>286</v>
       </c>
-      <c r="E344" s="26" t="s">
+      <c r="F344" s="26" t="s">
         <v>287</v>
-      </c>
-      <c r="F344" s="26" t="s">
-        <v>288</v>
       </c>
       <c r="G344" s="16" t="s">
         <v>58</v>
@@ -11819,22 +11823,22 @@
         <v>34</v>
       </c>
       <c r="I344" s="18" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="J344" s="1" t="s">
         <v>83</v>
       </c>
       <c r="K344" s="19" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="L344" s="18" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="M344" s="1" t="s">
         <v>71</v>
       </c>
       <c r="N344" s="19" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="345" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -11949,22 +11953,22 @@
     </row>
     <row r="350" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A350" s="36" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B350" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C350" s="14" t="s">
+        <v>290</v>
+      </c>
+      <c r="D350" s="15" t="s">
         <v>291</v>
       </c>
-      <c r="D350" s="15" t="s">
+      <c r="E350" s="15" t="s">
         <v>292</v>
       </c>
-      <c r="E350" s="15" t="s">
+      <c r="F350" s="15" t="s">
         <v>293</v>
-      </c>
-      <c r="F350" s="15" t="s">
-        <v>294</v>
       </c>
       <c r="G350" s="16" t="s">
         <v>58</v>
@@ -11973,7 +11977,7 @@
         <v>34</v>
       </c>
       <c r="I350" s="18" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="J350" s="1" t="s">
         <v>71</v>
@@ -12095,22 +12099,22 @@
     </row>
     <row r="356" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A356" s="36" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B356" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C356" s="25" t="s">
+        <v>294</v>
+      </c>
+      <c r="D356" s="26" t="s">
         <v>295</v>
       </c>
-      <c r="D356" s="26" t="s">
+      <c r="E356" s="26" t="s">
         <v>296</v>
       </c>
-      <c r="E356" s="26" t="s">
+      <c r="F356" s="26" t="s">
         <v>297</v>
-      </c>
-      <c r="F356" s="26" t="s">
-        <v>298</v>
       </c>
       <c r="G356" s="16" t="s">
         <v>58</v>
@@ -12239,22 +12243,22 @@
     </row>
     <row r="362" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A362" s="36" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B362" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C362" s="14" t="s">
+        <v>298</v>
+      </c>
+      <c r="D362" s="15" t="s">
         <v>299</v>
       </c>
-      <c r="D362" s="15" t="s">
+      <c r="E362" s="15" t="s">
         <v>300</v>
       </c>
-      <c r="E362" s="15" t="s">
-        <v>301</v>
-      </c>
       <c r="F362" s="15" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="G362" s="16" t="s">
         <v>58</v>
@@ -12385,22 +12389,22 @@
     </row>
     <row r="368" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A368" s="36" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B368" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C368" s="25" t="s">
+        <v>301</v>
+      </c>
+      <c r="D368" s="26" t="s">
         <v>302</v>
       </c>
-      <c r="D368" s="26" t="s">
+      <c r="E368" s="26" t="s">
         <v>303</v>
       </c>
-      <c r="E368" s="26" t="s">
+      <c r="F368" s="26" t="s">
         <v>304</v>
-      </c>
-      <c r="F368" s="26" t="s">
-        <v>305</v>
       </c>
       <c r="G368" s="16" t="s">
         <v>58</v>
@@ -12409,7 +12413,7 @@
         <v>34</v>
       </c>
       <c r="I368" s="18" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="J368" s="1" t="s">
         <v>71</v>
@@ -12531,22 +12535,22 @@
     </row>
     <row r="374" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A374" s="36" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B374" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C374" s="14" t="s">
+        <v>305</v>
+      </c>
+      <c r="D374" s="15" t="s">
         <v>306</v>
       </c>
-      <c r="D374" s="15" t="s">
+      <c r="E374" s="15" t="s">
         <v>307</v>
       </c>
-      <c r="E374" s="15" t="s">
+      <c r="F374" s="15" t="s">
         <v>308</v>
-      </c>
-      <c r="F374" s="15" t="s">
-        <v>309</v>
       </c>
       <c r="G374" s="16" t="s">
         <v>58</v>
@@ -12677,22 +12681,22 @@
     </row>
     <row r="380" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A380" s="36" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B380" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C380" s="25" t="s">
+        <v>309</v>
+      </c>
+      <c r="D380" s="26" t="s">
         <v>310</v>
       </c>
-      <c r="D380" s="26" t="s">
+      <c r="E380" s="26" t="s">
         <v>311</v>
       </c>
-      <c r="E380" s="26" t="s">
+      <c r="F380" s="26" t="s">
         <v>312</v>
-      </c>
-      <c r="F380" s="26" t="s">
-        <v>313</v>
       </c>
       <c r="G380" s="16" t="s">
         <v>58</v>
@@ -12701,7 +12705,7 @@
         <v>34</v>
       </c>
       <c r="I380" s="18" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="J380" s="1" t="s">
         <v>71</v>
@@ -12823,22 +12827,22 @@
     </row>
     <row r="386" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A386" s="36" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B386" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C386" s="14" t="s">
+        <v>313</v>
+      </c>
+      <c r="D386" s="15" t="s">
         <v>314</v>
       </c>
-      <c r="D386" s="15" t="s">
+      <c r="E386" s="15" t="s">
         <v>315</v>
       </c>
-      <c r="E386" s="15" t="s">
+      <c r="F386" s="15" t="s">
         <v>316</v>
-      </c>
-      <c r="F386" s="15" t="s">
-        <v>317</v>
       </c>
       <c r="G386" s="16" t="s">
         <v>58</v>
@@ -12847,7 +12851,7 @@
         <v>34</v>
       </c>
       <c r="I386" s="18" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="J386" s="1" t="s">
         <v>71</v>
@@ -12969,22 +12973,22 @@
     </row>
     <row r="392" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A392" s="36" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B392" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C392" s="25" t="s">
+        <v>317</v>
+      </c>
+      <c r="D392" s="26" t="s">
         <v>318</v>
       </c>
-      <c r="D392" s="26" t="s">
+      <c r="E392" s="26" t="s">
         <v>319</v>
       </c>
-      <c r="E392" s="26" t="s">
+      <c r="F392" s="26" t="s">
         <v>320</v>
-      </c>
-      <c r="F392" s="26" t="s">
-        <v>321</v>
       </c>
       <c r="G392" s="16" t="s">
         <v>58</v>
@@ -12999,7 +13003,7 @@
         <v>83</v>
       </c>
       <c r="K392" s="19" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="L392" s="18" t="s">
         <v>135</v>
@@ -13008,7 +13012,7 @@
         <v>71</v>
       </c>
       <c r="N392" s="19" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="393" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -13123,22 +13127,22 @@
     </row>
     <row r="398" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A398" s="37" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B398" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C398" s="14" t="s">
+        <v>324</v>
+      </c>
+      <c r="D398" s="15" t="s">
         <v>325</v>
       </c>
-      <c r="D398" s="15" t="s">
+      <c r="E398" s="15" t="s">
         <v>326</v>
       </c>
-      <c r="E398" s="15" t="s">
+      <c r="F398" s="15" t="s">
         <v>327</v>
-      </c>
-      <c r="F398" s="15" t="s">
-        <v>328</v>
       </c>
       <c r="G398" s="16" t="s">
         <v>58</v>
@@ -13146,9 +13150,11 @@
       <c r="H398" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="I398" s="18"/>
+      <c r="I398" s="18" t="s">
+        <v>82</v>
+      </c>
       <c r="J398" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K398" s="19"/>
       <c r="L398" s="18"/>
@@ -13279,13 +13285,13 @@
         <v>34</v>
       </c>
       <c r="I404" s="18" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="J404" s="1" t="s">
         <v>71</v>
       </c>
       <c r="K404" s="19" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="L404" s="18"/>
       <c r="M404" s="1"/>
@@ -13667,22 +13673,22 @@
     </row>
     <row r="422" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A422" s="37" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B422" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C422" s="25" t="s">
+        <v>330</v>
+      </c>
+      <c r="D422" s="26" t="s">
         <v>331</v>
       </c>
-      <c r="D422" s="26" t="s">
+      <c r="E422" s="26" t="s">
         <v>332</v>
       </c>
-      <c r="E422" s="26" t="s">
+      <c r="F422" s="26" t="s">
         <v>333</v>
-      </c>
-      <c r="F422" s="26" t="s">
-        <v>334</v>
       </c>
       <c r="G422" s="16" t="s">
         <v>58</v>
@@ -13691,7 +13697,7 @@
         <v>34</v>
       </c>
       <c r="I422" s="18" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="J422" s="1" t="s">
         <v>71</v>
@@ -13813,22 +13819,22 @@
     </row>
     <row r="428" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A428" s="37" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B428" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C428" s="14" t="s">
+        <v>335</v>
+      </c>
+      <c r="D428" s="15" t="s">
         <v>336</v>
       </c>
-      <c r="D428" s="15" t="s">
+      <c r="E428" s="15" t="s">
         <v>337</v>
       </c>
-      <c r="E428" s="15" t="s">
+      <c r="F428" s="15" t="s">
         <v>338</v>
-      </c>
-      <c r="F428" s="15" t="s">
-        <v>339</v>
       </c>
       <c r="G428" s="16" t="s">
         <v>58</v>
@@ -13843,7 +13849,7 @@
         <v>71</v>
       </c>
       <c r="K428" s="19" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="L428" s="18"/>
       <c r="M428" s="1"/>
@@ -13961,22 +13967,22 @@
     </row>
     <row r="434" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A434" s="37" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B434" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C434" s="25" t="s">
+        <v>340</v>
+      </c>
+      <c r="D434" s="26" t="s">
         <v>341</v>
       </c>
-      <c r="D434" s="26" t="s">
+      <c r="E434" s="26" t="s">
         <v>342</v>
       </c>
-      <c r="E434" s="26" t="s">
+      <c r="F434" s="26" t="s">
         <v>343</v>
-      </c>
-      <c r="F434" s="26" t="s">
-        <v>344</v>
       </c>
       <c r="G434" s="16" t="s">
         <v>58</v>
@@ -13991,7 +13997,7 @@
         <v>83</v>
       </c>
       <c r="K434" s="19" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="L434" s="18"/>
       <c r="M434" s="1"/>
@@ -14109,22 +14115,22 @@
     </row>
     <row r="440" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A440" s="37" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B440" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C440" s="14" t="s">
+        <v>345</v>
+      </c>
+      <c r="D440" s="15" t="s">
         <v>346</v>
       </c>
-      <c r="D440" s="15" t="s">
+      <c r="E440" s="15" t="s">
         <v>347</v>
       </c>
-      <c r="E440" s="15" t="s">
+      <c r="F440" s="15" t="s">
         <v>348</v>
-      </c>
-      <c r="F440" s="15" t="s">
-        <v>349</v>
       </c>
       <c r="G440" s="16" t="s">
         <v>58</v>
@@ -14255,22 +14261,22 @@
     </row>
     <row r="446" ht="77" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A446" s="37" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B446" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C446" s="25" t="s">
+        <v>349</v>
+      </c>
+      <c r="D446" s="26" t="s">
         <v>350</v>
       </c>
-      <c r="D446" s="26" t="s">
+      <c r="E446" s="26" t="s">
         <v>351</v>
       </c>
-      <c r="E446" s="26" t="s">
+      <c r="F446" s="26" t="s">
         <v>352</v>
-      </c>
-      <c r="F446" s="26" t="s">
-        <v>353</v>
       </c>
       <c r="G446" s="16" t="s">
         <v>58</v>
@@ -14279,22 +14285,22 @@
         <v>34</v>
       </c>
       <c r="I446" s="18" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="J446" s="1" t="s">
         <v>83</v>
       </c>
       <c r="K446" s="19" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="L446" s="18" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="M446" s="1" t="s">
         <v>71</v>
       </c>
       <c r="N446" s="19" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="447" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -14409,22 +14415,22 @@
     </row>
     <row r="452" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A452" s="37" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B452" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C452" s="14" t="s">
+        <v>355</v>
+      </c>
+      <c r="D452" s="15" t="s">
         <v>356</v>
       </c>
-      <c r="D452" s="15" t="s">
+      <c r="E452" s="15" t="s">
         <v>357</v>
       </c>
-      <c r="E452" s="15" t="s">
+      <c r="F452" s="15" t="s">
         <v>358</v>
-      </c>
-      <c r="F452" s="15" t="s">
-        <v>359</v>
       </c>
       <c r="G452" s="16" t="s">
         <v>58</v>
@@ -14555,22 +14561,22 @@
     </row>
     <row r="458" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A458" s="37" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B458" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C458" s="25" t="s">
+        <v>359</v>
+      </c>
+      <c r="D458" s="26" t="s">
         <v>360</v>
       </c>
-      <c r="D458" s="26" t="s">
+      <c r="E458" s="26" t="s">
         <v>361</v>
       </c>
-      <c r="E458" s="26" t="s">
+      <c r="F458" s="26" t="s">
         <v>362</v>
-      </c>
-      <c r="F458" s="26" t="s">
-        <v>363</v>
       </c>
       <c r="G458" s="16" t="s">
         <v>58</v>
@@ -14701,22 +14707,22 @@
     </row>
     <row r="464" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A464" s="37" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B464" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C464" s="14" t="s">
+        <v>363</v>
+      </c>
+      <c r="D464" s="15" t="s">
         <v>364</v>
       </c>
-      <c r="D464" s="15" t="s">
+      <c r="E464" s="15" t="s">
         <v>365</v>
       </c>
-      <c r="E464" s="15" t="s">
+      <c r="F464" s="15" t="s">
         <v>366</v>
-      </c>
-      <c r="F464" s="15" t="s">
-        <v>367</v>
       </c>
       <c r="G464" s="16" t="s">
         <v>58</v>
@@ -14847,22 +14853,22 @@
     </row>
     <row r="470" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A470" s="37" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B470" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C470" s="25" t="s">
+        <v>367</v>
+      </c>
+      <c r="D470" s="26" t="s">
         <v>368</v>
       </c>
-      <c r="D470" s="26" t="s">
+      <c r="E470" s="26" t="s">
         <v>369</v>
       </c>
-      <c r="E470" s="26" t="s">
+      <c r="F470" s="26" t="s">
         <v>370</v>
-      </c>
-      <c r="F470" s="26" t="s">
-        <v>371</v>
       </c>
       <c r="G470" s="16" t="s">
         <v>58</v>
@@ -14871,7 +14877,7 @@
         <v>34</v>
       </c>
       <c r="I470" s="18" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="J470" s="1" t="s">
         <v>71</v>
@@ -14993,22 +14999,22 @@
     </row>
     <row r="476" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A476" s="38" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B476" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C476" s="14" t="s">
+        <v>372</v>
+      </c>
+      <c r="D476" s="15" t="s">
         <v>373</v>
       </c>
-      <c r="D476" s="15" t="s">
+      <c r="E476" s="15" t="s">
         <v>374</v>
       </c>
-      <c r="E476" s="15" t="s">
+      <c r="F476" s="15" t="s">
         <v>375</v>
-      </c>
-      <c r="F476" s="15" t="s">
-        <v>376</v>
       </c>
       <c r="G476" s="16" t="s">
         <v>58</v>
@@ -15017,13 +15023,13 @@
         <v>34</v>
       </c>
       <c r="I476" s="18" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="J476" s="1" t="s">
         <v>71</v>
       </c>
       <c r="K476" s="19" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="L476" s="18"/>
       <c r="M476" s="1"/>
@@ -15141,22 +15147,22 @@
     </row>
     <row r="482" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A482" s="38" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B482" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C482" s="25" t="s">
+        <v>377</v>
+      </c>
+      <c r="D482" s="26" t="s">
         <v>378</v>
       </c>
-      <c r="D482" s="26" t="s">
+      <c r="E482" s="26" t="s">
         <v>379</v>
       </c>
-      <c r="E482" s="26" t="s">
+      <c r="F482" s="26" t="s">
         <v>380</v>
-      </c>
-      <c r="F482" s="26" t="s">
-        <v>381</v>
       </c>
       <c r="G482" s="16" t="s">
         <v>58</v>
@@ -15165,13 +15171,13 @@
         <v>34</v>
       </c>
       <c r="I482" s="18" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="J482" s="1" t="s">
         <v>71</v>
       </c>
       <c r="K482" s="19" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="L482" s="18"/>
       <c r="M482" s="1"/>
@@ -15289,22 +15295,22 @@
     </row>
     <row r="488" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A488" s="38" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B488" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C488" s="14" t="s">
+        <v>382</v>
+      </c>
+      <c r="D488" s="15" t="s">
         <v>383</v>
       </c>
-      <c r="D488" s="15" t="s">
+      <c r="E488" s="15" t="s">
         <v>384</v>
       </c>
-      <c r="E488" s="15" t="s">
+      <c r="F488" s="15" t="s">
         <v>385</v>
-      </c>
-      <c r="F488" s="15" t="s">
-        <v>386</v>
       </c>
       <c r="G488" s="16" t="s">
         <v>58</v>
@@ -15313,7 +15319,7 @@
         <v>34</v>
       </c>
       <c r="I488" s="18" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="J488" s="1" t="s">
         <v>71</v>
@@ -15435,22 +15441,22 @@
     </row>
     <row r="494" ht="110" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A494" s="38" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B494" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C494" s="25" t="s">
+        <v>386</v>
+      </c>
+      <c r="D494" s="26" t="s">
         <v>387</v>
       </c>
-      <c r="D494" s="26" t="s">
+      <c r="E494" s="26" t="s">
         <v>388</v>
       </c>
-      <c r="E494" s="26" t="s">
+      <c r="F494" s="26" t="s">
         <v>389</v>
-      </c>
-      <c r="F494" s="26" t="s">
-        <v>390</v>
       </c>
       <c r="G494" s="16" t="s">
         <v>58</v>
@@ -15465,7 +15471,7 @@
         <v>83</v>
       </c>
       <c r="K494" s="19" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
       <c r="L494" s="18" t="s">
         <v>82</v>
@@ -15474,7 +15480,7 @@
         <v>71</v>
       </c>
       <c r="N494" s="19" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="495" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -15589,22 +15595,22 @@
     </row>
     <row r="500" ht="96" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A500" s="38" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B500" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C500" s="14" t="s">
+        <v>392</v>
+      </c>
+      <c r="D500" s="15" t="s">
         <v>393</v>
       </c>
-      <c r="D500" s="15" t="s">
+      <c r="E500" s="15" t="s">
         <v>394</v>
       </c>
-      <c r="E500" s="15" t="s">
+      <c r="F500" s="15" t="s">
         <v>395</v>
-      </c>
-      <c r="F500" s="15" t="s">
-        <v>396</v>
       </c>
       <c r="G500" s="16" t="s">
         <v>58</v>
@@ -15619,7 +15625,7 @@
         <v>83</v>
       </c>
       <c r="K500" s="19" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="L500" s="18" t="s">
         <v>82</v>
@@ -15628,7 +15634,7 @@
         <v>71</v>
       </c>
       <c r="N500" s="19" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
     </row>
     <row r="501" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -15743,22 +15749,22 @@
     </row>
     <row r="506" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A506" s="38" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B506" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C506" s="25" t="s">
+        <v>398</v>
+      </c>
+      <c r="D506" s="26" t="s">
         <v>399</v>
       </c>
-      <c r="D506" s="26" t="s">
+      <c r="E506" s="26" t="s">
+        <v>257</v>
+      </c>
+      <c r="F506" s="26" t="s">
         <v>400</v>
-      </c>
-      <c r="E506" s="26" t="s">
-        <v>258</v>
-      </c>
-      <c r="F506" s="26" t="s">
-        <v>401</v>
       </c>
       <c r="G506" s="16" t="s">
         <v>58</v>
@@ -15889,22 +15895,22 @@
     </row>
     <row r="512" ht="80" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A512" s="38" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B512" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C512" s="14" t="s">
+        <v>401</v>
+      </c>
+      <c r="D512" s="15" t="s">
         <v>402</v>
       </c>
-      <c r="D512" s="15" t="s">
+      <c r="E512" s="15" t="s">
         <v>403</v>
       </c>
-      <c r="E512" s="15" t="s">
+      <c r="F512" s="15" t="s">
         <v>404</v>
-      </c>
-      <c r="F512" s="15" t="s">
-        <v>405</v>
       </c>
       <c r="G512" s="16" t="s">
         <v>58</v>
@@ -15919,7 +15925,7 @@
         <v>83</v>
       </c>
       <c r="K512" s="19" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="L512" s="18" t="s">
         <v>82</v>
@@ -15928,7 +15934,7 @@
         <v>71</v>
       </c>
       <c r="N512" s="19" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="513" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -16043,22 +16049,22 @@
     </row>
     <row r="518" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A518" s="38" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B518" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C518" s="25" t="s">
+        <v>407</v>
+      </c>
+      <c r="D518" s="26" t="s">
         <v>408</v>
       </c>
-      <c r="D518" s="26" t="s">
+      <c r="E518" s="26" t="s">
         <v>409</v>
       </c>
-      <c r="E518" s="26" t="s">
+      <c r="F518" s="26" t="s">
         <v>410</v>
-      </c>
-      <c r="F518" s="26" t="s">
-        <v>411</v>
       </c>
       <c r="G518" s="16" t="s">
         <v>58</v>
@@ -16189,22 +16195,22 @@
     </row>
     <row r="524" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A524" s="38" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B524" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C524" s="14" t="s">
+        <v>411</v>
+      </c>
+      <c r="D524" s="15" t="s">
         <v>412</v>
       </c>
-      <c r="D524" s="15" t="s">
+      <c r="E524" s="15" t="s">
         <v>413</v>
       </c>
-      <c r="E524" s="15" t="s">
+      <c r="F524" s="15" t="s">
         <v>414</v>
-      </c>
-      <c r="F524" s="15" t="s">
-        <v>415</v>
       </c>
       <c r="G524" s="16" t="s">
         <v>58</v>
@@ -16213,7 +16219,7 @@
         <v>34</v>
       </c>
       <c r="I524" s="18" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="J524" s="1" t="s">
         <v>71</v>
@@ -16335,22 +16341,22 @@
     </row>
     <row r="530" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A530" s="38" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B530" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C530" s="25" t="s">
+        <v>415</v>
+      </c>
+      <c r="D530" s="26" t="s">
         <v>416</v>
       </c>
-      <c r="D530" s="26" t="s">
+      <c r="E530" s="26" t="s">
         <v>417</v>
       </c>
-      <c r="E530" s="26" t="s">
+      <c r="F530" s="26" t="s">
         <v>418</v>
-      </c>
-      <c r="F530" s="26" t="s">
-        <v>419</v>
       </c>
       <c r="G530" s="16" t="s">
         <v>58</v>
@@ -16359,7 +16365,7 @@
         <v>34</v>
       </c>
       <c r="I530" s="18" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="J530" s="1" t="s">
         <v>71</v>
@@ -16481,22 +16487,22 @@
     </row>
     <row r="536" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A536" s="38" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B536" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C536" s="14" t="s">
+        <v>419</v>
+      </c>
+      <c r="D536" s="15" t="s">
         <v>420</v>
       </c>
-      <c r="D536" s="15" t="s">
+      <c r="E536" s="15" t="s">
         <v>421</v>
       </c>
-      <c r="E536" s="15" t="s">
+      <c r="F536" s="15" t="s">
         <v>422</v>
-      </c>
-      <c r="F536" s="15" t="s">
-        <v>423</v>
       </c>
       <c r="G536" s="16" t="s">
         <v>58</v>
@@ -16505,7 +16511,7 @@
         <v>34</v>
       </c>
       <c r="I536" s="18" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="J536" s="1" t="s">
         <v>71</v>
@@ -16627,22 +16633,22 @@
     </row>
     <row r="542" ht="180" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A542" s="39" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="B542" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C542" s="25" t="s">
+        <v>424</v>
+      </c>
+      <c r="D542" s="26" t="s">
         <v>425</v>
       </c>
-      <c r="D542" s="26" t="s">
+      <c r="E542" s="26" t="s">
         <v>426</v>
       </c>
-      <c r="E542" s="26" t="s">
+      <c r="F542" s="26" t="s">
         <v>427</v>
-      </c>
-      <c r="F542" s="26" t="s">
-        <v>428</v>
       </c>
       <c r="G542" s="16" t="s">
         <v>58</v>
@@ -16651,13 +16657,13 @@
         <v>34</v>
       </c>
       <c r="I542" s="18" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="J542" s="1" t="s">
         <v>83</v>
       </c>
       <c r="K542" s="19" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="L542" s="18">
         <v>46264.91666666667</v>
@@ -16666,7 +16672,7 @@
         <v>71</v>
       </c>
       <c r="N542" s="19" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="543" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -16781,22 +16787,22 @@
     </row>
     <row r="548" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A548" s="39" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="B548" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C548" s="14" t="s">
+        <v>430</v>
+      </c>
+      <c r="D548" s="15" t="s">
         <v>431</v>
       </c>
-      <c r="D548" s="15" t="s">
+      <c r="E548" s="15" t="s">
         <v>432</v>
       </c>
-      <c r="E548" s="15" t="s">
+      <c r="F548" s="15" t="s">
         <v>433</v>
-      </c>
-      <c r="F548" s="15" t="s">
-        <v>434</v>
       </c>
       <c r="G548" s="16" t="s">
         <v>58</v>
@@ -16804,9 +16810,11 @@
       <c r="H548" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="I548" s="18"/>
+      <c r="I548" s="18" t="s">
+        <v>82</v>
+      </c>
       <c r="J548" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K548" s="19"/>
       <c r="L548" s="18"/>
@@ -16925,22 +16933,22 @@
     </row>
     <row r="554" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A554" s="39" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="B554" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C554" s="25" t="s">
+        <v>434</v>
+      </c>
+      <c r="D554" s="26" t="s">
         <v>435</v>
       </c>
-      <c r="D554" s="26" t="s">
+      <c r="E554" s="26" t="s">
         <v>436</v>
       </c>
-      <c r="E554" s="26" t="s">
+      <c r="F554" s="26" t="s">
         <v>437</v>
-      </c>
-      <c r="F554" s="26" t="s">
-        <v>438</v>
       </c>
       <c r="G554" s="16" t="s">
         <v>58</v>
@@ -17071,22 +17079,22 @@
     </row>
     <row r="560" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A560" s="39" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="B560" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C560" s="14" t="s">
+        <v>438</v>
+      </c>
+      <c r="D560" s="15" t="s">
         <v>439</v>
       </c>
-      <c r="D560" s="15" t="s">
+      <c r="E560" s="15" t="s">
         <v>440</v>
       </c>
-      <c r="E560" s="15" t="s">
+      <c r="F560" s="15" t="s">
         <v>441</v>
-      </c>
-      <c r="F560" s="15" t="s">
-        <v>442</v>
       </c>
       <c r="G560" s="16" t="s">
         <v>58</v>
@@ -17217,22 +17225,22 @@
     </row>
     <row r="566" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A566" s="39" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="B566" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C566" s="25" t="s">
+        <v>442</v>
+      </c>
+      <c r="D566" s="26" t="s">
         <v>443</v>
       </c>
-      <c r="D566" s="26" t="s">
+      <c r="E566" s="26" t="s">
         <v>444</v>
       </c>
-      <c r="E566" s="26" t="s">
+      <c r="F566" s="26" t="s">
         <v>445</v>
-      </c>
-      <c r="F566" s="26" t="s">
-        <v>446</v>
       </c>
       <c r="G566" s="16" t="s">
         <v>58</v>
@@ -17363,22 +17371,22 @@
     </row>
     <row r="572" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A572" s="39" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="B572" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C572" s="14" t="s">
+        <v>446</v>
+      </c>
+      <c r="D572" s="15" t="s">
         <v>447</v>
       </c>
-      <c r="D572" s="15" t="s">
+      <c r="E572" s="15" t="s">
         <v>448</v>
       </c>
-      <c r="E572" s="15" t="s">
+      <c r="F572" s="15" t="s">
         <v>449</v>
-      </c>
-      <c r="F572" s="15" t="s">
-        <v>450</v>
       </c>
       <c r="G572" s="16" t="s">
         <v>58</v>
@@ -17509,22 +17517,22 @@
     </row>
     <row r="578" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A578" s="39" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="B578" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C578" s="25" t="s">
+        <v>450</v>
+      </c>
+      <c r="D578" s="26" t="s">
         <v>451</v>
       </c>
-      <c r="D578" s="26" t="s">
+      <c r="E578" s="26" t="s">
         <v>452</v>
       </c>
-      <c r="E578" s="26" t="s">
+      <c r="F578" s="26" t="s">
         <v>453</v>
-      </c>
-      <c r="F578" s="26" t="s">
-        <v>454</v>
       </c>
       <c r="G578" s="16" t="s">
         <v>58</v>
@@ -17655,22 +17663,22 @@
     </row>
     <row r="584" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A584" s="39" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="B584" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C584" s="14" t="s">
+        <v>454</v>
+      </c>
+      <c r="D584" s="15" t="s">
         <v>455</v>
       </c>
-      <c r="D584" s="15" t="s">
+      <c r="E584" s="15" t="s">
         <v>456</v>
       </c>
-      <c r="E584" s="15" t="s">
+      <c r="F584" s="15" t="s">
         <v>457</v>
-      </c>
-      <c r="F584" s="15" t="s">
-        <v>458</v>
       </c>
       <c r="G584" s="16" t="s">
         <v>58</v>
@@ -17799,22 +17807,22 @@
     </row>
     <row r="590" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A590" s="39" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="B590" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C590" s="25" t="s">
+        <v>458</v>
+      </c>
+      <c r="D590" s="26" t="s">
         <v>459</v>
       </c>
-      <c r="D590" s="26" t="s">
+      <c r="E590" s="26" t="s">
         <v>460</v>
       </c>
-      <c r="E590" s="26" t="s">
+      <c r="F590" s="26" t="s">
         <v>461</v>
-      </c>
-      <c r="F590" s="26" t="s">
-        <v>462</v>
       </c>
       <c r="G590" s="16" t="s">
         <v>58</v>
@@ -17945,22 +17953,22 @@
     </row>
     <row r="596" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A596" s="40" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="B596" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C596" s="14" t="s">
+        <v>463</v>
+      </c>
+      <c r="D596" s="15" t="s">
         <v>464</v>
       </c>
-      <c r="D596" s="15" t="s">
+      <c r="E596" s="15" t="s">
         <v>465</v>
       </c>
-      <c r="E596" s="15" t="s">
+      <c r="F596" s="15" t="s">
         <v>466</v>
-      </c>
-      <c r="F596" s="15" t="s">
-        <v>467</v>
       </c>
       <c r="G596" s="16" t="s">
         <v>58</v>
@@ -17968,9 +17976,11 @@
       <c r="H596" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="I596" s="18"/>
+      <c r="I596" s="18" t="s">
+        <v>82</v>
+      </c>
       <c r="J596" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K596" s="19"/>
       <c r="L596" s="18"/>
@@ -18107,7 +18117,7 @@
         <v>83</v>
       </c>
       <c r="K602" s="19" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="L602" s="18">
         <v>46264.91666666667</v>
@@ -18116,7 +18126,7 @@
         <v>71</v>
       </c>
       <c r="N602" s="19" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
     </row>
     <row r="603" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -18495,22 +18505,22 @@
     </row>
     <row r="620" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A620" s="40" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="B620" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C620" s="25" t="s">
+        <v>469</v>
+      </c>
+      <c r="D620" s="26" t="s">
         <v>470</v>
       </c>
-      <c r="D620" s="26" t="s">
+      <c r="E620" s="26" t="s">
         <v>471</v>
       </c>
-      <c r="E620" s="26" t="s">
+      <c r="F620" s="26" t="s">
         <v>472</v>
-      </c>
-      <c r="F620" s="26" t="s">
-        <v>473</v>
       </c>
       <c r="G620" s="16" t="s">
         <v>58</v>
@@ -18641,22 +18651,22 @@
     </row>
     <row r="626" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A626" s="40" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="B626" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C626" s="14" t="s">
+        <v>473</v>
+      </c>
+      <c r="D626" s="15" t="s">
         <v>474</v>
       </c>
-      <c r="D626" s="15" t="s">
+      <c r="E626" s="15" t="s">
         <v>475</v>
       </c>
-      <c r="E626" s="15" t="s">
+      <c r="F626" s="15" t="s">
         <v>476</v>
-      </c>
-      <c r="F626" s="15" t="s">
-        <v>477</v>
       </c>
       <c r="G626" s="16" t="s">
         <v>58</v>
@@ -18787,22 +18797,22 @@
     </row>
     <row r="632" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A632" s="40" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="B632" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C632" s="25" t="s">
+        <v>477</v>
+      </c>
+      <c r="D632" s="26" t="s">
         <v>478</v>
       </c>
-      <c r="D632" s="26" t="s">
+      <c r="E632" s="26" t="s">
         <v>479</v>
       </c>
-      <c r="E632" s="26" t="s">
+      <c r="F632" s="26" t="s">
         <v>480</v>
-      </c>
-      <c r="F632" s="26" t="s">
-        <v>481</v>
       </c>
       <c r="G632" s="16" t="s">
         <v>58</v>
@@ -18933,22 +18943,22 @@
     </row>
     <row r="638" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A638" s="40" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="B638" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C638" s="14" t="s">
+        <v>481</v>
+      </c>
+      <c r="D638" s="15" t="s">
         <v>482</v>
       </c>
-      <c r="D638" s="15" t="s">
+      <c r="E638" s="15" t="s">
         <v>483</v>
       </c>
-      <c r="E638" s="15" t="s">
+      <c r="F638" s="15" t="s">
         <v>484</v>
-      </c>
-      <c r="F638" s="15" t="s">
-        <v>485</v>
       </c>
       <c r="G638" s="16" t="s">
         <v>58</v>
@@ -19079,22 +19089,22 @@
     </row>
     <row r="644" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A644" s="41" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="B644" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C644" s="25" t="s">
+        <v>486</v>
+      </c>
+      <c r="D644" s="26" t="s">
         <v>487</v>
       </c>
-      <c r="D644" s="26" t="s">
+      <c r="E644" s="26" t="s">
         <v>488</v>
       </c>
-      <c r="E644" s="26" t="s">
+      <c r="F644" s="26" t="s">
         <v>489</v>
-      </c>
-      <c r="F644" s="26" t="s">
-        <v>490</v>
       </c>
       <c r="G644" s="16" t="s">
         <v>58</v>
@@ -19102,9 +19112,11 @@
       <c r="H644" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="I644" s="18"/>
+      <c r="I644" s="18" t="s">
+        <v>82</v>
+      </c>
       <c r="J644" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K644" s="19"/>
       <c r="L644" s="18"/>
@@ -19621,22 +19633,22 @@
     </row>
     <row r="668" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A668" s="41" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="B668" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C668" s="14" t="s">
+        <v>490</v>
+      </c>
+      <c r="D668" s="15" t="s">
         <v>491</v>
       </c>
-      <c r="D668" s="15" t="s">
+      <c r="E668" s="15" t="s">
         <v>492</v>
       </c>
-      <c r="E668" s="15" t="s">
+      <c r="F668" s="15" t="s">
         <v>493</v>
-      </c>
-      <c r="F668" s="15" t="s">
-        <v>494</v>
       </c>
       <c r="G668" s="16" t="s">
         <v>58</v>
@@ -19767,22 +19779,22 @@
     </row>
     <row r="674" ht="88" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A674" s="41" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="B674" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C674" s="25" t="s">
+        <v>494</v>
+      </c>
+      <c r="D674" s="26" t="s">
         <v>495</v>
       </c>
-      <c r="D674" s="26" t="s">
+      <c r="E674" s="26" t="s">
         <v>496</v>
       </c>
-      <c r="E674" s="26" t="s">
+      <c r="F674" s="26" t="s">
         <v>497</v>
-      </c>
-      <c r="F674" s="26" t="s">
-        <v>498</v>
       </c>
       <c r="G674" s="16" t="s">
         <v>58</v>
@@ -19797,7 +19809,7 @@
         <v>83</v>
       </c>
       <c r="K674" s="19" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="L674" s="18" t="s">
         <v>82</v>
@@ -19806,7 +19818,7 @@
         <v>71</v>
       </c>
       <c r="N674" s="19" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
     </row>
     <row r="675" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -19921,22 +19933,22 @@
     </row>
     <row r="680" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A680" s="41" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="B680" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C680" s="14" t="s">
+        <v>500</v>
+      </c>
+      <c r="D680" s="15" t="s">
         <v>501</v>
       </c>
-      <c r="D680" s="15" t="s">
+      <c r="E680" s="15" t="s">
         <v>502</v>
       </c>
-      <c r="E680" s="15" t="s">
-        <v>503</v>
-      </c>
       <c r="F680" s="15" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="G680" s="16" t="s">
         <v>58</v>
@@ -20067,22 +20079,22 @@
     </row>
     <row r="686" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A686" s="41" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="B686" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C686" s="25" t="s">
+        <v>503</v>
+      </c>
+      <c r="D686" s="26" t="s">
         <v>504</v>
       </c>
-      <c r="D686" s="26" t="s">
+      <c r="E686" s="26" t="s">
         <v>505</v>
       </c>
-      <c r="E686" s="26" t="s">
+      <c r="F686" s="26" t="s">
         <v>506</v>
-      </c>
-      <c r="F686" s="26" t="s">
-        <v>507</v>
       </c>
       <c r="G686" s="16" t="s">
         <v>58</v>
@@ -20213,22 +20225,22 @@
     </row>
     <row r="692" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A692" s="42" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="B692" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C692" s="14" t="s">
+        <v>508</v>
+      </c>
+      <c r="D692" s="15" t="s">
         <v>509</v>
       </c>
-      <c r="D692" s="15" t="s">
+      <c r="E692" s="15" t="s">
         <v>510</v>
       </c>
-      <c r="E692" s="15" t="s">
+      <c r="F692" s="15" t="s">
         <v>511</v>
-      </c>
-      <c r="F692" s="15" t="s">
-        <v>512</v>
       </c>
       <c r="G692" s="16" t="s">
         <v>58</v>
@@ -20238,7 +20250,7 @@
       </c>
       <c r="I692" s="18"/>
       <c r="J692" s="1" t="s">
-        <v>60</v>
+        <v>512</v>
       </c>
       <c r="K692" s="19"/>
       <c r="L692" s="18"/>
@@ -20755,7 +20767,7 @@
     </row>
     <row r="716" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A716" s="42" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="B716" s="27" t="s">
         <v>92</v>
@@ -20901,7 +20913,7 @@
     </row>
     <row r="722" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A722" s="42" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="B722" s="27" t="s">
         <v>92</v>
@@ -21049,7 +21061,7 @@
     </row>
     <row r="728" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A728" s="42" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="B728" s="27" t="s">
         <v>92</v>
@@ -21058,13 +21070,13 @@
         <v>522</v>
       </c>
       <c r="D728" s="26" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="E728" s="26" t="s">
         <v>519</v>
       </c>
       <c r="F728" s="26" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="G728" s="16" t="s">
         <v>58</v>
@@ -30247,7 +30259,7 @@
     </row>
     <row r="7" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="57" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B7" s="1">
         <v>17</v>
@@ -30276,7 +30288,7 @@
     </row>
     <row r="8" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="58" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="B8" s="1">
         <v>10</v>
@@ -30305,7 +30317,7 @@
     </row>
     <row r="9" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="59" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B9" s="1">
         <v>11</v>
@@ -30334,7 +30346,7 @@
     </row>
     <row r="10" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="60" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="B10" s="1">
         <v>9</v>
@@ -30363,7 +30375,7 @@
     </row>
     <row r="11" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="61" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="B11" s="1">
         <v>5</v>
@@ -30392,7 +30404,7 @@
     </row>
     <row r="12" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="62" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="B12" s="1">
         <v>5</v>
@@ -30421,7 +30433,7 @@
     </row>
     <row r="13" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="63" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="B13" s="1">
         <v>4</v>
@@ -31103,7 +31115,7 @@
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>213</v>
+        <v>512</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
097 => fase IV => alta/edició usuari amb contrasenya (confirmació, força, ull; admin sense actual), check privacitat a Nou rol, ZUP-095 ZUP-099 ZUP-101–106 OK i ZUP-100 KO/corr (Chrome/ADMIN)
</commit_message>
<xml_diff>
--- a/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
+++ b/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4412" uniqueCount="755">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4425" uniqueCount="757">
   <si>
     <t>Zuppeto — Joc de probes manual (totes les pantalles)</t>
   </si>
@@ -1638,163 +1638,171 @@
     <t>Heading contacte, etiquetes i canal suport@zuppeto.fake</t>
   </si>
   <si>
+    <t>ZUP-096</t>
+  </si>
+  <si>
+    <t>Targetes de canals</t>
+  </si>
+  <si>
+    <t>Revisar graella Partnerships / Feedback / Ciutats</t>
+  </si>
+  <si>
+    <t>Targetes informatives amb text coherent</t>
+  </si>
+  <si>
+    <t>ZUP-097</t>
+  </si>
+  <si>
+    <t>Botó «Veure com funciona»</t>
+  </si>
+  <si>
+    <t>Clic enllaç</t>
+  </si>
+  <si>
+    <t>Navega a /ajuda</t>
+  </si>
+  <si>
+    <t>OK: «Veure com funciona» obre Ajuda. Copy de Contacte (provisional / .fake) anotat com a millora pendent; no s’ha canviat ara.</t>
+  </si>
+  <si>
+    <t>ZUP-098</t>
+  </si>
+  <si>
+    <t>Admin · Rols (/admin/rols)</t>
+  </si>
+  <si>
+    <t>ZUP-099</t>
+  </si>
+  <si>
+    <t>Catàleg de rols — llistat</t>
+  </si>
+  <si>
+    <t>ADMIN → /admin/rols</t>
+  </si>
+  <si>
+    <t>Títol «Catàleg de rols» i graella</t>
+  </si>
+  <si>
+    <t>ZUP-100</t>
+  </si>
+  <si>
+    <t>Alta rol nou</t>
+  </si>
+  <si>
+    <t>Crear rol amb clau única i nom visible</t>
+  </si>
+  <si>
+    <t>Rol apareix al catàleg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A Nou rol, Desar queda desactivat i no es pot crear el rol.
+Falta el requadre d’acceptar la privacitat (sí que hi és a països, ciutats i llocs).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Què s’ha fet: s’ha afegit el requadre «Accepto les condicions de privacitat d’aquest entorn intern» a l’alta de rol. Desar s’activa un cop marcat, com a la resta de catàlegs.
+Fitxers: src/Web/src/app/features/admin/pages/admin-console-page/admin-console-page.component.html; docs/ca/funcional-ca.md; docs/ca/tecnic-ca.md</t>
+  </si>
+  <si>
+    <t>ZUP-101</t>
+  </si>
+  <si>
+    <t>Editar rol existent</t>
+  </si>
+  <si>
+    <t>Canviar nom visible o estat actiu</t>
+  </si>
+  <si>
+    <t>Canvis desats</t>
+  </si>
+  <si>
+    <t>ZUP-102</t>
+  </si>
+  <si>
+    <t>Baixa rol sense dependències</t>
+  </si>
+  <si>
+    <t>Esborrar rol sense usuaris assignats</t>
+  </si>
+  <si>
+    <t>Rol eliminat</t>
+  </si>
+  <si>
+    <t>ZUP-103</t>
+  </si>
+  <si>
+    <t>Baixa rol amb usuaris</t>
+  </si>
+  <si>
+    <t>Intentar esborrar rol en ús</t>
+  </si>
+  <si>
+    <t>Operació rebutjada amb missatge clar</t>
+  </si>
+  <si>
+    <t>Admin · Usuaris (/admin/usuaris)</t>
+  </si>
+  <si>
+    <t>ZUP-104</t>
+  </si>
+  <si>
+    <t>Llistat usuaris</t>
+  </si>
+  <si>
+    <t>ADMIN → /admin/usuaris</t>
+  </si>
+  <si>
+    <t>Graella amb email, nom, rol, dates</t>
+  </si>
+  <si>
+    <t>ZUP-105</t>
+  </si>
+  <si>
+    <t>Usuari ADMIN existent</t>
+  </si>
+  <si>
+    <t>Buscar admin@admin.adm</t>
+  </si>
+  <si>
+    <t>Present amb rol ADMIN</t>
+  </si>
+  <si>
+    <t>ZUP-106</t>
+  </si>
+  <si>
+    <t>finestra crear usuari — validació</t>
+  </si>
+  <si>
+    <t>Obrir Crear usuari amb camps buits</t>
+  </si>
+  <si>
+    <t>Botó desactivat o validació fins omplir obligatoris</t>
+  </si>
+  <si>
+    <t>ZUP-107</t>
+  </si>
+  <si>
+    <t>Crear usuari VIEWER</t>
+  </si>
+  <si>
+    <t>Omplir formulari rol VIEWER → crear</t>
+  </si>
+  <si>
+    <t>Usuari nou a la graella</t>
+  </si>
+  <si>
+    <t>ZUP-108</t>
+  </si>
+  <si>
+    <t>Crear usuari USER</t>
+  </si>
+  <si>
+    <t>Alta amb rol USER</t>
+  </si>
+  <si>
+    <t>Usuari creat correctament</t>
+  </si>
+  <si>
     <t>EN CURS</t>
-  </si>
-  <si>
-    <t>ZUP-096</t>
-  </si>
-  <si>
-    <t>Targetes de canals</t>
-  </si>
-  <si>
-    <t>Revisar graella Partnerships / Feedback / Ciutats</t>
-  </si>
-  <si>
-    <t>Targetes informatives amb text coherent</t>
-  </si>
-  <si>
-    <t>ZUP-097</t>
-  </si>
-  <si>
-    <t>Botó «Veure com funciona»</t>
-  </si>
-  <si>
-    <t>Clic enllaç</t>
-  </si>
-  <si>
-    <t>Navega a /ajuda</t>
-  </si>
-  <si>
-    <t>OK: «Veure com funciona» obre Ajuda. Copy de Contacte (provisional / .fake) anotat com a millora pendent; no s’ha canviat ara.</t>
-  </si>
-  <si>
-    <t>ZUP-098</t>
-  </si>
-  <si>
-    <t>Admin · Rols (/admin/rols)</t>
-  </si>
-  <si>
-    <t>ZUP-099</t>
-  </si>
-  <si>
-    <t>Catàleg de rols — llistat</t>
-  </si>
-  <si>
-    <t>ADMIN → /admin/rols</t>
-  </si>
-  <si>
-    <t>Títol «Catàleg de rols» i graella</t>
-  </si>
-  <si>
-    <t>ZUP-100</t>
-  </si>
-  <si>
-    <t>Alta rol nou</t>
-  </si>
-  <si>
-    <t>Crear rol amb clau única i nom visible</t>
-  </si>
-  <si>
-    <t>Rol apareix al catàleg</t>
-  </si>
-  <si>
-    <t>ZUP-101</t>
-  </si>
-  <si>
-    <t>Editar rol existent</t>
-  </si>
-  <si>
-    <t>Canviar nom visible o estat actiu</t>
-  </si>
-  <si>
-    <t>Canvis desats</t>
-  </si>
-  <si>
-    <t>ZUP-102</t>
-  </si>
-  <si>
-    <t>Baixa rol sense dependències</t>
-  </si>
-  <si>
-    <t>Esborrar rol sense usuaris assignats</t>
-  </si>
-  <si>
-    <t>Rol eliminat</t>
-  </si>
-  <si>
-    <t>ZUP-103</t>
-  </si>
-  <si>
-    <t>Baixa rol amb usuaris</t>
-  </si>
-  <si>
-    <t>Intentar esborrar rol en ús</t>
-  </si>
-  <si>
-    <t>Operació rebutjada amb missatge clar</t>
-  </si>
-  <si>
-    <t>Admin · Usuaris (/admin/usuaris)</t>
-  </si>
-  <si>
-    <t>ZUP-104</t>
-  </si>
-  <si>
-    <t>Llistat usuaris</t>
-  </si>
-  <si>
-    <t>ADMIN → /admin/usuaris</t>
-  </si>
-  <si>
-    <t>Graella amb email, nom, rol, dates</t>
-  </si>
-  <si>
-    <t>ZUP-105</t>
-  </si>
-  <si>
-    <t>Usuari ADMIN existent</t>
-  </si>
-  <si>
-    <t>Buscar admin@admin.adm</t>
-  </si>
-  <si>
-    <t>Present amb rol ADMIN</t>
-  </si>
-  <si>
-    <t>ZUP-106</t>
-  </si>
-  <si>
-    <t>finestra crear usuari — validació</t>
-  </si>
-  <si>
-    <t>Obrir Crear usuari amb camps buits</t>
-  </si>
-  <si>
-    <t>Botó desactivat o validació fins omplir obligatoris</t>
-  </si>
-  <si>
-    <t>ZUP-107</t>
-  </si>
-  <si>
-    <t>Crear usuari VIEWER</t>
-  </si>
-  <si>
-    <t>Omplir formulari rol VIEWER → crear</t>
-  </si>
-  <si>
-    <t>Usuari nou a la graella</t>
-  </si>
-  <si>
-    <t>ZUP-108</t>
-  </si>
-  <si>
-    <t>Crear usuari USER</t>
-  </si>
-  <si>
-    <t>Alta amb rol USER</t>
-  </si>
-  <si>
-    <t>Usuari creat correctament</t>
   </si>
   <si>
     <t>ZUP-109</t>
@@ -20248,9 +20256,11 @@
       <c r="H692" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="I692" s="18"/>
+      <c r="I692" s="18" t="s">
+        <v>82</v>
+      </c>
       <c r="J692" s="1" t="s">
-        <v>512</v>
+        <v>71</v>
       </c>
       <c r="K692" s="19"/>
       <c r="L692" s="18"/>
@@ -20773,16 +20783,16 @@
         <v>92</v>
       </c>
       <c r="C716" s="25" t="s">
+        <v>512</v>
+      </c>
+      <c r="D716" s="26" t="s">
         <v>513</v>
       </c>
-      <c r="D716" s="26" t="s">
+      <c r="E716" s="26" t="s">
         <v>514</v>
       </c>
-      <c r="E716" s="26" t="s">
+      <c r="F716" s="26" t="s">
         <v>515</v>
-      </c>
-      <c r="F716" s="26" t="s">
-        <v>516</v>
       </c>
       <c r="G716" s="16" t="s">
         <v>58</v>
@@ -20919,16 +20929,16 @@
         <v>92</v>
       </c>
       <c r="C722" s="14" t="s">
+        <v>516</v>
+      </c>
+      <c r="D722" s="15" t="s">
         <v>517</v>
       </c>
-      <c r="D722" s="15" t="s">
+      <c r="E722" s="15" t="s">
         <v>518</v>
       </c>
-      <c r="E722" s="15" t="s">
+      <c r="F722" s="15" t="s">
         <v>519</v>
-      </c>
-      <c r="F722" s="15" t="s">
-        <v>520</v>
       </c>
       <c r="G722" s="16" t="s">
         <v>58</v>
@@ -20943,7 +20953,7 @@
         <v>71</v>
       </c>
       <c r="K722" s="19" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="L722" s="18"/>
       <c r="M722" s="1"/>
@@ -21067,13 +21077,13 @@
         <v>92</v>
       </c>
       <c r="C728" s="25" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="D728" s="26" t="s">
         <v>219</v>
       </c>
       <c r="E728" s="26" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="F728" s="26" t="s">
         <v>221</v>
@@ -21207,22 +21217,22 @@
     </row>
     <row r="734" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A734" s="43" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="B734" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C734" s="14" t="s">
+        <v>523</v>
+      </c>
+      <c r="D734" s="15" t="s">
         <v>524</v>
       </c>
-      <c r="D734" s="15" t="s">
+      <c r="E734" s="15" t="s">
         <v>525</v>
       </c>
-      <c r="E734" s="15" t="s">
+      <c r="F734" s="15" t="s">
         <v>526</v>
-      </c>
-      <c r="F734" s="15" t="s">
-        <v>527</v>
       </c>
       <c r="G734" s="16" t="s">
         <v>58</v>
@@ -21230,9 +21240,11 @@
       <c r="H734" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="I734" s="18"/>
+      <c r="I734" s="18" t="s">
+        <v>82</v>
+      </c>
       <c r="J734" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K734" s="19"/>
       <c r="L734" s="18"/>
@@ -21351,22 +21363,22 @@
     </row>
     <row r="740" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A740" s="43" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="B740" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C740" s="25" t="s">
+        <v>527</v>
+      </c>
+      <c r="D740" s="26" t="s">
         <v>528</v>
       </c>
-      <c r="D740" s="26" t="s">
+      <c r="E740" s="26" t="s">
         <v>529</v>
       </c>
-      <c r="E740" s="26" t="s">
+      <c r="F740" s="26" t="s">
         <v>530</v>
-      </c>
-      <c r="F740" s="26" t="s">
-        <v>531</v>
       </c>
       <c r="G740" s="16" t="s">
         <v>58</v>
@@ -21374,14 +21386,24 @@
       <c r="H740" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="I740" s="18"/>
+      <c r="I740" s="18" t="s">
+        <v>82</v>
+      </c>
       <c r="J740" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="K740" s="19"/>
-      <c r="L740" s="18"/>
-      <c r="M740" s="1"/>
-      <c r="N740" s="19"/>
+        <v>83</v>
+      </c>
+      <c r="K740" s="19" t="s">
+        <v>531</v>
+      </c>
+      <c r="L740" s="18" t="s">
+        <v>82</v>
+      </c>
+      <c r="M740" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="N740" s="19" t="s">
+        <v>532</v>
+      </c>
     </row>
     <row r="741" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A741" s="43"/>
@@ -21495,22 +21517,22 @@
     </row>
     <row r="746" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A746" s="43" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="B746" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C746" s="14" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="D746" s="15" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="E746" s="15" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="F746" s="15" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="G746" s="16" t="s">
         <v>58</v>
@@ -21518,9 +21540,11 @@
       <c r="H746" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="I746" s="18"/>
+      <c r="I746" s="18" t="s">
+        <v>82</v>
+      </c>
       <c r="J746" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K746" s="19"/>
       <c r="L746" s="18"/>
@@ -21639,22 +21663,22 @@
     </row>
     <row r="752" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A752" s="43" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="B752" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C752" s="25" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="D752" s="26" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="E752" s="26" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="F752" s="26" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="G752" s="16" t="s">
         <v>58</v>
@@ -21662,9 +21686,11 @@
       <c r="H752" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="I752" s="18"/>
+      <c r="I752" s="18" t="s">
+        <v>82</v>
+      </c>
       <c r="J752" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K752" s="19"/>
       <c r="L752" s="18"/>
@@ -21783,22 +21809,22 @@
     </row>
     <row r="758" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A758" s="43" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="B758" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C758" s="14" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="D758" s="15" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="E758" s="15" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="F758" s="15" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="G758" s="16" t="s">
         <v>58</v>
@@ -21806,9 +21832,11 @@
       <c r="H758" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="I758" s="18"/>
+      <c r="I758" s="18" t="s">
+        <v>82</v>
+      </c>
       <c r="J758" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K758" s="19"/>
       <c r="L758" s="18"/>
@@ -21927,22 +21955,22 @@
     </row>
     <row r="764" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A764" s="44" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="B764" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C764" s="25" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="D764" s="26" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="E764" s="26" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="F764" s="26" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="G764" s="16" t="s">
         <v>58</v>
@@ -21950,9 +21978,11 @@
       <c r="H764" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="I764" s="18"/>
+      <c r="I764" s="18" t="s">
+        <v>82</v>
+      </c>
       <c r="J764" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K764" s="19"/>
       <c r="L764" s="18"/>
@@ -22071,22 +22101,22 @@
     </row>
     <row r="770" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A770" s="44" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="B770" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C770" s="14" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="D770" s="15" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="E770" s="15" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="F770" s="15" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="G770" s="16" t="s">
         <v>58</v>
@@ -22094,9 +22124,11 @@
       <c r="H770" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="I770" s="18"/>
+      <c r="I770" s="18" t="s">
+        <v>82</v>
+      </c>
       <c r="J770" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K770" s="19"/>
       <c r="L770" s="18"/>
@@ -22215,22 +22247,22 @@
     </row>
     <row r="776" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A776" s="44" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="B776" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C776" s="25" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="D776" s="26" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="E776" s="26" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="F776" s="26" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="G776" s="16" t="s">
         <v>58</v>
@@ -22238,9 +22270,11 @@
       <c r="H776" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="I776" s="18"/>
+      <c r="I776" s="18" t="s">
+        <v>82</v>
+      </c>
       <c r="J776" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K776" s="19"/>
       <c r="L776" s="18"/>
@@ -22359,22 +22393,22 @@
     </row>
     <row r="782" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A782" s="44" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="B782" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C782" s="14" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="D782" s="15" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="E782" s="15" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="F782" s="15" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="G782" s="16" t="s">
         <v>58</v>
@@ -22503,22 +22537,22 @@
     </row>
     <row r="788" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A788" s="44" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="B788" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C788" s="25" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="D788" s="26" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="E788" s="26" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="F788" s="26" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="G788" s="16" t="s">
         <v>58</v>
@@ -22528,7 +22562,7 @@
       </c>
       <c r="I788" s="18"/>
       <c r="J788" s="1" t="s">
-        <v>60</v>
+        <v>566</v>
       </c>
       <c r="K788" s="19"/>
       <c r="L788" s="18"/>
@@ -22647,22 +22681,22 @@
     </row>
     <row r="794" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A794" s="44" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="B794" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C794" s="14" t="s">
+        <v>567</v>
+      </c>
+      <c r="D794" s="15" t="s">
+        <v>568</v>
+      </c>
+      <c r="E794" s="15" t="s">
+        <v>569</v>
+      </c>
+      <c r="F794" s="15" t="s">
         <v>565</v>
-      </c>
-      <c r="D794" s="15" t="s">
-        <v>566</v>
-      </c>
-      <c r="E794" s="15" t="s">
-        <v>567</v>
-      </c>
-      <c r="F794" s="15" t="s">
-        <v>564</v>
       </c>
       <c r="G794" s="16" t="s">
         <v>58</v>
@@ -22791,22 +22825,22 @@
     </row>
     <row r="800" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A800" s="44" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="B800" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C800" s="25" t="s">
-        <v>568</v>
+        <v>570</v>
       </c>
       <c r="D800" s="26" t="s">
-        <v>569</v>
+        <v>571</v>
       </c>
       <c r="E800" s="26" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
       <c r="F800" s="26" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
       <c r="G800" s="16" t="s">
         <v>58</v>
@@ -22935,22 +22969,22 @@
     </row>
     <row r="806" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A806" s="44" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="B806" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C806" s="14" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
       <c r="D806" s="15" t="s">
-        <v>573</v>
+        <v>575</v>
       </c>
       <c r="E806" s="15" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="F806" s="15" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="G806" s="16" t="s">
         <v>58</v>
@@ -23079,22 +23113,22 @@
     </row>
     <row r="812" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A812" s="44" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="B812" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C812" s="25" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="D812" s="26" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="E812" s="26" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="F812" s="26" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="G812" s="16" t="s">
         <v>58</v>
@@ -23223,22 +23257,22 @@
     </row>
     <row r="818" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A818" s="44" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="B818" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C818" s="14" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="D818" s="15" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="E818" s="15" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="F818" s="15" t="s">
-        <v>583</v>
+        <v>585</v>
       </c>
       <c r="G818" s="16" t="s">
         <v>58</v>
@@ -23367,22 +23401,22 @@
     </row>
     <row r="824" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A824" s="44" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="B824" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C824" s="25" t="s">
-        <v>584</v>
+        <v>586</v>
       </c>
       <c r="D824" s="26" t="s">
-        <v>585</v>
+        <v>587</v>
       </c>
       <c r="E824" s="26" t="s">
-        <v>586</v>
+        <v>588</v>
       </c>
       <c r="F824" s="26" t="s">
-        <v>587</v>
+        <v>589</v>
       </c>
       <c r="G824" s="16" t="s">
         <v>58</v>
@@ -23511,22 +23545,22 @@
     </row>
     <row r="830" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A830" s="44" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="B830" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C830" s="14" t="s">
-        <v>588</v>
+        <v>590</v>
       </c>
       <c r="D830" s="15" t="s">
-        <v>589</v>
+        <v>591</v>
       </c>
       <c r="E830" s="15" t="s">
-        <v>590</v>
+        <v>592</v>
       </c>
       <c r="F830" s="15" t="s">
-        <v>591</v>
+        <v>593</v>
       </c>
       <c r="G830" s="16" t="s">
         <v>58</v>
@@ -23655,22 +23689,22 @@
     </row>
     <row r="836" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A836" s="45" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
       <c r="B836" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C836" s="25" t="s">
-        <v>593</v>
+        <v>595</v>
       </c>
       <c r="D836" s="26" t="s">
-        <v>594</v>
+        <v>596</v>
       </c>
       <c r="E836" s="26" t="s">
-        <v>595</v>
+        <v>597</v>
       </c>
       <c r="F836" s="26" t="s">
-        <v>596</v>
+        <v>598</v>
       </c>
       <c r="G836" s="16" t="s">
         <v>58</v>
@@ -23799,22 +23833,22 @@
     </row>
     <row r="842" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A842" s="45" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
       <c r="B842" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C842" s="14" t="s">
-        <v>597</v>
+        <v>599</v>
       </c>
       <c r="D842" s="15" t="s">
-        <v>598</v>
+        <v>600</v>
       </c>
       <c r="E842" s="15" t="s">
-        <v>599</v>
+        <v>601</v>
       </c>
       <c r="F842" s="15" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="G842" s="16" t="s">
         <v>58</v>
@@ -23943,22 +23977,22 @@
     </row>
     <row r="848" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A848" s="45" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
       <c r="B848" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C848" s="25" t="s">
-        <v>600</v>
+        <v>602</v>
       </c>
       <c r="D848" s="26" t="s">
-        <v>601</v>
+        <v>603</v>
       </c>
       <c r="E848" s="26" t="s">
-        <v>602</v>
+        <v>604</v>
       </c>
       <c r="F848" s="26" t="s">
-        <v>603</v>
+        <v>605</v>
       </c>
       <c r="G848" s="16" t="s">
         <v>58</v>
@@ -24087,22 +24121,22 @@
     </row>
     <row r="854" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A854" s="45" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
       <c r="B854" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C854" s="14" t="s">
-        <v>604</v>
+        <v>606</v>
       </c>
       <c r="D854" s="15" t="s">
-        <v>605</v>
+        <v>607</v>
       </c>
       <c r="E854" s="15" t="s">
-        <v>606</v>
+        <v>608</v>
       </c>
       <c r="F854" s="15" t="s">
-        <v>607</v>
+        <v>609</v>
       </c>
       <c r="G854" s="16" t="s">
         <v>58</v>
@@ -24231,22 +24265,22 @@
     </row>
     <row r="860" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A860" s="46" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
       <c r="B860" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C860" s="25" t="s">
-        <v>609</v>
+        <v>611</v>
       </c>
       <c r="D860" s="26" t="s">
-        <v>610</v>
+        <v>612</v>
       </c>
       <c r="E860" s="26" t="s">
-        <v>611</v>
+        <v>613</v>
       </c>
       <c r="F860" s="26" t="s">
-        <v>612</v>
+        <v>614</v>
       </c>
       <c r="G860" s="16" t="s">
         <v>58</v>
@@ -24375,22 +24409,22 @@
     </row>
     <row r="866" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A866" s="46" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
       <c r="B866" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C866" s="14" t="s">
-        <v>613</v>
+        <v>615</v>
       </c>
       <c r="D866" s="15" t="s">
-        <v>614</v>
+        <v>616</v>
       </c>
       <c r="E866" s="15" t="s">
-        <v>615</v>
+        <v>617</v>
       </c>
       <c r="F866" s="15" t="s">
-        <v>616</v>
+        <v>618</v>
       </c>
       <c r="G866" s="16" t="s">
         <v>58</v>
@@ -24519,22 +24553,22 @@
     </row>
     <row r="872" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A872" s="46" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
       <c r="B872" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C872" s="25" t="s">
-        <v>617</v>
+        <v>619</v>
       </c>
       <c r="D872" s="26" t="s">
-        <v>618</v>
+        <v>620</v>
       </c>
       <c r="E872" s="26" t="s">
-        <v>619</v>
+        <v>621</v>
       </c>
       <c r="F872" s="26" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="G872" s="16" t="s">
         <v>58</v>
@@ -24663,22 +24697,22 @@
     </row>
     <row r="878" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A878" s="46" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
       <c r="B878" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C878" s="14" t="s">
-        <v>621</v>
+        <v>623</v>
       </c>
       <c r="D878" s="15" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
       <c r="E878" s="15" t="s">
-        <v>623</v>
+        <v>625</v>
       </c>
       <c r="F878" s="15" t="s">
-        <v>624</v>
+        <v>626</v>
       </c>
       <c r="G878" s="16" t="s">
         <v>58</v>
@@ -24807,22 +24841,22 @@
     </row>
     <row r="884" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A884" s="46" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
       <c r="B884" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C884" s="25" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
       <c r="D884" s="26" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
       <c r="E884" s="26" t="s">
-        <v>627</v>
+        <v>629</v>
       </c>
       <c r="F884" s="26" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
       <c r="G884" s="16" t="s">
         <v>58</v>
@@ -24951,22 +24985,22 @@
     </row>
     <row r="890" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A890" s="46" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
       <c r="B890" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C890" s="14" t="s">
-        <v>629</v>
+        <v>631</v>
       </c>
       <c r="D890" s="15" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
       <c r="E890" s="15" t="s">
-        <v>631</v>
+        <v>633</v>
       </c>
       <c r="F890" s="15" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
       <c r="G890" s="16" t="s">
         <v>58</v>
@@ -25095,22 +25129,22 @@
     </row>
     <row r="896" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A896" s="46" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
       <c r="B896" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C896" s="25" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="D896" s="26" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
       <c r="E896" s="26" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="F896" s="26" t="s">
-        <v>636</v>
+        <v>638</v>
       </c>
       <c r="G896" s="16" t="s">
         <v>58</v>
@@ -25239,22 +25273,22 @@
     </row>
     <row r="902" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A902" s="47" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="B902" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C902" s="14" t="s">
-        <v>638</v>
+        <v>640</v>
       </c>
       <c r="D902" s="15" t="s">
-        <v>639</v>
+        <v>641</v>
       </c>
       <c r="E902" s="15" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
       <c r="F902" s="15" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
       <c r="G902" s="16" t="s">
         <v>58</v>
@@ -25383,22 +25417,22 @@
     </row>
     <row r="908" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A908" s="47" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="B908" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C908" s="25" t="s">
-        <v>642</v>
+        <v>644</v>
       </c>
       <c r="D908" s="26" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
       <c r="E908" s="26" t="s">
-        <v>644</v>
+        <v>646</v>
       </c>
       <c r="F908" s="26" t="s">
-        <v>645</v>
+        <v>647</v>
       </c>
       <c r="G908" s="16" t="s">
         <v>58</v>
@@ -25527,22 +25561,22 @@
     </row>
     <row r="914" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A914" s="47" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="B914" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C914" s="14" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
       <c r="D914" s="15" t="s">
-        <v>647</v>
+        <v>649</v>
       </c>
       <c r="E914" s="15" t="s">
-        <v>648</v>
+        <v>650</v>
       </c>
       <c r="F914" s="15" t="s">
-        <v>649</v>
+        <v>651</v>
       </c>
       <c r="G914" s="16" t="s">
         <v>58</v>
@@ -25671,22 +25705,22 @@
     </row>
     <row r="920" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A920" s="47" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="B920" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C920" s="25" t="s">
-        <v>650</v>
+        <v>652</v>
       </c>
       <c r="D920" s="26" t="s">
-        <v>651</v>
+        <v>653</v>
       </c>
       <c r="E920" s="26" t="s">
-        <v>652</v>
+        <v>654</v>
       </c>
       <c r="F920" s="26" t="s">
-        <v>653</v>
+        <v>655</v>
       </c>
       <c r="G920" s="16" t="s">
         <v>58</v>
@@ -25815,22 +25849,22 @@
     </row>
     <row r="926" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A926" s="47" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="B926" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C926" s="14" t="s">
-        <v>654</v>
+        <v>656</v>
       </c>
       <c r="D926" s="15" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
       <c r="E926" s="15" t="s">
-        <v>656</v>
+        <v>658</v>
       </c>
       <c r="F926" s="15" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
       <c r="G926" s="16" t="s">
         <v>58</v>
@@ -25959,22 +25993,22 @@
     </row>
     <row r="932" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A932" s="47" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="B932" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C932" s="25" t="s">
-        <v>658</v>
+        <v>660</v>
       </c>
       <c r="D932" s="26" t="s">
-        <v>659</v>
+        <v>661</v>
       </c>
       <c r="E932" s="26" t="s">
-        <v>660</v>
+        <v>662</v>
       </c>
       <c r="F932" s="26" t="s">
-        <v>661</v>
+        <v>663</v>
       </c>
       <c r="G932" s="16" t="s">
         <v>58</v>
@@ -26103,22 +26137,22 @@
     </row>
     <row r="938" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A938" s="48" t="s">
-        <v>662</v>
+        <v>664</v>
       </c>
       <c r="B938" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C938" s="14" t="s">
-        <v>663</v>
+        <v>665</v>
       </c>
       <c r="D938" s="15" t="s">
-        <v>664</v>
+        <v>666</v>
       </c>
       <c r="E938" s="15" t="s">
-        <v>665</v>
+        <v>667</v>
       </c>
       <c r="F938" s="15" t="s">
-        <v>666</v>
+        <v>668</v>
       </c>
       <c r="G938" s="16" t="s">
         <v>58</v>
@@ -26247,22 +26281,22 @@
     </row>
     <row r="944" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A944" s="48" t="s">
-        <v>662</v>
+        <v>664</v>
       </c>
       <c r="B944" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C944" s="25" t="s">
-        <v>667</v>
+        <v>669</v>
       </c>
       <c r="D944" s="26" t="s">
-        <v>668</v>
+        <v>670</v>
       </c>
       <c r="E944" s="26" t="s">
-        <v>669</v>
+        <v>671</v>
       </c>
       <c r="F944" s="26" t="s">
-        <v>670</v>
+        <v>672</v>
       </c>
       <c r="G944" s="16" t="s">
         <v>58</v>
@@ -26391,22 +26425,22 @@
     </row>
     <row r="950" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A950" s="48" t="s">
-        <v>662</v>
+        <v>664</v>
       </c>
       <c r="B950" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C950" s="14" t="s">
-        <v>671</v>
+        <v>673</v>
       </c>
       <c r="D950" s="15" t="s">
-        <v>672</v>
+        <v>674</v>
       </c>
       <c r="E950" s="15" t="s">
-        <v>673</v>
+        <v>675</v>
       </c>
       <c r="F950" s="15" t="s">
-        <v>674</v>
+        <v>676</v>
       </c>
       <c r="G950" s="16" t="s">
         <v>58</v>
@@ -26535,22 +26569,22 @@
     </row>
     <row r="956" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A956" s="48" t="s">
-        <v>662</v>
+        <v>664</v>
       </c>
       <c r="B956" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C956" s="25" t="s">
-        <v>675</v>
+        <v>677</v>
       </c>
       <c r="D956" s="26" t="s">
-        <v>676</v>
+        <v>678</v>
       </c>
       <c r="E956" s="26" t="s">
-        <v>677</v>
+        <v>679</v>
       </c>
       <c r="F956" s="26" t="s">
-        <v>649</v>
+        <v>651</v>
       </c>
       <c r="G956" s="16" t="s">
         <v>58</v>
@@ -26679,22 +26713,22 @@
     </row>
     <row r="962" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A962" s="48" t="s">
-        <v>662</v>
+        <v>664</v>
       </c>
       <c r="B962" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C962" s="14" t="s">
-        <v>678</v>
+        <v>680</v>
       </c>
       <c r="D962" s="15" t="s">
-        <v>679</v>
+        <v>681</v>
       </c>
       <c r="E962" s="15" t="s">
-        <v>680</v>
+        <v>682</v>
       </c>
       <c r="F962" s="15" t="s">
-        <v>681</v>
+        <v>683</v>
       </c>
       <c r="G962" s="16" t="s">
         <v>58</v>
@@ -26823,22 +26857,22 @@
     </row>
     <row r="968" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A968" s="48" t="s">
-        <v>662</v>
+        <v>664</v>
       </c>
       <c r="B968" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C968" s="25" t="s">
-        <v>682</v>
+        <v>684</v>
       </c>
       <c r="D968" s="26" t="s">
-        <v>683</v>
+        <v>685</v>
       </c>
       <c r="E968" s="26" t="s">
-        <v>684</v>
+        <v>686</v>
       </c>
       <c r="F968" s="26" t="s">
-        <v>685</v>
+        <v>687</v>
       </c>
       <c r="G968" s="16" t="s">
         <v>58</v>
@@ -26967,22 +27001,22 @@
     </row>
     <row r="974" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A974" s="49" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
       <c r="B974" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C974" s="14" t="s">
-        <v>687</v>
+        <v>689</v>
       </c>
       <c r="D974" s="15" t="s">
-        <v>688</v>
+        <v>690</v>
       </c>
       <c r="E974" s="15" t="s">
-        <v>689</v>
+        <v>691</v>
       </c>
       <c r="F974" s="15" t="s">
-        <v>690</v>
+        <v>692</v>
       </c>
       <c r="G974" s="16" t="s">
         <v>58</v>
@@ -27111,22 +27145,22 @@
     </row>
     <row r="980" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A980" s="49" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
       <c r="B980" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C980" s="25" t="s">
-        <v>691</v>
+        <v>693</v>
       </c>
       <c r="D980" s="26" t="s">
-        <v>692</v>
+        <v>694</v>
       </c>
       <c r="E980" s="26" t="s">
-        <v>693</v>
+        <v>695</v>
       </c>
       <c r="F980" s="26" t="s">
-        <v>694</v>
+        <v>696</v>
       </c>
       <c r="G980" s="16" t="s">
         <v>58</v>
@@ -27255,22 +27289,22 @@
     </row>
     <row r="986" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A986" s="49" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
       <c r="B986" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C986" s="14" t="s">
-        <v>695</v>
+        <v>697</v>
       </c>
       <c r="D986" s="15" t="s">
-        <v>696</v>
+        <v>698</v>
       </c>
       <c r="E986" s="15" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
       <c r="F986" s="15" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
       <c r="G986" s="16" t="s">
         <v>58</v>
@@ -27399,22 +27433,22 @@
     </row>
     <row r="992" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A992" s="49" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
       <c r="B992" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C992" s="25" t="s">
-        <v>699</v>
+        <v>701</v>
       </c>
       <c r="D992" s="26" t="s">
-        <v>700</v>
+        <v>702</v>
       </c>
       <c r="E992" s="26" t="s">
-        <v>701</v>
+        <v>703</v>
       </c>
       <c r="F992" s="26" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="G992" s="16" t="s">
         <v>58</v>
@@ -27543,22 +27577,22 @@
     </row>
     <row r="998" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A998" s="49" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
       <c r="B998" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C998" s="14" t="s">
-        <v>703</v>
+        <v>705</v>
       </c>
       <c r="D998" s="15" t="s">
-        <v>704</v>
+        <v>706</v>
       </c>
       <c r="E998" s="15" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
       <c r="F998" s="15" t="s">
-        <v>706</v>
+        <v>708</v>
       </c>
       <c r="G998" s="16" t="s">
         <v>58</v>
@@ -27687,22 +27721,22 @@
     </row>
     <row r="1004" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1004" s="50" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
       <c r="B1004" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1004" s="25" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="D1004" s="26" t="s">
-        <v>709</v>
+        <v>711</v>
       </c>
       <c r="E1004" s="26" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="F1004" s="26" t="s">
-        <v>711</v>
+        <v>713</v>
       </c>
       <c r="G1004" s="16" t="s">
         <v>58</v>
@@ -27831,22 +27865,22 @@
     </row>
     <row r="1010" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1010" s="50" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
       <c r="B1010" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1010" s="14" t="s">
-        <v>712</v>
+        <v>714</v>
       </c>
       <c r="D1010" s="15" t="s">
-        <v>713</v>
+        <v>715</v>
       </c>
       <c r="E1010" s="15" t="s">
-        <v>714</v>
+        <v>716</v>
       </c>
       <c r="F1010" s="15" t="s">
-        <v>715</v>
+        <v>717</v>
       </c>
       <c r="G1010" s="16" t="s">
         <v>58</v>
@@ -27975,22 +28009,22 @@
     </row>
     <row r="1016" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1016" s="50" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
       <c r="B1016" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1016" s="25" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
       <c r="D1016" s="26" t="s">
-        <v>717</v>
+        <v>719</v>
       </c>
       <c r="E1016" s="26" t="s">
-        <v>718</v>
+        <v>720</v>
       </c>
       <c r="F1016" s="26" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
       <c r="G1016" s="16" t="s">
         <v>58</v>
@@ -28119,22 +28153,22 @@
     </row>
     <row r="1022" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1022" s="50" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
       <c r="B1022" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1022" s="14" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
       <c r="D1022" s="15" t="s">
-        <v>721</v>
+        <v>723</v>
       </c>
       <c r="E1022" s="15" t="s">
-        <v>722</v>
+        <v>724</v>
       </c>
       <c r="F1022" s="15" t="s">
-        <v>723</v>
+        <v>725</v>
       </c>
       <c r="G1022" s="16" t="s">
         <v>58</v>
@@ -28263,22 +28297,22 @@
     </row>
     <row r="1028" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1028" s="50" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
       <c r="B1028" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C1028" s="25" t="s">
-        <v>724</v>
+        <v>726</v>
       </c>
       <c r="D1028" s="26" t="s">
-        <v>725</v>
+        <v>727</v>
       </c>
       <c r="E1028" s="26" t="s">
-        <v>726</v>
+        <v>728</v>
       </c>
       <c r="F1028" s="26" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
       <c r="G1028" s="16" t="s">
         <v>58</v>
@@ -28407,22 +28441,22 @@
     </row>
     <row r="1034" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1034" s="50" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
       <c r="B1034" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C1034" s="14" t="s">
-        <v>728</v>
+        <v>730</v>
       </c>
       <c r="D1034" s="15" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
       <c r="E1034" s="15" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="F1034" s="15" t="s">
-        <v>731</v>
+        <v>733</v>
       </c>
       <c r="G1034" s="16" t="s">
         <v>58</v>
@@ -28551,22 +28585,22 @@
     </row>
     <row r="1040" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1040" s="51" t="s">
-        <v>732</v>
+        <v>734</v>
       </c>
       <c r="B1040" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C1040" s="25" t="s">
-        <v>733</v>
+        <v>735</v>
       </c>
       <c r="D1040" s="26" t="s">
-        <v>721</v>
+        <v>723</v>
       </c>
       <c r="E1040" s="26" t="s">
-        <v>734</v>
+        <v>736</v>
       </c>
       <c r="F1040" s="26" t="s">
-        <v>735</v>
+        <v>737</v>
       </c>
       <c r="G1040" s="16" t="s">
         <v>58</v>
@@ -28695,22 +28729,22 @@
     </row>
     <row r="1046" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1046" s="51" t="s">
-        <v>732</v>
+        <v>734</v>
       </c>
       <c r="B1046" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1046" s="14" t="s">
-        <v>736</v>
+        <v>738</v>
       </c>
       <c r="D1046" s="15" t="s">
-        <v>713</v>
+        <v>715</v>
       </c>
       <c r="E1046" s="15" t="s">
-        <v>737</v>
+        <v>739</v>
       </c>
       <c r="F1046" s="15" t="s">
-        <v>738</v>
+        <v>740</v>
       </c>
       <c r="G1046" s="16" t="s">
         <v>58</v>
@@ -28847,16 +28881,16 @@
         <v>53</v>
       </c>
       <c r="C1052" s="25" t="s">
-        <v>739</v>
+        <v>741</v>
       </c>
       <c r="D1052" s="26" t="s">
-        <v>740</v>
+        <v>742</v>
       </c>
       <c r="E1052" s="26" t="s">
-        <v>741</v>
+        <v>743</v>
       </c>
       <c r="F1052" s="26" t="s">
-        <v>742</v>
+        <v>744</v>
       </c>
       <c r="G1052" s="16" t="s">
         <v>58</v>
@@ -28993,16 +29027,16 @@
         <v>53</v>
       </c>
       <c r="C1058" s="14" t="s">
-        <v>743</v>
+        <v>745</v>
       </c>
       <c r="D1058" s="15" t="s">
-        <v>744</v>
+        <v>746</v>
       </c>
       <c r="E1058" s="15" t="s">
-        <v>745</v>
+        <v>747</v>
       </c>
       <c r="F1058" s="15" t="s">
-        <v>746</v>
+        <v>748</v>
       </c>
       <c r="G1058" s="16" t="s">
         <v>58</v>
@@ -30088,10 +30122,10 @@
         <v>39</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>747</v>
+        <v>749</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>748</v>
+        <v>750</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>53</v>
@@ -30109,7 +30143,7 @@
         <v>83</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>749</v>
+        <v>751</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -30462,7 +30496,7 @@
     </row>
     <row r="14" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="64" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="B14" s="1">
         <v>5</v>
@@ -30491,7 +30525,7 @@
     </row>
     <row r="15" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="65" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="B15" s="1">
         <v>12</v>
@@ -30520,7 +30554,7 @@
     </row>
     <row r="16" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="66" t="s">
-        <v>592</v>
+        <v>594</v>
       </c>
       <c r="B16" s="1">
         <v>4</v>
@@ -30549,7 +30583,7 @@
     </row>
     <row r="17" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="67" t="s">
-        <v>608</v>
+        <v>610</v>
       </c>
       <c r="B17" s="1">
         <v>7</v>
@@ -30578,7 +30612,7 @@
     </row>
     <row r="18" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="68" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="B18" s="1">
         <v>6</v>
@@ -30607,7 +30641,7 @@
     </row>
     <row r="19" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="69" t="s">
-        <v>662</v>
+        <v>664</v>
       </c>
       <c r="B19" s="1">
         <v>6</v>
@@ -30636,7 +30670,7 @@
     </row>
     <row r="20" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="70" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
       <c r="B20" s="1">
         <v>5</v>
@@ -30665,7 +30699,7 @@
     </row>
     <row r="21" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="71" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
       <c r="B21" s="1">
         <v>6</v>
@@ -30694,7 +30728,7 @@
     </row>
     <row r="22" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="72" t="s">
-        <v>732</v>
+        <v>734</v>
       </c>
       <c r="B22" s="1">
         <v>2</v>
@@ -30723,7 +30757,7 @@
     </row>
     <row r="23" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="73" t="s">
-        <v>750</v>
+        <v>752</v>
       </c>
       <c r="B23" s="73">
         <v>153</v>
@@ -30774,7 +30808,7 @@
         <v>44</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>748</v>
+        <v>750</v>
       </c>
       <c r="C1" s="10" t="s">
         <v>71</v>
@@ -30783,7 +30817,7 @@
         <v>83</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>749</v>
+        <v>751</v>
       </c>
       <c r="F1" s="10" t="s">
         <v>97</v>
@@ -30934,10 +30968,10 @@
         <v>45</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>751</v>
+        <v>753</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>748</v>
+        <v>750</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>71</v>
@@ -30946,7 +30980,7 @@
         <v>83</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>749</v>
+        <v>751</v>
       </c>
       <c r="G1" s="10" t="s">
         <v>97</v>
@@ -30957,7 +30991,7 @@
         <v>59</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>752</v>
+        <v>754</v>
       </c>
       <c r="C2" s="1">
         <f>COUNTIF(Proves!$H:$H,A2)</f>
@@ -31087,7 +31121,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="83" t="s">
-        <v>753</v>
+        <v>755</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -31095,7 +31129,7 @@
         <v>71</v>
       </c>
       <c r="B2" s="84" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
@@ -31115,7 +31149,7 @@
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>512</v>
+        <v>566</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
098 => fase IV => edició admin (PUT users/{id}, sense 403 ni check de privacitat), capçalera per rol, Bio→Comentaris (users.comments), ZUP-114 OK i ZUP-112 KO/corr (Chrome/ADMIN)
</commit_message>
<xml_diff>
--- a/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
+++ b/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4425" uniqueCount="757">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4434" uniqueCount="761">
   <si>
     <t>Zuppeto — Joc de probes manual (totes les pantalles)</t>
   </si>
@@ -1802,103 +1802,121 @@
     <t>Usuari creat correctament</t>
   </si>
   <si>
+    <t>04-09-2026</t>
+  </si>
+  <si>
+    <t>ZUP-109</t>
+  </si>
+  <si>
+    <t>Crear usuari DEVELOPER</t>
+  </si>
+  <si>
+    <t>Alta amb rol DEVELOPER</t>
+  </si>
+  <si>
+    <t>ZUP-110</t>
+  </si>
+  <si>
+    <t>Email duplicat</t>
+  </si>
+  <si>
+    <t>Intentar crear email ja existent</t>
+  </si>
+  <si>
+    <t>Error de conflicte informatiu</t>
+  </si>
+  <si>
+    <t>ZUP-111</t>
+  </si>
+  <si>
+    <t>Veure detall usuari</t>
+  </si>
+  <si>
+    <t>Clic fila o icona ull</t>
+  </si>
+  <si>
+    <t>Panell o finestra de detall amb dades editables</t>
+  </si>
+  <si>
+    <t>ZUP-112</t>
+  </si>
+  <si>
+    <t>Canvi de rol</t>
+  </si>
+  <si>
+    <t>Editar rol d'un usuari i desar</t>
+  </si>
+  <si>
+    <t>Canvi persistit després de refrescar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Desar desactivat pel check de privacitat tot i ser Administrador.
+En desar sortien dos errors «Accés denegat»: el canvi de fitxa anava a l’API del perfil propi, que no deixa editar un altre usuari.
+La bio tenia un mínim de 12 caràcters que no correspon (només no pot ser buida).</t>
+  </si>
+  <si>
+    <t>06-09-2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Què s’ha fet: si qui opera és Administrador, no es mostra ni es valida el check de condicions (policy AdminExemptPrivacyConsentPolicy, com al perfil).
+El desar de fitxa va a PUT /api/admin/users/{id} (UpdateAdminUserCommand + User.ReplaceProfile), no al perfil propi.
+La bio és obligatòria i sense mínim de longitud.
+En desar el rol, el menú/aspecte segueix el rol: Admin → intern, User → públic i Inici, TEST → sense menú intern (RoleChromePolicy).
+El camp visible «Bio» passa a «Comentaris»; a BD la columna users.bio es reanomena a users.comments.</t>
+  </si>
+  <si>
+    <t>ZUP-113</t>
+  </si>
+  <si>
+    <t>Avatar en alta usuari</t>
+  </si>
+  <si>
+    <t>Pujar imatge al crear usuari</t>
+  </si>
+  <si>
+    <t>Avatar desat i visible al detall</t>
+  </si>
+  <si>
+    <t>ZUP-114</t>
+  </si>
+  <si>
+    <t>Esborrar usuari</t>
+  </si>
+  <si>
+    <t>Icona esborrar → confirmar</t>
+  </si>
+  <si>
+    <t>Usuari eliminat de la graella</t>
+  </si>
+  <si>
+    <t>ZUP-115</t>
+  </si>
+  <si>
+    <t>DEVELOPER no accedeix</t>
+  </si>
+  <si>
+    <t>DEVELOPER → /admin/usuaris</t>
+  </si>
+  <si>
+    <t>Redirecció a home</t>
+  </si>
+  <si>
+    <t>Admin · Permisos (/admin/permisos)</t>
+  </si>
+  <si>
+    <t>ZUP-116</t>
+  </si>
+  <si>
+    <t>Pantalla permisos per rol</t>
+  </si>
+  <si>
+    <t>ADMIN → /admin/permisos</t>
+  </si>
+  <si>
+    <t>Matriu o llistat permisos per rol</t>
+  </si>
+  <si>
     <t>EN CURS</t>
-  </si>
-  <si>
-    <t>ZUP-109</t>
-  </si>
-  <si>
-    <t>Crear usuari DEVELOPER</t>
-  </si>
-  <si>
-    <t>Alta amb rol DEVELOPER</t>
-  </si>
-  <si>
-    <t>ZUP-110</t>
-  </si>
-  <si>
-    <t>Email duplicat</t>
-  </si>
-  <si>
-    <t>Intentar crear email ja existent</t>
-  </si>
-  <si>
-    <t>Error de conflicte informatiu</t>
-  </si>
-  <si>
-    <t>ZUP-111</t>
-  </si>
-  <si>
-    <t>Veure detall usuari</t>
-  </si>
-  <si>
-    <t>Clic fila o icona ull</t>
-  </si>
-  <si>
-    <t>Panell o finestra de detall amb dades editables</t>
-  </si>
-  <si>
-    <t>ZUP-112</t>
-  </si>
-  <si>
-    <t>Canvi de rol</t>
-  </si>
-  <si>
-    <t>Editar rol d'un usuari i desar</t>
-  </si>
-  <si>
-    <t>Canvi persistit després de refrescar</t>
-  </si>
-  <si>
-    <t>ZUP-113</t>
-  </si>
-  <si>
-    <t>Avatar en alta usuari</t>
-  </si>
-  <si>
-    <t>Pujar imatge al crear usuari</t>
-  </si>
-  <si>
-    <t>Avatar desat i visible al detall</t>
-  </si>
-  <si>
-    <t>ZUP-114</t>
-  </si>
-  <si>
-    <t>Esborrar usuari</t>
-  </si>
-  <si>
-    <t>Icona esborrar → confirmar</t>
-  </si>
-  <si>
-    <t>Usuari eliminat de la graella</t>
-  </si>
-  <si>
-    <t>ZUP-115</t>
-  </si>
-  <si>
-    <t>DEVELOPER no accedeix</t>
-  </si>
-  <si>
-    <t>DEVELOPER → /admin/usuaris</t>
-  </si>
-  <si>
-    <t>Redirecció a home</t>
-  </si>
-  <si>
-    <t>Admin · Permisos (/admin/permisos)</t>
-  </si>
-  <si>
-    <t>ZUP-116</t>
-  </si>
-  <si>
-    <t>Pantalla permisos per rol</t>
-  </si>
-  <si>
-    <t>ADMIN → /admin/permisos</t>
-  </si>
-  <si>
-    <t>Matriu o llistat permisos per rol</t>
   </si>
   <si>
     <t>ZUP-117</t>
@@ -2827,7 +2845,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="86">
+  <cellXfs count="85">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3079,9 +3097,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -22560,9 +22575,11 @@
       <c r="H788" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="I788" s="18"/>
+      <c r="I788" s="18" t="s">
+        <v>566</v>
+      </c>
       <c r="J788" s="1" t="s">
-        <v>566</v>
+        <v>71</v>
       </c>
       <c r="K788" s="19"/>
       <c r="L788" s="18"/>
@@ -22848,9 +22865,11 @@
       <c r="H800" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="I800" s="18"/>
+      <c r="I800" s="18" t="s">
+        <v>566</v>
+      </c>
       <c r="J800" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K800" s="19"/>
       <c r="L800" s="18"/>
@@ -22992,9 +23011,11 @@
       <c r="H806" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="I806" s="18"/>
+      <c r="I806" s="18" t="s">
+        <v>566</v>
+      </c>
       <c r="J806" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K806" s="19"/>
       <c r="L806" s="18"/>
@@ -23111,7 +23132,7 @@
       <c r="M811" s="1"/>
       <c r="N811" s="19"/>
     </row>
-    <row r="812" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="812" ht="90" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A812" s="44" t="s">
         <v>545</v>
       </c>
@@ -23136,14 +23157,24 @@
       <c r="H812" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="I812" s="18"/>
+      <c r="I812" s="18" t="s">
+        <v>566</v>
+      </c>
       <c r="J812" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="K812" s="19"/>
-      <c r="L812" s="18"/>
-      <c r="M812" s="1"/>
-      <c r="N812" s="19"/>
+        <v>83</v>
+      </c>
+      <c r="K812" s="19" t="s">
+        <v>582</v>
+      </c>
+      <c r="L812" s="18" t="s">
+        <v>583</v>
+      </c>
+      <c r="M812" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="N812" s="19" t="s">
+        <v>584</v>
+      </c>
     </row>
     <row r="813" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A813" s="44"/>
@@ -23263,16 +23294,16 @@
         <v>92</v>
       </c>
       <c r="C818" s="14" t="s">
-        <v>582</v>
+        <v>585</v>
       </c>
       <c r="D818" s="15" t="s">
-        <v>583</v>
+        <v>586</v>
       </c>
       <c r="E818" s="15" t="s">
-        <v>584</v>
+        <v>587</v>
       </c>
       <c r="F818" s="15" t="s">
-        <v>585</v>
+        <v>588</v>
       </c>
       <c r="G818" s="16" t="s">
         <v>58</v>
@@ -23407,16 +23438,16 @@
         <v>53</v>
       </c>
       <c r="C824" s="25" t="s">
-        <v>586</v>
+        <v>589</v>
       </c>
       <c r="D824" s="26" t="s">
-        <v>587</v>
+        <v>590</v>
       </c>
       <c r="E824" s="26" t="s">
-        <v>588</v>
+        <v>591</v>
       </c>
       <c r="F824" s="26" t="s">
-        <v>589</v>
+        <v>592</v>
       </c>
       <c r="G824" s="16" t="s">
         <v>58</v>
@@ -23424,9 +23455,11 @@
       <c r="H824" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="I824" s="18"/>
+      <c r="I824" s="18" t="s">
+        <v>583</v>
+      </c>
       <c r="J824" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K824" s="19"/>
       <c r="L824" s="18"/>
@@ -23551,16 +23584,16 @@
         <v>53</v>
       </c>
       <c r="C830" s="14" t="s">
-        <v>590</v>
+        <v>593</v>
       </c>
       <c r="D830" s="15" t="s">
-        <v>591</v>
+        <v>594</v>
       </c>
       <c r="E830" s="15" t="s">
-        <v>592</v>
+        <v>595</v>
       </c>
       <c r="F830" s="15" t="s">
-        <v>593</v>
+        <v>596</v>
       </c>
       <c r="G830" s="16" t="s">
         <v>58</v>
@@ -23689,22 +23722,22 @@
     </row>
     <row r="836" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A836" s="45" t="s">
-        <v>594</v>
+        <v>597</v>
       </c>
       <c r="B836" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C836" s="25" t="s">
-        <v>595</v>
+        <v>598</v>
       </c>
       <c r="D836" s="26" t="s">
-        <v>596</v>
+        <v>599</v>
       </c>
       <c r="E836" s="26" t="s">
-        <v>597</v>
+        <v>600</v>
       </c>
       <c r="F836" s="26" t="s">
-        <v>598</v>
+        <v>601</v>
       </c>
       <c r="G836" s="16" t="s">
         <v>58</v>
@@ -23714,7 +23747,7 @@
       </c>
       <c r="I836" s="18"/>
       <c r="J836" s="1" t="s">
-        <v>60</v>
+        <v>602</v>
       </c>
       <c r="K836" s="19"/>
       <c r="L836" s="18"/>
@@ -23833,19 +23866,19 @@
     </row>
     <row r="842" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A842" s="45" t="s">
-        <v>594</v>
+        <v>597</v>
       </c>
       <c r="B842" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C842" s="14" t="s">
-        <v>599</v>
+        <v>603</v>
       </c>
       <c r="D842" s="15" t="s">
-        <v>600</v>
+        <v>604</v>
       </c>
       <c r="E842" s="15" t="s">
-        <v>601</v>
+        <v>605</v>
       </c>
       <c r="F842" s="15" t="s">
         <v>536</v>
@@ -23977,22 +24010,22 @@
     </row>
     <row r="848" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A848" s="45" t="s">
-        <v>594</v>
+        <v>597</v>
       </c>
       <c r="B848" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C848" s="25" t="s">
-        <v>602</v>
+        <v>606</v>
       </c>
       <c r="D848" s="26" t="s">
-        <v>603</v>
+        <v>607</v>
       </c>
       <c r="E848" s="26" t="s">
-        <v>604</v>
+        <v>608</v>
       </c>
       <c r="F848" s="26" t="s">
-        <v>605</v>
+        <v>609</v>
       </c>
       <c r="G848" s="16" t="s">
         <v>58</v>
@@ -24121,22 +24154,22 @@
     </row>
     <row r="854" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A854" s="45" t="s">
-        <v>594</v>
+        <v>597</v>
       </c>
       <c r="B854" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C854" s="14" t="s">
-        <v>606</v>
+        <v>610</v>
       </c>
       <c r="D854" s="15" t="s">
-        <v>607</v>
+        <v>611</v>
       </c>
       <c r="E854" s="15" t="s">
-        <v>608</v>
+        <v>612</v>
       </c>
       <c r="F854" s="15" t="s">
-        <v>609</v>
+        <v>613</v>
       </c>
       <c r="G854" s="16" t="s">
         <v>58</v>
@@ -24265,22 +24298,22 @@
     </row>
     <row r="860" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A860" s="46" t="s">
-        <v>610</v>
+        <v>614</v>
       </c>
       <c r="B860" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C860" s="25" t="s">
-        <v>611</v>
+        <v>615</v>
       </c>
       <c r="D860" s="26" t="s">
-        <v>612</v>
+        <v>616</v>
       </c>
       <c r="E860" s="26" t="s">
-        <v>613</v>
+        <v>617</v>
       </c>
       <c r="F860" s="26" t="s">
-        <v>614</v>
+        <v>618</v>
       </c>
       <c r="G860" s="16" t="s">
         <v>58</v>
@@ -24409,22 +24442,22 @@
     </row>
     <row r="866" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A866" s="46" t="s">
-        <v>610</v>
+        <v>614</v>
       </c>
       <c r="B866" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C866" s="14" t="s">
-        <v>615</v>
+        <v>619</v>
       </c>
       <c r="D866" s="15" t="s">
-        <v>616</v>
+        <v>620</v>
       </c>
       <c r="E866" s="15" t="s">
-        <v>617</v>
+        <v>621</v>
       </c>
       <c r="F866" s="15" t="s">
-        <v>618</v>
+        <v>622</v>
       </c>
       <c r="G866" s="16" t="s">
         <v>58</v>
@@ -24553,22 +24586,22 @@
     </row>
     <row r="872" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A872" s="46" t="s">
-        <v>610</v>
+        <v>614</v>
       </c>
       <c r="B872" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C872" s="25" t="s">
-        <v>619</v>
+        <v>623</v>
       </c>
       <c r="D872" s="26" t="s">
-        <v>620</v>
+        <v>624</v>
       </c>
       <c r="E872" s="26" t="s">
-        <v>621</v>
+        <v>625</v>
       </c>
       <c r="F872" s="26" t="s">
-        <v>622</v>
+        <v>626</v>
       </c>
       <c r="G872" s="16" t="s">
         <v>58</v>
@@ -24697,22 +24730,22 @@
     </row>
     <row r="878" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A878" s="46" t="s">
-        <v>610</v>
+        <v>614</v>
       </c>
       <c r="B878" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C878" s="14" t="s">
-        <v>623</v>
+        <v>627</v>
       </c>
       <c r="D878" s="15" t="s">
-        <v>624</v>
+        <v>628</v>
       </c>
       <c r="E878" s="15" t="s">
-        <v>625</v>
+        <v>629</v>
       </c>
       <c r="F878" s="15" t="s">
-        <v>626</v>
+        <v>630</v>
       </c>
       <c r="G878" s="16" t="s">
         <v>58</v>
@@ -24841,22 +24874,22 @@
     </row>
     <row r="884" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A884" s="46" t="s">
-        <v>610</v>
+        <v>614</v>
       </c>
       <c r="B884" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C884" s="25" t="s">
-        <v>627</v>
+        <v>631</v>
       </c>
       <c r="D884" s="26" t="s">
-        <v>628</v>
+        <v>632</v>
       </c>
       <c r="E884" s="26" t="s">
-        <v>629</v>
+        <v>633</v>
       </c>
       <c r="F884" s="26" t="s">
-        <v>630</v>
+        <v>634</v>
       </c>
       <c r="G884" s="16" t="s">
         <v>58</v>
@@ -24985,22 +25018,22 @@
     </row>
     <row r="890" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A890" s="46" t="s">
-        <v>610</v>
+        <v>614</v>
       </c>
       <c r="B890" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C890" s="14" t="s">
-        <v>631</v>
+        <v>635</v>
       </c>
       <c r="D890" s="15" t="s">
-        <v>632</v>
+        <v>636</v>
       </c>
       <c r="E890" s="15" t="s">
-        <v>633</v>
+        <v>637</v>
       </c>
       <c r="F890" s="15" t="s">
-        <v>634</v>
+        <v>638</v>
       </c>
       <c r="G890" s="16" t="s">
         <v>58</v>
@@ -25129,22 +25162,22 @@
     </row>
     <row r="896" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A896" s="46" t="s">
-        <v>610</v>
+        <v>614</v>
       </c>
       <c r="B896" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C896" s="25" t="s">
-        <v>635</v>
+        <v>639</v>
       </c>
       <c r="D896" s="26" t="s">
-        <v>636</v>
+        <v>640</v>
       </c>
       <c r="E896" s="26" t="s">
-        <v>637</v>
+        <v>641</v>
       </c>
       <c r="F896" s="26" t="s">
-        <v>638</v>
+        <v>642</v>
       </c>
       <c r="G896" s="16" t="s">
         <v>58</v>
@@ -25273,22 +25306,22 @@
     </row>
     <row r="902" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A902" s="47" t="s">
-        <v>639</v>
+        <v>643</v>
       </c>
       <c r="B902" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C902" s="14" t="s">
-        <v>640</v>
+        <v>644</v>
       </c>
       <c r="D902" s="15" t="s">
-        <v>641</v>
+        <v>645</v>
       </c>
       <c r="E902" s="15" t="s">
-        <v>642</v>
+        <v>646</v>
       </c>
       <c r="F902" s="15" t="s">
-        <v>643</v>
+        <v>647</v>
       </c>
       <c r="G902" s="16" t="s">
         <v>58</v>
@@ -25417,22 +25450,22 @@
     </row>
     <row r="908" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A908" s="47" t="s">
-        <v>639</v>
+        <v>643</v>
       </c>
       <c r="B908" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C908" s="25" t="s">
-        <v>644</v>
+        <v>648</v>
       </c>
       <c r="D908" s="26" t="s">
-        <v>645</v>
+        <v>649</v>
       </c>
       <c r="E908" s="26" t="s">
-        <v>646</v>
+        <v>650</v>
       </c>
       <c r="F908" s="26" t="s">
-        <v>647</v>
+        <v>651</v>
       </c>
       <c r="G908" s="16" t="s">
         <v>58</v>
@@ -25561,22 +25594,22 @@
     </row>
     <row r="914" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A914" s="47" t="s">
-        <v>639</v>
+        <v>643</v>
       </c>
       <c r="B914" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C914" s="14" t="s">
-        <v>648</v>
+        <v>652</v>
       </c>
       <c r="D914" s="15" t="s">
-        <v>649</v>
+        <v>653</v>
       </c>
       <c r="E914" s="15" t="s">
-        <v>650</v>
+        <v>654</v>
       </c>
       <c r="F914" s="15" t="s">
-        <v>651</v>
+        <v>655</v>
       </c>
       <c r="G914" s="16" t="s">
         <v>58</v>
@@ -25705,22 +25738,22 @@
     </row>
     <row r="920" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A920" s="47" t="s">
-        <v>639</v>
+        <v>643</v>
       </c>
       <c r="B920" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C920" s="25" t="s">
-        <v>652</v>
+        <v>656</v>
       </c>
       <c r="D920" s="26" t="s">
-        <v>653</v>
+        <v>657</v>
       </c>
       <c r="E920" s="26" t="s">
-        <v>654</v>
+        <v>658</v>
       </c>
       <c r="F920" s="26" t="s">
-        <v>655</v>
+        <v>659</v>
       </c>
       <c r="G920" s="16" t="s">
         <v>58</v>
@@ -25849,22 +25882,22 @@
     </row>
     <row r="926" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A926" s="47" t="s">
-        <v>639</v>
+        <v>643</v>
       </c>
       <c r="B926" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C926" s="14" t="s">
-        <v>656</v>
+        <v>660</v>
       </c>
       <c r="D926" s="15" t="s">
-        <v>657</v>
+        <v>661</v>
       </c>
       <c r="E926" s="15" t="s">
-        <v>658</v>
+        <v>662</v>
       </c>
       <c r="F926" s="15" t="s">
-        <v>659</v>
+        <v>663</v>
       </c>
       <c r="G926" s="16" t="s">
         <v>58</v>
@@ -25993,22 +26026,22 @@
     </row>
     <row r="932" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A932" s="47" t="s">
-        <v>639</v>
+        <v>643</v>
       </c>
       <c r="B932" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C932" s="25" t="s">
-        <v>660</v>
+        <v>664</v>
       </c>
       <c r="D932" s="26" t="s">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="E932" s="26" t="s">
-        <v>662</v>
+        <v>666</v>
       </c>
       <c r="F932" s="26" t="s">
-        <v>663</v>
+        <v>667</v>
       </c>
       <c r="G932" s="16" t="s">
         <v>58</v>
@@ -26137,22 +26170,22 @@
     </row>
     <row r="938" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A938" s="48" t="s">
-        <v>664</v>
+        <v>668</v>
       </c>
       <c r="B938" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C938" s="14" t="s">
-        <v>665</v>
+        <v>669</v>
       </c>
       <c r="D938" s="15" t="s">
-        <v>666</v>
+        <v>670</v>
       </c>
       <c r="E938" s="15" t="s">
-        <v>667</v>
+        <v>671</v>
       </c>
       <c r="F938" s="15" t="s">
-        <v>668</v>
+        <v>672</v>
       </c>
       <c r="G938" s="16" t="s">
         <v>58</v>
@@ -26281,22 +26314,22 @@
     </row>
     <row r="944" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A944" s="48" t="s">
-        <v>664</v>
+        <v>668</v>
       </c>
       <c r="B944" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C944" s="25" t="s">
-        <v>669</v>
+        <v>673</v>
       </c>
       <c r="D944" s="26" t="s">
-        <v>670</v>
+        <v>674</v>
       </c>
       <c r="E944" s="26" t="s">
-        <v>671</v>
+        <v>675</v>
       </c>
       <c r="F944" s="26" t="s">
-        <v>672</v>
+        <v>676</v>
       </c>
       <c r="G944" s="16" t="s">
         <v>58</v>
@@ -26425,22 +26458,22 @@
     </row>
     <row r="950" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A950" s="48" t="s">
-        <v>664</v>
+        <v>668</v>
       </c>
       <c r="B950" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C950" s="14" t="s">
-        <v>673</v>
+        <v>677</v>
       </c>
       <c r="D950" s="15" t="s">
-        <v>674</v>
+        <v>678</v>
       </c>
       <c r="E950" s="15" t="s">
-        <v>675</v>
+        <v>679</v>
       </c>
       <c r="F950" s="15" t="s">
-        <v>676</v>
+        <v>680</v>
       </c>
       <c r="G950" s="16" t="s">
         <v>58</v>
@@ -26569,22 +26602,22 @@
     </row>
     <row r="956" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A956" s="48" t="s">
-        <v>664</v>
+        <v>668</v>
       </c>
       <c r="B956" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C956" s="25" t="s">
-        <v>677</v>
+        <v>681</v>
       </c>
       <c r="D956" s="26" t="s">
-        <v>678</v>
+        <v>682</v>
       </c>
       <c r="E956" s="26" t="s">
-        <v>679</v>
+        <v>683</v>
       </c>
       <c r="F956" s="26" t="s">
-        <v>651</v>
+        <v>655</v>
       </c>
       <c r="G956" s="16" t="s">
         <v>58</v>
@@ -26713,22 +26746,22 @@
     </row>
     <row r="962" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A962" s="48" t="s">
-        <v>664</v>
+        <v>668</v>
       </c>
       <c r="B962" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C962" s="14" t="s">
-        <v>680</v>
+        <v>684</v>
       </c>
       <c r="D962" s="15" t="s">
-        <v>681</v>
+        <v>685</v>
       </c>
       <c r="E962" s="15" t="s">
-        <v>682</v>
+        <v>686</v>
       </c>
       <c r="F962" s="15" t="s">
-        <v>683</v>
+        <v>687</v>
       </c>
       <c r="G962" s="16" t="s">
         <v>58</v>
@@ -26857,22 +26890,22 @@
     </row>
     <row r="968" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A968" s="48" t="s">
-        <v>664</v>
+        <v>668</v>
       </c>
       <c r="B968" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C968" s="25" t="s">
-        <v>684</v>
+        <v>688</v>
       </c>
       <c r="D968" s="26" t="s">
-        <v>685</v>
+        <v>689</v>
       </c>
       <c r="E968" s="26" t="s">
-        <v>686</v>
+        <v>690</v>
       </c>
       <c r="F968" s="26" t="s">
-        <v>687</v>
+        <v>691</v>
       </c>
       <c r="G968" s="16" t="s">
         <v>58</v>
@@ -27001,22 +27034,22 @@
     </row>
     <row r="974" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A974" s="49" t="s">
-        <v>688</v>
+        <v>692</v>
       </c>
       <c r="B974" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C974" s="14" t="s">
-        <v>689</v>
+        <v>693</v>
       </c>
       <c r="D974" s="15" t="s">
-        <v>690</v>
+        <v>694</v>
       </c>
       <c r="E974" s="15" t="s">
-        <v>691</v>
+        <v>695</v>
       </c>
       <c r="F974" s="15" t="s">
-        <v>692</v>
+        <v>696</v>
       </c>
       <c r="G974" s="16" t="s">
         <v>58</v>
@@ -27145,22 +27178,22 @@
     </row>
     <row r="980" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A980" s="49" t="s">
-        <v>688</v>
+        <v>692</v>
       </c>
       <c r="B980" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C980" s="25" t="s">
-        <v>693</v>
+        <v>697</v>
       </c>
       <c r="D980" s="26" t="s">
-        <v>694</v>
+        <v>698</v>
       </c>
       <c r="E980" s="26" t="s">
-        <v>695</v>
+        <v>699</v>
       </c>
       <c r="F980" s="26" t="s">
-        <v>696</v>
+        <v>700</v>
       </c>
       <c r="G980" s="16" t="s">
         <v>58</v>
@@ -27289,22 +27322,22 @@
     </row>
     <row r="986" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A986" s="49" t="s">
-        <v>688</v>
+        <v>692</v>
       </c>
       <c r="B986" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C986" s="14" t="s">
-        <v>697</v>
+        <v>701</v>
       </c>
       <c r="D986" s="15" t="s">
-        <v>698</v>
+        <v>702</v>
       </c>
       <c r="E986" s="15" t="s">
-        <v>699</v>
+        <v>703</v>
       </c>
       <c r="F986" s="15" t="s">
-        <v>700</v>
+        <v>704</v>
       </c>
       <c r="G986" s="16" t="s">
         <v>58</v>
@@ -27433,22 +27466,22 @@
     </row>
     <row r="992" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A992" s="49" t="s">
-        <v>688</v>
+        <v>692</v>
       </c>
       <c r="B992" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C992" s="25" t="s">
-        <v>701</v>
+        <v>705</v>
       </c>
       <c r="D992" s="26" t="s">
-        <v>702</v>
+        <v>706</v>
       </c>
       <c r="E992" s="26" t="s">
-        <v>703</v>
+        <v>707</v>
       </c>
       <c r="F992" s="26" t="s">
-        <v>704</v>
+        <v>708</v>
       </c>
       <c r="G992" s="16" t="s">
         <v>58</v>
@@ -27577,22 +27610,22 @@
     </row>
     <row r="998" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A998" s="49" t="s">
-        <v>688</v>
+        <v>692</v>
       </c>
       <c r="B998" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C998" s="14" t="s">
-        <v>705</v>
+        <v>709</v>
       </c>
       <c r="D998" s="15" t="s">
-        <v>706</v>
+        <v>710</v>
       </c>
       <c r="E998" s="15" t="s">
-        <v>707</v>
+        <v>711</v>
       </c>
       <c r="F998" s="15" t="s">
-        <v>708</v>
+        <v>712</v>
       </c>
       <c r="G998" s="16" t="s">
         <v>58</v>
@@ -27721,22 +27754,22 @@
     </row>
     <row r="1004" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1004" s="50" t="s">
-        <v>709</v>
+        <v>713</v>
       </c>
       <c r="B1004" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1004" s="25" t="s">
-        <v>710</v>
+        <v>714</v>
       </c>
       <c r="D1004" s="26" t="s">
-        <v>711</v>
+        <v>715</v>
       </c>
       <c r="E1004" s="26" t="s">
-        <v>712</v>
+        <v>716</v>
       </c>
       <c r="F1004" s="26" t="s">
-        <v>713</v>
+        <v>717</v>
       </c>
       <c r="G1004" s="16" t="s">
         <v>58</v>
@@ -27865,22 +27898,22 @@
     </row>
     <row r="1010" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1010" s="50" t="s">
-        <v>709</v>
+        <v>713</v>
       </c>
       <c r="B1010" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1010" s="14" t="s">
-        <v>714</v>
+        <v>718</v>
       </c>
       <c r="D1010" s="15" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="E1010" s="15" t="s">
-        <v>716</v>
+        <v>720</v>
       </c>
       <c r="F1010" s="15" t="s">
-        <v>717</v>
+        <v>721</v>
       </c>
       <c r="G1010" s="16" t="s">
         <v>58</v>
@@ -28009,22 +28042,22 @@
     </row>
     <row r="1016" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1016" s="50" t="s">
-        <v>709</v>
+        <v>713</v>
       </c>
       <c r="B1016" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1016" s="25" t="s">
-        <v>718</v>
+        <v>722</v>
       </c>
       <c r="D1016" s="26" t="s">
-        <v>719</v>
+        <v>723</v>
       </c>
       <c r="E1016" s="26" t="s">
-        <v>720</v>
+        <v>724</v>
       </c>
       <c r="F1016" s="26" t="s">
-        <v>721</v>
+        <v>725</v>
       </c>
       <c r="G1016" s="16" t="s">
         <v>58</v>
@@ -28153,22 +28186,22 @@
     </row>
     <row r="1022" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1022" s="50" t="s">
-        <v>709</v>
+        <v>713</v>
       </c>
       <c r="B1022" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1022" s="14" t="s">
-        <v>722</v>
+        <v>726</v>
       </c>
       <c r="D1022" s="15" t="s">
-        <v>723</v>
+        <v>727</v>
       </c>
       <c r="E1022" s="15" t="s">
-        <v>724</v>
+        <v>728</v>
       </c>
       <c r="F1022" s="15" t="s">
-        <v>725</v>
+        <v>729</v>
       </c>
       <c r="G1022" s="16" t="s">
         <v>58</v>
@@ -28297,22 +28330,22 @@
     </row>
     <row r="1028" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1028" s="50" t="s">
-        <v>709</v>
+        <v>713</v>
       </c>
       <c r="B1028" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C1028" s="25" t="s">
-        <v>726</v>
+        <v>730</v>
       </c>
       <c r="D1028" s="26" t="s">
-        <v>727</v>
+        <v>731</v>
       </c>
       <c r="E1028" s="26" t="s">
-        <v>728</v>
+        <v>732</v>
       </c>
       <c r="F1028" s="26" t="s">
-        <v>729</v>
+        <v>733</v>
       </c>
       <c r="G1028" s="16" t="s">
         <v>58</v>
@@ -28441,22 +28474,22 @@
     </row>
     <row r="1034" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1034" s="50" t="s">
-        <v>709</v>
+        <v>713</v>
       </c>
       <c r="B1034" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C1034" s="14" t="s">
-        <v>730</v>
+        <v>734</v>
       </c>
       <c r="D1034" s="15" t="s">
-        <v>731</v>
+        <v>735</v>
       </c>
       <c r="E1034" s="15" t="s">
-        <v>732</v>
+        <v>736</v>
       </c>
       <c r="F1034" s="15" t="s">
-        <v>733</v>
+        <v>737</v>
       </c>
       <c r="G1034" s="16" t="s">
         <v>58</v>
@@ -28585,22 +28618,22 @@
     </row>
     <row r="1040" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1040" s="51" t="s">
-        <v>734</v>
+        <v>738</v>
       </c>
       <c r="B1040" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C1040" s="25" t="s">
-        <v>735</v>
+        <v>739</v>
       </c>
       <c r="D1040" s="26" t="s">
-        <v>723</v>
+        <v>727</v>
       </c>
       <c r="E1040" s="26" t="s">
-        <v>736</v>
+        <v>740</v>
       </c>
       <c r="F1040" s="26" t="s">
-        <v>737</v>
+        <v>741</v>
       </c>
       <c r="G1040" s="16" t="s">
         <v>58</v>
@@ -28729,22 +28762,22 @@
     </row>
     <row r="1046" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1046" s="51" t="s">
-        <v>734</v>
+        <v>738</v>
       </c>
       <c r="B1046" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1046" s="14" t="s">
-        <v>738</v>
+        <v>742</v>
       </c>
       <c r="D1046" s="15" t="s">
-        <v>715</v>
+        <v>719</v>
       </c>
       <c r="E1046" s="15" t="s">
-        <v>739</v>
+        <v>743</v>
       </c>
       <c r="F1046" s="15" t="s">
-        <v>740</v>
+        <v>744</v>
       </c>
       <c r="G1046" s="16" t="s">
         <v>58</v>
@@ -28881,16 +28914,16 @@
         <v>53</v>
       </c>
       <c r="C1052" s="25" t="s">
-        <v>741</v>
+        <v>745</v>
       </c>
       <c r="D1052" s="26" t="s">
-        <v>742</v>
+        <v>746</v>
       </c>
       <c r="E1052" s="26" t="s">
-        <v>743</v>
+        <v>747</v>
       </c>
       <c r="F1052" s="26" t="s">
-        <v>744</v>
+        <v>748</v>
       </c>
       <c r="G1052" s="16" t="s">
         <v>58</v>
@@ -29027,16 +29060,16 @@
         <v>53</v>
       </c>
       <c r="C1058" s="14" t="s">
-        <v>745</v>
+        <v>749</v>
       </c>
       <c r="D1058" s="15" t="s">
-        <v>746</v>
+        <v>750</v>
       </c>
       <c r="E1058" s="15" t="s">
-        <v>747</v>
+        <v>751</v>
       </c>
       <c r="F1058" s="15" t="s">
-        <v>748</v>
+        <v>752</v>
       </c>
       <c r="G1058" s="16" t="s">
         <v>58</v>
@@ -30122,10 +30155,10 @@
         <v>39</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>749</v>
+        <v>753</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>750</v>
+        <v>754</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>53</v>
@@ -30143,7 +30176,7 @@
         <v>83</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>751</v>
+        <v>755</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -30554,7 +30587,7 @@
     </row>
     <row r="16" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="66" t="s">
-        <v>594</v>
+        <v>597</v>
       </c>
       <c r="B16" s="1">
         <v>4</v>
@@ -30583,7 +30616,7 @@
     </row>
     <row r="17" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="67" t="s">
-        <v>610</v>
+        <v>614</v>
       </c>
       <c r="B17" s="1">
         <v>7</v>
@@ -30612,7 +30645,7 @@
     </row>
     <row r="18" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="68" t="s">
-        <v>639</v>
+        <v>643</v>
       </c>
       <c r="B18" s="1">
         <v>6</v>
@@ -30641,7 +30674,7 @@
     </row>
     <row r="19" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="69" t="s">
-        <v>664</v>
+        <v>668</v>
       </c>
       <c r="B19" s="1">
         <v>6</v>
@@ -30670,7 +30703,7 @@
     </row>
     <row r="20" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="70" t="s">
-        <v>688</v>
+        <v>692</v>
       </c>
       <c r="B20" s="1">
         <v>5</v>
@@ -30699,7 +30732,7 @@
     </row>
     <row r="21" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="71" t="s">
-        <v>709</v>
+        <v>713</v>
       </c>
       <c r="B21" s="1">
         <v>6</v>
@@ -30728,7 +30761,7 @@
     </row>
     <row r="22" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="72" t="s">
-        <v>734</v>
+        <v>738</v>
       </c>
       <c r="B22" s="1">
         <v>2</v>
@@ -30757,7 +30790,7 @@
     </row>
     <row r="23" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="73" t="s">
-        <v>752</v>
+        <v>756</v>
       </c>
       <c r="B23" s="73">
         <v>153</v>
@@ -30808,7 +30841,7 @@
         <v>44</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>750</v>
+        <v>754</v>
       </c>
       <c r="C1" s="10" t="s">
         <v>71</v>
@@ -30817,7 +30850,7 @@
         <v>83</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>751</v>
+        <v>755</v>
       </c>
       <c r="F1" s="10" t="s">
         <v>97</v>
@@ -30968,10 +31001,10 @@
         <v>45</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>753</v>
+        <v>757</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>750</v>
+        <v>754</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>71</v>
@@ -30980,7 +31013,7 @@
         <v>83</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>751</v>
+        <v>755</v>
       </c>
       <c r="G1" s="10" t="s">
         <v>97</v>
@@ -30991,7 +31024,7 @@
         <v>59</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>754</v>
+        <v>758</v>
       </c>
       <c r="C2" s="1">
         <f>COUNTIF(Proves!$H:$H,A2)</f>
@@ -31121,7 +31154,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="83" t="s">
-        <v>755</v>
+        <v>759</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -31129,7 +31162,7 @@
         <v>71</v>
       </c>
       <c r="B2" s="84" t="s">
-        <v>756</v>
+        <v>760</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
@@ -31138,7 +31171,7 @@
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" s="85" t="s">
+      <c r="A4" s="1" t="s">
         <v>60</v>
       </c>
     </row>
@@ -31149,7 +31182,7 @@
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>566</v>
+        <v>602</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
`099 => fase IV => menús per rol (TEST veu assignats, seed no pisa F5), Desar només amb canvi, comentaris opcionals, ZUP-116–120 OK i ZUP-121 KO/corr (Chrome/ADMIN)`
</commit_message>
<xml_diff>
--- a/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
+++ b/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4434" uniqueCount="761">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4444" uniqueCount="763">
   <si>
     <t>Zuppeto — Joc de probes manual (totes les pantalles)</t>
   </si>
@@ -1916,79 +1916,99 @@
     <t>Matriu o llistat permisos per rol</t>
   </si>
   <si>
+    <t>ZUP-117</t>
+  </si>
+  <si>
+    <t>Editar permisos USER</t>
+  </si>
+  <si>
+    <t>Modificar permís i desar</t>
+  </si>
+  <si>
+    <t>ZUP-118</t>
+  </si>
+  <si>
+    <t>Editar permisos DEVELOPER</t>
+  </si>
+  <si>
+    <t>Donar/treure accés a documentació interna</t>
+  </si>
+  <si>
+    <t>Canvi reflectit en accés real</t>
+  </si>
+  <si>
+    <t>ZUP-119</t>
+  </si>
+  <si>
+    <t>Refresc menú després de permisos</t>
+  </si>
+  <si>
+    <t>Desar canvis que afecten menú</t>
+  </si>
+  <si>
+    <t>La capçalera es refresca sense tornar a iniciar sessió</t>
+  </si>
+  <si>
+    <t>Admin · Menús (/admin/menus)</t>
+  </si>
+  <si>
+    <t>ZUP-120</t>
+  </si>
+  <si>
+    <t>Pantalla menús — llistat</t>
+  </si>
+  <si>
+    <t>ADMIN → /admin/menus</t>
+  </si>
+  <si>
+    <t>Definicions i assignacions de menú</t>
+  </si>
+  <si>
+    <t>ZUP-121</t>
+  </si>
+  <si>
+    <t>Crear menú sota Ajuda</t>
+  </si>
+  <si>
+    <t>Nou menú dins d'Ajuda</t>
+  </si>
+  <si>
+    <t>Apareix dins submenú Ajuda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El menú creat per TEST (kkk) no surt a la capçalera ni sota Ajuda.
+Desar quedava apagat: el pare era el mateix menú (kkk) en lloc de help.
+El rol TEST només veia un menú fix (Inici/Ajuda) i no els fills d’Ajuda assignats.
+La foto de perfil (logo) no es desava: el PUT de fitxa tornava 400 amb comentaris buits (API encara exigia comentaris).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Què s’ha fet:
+Comentaris sempre opcionals (perfil i admin); el Desar de fitxa ja no exigeix text.
+Desar/Crear només s’activen si hi ha canvi i es compleixen les regles (FormCommitPolicy).
+Si només es canvia la contrasenya, no s’envia la fitxa (evita el 400).
+TEST carrega el menú de l’API: Inici + Ajuda + fills d’Ajuda assignats (pare = help, no el mateix menú).
+Validació de pare de menú: ha d’existir i no pot ser ell mateix.
+Cal reiniciar l’API (F5) perquè agafi el validador nou i el filtre de navegació.
+Què s'ha fet (retest OK):
+- TEST veu els menús assignats (principal si Pare buit; sota Ajuda si Pare = help)
+- DevelopmentIdentitySeeder ja no esborra menu_roles en cada F5
+- Capçalera mostra menú sense ruta (text)
+- docs/ca/funcional-ca.md, docs/ca/tecnic-ca.md</t>
+  </si>
+  <si>
+    <t>ZUP-122</t>
+  </si>
+  <si>
+    <t>Crear menú sota admin</t>
+  </si>
+  <si>
+    <t>Nou menú dins d'administració</t>
+  </si>
+  <si>
+    <t>Apareix a Del administrador</t>
+  </si>
+  <si>
     <t>EN CURS</t>
-  </si>
-  <si>
-    <t>ZUP-117</t>
-  </si>
-  <si>
-    <t>Editar permisos USER</t>
-  </si>
-  <si>
-    <t>Modificar permís i desar</t>
-  </si>
-  <si>
-    <t>ZUP-118</t>
-  </si>
-  <si>
-    <t>Editar permisos DEVELOPER</t>
-  </si>
-  <si>
-    <t>Donar/treure accés a documentació interna</t>
-  </si>
-  <si>
-    <t>Canvi reflectit en accés real</t>
-  </si>
-  <si>
-    <t>ZUP-119</t>
-  </si>
-  <si>
-    <t>Refresc menú després de permisos</t>
-  </si>
-  <si>
-    <t>Desar canvis que afecten menú</t>
-  </si>
-  <si>
-    <t>La capçalera es refresca sense tornar a iniciar sessió</t>
-  </si>
-  <si>
-    <t>Admin · Menús (/admin/menus)</t>
-  </si>
-  <si>
-    <t>ZUP-120</t>
-  </si>
-  <si>
-    <t>Pantalla menús — llistat</t>
-  </si>
-  <si>
-    <t>ADMIN → /admin/menus</t>
-  </si>
-  <si>
-    <t>Definicions i assignacions de menú</t>
-  </si>
-  <si>
-    <t>ZUP-121</t>
-  </si>
-  <si>
-    <t>Crear menú sota Ajuda</t>
-  </si>
-  <si>
-    <t>Nou menú dins d'Ajuda</t>
-  </si>
-  <si>
-    <t>Apareix dins submenú Ajuda</t>
-  </si>
-  <si>
-    <t>ZUP-122</t>
-  </si>
-  <si>
-    <t>Crear menú sota admin</t>
-  </si>
-  <si>
-    <t>Nou menú dins d'administració</t>
-  </si>
-  <si>
-    <t>Apareix a Del administrador</t>
   </si>
   <si>
     <t>ZUP-123</t>
@@ -23745,9 +23765,11 @@
       <c r="H836" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="I836" s="18"/>
+      <c r="I836" s="18" t="s">
+        <v>583</v>
+      </c>
       <c r="J836" s="1" t="s">
-        <v>602</v>
+        <v>71</v>
       </c>
       <c r="K836" s="19"/>
       <c r="L836" s="18"/>
@@ -23872,13 +23894,13 @@
         <v>53</v>
       </c>
       <c r="C842" s="14" t="s">
+        <v>602</v>
+      </c>
+      <c r="D842" s="15" t="s">
         <v>603</v>
       </c>
-      <c r="D842" s="15" t="s">
+      <c r="E842" s="15" t="s">
         <v>604</v>
-      </c>
-      <c r="E842" s="15" t="s">
-        <v>605</v>
       </c>
       <c r="F842" s="15" t="s">
         <v>536</v>
@@ -23889,9 +23911,11 @@
       <c r="H842" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="I842" s="18"/>
+      <c r="I842" s="18" t="s">
+        <v>583</v>
+      </c>
       <c r="J842" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K842" s="19"/>
       <c r="L842" s="18"/>
@@ -24016,16 +24040,16 @@
         <v>53</v>
       </c>
       <c r="C848" s="25" t="s">
+        <v>605</v>
+      </c>
+      <c r="D848" s="26" t="s">
         <v>606</v>
       </c>
-      <c r="D848" s="26" t="s">
+      <c r="E848" s="26" t="s">
         <v>607</v>
       </c>
-      <c r="E848" s="26" t="s">
+      <c r="F848" s="26" t="s">
         <v>608</v>
-      </c>
-      <c r="F848" s="26" t="s">
-        <v>609</v>
       </c>
       <c r="G848" s="16" t="s">
         <v>58</v>
@@ -24160,16 +24184,16 @@
         <v>53</v>
       </c>
       <c r="C854" s="14" t="s">
+        <v>609</v>
+      </c>
+      <c r="D854" s="15" t="s">
         <v>610</v>
       </c>
-      <c r="D854" s="15" t="s">
+      <c r="E854" s="15" t="s">
         <v>611</v>
       </c>
-      <c r="E854" s="15" t="s">
+      <c r="F854" s="15" t="s">
         <v>612</v>
-      </c>
-      <c r="F854" s="15" t="s">
-        <v>613</v>
       </c>
       <c r="G854" s="16" t="s">
         <v>58</v>
@@ -24177,9 +24201,11 @@
       <c r="H854" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="I854" s="18"/>
+      <c r="I854" s="18" t="s">
+        <v>583</v>
+      </c>
       <c r="J854" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K854" s="19"/>
       <c r="L854" s="18"/>
@@ -24298,22 +24324,22 @@
     </row>
     <row r="860" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A860" s="46" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="B860" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C860" s="25" t="s">
+        <v>614</v>
+      </c>
+      <c r="D860" s="26" t="s">
         <v>615</v>
       </c>
-      <c r="D860" s="26" t="s">
+      <c r="E860" s="26" t="s">
         <v>616</v>
       </c>
-      <c r="E860" s="26" t="s">
+      <c r="F860" s="26" t="s">
         <v>617</v>
-      </c>
-      <c r="F860" s="26" t="s">
-        <v>618</v>
       </c>
       <c r="G860" s="16" t="s">
         <v>58</v>
@@ -24321,9 +24347,11 @@
       <c r="H860" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="I860" s="18"/>
+      <c r="I860" s="18" t="s">
+        <v>583</v>
+      </c>
       <c r="J860" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K860" s="19"/>
       <c r="L860" s="18"/>
@@ -24442,22 +24470,22 @@
     </row>
     <row r="866" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A866" s="46" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="B866" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C866" s="14" t="s">
+        <v>618</v>
+      </c>
+      <c r="D866" s="15" t="s">
         <v>619</v>
       </c>
-      <c r="D866" s="15" t="s">
+      <c r="E866" s="15" t="s">
         <v>620</v>
       </c>
-      <c r="E866" s="15" t="s">
+      <c r="F866" s="15" t="s">
         <v>621</v>
-      </c>
-      <c r="F866" s="15" t="s">
-        <v>622</v>
       </c>
       <c r="G866" s="16" t="s">
         <v>58</v>
@@ -24465,14 +24493,24 @@
       <c r="H866" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="I866" s="18"/>
+      <c r="I866" s="18" t="s">
+        <v>583</v>
+      </c>
       <c r="J866" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="K866" s="19"/>
-      <c r="L866" s="18"/>
-      <c r="M866" s="1"/>
-      <c r="N866" s="19"/>
+        <v>83</v>
+      </c>
+      <c r="K866" s="19" t="s">
+        <v>622</v>
+      </c>
+      <c r="L866" s="18" t="s">
+        <v>583</v>
+      </c>
+      <c r="M866" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="N866" s="19" t="s">
+        <v>623</v>
+      </c>
     </row>
     <row r="867" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A867" s="46"/>
@@ -24586,22 +24624,22 @@
     </row>
     <row r="872" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A872" s="46" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="B872" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C872" s="25" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
       <c r="D872" s="26" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="E872" s="26" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="F872" s="26" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="G872" s="16" t="s">
         <v>58</v>
@@ -24609,9 +24647,11 @@
       <c r="H872" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="I872" s="18"/>
+      <c r="I872" s="18" t="s">
+        <v>583</v>
+      </c>
       <c r="J872" s="1" t="s">
-        <v>60</v>
+        <v>628</v>
       </c>
       <c r="K872" s="19"/>
       <c r="L872" s="18"/>
@@ -24730,22 +24770,22 @@
     </row>
     <row r="878" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A878" s="46" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="B878" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C878" s="14" t="s">
-        <v>627</v>
+        <v>629</v>
       </c>
       <c r="D878" s="15" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
       <c r="E878" s="15" t="s">
-        <v>629</v>
+        <v>631</v>
       </c>
       <c r="F878" s="15" t="s">
-        <v>630</v>
+        <v>632</v>
       </c>
       <c r="G878" s="16" t="s">
         <v>58</v>
@@ -24874,22 +24914,22 @@
     </row>
     <row r="884" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A884" s="46" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="B884" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C884" s="25" t="s">
-        <v>631</v>
+        <v>633</v>
       </c>
       <c r="D884" s="26" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
       <c r="E884" s="26" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="F884" s="26" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
       <c r="G884" s="16" t="s">
         <v>58</v>
@@ -25018,22 +25058,22 @@
     </row>
     <row r="890" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A890" s="46" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="B890" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C890" s="14" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="D890" s="15" t="s">
-        <v>636</v>
+        <v>638</v>
       </c>
       <c r="E890" s="15" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="F890" s="15" t="s">
-        <v>638</v>
+        <v>640</v>
       </c>
       <c r="G890" s="16" t="s">
         <v>58</v>
@@ -25162,22 +25202,22 @@
     </row>
     <row r="896" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A896" s="46" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="B896" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C896" s="25" t="s">
-        <v>639</v>
+        <v>641</v>
       </c>
       <c r="D896" s="26" t="s">
-        <v>640</v>
+        <v>642</v>
       </c>
       <c r="E896" s="26" t="s">
-        <v>641</v>
+        <v>643</v>
       </c>
       <c r="F896" s="26" t="s">
-        <v>642</v>
+        <v>644</v>
       </c>
       <c r="G896" s="16" t="s">
         <v>58</v>
@@ -25306,22 +25346,22 @@
     </row>
     <row r="902" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A902" s="47" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
       <c r="B902" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C902" s="14" t="s">
-        <v>644</v>
+        <v>646</v>
       </c>
       <c r="D902" s="15" t="s">
-        <v>645</v>
+        <v>647</v>
       </c>
       <c r="E902" s="15" t="s">
-        <v>646</v>
+        <v>648</v>
       </c>
       <c r="F902" s="15" t="s">
-        <v>647</v>
+        <v>649</v>
       </c>
       <c r="G902" s="16" t="s">
         <v>58</v>
@@ -25450,22 +25490,22 @@
     </row>
     <row r="908" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A908" s="47" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
       <c r="B908" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C908" s="25" t="s">
-        <v>648</v>
+        <v>650</v>
       </c>
       <c r="D908" s="26" t="s">
-        <v>649</v>
+        <v>651</v>
       </c>
       <c r="E908" s="26" t="s">
-        <v>650</v>
+        <v>652</v>
       </c>
       <c r="F908" s="26" t="s">
-        <v>651</v>
+        <v>653</v>
       </c>
       <c r="G908" s="16" t="s">
         <v>58</v>
@@ -25594,22 +25634,22 @@
     </row>
     <row r="914" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A914" s="47" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
       <c r="B914" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C914" s="14" t="s">
-        <v>652</v>
+        <v>654</v>
       </c>
       <c r="D914" s="15" t="s">
-        <v>653</v>
+        <v>655</v>
       </c>
       <c r="E914" s="15" t="s">
-        <v>654</v>
+        <v>656</v>
       </c>
       <c r="F914" s="15" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
       <c r="G914" s="16" t="s">
         <v>58</v>
@@ -25738,22 +25778,22 @@
     </row>
     <row r="920" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A920" s="47" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
       <c r="B920" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C920" s="25" t="s">
-        <v>656</v>
+        <v>658</v>
       </c>
       <c r="D920" s="26" t="s">
-        <v>657</v>
+        <v>659</v>
       </c>
       <c r="E920" s="26" t="s">
-        <v>658</v>
+        <v>660</v>
       </c>
       <c r="F920" s="26" t="s">
-        <v>659</v>
+        <v>661</v>
       </c>
       <c r="G920" s="16" t="s">
         <v>58</v>
@@ -25882,22 +25922,22 @@
     </row>
     <row r="926" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A926" s="47" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
       <c r="B926" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C926" s="14" t="s">
-        <v>660</v>
+        <v>662</v>
       </c>
       <c r="D926" s="15" t="s">
-        <v>661</v>
+        <v>663</v>
       </c>
       <c r="E926" s="15" t="s">
-        <v>662</v>
+        <v>664</v>
       </c>
       <c r="F926" s="15" t="s">
-        <v>663</v>
+        <v>665</v>
       </c>
       <c r="G926" s="16" t="s">
         <v>58</v>
@@ -26026,22 +26066,22 @@
     </row>
     <row r="932" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A932" s="47" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
       <c r="B932" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C932" s="25" t="s">
-        <v>664</v>
+        <v>666</v>
       </c>
       <c r="D932" s="26" t="s">
-        <v>665</v>
+        <v>667</v>
       </c>
       <c r="E932" s="26" t="s">
-        <v>666</v>
+        <v>668</v>
       </c>
       <c r="F932" s="26" t="s">
-        <v>667</v>
+        <v>669</v>
       </c>
       <c r="G932" s="16" t="s">
         <v>58</v>
@@ -26170,22 +26210,22 @@
     </row>
     <row r="938" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A938" s="48" t="s">
-        <v>668</v>
+        <v>670</v>
       </c>
       <c r="B938" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C938" s="14" t="s">
-        <v>669</v>
+        <v>671</v>
       </c>
       <c r="D938" s="15" t="s">
-        <v>670</v>
+        <v>672</v>
       </c>
       <c r="E938" s="15" t="s">
-        <v>671</v>
+        <v>673</v>
       </c>
       <c r="F938" s="15" t="s">
-        <v>672</v>
+        <v>674</v>
       </c>
       <c r="G938" s="16" t="s">
         <v>58</v>
@@ -26314,22 +26354,22 @@
     </row>
     <row r="944" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A944" s="48" t="s">
-        <v>668</v>
+        <v>670</v>
       </c>
       <c r="B944" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C944" s="25" t="s">
-        <v>673</v>
+        <v>675</v>
       </c>
       <c r="D944" s="26" t="s">
-        <v>674</v>
+        <v>676</v>
       </c>
       <c r="E944" s="26" t="s">
-        <v>675</v>
+        <v>677</v>
       </c>
       <c r="F944" s="26" t="s">
-        <v>676</v>
+        <v>678</v>
       </c>
       <c r="G944" s="16" t="s">
         <v>58</v>
@@ -26458,22 +26498,22 @@
     </row>
     <row r="950" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A950" s="48" t="s">
-        <v>668</v>
+        <v>670</v>
       </c>
       <c r="B950" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C950" s="14" t="s">
-        <v>677</v>
+        <v>679</v>
       </c>
       <c r="D950" s="15" t="s">
-        <v>678</v>
+        <v>680</v>
       </c>
       <c r="E950" s="15" t="s">
-        <v>679</v>
+        <v>681</v>
       </c>
       <c r="F950" s="15" t="s">
-        <v>680</v>
+        <v>682</v>
       </c>
       <c r="G950" s="16" t="s">
         <v>58</v>
@@ -26602,22 +26642,22 @@
     </row>
     <row r="956" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A956" s="48" t="s">
-        <v>668</v>
+        <v>670</v>
       </c>
       <c r="B956" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C956" s="25" t="s">
-        <v>681</v>
+        <v>683</v>
       </c>
       <c r="D956" s="26" t="s">
-        <v>682</v>
+        <v>684</v>
       </c>
       <c r="E956" s="26" t="s">
-        <v>683</v>
+        <v>685</v>
       </c>
       <c r="F956" s="26" t="s">
-        <v>655</v>
+        <v>657</v>
       </c>
       <c r="G956" s="16" t="s">
         <v>58</v>
@@ -26746,22 +26786,22 @@
     </row>
     <row r="962" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A962" s="48" t="s">
-        <v>668</v>
+        <v>670</v>
       </c>
       <c r="B962" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C962" s="14" t="s">
-        <v>684</v>
+        <v>686</v>
       </c>
       <c r="D962" s="15" t="s">
-        <v>685</v>
+        <v>687</v>
       </c>
       <c r="E962" s="15" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
       <c r="F962" s="15" t="s">
-        <v>687</v>
+        <v>689</v>
       </c>
       <c r="G962" s="16" t="s">
         <v>58</v>
@@ -26890,22 +26930,22 @@
     </row>
     <row r="968" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A968" s="48" t="s">
-        <v>668</v>
+        <v>670</v>
       </c>
       <c r="B968" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C968" s="25" t="s">
-        <v>688</v>
+        <v>690</v>
       </c>
       <c r="D968" s="26" t="s">
-        <v>689</v>
+        <v>691</v>
       </c>
       <c r="E968" s="26" t="s">
-        <v>690</v>
+        <v>692</v>
       </c>
       <c r="F968" s="26" t="s">
-        <v>691</v>
+        <v>693</v>
       </c>
       <c r="G968" s="16" t="s">
         <v>58</v>
@@ -27034,22 +27074,22 @@
     </row>
     <row r="974" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A974" s="49" t="s">
-        <v>692</v>
+        <v>694</v>
       </c>
       <c r="B974" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C974" s="14" t="s">
-        <v>693</v>
+        <v>695</v>
       </c>
       <c r="D974" s="15" t="s">
-        <v>694</v>
+        <v>696</v>
       </c>
       <c r="E974" s="15" t="s">
-        <v>695</v>
+        <v>697</v>
       </c>
       <c r="F974" s="15" t="s">
-        <v>696</v>
+        <v>698</v>
       </c>
       <c r="G974" s="16" t="s">
         <v>58</v>
@@ -27178,22 +27218,22 @@
     </row>
     <row r="980" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A980" s="49" t="s">
-        <v>692</v>
+        <v>694</v>
       </c>
       <c r="B980" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C980" s="25" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
       <c r="D980" s="26" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
       <c r="E980" s="26" t="s">
-        <v>699</v>
+        <v>701</v>
       </c>
       <c r="F980" s="26" t="s">
-        <v>700</v>
+        <v>702</v>
       </c>
       <c r="G980" s="16" t="s">
         <v>58</v>
@@ -27322,22 +27362,22 @@
     </row>
     <row r="986" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A986" s="49" t="s">
-        <v>692</v>
+        <v>694</v>
       </c>
       <c r="B986" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C986" s="14" t="s">
-        <v>701</v>
+        <v>703</v>
       </c>
       <c r="D986" s="15" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="E986" s="15" t="s">
-        <v>703</v>
+        <v>705</v>
       </c>
       <c r="F986" s="15" t="s">
-        <v>704</v>
+        <v>706</v>
       </c>
       <c r="G986" s="16" t="s">
         <v>58</v>
@@ -27466,22 +27506,22 @@
     </row>
     <row r="992" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A992" s="49" t="s">
-        <v>692</v>
+        <v>694</v>
       </c>
       <c r="B992" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C992" s="25" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
       <c r="D992" s="26" t="s">
-        <v>706</v>
+        <v>708</v>
       </c>
       <c r="E992" s="26" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
       <c r="F992" s="26" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="G992" s="16" t="s">
         <v>58</v>
@@ -27610,22 +27650,22 @@
     </row>
     <row r="998" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A998" s="49" t="s">
-        <v>692</v>
+        <v>694</v>
       </c>
       <c r="B998" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C998" s="14" t="s">
-        <v>709</v>
+        <v>711</v>
       </c>
       <c r="D998" s="15" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="E998" s="15" t="s">
-        <v>711</v>
+        <v>713</v>
       </c>
       <c r="F998" s="15" t="s">
-        <v>712</v>
+        <v>714</v>
       </c>
       <c r="G998" s="16" t="s">
         <v>58</v>
@@ -27754,22 +27794,22 @@
     </row>
     <row r="1004" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1004" s="50" t="s">
-        <v>713</v>
+        <v>715</v>
       </c>
       <c r="B1004" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1004" s="25" t="s">
-        <v>714</v>
+        <v>716</v>
       </c>
       <c r="D1004" s="26" t="s">
-        <v>715</v>
+        <v>717</v>
       </c>
       <c r="E1004" s="26" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
       <c r="F1004" s="26" t="s">
-        <v>717</v>
+        <v>719</v>
       </c>
       <c r="G1004" s="16" t="s">
         <v>58</v>
@@ -27898,22 +27938,22 @@
     </row>
     <row r="1010" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1010" s="50" t="s">
-        <v>713</v>
+        <v>715</v>
       </c>
       <c r="B1010" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1010" s="14" t="s">
-        <v>718</v>
+        <v>720</v>
       </c>
       <c r="D1010" s="15" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
       <c r="E1010" s="15" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
       <c r="F1010" s="15" t="s">
-        <v>721</v>
+        <v>723</v>
       </c>
       <c r="G1010" s="16" t="s">
         <v>58</v>
@@ -28042,22 +28082,22 @@
     </row>
     <row r="1016" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1016" s="50" t="s">
-        <v>713</v>
+        <v>715</v>
       </c>
       <c r="B1016" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1016" s="25" t="s">
-        <v>722</v>
+        <v>724</v>
       </c>
       <c r="D1016" s="26" t="s">
-        <v>723</v>
+        <v>725</v>
       </c>
       <c r="E1016" s="26" t="s">
-        <v>724</v>
+        <v>726</v>
       </c>
       <c r="F1016" s="26" t="s">
-        <v>725</v>
+        <v>727</v>
       </c>
       <c r="G1016" s="16" t="s">
         <v>58</v>
@@ -28186,22 +28226,22 @@
     </row>
     <row r="1022" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1022" s="50" t="s">
-        <v>713</v>
+        <v>715</v>
       </c>
       <c r="B1022" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1022" s="14" t="s">
-        <v>726</v>
+        <v>728</v>
       </c>
       <c r="D1022" s="15" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
       <c r="E1022" s="15" t="s">
-        <v>728</v>
+        <v>730</v>
       </c>
       <c r="F1022" s="15" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
       <c r="G1022" s="16" t="s">
         <v>58</v>
@@ -28330,22 +28370,22 @@
     </row>
     <row r="1028" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1028" s="50" t="s">
-        <v>713</v>
+        <v>715</v>
       </c>
       <c r="B1028" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C1028" s="25" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="D1028" s="26" t="s">
-        <v>731</v>
+        <v>733</v>
       </c>
       <c r="E1028" s="26" t="s">
-        <v>732</v>
+        <v>734</v>
       </c>
       <c r="F1028" s="26" t="s">
-        <v>733</v>
+        <v>735</v>
       </c>
       <c r="G1028" s="16" t="s">
         <v>58</v>
@@ -28474,22 +28514,22 @@
     </row>
     <row r="1034" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1034" s="50" t="s">
-        <v>713</v>
+        <v>715</v>
       </c>
       <c r="B1034" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C1034" s="14" t="s">
-        <v>734</v>
+        <v>736</v>
       </c>
       <c r="D1034" s="15" t="s">
-        <v>735</v>
+        <v>737</v>
       </c>
       <c r="E1034" s="15" t="s">
-        <v>736</v>
+        <v>738</v>
       </c>
       <c r="F1034" s="15" t="s">
-        <v>737</v>
+        <v>739</v>
       </c>
       <c r="G1034" s="16" t="s">
         <v>58</v>
@@ -28618,22 +28658,22 @@
     </row>
     <row r="1040" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1040" s="51" t="s">
-        <v>738</v>
+        <v>740</v>
       </c>
       <c r="B1040" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C1040" s="25" t="s">
-        <v>739</v>
+        <v>741</v>
       </c>
       <c r="D1040" s="26" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
       <c r="E1040" s="26" t="s">
-        <v>740</v>
+        <v>742</v>
       </c>
       <c r="F1040" s="26" t="s">
-        <v>741</v>
+        <v>743</v>
       </c>
       <c r="G1040" s="16" t="s">
         <v>58</v>
@@ -28762,22 +28802,22 @@
     </row>
     <row r="1046" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1046" s="51" t="s">
-        <v>738</v>
+        <v>740</v>
       </c>
       <c r="B1046" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1046" s="14" t="s">
-        <v>742</v>
+        <v>744</v>
       </c>
       <c r="D1046" s="15" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
       <c r="E1046" s="15" t="s">
-        <v>743</v>
+        <v>745</v>
       </c>
       <c r="F1046" s="15" t="s">
-        <v>744</v>
+        <v>746</v>
       </c>
       <c r="G1046" s="16" t="s">
         <v>58</v>
@@ -28914,16 +28954,16 @@
         <v>53</v>
       </c>
       <c r="C1052" s="25" t="s">
-        <v>745</v>
+        <v>747</v>
       </c>
       <c r="D1052" s="26" t="s">
-        <v>746</v>
+        <v>748</v>
       </c>
       <c r="E1052" s="26" t="s">
-        <v>747</v>
+        <v>749</v>
       </c>
       <c r="F1052" s="26" t="s">
-        <v>748</v>
+        <v>750</v>
       </c>
       <c r="G1052" s="16" t="s">
         <v>58</v>
@@ -29060,16 +29100,16 @@
         <v>53</v>
       </c>
       <c r="C1058" s="14" t="s">
-        <v>749</v>
+        <v>751</v>
       </c>
       <c r="D1058" s="15" t="s">
-        <v>750</v>
+        <v>752</v>
       </c>
       <c r="E1058" s="15" t="s">
-        <v>751</v>
+        <v>753</v>
       </c>
       <c r="F1058" s="15" t="s">
-        <v>752</v>
+        <v>754</v>
       </c>
       <c r="G1058" s="16" t="s">
         <v>58</v>
@@ -30155,10 +30195,10 @@
         <v>39</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>753</v>
+        <v>755</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>53</v>
@@ -30176,7 +30216,7 @@
         <v>83</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>755</v>
+        <v>757</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -30616,7 +30656,7 @@
     </row>
     <row r="17" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="67" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="B17" s="1">
         <v>7</v>
@@ -30645,7 +30685,7 @@
     </row>
     <row r="18" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="68" t="s">
-        <v>643</v>
+        <v>645</v>
       </c>
       <c r="B18" s="1">
         <v>6</v>
@@ -30674,7 +30714,7 @@
     </row>
     <row r="19" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="69" t="s">
-        <v>668</v>
+        <v>670</v>
       </c>
       <c r="B19" s="1">
         <v>6</v>
@@ -30703,7 +30743,7 @@
     </row>
     <row r="20" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="70" t="s">
-        <v>692</v>
+        <v>694</v>
       </c>
       <c r="B20" s="1">
         <v>5</v>
@@ -30732,7 +30772,7 @@
     </row>
     <row r="21" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="71" t="s">
-        <v>713</v>
+        <v>715</v>
       </c>
       <c r="B21" s="1">
         <v>6</v>
@@ -30761,7 +30801,7 @@
     </row>
     <row r="22" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="72" t="s">
-        <v>738</v>
+        <v>740</v>
       </c>
       <c r="B22" s="1">
         <v>2</v>
@@ -30790,7 +30830,7 @@
     </row>
     <row r="23" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="73" t="s">
-        <v>756</v>
+        <v>758</v>
       </c>
       <c r="B23" s="73">
         <v>153</v>
@@ -30841,7 +30881,7 @@
         <v>44</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="C1" s="10" t="s">
         <v>71</v>
@@ -30850,7 +30890,7 @@
         <v>83</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>755</v>
+        <v>757</v>
       </c>
       <c r="F1" s="10" t="s">
         <v>97</v>
@@ -31001,10 +31041,10 @@
         <v>45</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>757</v>
+        <v>759</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>71</v>
@@ -31013,7 +31053,7 @@
         <v>83</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>755</v>
+        <v>757</v>
       </c>
       <c r="G1" s="10" t="s">
         <v>97</v>
@@ -31024,7 +31064,7 @@
         <v>59</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>758</v>
+        <v>760</v>
       </c>
       <c r="C2" s="1">
         <f>COUNTIF(Proves!$H:$H,A2)</f>
@@ -31154,7 +31194,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="83" t="s">
-        <v>759</v>
+        <v>761</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -31162,7 +31202,7 @@
         <v>71</v>
       </c>
       <c r="B2" s="84" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
@@ -31182,7 +31222,7 @@
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>602</v>
+        <v>628</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
100 => fase IV => fitxa sense copy inventada (És una veterinària), xips botiga+vet, confirmar mascotes trucant, ZUP-058 KO/corr (Chrome/USER)
</commit_message>
<xml_diff>
--- a/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
+++ b/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4444" uniqueCount="763">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4447" uniqueCount="764">
   <si>
     <t>Zuppeto — Joc de probes manual (totes les pantalles)</t>
   </si>
@@ -1076,6 +1076,16 @@
   <si>
     <t xml:space="preserve">«Què hi trobaràs» buit (caixa blanca, sense etiquetes).
 Cal omplir característiques útils (gos dins / només terrassa / no es permet, etc.). Si no hi són a la BD, consultar web/detall del local. No deixar la targeta buida.</t>
+  </si>
+  <si>
+    <t>06-09-2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Què s'ha fet:
+- Què hi trobaràs: si és botiga d'animals, es mostren xips de botiga i es queden els de veterinària
+- Context ràpid: ja no s'inventa «És una veterinària.» (només text real de Google/web)
+- Abans d'anar-hi: si no hi ha dada pet-friendly, cal confirmar trucant al local
+- docs/ca/funcional-ca.md, docs/ca/tecnic-ca.md</t>
   </si>
   <si>
     <t>ZUP-059</t>
@@ -1855,9 +1865,6 @@
 La bio tenia un mínim de 12 caràcters que no correspon (només no pot ser buida).</t>
   </si>
   <si>
-    <t>06-09-2026</t>
-  </si>
-  <si>
     <t xml:space="preserve">Què s’ha fet: si qui opera és Administrador, no es mostra ni es valida el check de condicions (policy AdminExemptPrivacyConsentPolicy, com al perfil).
 El desar de fitxa va a PUT /api/admin/users/{id} (UpdateAdminUserCommand + User.ReplaceProfile), no al perfil propi.
 La bio és obligatòria i sense mínim de longitud.
@@ -2430,7 +2437,7 @@
     </font>
     <font>
       <b/>
-      <color rgb="FF1D4ED8"/>
+      <color rgb="FF166534"/>
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
@@ -2599,7 +2606,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFDBEAFE"/>
+        <fgColor rgb="FFDCFCE7"/>
       </patternFill>
     </fill>
     <fill>
@@ -14042,9 +14049,15 @@
       <c r="K434" s="19" t="s">
         <v>344</v>
       </c>
-      <c r="L434" s="18"/>
-      <c r="M434" s="1"/>
-      <c r="N434" s="19"/>
+      <c r="L434" s="18" t="s">
+        <v>345</v>
+      </c>
+      <c r="M434" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="N434" s="19" t="s">
+        <v>346</v>
+      </c>
     </row>
     <row r="435" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A435" s="37"/>
@@ -14164,16 +14177,16 @@
         <v>92</v>
       </c>
       <c r="C440" s="14" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="D440" s="15" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="E440" s="15" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="F440" s="15" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="G440" s="16" t="s">
         <v>58</v>
@@ -14310,16 +14323,16 @@
         <v>53</v>
       </c>
       <c r="C446" s="25" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="D446" s="26" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="E446" s="26" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="F446" s="26" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="G446" s="16" t="s">
         <v>58</v>
@@ -14334,7 +14347,7 @@
         <v>83</v>
       </c>
       <c r="K446" s="19" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="L446" s="18" t="s">
         <v>213</v>
@@ -14343,7 +14356,7 @@
         <v>71</v>
       </c>
       <c r="N446" s="19" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
     </row>
     <row r="447" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -14464,16 +14477,16 @@
         <v>92</v>
       </c>
       <c r="C452" s="14" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="D452" s="15" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="E452" s="15" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="F452" s="15" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="G452" s="16" t="s">
         <v>58</v>
@@ -14610,16 +14623,16 @@
         <v>92</v>
       </c>
       <c r="C458" s="25" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="D458" s="26" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="E458" s="26" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="F458" s="26" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="G458" s="16" t="s">
         <v>58</v>
@@ -14756,16 +14769,16 @@
         <v>92</v>
       </c>
       <c r="C464" s="14" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="D464" s="15" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="E464" s="15" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="F464" s="15" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="G464" s="16" t="s">
         <v>58</v>
@@ -14902,16 +14915,16 @@
         <v>53</v>
       </c>
       <c r="C470" s="25" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="D470" s="26" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="E470" s="26" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="F470" s="26" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="G470" s="16" t="s">
         <v>58</v>
@@ -15042,22 +15055,22 @@
     </row>
     <row r="476" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A476" s="38" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B476" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C476" s="14" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="D476" s="15" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="E476" s="15" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="F476" s="15" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="G476" s="16" t="s">
         <v>58</v>
@@ -15072,7 +15085,7 @@
         <v>71</v>
       </c>
       <c r="K476" s="19" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="L476" s="18"/>
       <c r="M476" s="1"/>
@@ -15190,22 +15203,22 @@
     </row>
     <row r="482" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A482" s="38" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B482" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C482" s="25" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="D482" s="26" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="E482" s="26" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="F482" s="26" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="G482" s="16" t="s">
         <v>58</v>
@@ -15220,7 +15233,7 @@
         <v>71</v>
       </c>
       <c r="K482" s="19" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="L482" s="18"/>
       <c r="M482" s="1"/>
@@ -15338,22 +15351,22 @@
     </row>
     <row r="488" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A488" s="38" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B488" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C488" s="14" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="D488" s="15" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="E488" s="15" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="F488" s="15" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="G488" s="16" t="s">
         <v>58</v>
@@ -15484,22 +15497,22 @@
     </row>
     <row r="494" ht="110" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A494" s="38" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B494" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C494" s="25" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="D494" s="26" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="E494" s="26" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="F494" s="26" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="G494" s="16" t="s">
         <v>58</v>
@@ -15514,7 +15527,7 @@
         <v>83</v>
       </c>
       <c r="K494" s="19" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="L494" s="18" t="s">
         <v>82</v>
@@ -15523,7 +15536,7 @@
         <v>71</v>
       </c>
       <c r="N494" s="19" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
     </row>
     <row r="495" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -15638,22 +15651,22 @@
     </row>
     <row r="500" ht="96" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A500" s="38" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B500" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C500" s="14" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="D500" s="15" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="E500" s="15" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="F500" s="15" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="G500" s="16" t="s">
         <v>58</v>
@@ -15668,7 +15681,7 @@
         <v>83</v>
       </c>
       <c r="K500" s="19" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="L500" s="18" t="s">
         <v>82</v>
@@ -15677,7 +15690,7 @@
         <v>71</v>
       </c>
       <c r="N500" s="19" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
     </row>
     <row r="501" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -15792,22 +15805,22 @@
     </row>
     <row r="506" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A506" s="38" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B506" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C506" s="25" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="D506" s="26" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="E506" s="26" t="s">
         <v>257</v>
       </c>
       <c r="F506" s="26" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="G506" s="16" t="s">
         <v>58</v>
@@ -15938,22 +15951,22 @@
     </row>
     <row r="512" ht="80" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A512" s="38" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B512" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C512" s="14" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="D512" s="15" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="E512" s="15" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="F512" s="15" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="G512" s="16" t="s">
         <v>58</v>
@@ -15968,7 +15981,7 @@
         <v>83</v>
       </c>
       <c r="K512" s="19" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="L512" s="18" t="s">
         <v>82</v>
@@ -15977,7 +15990,7 @@
         <v>71</v>
       </c>
       <c r="N512" s="19" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
     </row>
     <row r="513" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -16092,22 +16105,22 @@
     </row>
     <row r="518" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A518" s="38" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B518" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C518" s="25" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="D518" s="26" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="E518" s="26" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="F518" s="26" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="G518" s="16" t="s">
         <v>58</v>
@@ -16238,22 +16251,22 @@
     </row>
     <row r="524" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A524" s="38" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B524" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C524" s="14" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="D524" s="15" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="E524" s="15" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="F524" s="15" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="G524" s="16" t="s">
         <v>58</v>
@@ -16384,22 +16397,22 @@
     </row>
     <row r="530" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A530" s="38" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B530" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C530" s="25" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="D530" s="26" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="E530" s="26" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="F530" s="26" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="G530" s="16" t="s">
         <v>58</v>
@@ -16530,22 +16543,22 @@
     </row>
     <row r="536" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A536" s="38" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B536" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C536" s="14" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="D536" s="15" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="E536" s="15" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="F536" s="15" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="G536" s="16" t="s">
         <v>58</v>
@@ -16676,22 +16689,22 @@
     </row>
     <row r="542" ht="180" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A542" s="39" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B542" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C542" s="25" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="D542" s="26" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="E542" s="26" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="F542" s="26" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="G542" s="16" t="s">
         <v>58</v>
@@ -16706,7 +16719,7 @@
         <v>83</v>
       </c>
       <c r="K542" s="19" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="L542" s="18">
         <v>46264.91666666667</v>
@@ -16715,7 +16728,7 @@
         <v>71</v>
       </c>
       <c r="N542" s="19" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
     </row>
     <row r="543" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -16830,22 +16843,22 @@
     </row>
     <row r="548" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A548" s="39" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B548" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C548" s="14" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="D548" s="15" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="E548" s="15" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="F548" s="15" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="G548" s="16" t="s">
         <v>58</v>
@@ -16976,22 +16989,22 @@
     </row>
     <row r="554" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A554" s="39" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B554" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C554" s="25" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="D554" s="26" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="E554" s="26" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="F554" s="26" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="G554" s="16" t="s">
         <v>58</v>
@@ -17122,22 +17135,22 @@
     </row>
     <row r="560" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A560" s="39" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B560" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C560" s="14" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="D560" s="15" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="E560" s="15" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="F560" s="15" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="G560" s="16" t="s">
         <v>58</v>
@@ -17268,22 +17281,22 @@
     </row>
     <row r="566" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A566" s="39" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B566" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C566" s="25" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="D566" s="26" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="E566" s="26" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="F566" s="26" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="G566" s="16" t="s">
         <v>58</v>
@@ -17414,22 +17427,22 @@
     </row>
     <row r="572" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A572" s="39" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B572" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C572" s="14" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="D572" s="15" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="E572" s="15" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="F572" s="15" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="G572" s="16" t="s">
         <v>58</v>
@@ -17560,22 +17573,22 @@
     </row>
     <row r="578" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A578" s="39" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B578" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C578" s="25" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="D578" s="26" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="E578" s="26" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="F578" s="26" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="G578" s="16" t="s">
         <v>58</v>
@@ -17706,22 +17719,22 @@
     </row>
     <row r="584" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A584" s="39" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B584" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C584" s="14" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="D584" s="15" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="E584" s="15" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="F584" s="15" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="G584" s="16" t="s">
         <v>58</v>
@@ -17850,22 +17863,22 @@
     </row>
     <row r="590" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A590" s="39" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B590" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C590" s="25" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="D590" s="26" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="E590" s="26" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="F590" s="26" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="G590" s="16" t="s">
         <v>58</v>
@@ -17996,22 +18009,22 @@
     </row>
     <row r="596" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A596" s="40" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="B596" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C596" s="14" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="D596" s="15" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="E596" s="15" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="F596" s="15" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="G596" s="16" t="s">
         <v>58</v>
@@ -18160,7 +18173,7 @@
         <v>83</v>
       </c>
       <c r="K602" s="19" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="L602" s="18">
         <v>46264.91666666667</v>
@@ -18169,7 +18182,7 @@
         <v>71</v>
       </c>
       <c r="N602" s="19" t="s">
-        <v>468</v>
+        <v>470</v>
       </c>
     </row>
     <row r="603" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -18548,22 +18561,22 @@
     </row>
     <row r="620" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A620" s="40" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="B620" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C620" s="25" t="s">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="D620" s="26" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="E620" s="26" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="F620" s="26" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="G620" s="16" t="s">
         <v>58</v>
@@ -18694,22 +18707,22 @@
     </row>
     <row r="626" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A626" s="40" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="B626" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C626" s="14" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="D626" s="15" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="E626" s="15" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="F626" s="15" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="G626" s="16" t="s">
         <v>58</v>
@@ -18840,22 +18853,22 @@
     </row>
     <row r="632" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A632" s="40" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="B632" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C632" s="25" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="D632" s="26" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="E632" s="26" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="F632" s="26" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="G632" s="16" t="s">
         <v>58</v>
@@ -18986,22 +18999,22 @@
     </row>
     <row r="638" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A638" s="40" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="B638" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C638" s="14" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="D638" s="15" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="E638" s="15" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="F638" s="15" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="G638" s="16" t="s">
         <v>58</v>
@@ -19132,22 +19145,22 @@
     </row>
     <row r="644" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A644" s="41" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="B644" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C644" s="25" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="D644" s="26" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="E644" s="26" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="F644" s="26" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="G644" s="16" t="s">
         <v>58</v>
@@ -19676,22 +19689,22 @@
     </row>
     <row r="668" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A668" s="41" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="B668" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C668" s="14" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="D668" s="15" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="E668" s="15" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="F668" s="15" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="G668" s="16" t="s">
         <v>58</v>
@@ -19822,22 +19835,22 @@
     </row>
     <row r="674" ht="88" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A674" s="41" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="B674" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C674" s="25" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="D674" s="26" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="E674" s="26" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="F674" s="26" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="G674" s="16" t="s">
         <v>58</v>
@@ -19852,7 +19865,7 @@
         <v>83</v>
       </c>
       <c r="K674" s="19" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="L674" s="18" t="s">
         <v>82</v>
@@ -19861,7 +19874,7 @@
         <v>71</v>
       </c>
       <c r="N674" s="19" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
     </row>
     <row r="675" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -19976,22 +19989,22 @@
     </row>
     <row r="680" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A680" s="41" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="B680" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C680" s="14" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="D680" s="15" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="E680" s="15" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="F680" s="15" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="G680" s="16" t="s">
         <v>58</v>
@@ -20122,22 +20135,22 @@
     </row>
     <row r="686" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A686" s="41" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="B686" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C686" s="25" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="D686" s="26" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="E686" s="26" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="F686" s="26" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="G686" s="16" t="s">
         <v>58</v>
@@ -20268,22 +20281,22 @@
     </row>
     <row r="692" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A692" s="42" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="B692" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C692" s="14" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="D692" s="15" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="E692" s="15" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="F692" s="15" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="G692" s="16" t="s">
         <v>58</v>
@@ -20812,22 +20825,22 @@
     </row>
     <row r="716" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A716" s="42" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="B716" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C716" s="25" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="D716" s="26" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="E716" s="26" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="F716" s="26" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="G716" s="16" t="s">
         <v>58</v>
@@ -20958,22 +20971,22 @@
     </row>
     <row r="722" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A722" s="42" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="B722" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C722" s="14" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="D722" s="15" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="E722" s="15" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="F722" s="15" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="G722" s="16" t="s">
         <v>58</v>
@@ -20988,7 +21001,7 @@
         <v>71</v>
       </c>
       <c r="K722" s="19" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="L722" s="18"/>
       <c r="M722" s="1"/>
@@ -21106,19 +21119,19 @@
     </row>
     <row r="728" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A728" s="42" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="B728" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C728" s="25" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="D728" s="26" t="s">
         <v>219</v>
       </c>
       <c r="E728" s="26" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="F728" s="26" t="s">
         <v>221</v>
@@ -21252,22 +21265,22 @@
     </row>
     <row r="734" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A734" s="43" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="B734" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C734" s="14" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="D734" s="15" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="E734" s="15" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="F734" s="15" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="G734" s="16" t="s">
         <v>58</v>
@@ -21398,22 +21411,22 @@
     </row>
     <row r="740" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A740" s="43" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="B740" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C740" s="25" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="D740" s="26" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="E740" s="26" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="F740" s="26" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="G740" s="16" t="s">
         <v>58</v>
@@ -21428,7 +21441,7 @@
         <v>83</v>
       </c>
       <c r="K740" s="19" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="L740" s="18" t="s">
         <v>82</v>
@@ -21437,7 +21450,7 @@
         <v>71</v>
       </c>
       <c r="N740" s="19" t="s">
-        <v>532</v>
+        <v>534</v>
       </c>
     </row>
     <row r="741" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -21552,22 +21565,22 @@
     </row>
     <row r="746" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A746" s="43" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="B746" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C746" s="14" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="D746" s="15" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="E746" s="15" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="F746" s="15" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="G746" s="16" t="s">
         <v>58</v>
@@ -21698,22 +21711,22 @@
     </row>
     <row r="752" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A752" s="43" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="B752" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C752" s="25" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="D752" s="26" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="E752" s="26" t="s">
-        <v>539</v>
+        <v>541</v>
       </c>
       <c r="F752" s="26" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="G752" s="16" t="s">
         <v>58</v>
@@ -21844,22 +21857,22 @@
     </row>
     <row r="758" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A758" s="43" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="B758" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C758" s="14" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="D758" s="15" t="s">
-        <v>542</v>
+        <v>544</v>
       </c>
       <c r="E758" s="15" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="F758" s="15" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="G758" s="16" t="s">
         <v>58</v>
@@ -21990,22 +22003,22 @@
     </row>
     <row r="764" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A764" s="44" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="B764" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C764" s="25" t="s">
-        <v>546</v>
+        <v>548</v>
       </c>
       <c r="D764" s="26" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="E764" s="26" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="F764" s="26" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
       <c r="G764" s="16" t="s">
         <v>58</v>
@@ -22136,22 +22149,22 @@
     </row>
     <row r="770" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A770" s="44" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="B770" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C770" s="14" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="D770" s="15" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="E770" s="15" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="F770" s="15" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="G770" s="16" t="s">
         <v>58</v>
@@ -22282,22 +22295,22 @@
     </row>
     <row r="776" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A776" s="44" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="B776" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C776" s="25" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="D776" s="26" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="E776" s="26" t="s">
-        <v>556</v>
+        <v>558</v>
       </c>
       <c r="F776" s="26" t="s">
-        <v>557</v>
+        <v>559</v>
       </c>
       <c r="G776" s="16" t="s">
         <v>58</v>
@@ -22428,22 +22441,22 @@
     </row>
     <row r="782" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A782" s="44" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="B782" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C782" s="14" t="s">
-        <v>558</v>
+        <v>560</v>
       </c>
       <c r="D782" s="15" t="s">
-        <v>559</v>
+        <v>561</v>
       </c>
       <c r="E782" s="15" t="s">
-        <v>560</v>
+        <v>562</v>
       </c>
       <c r="F782" s="15" t="s">
-        <v>561</v>
+        <v>563</v>
       </c>
       <c r="G782" s="16" t="s">
         <v>58</v>
@@ -22572,22 +22585,22 @@
     </row>
     <row r="788" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A788" s="44" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="B788" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C788" s="25" t="s">
-        <v>562</v>
+        <v>564</v>
       </c>
       <c r="D788" s="26" t="s">
-        <v>563</v>
+        <v>565</v>
       </c>
       <c r="E788" s="26" t="s">
-        <v>564</v>
+        <v>566</v>
       </c>
       <c r="F788" s="26" t="s">
-        <v>565</v>
+        <v>567</v>
       </c>
       <c r="G788" s="16" t="s">
         <v>58</v>
@@ -22596,7 +22609,7 @@
         <v>81</v>
       </c>
       <c r="I788" s="18" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="J788" s="1" t="s">
         <v>71</v>
@@ -22718,22 +22731,22 @@
     </row>
     <row r="794" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A794" s="44" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="B794" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C794" s="14" t="s">
+        <v>569</v>
+      </c>
+      <c r="D794" s="15" t="s">
+        <v>570</v>
+      </c>
+      <c r="E794" s="15" t="s">
+        <v>571</v>
+      </c>
+      <c r="F794" s="15" t="s">
         <v>567</v>
-      </c>
-      <c r="D794" s="15" t="s">
-        <v>568</v>
-      </c>
-      <c r="E794" s="15" t="s">
-        <v>569</v>
-      </c>
-      <c r="F794" s="15" t="s">
-        <v>565</v>
       </c>
       <c r="G794" s="16" t="s">
         <v>58</v>
@@ -22862,22 +22875,22 @@
     </row>
     <row r="800" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A800" s="44" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="B800" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C800" s="25" t="s">
-        <v>570</v>
+        <v>572</v>
       </c>
       <c r="D800" s="26" t="s">
-        <v>571</v>
+        <v>573</v>
       </c>
       <c r="E800" s="26" t="s">
-        <v>572</v>
+        <v>574</v>
       </c>
       <c r="F800" s="26" t="s">
-        <v>573</v>
+        <v>575</v>
       </c>
       <c r="G800" s="16" t="s">
         <v>58</v>
@@ -22886,7 +22899,7 @@
         <v>81</v>
       </c>
       <c r="I800" s="18" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="J800" s="1" t="s">
         <v>71</v>
@@ -23008,22 +23021,22 @@
     </row>
     <row r="806" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A806" s="44" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="B806" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C806" s="14" t="s">
-        <v>574</v>
+        <v>576</v>
       </c>
       <c r="D806" s="15" t="s">
-        <v>575</v>
+        <v>577</v>
       </c>
       <c r="E806" s="15" t="s">
-        <v>576</v>
+        <v>578</v>
       </c>
       <c r="F806" s="15" t="s">
-        <v>577</v>
+        <v>579</v>
       </c>
       <c r="G806" s="16" t="s">
         <v>58</v>
@@ -23032,7 +23045,7 @@
         <v>81</v>
       </c>
       <c r="I806" s="18" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="J806" s="1" t="s">
         <v>71</v>
@@ -23154,22 +23167,22 @@
     </row>
     <row r="812" ht="90" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A812" s="44" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="B812" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C812" s="25" t="s">
-        <v>578</v>
+        <v>580</v>
       </c>
       <c r="D812" s="26" t="s">
-        <v>579</v>
+        <v>581</v>
       </c>
       <c r="E812" s="26" t="s">
-        <v>580</v>
+        <v>582</v>
       </c>
       <c r="F812" s="26" t="s">
-        <v>581</v>
+        <v>583</v>
       </c>
       <c r="G812" s="16" t="s">
         <v>58</v>
@@ -23178,22 +23191,22 @@
         <v>81</v>
       </c>
       <c r="I812" s="18" t="s">
-        <v>566</v>
+        <v>568</v>
       </c>
       <c r="J812" s="1" t="s">
         <v>83</v>
       </c>
       <c r="K812" s="19" t="s">
-        <v>582</v>
+        <v>584</v>
       </c>
       <c r="L812" s="18" t="s">
-        <v>583</v>
+        <v>345</v>
       </c>
       <c r="M812" s="1" t="s">
         <v>71</v>
       </c>
       <c r="N812" s="19" t="s">
-        <v>584</v>
+        <v>585</v>
       </c>
     </row>
     <row r="813" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -23308,22 +23321,22 @@
     </row>
     <row r="818" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A818" s="44" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="B818" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C818" s="14" t="s">
-        <v>585</v>
+        <v>586</v>
       </c>
       <c r="D818" s="15" t="s">
-        <v>586</v>
+        <v>587</v>
       </c>
       <c r="E818" s="15" t="s">
-        <v>587</v>
+        <v>588</v>
       </c>
       <c r="F818" s="15" t="s">
-        <v>588</v>
+        <v>589</v>
       </c>
       <c r="G818" s="16" t="s">
         <v>58</v>
@@ -23452,22 +23465,22 @@
     </row>
     <row r="824" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A824" s="44" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="B824" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C824" s="25" t="s">
-        <v>589</v>
+        <v>590</v>
       </c>
       <c r="D824" s="26" t="s">
-        <v>590</v>
+        <v>591</v>
       </c>
       <c r="E824" s="26" t="s">
-        <v>591</v>
+        <v>592</v>
       </c>
       <c r="F824" s="26" t="s">
-        <v>592</v>
+        <v>593</v>
       </c>
       <c r="G824" s="16" t="s">
         <v>58</v>
@@ -23476,7 +23489,7 @@
         <v>81</v>
       </c>
       <c r="I824" s="18" t="s">
-        <v>583</v>
+        <v>345</v>
       </c>
       <c r="J824" s="1" t="s">
         <v>71</v>
@@ -23598,22 +23611,22 @@
     </row>
     <row r="830" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A830" s="44" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="B830" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C830" s="14" t="s">
-        <v>593</v>
+        <v>594</v>
       </c>
       <c r="D830" s="15" t="s">
-        <v>594</v>
+        <v>595</v>
       </c>
       <c r="E830" s="15" t="s">
-        <v>595</v>
+        <v>596</v>
       </c>
       <c r="F830" s="15" t="s">
-        <v>596</v>
+        <v>597</v>
       </c>
       <c r="G830" s="16" t="s">
         <v>58</v>
@@ -23742,22 +23755,22 @@
     </row>
     <row r="836" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A836" s="45" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="B836" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C836" s="25" t="s">
-        <v>598</v>
+        <v>599</v>
       </c>
       <c r="D836" s="26" t="s">
-        <v>599</v>
+        <v>600</v>
       </c>
       <c r="E836" s="26" t="s">
-        <v>600</v>
+        <v>601</v>
       </c>
       <c r="F836" s="26" t="s">
-        <v>601</v>
+        <v>602</v>
       </c>
       <c r="G836" s="16" t="s">
         <v>58</v>
@@ -23766,7 +23779,7 @@
         <v>81</v>
       </c>
       <c r="I836" s="18" t="s">
-        <v>583</v>
+        <v>345</v>
       </c>
       <c r="J836" s="1" t="s">
         <v>71</v>
@@ -23888,22 +23901,22 @@
     </row>
     <row r="842" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A842" s="45" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="B842" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C842" s="14" t="s">
-        <v>602</v>
+        <v>603</v>
       </c>
       <c r="D842" s="15" t="s">
-        <v>603</v>
+        <v>604</v>
       </c>
       <c r="E842" s="15" t="s">
-        <v>604</v>
+        <v>605</v>
       </c>
       <c r="F842" s="15" t="s">
-        <v>536</v>
+        <v>538</v>
       </c>
       <c r="G842" s="16" t="s">
         <v>58</v>
@@ -23912,7 +23925,7 @@
         <v>81</v>
       </c>
       <c r="I842" s="18" t="s">
-        <v>583</v>
+        <v>345</v>
       </c>
       <c r="J842" s="1" t="s">
         <v>71</v>
@@ -24034,22 +24047,22 @@
     </row>
     <row r="848" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A848" s="45" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="B848" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C848" s="25" t="s">
-        <v>605</v>
+        <v>606</v>
       </c>
       <c r="D848" s="26" t="s">
-        <v>606</v>
+        <v>607</v>
       </c>
       <c r="E848" s="26" t="s">
-        <v>607</v>
+        <v>608</v>
       </c>
       <c r="F848" s="26" t="s">
-        <v>608</v>
+        <v>609</v>
       </c>
       <c r="G848" s="16" t="s">
         <v>58</v>
@@ -24178,22 +24191,22 @@
     </row>
     <row r="854" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A854" s="45" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="B854" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C854" s="14" t="s">
-        <v>609</v>
+        <v>610</v>
       </c>
       <c r="D854" s="15" t="s">
-        <v>610</v>
+        <v>611</v>
       </c>
       <c r="E854" s="15" t="s">
-        <v>611</v>
+        <v>612</v>
       </c>
       <c r="F854" s="15" t="s">
-        <v>612</v>
+        <v>613</v>
       </c>
       <c r="G854" s="16" t="s">
         <v>58</v>
@@ -24202,7 +24215,7 @@
         <v>81</v>
       </c>
       <c r="I854" s="18" t="s">
-        <v>583</v>
+        <v>345</v>
       </c>
       <c r="J854" s="1" t="s">
         <v>71</v>
@@ -24324,22 +24337,22 @@
     </row>
     <row r="860" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A860" s="46" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="B860" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C860" s="25" t="s">
-        <v>614</v>
+        <v>615</v>
       </c>
       <c r="D860" s="26" t="s">
-        <v>615</v>
+        <v>616</v>
       </c>
       <c r="E860" s="26" t="s">
-        <v>616</v>
+        <v>617</v>
       </c>
       <c r="F860" s="26" t="s">
-        <v>617</v>
+        <v>618</v>
       </c>
       <c r="G860" s="16" t="s">
         <v>58</v>
@@ -24348,7 +24361,7 @@
         <v>81</v>
       </c>
       <c r="I860" s="18" t="s">
-        <v>583</v>
+        <v>345</v>
       </c>
       <c r="J860" s="1" t="s">
         <v>71</v>
@@ -24470,22 +24483,22 @@
     </row>
     <row r="866" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A866" s="46" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="B866" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C866" s="14" t="s">
-        <v>618</v>
+        <v>619</v>
       </c>
       <c r="D866" s="15" t="s">
-        <v>619</v>
+        <v>620</v>
       </c>
       <c r="E866" s="15" t="s">
-        <v>620</v>
+        <v>621</v>
       </c>
       <c r="F866" s="15" t="s">
-        <v>621</v>
+        <v>622</v>
       </c>
       <c r="G866" s="16" t="s">
         <v>58</v>
@@ -24494,22 +24507,22 @@
         <v>81</v>
       </c>
       <c r="I866" s="18" t="s">
-        <v>583</v>
+        <v>345</v>
       </c>
       <c r="J866" s="1" t="s">
         <v>83</v>
       </c>
       <c r="K866" s="19" t="s">
-        <v>622</v>
+        <v>623</v>
       </c>
       <c r="L866" s="18" t="s">
-        <v>583</v>
+        <v>345</v>
       </c>
       <c r="M866" s="1" t="s">
         <v>71</v>
       </c>
       <c r="N866" s="19" t="s">
-        <v>623</v>
+        <v>624</v>
       </c>
     </row>
     <row r="867" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
@@ -24624,22 +24637,22 @@
     </row>
     <row r="872" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A872" s="46" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="B872" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C872" s="25" t="s">
-        <v>624</v>
+        <v>625</v>
       </c>
       <c r="D872" s="26" t="s">
-        <v>625</v>
+        <v>626</v>
       </c>
       <c r="E872" s="26" t="s">
-        <v>626</v>
+        <v>627</v>
       </c>
       <c r="F872" s="26" t="s">
-        <v>627</v>
+        <v>628</v>
       </c>
       <c r="G872" s="16" t="s">
         <v>58</v>
@@ -24648,10 +24661,10 @@
         <v>81</v>
       </c>
       <c r="I872" s="18" t="s">
-        <v>583</v>
+        <v>345</v>
       </c>
       <c r="J872" s="1" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
       <c r="K872" s="19"/>
       <c r="L872" s="18"/>
@@ -24770,22 +24783,22 @@
     </row>
     <row r="878" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A878" s="46" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="B878" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C878" s="14" t="s">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="D878" s="15" t="s">
-        <v>630</v>
+        <v>631</v>
       </c>
       <c r="E878" s="15" t="s">
-        <v>631</v>
+        <v>632</v>
       </c>
       <c r="F878" s="15" t="s">
-        <v>632</v>
+        <v>633</v>
       </c>
       <c r="G878" s="16" t="s">
         <v>58</v>
@@ -24914,22 +24927,22 @@
     </row>
     <row r="884" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A884" s="46" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="B884" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C884" s="25" t="s">
-        <v>633</v>
+        <v>634</v>
       </c>
       <c r="D884" s="26" t="s">
-        <v>634</v>
+        <v>635</v>
       </c>
       <c r="E884" s="26" t="s">
-        <v>635</v>
+        <v>636</v>
       </c>
       <c r="F884" s="26" t="s">
-        <v>636</v>
+        <v>637</v>
       </c>
       <c r="G884" s="16" t="s">
         <v>58</v>
@@ -25058,22 +25071,22 @@
     </row>
     <row r="890" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A890" s="46" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="B890" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C890" s="14" t="s">
-        <v>637</v>
+        <v>638</v>
       </c>
       <c r="D890" s="15" t="s">
-        <v>638</v>
+        <v>639</v>
       </c>
       <c r="E890" s="15" t="s">
-        <v>639</v>
+        <v>640</v>
       </c>
       <c r="F890" s="15" t="s">
-        <v>640</v>
+        <v>641</v>
       </c>
       <c r="G890" s="16" t="s">
         <v>58</v>
@@ -25202,22 +25215,22 @@
     </row>
     <row r="896" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A896" s="46" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="B896" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C896" s="25" t="s">
-        <v>641</v>
+        <v>642</v>
       </c>
       <c r="D896" s="26" t="s">
-        <v>642</v>
+        <v>643</v>
       </c>
       <c r="E896" s="26" t="s">
-        <v>643</v>
+        <v>644</v>
       </c>
       <c r="F896" s="26" t="s">
-        <v>644</v>
+        <v>645</v>
       </c>
       <c r="G896" s="16" t="s">
         <v>58</v>
@@ -25346,22 +25359,22 @@
     </row>
     <row r="902" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A902" s="47" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="B902" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C902" s="14" t="s">
-        <v>646</v>
+        <v>647</v>
       </c>
       <c r="D902" s="15" t="s">
-        <v>647</v>
+        <v>648</v>
       </c>
       <c r="E902" s="15" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="F902" s="15" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="G902" s="16" t="s">
         <v>58</v>
@@ -25490,22 +25503,22 @@
     </row>
     <row r="908" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A908" s="47" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="B908" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C908" s="25" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="D908" s="26" t="s">
-        <v>651</v>
+        <v>652</v>
       </c>
       <c r="E908" s="26" t="s">
-        <v>652</v>
+        <v>653</v>
       </c>
       <c r="F908" s="26" t="s">
-        <v>653</v>
+        <v>654</v>
       </c>
       <c r="G908" s="16" t="s">
         <v>58</v>
@@ -25634,22 +25647,22 @@
     </row>
     <row r="914" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A914" s="47" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="B914" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C914" s="14" t="s">
-        <v>654</v>
+        <v>655</v>
       </c>
       <c r="D914" s="15" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="E914" s="15" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="F914" s="15" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="G914" s="16" t="s">
         <v>58</v>
@@ -25778,22 +25791,22 @@
     </row>
     <row r="920" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A920" s="47" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="B920" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C920" s="25" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="D920" s="26" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="E920" s="26" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="F920" s="26" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="G920" s="16" t="s">
         <v>58</v>
@@ -25922,22 +25935,22 @@
     </row>
     <row r="926" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A926" s="47" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="B926" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C926" s="14" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="D926" s="15" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="E926" s="15" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="F926" s="15" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="G926" s="16" t="s">
         <v>58</v>
@@ -26066,22 +26079,22 @@
     </row>
     <row r="932" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A932" s="47" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="B932" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C932" s="25" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="D932" s="26" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="E932" s="26" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="F932" s="26" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="G932" s="16" t="s">
         <v>58</v>
@@ -26210,22 +26223,22 @@
     </row>
     <row r="938" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A938" s="48" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="B938" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C938" s="14" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="D938" s="15" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="E938" s="15" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="F938" s="15" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="G938" s="16" t="s">
         <v>58</v>
@@ -26354,22 +26367,22 @@
     </row>
     <row r="944" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A944" s="48" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="B944" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C944" s="25" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="D944" s="26" t="s">
-        <v>676</v>
+        <v>677</v>
       </c>
       <c r="E944" s="26" t="s">
-        <v>677</v>
+        <v>678</v>
       </c>
       <c r="F944" s="26" t="s">
-        <v>678</v>
+        <v>679</v>
       </c>
       <c r="G944" s="16" t="s">
         <v>58</v>
@@ -26498,22 +26511,22 @@
     </row>
     <row r="950" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A950" s="48" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="B950" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C950" s="14" t="s">
-        <v>679</v>
+        <v>680</v>
       </c>
       <c r="D950" s="15" t="s">
-        <v>680</v>
+        <v>681</v>
       </c>
       <c r="E950" s="15" t="s">
-        <v>681</v>
+        <v>682</v>
       </c>
       <c r="F950" s="15" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="G950" s="16" t="s">
         <v>58</v>
@@ -26642,22 +26655,22 @@
     </row>
     <row r="956" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A956" s="48" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="B956" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C956" s="25" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="D956" s="26" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="E956" s="26" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="F956" s="26" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="G956" s="16" t="s">
         <v>58</v>
@@ -26786,22 +26799,22 @@
     </row>
     <row r="962" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A962" s="48" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="B962" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C962" s="14" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="D962" s="15" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="E962" s="15" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="F962" s="15" t="s">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="G962" s="16" t="s">
         <v>58</v>
@@ -26930,22 +26943,22 @@
     </row>
     <row r="968" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A968" s="48" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="B968" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C968" s="25" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="D968" s="26" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="E968" s="26" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="F968" s="26" t="s">
-        <v>693</v>
+        <v>694</v>
       </c>
       <c r="G968" s="16" t="s">
         <v>58</v>
@@ -27074,22 +27087,22 @@
     </row>
     <row r="974" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A974" s="49" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="B974" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C974" s="14" t="s">
-        <v>695</v>
+        <v>696</v>
       </c>
       <c r="D974" s="15" t="s">
-        <v>696</v>
+        <v>697</v>
       </c>
       <c r="E974" s="15" t="s">
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="F974" s="15" t="s">
-        <v>698</v>
+        <v>699</v>
       </c>
       <c r="G974" s="16" t="s">
         <v>58</v>
@@ -27218,22 +27231,22 @@
     </row>
     <row r="980" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A980" s="49" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="B980" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C980" s="25" t="s">
-        <v>699</v>
+        <v>700</v>
       </c>
       <c r="D980" s="26" t="s">
-        <v>700</v>
+        <v>701</v>
       </c>
       <c r="E980" s="26" t="s">
-        <v>701</v>
+        <v>702</v>
       </c>
       <c r="F980" s="26" t="s">
-        <v>702</v>
+        <v>703</v>
       </c>
       <c r="G980" s="16" t="s">
         <v>58</v>
@@ -27362,22 +27375,22 @@
     </row>
     <row r="986" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A986" s="49" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="B986" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C986" s="14" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="D986" s="15" t="s">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="E986" s="15" t="s">
-        <v>705</v>
+        <v>706</v>
       </c>
       <c r="F986" s="15" t="s">
-        <v>706</v>
+        <v>707</v>
       </c>
       <c r="G986" s="16" t="s">
         <v>58</v>
@@ -27506,22 +27519,22 @@
     </row>
     <row r="992" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A992" s="49" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="B992" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C992" s="25" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="D992" s="26" t="s">
-        <v>708</v>
+        <v>709</v>
       </c>
       <c r="E992" s="26" t="s">
-        <v>709</v>
+        <v>710</v>
       </c>
       <c r="F992" s="26" t="s">
-        <v>710</v>
+        <v>711</v>
       </c>
       <c r="G992" s="16" t="s">
         <v>58</v>
@@ -27650,22 +27663,22 @@
     </row>
     <row r="998" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A998" s="49" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="B998" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C998" s="14" t="s">
-        <v>711</v>
+        <v>712</v>
       </c>
       <c r="D998" s="15" t="s">
-        <v>712</v>
+        <v>713</v>
       </c>
       <c r="E998" s="15" t="s">
-        <v>713</v>
+        <v>714</v>
       </c>
       <c r="F998" s="15" t="s">
-        <v>714</v>
+        <v>715</v>
       </c>
       <c r="G998" s="16" t="s">
         <v>58</v>
@@ -27794,22 +27807,22 @@
     </row>
     <row r="1004" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1004" s="50" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="B1004" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1004" s="25" t="s">
-        <v>716</v>
+        <v>717</v>
       </c>
       <c r="D1004" s="26" t="s">
-        <v>717</v>
+        <v>718</v>
       </c>
       <c r="E1004" s="26" t="s">
-        <v>718</v>
+        <v>719</v>
       </c>
       <c r="F1004" s="26" t="s">
-        <v>719</v>
+        <v>720</v>
       </c>
       <c r="G1004" s="16" t="s">
         <v>58</v>
@@ -27938,22 +27951,22 @@
     </row>
     <row r="1010" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1010" s="50" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="B1010" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1010" s="14" t="s">
-        <v>720</v>
+        <v>721</v>
       </c>
       <c r="D1010" s="15" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="E1010" s="15" t="s">
-        <v>722</v>
+        <v>723</v>
       </c>
       <c r="F1010" s="15" t="s">
-        <v>723</v>
+        <v>724</v>
       </c>
       <c r="G1010" s="16" t="s">
         <v>58</v>
@@ -28082,22 +28095,22 @@
     </row>
     <row r="1016" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1016" s="50" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="B1016" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1016" s="25" t="s">
-        <v>724</v>
+        <v>725</v>
       </c>
       <c r="D1016" s="26" t="s">
-        <v>725</v>
+        <v>726</v>
       </c>
       <c r="E1016" s="26" t="s">
-        <v>726</v>
+        <v>727</v>
       </c>
       <c r="F1016" s="26" t="s">
-        <v>727</v>
+        <v>728</v>
       </c>
       <c r="G1016" s="16" t="s">
         <v>58</v>
@@ -28226,22 +28239,22 @@
     </row>
     <row r="1022" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1022" s="50" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="B1022" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1022" s="14" t="s">
-        <v>728</v>
+        <v>729</v>
       </c>
       <c r="D1022" s="15" t="s">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="E1022" s="15" t="s">
-        <v>730</v>
+        <v>731</v>
       </c>
       <c r="F1022" s="15" t="s">
-        <v>731</v>
+        <v>732</v>
       </c>
       <c r="G1022" s="16" t="s">
         <v>58</v>
@@ -28370,22 +28383,22 @@
     </row>
     <row r="1028" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1028" s="50" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="B1028" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C1028" s="25" t="s">
-        <v>732</v>
+        <v>733</v>
       </c>
       <c r="D1028" s="26" t="s">
-        <v>733</v>
+        <v>734</v>
       </c>
       <c r="E1028" s="26" t="s">
-        <v>734</v>
+        <v>735</v>
       </c>
       <c r="F1028" s="26" t="s">
-        <v>735</v>
+        <v>736</v>
       </c>
       <c r="G1028" s="16" t="s">
         <v>58</v>
@@ -28514,22 +28527,22 @@
     </row>
     <row r="1034" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1034" s="50" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="B1034" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C1034" s="14" t="s">
-        <v>736</v>
+        <v>737</v>
       </c>
       <c r="D1034" s="15" t="s">
-        <v>737</v>
+        <v>738</v>
       </c>
       <c r="E1034" s="15" t="s">
-        <v>738</v>
+        <v>739</v>
       </c>
       <c r="F1034" s="15" t="s">
-        <v>739</v>
+        <v>740</v>
       </c>
       <c r="G1034" s="16" t="s">
         <v>58</v>
@@ -28658,22 +28671,22 @@
     </row>
     <row r="1040" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1040" s="51" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="B1040" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C1040" s="25" t="s">
-        <v>741</v>
+        <v>742</v>
       </c>
       <c r="D1040" s="26" t="s">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="E1040" s="26" t="s">
-        <v>742</v>
+        <v>743</v>
       </c>
       <c r="F1040" s="26" t="s">
-        <v>743</v>
+        <v>744</v>
       </c>
       <c r="G1040" s="16" t="s">
         <v>58</v>
@@ -28802,22 +28815,22 @@
     </row>
     <row r="1046" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1046" s="51" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="B1046" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1046" s="14" t="s">
-        <v>744</v>
+        <v>745</v>
       </c>
       <c r="D1046" s="15" t="s">
-        <v>721</v>
+        <v>722</v>
       </c>
       <c r="E1046" s="15" t="s">
-        <v>745</v>
+        <v>746</v>
       </c>
       <c r="F1046" s="15" t="s">
-        <v>746</v>
+        <v>747</v>
       </c>
       <c r="G1046" s="16" t="s">
         <v>58</v>
@@ -28954,16 +28967,16 @@
         <v>53</v>
       </c>
       <c r="C1052" s="25" t="s">
-        <v>747</v>
+        <v>748</v>
       </c>
       <c r="D1052" s="26" t="s">
-        <v>748</v>
+        <v>749</v>
       </c>
       <c r="E1052" s="26" t="s">
-        <v>749</v>
+        <v>750</v>
       </c>
       <c r="F1052" s="26" t="s">
-        <v>750</v>
+        <v>751</v>
       </c>
       <c r="G1052" s="16" t="s">
         <v>58</v>
@@ -29100,16 +29113,16 @@
         <v>53</v>
       </c>
       <c r="C1058" s="14" t="s">
-        <v>751</v>
+        <v>752</v>
       </c>
       <c r="D1058" s="15" t="s">
-        <v>752</v>
+        <v>753</v>
       </c>
       <c r="E1058" s="15" t="s">
-        <v>753</v>
+        <v>754</v>
       </c>
       <c r="F1058" s="15" t="s">
-        <v>754</v>
+        <v>755</v>
       </c>
       <c r="G1058" s="16" t="s">
         <v>58</v>
@@ -30195,10 +30208,10 @@
         <v>39</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>755</v>
+        <v>756</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>756</v>
+        <v>757</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>53</v>
@@ -30216,7 +30229,7 @@
         <v>83</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>757</v>
+        <v>758</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -30424,7 +30437,7 @@
     </row>
     <row r="9" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="59" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B9" s="1">
         <v>11</v>
@@ -30453,7 +30466,7 @@
     </row>
     <row r="10" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="60" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B10" s="1">
         <v>9</v>
@@ -30482,7 +30495,7 @@
     </row>
     <row r="11" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="61" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="B11" s="1">
         <v>5</v>
@@ -30511,7 +30524,7 @@
     </row>
     <row r="12" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="62" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="B12" s="1">
         <v>5</v>
@@ -30540,7 +30553,7 @@
     </row>
     <row r="13" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="63" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="B13" s="1">
         <v>4</v>
@@ -30569,7 +30582,7 @@
     </row>
     <row r="14" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="64" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="B14" s="1">
         <v>5</v>
@@ -30598,7 +30611,7 @@
     </row>
     <row r="15" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="65" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="B15" s="1">
         <v>12</v>
@@ -30627,7 +30640,7 @@
     </row>
     <row r="16" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="66" t="s">
-        <v>597</v>
+        <v>598</v>
       </c>
       <c r="B16" s="1">
         <v>4</v>
@@ -30656,7 +30669,7 @@
     </row>
     <row r="17" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" s="67" t="s">
-        <v>613</v>
+        <v>614</v>
       </c>
       <c r="B17" s="1">
         <v>7</v>
@@ -30685,7 +30698,7 @@
     </row>
     <row r="18" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="68" t="s">
-        <v>645</v>
+        <v>646</v>
       </c>
       <c r="B18" s="1">
         <v>6</v>
@@ -30714,7 +30727,7 @@
     </row>
     <row r="19" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="69" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="B19" s="1">
         <v>6</v>
@@ -30743,7 +30756,7 @@
     </row>
     <row r="20" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="70" t="s">
-        <v>694</v>
+        <v>695</v>
       </c>
       <c r="B20" s="1">
         <v>5</v>
@@ -30772,7 +30785,7 @@
     </row>
     <row r="21" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="71" t="s">
-        <v>715</v>
+        <v>716</v>
       </c>
       <c r="B21" s="1">
         <v>6</v>
@@ -30801,7 +30814,7 @@
     </row>
     <row r="22" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="72" t="s">
-        <v>740</v>
+        <v>741</v>
       </c>
       <c r="B22" s="1">
         <v>2</v>
@@ -30830,7 +30843,7 @@
     </row>
     <row r="23" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="73" t="s">
-        <v>758</v>
+        <v>759</v>
       </c>
       <c r="B23" s="73">
         <v>153</v>
@@ -30881,7 +30894,7 @@
         <v>44</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>756</v>
+        <v>757</v>
       </c>
       <c r="C1" s="10" t="s">
         <v>71</v>
@@ -30890,7 +30903,7 @@
         <v>83</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="F1" s="10" t="s">
         <v>97</v>
@@ -31041,10 +31054,10 @@
         <v>45</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>759</v>
+        <v>760</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>756</v>
+        <v>757</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>71</v>
@@ -31053,7 +31066,7 @@
         <v>83</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>757</v>
+        <v>758</v>
       </c>
       <c r="G1" s="10" t="s">
         <v>97</v>
@@ -31064,7 +31077,7 @@
         <v>59</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>760</v>
+        <v>761</v>
       </c>
       <c r="C2" s="1">
         <f>COUNTIF(Proves!$H:$H,A2)</f>
@@ -31194,7 +31207,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="83" t="s">
-        <v>761</v>
+        <v>762</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -31202,7 +31215,7 @@
         <v>71</v>
       </c>
       <c r="B2" s="84" t="s">
-        <v>762</v>
+        <v>763</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
@@ -31222,7 +31235,7 @@
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>628</v>
+        <v>629</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
101 => fase IV => apartats de menú sense ruta com Negoci, ZUP-122 ZUP-124 OK (Chrome/ADMIN)
</commit_message>
<xml_diff>
--- a/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
+++ b/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4447" uniqueCount="764">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4449" uniqueCount="764">
   <si>
     <t>Zuppeto — Joc de probes manual (totes les pantalles)</t>
   </si>
@@ -2015,43 +2015,43 @@
     <t>Apareix a Del administrador</t>
   </si>
   <si>
+    <t>ZUP-123</t>
+  </si>
+  <si>
+    <t>Canvi de label</t>
+  </si>
+  <si>
+    <t>Editar label i desar</t>
+  </si>
+  <si>
+    <t>Text actualitzat a la capçalera</t>
+  </si>
+  <si>
+    <t>ZUP-124</t>
+  </si>
+  <si>
+    <t>Desactivar menú</t>
+  </si>
+  <si>
+    <t>marcar com a inactiu → desar</t>
+  </si>
+  <si>
+    <t>Opció desapareix de la capçalera</t>
+  </si>
+  <si>
+    <t>ZUP-125</t>
+  </si>
+  <si>
+    <t>Assignació per rol</t>
+  </si>
+  <si>
+    <t>Menú només ADMIN</t>
+  </si>
+  <si>
+    <t>Només ADMIN el veu</t>
+  </si>
+  <si>
     <t>EN CURS</t>
-  </si>
-  <si>
-    <t>ZUP-123</t>
-  </si>
-  <si>
-    <t>Canvi de label</t>
-  </si>
-  <si>
-    <t>Editar label i desar</t>
-  </si>
-  <si>
-    <t>Text actualitzat a la capçalera</t>
-  </si>
-  <si>
-    <t>ZUP-124</t>
-  </si>
-  <si>
-    <t>Desactivar menú</t>
-  </si>
-  <si>
-    <t>marcar com a inactiu → desar</t>
-  </si>
-  <si>
-    <t>Opció desapareix de la capçalera</t>
-  </si>
-  <si>
-    <t>ZUP-125</t>
-  </si>
-  <si>
-    <t>Assignació per rol</t>
-  </si>
-  <si>
-    <t>Menú només ADMIN</t>
-  </si>
-  <si>
-    <t>Només ADMIN el veu</t>
   </si>
   <si>
     <t>ZUP-126</t>
@@ -2437,7 +2437,7 @@
     </font>
     <font>
       <b/>
-      <color rgb="FF166534"/>
+      <color rgb="FF1D4ED8"/>
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
@@ -2606,7 +2606,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFDCFCE7"/>
+        <fgColor rgb="FFDBEAFE"/>
       </patternFill>
     </fill>
     <fill>
@@ -24664,7 +24664,7 @@
         <v>345</v>
       </c>
       <c r="J872" s="1" t="s">
-        <v>629</v>
+        <v>71</v>
       </c>
       <c r="K872" s="19"/>
       <c r="L872" s="18"/>
@@ -24789,16 +24789,16 @@
         <v>92</v>
       </c>
       <c r="C878" s="14" t="s">
+        <v>629</v>
+      </c>
+      <c r="D878" s="15" t="s">
         <v>630</v>
       </c>
-      <c r="D878" s="15" t="s">
+      <c r="E878" s="15" t="s">
         <v>631</v>
       </c>
-      <c r="E878" s="15" t="s">
+      <c r="F878" s="15" t="s">
         <v>632</v>
-      </c>
-      <c r="F878" s="15" t="s">
-        <v>633</v>
       </c>
       <c r="G878" s="16" t="s">
         <v>58</v>
@@ -24933,16 +24933,16 @@
         <v>53</v>
       </c>
       <c r="C884" s="25" t="s">
+        <v>633</v>
+      </c>
+      <c r="D884" s="26" t="s">
         <v>634</v>
       </c>
-      <c r="D884" s="26" t="s">
+      <c r="E884" s="26" t="s">
         <v>635</v>
       </c>
-      <c r="E884" s="26" t="s">
+      <c r="F884" s="26" t="s">
         <v>636</v>
-      </c>
-      <c r="F884" s="26" t="s">
-        <v>637</v>
       </c>
       <c r="G884" s="16" t="s">
         <v>58</v>
@@ -24950,9 +24950,11 @@
       <c r="H884" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="I884" s="18"/>
+      <c r="I884" s="18" t="s">
+        <v>345</v>
+      </c>
       <c r="J884" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K884" s="19"/>
       <c r="L884" s="18"/>
@@ -25077,16 +25079,16 @@
         <v>53</v>
       </c>
       <c r="C890" s="14" t="s">
+        <v>637</v>
+      </c>
+      <c r="D890" s="15" t="s">
         <v>638</v>
       </c>
-      <c r="D890" s="15" t="s">
+      <c r="E890" s="15" t="s">
         <v>639</v>
       </c>
-      <c r="E890" s="15" t="s">
+      <c r="F890" s="15" t="s">
         <v>640</v>
-      </c>
-      <c r="F890" s="15" t="s">
-        <v>641</v>
       </c>
       <c r="G890" s="16" t="s">
         <v>58</v>
@@ -25094,9 +25096,11 @@
       <c r="H890" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="I890" s="18"/>
+      <c r="I890" s="18" t="s">
+        <v>345</v>
+      </c>
       <c r="J890" s="1" t="s">
-        <v>60</v>
+        <v>641</v>
       </c>
       <c r="K890" s="19"/>
       <c r="L890" s="18"/>
@@ -31235,7 +31239,7 @@
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>629</v>
+        <v>641</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
102 => fase IV => codi de país a 20 i maxlength als textos de BD, toast visible sobre el modal, ZUP-128 KO/corr i ZUP-129–131 OK (Chrome/ADMIN)
</commit_message>
<xml_diff>
--- a/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
+++ b/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4449" uniqueCount="764">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4459" uniqueCount="766">
   <si>
     <t>Zuppeto — Joc de probes manual (totes les pantalles)</t>
   </si>
@@ -2051,109 +2051,124 @@
     <t>Només ADMIN el veu</t>
   </si>
   <si>
+    <t>ZUP-126</t>
+  </si>
+  <si>
+    <t>Refresc automàtic capçalera</t>
+  </si>
+  <si>
+    <t>Desar canvis a Menús</t>
+  </si>
+  <si>
+    <t>Menú superior actualitzat</t>
+  </si>
+  <si>
+    <t>Admin · Països (/admin/paisos)</t>
+  </si>
+  <si>
+    <t>ZUP-127</t>
+  </si>
+  <si>
+    <t>Catàleg de països — llistat</t>
+  </si>
+  <si>
+    <t>ADMIN → /admin/paisos</t>
+  </si>
+  <si>
+    <t>Graella països amb codi, ordre, actiu</t>
+  </si>
+  <si>
+    <t>ZUP-128</t>
+  </si>
+  <si>
+    <t>Alta país</t>
+  </si>
+  <si>
+    <t>Crear país amb codi únic (p.ex. ES)</t>
+  </si>
+  <si>
+    <t>País nou a la llista</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alta amb Codi «Catalunya» (9 lletres): error i toasts vermells.
+El Codi ha de tenir entre 2 i 8 caràcters (p. ex. ES, CAT). El requadre taronja diu «camps obligatoris» i no explica la regla del codi. El missatge de l’API surt en anglès.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Què s'ha fet:
+- Codi de país: 2 a 20 caràcters (abans 8); countries.code varchar(20)
+- El camp Codi talla a 20 (maxlength); sense error extra en Desar
+- Mateix criteri a la resta de textos amb límit de columna (usuaris, perfil, menús, rols, permisos, llocs, països, ciutats)
+- En gravar, ClampStringMaxLengthInterceptor talla al HasMaxLength (no peta la BD)
+- src/Backend/Domain/Geography/CountryCodeRules.cs
+- src/Web/src/app/shared/policies/db-field-max-length.ts
+- migració 20260906200000_WidenCountryCodeTo20
+- docs/ca/funcional-ca.md, docs/ca/tecnic-ca.md</t>
+  </si>
+  <si>
+    <t>ZUP-129</t>
+  </si>
+  <si>
+    <t>Editar país</t>
+  </si>
+  <si>
+    <t>Modificar nom o ordre → desar</t>
+  </si>
+  <si>
+    <t>Canvis persistits</t>
+  </si>
+  <si>
+    <t>ZUP-130</t>
+  </si>
+  <si>
+    <t>Desactivar país</t>
+  </si>
+  <si>
+    <t>Marcar inactiu</t>
+  </si>
+  <si>
+    <t>Estat actualitzat; coherent amb les llistes desplegables</t>
+  </si>
+  <si>
+    <t>ZUP-131</t>
+  </si>
+  <si>
+    <t>Codi duplicat</t>
+  </si>
+  <si>
+    <t>Alta amb codi ja existent</t>
+  </si>
+  <si>
+    <t>Error de validació</t>
+  </si>
+  <si>
+    <t>ZUP-132</t>
+  </si>
+  <si>
+    <t>Baixa país sense ciutats</t>
+  </si>
+  <si>
+    <t>Esborrar país sense dependències</t>
+  </si>
+  <si>
+    <t>Eliminat correctament</t>
+  </si>
+  <si>
+    <t>Admin · Ciutats (/admin/ciutats)</t>
+  </si>
+  <si>
+    <t>ZUP-133</t>
+  </si>
+  <si>
+    <t>Catàleg de ciutats — llistat</t>
+  </si>
+  <si>
+    <t>ADMIN → /admin/ciutats</t>
+  </si>
+  <si>
+    <t>Graella ciutats per país</t>
+  </si>
+  <si>
     <t>EN CURS</t>
-  </si>
-  <si>
-    <t>ZUP-126</t>
-  </si>
-  <si>
-    <t>Refresc automàtic capçalera</t>
-  </si>
-  <si>
-    <t>Desar canvis a Menús</t>
-  </si>
-  <si>
-    <t>Menú superior actualitzat</t>
-  </si>
-  <si>
-    <t>Admin · Països (/admin/paisos)</t>
-  </si>
-  <si>
-    <t>ZUP-127</t>
-  </si>
-  <si>
-    <t>Catàleg de països — llistat</t>
-  </si>
-  <si>
-    <t>ADMIN → /admin/paisos</t>
-  </si>
-  <si>
-    <t>Graella països amb codi, ordre, actiu</t>
-  </si>
-  <si>
-    <t>ZUP-128</t>
-  </si>
-  <si>
-    <t>Alta país</t>
-  </si>
-  <si>
-    <t>Crear país amb codi únic (p.ex. ES)</t>
-  </si>
-  <si>
-    <t>País nou a la llista</t>
-  </si>
-  <si>
-    <t>ZUP-129</t>
-  </si>
-  <si>
-    <t>Editar país</t>
-  </si>
-  <si>
-    <t>Modificar nom o ordre → desar</t>
-  </si>
-  <si>
-    <t>Canvis persistits</t>
-  </si>
-  <si>
-    <t>ZUP-130</t>
-  </si>
-  <si>
-    <t>Desactivar país</t>
-  </si>
-  <si>
-    <t>Marcar inactiu</t>
-  </si>
-  <si>
-    <t>Estat actualitzat; coherent amb les llistes desplegables</t>
-  </si>
-  <si>
-    <t>ZUP-131</t>
-  </si>
-  <si>
-    <t>Codi duplicat</t>
-  </si>
-  <si>
-    <t>Alta amb codi ja existent</t>
-  </si>
-  <si>
-    <t>Error de validació</t>
-  </si>
-  <si>
-    <t>ZUP-132</t>
-  </si>
-  <si>
-    <t>Baixa país sense ciutats</t>
-  </si>
-  <si>
-    <t>Esborrar país sense dependències</t>
-  </si>
-  <si>
-    <t>Eliminat correctament</t>
-  </si>
-  <si>
-    <t>Admin · Ciutats (/admin/ciutats)</t>
-  </si>
-  <si>
-    <t>ZUP-133</t>
-  </si>
-  <si>
-    <t>Catàleg de ciutats — llistat</t>
-  </si>
-  <si>
-    <t>ADMIN → /admin/ciutats</t>
-  </si>
-  <si>
-    <t>Graella ciutats per país</t>
   </si>
   <si>
     <t>ZUP-134</t>
@@ -25100,7 +25115,7 @@
         <v>345</v>
       </c>
       <c r="J890" s="1" t="s">
-        <v>641</v>
+        <v>71</v>
       </c>
       <c r="K890" s="19"/>
       <c r="L890" s="18"/>
@@ -25225,16 +25240,16 @@
         <v>53</v>
       </c>
       <c r="C896" s="25" t="s">
+        <v>641</v>
+      </c>
+      <c r="D896" s="26" t="s">
         <v>642</v>
       </c>
-      <c r="D896" s="26" t="s">
+      <c r="E896" s="26" t="s">
         <v>643</v>
       </c>
-      <c r="E896" s="26" t="s">
+      <c r="F896" s="26" t="s">
         <v>644</v>
-      </c>
-      <c r="F896" s="26" t="s">
-        <v>645</v>
       </c>
       <c r="G896" s="16" t="s">
         <v>58</v>
@@ -25242,9 +25257,11 @@
       <c r="H896" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="I896" s="18"/>
+      <c r="I896" s="18" t="s">
+        <v>345</v>
+      </c>
       <c r="J896" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K896" s="19"/>
       <c r="L896" s="18"/>
@@ -25363,22 +25380,22 @@
     </row>
     <row r="902" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A902" s="47" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="B902" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C902" s="14" t="s">
+        <v>646</v>
+      </c>
+      <c r="D902" s="15" t="s">
         <v>647</v>
       </c>
-      <c r="D902" s="15" t="s">
+      <c r="E902" s="15" t="s">
         <v>648</v>
       </c>
-      <c r="E902" s="15" t="s">
+      <c r="F902" s="15" t="s">
         <v>649</v>
-      </c>
-      <c r="F902" s="15" t="s">
-        <v>650</v>
       </c>
       <c r="G902" s="16" t="s">
         <v>58</v>
@@ -25386,9 +25403,11 @@
       <c r="H902" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="I902" s="18"/>
+      <c r="I902" s="18" t="s">
+        <v>345</v>
+      </c>
       <c r="J902" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K902" s="19"/>
       <c r="L902" s="18"/>
@@ -25507,22 +25526,22 @@
     </row>
     <row r="908" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A908" s="47" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="B908" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C908" s="25" t="s">
+        <v>650</v>
+      </c>
+      <c r="D908" s="26" t="s">
         <v>651</v>
       </c>
-      <c r="D908" s="26" t="s">
+      <c r="E908" s="26" t="s">
         <v>652</v>
       </c>
-      <c r="E908" s="26" t="s">
+      <c r="F908" s="26" t="s">
         <v>653</v>
-      </c>
-      <c r="F908" s="26" t="s">
-        <v>654</v>
       </c>
       <c r="G908" s="16" t="s">
         <v>58</v>
@@ -25530,14 +25549,24 @@
       <c r="H908" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="I908" s="18"/>
+      <c r="I908" s="18" t="s">
+        <v>345</v>
+      </c>
       <c r="J908" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="K908" s="19"/>
-      <c r="L908" s="18"/>
-      <c r="M908" s="1"/>
-      <c r="N908" s="19"/>
+        <v>83</v>
+      </c>
+      <c r="K908" s="19" t="s">
+        <v>654</v>
+      </c>
+      <c r="L908" s="18" t="s">
+        <v>345</v>
+      </c>
+      <c r="M908" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="N908" s="19" t="s">
+        <v>655</v>
+      </c>
     </row>
     <row r="909" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A909" s="47"/>
@@ -25651,22 +25680,22 @@
     </row>
     <row r="914" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A914" s="47" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="B914" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C914" s="14" t="s">
-        <v>655</v>
+        <v>656</v>
       </c>
       <c r="D914" s="15" t="s">
-        <v>656</v>
+        <v>657</v>
       </c>
       <c r="E914" s="15" t="s">
-        <v>657</v>
+        <v>658</v>
       </c>
       <c r="F914" s="15" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="G914" s="16" t="s">
         <v>58</v>
@@ -25674,9 +25703,11 @@
       <c r="H914" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="I914" s="18"/>
+      <c r="I914" s="18" t="s">
+        <v>345</v>
+      </c>
       <c r="J914" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K914" s="19"/>
       <c r="L914" s="18"/>
@@ -25795,22 +25826,22 @@
     </row>
     <row r="920" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A920" s="47" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="B920" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C920" s="25" t="s">
-        <v>659</v>
+        <v>660</v>
       </c>
       <c r="D920" s="26" t="s">
-        <v>660</v>
+        <v>661</v>
       </c>
       <c r="E920" s="26" t="s">
-        <v>661</v>
+        <v>662</v>
       </c>
       <c r="F920" s="26" t="s">
-        <v>662</v>
+        <v>663</v>
       </c>
       <c r="G920" s="16" t="s">
         <v>58</v>
@@ -25818,9 +25849,11 @@
       <c r="H920" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="I920" s="18"/>
+      <c r="I920" s="18" t="s">
+        <v>345</v>
+      </c>
       <c r="J920" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K920" s="19"/>
       <c r="L920" s="18"/>
@@ -25939,22 +25972,22 @@
     </row>
     <row r="926" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A926" s="47" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="B926" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C926" s="14" t="s">
-        <v>663</v>
+        <v>664</v>
       </c>
       <c r="D926" s="15" t="s">
-        <v>664</v>
+        <v>665</v>
       </c>
       <c r="E926" s="15" t="s">
-        <v>665</v>
+        <v>666</v>
       </c>
       <c r="F926" s="15" t="s">
-        <v>666</v>
+        <v>667</v>
       </c>
       <c r="G926" s="16" t="s">
         <v>58</v>
@@ -25962,9 +25995,11 @@
       <c r="H926" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="I926" s="18"/>
+      <c r="I926" s="18" t="s">
+        <v>345</v>
+      </c>
       <c r="J926" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K926" s="19"/>
       <c r="L926" s="18"/>
@@ -26083,22 +26118,22 @@
     </row>
     <row r="932" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A932" s="47" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="B932" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C932" s="25" t="s">
-        <v>667</v>
+        <v>668</v>
       </c>
       <c r="D932" s="26" t="s">
-        <v>668</v>
+        <v>669</v>
       </c>
       <c r="E932" s="26" t="s">
-        <v>669</v>
+        <v>670</v>
       </c>
       <c r="F932" s="26" t="s">
-        <v>670</v>
+        <v>671</v>
       </c>
       <c r="G932" s="16" t="s">
         <v>58</v>
@@ -26227,22 +26262,22 @@
     </row>
     <row r="938" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A938" s="48" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="B938" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C938" s="14" t="s">
-        <v>672</v>
+        <v>673</v>
       </c>
       <c r="D938" s="15" t="s">
-        <v>673</v>
+        <v>674</v>
       </c>
       <c r="E938" s="15" t="s">
-        <v>674</v>
+        <v>675</v>
       </c>
       <c r="F938" s="15" t="s">
-        <v>675</v>
+        <v>676</v>
       </c>
       <c r="G938" s="16" t="s">
         <v>58</v>
@@ -26252,7 +26287,7 @@
       </c>
       <c r="I938" s="18"/>
       <c r="J938" s="1" t="s">
-        <v>60</v>
+        <v>677</v>
       </c>
       <c r="K938" s="19"/>
       <c r="L938" s="18"/>
@@ -26371,22 +26406,22 @@
     </row>
     <row r="944" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A944" s="48" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="B944" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C944" s="25" t="s">
-        <v>676</v>
+        <v>678</v>
       </c>
       <c r="D944" s="26" t="s">
-        <v>677</v>
+        <v>679</v>
       </c>
       <c r="E944" s="26" t="s">
-        <v>678</v>
+        <v>680</v>
       </c>
       <c r="F944" s="26" t="s">
-        <v>679</v>
+        <v>681</v>
       </c>
       <c r="G944" s="16" t="s">
         <v>58</v>
@@ -26515,22 +26550,22 @@
     </row>
     <row r="950" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A950" s="48" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="B950" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C950" s="14" t="s">
-        <v>680</v>
+        <v>682</v>
       </c>
       <c r="D950" s="15" t="s">
-        <v>681</v>
+        <v>683</v>
       </c>
       <c r="E950" s="15" t="s">
-        <v>682</v>
+        <v>684</v>
       </c>
       <c r="F950" s="15" t="s">
-        <v>683</v>
+        <v>685</v>
       </c>
       <c r="G950" s="16" t="s">
         <v>58</v>
@@ -26659,22 +26694,22 @@
     </row>
     <row r="956" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A956" s="48" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="B956" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C956" s="25" t="s">
-        <v>684</v>
+        <v>686</v>
       </c>
       <c r="D956" s="26" t="s">
-        <v>685</v>
+        <v>687</v>
       </c>
       <c r="E956" s="26" t="s">
-        <v>686</v>
+        <v>688</v>
       </c>
       <c r="F956" s="26" t="s">
-        <v>658</v>
+        <v>659</v>
       </c>
       <c r="G956" s="16" t="s">
         <v>58</v>
@@ -26803,22 +26838,22 @@
     </row>
     <row r="962" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A962" s="48" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="B962" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C962" s="14" t="s">
-        <v>687</v>
+        <v>689</v>
       </c>
       <c r="D962" s="15" t="s">
-        <v>688</v>
+        <v>690</v>
       </c>
       <c r="E962" s="15" t="s">
-        <v>689</v>
+        <v>691</v>
       </c>
       <c r="F962" s="15" t="s">
-        <v>690</v>
+        <v>692</v>
       </c>
       <c r="G962" s="16" t="s">
         <v>58</v>
@@ -26947,22 +26982,22 @@
     </row>
     <row r="968" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A968" s="48" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="B968" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C968" s="25" t="s">
-        <v>691</v>
+        <v>693</v>
       </c>
       <c r="D968" s="26" t="s">
-        <v>692</v>
+        <v>694</v>
       </c>
       <c r="E968" s="26" t="s">
-        <v>693</v>
+        <v>695</v>
       </c>
       <c r="F968" s="26" t="s">
-        <v>694</v>
+        <v>696</v>
       </c>
       <c r="G968" s="16" t="s">
         <v>58</v>
@@ -27091,22 +27126,22 @@
     </row>
     <row r="974" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A974" s="49" t="s">
-        <v>695</v>
+        <v>697</v>
       </c>
       <c r="B974" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C974" s="14" t="s">
-        <v>696</v>
+        <v>698</v>
       </c>
       <c r="D974" s="15" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
       <c r="E974" s="15" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
       <c r="F974" s="15" t="s">
-        <v>699</v>
+        <v>701</v>
       </c>
       <c r="G974" s="16" t="s">
         <v>58</v>
@@ -27235,22 +27270,22 @@
     </row>
     <row r="980" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A980" s="49" t="s">
-        <v>695</v>
+        <v>697</v>
       </c>
       <c r="B980" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C980" s="25" t="s">
-        <v>700</v>
+        <v>702</v>
       </c>
       <c r="D980" s="26" t="s">
-        <v>701</v>
+        <v>703</v>
       </c>
       <c r="E980" s="26" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="F980" s="26" t="s">
-        <v>703</v>
+        <v>705</v>
       </c>
       <c r="G980" s="16" t="s">
         <v>58</v>
@@ -27379,22 +27414,22 @@
     </row>
     <row r="986" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A986" s="49" t="s">
-        <v>695</v>
+        <v>697</v>
       </c>
       <c r="B986" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C986" s="14" t="s">
-        <v>704</v>
+        <v>706</v>
       </c>
       <c r="D986" s="15" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
       <c r="E986" s="15" t="s">
-        <v>706</v>
+        <v>708</v>
       </c>
       <c r="F986" s="15" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
       <c r="G986" s="16" t="s">
         <v>58</v>
@@ -27523,22 +27558,22 @@
     </row>
     <row r="992" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A992" s="49" t="s">
-        <v>695</v>
+        <v>697</v>
       </c>
       <c r="B992" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C992" s="25" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="D992" s="26" t="s">
-        <v>709</v>
+        <v>711</v>
       </c>
       <c r="E992" s="26" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="F992" s="26" t="s">
-        <v>711</v>
+        <v>713</v>
       </c>
       <c r="G992" s="16" t="s">
         <v>58</v>
@@ -27667,22 +27702,22 @@
     </row>
     <row r="998" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A998" s="49" t="s">
-        <v>695</v>
+        <v>697</v>
       </c>
       <c r="B998" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C998" s="14" t="s">
-        <v>712</v>
+        <v>714</v>
       </c>
       <c r="D998" s="15" t="s">
-        <v>713</v>
+        <v>715</v>
       </c>
       <c r="E998" s="15" t="s">
-        <v>714</v>
+        <v>716</v>
       </c>
       <c r="F998" s="15" t="s">
-        <v>715</v>
+        <v>717</v>
       </c>
       <c r="G998" s="16" t="s">
         <v>58</v>
@@ -27811,22 +27846,22 @@
     </row>
     <row r="1004" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1004" s="50" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
       <c r="B1004" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1004" s="25" t="s">
-        <v>717</v>
+        <v>719</v>
       </c>
       <c r="D1004" s="26" t="s">
-        <v>718</v>
+        <v>720</v>
       </c>
       <c r="E1004" s="26" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
       <c r="F1004" s="26" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
       <c r="G1004" s="16" t="s">
         <v>58</v>
@@ -27955,22 +27990,22 @@
     </row>
     <row r="1010" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1010" s="50" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
       <c r="B1010" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1010" s="14" t="s">
-        <v>721</v>
+        <v>723</v>
       </c>
       <c r="D1010" s="15" t="s">
-        <v>722</v>
+        <v>724</v>
       </c>
       <c r="E1010" s="15" t="s">
-        <v>723</v>
+        <v>725</v>
       </c>
       <c r="F1010" s="15" t="s">
-        <v>724</v>
+        <v>726</v>
       </c>
       <c r="G1010" s="16" t="s">
         <v>58</v>
@@ -28099,22 +28134,22 @@
     </row>
     <row r="1016" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1016" s="50" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
       <c r="B1016" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1016" s="25" t="s">
-        <v>725</v>
+        <v>727</v>
       </c>
       <c r="D1016" s="26" t="s">
-        <v>726</v>
+        <v>728</v>
       </c>
       <c r="E1016" s="26" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
       <c r="F1016" s="26" t="s">
-        <v>728</v>
+        <v>730</v>
       </c>
       <c r="G1016" s="16" t="s">
         <v>58</v>
@@ -28243,22 +28278,22 @@
     </row>
     <row r="1022" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1022" s="50" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
       <c r="B1022" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1022" s="14" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
       <c r="D1022" s="15" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="E1022" s="15" t="s">
-        <v>731</v>
+        <v>733</v>
       </c>
       <c r="F1022" s="15" t="s">
-        <v>732</v>
+        <v>734</v>
       </c>
       <c r="G1022" s="16" t="s">
         <v>58</v>
@@ -28387,22 +28422,22 @@
     </row>
     <row r="1028" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1028" s="50" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
       <c r="B1028" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C1028" s="25" t="s">
-        <v>733</v>
+        <v>735</v>
       </c>
       <c r="D1028" s="26" t="s">
-        <v>734</v>
+        <v>736</v>
       </c>
       <c r="E1028" s="26" t="s">
-        <v>735</v>
+        <v>737</v>
       </c>
       <c r="F1028" s="26" t="s">
-        <v>736</v>
+        <v>738</v>
       </c>
       <c r="G1028" s="16" t="s">
         <v>58</v>
@@ -28531,22 +28566,22 @@
     </row>
     <row r="1034" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1034" s="50" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
       <c r="B1034" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C1034" s="14" t="s">
-        <v>737</v>
+        <v>739</v>
       </c>
       <c r="D1034" s="15" t="s">
-        <v>738</v>
+        <v>740</v>
       </c>
       <c r="E1034" s="15" t="s">
-        <v>739</v>
+        <v>741</v>
       </c>
       <c r="F1034" s="15" t="s">
-        <v>740</v>
+        <v>742</v>
       </c>
       <c r="G1034" s="16" t="s">
         <v>58</v>
@@ -28675,22 +28710,22 @@
     </row>
     <row r="1040" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1040" s="51" t="s">
-        <v>741</v>
+        <v>743</v>
       </c>
       <c r="B1040" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C1040" s="25" t="s">
-        <v>742</v>
+        <v>744</v>
       </c>
       <c r="D1040" s="26" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="E1040" s="26" t="s">
-        <v>743</v>
+        <v>745</v>
       </c>
       <c r="F1040" s="26" t="s">
-        <v>744</v>
+        <v>746</v>
       </c>
       <c r="G1040" s="16" t="s">
         <v>58</v>
@@ -28819,22 +28854,22 @@
     </row>
     <row r="1046" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1046" s="51" t="s">
-        <v>741</v>
+        <v>743</v>
       </c>
       <c r="B1046" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1046" s="14" t="s">
-        <v>745</v>
+        <v>747</v>
       </c>
       <c r="D1046" s="15" t="s">
-        <v>722</v>
+        <v>724</v>
       </c>
       <c r="E1046" s="15" t="s">
-        <v>746</v>
+        <v>748</v>
       </c>
       <c r="F1046" s="15" t="s">
-        <v>747</v>
+        <v>749</v>
       </c>
       <c r="G1046" s="16" t="s">
         <v>58</v>
@@ -28971,16 +29006,16 @@
         <v>53</v>
       </c>
       <c r="C1052" s="25" t="s">
-        <v>748</v>
+        <v>750</v>
       </c>
       <c r="D1052" s="26" t="s">
-        <v>749</v>
+        <v>751</v>
       </c>
       <c r="E1052" s="26" t="s">
-        <v>750</v>
+        <v>752</v>
       </c>
       <c r="F1052" s="26" t="s">
-        <v>751</v>
+        <v>753</v>
       </c>
       <c r="G1052" s="16" t="s">
         <v>58</v>
@@ -29117,16 +29152,16 @@
         <v>53</v>
       </c>
       <c r="C1058" s="14" t="s">
-        <v>752</v>
+        <v>754</v>
       </c>
       <c r="D1058" s="15" t="s">
-        <v>753</v>
+        <v>755</v>
       </c>
       <c r="E1058" s="15" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="F1058" s="15" t="s">
-        <v>755</v>
+        <v>757</v>
       </c>
       <c r="G1058" s="16" t="s">
         <v>58</v>
@@ -30212,10 +30247,10 @@
         <v>39</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>756</v>
+        <v>758</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>757</v>
+        <v>759</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>53</v>
@@ -30233,7 +30268,7 @@
         <v>83</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>758</v>
+        <v>760</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -30702,7 +30737,7 @@
     </row>
     <row r="18" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" s="68" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="B18" s="1">
         <v>6</v>
@@ -30731,7 +30766,7 @@
     </row>
     <row r="19" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" s="69" t="s">
-        <v>671</v>
+        <v>672</v>
       </c>
       <c r="B19" s="1">
         <v>6</v>
@@ -30760,7 +30795,7 @@
     </row>
     <row r="20" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="70" t="s">
-        <v>695</v>
+        <v>697</v>
       </c>
       <c r="B20" s="1">
         <v>5</v>
@@ -30789,7 +30824,7 @@
     </row>
     <row r="21" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="71" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
       <c r="B21" s="1">
         <v>6</v>
@@ -30818,7 +30853,7 @@
     </row>
     <row r="22" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="72" t="s">
-        <v>741</v>
+        <v>743</v>
       </c>
       <c r="B22" s="1">
         <v>2</v>
@@ -30847,7 +30882,7 @@
     </row>
     <row r="23" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="73" t="s">
-        <v>759</v>
+        <v>761</v>
       </c>
       <c r="B23" s="73">
         <v>153</v>
@@ -30898,7 +30933,7 @@
         <v>44</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>757</v>
+        <v>759</v>
       </c>
       <c r="C1" s="10" t="s">
         <v>71</v>
@@ -30907,7 +30942,7 @@
         <v>83</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>758</v>
+        <v>760</v>
       </c>
       <c r="F1" s="10" t="s">
         <v>97</v>
@@ -31058,10 +31093,10 @@
         <v>45</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>757</v>
+        <v>759</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>71</v>
@@ -31070,7 +31105,7 @@
         <v>83</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>758</v>
+        <v>760</v>
       </c>
       <c r="G1" s="10" t="s">
         <v>97</v>
@@ -31081,7 +31116,7 @@
         <v>59</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>761</v>
+        <v>763</v>
       </c>
       <c r="C2" s="1">
         <f>COUNTIF(Proves!$H:$H,A2)</f>
@@ -31211,7 +31246,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="83" t="s">
-        <v>762</v>
+        <v>764</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -31219,7 +31254,7 @@
         <v>71</v>
       </c>
       <c r="B2" s="84" t="s">
-        <v>763</v>
+        <v>765</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
@@ -31239,7 +31274,7 @@
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>641</v>
+        <v>677</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
103 => fase IV => missatges d’API en català, lat/long només decimals, ZUP-133 ZUP-135 OK i ZUP-134 KO/corr (Chrome/ADMIN)
</commit_message>
<xml_diff>
--- a/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
+++ b/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4459" uniqueCount="766">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4466" uniqueCount="768">
   <si>
     <t>Zuppeto — Joc de probes manual (totes les pantalles)</t>
   </si>
@@ -2168,52 +2168,64 @@
     <t>Graella ciutats per país</t>
   </si>
   <si>
+    <t>ZUP-134</t>
+  </si>
+  <si>
+    <t>Alta ciutat</t>
+  </si>
+  <si>
+    <t>Crear ciutat amb país i nom normalitzat</t>
+  </si>
+  <si>
+    <t>Ciutat nova visible</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Latitud i longitud acceptaven lletres (text lliure).
+Han de ser només decimals (signe i punt), com 41.387 / 2.170.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Què s'ha fet:
+- Latitud i longitud només accepten decimals (signe, números i un punt)
+- Les lletres no s'escriuen ni s'enganxen
+- En sortir del camp, un enter es mostra com a decimal (21 → 21.0)
+- src/Web/src/app/shared/policies/decimal-coordinate.policy.ts
+- docs/ca/funcional-ca.md, docs/ca/tecnic-ca.md</t>
+  </si>
+  <si>
+    <t>ZUP-135</t>
+  </si>
+  <si>
+    <t>Coordenades opcionals</t>
+  </si>
+  <si>
+    <t>Afegir lat/long a una ciutat</t>
+  </si>
+  <si>
+    <t>Coordenades desades</t>
+  </si>
+  <si>
+    <t>ZUP-136</t>
+  </si>
+  <si>
+    <t>Editar ciutat</t>
+  </si>
+  <si>
+    <t>Canviar nom o coordenades</t>
+  </si>
+  <si>
+    <t>ZUP-137</t>
+  </si>
+  <si>
+    <t>Unicitat nom dins país</t>
+  </si>
+  <si>
+    <t>Duplicar nom normalitzat mateix país</t>
+  </si>
+  <si>
+    <t>Error de conflicte</t>
+  </si>
+  <si>
     <t>EN CURS</t>
-  </si>
-  <si>
-    <t>ZUP-134</t>
-  </si>
-  <si>
-    <t>Alta ciutat</t>
-  </si>
-  <si>
-    <t>Crear ciutat amb país i nom normalitzat</t>
-  </si>
-  <si>
-    <t>Ciutat nova visible</t>
-  </si>
-  <si>
-    <t>ZUP-135</t>
-  </si>
-  <si>
-    <t>Coordenades opcionals</t>
-  </si>
-  <si>
-    <t>Afegir lat/long a una ciutat</t>
-  </si>
-  <si>
-    <t>Coordenades desades</t>
-  </si>
-  <si>
-    <t>ZUP-136</t>
-  </si>
-  <si>
-    <t>Editar ciutat</t>
-  </si>
-  <si>
-    <t>Canviar nom o coordenades</t>
-  </si>
-  <si>
-    <t>ZUP-137</t>
-  </si>
-  <si>
-    <t>Unicitat nom dins país</t>
-  </si>
-  <si>
-    <t>Duplicar nom normalitzat mateix país</t>
-  </si>
-  <si>
-    <t>Error de conflicte</t>
   </si>
   <si>
     <t>ZUP-138</t>
@@ -26285,9 +26297,11 @@
       <c r="H938" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="I938" s="18"/>
+      <c r="I938" s="18" t="s">
+        <v>345</v>
+      </c>
       <c r="J938" s="1" t="s">
-        <v>677</v>
+        <v>71</v>
       </c>
       <c r="K938" s="19"/>
       <c r="L938" s="18"/>
@@ -26412,16 +26426,16 @@
         <v>53</v>
       </c>
       <c r="C944" s="25" t="s">
+        <v>677</v>
+      </c>
+      <c r="D944" s="26" t="s">
         <v>678</v>
       </c>
-      <c r="D944" s="26" t="s">
+      <c r="E944" s="26" t="s">
         <v>679</v>
       </c>
-      <c r="E944" s="26" t="s">
+      <c r="F944" s="26" t="s">
         <v>680</v>
-      </c>
-      <c r="F944" s="26" t="s">
-        <v>681</v>
       </c>
       <c r="G944" s="16" t="s">
         <v>58</v>
@@ -26429,14 +26443,24 @@
       <c r="H944" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="I944" s="18"/>
+      <c r="I944" s="18" t="s">
+        <v>345</v>
+      </c>
       <c r="J944" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="K944" s="19"/>
-      <c r="L944" s="18"/>
-      <c r="M944" s="1"/>
-      <c r="N944" s="19"/>
+        <v>83</v>
+      </c>
+      <c r="K944" s="19" t="s">
+        <v>681</v>
+      </c>
+      <c r="L944" s="18" t="s">
+        <v>345</v>
+      </c>
+      <c r="M944" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="N944" s="19" t="s">
+        <v>682</v>
+      </c>
     </row>
     <row r="945" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A945" s="48"/>
@@ -26556,16 +26580,16 @@
         <v>53</v>
       </c>
       <c r="C950" s="14" t="s">
-        <v>682</v>
+        <v>683</v>
       </c>
       <c r="D950" s="15" t="s">
-        <v>683</v>
+        <v>684</v>
       </c>
       <c r="E950" s="15" t="s">
-        <v>684</v>
+        <v>685</v>
       </c>
       <c r="F950" s="15" t="s">
-        <v>685</v>
+        <v>686</v>
       </c>
       <c r="G950" s="16" t="s">
         <v>58</v>
@@ -26573,9 +26597,11 @@
       <c r="H950" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="I950" s="18"/>
+      <c r="I950" s="18" t="s">
+        <v>345</v>
+      </c>
       <c r="J950" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K950" s="19"/>
       <c r="L950" s="18"/>
@@ -26700,13 +26726,13 @@
         <v>92</v>
       </c>
       <c r="C956" s="25" t="s">
-        <v>686</v>
+        <v>687</v>
       </c>
       <c r="D956" s="26" t="s">
-        <v>687</v>
+        <v>688</v>
       </c>
       <c r="E956" s="26" t="s">
-        <v>688</v>
+        <v>689</v>
       </c>
       <c r="F956" s="26" t="s">
         <v>659</v>
@@ -26844,16 +26870,16 @@
         <v>53</v>
       </c>
       <c r="C962" s="14" t="s">
-        <v>689</v>
+        <v>690</v>
       </c>
       <c r="D962" s="15" t="s">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="E962" s="15" t="s">
-        <v>691</v>
+        <v>692</v>
       </c>
       <c r="F962" s="15" t="s">
-        <v>692</v>
+        <v>693</v>
       </c>
       <c r="G962" s="16" t="s">
         <v>58</v>
@@ -26863,7 +26889,7 @@
       </c>
       <c r="I962" s="18"/>
       <c r="J962" s="1" t="s">
-        <v>60</v>
+        <v>694</v>
       </c>
       <c r="K962" s="19"/>
       <c r="L962" s="18"/>
@@ -26988,16 +27014,16 @@
         <v>92</v>
       </c>
       <c r="C968" s="25" t="s">
-        <v>693</v>
+        <v>695</v>
       </c>
       <c r="D968" s="26" t="s">
-        <v>694</v>
+        <v>696</v>
       </c>
       <c r="E968" s="26" t="s">
-        <v>695</v>
+        <v>697</v>
       </c>
       <c r="F968" s="26" t="s">
-        <v>696</v>
+        <v>698</v>
       </c>
       <c r="G968" s="16" t="s">
         <v>58</v>
@@ -27126,22 +27152,22 @@
     </row>
     <row r="974" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A974" s="49" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
       <c r="B974" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C974" s="14" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
       <c r="D974" s="15" t="s">
-        <v>699</v>
+        <v>701</v>
       </c>
       <c r="E974" s="15" t="s">
-        <v>700</v>
+        <v>702</v>
       </c>
       <c r="F974" s="15" t="s">
-        <v>701</v>
+        <v>703</v>
       </c>
       <c r="G974" s="16" t="s">
         <v>58</v>
@@ -27270,22 +27296,22 @@
     </row>
     <row r="980" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A980" s="49" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
       <c r="B980" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C980" s="25" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="D980" s="26" t="s">
-        <v>703</v>
+        <v>705</v>
       </c>
       <c r="E980" s="26" t="s">
-        <v>704</v>
+        <v>706</v>
       </c>
       <c r="F980" s="26" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
       <c r="G980" s="16" t="s">
         <v>58</v>
@@ -27414,22 +27440,22 @@
     </row>
     <row r="986" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A986" s="49" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
       <c r="B986" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C986" s="14" t="s">
-        <v>706</v>
+        <v>708</v>
       </c>
       <c r="D986" s="15" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
       <c r="E986" s="15" t="s">
-        <v>708</v>
+        <v>710</v>
       </c>
       <c r="F986" s="15" t="s">
-        <v>709</v>
+        <v>711</v>
       </c>
       <c r="G986" s="16" t="s">
         <v>58</v>
@@ -27558,22 +27584,22 @@
     </row>
     <row r="992" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A992" s="49" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
       <c r="B992" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C992" s="25" t="s">
-        <v>710</v>
+        <v>712</v>
       </c>
       <c r="D992" s="26" t="s">
-        <v>711</v>
+        <v>713</v>
       </c>
       <c r="E992" s="26" t="s">
-        <v>712</v>
+        <v>714</v>
       </c>
       <c r="F992" s="26" t="s">
-        <v>713</v>
+        <v>715</v>
       </c>
       <c r="G992" s="16" t="s">
         <v>58</v>
@@ -27702,22 +27728,22 @@
     </row>
     <row r="998" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A998" s="49" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
       <c r="B998" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C998" s="14" t="s">
-        <v>714</v>
+        <v>716</v>
       </c>
       <c r="D998" s="15" t="s">
-        <v>715</v>
+        <v>717</v>
       </c>
       <c r="E998" s="15" t="s">
-        <v>716</v>
+        <v>718</v>
       </c>
       <c r="F998" s="15" t="s">
-        <v>717</v>
+        <v>719</v>
       </c>
       <c r="G998" s="16" t="s">
         <v>58</v>
@@ -27846,22 +27872,22 @@
     </row>
     <row r="1004" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1004" s="50" t="s">
-        <v>718</v>
+        <v>720</v>
       </c>
       <c r="B1004" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1004" s="25" t="s">
-        <v>719</v>
+        <v>721</v>
       </c>
       <c r="D1004" s="26" t="s">
-        <v>720</v>
+        <v>722</v>
       </c>
       <c r="E1004" s="26" t="s">
-        <v>721</v>
+        <v>723</v>
       </c>
       <c r="F1004" s="26" t="s">
-        <v>722</v>
+        <v>724</v>
       </c>
       <c r="G1004" s="16" t="s">
         <v>58</v>
@@ -27990,22 +28016,22 @@
     </row>
     <row r="1010" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1010" s="50" t="s">
-        <v>718</v>
+        <v>720</v>
       </c>
       <c r="B1010" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1010" s="14" t="s">
-        <v>723</v>
+        <v>725</v>
       </c>
       <c r="D1010" s="15" t="s">
-        <v>724</v>
+        <v>726</v>
       </c>
       <c r="E1010" s="15" t="s">
-        <v>725</v>
+        <v>727</v>
       </c>
       <c r="F1010" s="15" t="s">
-        <v>726</v>
+        <v>728</v>
       </c>
       <c r="G1010" s="16" t="s">
         <v>58</v>
@@ -28134,22 +28160,22 @@
     </row>
     <row r="1016" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1016" s="50" t="s">
-        <v>718</v>
+        <v>720</v>
       </c>
       <c r="B1016" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1016" s="25" t="s">
-        <v>727</v>
+        <v>729</v>
       </c>
       <c r="D1016" s="26" t="s">
-        <v>728</v>
+        <v>730</v>
       </c>
       <c r="E1016" s="26" t="s">
-        <v>729</v>
+        <v>731</v>
       </c>
       <c r="F1016" s="26" t="s">
-        <v>730</v>
+        <v>732</v>
       </c>
       <c r="G1016" s="16" t="s">
         <v>58</v>
@@ -28278,22 +28304,22 @@
     </row>
     <row r="1022" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1022" s="50" t="s">
-        <v>718</v>
+        <v>720</v>
       </c>
       <c r="B1022" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1022" s="14" t="s">
-        <v>731</v>
+        <v>733</v>
       </c>
       <c r="D1022" s="15" t="s">
-        <v>732</v>
+        <v>734</v>
       </c>
       <c r="E1022" s="15" t="s">
-        <v>733</v>
+        <v>735</v>
       </c>
       <c r="F1022" s="15" t="s">
-        <v>734</v>
+        <v>736</v>
       </c>
       <c r="G1022" s="16" t="s">
         <v>58</v>
@@ -28422,22 +28448,22 @@
     </row>
     <row r="1028" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1028" s="50" t="s">
-        <v>718</v>
+        <v>720</v>
       </c>
       <c r="B1028" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C1028" s="25" t="s">
-        <v>735</v>
+        <v>737</v>
       </c>
       <c r="D1028" s="26" t="s">
-        <v>736</v>
+        <v>738</v>
       </c>
       <c r="E1028" s="26" t="s">
-        <v>737</v>
+        <v>739</v>
       </c>
       <c r="F1028" s="26" t="s">
-        <v>738</v>
+        <v>740</v>
       </c>
       <c r="G1028" s="16" t="s">
         <v>58</v>
@@ -28566,22 +28592,22 @@
     </row>
     <row r="1034" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1034" s="50" t="s">
-        <v>718</v>
+        <v>720</v>
       </c>
       <c r="B1034" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C1034" s="14" t="s">
-        <v>739</v>
+        <v>741</v>
       </c>
       <c r="D1034" s="15" t="s">
-        <v>740</v>
+        <v>742</v>
       </c>
       <c r="E1034" s="15" t="s">
-        <v>741</v>
+        <v>743</v>
       </c>
       <c r="F1034" s="15" t="s">
-        <v>742</v>
+        <v>744</v>
       </c>
       <c r="G1034" s="16" t="s">
         <v>58</v>
@@ -28710,22 +28736,22 @@
     </row>
     <row r="1040" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1040" s="51" t="s">
-        <v>743</v>
+        <v>745</v>
       </c>
       <c r="B1040" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C1040" s="25" t="s">
-        <v>744</v>
+        <v>746</v>
       </c>
       <c r="D1040" s="26" t="s">
-        <v>732</v>
+        <v>734</v>
       </c>
       <c r="E1040" s="26" t="s">
-        <v>745</v>
+        <v>747</v>
       </c>
       <c r="F1040" s="26" t="s">
-        <v>746</v>
+        <v>748</v>
       </c>
       <c r="G1040" s="16" t="s">
         <v>58</v>
@@ -28854,22 +28880,22 @@
     </row>
     <row r="1046" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1046" s="51" t="s">
-        <v>743</v>
+        <v>745</v>
       </c>
       <c r="B1046" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1046" s="14" t="s">
-        <v>747</v>
+        <v>749</v>
       </c>
       <c r="D1046" s="15" t="s">
-        <v>724</v>
+        <v>726</v>
       </c>
       <c r="E1046" s="15" t="s">
-        <v>748</v>
+        <v>750</v>
       </c>
       <c r="F1046" s="15" t="s">
-        <v>749</v>
+        <v>751</v>
       </c>
       <c r="G1046" s="16" t="s">
         <v>58</v>
@@ -29006,16 +29032,16 @@
         <v>53</v>
       </c>
       <c r="C1052" s="25" t="s">
-        <v>750</v>
+        <v>752</v>
       </c>
       <c r="D1052" s="26" t="s">
-        <v>751</v>
+        <v>753</v>
       </c>
       <c r="E1052" s="26" t="s">
-        <v>752</v>
+        <v>754</v>
       </c>
       <c r="F1052" s="26" t="s">
-        <v>753</v>
+        <v>755</v>
       </c>
       <c r="G1052" s="16" t="s">
         <v>58</v>
@@ -29152,16 +29178,16 @@
         <v>53</v>
       </c>
       <c r="C1058" s="14" t="s">
-        <v>754</v>
+        <v>756</v>
       </c>
       <c r="D1058" s="15" t="s">
-        <v>755</v>
+        <v>757</v>
       </c>
       <c r="E1058" s="15" t="s">
-        <v>756</v>
+        <v>758</v>
       </c>
       <c r="F1058" s="15" t="s">
-        <v>757</v>
+        <v>759</v>
       </c>
       <c r="G1058" s="16" t="s">
         <v>58</v>
@@ -30247,10 +30273,10 @@
         <v>39</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>758</v>
+        <v>760</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>759</v>
+        <v>761</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>53</v>
@@ -30268,7 +30294,7 @@
         <v>83</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -30795,7 +30821,7 @@
     </row>
     <row r="20" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="70" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
       <c r="B20" s="1">
         <v>5</v>
@@ -30824,7 +30850,7 @@
     </row>
     <row r="21" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="71" t="s">
-        <v>718</v>
+        <v>720</v>
       </c>
       <c r="B21" s="1">
         <v>6</v>
@@ -30853,7 +30879,7 @@
     </row>
     <row r="22" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="72" t="s">
-        <v>743</v>
+        <v>745</v>
       </c>
       <c r="B22" s="1">
         <v>2</v>
@@ -30882,7 +30908,7 @@
     </row>
     <row r="23" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="73" t="s">
-        <v>761</v>
+        <v>763</v>
       </c>
       <c r="B23" s="73">
         <v>153</v>
@@ -30933,7 +30959,7 @@
         <v>44</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>759</v>
+        <v>761</v>
       </c>
       <c r="C1" s="10" t="s">
         <v>71</v>
@@ -30942,7 +30968,7 @@
         <v>83</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
       <c r="F1" s="10" t="s">
         <v>97</v>
@@ -31093,10 +31119,10 @@
         <v>45</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>762</v>
+        <v>764</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>759</v>
+        <v>761</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>71</v>
@@ -31105,7 +31131,7 @@
         <v>83</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>760</v>
+        <v>762</v>
       </c>
       <c r="G1" s="10" t="s">
         <v>97</v>
@@ -31116,7 +31142,7 @@
         <v>59</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>763</v>
+        <v>765</v>
       </c>
       <c r="C2" s="1">
         <f>COUNTIF(Proves!$H:$H,A2)</f>
@@ -31246,7 +31272,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="83" t="s">
-        <v>764</v>
+        <v>766</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -31254,7 +31280,7 @@
         <v>71</v>
       </c>
       <c r="B2" s="84" t="s">
-        <v>765</v>
+        <v>767</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
@@ -31274,7 +31300,7 @@
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>677</v>
+        <v>694</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
104 => fase IV => toasts i excepcions d’API en català (ciutat duplicada), ZUP-137 KO/corr i ZUP-139 OK (Chrome/ADMIN)
</commit_message>
<xml_diff>
--- a/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
+++ b/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4466" uniqueCount="768">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4472" uniqueCount="771">
   <si>
     <t>Zuppeto — Joc de probes manual (totes les pantalles)</t>
   </si>
@@ -2225,46 +2225,55 @@
     <t>Error de conflicte</t>
   </si>
   <si>
+    <t>07-09-2026</t>
+  </si>
+  <si>
+    <t>El duplicat es detecta (409 Conflicte), però el cos del toast surt en anglès: «City name already exists in this country.» La resta de la UI és en català.</t>
+  </si>
+  <si>
+    <t>Què s'ha fet: El 409 de nom de ciutat duplicat ja no reenvia el text anglès de l’excepció; el missatge fix és «Ja existeix una ciutat amb aquest nom en aquest país.» El front tradueix cossos anglesos residuals al toast (p. ex. City name already exists…). També s’han passat a català les excepcions de domini que podien filtrar-se. Fitxers: GeographicAdminAppService.cs, GeographicCatalogRepository.cs, api-message-ca.policy.ts, error-notifications.service.ts, excepcions de Domain/Infrastructure, docs/ca/funcional-ca.md, docs/ca/tecnic-ca.md.</t>
+  </si>
+  <si>
+    <t>ZUP-138</t>
+  </si>
+  <si>
+    <t>Ciutat a la llista desplegable de llocs</t>
+  </si>
+  <si>
+    <t>Ciutat creada → provar la llista de ciutats a /places</t>
+  </si>
+  <si>
+    <t>Ciutat disponible a la cerca</t>
+  </si>
+  <si>
+    <t>Admin · Llocs (/admin/llocs)</t>
+  </si>
+  <si>
+    <t>ZUP-139</t>
+  </si>
+  <si>
+    <t>Catàleg de llocs — llistat</t>
+  </si>
+  <si>
+    <t>ADMIN → /admin/llocs</t>
+  </si>
+  <si>
+    <t>Graella manteniment llocs</t>
+  </si>
+  <si>
+    <t>ZUP-140</t>
+  </si>
+  <si>
+    <t>Alta lloc manual</t>
+  </si>
+  <si>
+    <t>Crear lloc amb dades mínimes obligatòries</t>
+  </si>
+  <si>
+    <t>Lloc al catàleg i visible a /places</t>
+  </si>
+  <si>
     <t>EN CURS</t>
-  </si>
-  <si>
-    <t>ZUP-138</t>
-  </si>
-  <si>
-    <t>Ciutat a la llista desplegable de llocs</t>
-  </si>
-  <si>
-    <t>Ciutat creada → provar la llista de ciutats a /places</t>
-  </si>
-  <si>
-    <t>Ciutat disponible a la cerca</t>
-  </si>
-  <si>
-    <t>Admin · Llocs (/admin/llocs)</t>
-  </si>
-  <si>
-    <t>ZUP-139</t>
-  </si>
-  <si>
-    <t>Catàleg de llocs — llistat</t>
-  </si>
-  <si>
-    <t>ADMIN → /admin/llocs</t>
-  </si>
-  <si>
-    <t>Graella manteniment llocs</t>
-  </si>
-  <si>
-    <t>ZUP-140</t>
-  </si>
-  <si>
-    <t>Alta lloc manual</t>
-  </si>
-  <si>
-    <t>Crear lloc amb dades mínimes obligatòries</t>
-  </si>
-  <si>
-    <t>Lloc al catàleg i visible a /places</t>
   </si>
   <si>
     <t>ZUP-141</t>
@@ -26887,14 +26896,24 @@
       <c r="H962" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="I962" s="18"/>
+      <c r="I962" s="18" t="s">
+        <v>694</v>
+      </c>
       <c r="J962" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="K962" s="19" t="s">
+        <v>695</v>
+      </c>
+      <c r="L962" s="18" t="s">
         <v>694</v>
       </c>
-      <c r="K962" s="19"/>
-      <c r="L962" s="18"/>
-      <c r="M962" s="1"/>
-      <c r="N962" s="19"/>
+      <c r="M962" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="N962" s="19" t="s">
+        <v>696</v>
+      </c>
     </row>
     <row r="963" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A963" s="48"/>
@@ -27014,16 +27033,16 @@
         <v>92</v>
       </c>
       <c r="C968" s="25" t="s">
-        <v>695</v>
+        <v>697</v>
       </c>
       <c r="D968" s="26" t="s">
-        <v>696</v>
+        <v>698</v>
       </c>
       <c r="E968" s="26" t="s">
-        <v>697</v>
+        <v>699</v>
       </c>
       <c r="F968" s="26" t="s">
-        <v>698</v>
+        <v>700</v>
       </c>
       <c r="G968" s="16" t="s">
         <v>58</v>
@@ -27152,22 +27171,22 @@
     </row>
     <row r="974" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A974" s="49" t="s">
-        <v>699</v>
+        <v>701</v>
       </c>
       <c r="B974" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C974" s="14" t="s">
-        <v>700</v>
+        <v>702</v>
       </c>
       <c r="D974" s="15" t="s">
-        <v>701</v>
+        <v>703</v>
       </c>
       <c r="E974" s="15" t="s">
-        <v>702</v>
+        <v>704</v>
       </c>
       <c r="F974" s="15" t="s">
-        <v>703</v>
+        <v>705</v>
       </c>
       <c r="G974" s="16" t="s">
         <v>58</v>
@@ -27175,9 +27194,11 @@
       <c r="H974" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="I974" s="18"/>
+      <c r="I974" s="18" t="s">
+        <v>694</v>
+      </c>
       <c r="J974" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K974" s="19"/>
       <c r="L974" s="18"/>
@@ -27296,22 +27317,22 @@
     </row>
     <row r="980" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A980" s="49" t="s">
-        <v>699</v>
+        <v>701</v>
       </c>
       <c r="B980" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C980" s="25" t="s">
-        <v>704</v>
+        <v>706</v>
       </c>
       <c r="D980" s="26" t="s">
-        <v>705</v>
+        <v>707</v>
       </c>
       <c r="E980" s="26" t="s">
-        <v>706</v>
+        <v>708</v>
       </c>
       <c r="F980" s="26" t="s">
-        <v>707</v>
+        <v>709</v>
       </c>
       <c r="G980" s="16" t="s">
         <v>58</v>
@@ -27321,7 +27342,7 @@
       </c>
       <c r="I980" s="18"/>
       <c r="J980" s="1" t="s">
-        <v>60</v>
+        <v>710</v>
       </c>
       <c r="K980" s="19"/>
       <c r="L980" s="18"/>
@@ -27440,22 +27461,22 @@
     </row>
     <row r="986" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A986" s="49" t="s">
-        <v>699</v>
+        <v>701</v>
       </c>
       <c r="B986" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C986" s="14" t="s">
-        <v>708</v>
+        <v>711</v>
       </c>
       <c r="D986" s="15" t="s">
-        <v>709</v>
+        <v>712</v>
       </c>
       <c r="E986" s="15" t="s">
-        <v>710</v>
+        <v>713</v>
       </c>
       <c r="F986" s="15" t="s">
-        <v>711</v>
+        <v>714</v>
       </c>
       <c r="G986" s="16" t="s">
         <v>58</v>
@@ -27584,22 +27605,22 @@
     </row>
     <row r="992" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A992" s="49" t="s">
-        <v>699</v>
+        <v>701</v>
       </c>
       <c r="B992" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C992" s="25" t="s">
-        <v>712</v>
+        <v>715</v>
       </c>
       <c r="D992" s="26" t="s">
-        <v>713</v>
+        <v>716</v>
       </c>
       <c r="E992" s="26" t="s">
-        <v>714</v>
+        <v>717</v>
       </c>
       <c r="F992" s="26" t="s">
-        <v>715</v>
+        <v>718</v>
       </c>
       <c r="G992" s="16" t="s">
         <v>58</v>
@@ -27728,22 +27749,22 @@
     </row>
     <row r="998" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A998" s="49" t="s">
-        <v>699</v>
+        <v>701</v>
       </c>
       <c r="B998" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C998" s="14" t="s">
-        <v>716</v>
+        <v>719</v>
       </c>
       <c r="D998" s="15" t="s">
-        <v>717</v>
+        <v>720</v>
       </c>
       <c r="E998" s="15" t="s">
-        <v>718</v>
+        <v>721</v>
       </c>
       <c r="F998" s="15" t="s">
-        <v>719</v>
+        <v>722</v>
       </c>
       <c r="G998" s="16" t="s">
         <v>58</v>
@@ -27872,22 +27893,22 @@
     </row>
     <row r="1004" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1004" s="50" t="s">
-        <v>720</v>
+        <v>723</v>
       </c>
       <c r="B1004" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1004" s="25" t="s">
-        <v>721</v>
+        <v>724</v>
       </c>
       <c r="D1004" s="26" t="s">
-        <v>722</v>
+        <v>725</v>
       </c>
       <c r="E1004" s="26" t="s">
-        <v>723</v>
+        <v>726</v>
       </c>
       <c r="F1004" s="26" t="s">
-        <v>724</v>
+        <v>727</v>
       </c>
       <c r="G1004" s="16" t="s">
         <v>58</v>
@@ -28016,22 +28037,22 @@
     </row>
     <row r="1010" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1010" s="50" t="s">
-        <v>720</v>
+        <v>723</v>
       </c>
       <c r="B1010" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1010" s="14" t="s">
-        <v>725</v>
+        <v>728</v>
       </c>
       <c r="D1010" s="15" t="s">
-        <v>726</v>
+        <v>729</v>
       </c>
       <c r="E1010" s="15" t="s">
-        <v>727</v>
+        <v>730</v>
       </c>
       <c r="F1010" s="15" t="s">
-        <v>728</v>
+        <v>731</v>
       </c>
       <c r="G1010" s="16" t="s">
         <v>58</v>
@@ -28160,22 +28181,22 @@
     </row>
     <row r="1016" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1016" s="50" t="s">
-        <v>720</v>
+        <v>723</v>
       </c>
       <c r="B1016" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1016" s="25" t="s">
-        <v>729</v>
+        <v>732</v>
       </c>
       <c r="D1016" s="26" t="s">
-        <v>730</v>
+        <v>733</v>
       </c>
       <c r="E1016" s="26" t="s">
-        <v>731</v>
+        <v>734</v>
       </c>
       <c r="F1016" s="26" t="s">
-        <v>732</v>
+        <v>735</v>
       </c>
       <c r="G1016" s="16" t="s">
         <v>58</v>
@@ -28304,22 +28325,22 @@
     </row>
     <row r="1022" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1022" s="50" t="s">
-        <v>720</v>
+        <v>723</v>
       </c>
       <c r="B1022" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1022" s="14" t="s">
-        <v>733</v>
+        <v>736</v>
       </c>
       <c r="D1022" s="15" t="s">
-        <v>734</v>
+        <v>737</v>
       </c>
       <c r="E1022" s="15" t="s">
-        <v>735</v>
+        <v>738</v>
       </c>
       <c r="F1022" s="15" t="s">
-        <v>736</v>
+        <v>739</v>
       </c>
       <c r="G1022" s="16" t="s">
         <v>58</v>
@@ -28448,22 +28469,22 @@
     </row>
     <row r="1028" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1028" s="50" t="s">
-        <v>720</v>
+        <v>723</v>
       </c>
       <c r="B1028" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C1028" s="25" t="s">
-        <v>737</v>
+        <v>740</v>
       </c>
       <c r="D1028" s="26" t="s">
-        <v>738</v>
+        <v>741</v>
       </c>
       <c r="E1028" s="26" t="s">
-        <v>739</v>
+        <v>742</v>
       </c>
       <c r="F1028" s="26" t="s">
-        <v>740</v>
+        <v>743</v>
       </c>
       <c r="G1028" s="16" t="s">
         <v>58</v>
@@ -28592,22 +28613,22 @@
     </row>
     <row r="1034" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1034" s="50" t="s">
-        <v>720</v>
+        <v>723</v>
       </c>
       <c r="B1034" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C1034" s="14" t="s">
-        <v>741</v>
+        <v>744</v>
       </c>
       <c r="D1034" s="15" t="s">
-        <v>742</v>
+        <v>745</v>
       </c>
       <c r="E1034" s="15" t="s">
-        <v>743</v>
+        <v>746</v>
       </c>
       <c r="F1034" s="15" t="s">
-        <v>744</v>
+        <v>747</v>
       </c>
       <c r="G1034" s="16" t="s">
         <v>58</v>
@@ -28736,22 +28757,22 @@
     </row>
     <row r="1040" ht="36" customHeight="1" hidden="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1040" s="51" t="s">
-        <v>745</v>
+        <v>748</v>
       </c>
       <c r="B1040" s="27" t="s">
         <v>92</v>
       </c>
       <c r="C1040" s="25" t="s">
-        <v>746</v>
+        <v>749</v>
       </c>
       <c r="D1040" s="26" t="s">
-        <v>734</v>
+        <v>737</v>
       </c>
       <c r="E1040" s="26" t="s">
-        <v>747</v>
+        <v>750</v>
       </c>
       <c r="F1040" s="26" t="s">
-        <v>748</v>
+        <v>751</v>
       </c>
       <c r="G1040" s="16" t="s">
         <v>58</v>
@@ -28880,22 +28901,22 @@
     </row>
     <row r="1046" ht="36" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1046" s="51" t="s">
-        <v>745</v>
+        <v>748</v>
       </c>
       <c r="B1046" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C1046" s="14" t="s">
-        <v>749</v>
+        <v>752</v>
       </c>
       <c r="D1046" s="15" t="s">
-        <v>726</v>
+        <v>729</v>
       </c>
       <c r="E1046" s="15" t="s">
-        <v>750</v>
+        <v>753</v>
       </c>
       <c r="F1046" s="15" t="s">
-        <v>751</v>
+        <v>754</v>
       </c>
       <c r="G1046" s="16" t="s">
         <v>58</v>
@@ -29032,16 +29053,16 @@
         <v>53</v>
       </c>
       <c r="C1052" s="25" t="s">
-        <v>752</v>
+        <v>755</v>
       </c>
       <c r="D1052" s="26" t="s">
-        <v>753</v>
+        <v>756</v>
       </c>
       <c r="E1052" s="26" t="s">
-        <v>754</v>
+        <v>757</v>
       </c>
       <c r="F1052" s="26" t="s">
-        <v>755</v>
+        <v>758</v>
       </c>
       <c r="G1052" s="16" t="s">
         <v>58</v>
@@ -29178,16 +29199,16 @@
         <v>53</v>
       </c>
       <c r="C1058" s="14" t="s">
-        <v>756</v>
+        <v>759</v>
       </c>
       <c r="D1058" s="15" t="s">
-        <v>757</v>
+        <v>760</v>
       </c>
       <c r="E1058" s="15" t="s">
-        <v>758</v>
+        <v>761</v>
       </c>
       <c r="F1058" s="15" t="s">
-        <v>759</v>
+        <v>762</v>
       </c>
       <c r="G1058" s="16" t="s">
         <v>58</v>
@@ -30273,10 +30294,10 @@
         <v>39</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>760</v>
+        <v>763</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>761</v>
+        <v>764</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>53</v>
@@ -30294,7 +30315,7 @@
         <v>83</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>762</v>
+        <v>765</v>
       </c>
     </row>
     <row r="2" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
@@ -30821,7 +30842,7 @@
     </row>
     <row r="20" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" s="70" t="s">
-        <v>699</v>
+        <v>701</v>
       </c>
       <c r="B20" s="1">
         <v>5</v>
@@ -30850,7 +30871,7 @@
     </row>
     <row r="21" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" s="71" t="s">
-        <v>720</v>
+        <v>723</v>
       </c>
       <c r="B21" s="1">
         <v>6</v>
@@ -30879,7 +30900,7 @@
     </row>
     <row r="22" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" s="72" t="s">
-        <v>745</v>
+        <v>748</v>
       </c>
       <c r="B22" s="1">
         <v>2</v>
@@ -30908,7 +30929,7 @@
     </row>
     <row r="23" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" s="73" t="s">
-        <v>763</v>
+        <v>766</v>
       </c>
       <c r="B23" s="73">
         <v>153</v>
@@ -30959,7 +30980,7 @@
         <v>44</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>761</v>
+        <v>764</v>
       </c>
       <c r="C1" s="10" t="s">
         <v>71</v>
@@ -30968,7 +30989,7 @@
         <v>83</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>762</v>
+        <v>765</v>
       </c>
       <c r="F1" s="10" t="s">
         <v>97</v>
@@ -31119,10 +31140,10 @@
         <v>45</v>
       </c>
       <c r="B1" s="10" t="s">
+        <v>767</v>
+      </c>
+      <c r="C1" s="10" t="s">
         <v>764</v>
-      </c>
-      <c r="C1" s="10" t="s">
-        <v>761</v>
       </c>
       <c r="D1" s="10" t="s">
         <v>71</v>
@@ -31131,7 +31152,7 @@
         <v>83</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>762</v>
+        <v>765</v>
       </c>
       <c r="G1" s="10" t="s">
         <v>97</v>
@@ -31142,7 +31163,7 @@
         <v>59</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>765</v>
+        <v>768</v>
       </c>
       <c r="C2" s="1">
         <f>COUNTIF(Proves!$H:$H,A2)</f>
@@ -31272,7 +31293,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="83" t="s">
-        <v>766</v>
+        <v>769</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -31280,7 +31301,7 @@
         <v>71</v>
       </c>
       <c r="B2" s="84" t="s">
-        <v>767</v>
+        <v>770</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
@@ -31300,7 +31321,7 @@
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>694</v>
+        <v>710</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
107 => fase IV => filtre SQL per país i combo de ciutats amb pins+BD+GeoNames+catàleg, format Ciutat (País) sense CP; ZUP-138 KO/corr i ZUP-143 ZUP-148–150 OK (Chrome/ADMIN)
</commit_message>
<xml_diff>
--- a/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
+++ b/docs/probes-e2e/probes-pagines/MAIN_PROBES_ZUPETTO.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4500" uniqueCount="780">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4504" uniqueCount="780">
   <si>
     <t>Zuppeto — Joc de probes manual (totes les pantalles)</t>
   </si>
@@ -27869,9 +27869,11 @@
       <c r="H998" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="I998" s="18"/>
+      <c r="I998" s="18" t="s">
+        <v>702</v>
+      </c>
       <c r="J998" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K998" s="19"/>
       <c r="L998" s="18"/>
@@ -28601,9 +28603,11 @@
       <c r="H1028" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="I1028" s="18"/>
+      <c r="I1028" s="18" t="s">
+        <v>702</v>
+      </c>
       <c r="J1028" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K1028" s="19"/>
       <c r="L1028" s="18"/>
@@ -28745,9 +28749,11 @@
       <c r="H1034" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="I1034" s="18"/>
+      <c r="I1034" s="18" t="s">
+        <v>702</v>
+      </c>
       <c r="J1034" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K1034" s="19"/>
       <c r="L1034" s="18"/>
@@ -28889,9 +28895,11 @@
       <c r="H1040" s="23" t="s">
         <v>81</v>
       </c>
-      <c r="I1040" s="18"/>
+      <c r="I1040" s="18" t="s">
+        <v>702</v>
+      </c>
       <c r="J1040" s="1" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="K1040" s="19"/>
       <c r="L1040" s="18"/>

</xml_diff>